<commit_message>
websocket auto send ping
</commit_message>
<xml_diff>
--- a/ExLibris/test_excel/exlibris_test.xlsx
+++ b/ExLibris/test_excel/exlibris_test.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\mugen\git\ex-libris\ExLibris\test_excel\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A763B134-04A3-4713-B9B5-8116F35683FF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3AA317F5-F581-4347-9A4A-71A15988A1B5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="270" yWindow="735" windowWidth="14160" windowHeight="11385" activeTab="1" xr2:uid="{705CD0B7-27A9-4291-85BD-6034C0FEE3E4}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" activeTab="1" xr2:uid="{705CD0B7-27A9-4291-85BD-6034C0FEE3E4}"/>
   </bookViews>
   <sheets>
     <sheet name="json_test" sheetId="1" r:id="rId1"/>
@@ -408,10 +408,6 @@
     <phoneticPr fontId="1"/>
   </si>
   <si>
-    <t>socket</t>
-    <phoneticPr fontId="1"/>
-  </si>
-  <si>
     <t>message 0</t>
     <phoneticPr fontId="1"/>
   </si>
@@ -432,6 +428,10 @@
   </si>
   <si>
     <t>message 6</t>
+  </si>
+  <si>
+    <t>client0</t>
+    <phoneticPr fontId="1"/>
   </si>
 </sst>
 </file>
@@ -537,328 +537,336 @@
 <file path=xl/volatileDependencies.xml><?xml version="1.0" encoding="utf-8"?>
 <volTypes xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <volType type="realTimeData">
-    <main first="rtdsrv.46c5753678554062b36cfbc3a8309d90">
-      <tp>
-        <v>1</v>
-        <stp/>
-        <stp>2dc2dd4b-711d-4c23-82ae-0ebc7a0fcb4e</stp>
+    <main first="rtdsrv.da30af61cf3e4a5a94195f27fdd074ca">
+      <tp>
+        <v>1</v>
+        <stp/>
+        <stp>8215b3c4-c6dd-45ca-955f-7abcf8c59b10</stp>
+        <tr r="G43" s="1"/>
+      </tp>
+    </main>
+    <main first="rtdsrv.da30af61cf3e4a5a94195f27fdd074ca">
+      <tp>
+        <v>1</v>
+        <stp/>
+        <stp>9b0f7522-fb02-492c-b49e-ee514a0afb74</stp>
+        <tr r="I19" s="1"/>
+      </tp>
+      <tp>
+        <v>1</v>
+        <stp/>
+        <stp>b2906bc6-1c00-408e-b9af-029ad8a22c8a</stp>
+        <tr r="G45" s="1"/>
+      </tp>
+    </main>
+    <main first="rtdsrv.da30af61cf3e4a5a94195f27fdd074ca">
+      <tp>
+        <v>1</v>
+        <stp/>
+        <stp>d41359cf-4f1b-4c32-b7a6-ae72bc604c0c</stp>
+        <tr r="E4" s="3"/>
+      </tp>
+      <tp>
+        <v>1</v>
+        <stp/>
+        <stp>d0e61287-ce66-4238-973b-50d98efec0b0</stp>
+        <tr r="G21" s="1"/>
+      </tp>
+    </main>
+    <main first="rtdsrv.da30af61cf3e4a5a94195f27fdd074ca">
+      <tp>
+        <v>1</v>
+        <stp/>
+        <stp>8f86837d-5995-4ea9-b8df-554737d4a4c4</stp>
+        <tr r="G23" s="1"/>
+      </tp>
+    </main>
+    <main first="rtdsrv.da30af61cf3e4a5a94195f27fdd074ca">
+      <tp>
+        <v>1</v>
+        <stp/>
+        <stp>09a9dcdd-c4f5-4f8d-972c-09e588239e14</stp>
+        <tr r="G57" s="1"/>
+      </tp>
+    </main>
+    <main first="rtdsrv.da30af61cf3e4a5a94195f27fdd074ca">
+      <tp>
+        <v>1</v>
+        <stp/>
+        <stp>908e95de-4bbf-44e4-9ba9-cb11708173c0</stp>
+        <tr r="G50" s="1"/>
+      </tp>
+    </main>
+    <main first="rtdsrv.da30af61cf3e4a5a94195f27fdd074ca">
+      <tp>
+        <v>1</v>
+        <stp/>
+        <stp>fe13b170-c101-4957-b8f0-2344d475cd18</stp>
+        <tr r="G55" s="1"/>
+      </tp>
+    </main>
+    <main first="rtdsrv.da30af61cf3e4a5a94195f27fdd074ca">
+      <tp>
+        <v>1</v>
+        <stp/>
+        <stp>2dcfdd96-f37f-4170-82b6-ff69bd97a210</stp>
+        <tr r="G35" s="1"/>
+      </tp>
+    </main>
+    <main first="rtdsrv.da30af61cf3e4a5a94195f27fdd074ca">
+      <tp>
+        <v>1</v>
+        <stp/>
+        <stp>5dc1d79c-6026-4851-abc6-80c7ee5b8ffa</stp>
+        <tr r="G26" s="1"/>
+      </tp>
+    </main>
+    <main first="rtdsrv.da30af61cf3e4a5a94195f27fdd074ca">
+      <tp>
+        <v>1</v>
+        <stp/>
+        <stp>82df0738-be39-4c04-82c3-4481c4d2f4f8</stp>
+        <tr r="G22" s="1"/>
+      </tp>
+    </main>
+    <main first="rtdsrv.da30af61cf3e4a5a94195f27fdd074ca">
+      <tp>
+        <v>1</v>
+        <stp/>
+        <stp>f7de2308-d966-4801-a61c-58826fc62941</stp>
+        <tr r="G31" s="1"/>
+      </tp>
+      <tp>
+        <v>1</v>
+        <stp/>
+        <stp>a34588c1-98f5-481d-b7d7-5337dc465e85</stp>
+        <tr r="G25" s="1"/>
+      </tp>
+    </main>
+    <main first="rtdsrv.da30af61cf3e4a5a94195f27fdd074ca">
+      <tp>
+        <v>1</v>
+        <stp/>
+        <stp>670267aa-3ac1-46f0-ac72-02bce736a7db</stp>
+        <tr r="G20" s="1"/>
+      </tp>
+    </main>
+    <main first="rtdsrv.da30af61cf3e4a5a94195f27fdd074ca">
+      <tp>
+        <v>1</v>
+        <stp/>
+        <stp>ac050767-4cd9-4979-a898-5d8733ee87cf</stp>
+        <tr r="G40" s="1"/>
+      </tp>
+      <tp>
+        <v>1</v>
+        <stp/>
+        <stp>ddeffaa2-ae8d-425d-9c29-c186f1411270</stp>
+        <tr r="G36" s="1"/>
+      </tp>
+      <tp>
+        <v>1</v>
+        <stp/>
+        <stp>05defc1e-b383-4186-8ac9-cd415369b65f</stp>
+        <tr r="I28" s="1"/>
+      </tp>
+      <tp>
+        <v>1</v>
+        <stp/>
+        <stp>2955d900-acde-459e-acc1-fd4531d0f232</stp>
+        <tr r="G38" s="1"/>
+      </tp>
+      <tp>
+        <v>1</v>
+        <stp/>
+        <stp>0d440dbe-5192-41d7-8815-9fbdd79aeb45</stp>
         <tr r="G49" s="1"/>
       </tp>
+      <tp>
+        <v>1</v>
+        <stp/>
+        <stp>6a3f0ae0-3bb0-4ddd-a9b0-a4e36d650f44</stp>
+        <tr r="G34" s="1"/>
+      </tp>
+      <tp>
+        <v>1</v>
+        <stp/>
+        <stp>76dc2e7d-4326-486e-8454-c0d1d05834c7</stp>
+        <tr r="G47" s="1"/>
+      </tp>
     </main>
-    <main first="rtdsrv.46c5753678554062b36cfbc3a8309d90">
-      <tp>
-        <v>1</v>
-        <stp/>
-        <stp>0dfbf2ac-93d8-48ae-9644-3e7db83bbb3f</stp>
+    <main first="rtdsrv.da30af61cf3e4a5a94195f27fdd074ca">
+      <tp>
+        <v>1</v>
+        <stp/>
+        <stp>7b64e19d-80a1-4c63-80d7-c0bb18ec56ba</stp>
+        <tr r="G42" s="1"/>
+      </tp>
+    </main>
+    <main first="rtdsrv.da30af61cf3e4a5a94195f27fdd074ca">
+      <tp>
+        <v>1</v>
+        <stp/>
+        <stp>40186b44-8817-45bd-b30c-66a836a08b81</stp>
+        <tr r="C2" s="2"/>
+      </tp>
+      <tp>
+        <v>1</v>
+        <stp/>
+        <stp>1b1fadc6-7e5c-4ad1-939f-63f1a4d15a17</stp>
         <tr r="G30" s="1"/>
       </tp>
       <tp>
         <v>1</v>
         <stp/>
-        <stp>03a6be81-6ca6-4265-9318-53f5bbae1498</stp>
+        <stp>fd326be5-bf91-4ef0-b1fa-f21fa8946f08</stp>
+        <tr r="G19" s="1"/>
+      </tp>
+      <tp>
+        <v>1</v>
+        <stp/>
+        <stp>6850bd1c-6e8c-40a3-8534-f66c8738c5ba</stp>
+        <tr r="G46" s="1"/>
+      </tp>
+      <tp>
+        <v>1</v>
+        <stp/>
+        <stp>e8e3f255-6c48-4e13-a2c3-966ed6bf42fc</stp>
         <tr r="G39" s="1"/>
       </tp>
       <tp>
-        <v>1</v>
-        <stp/>
-        <stp>318900f7-db95-4a26-8522-86fb0aa92689</stp>
-        <tr r="G35" s="1"/>
+        <v>10</v>
+        <stp/>
+        <stp>37de08e9-0167-4fbc-8c01-65486a4edf0f</stp>
+        <tr r="E7" s="3"/>
       </tp>
     </main>
-    <main first="rtdsrv.46c5753678554062b36cfbc3a8309d90">
-      <tp>
-        <v>1</v>
-        <stp/>
-        <stp>b8f5d4bb-2177-43ea-8bed-4d18d9e22ad3</stp>
-        <tr r="G19" s="1"/>
+    <main first="rtdsrv.da30af61cf3e4a5a94195f27fdd074ca">
+      <tp>
+        <v>1</v>
+        <stp/>
+        <stp>98a7fab1-a0a9-4330-a4eb-12261bc61dd8</stp>
+        <tr r="G44" s="1"/>
+      </tp>
+      <tp>
+        <v>1</v>
+        <stp/>
+        <stp>fed5a1d5-22bf-445e-b6a4-249329dcc638</stp>
+        <tr r="G27" s="1"/>
       </tp>
     </main>
-    <main first="rtdsrv.46c5753678554062b36cfbc3a8309d90">
-      <tp>
-        <v>1</v>
-        <stp/>
-        <stp>379ec024-27d1-4c65-b4a5-b7f7d24bfb04</stp>
-        <tr r="I28" s="1"/>
+    <main first="rtdsrv.da30af61cf3e4a5a94195f27fdd074ca">
+      <tp>
+        <v>1</v>
+        <stp/>
+        <stp>ce470760-a3c9-441d-885a-375979c3d4d3</stp>
+        <tr r="G28" s="1"/>
       </tp>
     </main>
-    <main first="rtdsrv.46c5753678554062b36cfbc3a8309d90">
-      <tp>
-        <v>18</v>
-        <stp/>
-        <stp>936a91b3-cc90-451a-922a-ab40918d6d96</stp>
-        <tr r="E7" s="3"/>
-      </tp>
-      <tp>
-        <v>1</v>
-        <stp/>
-        <stp>51de8610-3af4-4bc1-a0f2-9d303567b7fe</stp>
-        <tr r="G43" s="1"/>
-      </tp>
-      <tp>
-        <v>1</v>
-        <stp/>
-        <stp>edc04af2-bfdd-45da-8b25-3a6a8c4bc32a</stp>
+    <main first="rtdsrv.da30af61cf3e4a5a94195f27fdd074ca">
+      <tp>
+        <v>1</v>
+        <stp/>
+        <stp>4835f6a1-87a1-4740-a8cb-692464f720b9</stp>
+        <tr r="G24" s="1"/>
+      </tp>
+    </main>
+    <main first="rtdsrv.da30af61cf3e4a5a94195f27fdd074ca">
+      <tp>
+        <v>1</v>
+        <stp/>
+        <stp>6ce81161-9f0d-4c2f-be8c-d82e6a33a714</stp>
+        <tr r="F6" s="1"/>
+      </tp>
+    </main>
+    <main first="rtdsrv.da30af61cf3e4a5a94195f27fdd074ca">
+      <tp>
+        <v>1</v>
+        <stp/>
+        <stp>73ae7014-afde-41b8-b204-a3274c78da62</stp>
+        <tr r="G51" s="1"/>
+      </tp>
+    </main>
+    <main first="rtdsrv.da30af61cf3e4a5a94195f27fdd074ca">
+      <tp>
+        <v>1</v>
+        <stp/>
+        <stp>aee4a2c5-6ce5-4bf4-97df-3dbc85d1b6b2</stp>
+        <tr r="G32" s="1"/>
+      </tp>
+      <tp>
+        <v>1</v>
+        <stp/>
+        <stp>a7d8db76-c84c-4464-80fe-a54eac2b5d35</stp>
+        <tr r="G54" s="1"/>
+      </tp>
+    </main>
+    <main first="rtdsrv.da30af61cf3e4a5a94195f27fdd074ca">
+      <tp>
+        <v>1</v>
+        <stp/>
+        <stp>2c6e798c-8edd-432e-a52d-ae56d324d222</stp>
+        <tr r="G41" s="1"/>
+      </tp>
+    </main>
+    <main first="rtdsrv.da30af61cf3e4a5a94195f27fdd074ca">
+      <tp>
+        <v>1</v>
+        <stp/>
+        <stp>9ff95a53-ffbd-4161-b650-60bd0c030f8d</stp>
+        <tr r="G33" s="1"/>
+      </tp>
+      <tp>
+        <v>1</v>
+        <stp/>
+        <stp>b0e8efc0-1416-4f37-a3ca-10473dbcc75b</stp>
+        <tr r="G48" s="1"/>
+      </tp>
+      <tp>
+        <v>1</v>
+        <stp/>
+        <stp>dccd6470-d289-48aa-bc03-b321c62a37c1</stp>
+        <tr r="G29" s="1"/>
+      </tp>
+      <tp>
+        <v>1</v>
+        <stp/>
+        <stp>225fcc00-4787-49f2-a7a9-7370849adbf3</stp>
         <tr r="F1" s="1"/>
       </tp>
       <tp>
-        <v>3</v>
-        <stp/>
-        <stp>bad58e35-d7a5-43ca-9dbf-8da0c5a22604</stp>
+        <v>1</v>
+        <stp/>
+        <stp>f5a74a31-566f-4441-b55b-97dc9d4a5e8d</stp>
+        <tr r="G52" s="1"/>
+      </tp>
+    </main>
+    <main first="rtdsrv.da30af61cf3e4a5a94195f27fdd074ca">
+      <tp>
+        <v>1</v>
+        <stp/>
+        <stp>9016b188-060e-413c-9ea9-7ecc70f0d504</stp>
+        <tr r="G56" s="1"/>
+      </tp>
+      <tp>
+        <v>2</v>
+        <stp/>
+        <stp>0fa64373-1b60-4726-8d69-53d71fdacb5e</stp>
         <tr r="E6" s="3"/>
       </tp>
       <tp>
         <v>1</v>
         <stp/>
-        <stp>2bfd876b-4387-4916-a098-20c716433c2b</stp>
-        <tr r="G40" s="1"/>
-      </tp>
-      <tp>
-        <v>1</v>
-        <stp/>
-        <stp>776c6a0a-a1a1-4ff5-9c27-886434d93721</stp>
-        <tr r="G54" s="1"/>
+        <stp>d1e9d6b5-9d39-4b5b-999d-4a2a9ea26375</stp>
+        <tr r="G53" s="1"/>
       </tp>
     </main>
-    <main first="rtdsrv.46c5753678554062b36cfbc3a8309d90">
-      <tp>
-        <v>1</v>
-        <stp/>
-        <stp>274a0086-ec7e-4c4d-8a0a-012ec4afa828</stp>
-        <tr r="G42" s="1"/>
-      </tp>
-      <tp>
-        <v>1</v>
-        <stp/>
-        <stp>17adb89a-66cb-427b-a1a8-17450ef41b63</stp>
-        <tr r="G44" s="1"/>
-      </tp>
-    </main>
-    <main first="rtdsrv.46c5753678554062b36cfbc3a8309d90">
-      <tp>
-        <v>1</v>
-        <stp/>
-        <stp>30a42af1-3e0b-455e-9030-4b2a2d1fd8e9</stp>
-        <tr r="G33" s="1"/>
-      </tp>
-      <tp>
-        <v>1</v>
-        <stp/>
-        <stp>3fcd1e2f-0e95-4a4c-a61d-c73bb9e88e22</stp>
-        <tr r="G41" s="1"/>
-      </tp>
-      <tp>
-        <v>1</v>
-        <stp/>
-        <stp>43ee96d1-0bb0-45a2-a649-a55859b6d557</stp>
-        <tr r="G48" s="1"/>
-      </tp>
-      <tp>
-        <v>1</v>
-        <stp/>
-        <stp>65e152c0-8346-4cc1-a0a2-82addda84395</stp>
-        <tr r="G47" s="1"/>
-      </tp>
-      <tp>
-        <v>1</v>
-        <stp/>
-        <stp>a6e0b538-5461-45b0-9671-978c540d385a</stp>
-        <tr r="G29" s="1"/>
-      </tp>
-    </main>
-    <main first="rtdsrv.46c5753678554062b36cfbc3a8309d90">
-      <tp>
-        <v>1</v>
-        <stp/>
-        <stp>bd82148e-9f60-4095-918d-0df7d9e0c07a</stp>
-        <tr r="G38" s="1"/>
-      </tp>
-    </main>
-    <main first="rtdsrv.46c5753678554062b36cfbc3a8309d90">
-      <tp>
-        <v>1</v>
-        <stp/>
-        <stp>6bb44877-5462-4807-be1d-a3bf1d8fc6da</stp>
-        <tr r="G53" s="1"/>
-      </tp>
-    </main>
-    <main first="rtdsrv.46c5753678554062b36cfbc3a8309d90">
-      <tp>
-        <v>1</v>
-        <stp/>
-        <stp>934a9244-37ca-4ea0-8fda-8d8828dec2a6</stp>
-        <tr r="F6" s="1"/>
-      </tp>
-    </main>
-    <main first="rtdsrv.46c5753678554062b36cfbc3a8309d90">
-      <tp>
-        <v>1</v>
-        <stp/>
-        <stp>b335ad67-ee29-4296-a3f9-793f1ebf016b</stp>
-        <tr r="G25" s="1"/>
-      </tp>
-    </main>
-    <main first="rtdsrv.46c5753678554062b36cfbc3a8309d90">
-      <tp>
-        <v>1</v>
-        <stp/>
-        <stp>cd7f3252-0b10-4b0b-b29d-aa146b57c3b7</stp>
-        <tr r="G23" s="1"/>
-      </tp>
-      <tp>
-        <v>1</v>
-        <stp/>
-        <stp>5fde92ed-2ab9-4c45-ac71-9ded4c5c702a</stp>
-        <tr r="G20" s="1"/>
-      </tp>
-    </main>
-    <main first="rtdsrv.46c5753678554062b36cfbc3a8309d90">
-      <tp>
-        <v>1</v>
-        <stp/>
-        <stp>585b1bd3-9fa9-4ffb-8cdf-1d97ef08076c</stp>
-        <tr r="G24" s="1"/>
-      </tp>
-    </main>
-    <main first="rtdsrv.46c5753678554062b36cfbc3a8309d90">
-      <tp>
-        <v>1</v>
-        <stp/>
-        <stp>2f625adf-eb80-48fc-bd1f-e43b62acbaf2</stp>
-        <tr r="G34" s="1"/>
-      </tp>
-      <tp>
-        <v>1</v>
-        <stp/>
-        <stp>a41d147a-d3fa-4e83-afee-6433fb9bd32b</stp>
-        <tr r="G51" s="1"/>
-      </tp>
-    </main>
-    <main first="rtdsrv.46c5753678554062b36cfbc3a8309d90">
-      <tp>
-        <v>1</v>
-        <stp/>
-        <stp>39b81c11-98ad-429a-abcd-1ff4d00c8a8a</stp>
-        <tr r="G36" s="1"/>
-      </tp>
-    </main>
-    <main first="rtdsrv.46c5753678554062b36cfbc3a8309d90">
-      <tp>
-        <v>1</v>
-        <stp/>
-        <stp>fe7f2634-502a-4360-a0e2-6a16877693ff</stp>
-        <tr r="G26" s="1"/>
-      </tp>
-      <tp>
-        <v>1</v>
-        <stp/>
-        <stp>c2df1639-7beb-4edf-be6e-7869e6f00857</stp>
-        <tr r="I19" s="1"/>
-      </tp>
-      <tp>
-        <v>1</v>
-        <stp/>
-        <stp>aec6adf7-7e5f-43c0-b1d1-b5f83cc3ca44</stp>
-        <tr r="G45" s="1"/>
-      </tp>
-      <tp>
-        <v>1</v>
-        <stp/>
-        <stp>264978d6-3a7d-4a29-961a-da7a983c490c</stp>
+    <main first="rtdsrv.da30af61cf3e4a5a94195f27fdd074ca">
+      <tp>
+        <v>1</v>
+        <stp/>
+        <stp>7edd312f-2579-4474-9061-b6595b0a7bab</stp>
         <tr r="G37" s="1"/>
-      </tp>
-      <tp>
-        <v>1</v>
-        <stp/>
-        <stp>bd814d20-b495-410f-b934-07075cddd662</stp>
-        <tr r="G22" s="1"/>
-      </tp>
-      <tp>
-        <v>1</v>
-        <stp/>
-        <stp>2387c2fd-a8db-444e-ba72-4990487e3f19</stp>
-        <tr r="G32" s="1"/>
-      </tp>
-    </main>
-    <main first="rtdsrv.46c5753678554062b36cfbc3a8309d90">
-      <tp>
-        <v>1</v>
-        <stp/>
-        <stp>da1ab319-cafc-4a58-a41d-a0b13c40d069</stp>
-        <tr r="G57" s="1"/>
-      </tp>
-      <tp>
-        <v>1</v>
-        <stp/>
-        <stp>5f265889-653c-4b82-95bc-844eac7c9448</stp>
-        <tr r="G55" s="1"/>
-      </tp>
-      <tp>
-        <v>1</v>
-        <stp/>
-        <stp>87ab3c8c-9cc4-429c-b257-542461f5ee57</stp>
-        <tr r="E4" s="3"/>
-      </tp>
-      <tp>
-        <v>1</v>
-        <stp/>
-        <stp>ba7be99f-3a1f-4f83-bc7d-c42285221499</stp>
-        <tr r="G50" s="1"/>
-      </tp>
-      <tp>
-        <v>1</v>
-        <stp/>
-        <stp>3e9f3533-dfc8-4431-9182-dc686012d771</stp>
-        <tr r="G27" s="1"/>
-      </tp>
-    </main>
-    <main first="rtdsrv.46c5753678554062b36cfbc3a8309d90">
-      <tp>
-        <v>1</v>
-        <stp/>
-        <stp>d06d2b2e-f153-4bdf-b4f6-f4985a3a79f8</stp>
-        <tr r="G56" s="1"/>
-      </tp>
-    </main>
-    <main first="rtdsrv.46c5753678554062b36cfbc3a8309d90">
-      <tp>
-        <v>1</v>
-        <stp/>
-        <stp>1b81d318-90ab-4054-82b1-9af22a6cba22</stp>
-        <tr r="G21" s="1"/>
-      </tp>
-    </main>
-    <main first="rtdsrv.46c5753678554062b36cfbc3a8309d90">
-      <tp>
-        <v>1</v>
-        <stp/>
-        <stp>5a22fc47-b587-454e-80b7-897db18e011b</stp>
-        <tr r="G52" s="1"/>
-      </tp>
-    </main>
-    <main first="rtdsrv.46c5753678554062b36cfbc3a8309d90">
-      <tp>
-        <v>1</v>
-        <stp/>
-        <stp>ae4eb2dc-c3b2-4024-a534-f99fec10d4ad</stp>
-        <tr r="G28" s="1"/>
-      </tp>
-      <tp>
-        <v>1</v>
-        <stp/>
-        <stp>61ddc3bc-5f4e-4429-a4ab-d9c028d1523e</stp>
-        <tr r="G46" s="1"/>
-      </tp>
-      <tp>
-        <v>1</v>
-        <stp/>
-        <stp>69584146-cb8d-4689-a1ca-35b3a98a0a3e</stp>
-        <tr r="G31" s="1"/>
-      </tp>
-      <tp>
-        <v>1</v>
-        <stp/>
-        <stp>4c217539-8bbe-436d-bb7d-f019fd9fe5cb</stp>
-        <tr r="C2" s="2"/>
       </tp>
     </main>
   </volType>
@@ -1187,11 +1195,11 @@
       </c>
       <c r="F1" t="str" cm="1">
         <f t="array" ref="F1">_xll.ExLibris.Json.CreateJsonObject(E3:F6, EXLIBRIS_CONFIGURATION)</f>
-        <v>JsonObject:6B86012C-4633-4710-86A4-5526174543C9</v>
+        <v>JsonObject:4CBE4E84-D038-4955-8393-CE04A80A3583</v>
       </c>
       <c r="K1" t="str">
         <f>EXLIBRIS_CONFIGURATION</f>
-        <v>ExLibris.Core.ExLibrisConfiguration:41DE7111-6A92-4854-9FC9-1FC8091CB7CD</v>
+        <v>ExLibris.Core.ExLibrisConfiguration:E8DCA9AB-6EBC-4C98-8C3A-029399E3EB11</v>
       </c>
     </row>
     <row r="2" spans="2:25" x14ac:dyDescent="0.4">
@@ -1261,7 +1269,7 @@
       </c>
       <c r="F6" t="str" cm="1">
         <f t="array" ref="F6">_xll.ExLibris.Json.CreateJsonArray(E8:J14, EXLIBRIS_CONFIGURATION)</f>
-        <v>JsonObject:C9086EB2-CC40-4366-93FB-B5BC53FFB3B3</v>
+        <v>JsonObject:B058ED14-E401-4142-AB75-B5F6A0D6467C</v>
       </c>
       <c r="L6" t="s">
         <v>68</v>
@@ -1486,7 +1494,7 @@
       </c>
       <c r="I19" t="str" cm="1">
         <f t="array" ref="I19">_xll.ExLibris.Json.GetJsonValue(F1,E6, EXLIBRIS_CONFIGURATION)</f>
-        <v>JsonObject:970AC73C-D764-4FC1-815E-3CFE212730D5</v>
+        <v>JsonObject:F3637329-E835-40D6-98B6-1A8D47A1CCA3</v>
       </c>
       <c r="P19" t="s">
         <v>14</v>
@@ -2208,7 +2216,7 @@
       </c>
       <c r="I28" t="str" cm="1">
         <f t="array" ref="I28">_xll.ExLibris.Json.GetJsonValue(I19,"[2]", EXLIBRIS_CONFIGURATION)</f>
-        <v>JsonObject:D9CC4637-154F-4012-8AAA-EA0737B72E93</v>
+        <v>JsonObject:FEEEC164-0563-4FDB-931A-8D59613C5F83</v>
       </c>
       <c r="P28" t="s">
         <v>38</v>
@@ -3335,11 +3343,11 @@
     </row>
     <row r="4" spans="2:5" x14ac:dyDescent="0.4">
       <c r="D4" t="s">
-        <v>104</v>
+        <v>111</v>
       </c>
       <c r="E4" t="str" cm="1">
-        <f t="array" ref="E4">_xll.ExLibris.WebSockets.OpenWebSocket("ws://localhost:10101" )</f>
-        <v>ExLibris.Core.WebSockets.WebsocketClient:9CA7641C-311D-47BD-911C-A7A7C7A8CE94</v>
+        <f t="array" ref="E4">_xll.ExLibris.WebSockets.OpenWebSocket("ws://localhost:10101",D4)</f>
+        <v>ExLibris.Core.WebSockets.WebsocketClient:4DF9B095-61CC-4272-AF17-953246EC0EF5</v>
       </c>
     </row>
     <row r="6" spans="2:5" x14ac:dyDescent="0.4">
@@ -3348,7 +3356,7 @@
       </c>
       <c r="E6" t="str" cm="1">
         <f t="array" ref="E6">_xll.ExLibris.WebSockets.ObserveWebSocketStatus(E4,1000)</f>
-        <v>Closed</v>
+        <v>Open</v>
       </c>
     </row>
     <row r="7" spans="2:5" x14ac:dyDescent="0.4">
@@ -3357,70 +3365,70 @@
       </c>
       <c r="E7" t="str" cm="1">
         <f t="array" ref="E7">_xll.ExLibris.WebSockets.ObserveWebSocketMessage(E4)</f>
-        <v>push_event 23:11:04</v>
+        <v>push_event 23:42:24</v>
       </c>
     </row>
     <row r="9" spans="2:5" x14ac:dyDescent="0.4">
       <c r="D9" t="s">
-        <v>105</v>
-      </c>
-      <c r="E9" t="e" cm="1">
+        <v>104</v>
+      </c>
+      <c r="E9" t="str" cm="1">
         <f t="array" ref="E9">_xll.ExLibris.WebSockets.SendWebSocketMessage(E4,"test "&amp;D9,E6="Open")</f>
-        <v>#N/A</v>
+        <v>message sent : 2021-09-15T11:42:08.610</v>
       </c>
     </row>
     <row r="10" spans="2:5" x14ac:dyDescent="0.4">
       <c r="D10" t="s">
-        <v>106</v>
-      </c>
-      <c r="E10" t="e" cm="1">
+        <v>105</v>
+      </c>
+      <c r="E10" t="str" cm="1">
         <f t="array" ref="E10">_xll.ExLibris.WebSockets.SendWebSocketMessage($E$4,"test next "&amp;D10,E9)</f>
-        <v>#N/A</v>
+        <v>message sent : 2021-09-15T11:42:08.610</v>
       </c>
     </row>
     <row r="11" spans="2:5" x14ac:dyDescent="0.4">
       <c r="D11" t="s">
-        <v>107</v>
-      </c>
-      <c r="E11" t="e" cm="1">
+        <v>106</v>
+      </c>
+      <c r="E11" t="str" cm="1">
         <f t="array" ref="E11">_xll.ExLibris.WebSockets.SendWebSocketMessage($E$4,"test next "&amp;D11,E10)</f>
-        <v>#N/A</v>
+        <v>message sent : 2021-09-15T11:42:08.610</v>
       </c>
     </row>
     <row r="12" spans="2:5" x14ac:dyDescent="0.4">
       <c r="D12" t="s">
-        <v>108</v>
-      </c>
-      <c r="E12" t="e" cm="1">
+        <v>107</v>
+      </c>
+      <c r="E12" t="str" cm="1">
         <f t="array" ref="E12">_xll.ExLibris.WebSockets.SendWebSocketMessage($E$4,"test next "&amp;D12,E11)</f>
-        <v>#N/A</v>
+        <v>message sent : 2021-09-15T11:42:08.610</v>
       </c>
     </row>
     <row r="13" spans="2:5" x14ac:dyDescent="0.4">
       <c r="D13" t="s">
-        <v>109</v>
-      </c>
-      <c r="E13" t="e" cm="1">
+        <v>108</v>
+      </c>
+      <c r="E13" t="str" cm="1">
         <f t="array" ref="E13">_xll.ExLibris.WebSockets.SendWebSocketMessage($E$4,"test next "&amp;D13,E12)</f>
-        <v>#N/A</v>
+        <v>message sent : 2021-09-15T11:42:08.611</v>
       </c>
     </row>
     <row r="14" spans="2:5" x14ac:dyDescent="0.4">
       <c r="D14" t="s">
-        <v>110</v>
-      </c>
-      <c r="E14" t="e" cm="1">
+        <v>109</v>
+      </c>
+      <c r="E14" t="str" cm="1">
         <f t="array" ref="E14">_xll.ExLibris.WebSockets.SendWebSocketMessage($E$4,"test next "&amp;D14,E13)</f>
-        <v>#N/A</v>
+        <v>message sent : 2021-09-15T11:42:08.611</v>
       </c>
     </row>
     <row r="15" spans="2:5" x14ac:dyDescent="0.4">
       <c r="D15" t="s">
-        <v>111</v>
-      </c>
-      <c r="E15" t="e" cm="1">
+        <v>110</v>
+      </c>
+      <c r="E15" t="str" cm="1">
         <f t="array" ref="E15">_xll.ExLibris.WebSockets.SendWebSocketMessage($E$4,"test next "&amp;D15,E14)</f>
-        <v>#N/A</v>
+        <v>message sent : 2021-09-15T11:42:08.611</v>
       </c>
     </row>
   </sheetData>
@@ -3447,7 +3455,7 @@
       </c>
       <c r="C2" t="str" cm="1">
         <f t="array" ref="C2">_xll.ExLibris.LoadConfiguration(B6:C15)</f>
-        <v>ExLibris.Core.ExLibrisConfiguration:41DE7111-6A92-4854-9FC9-1FC8091CB7CD</v>
+        <v>ExLibris.Core.ExLibrisConfiguration:E8DCA9AB-6EBC-4C98-8C3A-029399E3EB11</v>
       </c>
     </row>
     <row r="4" spans="2:6" s="4" customFormat="1" ht="18" x14ac:dyDescent="0.4">

</xml_diff>

<commit_message>
refactoring : small refactoring
</commit_message>
<xml_diff>
--- a/ExLibris/test_excel/exlibris_test.xlsx
+++ b/ExLibris/test_excel/exlibris_test.xlsx
@@ -8,14 +8,15 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\mugen\git\ex-libris\ExLibris\test_excel\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3AA317F5-F581-4347-9A4A-71A15988A1B5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1EC2873F-5E94-4754-9542-2E2FFC115C15}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" activeTab="1" xr2:uid="{705CD0B7-27A9-4291-85BD-6034C0FEE3E4}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{705CD0B7-27A9-4291-85BD-6034C0FEE3E4}"/>
   </bookViews>
   <sheets>
     <sheet name="json_test" sheetId="1" r:id="rId1"/>
-    <sheet name="websocket" sheetId="3" r:id="rId2"/>
-    <sheet name="configuration" sheetId="2" r:id="rId3"/>
+    <sheet name="json_w_conf_test" sheetId="4" r:id="rId2"/>
+    <sheet name="websocket" sheetId="3" r:id="rId3"/>
+    <sheet name="configuration" sheetId="2" r:id="rId4"/>
   </sheets>
   <definedNames>
     <definedName name="EXLIBRIS_CONFIGURATION">configuration!$C$2</definedName>
@@ -39,7 +40,7 @@
 </file>
 
 <file path=xl/metadata.xml><?xml version="1.0" encoding="utf-8"?>
-<metadata xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xda="http://schemas.microsoft.com/office/spreadsheetml/2017/dynamicarray">
+<metadata xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xlrd="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata" xmlns:xda="http://schemas.microsoft.com/office/spreadsheetml/2017/dynamicarray">
   <metadataTypes count="1">
     <metadataType name="XLDAPR" minSupportedVersion="120000" copy="1" pasteAll="1" pasteValues="1" merge="1" splitFirst="1" rowColShift="1" clearFormats="1" clearComments="1" assign="1" coerce="1" cellMeta="1"/>
   </metadataTypes>
@@ -61,7 +62,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="205" uniqueCount="112">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="319" uniqueCount="113">
   <si>
     <t>payment _date</t>
   </si>
@@ -432,6 +433,9 @@
   <si>
     <t>client0</t>
     <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>{"trade_code":"money_00001","couter_party":"CP00001","fixed_leg":{"pay_or_recieve":"Receive","cashflows":[{"payment _date":44632,"start_date":44452,"end_date":44632,"day_count_type":"ACT/360","amout":10000000,"fixed_rate":0.001},{"payment _date":44812,"start_date":44632,"end_date":44812,"day_count_type":"ACT/360","amout":11000000,"fixed_rate":0.001},{"payment _date":44992,"start_date":44812,"end_date":44992,"day_count_type":"ACT/360","amout":12000000,"fixed_rate":0.001},{"payment _date":45172,"start_date":44992,"end_date":45172,"day_count_type":"ACT/360","amout":13000000,"fixed_rate":0.001},{"payment _date":45352,"start_date":45172,"end_date":45352,"day_count_type":"ACT/360","amout":14000000,"fixed_rate":0.001},{"payment _date":45532,"start_date":45352,"end_date":45532,"day_count_type":"ACT/360","amout":15000000,"fixed_rate":0.001}]}}</t>
   </si>
 </sst>
 </file>
@@ -537,336 +541,608 @@
 <file path=xl/volatileDependencies.xml><?xml version="1.0" encoding="utf-8"?>
 <volTypes xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <volType type="realTimeData">
-    <main first="rtdsrv.da30af61cf3e4a5a94195f27fdd074ca">
-      <tp>
-        <v>1</v>
-        <stp/>
-        <stp>8215b3c4-c6dd-45ca-955f-7abcf8c59b10</stp>
+    <main first="rtdsrv.4b8ef99e016b447da4df1f9adeb95e96">
+      <tp>
+        <v>1</v>
+        <stp/>
+        <stp>686bc1c5-323e-4744-b701-e3b327147ccf</stp>
+        <tr r="G25" s="1"/>
+      </tp>
+      <tp>
+        <v>1</v>
+        <stp/>
+        <stp>5762ea02-f98e-44f5-8af4-a01b12463914</stp>
+        <tr r="G27" s="1"/>
+      </tp>
+      <tp>
+        <v>1</v>
+        <stp/>
+        <stp>9e6fa9bf-d626-4b10-82fe-5ae1ccc2a423</stp>
+        <tr r="F6" s="4"/>
+      </tp>
+      <tp>
+        <v>1</v>
+        <stp/>
+        <stp>c66e509e-94f6-48c2-bb0c-af5f357b7664</stp>
+        <tr r="G36" s="4"/>
+      </tp>
+    </main>
+    <main first="rtdsrv.4b8ef99e016b447da4df1f9adeb95e96">
+      <tp>
+        <v>1</v>
+        <stp/>
+        <stp>4efd792c-b43e-4209-8e80-ae43236ba2e3</stp>
+        <tr r="G25" s="4"/>
+      </tp>
+      <tp>
+        <v>1</v>
+        <stp/>
+        <stp>f37079ca-e529-4b73-87fe-b232caac12c5</stp>
+        <tr r="G52" s="1"/>
+      </tp>
+    </main>
+    <main first="rtdsrv.4b8ef99e016b447da4df1f9adeb95e96">
+      <tp>
+        <v>1</v>
+        <stp/>
+        <stp>67012ff4-1270-4eaa-848e-a22e52fa8b2f</stp>
+        <tr r="G57" s="1"/>
+      </tp>
+      <tp>
+        <v>1</v>
+        <stp/>
+        <stp>52b667d1-6ce4-459f-a6a2-45793c0028d3</stp>
+        <tr r="G27" s="4"/>
+      </tp>
+      <tp>
+        <v>1</v>
+        <stp/>
+        <stp>89f8e619-fafb-409f-90e0-e43c009a0489</stp>
+        <tr r="G21" s="1"/>
+      </tp>
+      <tp>
+        <v>1</v>
+        <stp/>
+        <stp>caf4d30a-a402-4fc3-ab09-07cb89345da7</stp>
+        <tr r="G31" s="1"/>
+      </tp>
+      <tp>
+        <v>1</v>
+        <stp/>
+        <stp>e2b50a7f-c0b4-4e28-9c5c-063f6a32e76f</stp>
+        <tr r="G56" s="1"/>
+      </tp>
+      <tp>
+        <v>1</v>
+        <stp/>
+        <stp>cbcf9cab-f3ec-4461-93f7-4573f961aae4</stp>
+        <tr r="G53" s="1"/>
+      </tp>
+      <tp>
+        <v>1</v>
+        <stp/>
+        <stp>cee9e8aa-3e79-4832-985b-74cc2e842de4</stp>
+        <tr r="G42" s="1"/>
+      </tp>
+      <tp>
+        <v>1</v>
+        <stp/>
+        <stp>2af9c600-62cb-44c1-9d7b-384dc2c5a1af</stp>
+        <tr r="C2" s="2"/>
+      </tp>
+      <tp>
+        <v>1</v>
+        <stp/>
+        <stp>5dc5449c-285b-4969-ac73-7ffb4492dbf4</stp>
+        <tr r="G40" s="4"/>
+      </tp>
+      <tp>
+        <v>1</v>
+        <stp/>
+        <stp>5f6eacb5-697b-434b-86f6-2975cb268086</stp>
+        <tr r="G31" s="4"/>
+      </tp>
+      <tp>
+        <v>1</v>
+        <stp/>
+        <stp>d934f17e-44de-4792-82e5-5be9e73f9b4b</stp>
+        <tr r="G33" s="4"/>
+      </tp>
+    </main>
+    <main first="rtdsrv.4b8ef99e016b447da4df1f9adeb95e96">
+      <tp>
+        <v>1</v>
+        <stp/>
+        <stp>a2f0394e-7e61-43f9-89d0-d9d2373de0e2</stp>
+        <tr r="G26" s="4"/>
+      </tp>
+    </main>
+    <main first="rtdsrv.4b8ef99e016b447da4df1f9adeb95e96">
+      <tp>
+        <v>2</v>
+        <stp/>
+        <stp>f683902d-4f5d-4695-85c9-70a6227ad9a1</stp>
+        <tr r="E6" s="3"/>
+      </tp>
+      <tp>
+        <v>1</v>
+        <stp/>
+        <stp>5fa7ab49-a894-483f-8180-4a54afb86ba1</stp>
+        <tr r="G38" s="1"/>
+      </tp>
+      <tp>
+        <v>1</v>
+        <stp/>
+        <stp>35d80511-c89c-44f5-a8c7-c5d9f8158ffa</stp>
+        <tr r="G20" s="1"/>
+      </tp>
+      <tp>
+        <v>1</v>
+        <stp/>
+        <stp>3ab4ebe7-a21c-4702-a280-5211f04df4ba</stp>
+        <tr r="G20" s="4"/>
+      </tp>
+    </main>
+    <main first="rtdsrv.4b8ef99e016b447da4df1f9adeb95e96">
+      <tp>
+        <v>1</v>
+        <stp/>
+        <stp>07592be1-25ec-418a-ad74-727bdc56510f</stp>
+        <tr r="G49" s="1"/>
+      </tp>
+    </main>
+    <main first="rtdsrv.4b8ef99e016b447da4df1f9adeb95e96">
+      <tp>
+        <v>1</v>
+        <stp/>
+        <stp>60c987a5-d7f3-4535-afaa-606e762cead9</stp>
+        <tr r="G32" s="1"/>
+      </tp>
+    </main>
+    <main first="rtdsrv.4b8ef99e016b447da4df1f9adeb95e96">
+      <tp>
+        <v>1</v>
+        <stp/>
+        <stp>7f546308-9bd8-4b30-933e-3dbe38580c81</stp>
+        <tr r="G19" s="1"/>
+      </tp>
+    </main>
+    <main first="rtdsrv.4b8ef99e016b447da4df1f9adeb95e96">
+      <tp>
+        <v>1</v>
+        <stp/>
+        <stp>a7d76aee-c7f5-4013-9c34-80a4dc321638</stp>
+        <tr r="G35" s="4"/>
+      </tp>
+      <tp>
+        <v>1</v>
+        <stp/>
+        <stp>de0d9157-bea8-4204-b7dd-1e3c62770aa4</stp>
+        <tr r="G24" s="1"/>
+      </tp>
+    </main>
+    <main first="rtdsrv.4b8ef99e016b447da4df1f9adeb95e96">
+      <tp>
+        <v>1</v>
+        <stp/>
+        <stp>e3b96405-cf09-4807-ac9a-f910d3788301</stp>
+        <tr r="G45" s="4"/>
+      </tp>
+      <tp>
+        <v>1</v>
+        <stp/>
+        <stp>24e2d18f-48ce-4cf4-8914-9ef68226412e</stp>
+        <tr r="G24" s="4"/>
+      </tp>
+    </main>
+    <main first="rtdsrv.4b8ef99e016b447da4df1f9adeb95e96">
+      <tp>
+        <v>1</v>
+        <stp/>
+        <stp>a99f1cad-dbb1-4d0b-87d2-37a1ceb188fb</stp>
+        <tr r="G47" s="4"/>
+      </tp>
+      <tp>
+        <v>1</v>
+        <stp/>
+        <stp>dfe1bc29-d3b7-44be-a4ed-15290cd27b46</stp>
+        <tr r="G41" s="4"/>
+      </tp>
+    </main>
+    <main first="rtdsrv.4b8ef99e016b447da4df1f9adeb95e96">
+      <tp>
+        <v>1</v>
+        <stp/>
+        <stp>e2fb3df6-7928-4ed2-8d99-4288b8aa348e</stp>
+        <tr r="G51" s="4"/>
+      </tp>
+      <tp>
+        <v>1</v>
+        <stp/>
+        <stp>b06dd595-b7b5-404f-80bc-57d58bb87b99</stp>
+        <tr r="G30" s="4"/>
+      </tp>
+    </main>
+    <main first="rtdsrv.4b8ef99e016b447da4df1f9adeb95e96">
+      <tp>
+        <v>1</v>
+        <stp/>
+        <stp>75eb7dcb-1240-4813-b3cd-ef943785f6ce</stp>
+        <tr r="G47" s="1"/>
+      </tp>
+      <tp>
+        <v>1</v>
+        <stp/>
+        <stp>1fc5db0e-0951-487a-b35f-6615274cf683</stp>
+        <tr r="G28" s="4"/>
+      </tp>
+      <tp>
+        <v>1</v>
+        <stp/>
+        <stp>3f7b3da9-67a8-4255-b1be-ae7e3397cbab</stp>
+        <tr r="G37" s="4"/>
+      </tp>
+      <tp>
+        <v>1</v>
+        <stp/>
+        <stp>5f50dafc-460c-4064-833d-a02370dd9c49</stp>
+        <tr r="G21" s="4"/>
+      </tp>
+      <tp>
+        <v>1</v>
+        <stp/>
+        <stp>bcbafea3-e434-44bc-be00-e66713672c7e</stp>
+        <tr r="G50" s="1"/>
+      </tp>
+      <tp>
+        <v>1</v>
+        <stp/>
+        <stp>a1062289-db09-428b-8629-af3da22f05da</stp>
+        <tr r="G54" s="1"/>
+      </tp>
+    </main>
+    <main first="rtdsrv.4b8ef99e016b447da4df1f9adeb95e96">
+      <tp>
+        <v>1</v>
+        <stp/>
+        <stp>707587d9-6fc6-4bc9-9b16-c8ffd6afbafd</stp>
+        <tr r="G43" s="4"/>
+      </tp>
+      <tp>
+        <v>1</v>
+        <stp/>
+        <stp>e18d8c9e-c7ef-4783-8616-b9c95aaafb8b</stp>
+        <tr r="G42" s="4"/>
+      </tp>
+      <tp>
+        <v>1</v>
+        <stp/>
+        <stp>d6663a89-5a23-4a77-ab92-71ebb7412c5d</stp>
+        <tr r="G49" s="4"/>
+      </tp>
+      <tp>
+        <v>1</v>
+        <stp/>
+        <stp>286aafc8-7969-4e4a-8158-37f692fa413a</stp>
+        <tr r="F6" s="1"/>
+      </tp>
+    </main>
+    <main first="rtdsrv.4b8ef99e016b447da4df1f9adeb95e96">
+      <tp>
+        <v>1</v>
+        <stp/>
+        <stp>b422dca2-8e2c-4b43-9da5-ba427a1f059b</stp>
+        <tr r="I19" s="1"/>
+      </tp>
+      <tp>
+        <v>1</v>
+        <stp/>
+        <stp>973f232f-a5fe-4d22-87e0-492d5091f33a</stp>
+        <tr r="G52" s="4"/>
+      </tp>
+      <tp>
+        <v>1</v>
+        <stp/>
+        <stp>dfc230f6-10a5-4eda-aa34-c9b742da8661</stp>
+        <tr r="G22" s="1"/>
+      </tp>
+      <tp>
+        <v>1</v>
+        <stp/>
+        <stp>0168d52e-0b73-4b49-998d-c7f218970209</stp>
+        <tr r="G48" s="1"/>
+      </tp>
+    </main>
+    <main first="rtdsrv.4b8ef99e016b447da4df1f9adeb95e96">
+      <tp>
+        <v>1</v>
+        <stp/>
+        <stp>b4d8df59-58b8-4ca4-831e-c49829f09db5</stp>
+        <tr r="G46" s="1"/>
+      </tp>
+      <tp>
+        <v>1</v>
+        <stp/>
+        <stp>e86b73fe-6b46-4c47-8271-abf34dc84018</stp>
+        <tr r="G30" s="1"/>
+      </tp>
+      <tp>
+        <v>1</v>
+        <stp/>
+        <stp>417fc574-e091-4fdb-a48d-f67ad5e8c32e</stp>
+        <tr r="G45" s="1"/>
+      </tp>
+      <tp>
+        <v>1</v>
+        <stp/>
+        <stp>865af7e0-1550-485c-b1a5-218d1075a9da</stp>
+        <tr r="G37" s="1"/>
+      </tp>
+      <tp>
+        <v>1</v>
+        <stp/>
+        <stp>76b07320-f83c-4689-894b-6c28860fe15b</stp>
+        <tr r="G36" s="1"/>
+      </tp>
+    </main>
+    <main first="rtdsrv.4b8ef99e016b447da4df1f9adeb95e96">
+      <tp>
+        <v>1</v>
+        <stp/>
+        <stp>6b449903-bc31-4f60-95aa-7dc19c10ee4e</stp>
+        <tr r="G57" s="4"/>
+      </tp>
+    </main>
+    <main first="rtdsrv.4b8ef99e016b447da4df1f9adeb95e96">
+      <tp>
+        <v>1</v>
+        <stp/>
+        <stp>ea1c0135-b590-4337-8ab2-961da8091d6b</stp>
+        <tr r="G39" s="1"/>
+      </tp>
+    </main>
+    <main first="rtdsrv.4b8ef99e016b447da4df1f9adeb95e96">
+      <tp>
+        <v>1</v>
+        <stp/>
+        <stp>939e3515-f4df-4f0b-b75c-65eb29c357c5</stp>
+        <tr r="I28" s="4"/>
+      </tp>
+    </main>
+    <main first="rtdsrv.4b8ef99e016b447da4df1f9adeb95e96">
+      <tp>
+        <v>1</v>
+        <stp/>
+        <stp>fc7bacc0-7b10-4c5a-ac91-a0d0be715610</stp>
+        <tr r="G46" s="4"/>
+      </tp>
+    </main>
+    <main first="rtdsrv.4b8ef99e016b447da4df1f9adeb95e96">
+      <tp>
+        <v>1</v>
+        <stp/>
+        <stp>36e58f36-0b31-4d70-8478-59c7f352eb23</stp>
+        <tr r="G19" s="4"/>
+      </tp>
+    </main>
+    <main first="rtdsrv.4b8ef99e016b447da4df1f9adeb95e96">
+      <tp>
+        <v>1</v>
+        <stp/>
+        <stp>a27287b1-9ad8-4cdd-a84f-9163a71d1d9f</stp>
+        <tr r="G56" s="4"/>
+      </tp>
+      <tp>
+        <v>1</v>
+        <stp/>
+        <stp>4f4f6569-5531-4084-8239-b724ae377229</stp>
+        <tr r="G35" s="1"/>
+      </tp>
+      <tp>
+        <v>1</v>
+        <stp/>
+        <stp>d686cd8e-4bda-4864-a9a4-8fec273e7c27</stp>
+        <tr r="G29" s="4"/>
+      </tp>
+      <tp>
+        <v>1</v>
+        <stp/>
+        <stp>bb76ab39-1507-4cd5-8ffc-5a599d4b8f8e</stp>
+        <tr r="G50" s="4"/>
+      </tp>
+      <tp>
+        <v>1</v>
+        <stp/>
+        <stp>737fdd70-fa54-4068-bb99-a5a3dbd02f5a</stp>
+        <tr r="G44" s="1"/>
+      </tp>
+      <tp>
+        <v>1</v>
+        <stp/>
+        <stp>9319eabb-8ddd-43c6-9111-e02b98c07d5e</stp>
+        <tr r="G44" s="4"/>
+      </tp>
+      <tp>
+        <v>1</v>
+        <stp/>
+        <stp>bebc2de1-60ea-40bb-8a46-521efe0f458e</stp>
+        <tr r="G41" s="1"/>
+      </tp>
+      <tp>
+        <v>1</v>
+        <stp/>
+        <stp>29f95f6a-8c35-4d6b-9c18-f67c942ba582</stp>
+        <tr r="G22" s="4"/>
+      </tp>
+      <tp>
+        <v>1</v>
+        <stp/>
+        <stp>21f26eb4-332f-4579-a19f-7b05db019d10</stp>
+        <tr r="E4" s="3"/>
+      </tp>
+      <tp>
+        <v>1</v>
+        <stp/>
+        <stp>45f70452-a4c1-48af-8087-beebc9e9fa7e</stp>
+        <tr r="G38" s="4"/>
+      </tp>
+      <tp>
+        <v>1</v>
+        <stp/>
+        <stp>cb75bec1-4e61-4348-b7c1-7d0d579e9979</stp>
+        <tr r="G26" s="1"/>
+      </tp>
+    </main>
+    <main first="rtdsrv.4b8ef99e016b447da4df1f9adeb95e96">
+      <tp>
+        <v>1</v>
+        <stp/>
+        <stp>d40bbdc3-504c-43f0-a54d-e58652259d10</stp>
+        <tr r="G34" s="1"/>
+      </tp>
+      <tp>
+        <v>1</v>
+        <stp/>
+        <stp>000049d3-ca0c-4109-a973-0713aa7ad004</stp>
+        <tr r="G23" s="1"/>
+      </tp>
+      <tp>
+        <v>101</v>
+        <stp/>
+        <stp>a0770d64-0cc0-4d63-a9c0-72192be5bf75</stp>
+        <tr r="E7" s="3"/>
+      </tp>
+      <tp>
+        <v>1</v>
+        <stp/>
+        <stp>9f0b6f53-f245-405d-83f1-d57507822dbc</stp>
+        <tr r="I19" s="4"/>
+      </tp>
+      <tp>
+        <v>1</v>
+        <stp/>
+        <stp>6e91c3b5-e1e9-4efe-93bb-46c26a0a6a2c</stp>
+        <tr r="G51" s="1"/>
+      </tp>
+      <tp>
+        <v>1</v>
+        <stp/>
+        <stp>f91acaf9-ab77-44af-9389-6eef20a9a0ac</stp>
+        <tr r="G53" s="4"/>
+      </tp>
+    </main>
+    <main first="rtdsrv.4b8ef99e016b447da4df1f9adeb95e96">
+      <tp>
+        <v>1</v>
+        <stp/>
+        <stp>1e20d4de-2006-41bf-9f80-48b93da56c4b</stp>
+        <tr r="G23" s="4"/>
+      </tp>
+      <tp>
+        <v>1</v>
+        <stp/>
+        <stp>ce261162-24ce-4c6d-a0ab-2cd83d335a7c</stp>
+        <tr r="G34" s="4"/>
+      </tp>
+      <tp>
+        <v>1</v>
+        <stp/>
+        <stp>1fe8571a-1322-4957-a257-27722b06f2ec</stp>
+        <tr r="F1" s="4"/>
+      </tp>
+      <tp>
+        <v>1</v>
+        <stp/>
+        <stp>6ab7d9c1-044d-4c95-8eee-209aa8eda5dc</stp>
+        <tr r="G32" s="4"/>
+      </tp>
+    </main>
+    <main first="rtdsrv.4b8ef99e016b447da4df1f9adeb95e96">
+      <tp>
+        <v>1</v>
+        <stp/>
+        <stp>50a5dade-ed33-482e-a207-4ac937b8d260</stp>
         <tr r="G43" s="1"/>
       </tp>
+      <tp>
+        <v>1</v>
+        <stp/>
+        <stp>9b1b9ee4-4a7f-4a10-9faf-e205c6243c5a</stp>
+        <tr r="G33" s="1"/>
+      </tp>
+      <tp>
+        <v>1</v>
+        <stp/>
+        <stp>10487dcd-ca18-4168-91ef-9969c4be5c62</stp>
+        <tr r="G29" s="1"/>
+      </tp>
     </main>
-    <main first="rtdsrv.da30af61cf3e4a5a94195f27fdd074ca">
-      <tp>
-        <v>1</v>
-        <stp/>
-        <stp>9b0f7522-fb02-492c-b49e-ee514a0afb74</stp>
-        <tr r="I19" s="1"/>
-      </tp>
-      <tp>
-        <v>1</v>
-        <stp/>
-        <stp>b2906bc6-1c00-408e-b9af-029ad8a22c8a</stp>
-        <tr r="G45" s="1"/>
+    <main first="rtdsrv.4b8ef99e016b447da4df1f9adeb95e96">
+      <tp>
+        <v>1</v>
+        <stp/>
+        <stp>68817488-5a6f-4517-8f05-abe5eae029a3</stp>
+        <tr r="G55" s="4"/>
       </tp>
     </main>
-    <main first="rtdsrv.da30af61cf3e4a5a94195f27fdd074ca">
-      <tp>
-        <v>1</v>
-        <stp/>
-        <stp>d41359cf-4f1b-4c32-b7a6-ae72bc604c0c</stp>
-        <tr r="E4" s="3"/>
-      </tp>
-      <tp>
-        <v>1</v>
-        <stp/>
-        <stp>d0e61287-ce66-4238-973b-50d98efec0b0</stp>
-        <tr r="G21" s="1"/>
+    <main first="rtdsrv.4b8ef99e016b447da4df1f9adeb95e96">
+      <tp>
+        <v>1</v>
+        <stp/>
+        <stp>5dd97d21-88d3-495d-a3ec-ab00bd0b884d</stp>
+        <tr r="F1" s="1"/>
       </tp>
     </main>
-    <main first="rtdsrv.da30af61cf3e4a5a94195f27fdd074ca">
-      <tp>
-        <v>1</v>
-        <stp/>
-        <stp>8f86837d-5995-4ea9-b8df-554737d4a4c4</stp>
-        <tr r="G23" s="1"/>
+    <main first="rtdsrv.4b8ef99e016b447da4df1f9adeb95e96">
+      <tp>
+        <v>1</v>
+        <stp/>
+        <stp>ec33074b-202c-4cda-8fd4-da68ad1c0a3f</stp>
+        <tr r="I28" s="1"/>
       </tp>
     </main>
-    <main first="rtdsrv.da30af61cf3e4a5a94195f27fdd074ca">
-      <tp>
-        <v>1</v>
-        <stp/>
-        <stp>09a9dcdd-c4f5-4f8d-972c-09e588239e14</stp>
-        <tr r="G57" s="1"/>
+    <main first="rtdsrv.4b8ef99e016b447da4df1f9adeb95e96">
+      <tp>
+        <v>1</v>
+        <stp/>
+        <stp>2ed72686-3229-4c7b-9b5a-2dabef48625d</stp>
+        <tr r="G28" s="1"/>
+      </tp>
+      <tp>
+        <v>1</v>
+        <stp/>
+        <stp>ad36159f-d95a-408b-a01c-a0ad60f46a87</stp>
+        <tr r="G40" s="1"/>
+      </tp>
+      <tp>
+        <v>1</v>
+        <stp/>
+        <stp>3b855b64-7082-46e7-9617-789a87d58986</stp>
+        <tr r="G54" s="4"/>
       </tp>
     </main>
-    <main first="rtdsrv.da30af61cf3e4a5a94195f27fdd074ca">
-      <tp>
-        <v>1</v>
-        <stp/>
-        <stp>908e95de-4bbf-44e4-9ba9-cb11708173c0</stp>
-        <tr r="G50" s="1"/>
+    <main first="rtdsrv.4b8ef99e016b447da4df1f9adeb95e96">
+      <tp>
+        <v>1</v>
+        <stp/>
+        <stp>4fca72d5-313d-4a80-ac8b-cde084ac485b</stp>
+        <tr r="G39" s="4"/>
       </tp>
     </main>
-    <main first="rtdsrv.da30af61cf3e4a5a94195f27fdd074ca">
-      <tp>
-        <v>1</v>
-        <stp/>
-        <stp>fe13b170-c101-4957-b8f0-2344d475cd18</stp>
+    <main first="rtdsrv.4b8ef99e016b447da4df1f9adeb95e96">
+      <tp>
+        <v>1</v>
+        <stp/>
+        <stp>a28a91ab-2972-417f-8575-1cd8af371c3f</stp>
+        <tr r="G48" s="4"/>
+      </tp>
+    </main>
+    <main first="rtdsrv.4b8ef99e016b447da4df1f9adeb95e96">
+      <tp>
+        <v>1</v>
+        <stp/>
+        <stp>ca9757e3-7740-4471-bd1f-59b2b8403f6c</stp>
         <tr r="G55" s="1"/>
-      </tp>
-    </main>
-    <main first="rtdsrv.da30af61cf3e4a5a94195f27fdd074ca">
-      <tp>
-        <v>1</v>
-        <stp/>
-        <stp>2dcfdd96-f37f-4170-82b6-ff69bd97a210</stp>
-        <tr r="G35" s="1"/>
-      </tp>
-    </main>
-    <main first="rtdsrv.da30af61cf3e4a5a94195f27fdd074ca">
-      <tp>
-        <v>1</v>
-        <stp/>
-        <stp>5dc1d79c-6026-4851-abc6-80c7ee5b8ffa</stp>
-        <tr r="G26" s="1"/>
-      </tp>
-    </main>
-    <main first="rtdsrv.da30af61cf3e4a5a94195f27fdd074ca">
-      <tp>
-        <v>1</v>
-        <stp/>
-        <stp>82df0738-be39-4c04-82c3-4481c4d2f4f8</stp>
-        <tr r="G22" s="1"/>
-      </tp>
-    </main>
-    <main first="rtdsrv.da30af61cf3e4a5a94195f27fdd074ca">
-      <tp>
-        <v>1</v>
-        <stp/>
-        <stp>f7de2308-d966-4801-a61c-58826fc62941</stp>
-        <tr r="G31" s="1"/>
-      </tp>
-      <tp>
-        <v>1</v>
-        <stp/>
-        <stp>a34588c1-98f5-481d-b7d7-5337dc465e85</stp>
-        <tr r="G25" s="1"/>
-      </tp>
-    </main>
-    <main first="rtdsrv.da30af61cf3e4a5a94195f27fdd074ca">
-      <tp>
-        <v>1</v>
-        <stp/>
-        <stp>670267aa-3ac1-46f0-ac72-02bce736a7db</stp>
-        <tr r="G20" s="1"/>
-      </tp>
-    </main>
-    <main first="rtdsrv.da30af61cf3e4a5a94195f27fdd074ca">
-      <tp>
-        <v>1</v>
-        <stp/>
-        <stp>ac050767-4cd9-4979-a898-5d8733ee87cf</stp>
-        <tr r="G40" s="1"/>
-      </tp>
-      <tp>
-        <v>1</v>
-        <stp/>
-        <stp>ddeffaa2-ae8d-425d-9c29-c186f1411270</stp>
-        <tr r="G36" s="1"/>
-      </tp>
-      <tp>
-        <v>1</v>
-        <stp/>
-        <stp>05defc1e-b383-4186-8ac9-cd415369b65f</stp>
-        <tr r="I28" s="1"/>
-      </tp>
-      <tp>
-        <v>1</v>
-        <stp/>
-        <stp>2955d900-acde-459e-acc1-fd4531d0f232</stp>
-        <tr r="G38" s="1"/>
-      </tp>
-      <tp>
-        <v>1</v>
-        <stp/>
-        <stp>0d440dbe-5192-41d7-8815-9fbdd79aeb45</stp>
-        <tr r="G49" s="1"/>
-      </tp>
-      <tp>
-        <v>1</v>
-        <stp/>
-        <stp>6a3f0ae0-3bb0-4ddd-a9b0-a4e36d650f44</stp>
-        <tr r="G34" s="1"/>
-      </tp>
-      <tp>
-        <v>1</v>
-        <stp/>
-        <stp>76dc2e7d-4326-486e-8454-c0d1d05834c7</stp>
-        <tr r="G47" s="1"/>
-      </tp>
-    </main>
-    <main first="rtdsrv.da30af61cf3e4a5a94195f27fdd074ca">
-      <tp>
-        <v>1</v>
-        <stp/>
-        <stp>7b64e19d-80a1-4c63-80d7-c0bb18ec56ba</stp>
-        <tr r="G42" s="1"/>
-      </tp>
-    </main>
-    <main first="rtdsrv.da30af61cf3e4a5a94195f27fdd074ca">
-      <tp>
-        <v>1</v>
-        <stp/>
-        <stp>40186b44-8817-45bd-b30c-66a836a08b81</stp>
-        <tr r="C2" s="2"/>
-      </tp>
-      <tp>
-        <v>1</v>
-        <stp/>
-        <stp>1b1fadc6-7e5c-4ad1-939f-63f1a4d15a17</stp>
-        <tr r="G30" s="1"/>
-      </tp>
-      <tp>
-        <v>1</v>
-        <stp/>
-        <stp>fd326be5-bf91-4ef0-b1fa-f21fa8946f08</stp>
-        <tr r="G19" s="1"/>
-      </tp>
-      <tp>
-        <v>1</v>
-        <stp/>
-        <stp>6850bd1c-6e8c-40a3-8534-f66c8738c5ba</stp>
-        <tr r="G46" s="1"/>
-      </tp>
-      <tp>
-        <v>1</v>
-        <stp/>
-        <stp>e8e3f255-6c48-4e13-a2c3-966ed6bf42fc</stp>
-        <tr r="G39" s="1"/>
-      </tp>
-      <tp>
-        <v>10</v>
-        <stp/>
-        <stp>37de08e9-0167-4fbc-8c01-65486a4edf0f</stp>
-        <tr r="E7" s="3"/>
-      </tp>
-    </main>
-    <main first="rtdsrv.da30af61cf3e4a5a94195f27fdd074ca">
-      <tp>
-        <v>1</v>
-        <stp/>
-        <stp>98a7fab1-a0a9-4330-a4eb-12261bc61dd8</stp>
-        <tr r="G44" s="1"/>
-      </tp>
-      <tp>
-        <v>1</v>
-        <stp/>
-        <stp>fed5a1d5-22bf-445e-b6a4-249329dcc638</stp>
-        <tr r="G27" s="1"/>
-      </tp>
-    </main>
-    <main first="rtdsrv.da30af61cf3e4a5a94195f27fdd074ca">
-      <tp>
-        <v>1</v>
-        <stp/>
-        <stp>ce470760-a3c9-441d-885a-375979c3d4d3</stp>
-        <tr r="G28" s="1"/>
-      </tp>
-    </main>
-    <main first="rtdsrv.da30af61cf3e4a5a94195f27fdd074ca">
-      <tp>
-        <v>1</v>
-        <stp/>
-        <stp>4835f6a1-87a1-4740-a8cb-692464f720b9</stp>
-        <tr r="G24" s="1"/>
-      </tp>
-    </main>
-    <main first="rtdsrv.da30af61cf3e4a5a94195f27fdd074ca">
-      <tp>
-        <v>1</v>
-        <stp/>
-        <stp>6ce81161-9f0d-4c2f-be8c-d82e6a33a714</stp>
-        <tr r="F6" s="1"/>
-      </tp>
-    </main>
-    <main first="rtdsrv.da30af61cf3e4a5a94195f27fdd074ca">
-      <tp>
-        <v>1</v>
-        <stp/>
-        <stp>73ae7014-afde-41b8-b204-a3274c78da62</stp>
-        <tr r="G51" s="1"/>
-      </tp>
-    </main>
-    <main first="rtdsrv.da30af61cf3e4a5a94195f27fdd074ca">
-      <tp>
-        <v>1</v>
-        <stp/>
-        <stp>aee4a2c5-6ce5-4bf4-97df-3dbc85d1b6b2</stp>
-        <tr r="G32" s="1"/>
-      </tp>
-      <tp>
-        <v>1</v>
-        <stp/>
-        <stp>a7d8db76-c84c-4464-80fe-a54eac2b5d35</stp>
-        <tr r="G54" s="1"/>
-      </tp>
-    </main>
-    <main first="rtdsrv.da30af61cf3e4a5a94195f27fdd074ca">
-      <tp>
-        <v>1</v>
-        <stp/>
-        <stp>2c6e798c-8edd-432e-a52d-ae56d324d222</stp>
-        <tr r="G41" s="1"/>
-      </tp>
-    </main>
-    <main first="rtdsrv.da30af61cf3e4a5a94195f27fdd074ca">
-      <tp>
-        <v>1</v>
-        <stp/>
-        <stp>9ff95a53-ffbd-4161-b650-60bd0c030f8d</stp>
-        <tr r="G33" s="1"/>
-      </tp>
-      <tp>
-        <v>1</v>
-        <stp/>
-        <stp>b0e8efc0-1416-4f37-a3ca-10473dbcc75b</stp>
-        <tr r="G48" s="1"/>
-      </tp>
-      <tp>
-        <v>1</v>
-        <stp/>
-        <stp>dccd6470-d289-48aa-bc03-b321c62a37c1</stp>
-        <tr r="G29" s="1"/>
-      </tp>
-      <tp>
-        <v>1</v>
-        <stp/>
-        <stp>225fcc00-4787-49f2-a7a9-7370849adbf3</stp>
-        <tr r="F1" s="1"/>
-      </tp>
-      <tp>
-        <v>1</v>
-        <stp/>
-        <stp>f5a74a31-566f-4441-b55b-97dc9d4a5e8d</stp>
-        <tr r="G52" s="1"/>
-      </tp>
-    </main>
-    <main first="rtdsrv.da30af61cf3e4a5a94195f27fdd074ca">
-      <tp>
-        <v>1</v>
-        <stp/>
-        <stp>9016b188-060e-413c-9ea9-7ecc70f0d504</stp>
-        <tr r="G56" s="1"/>
-      </tp>
-      <tp>
-        <v>2</v>
-        <stp/>
-        <stp>0fa64373-1b60-4726-8d69-53d71fdacb5e</stp>
-        <tr r="E6" s="3"/>
-      </tp>
-      <tp>
-        <v>1</v>
-        <stp/>
-        <stp>d1e9d6b5-9d39-4b5b-999d-4a2a9ea26375</stp>
-        <tr r="G53" s="1"/>
-      </tp>
-    </main>
-    <main first="rtdsrv.da30af61cf3e4a5a94195f27fdd074ca">
-      <tp>
-        <v>1</v>
-        <stp/>
-        <stp>7edd312f-2579-4474-9061-b6595b0a7bab</stp>
-        <tr r="G37" s="1"/>
       </tp>
     </main>
   </volType>
@@ -1194,12 +1470,12 @@
         <v>27</v>
       </c>
       <c r="F1" t="str" cm="1">
-        <f t="array" ref="F1">_xll.ExLibris.Json.CreateJsonObject(E3:F6, EXLIBRIS_CONFIGURATION)</f>
-        <v>JsonObject:4CBE4E84-D038-4955-8393-CE04A80A3583</v>
+        <f t="array" ref="F1">_xll.ExLibris.Json.CreateJsonObject(E3:F6)</f>
+        <v>JsonObject:BE1FC4FB-547E-4869-A7F0-521890319C3A</v>
       </c>
       <c r="K1" t="str">
         <f>EXLIBRIS_CONFIGURATION</f>
-        <v>ExLibris.Core.ExLibrisConfiguration:E8DCA9AB-6EBC-4C98-8C3A-029399E3EB11</v>
+        <v>ExLibris.Core.ExLibrisConfiguration:78976E74-B484-403F-9AE1-F5D51D57D63F</v>
       </c>
     </row>
     <row r="2" spans="2:25" x14ac:dyDescent="0.4">
@@ -1268,15 +1544,15 @@
         <v>26</v>
       </c>
       <c r="F6" t="str" cm="1">
-        <f t="array" ref="F6">_xll.ExLibris.Json.CreateJsonArray(E8:J14, EXLIBRIS_CONFIGURATION)</f>
-        <v>JsonObject:B058ED14-E401-4142-AB75-B5F6A0D6467C</v>
+        <f t="array" ref="F6">_xll.ExLibris.Json.CreateJsonArray(E8:J14)</f>
+        <v>JsonObject:7FD63C57-393E-49CA-A58E-C4F2225A9BAA</v>
       </c>
       <c r="L6" t="s">
         <v>68</v>
       </c>
       <c r="M6" t="str" cm="1">
         <f t="array" ref="M6">_xll.ExLibris.Json.ShowJsonText(F1)</f>
-        <v>{"trade_code":"money_00001","couter_party":"CP00001","fixed_leg":{"pay_or_recieve":"Receive","cashflows":[{"payment _date":"2022-03-12","start_date":"2021-09-13","end_date":"2022-03-12","day_count_type":"ACT/360","amout":10000000,"fixed_rate":0.001},{"payment _date":"2022-09-08","start_date":"2022-03-12","end_date":"2022-09-08","day_count_type":"ACT/360","amout":11000000,"fixed_rate":0.001},{"payment _date":"2023-03-07","start_date":"2022-09-08","end_date":"2023-03-07","day_count_type":"ACT/360","amout":12000000,"fixed_rate":0.001},{"payment _date":"2023-09-03","start_date":"2023-03-07","end_date":"2023-09-03","day_count_type":"ACT/360","amout":13000000,"fixed_rate":0.001},{"payment _date":"2024-03-01","start_date":"2023-09-03","end_date":"2024-03-01","day_count_type":"ACT/360","amout":14000000,"fixed_rate":0.001},{"payment _date":"2024-08-28","start_date":"2024-03-01","end_date":"2024-08-28","day_count_type":"ACT/360","amout":15000000,"fixed_rate":0.001}]}}</v>
+        <v>{"trade_code":"money_00001","couter_party":"CP00001","fixed_leg":{"pay_or_recieve":"Receive","cashflows":[{"payment _date":44632,"start_date":44452,"end_date":44632,"day_count_type":"ACT/360","amout":10000000,"fixed_rate":0.001},{"payment _date":44812,"start_date":44632,"end_date":44812,"day_count_type":"ACT/360","amout":11000000,"fixed_rate":0.001},{"payment _date":44992,"start_date":44812,"end_date":44992,"day_count_type":"ACT/360","amout":12000000,"fixed_rate":0.001},{"payment _date":45172,"start_date":44992,"end_date":45172,"day_count_type":"ACT/360","amout":13000000,"fixed_rate":0.001},{"payment _date":45352,"start_date":45172,"end_date":45352,"day_count_type":"ACT/360","amout":14000000,"fixed_rate":0.001},{"payment _date":45532,"start_date":45352,"end_date":45532,"day_count_type":"ACT/360","amout":15000000,"fixed_rate":0.001}]}}</v>
       </c>
     </row>
     <row r="7" spans="2:25" x14ac:dyDescent="0.4">
@@ -1284,7 +1560,7 @@
         <v>74</v>
       </c>
       <c r="M7" t="s">
-        <v>100</v>
+        <v>112</v>
       </c>
     </row>
     <row r="8" spans="2:25" x14ac:dyDescent="0.4">
@@ -1482,19 +1758,19 @@
     </row>
     <row r="19" spans="5:36" x14ac:dyDescent="0.4">
       <c r="E19" t="str" cm="1">
-        <f t="array" ref="E19:F57">_xll.ExLibris.Json.GetJsonKeyValues(F1, EXLIBRIS_CONFIGURATION)</f>
+        <f t="array" ref="E19:F57">_xll.ExLibris.Json.GetJsonKeyValues(F1)</f>
         <v>trade_code</v>
       </c>
       <c r="F19" t="str">
         <v>money_00001</v>
       </c>
       <c r="G19" t="str" cm="1">
-        <f t="array" ref="G19">_xll.ExLibris.Json.GetJsonValue($F$1,E19, EXLIBRIS_CONFIGURATION)</f>
+        <f t="array" ref="G19">_xll.ExLibris.Json.GetJsonValue($F$1,E19)</f>
         <v>money_00001</v>
       </c>
       <c r="I19" t="str" cm="1">
-        <f t="array" ref="I19">_xll.ExLibris.Json.GetJsonValue(F1,E6, EXLIBRIS_CONFIGURATION)</f>
-        <v>JsonObject:F3637329-E835-40D6-98B6-1A8D47A1CCA3</v>
+        <f t="array" ref="I19">_xll.ExLibris.Json.GetJsonValue(F1,E6)</f>
+        <v>JsonObject:854737B1-0B9E-4F70-9A82-B16823CD8333</v>
       </c>
       <c r="P19" t="s">
         <v>14</v>
@@ -1526,11 +1802,11 @@
         <v>CP00001</v>
       </c>
       <c r="G20" t="str" cm="1">
-        <f t="array" ref="G20">_xll.ExLibris.Json.GetJsonValue($F$1,E20, EXLIBRIS_CONFIGURATION)</f>
+        <f t="array" ref="G20">_xll.ExLibris.Json.GetJsonValue($F$1,E20)</f>
         <v>CP00001</v>
       </c>
       <c r="I20" t="str" cm="1">
-        <f t="array" ref="I20:N26">_xll.ExLibris.Json.GetJsonTable(I19, EXLIBRIS_CONFIGURATION)</f>
+        <f t="array" ref="I20:N26">_xll.ExLibris.Json.GetJsonTable(I19)</f>
         <v>payment _date</v>
       </c>
       <c r="J20" t="str">
@@ -1620,17 +1896,17 @@
         <v>Receive</v>
       </c>
       <c r="G21" t="str" cm="1">
-        <f t="array" ref="G21">_xll.ExLibris.Json.GetJsonValue($F$1,E21, EXLIBRIS_CONFIGURATION)</f>
+        <f t="array" ref="G21">_xll.ExLibris.Json.GetJsonValue($F$1,E21)</f>
         <v>Receive</v>
       </c>
-      <c r="I21" t="str">
-        <v>2022-03-12</v>
-      </c>
-      <c r="J21" t="str">
-        <v>2021-09-13</v>
-      </c>
-      <c r="K21" t="str">
-        <v>2022-03-12</v>
+      <c r="I21">
+        <v>44632</v>
+      </c>
+      <c r="J21">
+        <v>44452</v>
+      </c>
+      <c r="K21">
+        <v>44632</v>
       </c>
       <c r="L21" t="str">
         <v>ACT/360</v>
@@ -1650,14 +1926,14 @@
       <c r="R21" t="s">
         <v>24</v>
       </c>
-      <c r="T21" t="s">
-        <v>93</v>
-      </c>
-      <c r="U21" t="s">
-        <v>94</v>
-      </c>
-      <c r="V21" t="s">
-        <v>93</v>
+      <c r="T21">
+        <v>44632</v>
+      </c>
+      <c r="U21">
+        <v>44452</v>
+      </c>
+      <c r="V21">
+        <v>44632</v>
       </c>
       <c r="W21" t="s">
         <v>8</v>
@@ -1709,21 +1985,21 @@
       <c r="E22" t="str">
         <v>fixed_leg.cashflows.[0].payment _date</v>
       </c>
-      <c r="F22" t="str">
-        <v>2022-03-12</v>
-      </c>
-      <c r="G22" s="1" t="str" cm="1">
-        <f t="array" ref="G22">_xll.ExLibris.Json.GetJsonValue($F$1,E22, EXLIBRIS_CONFIGURATION)</f>
-        <v>2022-03-12</v>
-      </c>
-      <c r="I22" t="str">
-        <v>2022-09-08</v>
-      </c>
-      <c r="J22" t="str">
-        <v>2022-03-12</v>
-      </c>
-      <c r="K22" t="str">
-        <v>2022-09-08</v>
+      <c r="F22">
+        <v>44632</v>
+      </c>
+      <c r="G22" cm="1">
+        <f t="array" ref="G22">_xll.ExLibris.Json.GetJsonValue($F$1,E22)</f>
+        <v>44632</v>
+      </c>
+      <c r="I22">
+        <v>44812</v>
+      </c>
+      <c r="J22">
+        <v>44632</v>
+      </c>
+      <c r="K22">
+        <v>44812</v>
       </c>
       <c r="L22" t="str">
         <v>ACT/360</v>
@@ -1737,20 +2013,20 @@
       <c r="P22" t="s">
         <v>32</v>
       </c>
-      <c r="Q22" t="s">
-        <v>93</v>
-      </c>
-      <c r="R22" t="s">
-        <v>93</v>
-      </c>
-      <c r="T22" t="s">
-        <v>95</v>
-      </c>
-      <c r="U22" t="s">
-        <v>93</v>
-      </c>
-      <c r="V22" t="s">
-        <v>95</v>
+      <c r="Q22">
+        <v>44632</v>
+      </c>
+      <c r="R22">
+        <v>44632</v>
+      </c>
+      <c r="T22">
+        <v>44812</v>
+      </c>
+      <c r="U22">
+        <v>44632</v>
+      </c>
+      <c r="V22">
+        <v>44812</v>
       </c>
       <c r="W22" t="s">
         <v>8</v>
@@ -1802,21 +2078,21 @@
       <c r="E23" t="str">
         <v>fixed_leg.cashflows.[0].start_date</v>
       </c>
-      <c r="F23" t="str">
-        <v>2021-09-13</v>
-      </c>
-      <c r="G23" t="str" cm="1">
-        <f t="array" ref="G23">_xll.ExLibris.Json.GetJsonValue($F$1,E23, EXLIBRIS_CONFIGURATION)</f>
-        <v>2021-09-13</v>
-      </c>
-      <c r="I23" t="str">
-        <v>2023-03-07</v>
-      </c>
-      <c r="J23" t="str">
-        <v>2022-09-08</v>
-      </c>
-      <c r="K23" t="str">
-        <v>2023-03-07</v>
+      <c r="F23">
+        <v>44452</v>
+      </c>
+      <c r="G23" cm="1">
+        <f t="array" ref="G23">_xll.ExLibris.Json.GetJsonValue($F$1,E23)</f>
+        <v>44452</v>
+      </c>
+      <c r="I23">
+        <v>44992</v>
+      </c>
+      <c r="J23">
+        <v>44812</v>
+      </c>
+      <c r="K23">
+        <v>44992</v>
       </c>
       <c r="L23" t="str">
         <v>ACT/360</v>
@@ -1830,20 +2106,20 @@
       <c r="P23" t="s">
         <v>33</v>
       </c>
-      <c r="Q23" t="s">
-        <v>94</v>
-      </c>
-      <c r="R23" t="s">
-        <v>94</v>
-      </c>
-      <c r="T23" t="s">
-        <v>96</v>
-      </c>
-      <c r="U23" t="s">
-        <v>95</v>
-      </c>
-      <c r="V23" t="s">
-        <v>96</v>
+      <c r="Q23">
+        <v>44452</v>
+      </c>
+      <c r="R23">
+        <v>44452</v>
+      </c>
+      <c r="T23">
+        <v>44992</v>
+      </c>
+      <c r="U23">
+        <v>44812</v>
+      </c>
+      <c r="V23">
+        <v>44992</v>
       </c>
       <c r="W23" t="s">
         <v>8</v>
@@ -1895,21 +2171,21 @@
       <c r="E24" t="str">
         <v>fixed_leg.cashflows.[0].end_date</v>
       </c>
-      <c r="F24" t="str">
-        <v>2022-03-12</v>
-      </c>
-      <c r="G24" t="str" cm="1">
-        <f t="array" ref="G24">_xll.ExLibris.Json.GetJsonValue($F$1,E24, EXLIBRIS_CONFIGURATION)</f>
-        <v>2022-03-12</v>
-      </c>
-      <c r="I24" t="str">
-        <v>2023-09-03</v>
-      </c>
-      <c r="J24" t="str">
-        <v>2023-03-07</v>
-      </c>
-      <c r="K24" t="str">
-        <v>2023-09-03</v>
+      <c r="F24">
+        <v>44632</v>
+      </c>
+      <c r="G24" cm="1">
+        <f t="array" ref="G24">_xll.ExLibris.Json.GetJsonValue($F$1,E24)</f>
+        <v>44632</v>
+      </c>
+      <c r="I24">
+        <v>45172</v>
+      </c>
+      <c r="J24">
+        <v>44992</v>
+      </c>
+      <c r="K24">
+        <v>45172</v>
       </c>
       <c r="L24" t="str">
         <v>ACT/360</v>
@@ -1923,20 +2199,20 @@
       <c r="P24" t="s">
         <v>34</v>
       </c>
-      <c r="Q24" t="s">
-        <v>93</v>
-      </c>
-      <c r="R24" t="s">
-        <v>93</v>
-      </c>
-      <c r="T24" t="s">
-        <v>97</v>
-      </c>
-      <c r="U24" t="s">
-        <v>96</v>
-      </c>
-      <c r="V24" t="s">
-        <v>97</v>
+      <c r="Q24">
+        <v>44632</v>
+      </c>
+      <c r="R24">
+        <v>44632</v>
+      </c>
+      <c r="T24">
+        <v>45172</v>
+      </c>
+      <c r="U24">
+        <v>44992</v>
+      </c>
+      <c r="V24">
+        <v>45172</v>
       </c>
       <c r="W24" t="s">
         <v>8</v>
@@ -1992,17 +2268,17 @@
         <v>ACT/360</v>
       </c>
       <c r="G25" t="str" cm="1">
-        <f t="array" ref="G25">_xll.ExLibris.Json.GetJsonValue($F$1,E25, EXLIBRIS_CONFIGURATION)</f>
+        <f t="array" ref="G25">_xll.ExLibris.Json.GetJsonValue($F$1,E25)</f>
         <v>ACT/360</v>
       </c>
-      <c r="I25" t="str">
-        <v>2024-03-01</v>
-      </c>
-      <c r="J25" t="str">
-        <v>2023-09-03</v>
-      </c>
-      <c r="K25" t="str">
-        <v>2024-03-01</v>
+      <c r="I25">
+        <v>45352</v>
+      </c>
+      <c r="J25">
+        <v>45172</v>
+      </c>
+      <c r="K25">
+        <v>45352</v>
       </c>
       <c r="L25" t="str">
         <v>ACT/360</v>
@@ -2022,14 +2298,14 @@
       <c r="R25" t="s">
         <v>8</v>
       </c>
-      <c r="T25" t="s">
-        <v>98</v>
-      </c>
-      <c r="U25" t="s">
-        <v>97</v>
-      </c>
-      <c r="V25" t="s">
-        <v>98</v>
+      <c r="T25">
+        <v>45352</v>
+      </c>
+      <c r="U25">
+        <v>45172</v>
+      </c>
+      <c r="V25">
+        <v>45352</v>
       </c>
       <c r="W25" t="s">
         <v>8</v>
@@ -2085,17 +2361,17 @@
         <v>10000000</v>
       </c>
       <c r="G26" cm="1">
-        <f t="array" ref="G26">_xll.ExLibris.Json.GetJsonValue($F$1,E26, EXLIBRIS_CONFIGURATION)</f>
+        <f t="array" ref="G26">_xll.ExLibris.Json.GetJsonValue($F$1,E26)</f>
         <v>10000000</v>
       </c>
-      <c r="I26" t="str">
-        <v>2024-08-28</v>
-      </c>
-      <c r="J26" t="str">
-        <v>2024-03-01</v>
-      </c>
-      <c r="K26" t="str">
-        <v>2024-08-28</v>
+      <c r="I26">
+        <v>45532</v>
+      </c>
+      <c r="J26">
+        <v>45352</v>
+      </c>
+      <c r="K26">
+        <v>45532</v>
       </c>
       <c r="L26" t="str">
         <v>ACT/360</v>
@@ -2115,14 +2391,14 @@
       <c r="R26">
         <v>10000000</v>
       </c>
-      <c r="T26" t="s">
-        <v>99</v>
-      </c>
-      <c r="U26" t="s">
-        <v>98</v>
-      </c>
-      <c r="V26" t="s">
-        <v>99</v>
+      <c r="T26">
+        <v>45532</v>
+      </c>
+      <c r="U26">
+        <v>45352</v>
+      </c>
+      <c r="V26">
+        <v>45532</v>
       </c>
       <c r="W26" t="s">
         <v>8</v>
@@ -2178,7 +2454,7 @@
         <v>1E-3</v>
       </c>
       <c r="G27" cm="1">
-        <f t="array" ref="G27">_xll.ExLibris.Json.GetJsonValue($F$1,E27, EXLIBRIS_CONFIGURATION)</f>
+        <f t="array" ref="G27">_xll.ExLibris.Json.GetJsonValue($F$1,E27)</f>
         <v>1E-3</v>
       </c>
       <c r="P27" t="s">
@@ -2207,25 +2483,25 @@
       <c r="E28" t="str">
         <v>fixed_leg.cashflows.[1].payment _date</v>
       </c>
-      <c r="F28" t="str">
-        <v>2022-09-08</v>
-      </c>
-      <c r="G28" t="str" cm="1">
-        <f t="array" ref="G28">_xll.ExLibris.Json.GetJsonValue($F$1,E28, EXLIBRIS_CONFIGURATION)</f>
-        <v>2022-09-08</v>
+      <c r="F28">
+        <v>44812</v>
+      </c>
+      <c r="G28" cm="1">
+        <f t="array" ref="G28">_xll.ExLibris.Json.GetJsonValue($F$1,E28)</f>
+        <v>44812</v>
       </c>
       <c r="I28" t="str" cm="1">
-        <f t="array" ref="I28">_xll.ExLibris.Json.GetJsonValue(I19,"[2]", EXLIBRIS_CONFIGURATION)</f>
-        <v>JsonObject:FEEEC164-0563-4FDB-931A-8D59613C5F83</v>
+        <f t="array" ref="I28">_xll.ExLibris.Json.GetJsonValue(I19,"[2]")</f>
+        <v>JsonObject:1676224C-EAA0-4A14-9F89-A758F8BDAE9D</v>
       </c>
       <c r="P28" t="s">
         <v>38</v>
       </c>
-      <c r="Q28" t="s">
-        <v>95</v>
-      </c>
-      <c r="R28" t="s">
-        <v>95</v>
+      <c r="Q28">
+        <v>44812</v>
+      </c>
+      <c r="R28">
+        <v>44812</v>
       </c>
       <c r="AA28" t="b">
         <f t="shared" si="4"/>
@@ -2244,15 +2520,15 @@
       <c r="E29" t="str">
         <v>fixed_leg.cashflows.[1].start_date</v>
       </c>
-      <c r="F29" t="str">
-        <v>2022-03-12</v>
-      </c>
-      <c r="G29" t="str" cm="1">
-        <f t="array" ref="G29">_xll.ExLibris.Json.GetJsonValue($F$1,E29, EXLIBRIS_CONFIGURATION)</f>
-        <v>2022-03-12</v>
+      <c r="F29">
+        <v>44632</v>
+      </c>
+      <c r="G29" cm="1">
+        <f t="array" ref="G29">_xll.ExLibris.Json.GetJsonValue($F$1,E29)</f>
+        <v>44632</v>
       </c>
       <c r="I29" t="str" cm="1">
-        <f t="array" ref="I29:N30">_xll.ExLibris.Json.GetJsonTable(I28, EXLIBRIS_CONFIGURATION)</f>
+        <f t="array" ref="I29:N30">_xll.ExLibris.Json.GetJsonTable(I28)</f>
         <v>payment _date</v>
       </c>
       <c r="J29" t="str">
@@ -2273,11 +2549,11 @@
       <c r="P29" t="s">
         <v>39</v>
       </c>
-      <c r="Q29" t="s">
-        <v>93</v>
-      </c>
-      <c r="R29" t="s">
-        <v>93</v>
+      <c r="Q29">
+        <v>44632</v>
+      </c>
+      <c r="R29">
+        <v>44632</v>
       </c>
       <c r="T29" t="s">
         <v>0</v>
@@ -2338,21 +2614,21 @@
       <c r="E30" t="str">
         <v>fixed_leg.cashflows.[1].end_date</v>
       </c>
-      <c r="F30" t="str">
-        <v>2022-09-08</v>
-      </c>
-      <c r="G30" t="str" cm="1">
-        <f t="array" ref="G30">_xll.ExLibris.Json.GetJsonValue($F$1,E30, EXLIBRIS_CONFIGURATION)</f>
-        <v>2022-09-08</v>
-      </c>
-      <c r="I30" t="str">
-        <v>2023-03-07</v>
-      </c>
-      <c r="J30" t="str">
-        <v>2022-09-08</v>
-      </c>
-      <c r="K30" t="str">
-        <v>2023-03-07</v>
+      <c r="F30">
+        <v>44812</v>
+      </c>
+      <c r="G30" cm="1">
+        <f t="array" ref="G30">_xll.ExLibris.Json.GetJsonValue($F$1,E30)</f>
+        <v>44812</v>
+      </c>
+      <c r="I30">
+        <v>44992</v>
+      </c>
+      <c r="J30">
+        <v>44812</v>
+      </c>
+      <c r="K30">
+        <v>44992</v>
       </c>
       <c r="L30" t="str">
         <v>ACT/360</v>
@@ -2366,20 +2642,20 @@
       <c r="P30" t="s">
         <v>40</v>
       </c>
-      <c r="Q30" t="s">
-        <v>95</v>
-      </c>
-      <c r="R30" t="s">
-        <v>95</v>
-      </c>
-      <c r="T30" t="s">
-        <v>96</v>
-      </c>
-      <c r="U30" t="s">
-        <v>95</v>
-      </c>
-      <c r="V30" t="s">
-        <v>96</v>
+      <c r="Q30">
+        <v>44812</v>
+      </c>
+      <c r="R30">
+        <v>44812</v>
+      </c>
+      <c r="T30">
+        <v>44992</v>
+      </c>
+      <c r="U30">
+        <v>44812</v>
+      </c>
+      <c r="V30">
+        <v>44992</v>
       </c>
       <c r="W30" t="s">
         <v>8</v>
@@ -2435,7 +2711,7 @@
         <v>ACT/360</v>
       </c>
       <c r="G31" t="str" cm="1">
-        <f t="array" ref="G31">_xll.ExLibris.Json.GetJsonValue($F$1,E31, EXLIBRIS_CONFIGURATION)</f>
+        <f t="array" ref="G31">_xll.ExLibris.Json.GetJsonValue($F$1,E31)</f>
         <v>ACT/360</v>
       </c>
       <c r="P31" t="s">
@@ -2468,7 +2744,7 @@
         <v>11000000</v>
       </c>
       <c r="G32" cm="1">
-        <f t="array" ref="G32">_xll.ExLibris.Json.GetJsonValue($F$1,E32, EXLIBRIS_CONFIGURATION)</f>
+        <f t="array" ref="G32">_xll.ExLibris.Json.GetJsonValue($F$1,E32)</f>
         <v>11000000</v>
       </c>
       <c r="P32" t="s">
@@ -2501,7 +2777,7 @@
         <v>1E-3</v>
       </c>
       <c r="G33" cm="1">
-        <f t="array" ref="G33">_xll.ExLibris.Json.GetJsonValue($F$1,E33, EXLIBRIS_CONFIGURATION)</f>
+        <f t="array" ref="G33">_xll.ExLibris.Json.GetJsonValue($F$1,E33)</f>
         <v>1E-3</v>
       </c>
       <c r="P33" t="s">
@@ -2530,21 +2806,21 @@
       <c r="E34" t="str">
         <v>fixed_leg.cashflows.[2].payment _date</v>
       </c>
-      <c r="F34" t="str">
-        <v>2023-03-07</v>
-      </c>
-      <c r="G34" t="str" cm="1">
-        <f t="array" ref="G34">_xll.ExLibris.Json.GetJsonValue($F$1,E34, EXLIBRIS_CONFIGURATION)</f>
-        <v>2023-03-07</v>
+      <c r="F34">
+        <v>44992</v>
+      </c>
+      <c r="G34" cm="1">
+        <f t="array" ref="G34">_xll.ExLibris.Json.GetJsonValue($F$1,E34)</f>
+        <v>44992</v>
       </c>
       <c r="P34" t="s">
         <v>44</v>
       </c>
-      <c r="Q34" t="s">
-        <v>96</v>
-      </c>
-      <c r="R34" t="s">
-        <v>96</v>
+      <c r="Q34">
+        <v>44992</v>
+      </c>
+      <c r="R34">
+        <v>44992</v>
       </c>
       <c r="AA34" t="b">
         <f t="shared" si="4"/>
@@ -2563,21 +2839,21 @@
       <c r="E35" t="str">
         <v>fixed_leg.cashflows.[2].start_date</v>
       </c>
-      <c r="F35" t="str">
-        <v>2022-09-08</v>
-      </c>
-      <c r="G35" t="str" cm="1">
-        <f t="array" ref="G35">_xll.ExLibris.Json.GetJsonValue($F$1,E35, EXLIBRIS_CONFIGURATION)</f>
-        <v>2022-09-08</v>
+      <c r="F35">
+        <v>44812</v>
+      </c>
+      <c r="G35" cm="1">
+        <f t="array" ref="G35">_xll.ExLibris.Json.GetJsonValue($F$1,E35)</f>
+        <v>44812</v>
       </c>
       <c r="P35" t="s">
         <v>45</v>
       </c>
-      <c r="Q35" t="s">
-        <v>95</v>
-      </c>
-      <c r="R35" t="s">
-        <v>95</v>
+      <c r="Q35">
+        <v>44812</v>
+      </c>
+      <c r="R35">
+        <v>44812</v>
       </c>
       <c r="AA35" t="b">
         <f t="shared" si="4"/>
@@ -2596,21 +2872,21 @@
       <c r="E36" t="str">
         <v>fixed_leg.cashflows.[2].end_date</v>
       </c>
-      <c r="F36" t="str">
-        <v>2023-03-07</v>
-      </c>
-      <c r="G36" t="str" cm="1">
-        <f t="array" ref="G36">_xll.ExLibris.Json.GetJsonValue($F$1,E36, EXLIBRIS_CONFIGURATION)</f>
-        <v>2023-03-07</v>
+      <c r="F36">
+        <v>44992</v>
+      </c>
+      <c r="G36" cm="1">
+        <f t="array" ref="G36">_xll.ExLibris.Json.GetJsonValue($F$1,E36)</f>
+        <v>44992</v>
       </c>
       <c r="P36" t="s">
         <v>46</v>
       </c>
-      <c r="Q36" t="s">
-        <v>96</v>
-      </c>
-      <c r="R36" t="s">
-        <v>96</v>
+      <c r="Q36">
+        <v>44992</v>
+      </c>
+      <c r="R36">
+        <v>44992</v>
       </c>
       <c r="AA36" t="b">
         <f t="shared" si="4"/>
@@ -2633,7 +2909,7 @@
         <v>ACT/360</v>
       </c>
       <c r="G37" t="str" cm="1">
-        <f t="array" ref="G37">_xll.ExLibris.Json.GetJsonValue($F$1,E37, EXLIBRIS_CONFIGURATION)</f>
+        <f t="array" ref="G37">_xll.ExLibris.Json.GetJsonValue($F$1,E37)</f>
         <v>ACT/360</v>
       </c>
       <c r="P37" t="s">
@@ -2666,7 +2942,7 @@
         <v>12000000</v>
       </c>
       <c r="G38" cm="1">
-        <f t="array" ref="G38">_xll.ExLibris.Json.GetJsonValue($F$1,E38, EXLIBRIS_CONFIGURATION)</f>
+        <f t="array" ref="G38">_xll.ExLibris.Json.GetJsonValue($F$1,E38)</f>
         <v>12000000</v>
       </c>
       <c r="P38" t="s">
@@ -2699,7 +2975,7 @@
         <v>1E-3</v>
       </c>
       <c r="G39" cm="1">
-        <f t="array" ref="G39">_xll.ExLibris.Json.GetJsonValue($F$1,E39, EXLIBRIS_CONFIGURATION)</f>
+        <f t="array" ref="G39">_xll.ExLibris.Json.GetJsonValue($F$1,E39)</f>
         <v>1E-3</v>
       </c>
       <c r="P39" t="s">
@@ -2728,21 +3004,21 @@
       <c r="E40" t="str">
         <v>fixed_leg.cashflows.[3].payment _date</v>
       </c>
-      <c r="F40" t="str">
-        <v>2023-09-03</v>
-      </c>
-      <c r="G40" t="str" cm="1">
-        <f t="array" ref="G40">_xll.ExLibris.Json.GetJsonValue($F$1,E40, EXLIBRIS_CONFIGURATION)</f>
-        <v>2023-09-03</v>
+      <c r="F40">
+        <v>45172</v>
+      </c>
+      <c r="G40" cm="1">
+        <f t="array" ref="G40">_xll.ExLibris.Json.GetJsonValue($F$1,E40)</f>
+        <v>45172</v>
       </c>
       <c r="P40" t="s">
         <v>50</v>
       </c>
-      <c r="Q40" t="s">
-        <v>97</v>
-      </c>
-      <c r="R40" t="s">
-        <v>97</v>
+      <c r="Q40">
+        <v>45172</v>
+      </c>
+      <c r="R40">
+        <v>45172</v>
       </c>
       <c r="AA40" t="b">
         <f t="shared" si="4"/>
@@ -2761,21 +3037,21 @@
       <c r="E41" t="str">
         <v>fixed_leg.cashflows.[3].start_date</v>
       </c>
-      <c r="F41" t="str">
-        <v>2023-03-07</v>
-      </c>
-      <c r="G41" t="str" cm="1">
-        <f t="array" ref="G41">_xll.ExLibris.Json.GetJsonValue($F$1,E41, EXLIBRIS_CONFIGURATION)</f>
-        <v>2023-03-07</v>
+      <c r="F41">
+        <v>44992</v>
+      </c>
+      <c r="G41" cm="1">
+        <f t="array" ref="G41">_xll.ExLibris.Json.GetJsonValue($F$1,E41)</f>
+        <v>44992</v>
       </c>
       <c r="P41" t="s">
         <v>51</v>
       </c>
-      <c r="Q41" t="s">
-        <v>96</v>
-      </c>
-      <c r="R41" t="s">
-        <v>96</v>
+      <c r="Q41">
+        <v>44992</v>
+      </c>
+      <c r="R41">
+        <v>44992</v>
       </c>
       <c r="AA41" t="b">
         <f t="shared" si="4"/>
@@ -2794,21 +3070,21 @@
       <c r="E42" t="str">
         <v>fixed_leg.cashflows.[3].end_date</v>
       </c>
-      <c r="F42" t="str">
-        <v>2023-09-03</v>
-      </c>
-      <c r="G42" t="str" cm="1">
-        <f t="array" ref="G42">_xll.ExLibris.Json.GetJsonValue($F$1,E42, EXLIBRIS_CONFIGURATION)</f>
-        <v>2023-09-03</v>
+      <c r="F42">
+        <v>45172</v>
+      </c>
+      <c r="G42" cm="1">
+        <f t="array" ref="G42">_xll.ExLibris.Json.GetJsonValue($F$1,E42)</f>
+        <v>45172</v>
       </c>
       <c r="P42" t="s">
         <v>52</v>
       </c>
-      <c r="Q42" t="s">
-        <v>97</v>
-      </c>
-      <c r="R42" t="s">
-        <v>97</v>
+      <c r="Q42">
+        <v>45172</v>
+      </c>
+      <c r="R42">
+        <v>45172</v>
       </c>
       <c r="AA42" t="b">
         <f t="shared" si="4"/>
@@ -2831,7 +3107,7 @@
         <v>ACT/360</v>
       </c>
       <c r="G43" t="str" cm="1">
-        <f t="array" ref="G43">_xll.ExLibris.Json.GetJsonValue($F$1,E43, EXLIBRIS_CONFIGURATION)</f>
+        <f t="array" ref="G43">_xll.ExLibris.Json.GetJsonValue($F$1,E43)</f>
         <v>ACT/360</v>
       </c>
       <c r="P43" t="s">
@@ -2864,7 +3140,7 @@
         <v>13000000</v>
       </c>
       <c r="G44" cm="1">
-        <f t="array" ref="G44">_xll.ExLibris.Json.GetJsonValue($F$1,E44, EXLIBRIS_CONFIGURATION)</f>
+        <f t="array" ref="G44">_xll.ExLibris.Json.GetJsonValue($F$1,E44)</f>
         <v>13000000</v>
       </c>
       <c r="P44" t="s">
@@ -2897,7 +3173,7 @@
         <v>1E-3</v>
       </c>
       <c r="G45" cm="1">
-        <f t="array" ref="G45">_xll.ExLibris.Json.GetJsonValue($F$1,E45, EXLIBRIS_CONFIGURATION)</f>
+        <f t="array" ref="G45">_xll.ExLibris.Json.GetJsonValue($F$1,E45)</f>
         <v>1E-3</v>
       </c>
       <c r="P45" t="s">
@@ -2926,21 +3202,21 @@
       <c r="E46" t="str">
         <v>fixed_leg.cashflows.[4].payment _date</v>
       </c>
-      <c r="F46" t="str">
-        <v>2024-03-01</v>
-      </c>
-      <c r="G46" t="str" cm="1">
-        <f t="array" ref="G46">_xll.ExLibris.Json.GetJsonValue($F$1,E46, EXLIBRIS_CONFIGURATION)</f>
-        <v>2024-03-01</v>
+      <c r="F46">
+        <v>45352</v>
+      </c>
+      <c r="G46" cm="1">
+        <f t="array" ref="G46">_xll.ExLibris.Json.GetJsonValue($F$1,E46)</f>
+        <v>45352</v>
       </c>
       <c r="P46" t="s">
         <v>56</v>
       </c>
-      <c r="Q46" t="s">
-        <v>98</v>
-      </c>
-      <c r="R46" t="s">
-        <v>98</v>
+      <c r="Q46">
+        <v>45352</v>
+      </c>
+      <c r="R46">
+        <v>45352</v>
       </c>
       <c r="AA46" t="b">
         <f t="shared" si="4"/>
@@ -2959,21 +3235,21 @@
       <c r="E47" t="str">
         <v>fixed_leg.cashflows.[4].start_date</v>
       </c>
-      <c r="F47" t="str">
-        <v>2023-09-03</v>
-      </c>
-      <c r="G47" t="str" cm="1">
-        <f t="array" ref="G47">_xll.ExLibris.Json.GetJsonValue($F$1,E47, EXLIBRIS_CONFIGURATION)</f>
-        <v>2023-09-03</v>
+      <c r="F47">
+        <v>45172</v>
+      </c>
+      <c r="G47" cm="1">
+        <f t="array" ref="G47">_xll.ExLibris.Json.GetJsonValue($F$1,E47)</f>
+        <v>45172</v>
       </c>
       <c r="P47" t="s">
         <v>57</v>
       </c>
-      <c r="Q47" t="s">
-        <v>97</v>
-      </c>
-      <c r="R47" t="s">
-        <v>97</v>
+      <c r="Q47">
+        <v>45172</v>
+      </c>
+      <c r="R47">
+        <v>45172</v>
       </c>
       <c r="AA47" t="b">
         <f t="shared" si="4"/>
@@ -2992,21 +3268,21 @@
       <c r="E48" t="str">
         <v>fixed_leg.cashflows.[4].end_date</v>
       </c>
-      <c r="F48" t="str">
-        <v>2024-03-01</v>
-      </c>
-      <c r="G48" t="str" cm="1">
-        <f t="array" ref="G48">_xll.ExLibris.Json.GetJsonValue($F$1,E48, EXLIBRIS_CONFIGURATION)</f>
-        <v>2024-03-01</v>
+      <c r="F48">
+        <v>45352</v>
+      </c>
+      <c r="G48" cm="1">
+        <f t="array" ref="G48">_xll.ExLibris.Json.GetJsonValue($F$1,E48)</f>
+        <v>45352</v>
       </c>
       <c r="P48" t="s">
         <v>58</v>
       </c>
-      <c r="Q48" t="s">
-        <v>98</v>
-      </c>
-      <c r="R48" t="s">
-        <v>98</v>
+      <c r="Q48">
+        <v>45352</v>
+      </c>
+      <c r="R48">
+        <v>45352</v>
       </c>
       <c r="AA48" t="b">
         <f t="shared" si="4"/>
@@ -3029,7 +3305,7 @@
         <v>ACT/360</v>
       </c>
       <c r="G49" t="str" cm="1">
-        <f t="array" ref="G49">_xll.ExLibris.Json.GetJsonValue($F$1,E49, EXLIBRIS_CONFIGURATION)</f>
+        <f t="array" ref="G49">_xll.ExLibris.Json.GetJsonValue($F$1,E49)</f>
         <v>ACT/360</v>
       </c>
       <c r="P49" t="s">
@@ -3062,7 +3338,7 @@
         <v>14000000</v>
       </c>
       <c r="G50" cm="1">
-        <f t="array" ref="G50">_xll.ExLibris.Json.GetJsonValue($F$1,E50, EXLIBRIS_CONFIGURATION)</f>
+        <f t="array" ref="G50">_xll.ExLibris.Json.GetJsonValue($F$1,E50)</f>
         <v>14000000</v>
       </c>
       <c r="P50" t="s">
@@ -3095,7 +3371,7 @@
         <v>1E-3</v>
       </c>
       <c r="G51" cm="1">
-        <f t="array" ref="G51">_xll.ExLibris.Json.GetJsonValue($F$1,E51, EXLIBRIS_CONFIGURATION)</f>
+        <f t="array" ref="G51">_xll.ExLibris.Json.GetJsonValue($F$1,E51)</f>
         <v>1E-3</v>
       </c>
       <c r="P51" t="s">
@@ -3124,21 +3400,21 @@
       <c r="E52" t="str">
         <v>fixed_leg.cashflows.[5].payment _date</v>
       </c>
-      <c r="F52" t="str">
-        <v>2024-08-28</v>
-      </c>
-      <c r="G52" t="str" cm="1">
-        <f t="array" ref="G52">_xll.ExLibris.Json.GetJsonValue($F$1,E52, EXLIBRIS_CONFIGURATION)</f>
-        <v>2024-08-28</v>
+      <c r="F52">
+        <v>45532</v>
+      </c>
+      <c r="G52" cm="1">
+        <f t="array" ref="G52">_xll.ExLibris.Json.GetJsonValue($F$1,E52)</f>
+        <v>45532</v>
       </c>
       <c r="P52" t="s">
         <v>62</v>
       </c>
-      <c r="Q52" t="s">
-        <v>99</v>
-      </c>
-      <c r="R52" t="s">
-        <v>99</v>
+      <c r="Q52">
+        <v>45532</v>
+      </c>
+      <c r="R52">
+        <v>45532</v>
       </c>
       <c r="AA52" t="b">
         <f t="shared" si="4"/>
@@ -3157,21 +3433,21 @@
       <c r="E53" t="str">
         <v>fixed_leg.cashflows.[5].start_date</v>
       </c>
-      <c r="F53" t="str">
-        <v>2024-03-01</v>
-      </c>
-      <c r="G53" t="str" cm="1">
-        <f t="array" ref="G53">_xll.ExLibris.Json.GetJsonValue($F$1,E53, EXLIBRIS_CONFIGURATION)</f>
-        <v>2024-03-01</v>
+      <c r="F53">
+        <v>45352</v>
+      </c>
+      <c r="G53" cm="1">
+        <f t="array" ref="G53">_xll.ExLibris.Json.GetJsonValue($F$1,E53)</f>
+        <v>45352</v>
       </c>
       <c r="P53" t="s">
         <v>63</v>
       </c>
-      <c r="Q53" t="s">
-        <v>98</v>
-      </c>
-      <c r="R53" t="s">
-        <v>98</v>
+      <c r="Q53">
+        <v>45352</v>
+      </c>
+      <c r="R53">
+        <v>45352</v>
       </c>
       <c r="AA53" t="b">
         <f t="shared" si="4"/>
@@ -3190,21 +3466,21 @@
       <c r="E54" t="str">
         <v>fixed_leg.cashflows.[5].end_date</v>
       </c>
-      <c r="F54" t="str">
-        <v>2024-08-28</v>
-      </c>
-      <c r="G54" t="str" cm="1">
-        <f t="array" ref="G54">_xll.ExLibris.Json.GetJsonValue($F$1,E54, EXLIBRIS_CONFIGURATION)</f>
-        <v>2024-08-28</v>
+      <c r="F54">
+        <v>45532</v>
+      </c>
+      <c r="G54" cm="1">
+        <f t="array" ref="G54">_xll.ExLibris.Json.GetJsonValue($F$1,E54)</f>
+        <v>45532</v>
       </c>
       <c r="P54" t="s">
         <v>64</v>
       </c>
-      <c r="Q54" t="s">
-        <v>99</v>
-      </c>
-      <c r="R54" t="s">
-        <v>99</v>
+      <c r="Q54">
+        <v>45532</v>
+      </c>
+      <c r="R54">
+        <v>45532</v>
       </c>
       <c r="AA54" t="b">
         <f t="shared" si="4"/>
@@ -3227,7 +3503,7 @@
         <v>ACT/360</v>
       </c>
       <c r="G55" t="str" cm="1">
-        <f t="array" ref="G55">_xll.ExLibris.Json.GetJsonValue($F$1,E55, EXLIBRIS_CONFIGURATION)</f>
+        <f t="array" ref="G55">_xll.ExLibris.Json.GetJsonValue($F$1,E55)</f>
         <v>ACT/360</v>
       </c>
       <c r="P55" t="s">
@@ -3260,7 +3536,7 @@
         <v>15000000</v>
       </c>
       <c r="G56" cm="1">
-        <f t="array" ref="G56">_xll.ExLibris.Json.GetJsonValue($F$1,E56, EXLIBRIS_CONFIGURATION)</f>
+        <f t="array" ref="G56">_xll.ExLibris.Json.GetJsonValue($F$1,E56)</f>
         <v>15000000</v>
       </c>
       <c r="P56" t="s">
@@ -3293,7 +3569,7 @@
         <v>1E-3</v>
       </c>
       <c r="G57" cm="1">
-        <f t="array" ref="G57">_xll.ExLibris.Json.GetJsonValue($F$1,E57, EXLIBRIS_CONFIGURATION)</f>
+        <f t="array" ref="G57">_xll.ExLibris.Json.GetJsonValue($F$1,E57)</f>
         <v>1E-3</v>
       </c>
       <c r="P57" t="s">
@@ -3326,6 +3602,2163 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{040ED89E-C884-4680-AA73-D86C4BBD7CCE}">
+  <dimension ref="B1:AJ57"/>
+  <sheetFormatPr defaultRowHeight="18.75" x14ac:dyDescent="0.4"/>
+  <cols>
+    <col min="1" max="1" width="2.25" customWidth="1"/>
+    <col min="4" max="4" width="2.125" customWidth="1"/>
+    <col min="5" max="5" width="38.125" bestFit="1" customWidth="1"/>
+    <col min="6" max="7" width="13.25" customWidth="1"/>
+    <col min="8" max="8" width="15.5" bestFit="1" customWidth="1"/>
+    <col min="9" max="11" width="13.25" customWidth="1"/>
+    <col min="15" max="15" width="7.375" customWidth="1"/>
+    <col min="16" max="16" width="13.5" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="17" customWidth="1"/>
+    <col min="19" max="19" width="10.125" bestFit="1" customWidth="1"/>
+    <col min="20" max="20" width="9.5" bestFit="1" customWidth="1"/>
+    <col min="21" max="21" width="15.5" bestFit="1" customWidth="1"/>
+    <col min="22" max="22" width="9.5" bestFit="1" customWidth="1"/>
+    <col min="23" max="23" width="9.875" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="2:25" x14ac:dyDescent="0.4">
+      <c r="E1" t="s">
+        <v>27</v>
+      </c>
+      <c r="F1" t="str" cm="1">
+        <f t="array" ref="F1">_xll.ExLibris.Json.CreateJsonObject(E3:F6, EXLIBRIS_CONFIGURATION)</f>
+        <v>JsonObject:503E7613-4E07-4006-B2A7-CB6401DF8B02</v>
+      </c>
+      <c r="K1" t="str">
+        <f>EXLIBRIS_CONFIGURATION</f>
+        <v>ExLibris.Core.ExLibrisConfiguration:78976E74-B484-403F-9AE1-F5D51D57D63F</v>
+      </c>
+    </row>
+    <row r="2" spans="2:25" x14ac:dyDescent="0.4">
+      <c r="B2" s="5" t="s">
+        <v>70</v>
+      </c>
+      <c r="C2" s="5"/>
+    </row>
+    <row r="3" spans="2:25" x14ac:dyDescent="0.4">
+      <c r="B3" s="6" t="s">
+        <v>71</v>
+      </c>
+      <c r="C3" s="6">
+        <f>COUNTIF(AA19:AC57,FALSE)</f>
+        <v>0</v>
+      </c>
+      <c r="E3" t="s">
+        <v>15</v>
+      </c>
+      <c r="F3" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="4" spans="2:25" x14ac:dyDescent="0.4">
+      <c r="B4" s="6" t="s">
+        <v>72</v>
+      </c>
+      <c r="C4" s="6">
+        <f>COUNTIF(AE20:AJ26,FALSE)</f>
+        <v>0</v>
+      </c>
+      <c r="E4" t="s">
+        <v>19</v>
+      </c>
+      <c r="F4" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="5" spans="2:25" x14ac:dyDescent="0.4">
+      <c r="B5" s="6" t="s">
+        <v>73</v>
+      </c>
+      <c r="C5" s="6" t="str">
+        <f>IF(M6=M7,"ok","ng")</f>
+        <v>ok</v>
+      </c>
+      <c r="E5" t="s">
+        <v>23</v>
+      </c>
+      <c r="F5" t="s">
+        <v>25</v>
+      </c>
+      <c r="L5" t="s">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="6" spans="2:25" x14ac:dyDescent="0.4">
+      <c r="B6" s="6" t="s">
+        <v>75</v>
+      </c>
+      <c r="C6" s="6">
+        <f>COUNTIF(AE29:AJ30,FALSE)</f>
+        <v>0</v>
+      </c>
+      <c r="E6" t="s">
+        <v>26</v>
+      </c>
+      <c r="F6" t="str" cm="1">
+        <f t="array" ref="F6">_xll.ExLibris.Json.CreateJsonArray(E8:J14, EXLIBRIS_CONFIGURATION)</f>
+        <v>JsonObject:16334072-DD2A-4369-8330-48716197076D</v>
+      </c>
+      <c r="L6" t="s">
+        <v>68</v>
+      </c>
+      <c r="M6" t="str" cm="1">
+        <f t="array" ref="M6">_xll.ExLibris.Json.ShowJsonText(F1)</f>
+        <v>{"trade_code":"money_00001","couter_party":"CP00001","fixed_leg":{"pay_or_recieve":"Receive","cashflows":[{"payment _date":"2022-03-12","start_date":"2021-09-13","end_date":"2022-03-12","day_count_type":"ACT/360","amout":10000000,"fixed_rate":0.001},{"payment _date":"2022-09-08","start_date":"2022-03-12","end_date":"2022-09-08","day_count_type":"ACT/360","amout":11000000,"fixed_rate":0.001},{"payment _date":"2023-03-07","start_date":"2022-09-08","end_date":"2023-03-07","day_count_type":"ACT/360","amout":12000000,"fixed_rate":0.001},{"payment _date":"2023-09-03","start_date":"2023-03-07","end_date":"2023-09-03","day_count_type":"ACT/360","amout":13000000,"fixed_rate":0.001},{"payment _date":"2024-03-01","start_date":"2023-09-03","end_date":"2024-03-01","day_count_type":"ACT/360","amout":14000000,"fixed_rate":0.001},{"payment _date":"2024-08-28","start_date":"2024-03-01","end_date":"2024-08-28","day_count_type":"ACT/360","amout":15000000,"fixed_rate":0.001}]}}</v>
+      </c>
+    </row>
+    <row r="7" spans="2:25" x14ac:dyDescent="0.4">
+      <c r="L7" t="s">
+        <v>74</v>
+      </c>
+      <c r="M7" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="8" spans="2:25" x14ac:dyDescent="0.4">
+      <c r="E8" t="s">
+        <v>1</v>
+      </c>
+      <c r="F8" t="s">
+        <v>3</v>
+      </c>
+      <c r="G8" t="s">
+        <v>5</v>
+      </c>
+      <c r="H8" t="s">
+        <v>7</v>
+      </c>
+      <c r="I8" t="s">
+        <v>11</v>
+      </c>
+      <c r="J8" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="9" spans="2:25" x14ac:dyDescent="0.4">
+      <c r="E9" s="1">
+        <f>G9</f>
+        <v>44632</v>
+      </c>
+      <c r="F9" s="1">
+        <v>44452</v>
+      </c>
+      <c r="G9" s="1">
+        <f>F9+180</f>
+        <v>44632</v>
+      </c>
+      <c r="H9" t="s">
+        <v>9</v>
+      </c>
+      <c r="I9" s="2">
+        <v>10000000</v>
+      </c>
+      <c r="J9" s="3">
+        <v>1E-3</v>
+      </c>
+    </row>
+    <row r="10" spans="2:25" x14ac:dyDescent="0.4">
+      <c r="E10" s="1">
+        <f>G10</f>
+        <v>44812</v>
+      </c>
+      <c r="F10" s="1">
+        <f>G9</f>
+        <v>44632</v>
+      </c>
+      <c r="G10" s="1">
+        <f>F10+180</f>
+        <v>44812</v>
+      </c>
+      <c r="H10" t="s">
+        <v>9</v>
+      </c>
+      <c r="I10" s="2">
+        <f>I9+1000000</f>
+        <v>11000000</v>
+      </c>
+      <c r="J10" s="3">
+        <v>1E-3</v>
+      </c>
+    </row>
+    <row r="11" spans="2:25" x14ac:dyDescent="0.4">
+      <c r="E11" s="1">
+        <f t="shared" ref="E11:E14" si="0">G11</f>
+        <v>44992</v>
+      </c>
+      <c r="F11" s="1">
+        <f t="shared" ref="F11:F14" si="1">G10</f>
+        <v>44812</v>
+      </c>
+      <c r="G11" s="1">
+        <f t="shared" ref="G11:G14" si="2">F11+180</f>
+        <v>44992</v>
+      </c>
+      <c r="H11" t="s">
+        <v>9</v>
+      </c>
+      <c r="I11" s="2">
+        <f t="shared" ref="I11:I14" si="3">I10+1000000</f>
+        <v>12000000</v>
+      </c>
+      <c r="J11" s="3">
+        <v>1E-3</v>
+      </c>
+    </row>
+    <row r="12" spans="2:25" x14ac:dyDescent="0.4">
+      <c r="E12" s="1">
+        <f t="shared" si="0"/>
+        <v>45172</v>
+      </c>
+      <c r="F12" s="1">
+        <f t="shared" si="1"/>
+        <v>44992</v>
+      </c>
+      <c r="G12" s="1">
+        <f t="shared" si="2"/>
+        <v>45172</v>
+      </c>
+      <c r="H12" t="s">
+        <v>9</v>
+      </c>
+      <c r="I12" s="2">
+        <f t="shared" si="3"/>
+        <v>13000000</v>
+      </c>
+      <c r="J12" s="3">
+        <v>1E-3</v>
+      </c>
+    </row>
+    <row r="13" spans="2:25" x14ac:dyDescent="0.4">
+      <c r="E13" s="1">
+        <f t="shared" si="0"/>
+        <v>45352</v>
+      </c>
+      <c r="F13" s="1">
+        <f t="shared" si="1"/>
+        <v>45172</v>
+      </c>
+      <c r="G13" s="1">
+        <f t="shared" si="2"/>
+        <v>45352</v>
+      </c>
+      <c r="H13" t="s">
+        <v>9</v>
+      </c>
+      <c r="I13" s="2">
+        <f t="shared" si="3"/>
+        <v>14000000</v>
+      </c>
+      <c r="J13" s="3">
+        <v>1E-3</v>
+      </c>
+    </row>
+    <row r="14" spans="2:25" x14ac:dyDescent="0.4">
+      <c r="E14" s="1">
+        <f t="shared" si="0"/>
+        <v>45532</v>
+      </c>
+      <c r="F14" s="1">
+        <f t="shared" si="1"/>
+        <v>45352</v>
+      </c>
+      <c r="G14" s="1">
+        <f t="shared" si="2"/>
+        <v>45532</v>
+      </c>
+      <c r="H14" t="s">
+        <v>9</v>
+      </c>
+      <c r="I14" s="2">
+        <f t="shared" si="3"/>
+        <v>15000000</v>
+      </c>
+      <c r="J14" s="3">
+        <v>1E-3</v>
+      </c>
+    </row>
+    <row r="16" spans="2:25" s="4" customFormat="1" ht="18" x14ac:dyDescent="0.4">
+      <c r="E16" s="4" t="s">
+        <v>68</v>
+      </c>
+      <c r="P16" s="4" t="s">
+        <v>69</v>
+      </c>
+      <c r="Y16" s="4" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="18" spans="5:36" x14ac:dyDescent="0.4">
+      <c r="E18" t="s">
+        <v>29</v>
+      </c>
+      <c r="I18" t="s">
+        <v>31</v>
+      </c>
+      <c r="P18" t="s">
+        <v>28</v>
+      </c>
+      <c r="T18" t="s">
+        <v>30</v>
+      </c>
+      <c r="AA18" t="s">
+        <v>28</v>
+      </c>
+      <c r="AE18" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="19" spans="5:36" x14ac:dyDescent="0.4">
+      <c r="E19" t="str" cm="1">
+        <f t="array" ref="E19:F57">_xll.ExLibris.Json.GetJsonKeyValues(F1, EXLIBRIS_CONFIGURATION)</f>
+        <v>trade_code</v>
+      </c>
+      <c r="F19" t="str">
+        <v>money_00001</v>
+      </c>
+      <c r="G19" t="str" cm="1">
+        <f t="array" ref="G19">_xll.ExLibris.Json.GetJsonValue($F$1,E19, EXLIBRIS_CONFIGURATION)</f>
+        <v>money_00001</v>
+      </c>
+      <c r="I19" t="str" cm="1">
+        <f t="array" ref="I19">_xll.ExLibris.Json.GetJsonValue(F1,E6, EXLIBRIS_CONFIGURATION)</f>
+        <v>JsonObject:CF6400C5-7AED-47FD-98B7-BD0CD6EEF736</v>
+      </c>
+      <c r="P19" t="s">
+        <v>14</v>
+      </c>
+      <c r="Q19" t="s">
+        <v>16</v>
+      </c>
+      <c r="R19" t="s">
+        <v>16</v>
+      </c>
+      <c r="AA19" t="b">
+        <f t="shared" ref="AA19:AA57" si="4">E19=P19</f>
+        <v>1</v>
+      </c>
+      <c r="AB19" t="b">
+        <f t="shared" ref="AB19:AC57" si="5">E19=P19</f>
+        <v>1</v>
+      </c>
+      <c r="AC19" t="b">
+        <f t="shared" si="5"/>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="20" spans="5:36" x14ac:dyDescent="0.4">
+      <c r="E20" t="str">
+        <v>couter_party</v>
+      </c>
+      <c r="F20" t="str">
+        <v>CP00001</v>
+      </c>
+      <c r="G20" t="str" cm="1">
+        <f t="array" ref="G20">_xll.ExLibris.Json.GetJsonValue($F$1,E20, EXLIBRIS_CONFIGURATION)</f>
+        <v>CP00001</v>
+      </c>
+      <c r="I20" t="str" cm="1">
+        <f t="array" ref="I20:N26">_xll.ExLibris.Json.GetJsonTable(I19, EXLIBRIS_CONFIGURATION)</f>
+        <v>payment _date</v>
+      </c>
+      <c r="J20" t="str">
+        <v>start_date</v>
+      </c>
+      <c r="K20" t="str">
+        <v>end_date</v>
+      </c>
+      <c r="L20" t="str">
+        <v>day_count_type</v>
+      </c>
+      <c r="M20" t="str">
+        <v>amout</v>
+      </c>
+      <c r="N20" t="str">
+        <v>fixed_rate</v>
+      </c>
+      <c r="P20" t="s">
+        <v>18</v>
+      </c>
+      <c r="Q20" t="s">
+        <v>20</v>
+      </c>
+      <c r="R20" t="s">
+        <v>20</v>
+      </c>
+      <c r="T20" t="s">
+        <v>0</v>
+      </c>
+      <c r="U20" t="s">
+        <v>2</v>
+      </c>
+      <c r="V20" t="s">
+        <v>4</v>
+      </c>
+      <c r="W20" t="s">
+        <v>6</v>
+      </c>
+      <c r="X20" t="s">
+        <v>10</v>
+      </c>
+      <c r="Y20" t="s">
+        <v>12</v>
+      </c>
+      <c r="AA20" t="b">
+        <f t="shared" si="4"/>
+        <v>1</v>
+      </c>
+      <c r="AB20" t="b">
+        <f t="shared" si="5"/>
+        <v>1</v>
+      </c>
+      <c r="AC20" t="b">
+        <f t="shared" si="5"/>
+        <v>1</v>
+      </c>
+      <c r="AE20" t="b">
+        <f t="shared" ref="AE20:AJ26" si="6">I20=T20</f>
+        <v>1</v>
+      </c>
+      <c r="AF20" t="b">
+        <f t="shared" si="6"/>
+        <v>1</v>
+      </c>
+      <c r="AG20" t="b">
+        <f t="shared" si="6"/>
+        <v>1</v>
+      </c>
+      <c r="AH20" t="b">
+        <f t="shared" si="6"/>
+        <v>1</v>
+      </c>
+      <c r="AI20" t="b">
+        <f t="shared" si="6"/>
+        <v>1</v>
+      </c>
+      <c r="AJ20" t="b">
+        <f t="shared" si="6"/>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="21" spans="5:36" x14ac:dyDescent="0.4">
+      <c r="E21" t="str">
+        <v>fixed_leg.pay_or_recieve</v>
+      </c>
+      <c r="F21" t="str">
+        <v>Receive</v>
+      </c>
+      <c r="G21" t="str" cm="1">
+        <f t="array" ref="G21">_xll.ExLibris.Json.GetJsonValue($F$1,E21, EXLIBRIS_CONFIGURATION)</f>
+        <v>Receive</v>
+      </c>
+      <c r="I21" t="str">
+        <v>2022-03-12</v>
+      </c>
+      <c r="J21" t="str">
+        <v>2021-09-13</v>
+      </c>
+      <c r="K21" t="str">
+        <v>2022-03-12</v>
+      </c>
+      <c r="L21" t="str">
+        <v>ACT/360</v>
+      </c>
+      <c r="M21">
+        <v>10000000</v>
+      </c>
+      <c r="N21">
+        <v>1E-3</v>
+      </c>
+      <c r="P21" t="s">
+        <v>22</v>
+      </c>
+      <c r="Q21" t="s">
+        <v>24</v>
+      </c>
+      <c r="R21" t="s">
+        <v>24</v>
+      </c>
+      <c r="T21" t="s">
+        <v>93</v>
+      </c>
+      <c r="U21" t="s">
+        <v>94</v>
+      </c>
+      <c r="V21" t="s">
+        <v>93</v>
+      </c>
+      <c r="W21" t="s">
+        <v>8</v>
+      </c>
+      <c r="X21">
+        <v>10000000</v>
+      </c>
+      <c r="Y21">
+        <v>1E-3</v>
+      </c>
+      <c r="AA21" t="b">
+        <f t="shared" si="4"/>
+        <v>1</v>
+      </c>
+      <c r="AB21" t="b">
+        <f t="shared" si="5"/>
+        <v>1</v>
+      </c>
+      <c r="AC21" t="b">
+        <f t="shared" si="5"/>
+        <v>1</v>
+      </c>
+      <c r="AE21" t="b">
+        <f t="shared" si="6"/>
+        <v>1</v>
+      </c>
+      <c r="AF21" t="b">
+        <f t="shared" si="6"/>
+        <v>1</v>
+      </c>
+      <c r="AG21" t="b">
+        <f t="shared" si="6"/>
+        <v>1</v>
+      </c>
+      <c r="AH21" t="b">
+        <f t="shared" si="6"/>
+        <v>1</v>
+      </c>
+      <c r="AI21" t="b">
+        <f t="shared" si="6"/>
+        <v>1</v>
+      </c>
+      <c r="AJ21" t="b">
+        <f t="shared" si="6"/>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="22" spans="5:36" x14ac:dyDescent="0.4">
+      <c r="E22" t="str">
+        <v>fixed_leg.cashflows.[0].payment _date</v>
+      </c>
+      <c r="F22" t="str">
+        <v>2022-03-12</v>
+      </c>
+      <c r="G22" s="1" t="str" cm="1">
+        <f t="array" ref="G22">_xll.ExLibris.Json.GetJsonValue($F$1,E22, EXLIBRIS_CONFIGURATION)</f>
+        <v>2022-03-12</v>
+      </c>
+      <c r="I22" t="str">
+        <v>2022-09-08</v>
+      </c>
+      <c r="J22" t="str">
+        <v>2022-03-12</v>
+      </c>
+      <c r="K22" t="str">
+        <v>2022-09-08</v>
+      </c>
+      <c r="L22" t="str">
+        <v>ACT/360</v>
+      </c>
+      <c r="M22">
+        <v>11000000</v>
+      </c>
+      <c r="N22">
+        <v>1E-3</v>
+      </c>
+      <c r="P22" t="s">
+        <v>32</v>
+      </c>
+      <c r="Q22" t="s">
+        <v>93</v>
+      </c>
+      <c r="R22" t="s">
+        <v>93</v>
+      </c>
+      <c r="T22" t="s">
+        <v>95</v>
+      </c>
+      <c r="U22" t="s">
+        <v>93</v>
+      </c>
+      <c r="V22" t="s">
+        <v>95</v>
+      </c>
+      <c r="W22" t="s">
+        <v>8</v>
+      </c>
+      <c r="X22">
+        <v>11000000</v>
+      </c>
+      <c r="Y22">
+        <v>1E-3</v>
+      </c>
+      <c r="AA22" t="b">
+        <f t="shared" si="4"/>
+        <v>1</v>
+      </c>
+      <c r="AB22" t="b">
+        <f t="shared" si="5"/>
+        <v>1</v>
+      </c>
+      <c r="AC22" t="b">
+        <f t="shared" si="5"/>
+        <v>1</v>
+      </c>
+      <c r="AE22" t="b">
+        <f t="shared" si="6"/>
+        <v>1</v>
+      </c>
+      <c r="AF22" t="b">
+        <f t="shared" si="6"/>
+        <v>1</v>
+      </c>
+      <c r="AG22" t="b">
+        <f t="shared" si="6"/>
+        <v>1</v>
+      </c>
+      <c r="AH22" t="b">
+        <f t="shared" si="6"/>
+        <v>1</v>
+      </c>
+      <c r="AI22" t="b">
+        <f t="shared" si="6"/>
+        <v>1</v>
+      </c>
+      <c r="AJ22" t="b">
+        <f t="shared" si="6"/>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="23" spans="5:36" x14ac:dyDescent="0.4">
+      <c r="E23" t="str">
+        <v>fixed_leg.cashflows.[0].start_date</v>
+      </c>
+      <c r="F23" t="str">
+        <v>2021-09-13</v>
+      </c>
+      <c r="G23" t="str" cm="1">
+        <f t="array" ref="G23">_xll.ExLibris.Json.GetJsonValue($F$1,E23, EXLIBRIS_CONFIGURATION)</f>
+        <v>2021-09-13</v>
+      </c>
+      <c r="I23" t="str">
+        <v>2023-03-07</v>
+      </c>
+      <c r="J23" t="str">
+        <v>2022-09-08</v>
+      </c>
+      <c r="K23" t="str">
+        <v>2023-03-07</v>
+      </c>
+      <c r="L23" t="str">
+        <v>ACT/360</v>
+      </c>
+      <c r="M23">
+        <v>12000000</v>
+      </c>
+      <c r="N23">
+        <v>1E-3</v>
+      </c>
+      <c r="P23" t="s">
+        <v>33</v>
+      </c>
+      <c r="Q23" t="s">
+        <v>94</v>
+      </c>
+      <c r="R23" t="s">
+        <v>94</v>
+      </c>
+      <c r="T23" t="s">
+        <v>96</v>
+      </c>
+      <c r="U23" t="s">
+        <v>95</v>
+      </c>
+      <c r="V23" t="s">
+        <v>96</v>
+      </c>
+      <c r="W23" t="s">
+        <v>8</v>
+      </c>
+      <c r="X23">
+        <v>12000000</v>
+      </c>
+      <c r="Y23">
+        <v>1E-3</v>
+      </c>
+      <c r="AA23" t="b">
+        <f t="shared" si="4"/>
+        <v>1</v>
+      </c>
+      <c r="AB23" t="b">
+        <f t="shared" si="5"/>
+        <v>1</v>
+      </c>
+      <c r="AC23" t="b">
+        <f t="shared" si="5"/>
+        <v>1</v>
+      </c>
+      <c r="AE23" t="b">
+        <f t="shared" si="6"/>
+        <v>1</v>
+      </c>
+      <c r="AF23" t="b">
+        <f t="shared" si="6"/>
+        <v>1</v>
+      </c>
+      <c r="AG23" t="b">
+        <f t="shared" si="6"/>
+        <v>1</v>
+      </c>
+      <c r="AH23" t="b">
+        <f t="shared" si="6"/>
+        <v>1</v>
+      </c>
+      <c r="AI23" t="b">
+        <f t="shared" si="6"/>
+        <v>1</v>
+      </c>
+      <c r="AJ23" t="b">
+        <f t="shared" si="6"/>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="24" spans="5:36" x14ac:dyDescent="0.4">
+      <c r="E24" t="str">
+        <v>fixed_leg.cashflows.[0].end_date</v>
+      </c>
+      <c r="F24" t="str">
+        <v>2022-03-12</v>
+      </c>
+      <c r="G24" t="str" cm="1">
+        <f t="array" ref="G24">_xll.ExLibris.Json.GetJsonValue($F$1,E24, EXLIBRIS_CONFIGURATION)</f>
+        <v>2022-03-12</v>
+      </c>
+      <c r="I24" t="str">
+        <v>2023-09-03</v>
+      </c>
+      <c r="J24" t="str">
+        <v>2023-03-07</v>
+      </c>
+      <c r="K24" t="str">
+        <v>2023-09-03</v>
+      </c>
+      <c r="L24" t="str">
+        <v>ACT/360</v>
+      </c>
+      <c r="M24">
+        <v>13000000</v>
+      </c>
+      <c r="N24">
+        <v>1E-3</v>
+      </c>
+      <c r="P24" t="s">
+        <v>34</v>
+      </c>
+      <c r="Q24" t="s">
+        <v>93</v>
+      </c>
+      <c r="R24" t="s">
+        <v>93</v>
+      </c>
+      <c r="T24" t="s">
+        <v>97</v>
+      </c>
+      <c r="U24" t="s">
+        <v>96</v>
+      </c>
+      <c r="V24" t="s">
+        <v>97</v>
+      </c>
+      <c r="W24" t="s">
+        <v>8</v>
+      </c>
+      <c r="X24">
+        <v>13000000</v>
+      </c>
+      <c r="Y24">
+        <v>1E-3</v>
+      </c>
+      <c r="AA24" t="b">
+        <f t="shared" si="4"/>
+        <v>1</v>
+      </c>
+      <c r="AB24" t="b">
+        <f t="shared" si="5"/>
+        <v>1</v>
+      </c>
+      <c r="AC24" t="b">
+        <f t="shared" si="5"/>
+        <v>1</v>
+      </c>
+      <c r="AE24" t="b">
+        <f t="shared" si="6"/>
+        <v>1</v>
+      </c>
+      <c r="AF24" t="b">
+        <f t="shared" si="6"/>
+        <v>1</v>
+      </c>
+      <c r="AG24" t="b">
+        <f t="shared" si="6"/>
+        <v>1</v>
+      </c>
+      <c r="AH24" t="b">
+        <f t="shared" si="6"/>
+        <v>1</v>
+      </c>
+      <c r="AI24" t="b">
+        <f t="shared" si="6"/>
+        <v>1</v>
+      </c>
+      <c r="AJ24" t="b">
+        <f t="shared" si="6"/>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="25" spans="5:36" x14ac:dyDescent="0.4">
+      <c r="E25" t="str">
+        <v>fixed_leg.cashflows.[0].day_count_type</v>
+      </c>
+      <c r="F25" t="str">
+        <v>ACT/360</v>
+      </c>
+      <c r="G25" t="str" cm="1">
+        <f t="array" ref="G25">_xll.ExLibris.Json.GetJsonValue($F$1,E25, EXLIBRIS_CONFIGURATION)</f>
+        <v>ACT/360</v>
+      </c>
+      <c r="I25" t="str">
+        <v>2024-03-01</v>
+      </c>
+      <c r="J25" t="str">
+        <v>2023-09-03</v>
+      </c>
+      <c r="K25" t="str">
+        <v>2024-03-01</v>
+      </c>
+      <c r="L25" t="str">
+        <v>ACT/360</v>
+      </c>
+      <c r="M25">
+        <v>14000000</v>
+      </c>
+      <c r="N25">
+        <v>1E-3</v>
+      </c>
+      <c r="P25" t="s">
+        <v>35</v>
+      </c>
+      <c r="Q25" t="s">
+        <v>8</v>
+      </c>
+      <c r="R25" t="s">
+        <v>8</v>
+      </c>
+      <c r="T25" t="s">
+        <v>98</v>
+      </c>
+      <c r="U25" t="s">
+        <v>97</v>
+      </c>
+      <c r="V25" t="s">
+        <v>98</v>
+      </c>
+      <c r="W25" t="s">
+        <v>8</v>
+      </c>
+      <c r="X25">
+        <v>14000000</v>
+      </c>
+      <c r="Y25">
+        <v>1E-3</v>
+      </c>
+      <c r="AA25" t="b">
+        <f t="shared" si="4"/>
+        <v>1</v>
+      </c>
+      <c r="AB25" t="b">
+        <f t="shared" si="5"/>
+        <v>1</v>
+      </c>
+      <c r="AC25" t="b">
+        <f t="shared" si="5"/>
+        <v>1</v>
+      </c>
+      <c r="AE25" t="b">
+        <f t="shared" si="6"/>
+        <v>1</v>
+      </c>
+      <c r="AF25" t="b">
+        <f t="shared" si="6"/>
+        <v>1</v>
+      </c>
+      <c r="AG25" t="b">
+        <f t="shared" si="6"/>
+        <v>1</v>
+      </c>
+      <c r="AH25" t="b">
+        <f t="shared" si="6"/>
+        <v>1</v>
+      </c>
+      <c r="AI25" t="b">
+        <f t="shared" si="6"/>
+        <v>1</v>
+      </c>
+      <c r="AJ25" t="b">
+        <f t="shared" si="6"/>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="26" spans="5:36" x14ac:dyDescent="0.4">
+      <c r="E26" t="str">
+        <v>fixed_leg.cashflows.[0].amout</v>
+      </c>
+      <c r="F26">
+        <v>10000000</v>
+      </c>
+      <c r="G26" cm="1">
+        <f t="array" ref="G26">_xll.ExLibris.Json.GetJsonValue($F$1,E26, EXLIBRIS_CONFIGURATION)</f>
+        <v>10000000</v>
+      </c>
+      <c r="I26" t="str">
+        <v>2024-08-28</v>
+      </c>
+      <c r="J26" t="str">
+        <v>2024-03-01</v>
+      </c>
+      <c r="K26" t="str">
+        <v>2024-08-28</v>
+      </c>
+      <c r="L26" t="str">
+        <v>ACT/360</v>
+      </c>
+      <c r="M26">
+        <v>15000000</v>
+      </c>
+      <c r="N26">
+        <v>1E-3</v>
+      </c>
+      <c r="P26" t="s">
+        <v>36</v>
+      </c>
+      <c r="Q26">
+        <v>10000000</v>
+      </c>
+      <c r="R26">
+        <v>10000000</v>
+      </c>
+      <c r="T26" t="s">
+        <v>99</v>
+      </c>
+      <c r="U26" t="s">
+        <v>98</v>
+      </c>
+      <c r="V26" t="s">
+        <v>99</v>
+      </c>
+      <c r="W26" t="s">
+        <v>8</v>
+      </c>
+      <c r="X26">
+        <v>15000000</v>
+      </c>
+      <c r="Y26">
+        <v>1E-3</v>
+      </c>
+      <c r="AA26" t="b">
+        <f t="shared" si="4"/>
+        <v>1</v>
+      </c>
+      <c r="AB26" t="b">
+        <f t="shared" si="5"/>
+        <v>1</v>
+      </c>
+      <c r="AC26" t="b">
+        <f t="shared" si="5"/>
+        <v>1</v>
+      </c>
+      <c r="AE26" t="b">
+        <f t="shared" si="6"/>
+        <v>1</v>
+      </c>
+      <c r="AF26" t="b">
+        <f t="shared" si="6"/>
+        <v>1</v>
+      </c>
+      <c r="AG26" t="b">
+        <f t="shared" si="6"/>
+        <v>1</v>
+      </c>
+      <c r="AH26" t="b">
+        <f t="shared" si="6"/>
+        <v>1</v>
+      </c>
+      <c r="AI26" t="b">
+        <f t="shared" si="6"/>
+        <v>1</v>
+      </c>
+      <c r="AJ26" t="b">
+        <f t="shared" si="6"/>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="27" spans="5:36" x14ac:dyDescent="0.4">
+      <c r="E27" t="str">
+        <v>fixed_leg.cashflows.[0].fixed_rate</v>
+      </c>
+      <c r="F27">
+        <v>1E-3</v>
+      </c>
+      <c r="G27" cm="1">
+        <f t="array" ref="G27">_xll.ExLibris.Json.GetJsonValue($F$1,E27, EXLIBRIS_CONFIGURATION)</f>
+        <v>1E-3</v>
+      </c>
+      <c r="P27" t="s">
+        <v>37</v>
+      </c>
+      <c r="Q27">
+        <v>1E-3</v>
+      </c>
+      <c r="R27">
+        <v>1E-3</v>
+      </c>
+      <c r="AA27" t="b">
+        <f t="shared" si="4"/>
+        <v>1</v>
+      </c>
+      <c r="AB27" t="b">
+        <f t="shared" si="5"/>
+        <v>1</v>
+      </c>
+      <c r="AC27" t="b">
+        <f t="shared" si="5"/>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="28" spans="5:36" x14ac:dyDescent="0.4">
+      <c r="E28" t="str">
+        <v>fixed_leg.cashflows.[1].payment _date</v>
+      </c>
+      <c r="F28" t="str">
+        <v>2022-09-08</v>
+      </c>
+      <c r="G28" t="str" cm="1">
+        <f t="array" ref="G28">_xll.ExLibris.Json.GetJsonValue($F$1,E28, EXLIBRIS_CONFIGURATION)</f>
+        <v>2022-09-08</v>
+      </c>
+      <c r="I28" t="str" cm="1">
+        <f t="array" ref="I28">_xll.ExLibris.Json.GetJsonValue(I19,"[2]", EXLIBRIS_CONFIGURATION)</f>
+        <v>JsonObject:391EFAB2-D899-4E8E-B0E6-36E35FB16A7E</v>
+      </c>
+      <c r="P28" t="s">
+        <v>38</v>
+      </c>
+      <c r="Q28" t="s">
+        <v>95</v>
+      </c>
+      <c r="R28" t="s">
+        <v>95</v>
+      </c>
+      <c r="AA28" t="b">
+        <f t="shared" si="4"/>
+        <v>1</v>
+      </c>
+      <c r="AB28" t="b">
+        <f t="shared" si="5"/>
+        <v>1</v>
+      </c>
+      <c r="AC28" t="b">
+        <f t="shared" si="5"/>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="29" spans="5:36" x14ac:dyDescent="0.4">
+      <c r="E29" t="str">
+        <v>fixed_leg.cashflows.[1].start_date</v>
+      </c>
+      <c r="F29" t="str">
+        <v>2022-03-12</v>
+      </c>
+      <c r="G29" t="str" cm="1">
+        <f t="array" ref="G29">_xll.ExLibris.Json.GetJsonValue($F$1,E29, EXLIBRIS_CONFIGURATION)</f>
+        <v>2022-03-12</v>
+      </c>
+      <c r="I29" t="str" cm="1">
+        <f t="array" ref="I29:N30">_xll.ExLibris.Json.GetJsonTable(I28, EXLIBRIS_CONFIGURATION)</f>
+        <v>payment _date</v>
+      </c>
+      <c r="J29" t="str">
+        <v>start_date</v>
+      </c>
+      <c r="K29" t="str">
+        <v>end_date</v>
+      </c>
+      <c r="L29" t="str">
+        <v>day_count_type</v>
+      </c>
+      <c r="M29" t="str">
+        <v>amout</v>
+      </c>
+      <c r="N29" t="str">
+        <v>fixed_rate</v>
+      </c>
+      <c r="P29" t="s">
+        <v>39</v>
+      </c>
+      <c r="Q29" t="s">
+        <v>93</v>
+      </c>
+      <c r="R29" t="s">
+        <v>93</v>
+      </c>
+      <c r="T29" t="s">
+        <v>0</v>
+      </c>
+      <c r="U29" t="s">
+        <v>2</v>
+      </c>
+      <c r="V29" t="s">
+        <v>4</v>
+      </c>
+      <c r="W29" t="s">
+        <v>6</v>
+      </c>
+      <c r="X29" t="s">
+        <v>10</v>
+      </c>
+      <c r="Y29" t="s">
+        <v>12</v>
+      </c>
+      <c r="AA29" t="b">
+        <f t="shared" si="4"/>
+        <v>1</v>
+      </c>
+      <c r="AB29" t="b">
+        <f t="shared" si="5"/>
+        <v>1</v>
+      </c>
+      <c r="AC29" t="b">
+        <f t="shared" si="5"/>
+        <v>1</v>
+      </c>
+      <c r="AE29" t="b">
+        <f t="shared" ref="AE29:AJ30" si="7">I29=T29</f>
+        <v>1</v>
+      </c>
+      <c r="AF29" t="b">
+        <f t="shared" si="7"/>
+        <v>1</v>
+      </c>
+      <c r="AG29" t="b">
+        <f t="shared" si="7"/>
+        <v>1</v>
+      </c>
+      <c r="AH29" t="b">
+        <f t="shared" si="7"/>
+        <v>1</v>
+      </c>
+      <c r="AI29" t="b">
+        <f t="shared" si="7"/>
+        <v>1</v>
+      </c>
+      <c r="AJ29" t="b">
+        <f t="shared" si="7"/>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="30" spans="5:36" x14ac:dyDescent="0.4">
+      <c r="E30" t="str">
+        <v>fixed_leg.cashflows.[1].end_date</v>
+      </c>
+      <c r="F30" t="str">
+        <v>2022-09-08</v>
+      </c>
+      <c r="G30" t="str" cm="1">
+        <f t="array" ref="G30">_xll.ExLibris.Json.GetJsonValue($F$1,E30, EXLIBRIS_CONFIGURATION)</f>
+        <v>2022-09-08</v>
+      </c>
+      <c r="I30" t="str">
+        <v>2023-03-07</v>
+      </c>
+      <c r="J30" t="str">
+        <v>2022-09-08</v>
+      </c>
+      <c r="K30" t="str">
+        <v>2023-03-07</v>
+      </c>
+      <c r="L30" t="str">
+        <v>ACT/360</v>
+      </c>
+      <c r="M30">
+        <v>12000000</v>
+      </c>
+      <c r="N30">
+        <v>1E-3</v>
+      </c>
+      <c r="P30" t="s">
+        <v>40</v>
+      </c>
+      <c r="Q30" t="s">
+        <v>95</v>
+      </c>
+      <c r="R30" t="s">
+        <v>95</v>
+      </c>
+      <c r="T30" t="s">
+        <v>96</v>
+      </c>
+      <c r="U30" t="s">
+        <v>95</v>
+      </c>
+      <c r="V30" t="s">
+        <v>96</v>
+      </c>
+      <c r="W30" t="s">
+        <v>8</v>
+      </c>
+      <c r="X30">
+        <v>12000000</v>
+      </c>
+      <c r="Y30">
+        <v>1E-3</v>
+      </c>
+      <c r="AA30" t="b">
+        <f t="shared" si="4"/>
+        <v>1</v>
+      </c>
+      <c r="AB30" t="b">
+        <f t="shared" si="5"/>
+        <v>1</v>
+      </c>
+      <c r="AC30" t="b">
+        <f t="shared" si="5"/>
+        <v>1</v>
+      </c>
+      <c r="AE30" t="b">
+        <f t="shared" si="7"/>
+        <v>1</v>
+      </c>
+      <c r="AF30" t="b">
+        <f t="shared" si="7"/>
+        <v>1</v>
+      </c>
+      <c r="AG30" t="b">
+        <f t="shared" si="7"/>
+        <v>1</v>
+      </c>
+      <c r="AH30" t="b">
+        <f t="shared" si="7"/>
+        <v>1</v>
+      </c>
+      <c r="AI30" t="b">
+        <f t="shared" si="7"/>
+        <v>1</v>
+      </c>
+      <c r="AJ30" t="b">
+        <f t="shared" si="7"/>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="31" spans="5:36" x14ac:dyDescent="0.4">
+      <c r="E31" t="str">
+        <v>fixed_leg.cashflows.[1].day_count_type</v>
+      </c>
+      <c r="F31" t="str">
+        <v>ACT/360</v>
+      </c>
+      <c r="G31" t="str" cm="1">
+        <f t="array" ref="G31">_xll.ExLibris.Json.GetJsonValue($F$1,E31, EXLIBRIS_CONFIGURATION)</f>
+        <v>ACT/360</v>
+      </c>
+      <c r="P31" t="s">
+        <v>41</v>
+      </c>
+      <c r="Q31" t="s">
+        <v>8</v>
+      </c>
+      <c r="R31" t="s">
+        <v>8</v>
+      </c>
+      <c r="AA31" t="b">
+        <f t="shared" si="4"/>
+        <v>1</v>
+      </c>
+      <c r="AB31" t="b">
+        <f t="shared" si="5"/>
+        <v>1</v>
+      </c>
+      <c r="AC31" t="b">
+        <f t="shared" si="5"/>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="32" spans="5:36" x14ac:dyDescent="0.4">
+      <c r="E32" t="str">
+        <v>fixed_leg.cashflows.[1].amout</v>
+      </c>
+      <c r="F32">
+        <v>11000000</v>
+      </c>
+      <c r="G32" cm="1">
+        <f t="array" ref="G32">_xll.ExLibris.Json.GetJsonValue($F$1,E32, EXLIBRIS_CONFIGURATION)</f>
+        <v>11000000</v>
+      </c>
+      <c r="P32" t="s">
+        <v>42</v>
+      </c>
+      <c r="Q32">
+        <v>11000000</v>
+      </c>
+      <c r="R32">
+        <v>11000000</v>
+      </c>
+      <c r="AA32" t="b">
+        <f t="shared" si="4"/>
+        <v>1</v>
+      </c>
+      <c r="AB32" t="b">
+        <f t="shared" si="5"/>
+        <v>1</v>
+      </c>
+      <c r="AC32" t="b">
+        <f t="shared" si="5"/>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="33" spans="5:29" x14ac:dyDescent="0.4">
+      <c r="E33" t="str">
+        <v>fixed_leg.cashflows.[1].fixed_rate</v>
+      </c>
+      <c r="F33">
+        <v>1E-3</v>
+      </c>
+      <c r="G33" cm="1">
+        <f t="array" ref="G33">_xll.ExLibris.Json.GetJsonValue($F$1,E33, EXLIBRIS_CONFIGURATION)</f>
+        <v>1E-3</v>
+      </c>
+      <c r="P33" t="s">
+        <v>43</v>
+      </c>
+      <c r="Q33">
+        <v>1E-3</v>
+      </c>
+      <c r="R33">
+        <v>1E-3</v>
+      </c>
+      <c r="AA33" t="b">
+        <f t="shared" si="4"/>
+        <v>1</v>
+      </c>
+      <c r="AB33" t="b">
+        <f t="shared" si="5"/>
+        <v>1</v>
+      </c>
+      <c r="AC33" t="b">
+        <f t="shared" si="5"/>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="34" spans="5:29" x14ac:dyDescent="0.4">
+      <c r="E34" t="str">
+        <v>fixed_leg.cashflows.[2].payment _date</v>
+      </c>
+      <c r="F34" t="str">
+        <v>2023-03-07</v>
+      </c>
+      <c r="G34" t="str" cm="1">
+        <f t="array" ref="G34">_xll.ExLibris.Json.GetJsonValue($F$1,E34, EXLIBRIS_CONFIGURATION)</f>
+        <v>2023-03-07</v>
+      </c>
+      <c r="P34" t="s">
+        <v>44</v>
+      </c>
+      <c r="Q34" t="s">
+        <v>96</v>
+      </c>
+      <c r="R34" t="s">
+        <v>96</v>
+      </c>
+      <c r="AA34" t="b">
+        <f t="shared" si="4"/>
+        <v>1</v>
+      </c>
+      <c r="AB34" t="b">
+        <f t="shared" si="5"/>
+        <v>1</v>
+      </c>
+      <c r="AC34" t="b">
+        <f t="shared" si="5"/>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="35" spans="5:29" x14ac:dyDescent="0.4">
+      <c r="E35" t="str">
+        <v>fixed_leg.cashflows.[2].start_date</v>
+      </c>
+      <c r="F35" t="str">
+        <v>2022-09-08</v>
+      </c>
+      <c r="G35" t="str" cm="1">
+        <f t="array" ref="G35">_xll.ExLibris.Json.GetJsonValue($F$1,E35, EXLIBRIS_CONFIGURATION)</f>
+        <v>2022-09-08</v>
+      </c>
+      <c r="P35" t="s">
+        <v>45</v>
+      </c>
+      <c r="Q35" t="s">
+        <v>95</v>
+      </c>
+      <c r="R35" t="s">
+        <v>95</v>
+      </c>
+      <c r="AA35" t="b">
+        <f t="shared" si="4"/>
+        <v>1</v>
+      </c>
+      <c r="AB35" t="b">
+        <f t="shared" si="5"/>
+        <v>1</v>
+      </c>
+      <c r="AC35" t="b">
+        <f t="shared" si="5"/>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="36" spans="5:29" x14ac:dyDescent="0.4">
+      <c r="E36" t="str">
+        <v>fixed_leg.cashflows.[2].end_date</v>
+      </c>
+      <c r="F36" t="str">
+        <v>2023-03-07</v>
+      </c>
+      <c r="G36" t="str" cm="1">
+        <f t="array" ref="G36">_xll.ExLibris.Json.GetJsonValue($F$1,E36, EXLIBRIS_CONFIGURATION)</f>
+        <v>2023-03-07</v>
+      </c>
+      <c r="P36" t="s">
+        <v>46</v>
+      </c>
+      <c r="Q36" t="s">
+        <v>96</v>
+      </c>
+      <c r="R36" t="s">
+        <v>96</v>
+      </c>
+      <c r="AA36" t="b">
+        <f t="shared" si="4"/>
+        <v>1</v>
+      </c>
+      <c r="AB36" t="b">
+        <f t="shared" si="5"/>
+        <v>1</v>
+      </c>
+      <c r="AC36" t="b">
+        <f t="shared" si="5"/>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="37" spans="5:29" x14ac:dyDescent="0.4">
+      <c r="E37" t="str">
+        <v>fixed_leg.cashflows.[2].day_count_type</v>
+      </c>
+      <c r="F37" t="str">
+        <v>ACT/360</v>
+      </c>
+      <c r="G37" t="str" cm="1">
+        <f t="array" ref="G37">_xll.ExLibris.Json.GetJsonValue($F$1,E37, EXLIBRIS_CONFIGURATION)</f>
+        <v>ACT/360</v>
+      </c>
+      <c r="P37" t="s">
+        <v>47</v>
+      </c>
+      <c r="Q37" t="s">
+        <v>8</v>
+      </c>
+      <c r="R37" t="s">
+        <v>8</v>
+      </c>
+      <c r="AA37" t="b">
+        <f t="shared" si="4"/>
+        <v>1</v>
+      </c>
+      <c r="AB37" t="b">
+        <f t="shared" si="5"/>
+        <v>1</v>
+      </c>
+      <c r="AC37" t="b">
+        <f t="shared" si="5"/>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="38" spans="5:29" x14ac:dyDescent="0.4">
+      <c r="E38" t="str">
+        <v>fixed_leg.cashflows.[2].amout</v>
+      </c>
+      <c r="F38">
+        <v>12000000</v>
+      </c>
+      <c r="G38" cm="1">
+        <f t="array" ref="G38">_xll.ExLibris.Json.GetJsonValue($F$1,E38, EXLIBRIS_CONFIGURATION)</f>
+        <v>12000000</v>
+      </c>
+      <c r="P38" t="s">
+        <v>48</v>
+      </c>
+      <c r="Q38">
+        <v>12000000</v>
+      </c>
+      <c r="R38">
+        <v>12000000</v>
+      </c>
+      <c r="AA38" t="b">
+        <f t="shared" si="4"/>
+        <v>1</v>
+      </c>
+      <c r="AB38" t="b">
+        <f t="shared" si="5"/>
+        <v>1</v>
+      </c>
+      <c r="AC38" t="b">
+        <f t="shared" si="5"/>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="39" spans="5:29" x14ac:dyDescent="0.4">
+      <c r="E39" t="str">
+        <v>fixed_leg.cashflows.[2].fixed_rate</v>
+      </c>
+      <c r="F39">
+        <v>1E-3</v>
+      </c>
+      <c r="G39" cm="1">
+        <f t="array" ref="G39">_xll.ExLibris.Json.GetJsonValue($F$1,E39, EXLIBRIS_CONFIGURATION)</f>
+        <v>1E-3</v>
+      </c>
+      <c r="P39" t="s">
+        <v>49</v>
+      </c>
+      <c r="Q39">
+        <v>1E-3</v>
+      </c>
+      <c r="R39">
+        <v>1E-3</v>
+      </c>
+      <c r="AA39" t="b">
+        <f t="shared" si="4"/>
+        <v>1</v>
+      </c>
+      <c r="AB39" t="b">
+        <f t="shared" si="5"/>
+        <v>1</v>
+      </c>
+      <c r="AC39" t="b">
+        <f t="shared" si="5"/>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="40" spans="5:29" x14ac:dyDescent="0.4">
+      <c r="E40" t="str">
+        <v>fixed_leg.cashflows.[3].payment _date</v>
+      </c>
+      <c r="F40" t="str">
+        <v>2023-09-03</v>
+      </c>
+      <c r="G40" t="str" cm="1">
+        <f t="array" ref="G40">_xll.ExLibris.Json.GetJsonValue($F$1,E40, EXLIBRIS_CONFIGURATION)</f>
+        <v>2023-09-03</v>
+      </c>
+      <c r="P40" t="s">
+        <v>50</v>
+      </c>
+      <c r="Q40" t="s">
+        <v>97</v>
+      </c>
+      <c r="R40" t="s">
+        <v>97</v>
+      </c>
+      <c r="AA40" t="b">
+        <f t="shared" si="4"/>
+        <v>1</v>
+      </c>
+      <c r="AB40" t="b">
+        <f t="shared" si="5"/>
+        <v>1</v>
+      </c>
+      <c r="AC40" t="b">
+        <f t="shared" si="5"/>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="41" spans="5:29" x14ac:dyDescent="0.4">
+      <c r="E41" t="str">
+        <v>fixed_leg.cashflows.[3].start_date</v>
+      </c>
+      <c r="F41" t="str">
+        <v>2023-03-07</v>
+      </c>
+      <c r="G41" t="str" cm="1">
+        <f t="array" ref="G41">_xll.ExLibris.Json.GetJsonValue($F$1,E41, EXLIBRIS_CONFIGURATION)</f>
+        <v>2023-03-07</v>
+      </c>
+      <c r="P41" t="s">
+        <v>51</v>
+      </c>
+      <c r="Q41" t="s">
+        <v>96</v>
+      </c>
+      <c r="R41" t="s">
+        <v>96</v>
+      </c>
+      <c r="AA41" t="b">
+        <f t="shared" si="4"/>
+        <v>1</v>
+      </c>
+      <c r="AB41" t="b">
+        <f t="shared" si="5"/>
+        <v>1</v>
+      </c>
+      <c r="AC41" t="b">
+        <f t="shared" si="5"/>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="42" spans="5:29" x14ac:dyDescent="0.4">
+      <c r="E42" t="str">
+        <v>fixed_leg.cashflows.[3].end_date</v>
+      </c>
+      <c r="F42" t="str">
+        <v>2023-09-03</v>
+      </c>
+      <c r="G42" t="str" cm="1">
+        <f t="array" ref="G42">_xll.ExLibris.Json.GetJsonValue($F$1,E42, EXLIBRIS_CONFIGURATION)</f>
+        <v>2023-09-03</v>
+      </c>
+      <c r="P42" t="s">
+        <v>52</v>
+      </c>
+      <c r="Q42" t="s">
+        <v>97</v>
+      </c>
+      <c r="R42" t="s">
+        <v>97</v>
+      </c>
+      <c r="AA42" t="b">
+        <f t="shared" si="4"/>
+        <v>1</v>
+      </c>
+      <c r="AB42" t="b">
+        <f t="shared" si="5"/>
+        <v>1</v>
+      </c>
+      <c r="AC42" t="b">
+        <f t="shared" si="5"/>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="43" spans="5:29" x14ac:dyDescent="0.4">
+      <c r="E43" t="str">
+        <v>fixed_leg.cashflows.[3].day_count_type</v>
+      </c>
+      <c r="F43" t="str">
+        <v>ACT/360</v>
+      </c>
+      <c r="G43" t="str" cm="1">
+        <f t="array" ref="G43">_xll.ExLibris.Json.GetJsonValue($F$1,E43, EXLIBRIS_CONFIGURATION)</f>
+        <v>ACT/360</v>
+      </c>
+      <c r="P43" t="s">
+        <v>53</v>
+      </c>
+      <c r="Q43" t="s">
+        <v>8</v>
+      </c>
+      <c r="R43" t="s">
+        <v>8</v>
+      </c>
+      <c r="AA43" t="b">
+        <f t="shared" si="4"/>
+        <v>1</v>
+      </c>
+      <c r="AB43" t="b">
+        <f t="shared" si="5"/>
+        <v>1</v>
+      </c>
+      <c r="AC43" t="b">
+        <f t="shared" si="5"/>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="44" spans="5:29" x14ac:dyDescent="0.4">
+      <c r="E44" t="str">
+        <v>fixed_leg.cashflows.[3].amout</v>
+      </c>
+      <c r="F44">
+        <v>13000000</v>
+      </c>
+      <c r="G44" cm="1">
+        <f t="array" ref="G44">_xll.ExLibris.Json.GetJsonValue($F$1,E44, EXLIBRIS_CONFIGURATION)</f>
+        <v>13000000</v>
+      </c>
+      <c r="P44" t="s">
+        <v>54</v>
+      </c>
+      <c r="Q44">
+        <v>13000000</v>
+      </c>
+      <c r="R44">
+        <v>13000000</v>
+      </c>
+      <c r="AA44" t="b">
+        <f t="shared" si="4"/>
+        <v>1</v>
+      </c>
+      <c r="AB44" t="b">
+        <f t="shared" si="5"/>
+        <v>1</v>
+      </c>
+      <c r="AC44" t="b">
+        <f t="shared" si="5"/>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="45" spans="5:29" x14ac:dyDescent="0.4">
+      <c r="E45" t="str">
+        <v>fixed_leg.cashflows.[3].fixed_rate</v>
+      </c>
+      <c r="F45">
+        <v>1E-3</v>
+      </c>
+      <c r="G45" cm="1">
+        <f t="array" ref="G45">_xll.ExLibris.Json.GetJsonValue($F$1,E45, EXLIBRIS_CONFIGURATION)</f>
+        <v>1E-3</v>
+      </c>
+      <c r="P45" t="s">
+        <v>55</v>
+      </c>
+      <c r="Q45">
+        <v>1E-3</v>
+      </c>
+      <c r="R45">
+        <v>1E-3</v>
+      </c>
+      <c r="AA45" t="b">
+        <f t="shared" si="4"/>
+        <v>1</v>
+      </c>
+      <c r="AB45" t="b">
+        <f t="shared" si="5"/>
+        <v>1</v>
+      </c>
+      <c r="AC45" t="b">
+        <f t="shared" si="5"/>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="46" spans="5:29" x14ac:dyDescent="0.4">
+      <c r="E46" t="str">
+        <v>fixed_leg.cashflows.[4].payment _date</v>
+      </c>
+      <c r="F46" t="str">
+        <v>2024-03-01</v>
+      </c>
+      <c r="G46" t="str" cm="1">
+        <f t="array" ref="G46">_xll.ExLibris.Json.GetJsonValue($F$1,E46, EXLIBRIS_CONFIGURATION)</f>
+        <v>2024-03-01</v>
+      </c>
+      <c r="P46" t="s">
+        <v>56</v>
+      </c>
+      <c r="Q46" t="s">
+        <v>98</v>
+      </c>
+      <c r="R46" t="s">
+        <v>98</v>
+      </c>
+      <c r="AA46" t="b">
+        <f t="shared" si="4"/>
+        <v>1</v>
+      </c>
+      <c r="AB46" t="b">
+        <f t="shared" si="5"/>
+        <v>1</v>
+      </c>
+      <c r="AC46" t="b">
+        <f t="shared" si="5"/>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="47" spans="5:29" x14ac:dyDescent="0.4">
+      <c r="E47" t="str">
+        <v>fixed_leg.cashflows.[4].start_date</v>
+      </c>
+      <c r="F47" t="str">
+        <v>2023-09-03</v>
+      </c>
+      <c r="G47" t="str" cm="1">
+        <f t="array" ref="G47">_xll.ExLibris.Json.GetJsonValue($F$1,E47, EXLIBRIS_CONFIGURATION)</f>
+        <v>2023-09-03</v>
+      </c>
+      <c r="P47" t="s">
+        <v>57</v>
+      </c>
+      <c r="Q47" t="s">
+        <v>97</v>
+      </c>
+      <c r="R47" t="s">
+        <v>97</v>
+      </c>
+      <c r="AA47" t="b">
+        <f t="shared" si="4"/>
+        <v>1</v>
+      </c>
+      <c r="AB47" t="b">
+        <f t="shared" si="5"/>
+        <v>1</v>
+      </c>
+      <c r="AC47" t="b">
+        <f t="shared" si="5"/>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="48" spans="5:29" x14ac:dyDescent="0.4">
+      <c r="E48" t="str">
+        <v>fixed_leg.cashflows.[4].end_date</v>
+      </c>
+      <c r="F48" t="str">
+        <v>2024-03-01</v>
+      </c>
+      <c r="G48" t="str" cm="1">
+        <f t="array" ref="G48">_xll.ExLibris.Json.GetJsonValue($F$1,E48, EXLIBRIS_CONFIGURATION)</f>
+        <v>2024-03-01</v>
+      </c>
+      <c r="P48" t="s">
+        <v>58</v>
+      </c>
+      <c r="Q48" t="s">
+        <v>98</v>
+      </c>
+      <c r="R48" t="s">
+        <v>98</v>
+      </c>
+      <c r="AA48" t="b">
+        <f t="shared" si="4"/>
+        <v>1</v>
+      </c>
+      <c r="AB48" t="b">
+        <f t="shared" si="5"/>
+        <v>1</v>
+      </c>
+      <c r="AC48" t="b">
+        <f t="shared" si="5"/>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="49" spans="5:29" x14ac:dyDescent="0.4">
+      <c r="E49" t="str">
+        <v>fixed_leg.cashflows.[4].day_count_type</v>
+      </c>
+      <c r="F49" t="str">
+        <v>ACT/360</v>
+      </c>
+      <c r="G49" t="str" cm="1">
+        <f t="array" ref="G49">_xll.ExLibris.Json.GetJsonValue($F$1,E49, EXLIBRIS_CONFIGURATION)</f>
+        <v>ACT/360</v>
+      </c>
+      <c r="P49" t="s">
+        <v>59</v>
+      </c>
+      <c r="Q49" t="s">
+        <v>8</v>
+      </c>
+      <c r="R49" t="s">
+        <v>8</v>
+      </c>
+      <c r="AA49" t="b">
+        <f t="shared" si="4"/>
+        <v>1</v>
+      </c>
+      <c r="AB49" t="b">
+        <f t="shared" si="5"/>
+        <v>1</v>
+      </c>
+      <c r="AC49" t="b">
+        <f t="shared" si="5"/>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="50" spans="5:29" x14ac:dyDescent="0.4">
+      <c r="E50" t="str">
+        <v>fixed_leg.cashflows.[4].amout</v>
+      </c>
+      <c r="F50">
+        <v>14000000</v>
+      </c>
+      <c r="G50" cm="1">
+        <f t="array" ref="G50">_xll.ExLibris.Json.GetJsonValue($F$1,E50, EXLIBRIS_CONFIGURATION)</f>
+        <v>14000000</v>
+      </c>
+      <c r="P50" t="s">
+        <v>60</v>
+      </c>
+      <c r="Q50">
+        <v>14000000</v>
+      </c>
+      <c r="R50">
+        <v>14000000</v>
+      </c>
+      <c r="AA50" t="b">
+        <f t="shared" si="4"/>
+        <v>1</v>
+      </c>
+      <c r="AB50" t="b">
+        <f t="shared" si="5"/>
+        <v>1</v>
+      </c>
+      <c r="AC50" t="b">
+        <f t="shared" si="5"/>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="51" spans="5:29" x14ac:dyDescent="0.4">
+      <c r="E51" t="str">
+        <v>fixed_leg.cashflows.[4].fixed_rate</v>
+      </c>
+      <c r="F51">
+        <v>1E-3</v>
+      </c>
+      <c r="G51" cm="1">
+        <f t="array" ref="G51">_xll.ExLibris.Json.GetJsonValue($F$1,E51, EXLIBRIS_CONFIGURATION)</f>
+        <v>1E-3</v>
+      </c>
+      <c r="P51" t="s">
+        <v>61</v>
+      </c>
+      <c r="Q51">
+        <v>1E-3</v>
+      </c>
+      <c r="R51">
+        <v>1E-3</v>
+      </c>
+      <c r="AA51" t="b">
+        <f t="shared" si="4"/>
+        <v>1</v>
+      </c>
+      <c r="AB51" t="b">
+        <f t="shared" si="5"/>
+        <v>1</v>
+      </c>
+      <c r="AC51" t="b">
+        <f t="shared" si="5"/>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="52" spans="5:29" x14ac:dyDescent="0.4">
+      <c r="E52" t="str">
+        <v>fixed_leg.cashflows.[5].payment _date</v>
+      </c>
+      <c r="F52" t="str">
+        <v>2024-08-28</v>
+      </c>
+      <c r="G52" t="str" cm="1">
+        <f t="array" ref="G52">_xll.ExLibris.Json.GetJsonValue($F$1,E52, EXLIBRIS_CONFIGURATION)</f>
+        <v>2024-08-28</v>
+      </c>
+      <c r="P52" t="s">
+        <v>62</v>
+      </c>
+      <c r="Q52" t="s">
+        <v>99</v>
+      </c>
+      <c r="R52" t="s">
+        <v>99</v>
+      </c>
+      <c r="AA52" t="b">
+        <f t="shared" si="4"/>
+        <v>1</v>
+      </c>
+      <c r="AB52" t="b">
+        <f t="shared" si="5"/>
+        <v>1</v>
+      </c>
+      <c r="AC52" t="b">
+        <f t="shared" si="5"/>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="53" spans="5:29" x14ac:dyDescent="0.4">
+      <c r="E53" t="str">
+        <v>fixed_leg.cashflows.[5].start_date</v>
+      </c>
+      <c r="F53" t="str">
+        <v>2024-03-01</v>
+      </c>
+      <c r="G53" t="str" cm="1">
+        <f t="array" ref="G53">_xll.ExLibris.Json.GetJsonValue($F$1,E53, EXLIBRIS_CONFIGURATION)</f>
+        <v>2024-03-01</v>
+      </c>
+      <c r="P53" t="s">
+        <v>63</v>
+      </c>
+      <c r="Q53" t="s">
+        <v>98</v>
+      </c>
+      <c r="R53" t="s">
+        <v>98</v>
+      </c>
+      <c r="AA53" t="b">
+        <f t="shared" si="4"/>
+        <v>1</v>
+      </c>
+      <c r="AB53" t="b">
+        <f t="shared" si="5"/>
+        <v>1</v>
+      </c>
+      <c r="AC53" t="b">
+        <f t="shared" si="5"/>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="54" spans="5:29" x14ac:dyDescent="0.4">
+      <c r="E54" t="str">
+        <v>fixed_leg.cashflows.[5].end_date</v>
+      </c>
+      <c r="F54" t="str">
+        <v>2024-08-28</v>
+      </c>
+      <c r="G54" t="str" cm="1">
+        <f t="array" ref="G54">_xll.ExLibris.Json.GetJsonValue($F$1,E54, EXLIBRIS_CONFIGURATION)</f>
+        <v>2024-08-28</v>
+      </c>
+      <c r="P54" t="s">
+        <v>64</v>
+      </c>
+      <c r="Q54" t="s">
+        <v>99</v>
+      </c>
+      <c r="R54" t="s">
+        <v>99</v>
+      </c>
+      <c r="AA54" t="b">
+        <f t="shared" si="4"/>
+        <v>1</v>
+      </c>
+      <c r="AB54" t="b">
+        <f t="shared" si="5"/>
+        <v>1</v>
+      </c>
+      <c r="AC54" t="b">
+        <f t="shared" si="5"/>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="55" spans="5:29" x14ac:dyDescent="0.4">
+      <c r="E55" t="str">
+        <v>fixed_leg.cashflows.[5].day_count_type</v>
+      </c>
+      <c r="F55" t="str">
+        <v>ACT/360</v>
+      </c>
+      <c r="G55" t="str" cm="1">
+        <f t="array" ref="G55">_xll.ExLibris.Json.GetJsonValue($F$1,E55, EXLIBRIS_CONFIGURATION)</f>
+        <v>ACT/360</v>
+      </c>
+      <c r="P55" t="s">
+        <v>65</v>
+      </c>
+      <c r="Q55" t="s">
+        <v>8</v>
+      </c>
+      <c r="R55" t="s">
+        <v>8</v>
+      </c>
+      <c r="AA55" t="b">
+        <f t="shared" si="4"/>
+        <v>1</v>
+      </c>
+      <c r="AB55" t="b">
+        <f t="shared" si="5"/>
+        <v>1</v>
+      </c>
+      <c r="AC55" t="b">
+        <f t="shared" si="5"/>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="56" spans="5:29" x14ac:dyDescent="0.4">
+      <c r="E56" t="str">
+        <v>fixed_leg.cashflows.[5].amout</v>
+      </c>
+      <c r="F56">
+        <v>15000000</v>
+      </c>
+      <c r="G56" cm="1">
+        <f t="array" ref="G56">_xll.ExLibris.Json.GetJsonValue($F$1,E56, EXLIBRIS_CONFIGURATION)</f>
+        <v>15000000</v>
+      </c>
+      <c r="P56" t="s">
+        <v>66</v>
+      </c>
+      <c r="Q56">
+        <v>15000000</v>
+      </c>
+      <c r="R56">
+        <v>15000000</v>
+      </c>
+      <c r="AA56" t="b">
+        <f t="shared" si="4"/>
+        <v>1</v>
+      </c>
+      <c r="AB56" t="b">
+        <f t="shared" si="5"/>
+        <v>1</v>
+      </c>
+      <c r="AC56" t="b">
+        <f t="shared" si="5"/>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="57" spans="5:29" x14ac:dyDescent="0.4">
+      <c r="E57" t="str">
+        <v>fixed_leg.cashflows.[5].fixed_rate</v>
+      </c>
+      <c r="F57">
+        <v>1E-3</v>
+      </c>
+      <c r="G57" cm="1">
+        <f t="array" ref="G57">_xll.ExLibris.Json.GetJsonValue($F$1,E57, EXLIBRIS_CONFIGURATION)</f>
+        <v>1E-3</v>
+      </c>
+      <c r="P57" t="s">
+        <v>67</v>
+      </c>
+      <c r="Q57">
+        <v>1E-3</v>
+      </c>
+      <c r="R57">
+        <v>1E-3</v>
+      </c>
+      <c r="AA57" t="b">
+        <f t="shared" si="4"/>
+        <v>1</v>
+      </c>
+      <c r="AB57" t="b">
+        <f t="shared" si="5"/>
+        <v>1</v>
+      </c>
+      <c r="AC57" t="b">
+        <f t="shared" si="5"/>
+        <v>1</v>
+      </c>
+    </row>
+  </sheetData>
+  <phoneticPr fontId="1"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C0D3ACF1-D52B-4405-9E6D-D2579DCD0199}">
   <dimension ref="B2:E15"/>
   <sheetFormatPr defaultRowHeight="18.75" x14ac:dyDescent="0.4"/>
@@ -3347,7 +5780,7 @@
       </c>
       <c r="E4" t="str" cm="1">
         <f t="array" ref="E4">_xll.ExLibris.WebSockets.OpenWebSocket("ws://localhost:10101",D4)</f>
-        <v>ExLibris.Core.WebSockets.WebsocketClient:4DF9B095-61CC-4272-AF17-953246EC0EF5</v>
+        <v>ExLibris.Core.WebSockets.WebsocketClient:AF651CF1-1F52-4171-B6DA-EE452997DBD2</v>
       </c>
     </row>
     <row r="6" spans="2:5" x14ac:dyDescent="0.4">
@@ -3365,7 +5798,7 @@
       </c>
       <c r="E7" t="str" cm="1">
         <f t="array" ref="E7">_xll.ExLibris.WebSockets.ObserveWebSocketMessage(E4)</f>
-        <v>push_event 23:42:24</v>
+        <v>push_event 22:04:25</v>
       </c>
     </row>
     <row r="9" spans="2:5" x14ac:dyDescent="0.4">
@@ -3374,7 +5807,7 @@
       </c>
       <c r="E9" t="str" cm="1">
         <f t="array" ref="E9">_xll.ExLibris.WebSockets.SendWebSocketMessage(E4,"test "&amp;D9,E6="Open")</f>
-        <v>message sent : 2021-09-15T11:42:08.610</v>
+        <v>message sent : 2021-09-20T10:01:04.926</v>
       </c>
     </row>
     <row r="10" spans="2:5" x14ac:dyDescent="0.4">
@@ -3383,7 +5816,7 @@
       </c>
       <c r="E10" t="str" cm="1">
         <f t="array" ref="E10">_xll.ExLibris.WebSockets.SendWebSocketMessage($E$4,"test next "&amp;D10,E9)</f>
-        <v>message sent : 2021-09-15T11:42:08.610</v>
+        <v>message sent : 2021-09-20T10:01:04.927</v>
       </c>
     </row>
     <row r="11" spans="2:5" x14ac:dyDescent="0.4">
@@ -3392,7 +5825,7 @@
       </c>
       <c r="E11" t="str" cm="1">
         <f t="array" ref="E11">_xll.ExLibris.WebSockets.SendWebSocketMessage($E$4,"test next "&amp;D11,E10)</f>
-        <v>message sent : 2021-09-15T11:42:08.610</v>
+        <v>message sent : 2021-09-20T10:01:04.931</v>
       </c>
     </row>
     <row r="12" spans="2:5" x14ac:dyDescent="0.4">
@@ -3401,7 +5834,7 @@
       </c>
       <c r="E12" t="str" cm="1">
         <f t="array" ref="E12">_xll.ExLibris.WebSockets.SendWebSocketMessage($E$4,"test next "&amp;D12,E11)</f>
-        <v>message sent : 2021-09-15T11:42:08.610</v>
+        <v>message sent : 2021-09-20T10:01:04.932</v>
       </c>
     </row>
     <row r="13" spans="2:5" x14ac:dyDescent="0.4">
@@ -3410,7 +5843,7 @@
       </c>
       <c r="E13" t="str" cm="1">
         <f t="array" ref="E13">_xll.ExLibris.WebSockets.SendWebSocketMessage($E$4,"test next "&amp;D13,E12)</f>
-        <v>message sent : 2021-09-15T11:42:08.611</v>
+        <v>message sent : 2021-09-20T10:01:04.946</v>
       </c>
     </row>
     <row r="14" spans="2:5" x14ac:dyDescent="0.4">
@@ -3419,7 +5852,7 @@
       </c>
       <c r="E14" t="str" cm="1">
         <f t="array" ref="E14">_xll.ExLibris.WebSockets.SendWebSocketMessage($E$4,"test next "&amp;D14,E13)</f>
-        <v>message sent : 2021-09-15T11:42:08.611</v>
+        <v>message sent : 2021-09-20T10:01:04.946</v>
       </c>
     </row>
     <row r="15" spans="2:5" x14ac:dyDescent="0.4">
@@ -3428,7 +5861,7 @@
       </c>
       <c r="E15" t="str" cm="1">
         <f t="array" ref="E15">_xll.ExLibris.WebSockets.SendWebSocketMessage($E$4,"test next "&amp;D15,E14)</f>
-        <v>message sent : 2021-09-15T11:42:08.611</v>
+        <v>message sent : 2021-09-20T10:01:04.947</v>
       </c>
     </row>
   </sheetData>
@@ -3438,7 +5871,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{92C31E65-5244-494C-A4E6-E2042CA25001}">
   <dimension ref="B2:F15"/>
   <sheetFormatPr defaultRowHeight="18.75" x14ac:dyDescent="0.4"/>
@@ -3455,7 +5888,7 @@
       </c>
       <c r="C2" t="str" cm="1">
         <f t="array" ref="C2">_xll.ExLibris.LoadConfiguration(B6:C15)</f>
-        <v>ExLibris.Core.ExLibrisConfiguration:E8DCA9AB-6EBC-4C98-8C3A-029399E3EB11</v>
+        <v>ExLibris.Core.ExLibrisConfiguration:78976E74-B484-403F-9AE1-F5D51D57D63F</v>
       </c>
     </row>
     <row r="4" spans="2:6" s="4" customFormat="1" ht="18" x14ac:dyDescent="0.4">

</xml_diff>

<commit_message>
refacotring : websocket client
</commit_message>
<xml_diff>
--- a/ExLibris/test_excel/exlibris_test.xlsx
+++ b/ExLibris/test_excel/exlibris_test.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\mugen\git\ex-libris\ExLibris\test_excel\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1EC2873F-5E94-4754-9542-2E2FFC115C15}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7660AA47-6101-403E-AA78-BDF81A98FB55}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{705CD0B7-27A9-4291-85BD-6034C0FEE3E4}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" activeTab="2" xr2:uid="{705CD0B7-27A9-4291-85BD-6034C0FEE3E4}"/>
   </bookViews>
   <sheets>
     <sheet name="json_test" sheetId="1" r:id="rId1"/>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/metadata.xml><?xml version="1.0" encoding="utf-8"?>
-<metadata xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xlrd="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata" xmlns:xda="http://schemas.microsoft.com/office/spreadsheetml/2017/dynamicarray">
+<metadata xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xda="http://schemas.microsoft.com/office/spreadsheetml/2017/dynamicarray">
   <metadataTypes count="1">
     <metadataType name="XLDAPR" minSupportedVersion="120000" copy="1" pasteAll="1" pasteValues="1" merge="1" splitFirst="1" rowColShift="1" clearFormats="1" clearComments="1" assign="1" coerce="1" cellMeta="1"/>
   </metadataTypes>
@@ -62,7 +62,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="319" uniqueCount="113">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="329" uniqueCount="114">
   <si>
     <t>payment _date</t>
   </si>
@@ -436,6 +436,10 @@
   </si>
   <si>
     <t>{"trade_code":"money_00001","couter_party":"CP00001","fixed_leg":{"pay_or_recieve":"Receive","cashflows":[{"payment _date":44632,"start_date":44452,"end_date":44632,"day_count_type":"ACT/360","amout":10000000,"fixed_rate":0.001},{"payment _date":44812,"start_date":44632,"end_date":44812,"day_count_type":"ACT/360","amout":11000000,"fixed_rate":0.001},{"payment _date":44992,"start_date":44812,"end_date":44992,"day_count_type":"ACT/360","amout":12000000,"fixed_rate":0.001},{"payment _date":45172,"start_date":44992,"end_date":45172,"day_count_type":"ACT/360","amout":13000000,"fixed_rate":0.001},{"payment _date":45352,"start_date":45172,"end_date":45352,"day_count_type":"ACT/360","amout":14000000,"fixed_rate":0.001},{"payment _date":45532,"start_date":45352,"end_date":45532,"day_count_type":"ACT/360","amout":15000000,"fixed_rate":0.001}]}}</t>
+  </si>
+  <si>
+    <t>client1</t>
+    <phoneticPr fontId="1"/>
   </si>
 </sst>
 </file>
@@ -541,608 +545,710 @@
 <file path=xl/volatileDependencies.xml><?xml version="1.0" encoding="utf-8"?>
 <volTypes xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <volType type="realTimeData">
-    <main first="rtdsrv.4b8ef99e016b447da4df1f9adeb95e96">
-      <tp>
-        <v>1</v>
-        <stp/>
-        <stp>686bc1c5-323e-4744-b701-e3b327147ccf</stp>
+    <main first="rtdsrv.db6c896509644de1836cdeb9db2ec598">
+      <tp>
+        <v>1</v>
+        <stp/>
+        <stp>93e4fdf8-ea4b-4a33-9856-402e5a7a8f6d</stp>
+        <tr r="I19" s="4"/>
+      </tp>
+      <tp>
+        <v>1</v>
+        <stp/>
+        <stp>e8acaa44-0dcd-43c8-a114-6c29dea55e3a</stp>
+        <tr r="G49" s="4"/>
+      </tp>
+      <tp>
+        <v>1</v>
+        <stp/>
+        <stp>5a2a29dc-3de8-4c41-a301-7bb0d809b344</stp>
+        <tr r="G56" s="1"/>
+      </tp>
+    </main>
+    <main first="rtdsrv.db6c896509644de1836cdeb9db2ec598">
+      <tp>
+        <v>1</v>
+        <stp/>
+        <stp>53e442f8-1e64-4293-beae-1e325f5ecbec</stp>
+        <tr r="G46" s="4"/>
+      </tp>
+      <tp>
+        <v>1</v>
+        <stp/>
+        <stp>4f349d4f-1fae-4c99-bcbe-bab9798d83cd</stp>
+        <tr r="G39" s="1"/>
+      </tp>
+    </main>
+    <main first="rtdsrv.db6c896509644de1836cdeb9db2ec598">
+      <tp>
+        <v>1</v>
+        <stp/>
+        <stp>504d5c0f-b001-4065-b635-5d8045acfea0</stp>
+        <tr r="G30" s="4"/>
+      </tp>
+    </main>
+    <main first="rtdsrv.db6c896509644de1836cdeb9db2ec598">
+      <tp>
+        <v>1</v>
+        <stp/>
+        <stp>7c7bd354-ab85-4455-8842-261c3d48dae9</stp>
+        <tr r="G35" s="1"/>
+      </tp>
+    </main>
+    <main first="rtdsrv.db6c896509644de1836cdeb9db2ec598">
+      <tp>
+        <v>1</v>
+        <stp/>
+        <stp>2968ccd6-9625-42b5-a471-457af3dbae56</stp>
+        <tr r="G55" s="4"/>
+      </tp>
+    </main>
+    <main first="rtdsrv.db6c896509644de1836cdeb9db2ec598">
+      <tp>
+        <v>2</v>
+        <stp/>
+        <stp>c1029caa-5f69-4f6c-b1ce-72e9fb3ca684</stp>
+        <tr r="E6" s="3"/>
+      </tp>
+    </main>
+    <main first="rtdsrv.db6c896509644de1836cdeb9db2ec598">
+      <tp>
+        <v>1</v>
+        <stp/>
+        <stp>a2b14fe0-d139-4a21-820c-8e41cb0a27d0</stp>
+        <tr r="G24" s="1"/>
+      </tp>
+    </main>
+    <main first="rtdsrv.db6c896509644de1836cdeb9db2ec598">
+      <tp>
+        <v>1</v>
+        <stp/>
+        <stp>6f896637-e3fc-4627-a6fe-81952e24d05a</stp>
+        <tr r="G56" s="4"/>
+      </tp>
+      <tp>
+        <v>1</v>
+        <stp/>
+        <stp>29496912-dc7f-40d5-a110-47ddafa0e132</stp>
+        <tr r="G20" s="4"/>
+      </tp>
+    </main>
+    <main first="rtdsrv.db6c896509644de1836cdeb9db2ec598">
+      <tp>
+        <v>1</v>
+        <stp/>
+        <stp>551c8c0d-5225-46cc-91bf-ffbfe4a050a5</stp>
+        <tr r="G27" s="4"/>
+      </tp>
+      <tp>
+        <v>1</v>
+        <stp/>
+        <stp>9e9c8fcb-9367-4aef-88ff-9383f9b360b8</stp>
+        <tr r="G30" s="1"/>
+      </tp>
+      <tp>
+        <v>1</v>
+        <stp/>
+        <stp>d011499e-23db-43e8-8821-223f024cb186</stp>
+        <tr r="G36" s="1"/>
+      </tp>
+    </main>
+    <main first="rtdsrv.db6c896509644de1836cdeb9db2ec598">
+      <tp>
+        <v>1</v>
+        <stp/>
+        <stp>6f23eb6e-df1b-4351-9f15-303cef7c7121</stp>
+        <tr r="G54" s="4"/>
+      </tp>
+    </main>
+    <main first="rtdsrv.db6c896509644de1836cdeb9db2ec598">
+      <tp>
+        <v>1</v>
+        <stp/>
+        <stp>4aec1dc5-779d-49d5-a68f-4ce569243b36</stp>
+        <tr r="G32" s="4"/>
+      </tp>
+    </main>
+    <main first="rtdsrv.db6c896509644de1836cdeb9db2ec598">
+      <tp>
+        <v>1</v>
+        <stp/>
+        <stp>1782e00d-b22d-428a-bb8a-696ccdd5ff83</stp>
+        <tr r="G46" s="1"/>
+      </tp>
+      <tp>
+        <v>1</v>
+        <stp/>
+        <stp>efd26363-f200-46fd-9f29-0c5c89fb19ad</stp>
+        <tr r="G27" s="1"/>
+      </tp>
+    </main>
+    <main first="rtdsrv.db6c896509644de1836cdeb9db2ec598">
+      <tp>
+        <v>1</v>
+        <stp/>
+        <stp>8bd66772-ad29-408e-9631-b9aa5df2f9d2</stp>
+        <tr r="G43" s="1"/>
+      </tp>
+    </main>
+    <main first="rtdsrv.db6c896509644de1836cdeb9db2ec598">
+      <tp>
+        <v>1</v>
+        <stp/>
+        <stp>95142b80-4415-47a4-9779-ce1af79e3449</stp>
+        <tr r="G47" s="1"/>
+      </tp>
+    </main>
+    <main first="rtdsrv.db6c896509644de1836cdeb9db2ec598">
+      <tp>
+        <v>1</v>
+        <stp/>
+        <stp>3e4e4201-0ee4-4226-a65e-c580dd7db32f</stp>
+        <tr r="G28" s="1"/>
+      </tp>
+    </main>
+    <main first="rtdsrv.db6c896509644de1836cdeb9db2ec598">
+      <tp>
+        <v>1</v>
+        <stp/>
+        <stp>bff6b94e-9c03-46b2-9eed-cc344e56d222</stp>
+        <tr r="G53" s="1"/>
+      </tp>
+    </main>
+    <main first="rtdsrv.db6c896509644de1836cdeb9db2ec598">
+      <tp>
+        <v>1</v>
+        <stp/>
+        <stp>bab19082-6465-45e4-bc5d-055a4ee743b4</stp>
+        <tr r="G51" s="1"/>
+      </tp>
+    </main>
+    <main first="rtdsrv.db6c896509644de1836cdeb9db2ec598">
+      <tp>
+        <v>1</v>
+        <stp/>
+        <stp>c1ab782e-3262-41ab-ace7-f2587264d994</stp>
+        <tr r="G45" s="1"/>
+      </tp>
+      <tp>
+        <v>1</v>
+        <stp/>
+        <stp>f13498c6-2a3b-40ae-aee9-791bd6624017</stp>
+        <tr r="G41" s="4"/>
+      </tp>
+      <tp>
+        <v>1</v>
+        <stp/>
+        <stp>f9bb4a82-312d-42e0-8a1c-78be3ede331c</stp>
+        <tr r="G19" s="1"/>
+      </tp>
+    </main>
+    <main first="rtdsrv.db6c896509644de1836cdeb9db2ec598">
+      <tp>
+        <v>1</v>
+        <stp/>
+        <stp>4d7dfdab-3dc6-4bb4-8acb-2b00a4d96622</stp>
+        <tr r="G47" s="4"/>
+      </tp>
+    </main>
+    <main first="rtdsrv.db6c896509644de1836cdeb9db2ec598">
+      <tp>
+        <v>1</v>
+        <stp/>
+        <stp>28fb6429-57d0-45f7-8ce0-d3a1babd9254</stp>
+        <tr r="C2" s="2"/>
+      </tp>
+    </main>
+    <main first="rtdsrv.db6c896509644de1836cdeb9db2ec598">
+      <tp>
+        <v>1</v>
+        <stp/>
+        <stp>091a4db0-cd9b-497d-a016-3b22d36f51d5</stp>
+        <tr r="G50" s="4"/>
+      </tp>
+    </main>
+    <main first="rtdsrv.db6c896509644de1836cdeb9db2ec598">
+      <tp>
+        <v>1</v>
+        <stp/>
+        <stp>f33f4e10-b854-48ac-b4f6-ab1b8857bae7</stp>
+        <tr r="G35" s="4"/>
+      </tp>
+    </main>
+    <main first="rtdsrv.db6c896509644de1836cdeb9db2ec598">
+      <tp>
+        <v>1</v>
+        <stp/>
+        <stp>3a36ae2d-94e0-48b5-879a-7a0dbba478e0</stp>
+        <tr r="G26" s="1"/>
+      </tp>
+    </main>
+    <main first="rtdsrv.db6c896509644de1836cdeb9db2ec598">
+      <tp>
+        <v>1</v>
+        <stp/>
+        <stp>2277a962-66f9-4117-a688-0e3a69a64da4</stp>
+        <tr r="G23" s="4"/>
+      </tp>
+    </main>
+    <main first="rtdsrv.db6c896509644de1836cdeb9db2ec598">
+      <tp>
+        <v>1</v>
+        <stp/>
+        <stp>a08fb980-3454-4361-b9fd-a32d0508ab0a</stp>
+        <tr r="G34" s="1"/>
+      </tp>
+    </main>
+    <main first="rtdsrv.db6c896509644de1836cdeb9db2ec598">
+      <tp>
+        <v>1</v>
+        <stp/>
+        <stp>9a816655-a342-4b9b-bb1d-f9b7a339ef5a</stp>
+        <tr r="G22" s="1"/>
+      </tp>
+    </main>
+    <main first="rtdsrv.db6c896509644de1836cdeb9db2ec598">
+      <tp>
+        <v>1</v>
+        <stp/>
+        <stp>b19c782b-0042-40d0-91ad-80e5fda6f4a2</stp>
+        <tr r="G25" s="4"/>
+      </tp>
+    </main>
+    <main first="rtdsrv.db6c896509644de1836cdeb9db2ec598">
+      <tp>
+        <v>1</v>
+        <stp/>
+        <stp>b85a7a21-b0b0-494f-b42b-cfc444add5ae</stp>
+        <tr r="G39" s="4"/>
+      </tp>
+    </main>
+    <main first="rtdsrv.db6c896509644de1836cdeb9db2ec598">
+      <tp>
+        <v>1</v>
+        <stp/>
+        <stp>76c5be7e-743b-4258-95bf-1e395d61676c</stp>
+        <tr r="I28" s="4"/>
+      </tp>
+    </main>
+    <main first="rtdsrv.db6c896509644de1836cdeb9db2ec598">
+      <tp>
+        <v>1</v>
+        <stp/>
+        <stp>2a3a333f-b28c-45eb-8eb6-d6594981706d</stp>
+        <tr r="G33" s="4"/>
+      </tp>
+    </main>
+    <main first="rtdsrv.db6c896509644de1836cdeb9db2ec598">
+      <tp>
+        <v>1</v>
+        <stp/>
+        <stp>da1c1356-3929-4a38-88f2-40fa114fc0f0</stp>
+        <tr r="G24" s="4"/>
+      </tp>
+    </main>
+    <main first="rtdsrv.db6c896509644de1836cdeb9db2ec598">
+      <tp>
+        <v>1</v>
+        <stp/>
+        <stp>6222d97f-d036-439d-9c74-7226652c2569</stp>
+        <tr r="G23" s="1"/>
+      </tp>
+    </main>
+    <main first="rtdsrv.db6c896509644de1836cdeb9db2ec598">
+      <tp>
+        <v>1</v>
+        <stp/>
+        <stp>12b869cc-cec4-4722-9b17-066b01e65b0a</stp>
+        <tr r="G29" s="1"/>
+      </tp>
+      <tp>
+        <v>1</v>
+        <stp/>
+        <stp>92bb4a05-ae6c-4ee4-83d6-516d0de979c5</stp>
+        <tr r="G34" s="4"/>
+      </tp>
+      <tp>
+        <v>1</v>
+        <stp/>
+        <stp>88ea1428-f268-4024-9e31-8a78014b9093</stp>
+        <tr r="G48" s="4"/>
+      </tp>
+    </main>
+    <main first="rtdsrv.db6c896509644de1836cdeb9db2ec598">
+      <tp>
+        <v>1</v>
+        <stp/>
+        <stp>0d1c1301-8da6-4f92-8d59-fe1de7726792</stp>
+        <tr r="G57" s="4"/>
+      </tp>
+    </main>
+    <main first="rtdsrv.db6c896509644de1836cdeb9db2ec598">
+      <tp>
+        <v>1</v>
+        <stp/>
+        <stp>1b8d049d-1206-4b59-89e8-c254f751533a</stp>
+        <tr r="G51" s="4"/>
+      </tp>
+    </main>
+    <main first="rtdsrv.db6c896509644de1836cdeb9db2ec598">
+      <tp>
+        <v>1</v>
+        <stp/>
+        <stp>a5280c10-ece9-44d3-9687-d60257d7a5e7</stp>
+        <tr r="G54" s="1"/>
+      </tp>
+    </main>
+    <main first="rtdsrv.db6c896509644de1836cdeb9db2ec598">
+      <tp>
+        <v>1</v>
+        <stp/>
+        <stp>f27a6d38-5f10-4dbe-86c1-842ba3af01b0</stp>
+        <tr r="G55" s="1"/>
+      </tp>
+    </main>
+    <main first="rtdsrv.db6c896509644de1836cdeb9db2ec598">
+      <tp>
+        <v>1</v>
+        <stp/>
+        <stp>b62de6d9-a006-4e40-944e-eb8aaa710527</stp>
+        <tr r="G38" s="4"/>
+      </tp>
+    </main>
+    <main first="rtdsrv.db6c896509644de1836cdeb9db2ec598">
+      <tp>
+        <v>1</v>
+        <stp/>
+        <stp>b6824a84-2ef6-4df3-a913-003e2204f717</stp>
+        <tr r="G37" s="4"/>
+      </tp>
+    </main>
+    <main first="rtdsrv.db6c896509644de1836cdeb9db2ec598">
+      <tp>
+        <v>1</v>
+        <stp/>
+        <stp>a3bd9f5f-ca26-4415-83fa-c5f1a15ba3dd</stp>
+        <tr r="I19" s="1"/>
+      </tp>
+    </main>
+    <main first="rtdsrv.db6c896509644de1836cdeb9db2ec598">
+      <tp>
+        <v>1</v>
+        <stp/>
+        <stp>7ae6c7da-264f-4bff-81f4-d26d678660f3</stp>
+        <tr r="G21" s="4"/>
+      </tp>
+    </main>
+    <main first="rtdsrv.db6c896509644de1836cdeb9db2ec598">
+      <tp>
+        <v>1</v>
+        <stp/>
+        <stp>57f54d62-dcd3-4f50-aa42-ae205a710fe5</stp>
+        <tr r="G44" s="1"/>
+      </tp>
+      <tp>
+        <v>1</v>
+        <stp/>
+        <stp>8f3e1fb4-74b9-4bf3-83d2-c78aa6ae602e</stp>
+        <tr r="F1" s="4"/>
+      </tp>
+    </main>
+    <main first="rtdsrv.db6c896509644de1836cdeb9db2ec598">
+      <tp>
+        <v>1</v>
+        <stp/>
+        <stp>315dfc22-af1a-4f1a-9a28-f19e7c870b2a</stp>
+        <tr r="G42" s="4"/>
+      </tp>
+    </main>
+    <main first="rtdsrv.db6c896509644de1836cdeb9db2ec598">
+      <tp>
+        <v>1</v>
+        <stp/>
+        <stp>4e09315d-4510-42f2-a06d-bcee0f6d41d8</stp>
+        <tr r="G29" s="4"/>
+      </tp>
+    </main>
+    <main first="rtdsrv.db6c896509644de1836cdeb9db2ec598">
+      <tp>
+        <v>1</v>
+        <stp/>
+        <stp>10c4e3f9-e426-448b-99ce-707b2d3a5c16</stp>
+        <tr r="G31" s="1"/>
+      </tp>
+    </main>
+    <main first="rtdsrv.db6c896509644de1836cdeb9db2ec598">
+      <tp>
+        <v>1</v>
+        <stp/>
+        <stp>1e14db47-388f-45d9-b46d-8c9e80a97821</stp>
+        <tr r="G52" s="4"/>
+      </tp>
+    </main>
+    <main first="rtdsrv.db6c896509644de1836cdeb9db2ec598">
+      <tp>
+        <v>1</v>
+        <stp/>
+        <stp>c9c03b22-315b-4838-90d3-ef567402514b</stp>
+        <tr r="G45" s="4"/>
+      </tp>
+    </main>
+    <main first="rtdsrv.db6c896509644de1836cdeb9db2ec598">
+      <tp>
+        <v>1</v>
+        <stp/>
+        <stp>506b75d2-3267-450b-9950-dcd5809f9e05</stp>
+        <tr r="F6" s="4"/>
+      </tp>
+    </main>
+    <main first="rtdsrv.db6c896509644de1836cdeb9db2ec598">
+      <tp>
+        <v>1</v>
+        <stp/>
+        <stp>decabe36-fb89-4fff-b5ef-fca842ec6ce7</stp>
+        <tr r="G31" s="4"/>
+      </tp>
+      <tp>
+        <v>1</v>
+        <stp/>
+        <stp>afd54d0d-3b6c-491d-8b40-ec5c1e99109b</stp>
+        <tr r="G38" s="1"/>
+      </tp>
+    </main>
+    <main first="rtdsrv.db6c896509644de1836cdeb9db2ec598">
+      <tp>
+        <v>1</v>
+        <stp/>
+        <stp>d8ef4749-9678-432a-85a5-c0d9e1fcfa55</stp>
+        <tr r="I28" s="1"/>
+      </tp>
+    </main>
+    <main first="rtdsrv.db6c896509644de1836cdeb9db2ec598">
+      <tp>
+        <v>1</v>
+        <stp/>
+        <stp>3ab1ff36-ac5f-47e2-9d49-4d86aa4293df</stp>
+        <tr r="G19" s="4"/>
+      </tp>
+    </main>
+    <main first="rtdsrv.db6c896509644de1836cdeb9db2ec598">
+      <tp>
+        <v>1</v>
+        <stp/>
+        <stp>825f6912-9896-40dc-a356-b128afbe4f6a</stp>
+        <tr r="F6" s="1"/>
+      </tp>
+    </main>
+    <main first="rtdsrv.db6c896509644de1836cdeb9db2ec598">
+      <tp>
+        <v>1</v>
+        <stp/>
+        <stp>ecce8449-e7d0-4515-9423-6274de14a768</stp>
+        <tr r="G48" s="1"/>
+      </tp>
+    </main>
+    <main first="rtdsrv.db6c896509644de1836cdeb9db2ec598">
+      <tp>
+        <v>1</v>
+        <stp/>
+        <stp>97656a24-fc6b-482d-b795-88030e6c5e49</stp>
+        <tr r="G52" s="1"/>
+      </tp>
+    </main>
+    <main first="rtdsrv.db6c896509644de1836cdeb9db2ec598">
+      <tp>
+        <v>1</v>
+        <stp/>
+        <stp>e629aec4-c8fd-4531-8a5f-55a006325bbe</stp>
+        <tr r="G40" s="4"/>
+      </tp>
+    </main>
+    <main first="rtdsrv.db6c896509644de1836cdeb9db2ec598">
+      <tp>
+        <v>1</v>
+        <stp/>
+        <stp>98a40869-1fb1-47dd-b1f3-54b3a3e52a2f</stp>
+        <tr r="G33" s="1"/>
+      </tp>
+      <tp>
+        <v>1</v>
+        <stp/>
+        <stp>64503075-1343-483c-94f5-dcfb0ca47e76</stp>
+        <tr r="G42" s="1"/>
+      </tp>
+    </main>
+    <main first="rtdsrv.db6c896509644de1836cdeb9db2ec598">
+      <tp>
+        <v>1</v>
+        <stp/>
+        <stp>76fa3ee3-cfa1-4f5c-83f1-9f9b0568625e</stp>
+        <tr r="G57" s="1"/>
+      </tp>
+      <tp>
+        <v>1</v>
+        <stp/>
+        <stp>7c6295a2-a7cd-415f-8858-5b108e4ac71c</stp>
+        <tr r="G40" s="1"/>
+      </tp>
+    </main>
+    <main first="rtdsrv.db6c896509644de1836cdeb9db2ec598">
+      <tp>
+        <v>3</v>
+        <stp/>
+        <stp>b3d12bcc-6fbc-4bd0-abfa-254cce48f5f0</stp>
+        <tr r="E19" s="3"/>
+      </tp>
+    </main>
+    <main first="rtdsrv.db6c896509644de1836cdeb9db2ec598">
+      <tp>
+        <v>1</v>
+        <stp/>
+        <stp>74934fcf-8a7e-41ba-bcd1-a91724df093d</stp>
+        <tr r="E7" s="3"/>
+      </tp>
+    </main>
+    <main first="rtdsrv.db6c896509644de1836cdeb9db2ec598">
+      <tp>
+        <v>7</v>
+        <stp/>
+        <stp>522ea8bf-b4f0-4f1e-aa6d-dbdc25f607df</stp>
+        <tr r="E20" s="3"/>
+      </tp>
+    </main>
+    <main first="rtdsrv.db6c896509644de1836cdeb9db2ec598">
+      <tp>
+        <v>1</v>
+        <stp/>
+        <stp>30039974-0675-42e9-a066-860b2b2ef95c</stp>
+        <tr r="G41" s="1"/>
+      </tp>
+    </main>
+    <main first="rtdsrv.db6c896509644de1836cdeb9db2ec598">
+      <tp>
+        <v>1</v>
+        <stp/>
+        <stp>4693423f-300f-4148-b9c3-1221eb577f1a</stp>
+        <tr r="G36" s="4"/>
+      </tp>
+    </main>
+    <main first="rtdsrv.db6c896509644de1836cdeb9db2ec598">
+      <tp>
+        <v>1</v>
+        <stp/>
+        <stp>8886342d-f032-4b80-8fde-e562d5902dde</stp>
+        <tr r="G28" s="4"/>
+      </tp>
+    </main>
+    <main first="rtdsrv.db6c896509644de1836cdeb9db2ec598">
+      <tp>
+        <v>1</v>
+        <stp/>
+        <stp>af87949d-cb15-4711-84ad-6b1d2ae2b8a3</stp>
+        <tr r="G21" s="1"/>
+      </tp>
+      <tp>
+        <v>1</v>
+        <stp/>
+        <stp>ea2c37bc-d1f3-4962-b8bd-f17be9f8f0f7</stp>
+        <tr r="G44" s="4"/>
+      </tp>
+    </main>
+    <main first="rtdsrv.db6c896509644de1836cdeb9db2ec598">
+      <tp>
+        <v>1</v>
+        <stp/>
+        <stp>d88eb260-959a-4938-857f-6762ddde06e5</stp>
+        <tr r="G43" s="4"/>
+      </tp>
+    </main>
+    <main first="rtdsrv.db6c896509644de1836cdeb9db2ec598">
+      <tp>
+        <v>1</v>
+        <stp/>
+        <stp>d84f3a65-1164-476f-a168-7fec914c4763</stp>
+        <tr r="G37" s="1"/>
+      </tp>
+    </main>
+    <main first="rtdsrv.db6c896509644de1836cdeb9db2ec598">
+      <tp>
+        <v>1</v>
+        <stp/>
+        <stp>07b1a09b-9452-4ee0-b77a-81f8fb60a506</stp>
+        <tr r="F1" s="1"/>
+      </tp>
+    </main>
+    <main first="rtdsrv.db6c896509644de1836cdeb9db2ec598">
+      <tp>
+        <v>1</v>
+        <stp/>
+        <stp>d9aa2161-ace6-4064-b321-2fcee4851b42</stp>
+        <tr r="G53" s="4"/>
+      </tp>
+    </main>
+    <main first="rtdsrv.db6c896509644de1836cdeb9db2ec598">
+      <tp>
+        <v>1</v>
+        <stp/>
+        <stp>25be8688-98bd-4a36-96f6-f790cd9d1f1a</stp>
+        <tr r="G20" s="1"/>
+      </tp>
+    </main>
+    <main first="rtdsrv.db6c896509644de1836cdeb9db2ec598">
+      <tp>
+        <v>1</v>
+        <stp/>
+        <stp>0e58d5a1-6aaa-4449-8f18-7c69ddc9b698</stp>
+        <tr r="G49" s="1"/>
+      </tp>
+    </main>
+    <main first="rtdsrv.db6c896509644de1836cdeb9db2ec598">
+      <tp>
+        <v>1</v>
+        <stp/>
+        <stp>a79d8d4a-e6ff-4b0e-898c-d6d5f625a441</stp>
+        <tr r="G32" s="1"/>
+      </tp>
+      <tp>
+        <v>1</v>
+        <stp/>
+        <stp>37ca0c03-57bb-4d6d-bb8b-4b9addc0fdf5</stp>
+        <tr r="E17" s="3"/>
+      </tp>
+    </main>
+    <main first="rtdsrv.db6c896509644de1836cdeb9db2ec598">
+      <tp>
+        <v>1</v>
+        <stp/>
+        <stp>3fad93a4-ff9f-4acd-aac1-909408d70aa4</stp>
+        <tr r="G26" s="4"/>
+      </tp>
+    </main>
+    <main first="rtdsrv.db6c896509644de1836cdeb9db2ec598">
+      <tp>
+        <v>1</v>
+        <stp/>
+        <stp>d46533dd-63c7-41b5-863c-c5911f7c48b8</stp>
+        <tr r="G50" s="1"/>
+      </tp>
+    </main>
+    <main first="rtdsrv.db6c896509644de1836cdeb9db2ec598">
+      <tp>
+        <v>1</v>
+        <stp/>
+        <stp>760ba543-24ab-4ebf-a11b-d39559e66075</stp>
         <tr r="G25" s="1"/>
       </tp>
       <tp>
         <v>1</v>
         <stp/>
-        <stp>5762ea02-f98e-44f5-8af4-a01b12463914</stp>
-        <tr r="G27" s="1"/>
-      </tp>
-      <tp>
-        <v>1</v>
-        <stp/>
-        <stp>9e6fa9bf-d626-4b10-82fe-5ae1ccc2a423</stp>
-        <tr r="F6" s="4"/>
-      </tp>
-      <tp>
-        <v>1</v>
-        <stp/>
-        <stp>c66e509e-94f6-48c2-bb0c-af5f357b7664</stp>
-        <tr r="G36" s="4"/>
-      </tp>
-    </main>
-    <main first="rtdsrv.4b8ef99e016b447da4df1f9adeb95e96">
-      <tp>
-        <v>1</v>
-        <stp/>
-        <stp>4efd792c-b43e-4209-8e80-ae43236ba2e3</stp>
-        <tr r="G25" s="4"/>
-      </tp>
-      <tp>
-        <v>1</v>
-        <stp/>
-        <stp>f37079ca-e529-4b73-87fe-b232caac12c5</stp>
-        <tr r="G52" s="1"/>
-      </tp>
-    </main>
-    <main first="rtdsrv.4b8ef99e016b447da4df1f9adeb95e96">
-      <tp>
-        <v>1</v>
-        <stp/>
-        <stp>67012ff4-1270-4eaa-848e-a22e52fa8b2f</stp>
-        <tr r="G57" s="1"/>
-      </tp>
-      <tp>
-        <v>1</v>
-        <stp/>
-        <stp>52b667d1-6ce4-459f-a6a2-45793c0028d3</stp>
-        <tr r="G27" s="4"/>
-      </tp>
-      <tp>
-        <v>1</v>
-        <stp/>
-        <stp>89f8e619-fafb-409f-90e0-e43c009a0489</stp>
-        <tr r="G21" s="1"/>
-      </tp>
-      <tp>
-        <v>1</v>
-        <stp/>
-        <stp>caf4d30a-a402-4fc3-ab09-07cb89345da7</stp>
-        <tr r="G31" s="1"/>
-      </tp>
-      <tp>
-        <v>1</v>
-        <stp/>
-        <stp>e2b50a7f-c0b4-4e28-9c5c-063f6a32e76f</stp>
-        <tr r="G56" s="1"/>
-      </tp>
-      <tp>
-        <v>1</v>
-        <stp/>
-        <stp>cbcf9cab-f3ec-4461-93f7-4573f961aae4</stp>
-        <tr r="G53" s="1"/>
-      </tp>
-      <tp>
-        <v>1</v>
-        <stp/>
-        <stp>cee9e8aa-3e79-4832-985b-74cc2e842de4</stp>
-        <tr r="G42" s="1"/>
-      </tp>
-      <tp>
-        <v>1</v>
-        <stp/>
-        <stp>2af9c600-62cb-44c1-9d7b-384dc2c5a1af</stp>
-        <tr r="C2" s="2"/>
-      </tp>
-      <tp>
-        <v>1</v>
-        <stp/>
-        <stp>5dc5449c-285b-4969-ac73-7ffb4492dbf4</stp>
-        <tr r="G40" s="4"/>
-      </tp>
-      <tp>
-        <v>1</v>
-        <stp/>
-        <stp>5f6eacb5-697b-434b-86f6-2975cb268086</stp>
-        <tr r="G31" s="4"/>
-      </tp>
-      <tp>
-        <v>1</v>
-        <stp/>
-        <stp>d934f17e-44de-4792-82e5-5be9e73f9b4b</stp>
-        <tr r="G33" s="4"/>
-      </tp>
-    </main>
-    <main first="rtdsrv.4b8ef99e016b447da4df1f9adeb95e96">
-      <tp>
-        <v>1</v>
-        <stp/>
-        <stp>a2f0394e-7e61-43f9-89d0-d9d2373de0e2</stp>
-        <tr r="G26" s="4"/>
-      </tp>
-    </main>
-    <main first="rtdsrv.4b8ef99e016b447da4df1f9adeb95e96">
-      <tp>
-        <v>2</v>
-        <stp/>
-        <stp>f683902d-4f5d-4695-85c9-70a6227ad9a1</stp>
-        <tr r="E6" s="3"/>
-      </tp>
-      <tp>
-        <v>1</v>
-        <stp/>
-        <stp>5fa7ab49-a894-483f-8180-4a54afb86ba1</stp>
-        <tr r="G38" s="1"/>
-      </tp>
-      <tp>
-        <v>1</v>
-        <stp/>
-        <stp>35d80511-c89c-44f5-a8c7-c5d9f8158ffa</stp>
-        <tr r="G20" s="1"/>
-      </tp>
-      <tp>
-        <v>1</v>
-        <stp/>
-        <stp>3ab4ebe7-a21c-4702-a280-5211f04df4ba</stp>
-        <tr r="G20" s="4"/>
-      </tp>
-    </main>
-    <main first="rtdsrv.4b8ef99e016b447da4df1f9adeb95e96">
-      <tp>
-        <v>1</v>
-        <stp/>
-        <stp>07592be1-25ec-418a-ad74-727bdc56510f</stp>
-        <tr r="G49" s="1"/>
-      </tp>
-    </main>
-    <main first="rtdsrv.4b8ef99e016b447da4df1f9adeb95e96">
-      <tp>
-        <v>1</v>
-        <stp/>
-        <stp>60c987a5-d7f3-4535-afaa-606e762cead9</stp>
-        <tr r="G32" s="1"/>
-      </tp>
-    </main>
-    <main first="rtdsrv.4b8ef99e016b447da4df1f9adeb95e96">
-      <tp>
-        <v>1</v>
-        <stp/>
-        <stp>7f546308-9bd8-4b30-933e-3dbe38580c81</stp>
-        <tr r="G19" s="1"/>
-      </tp>
-    </main>
-    <main first="rtdsrv.4b8ef99e016b447da4df1f9adeb95e96">
-      <tp>
-        <v>1</v>
-        <stp/>
-        <stp>a7d76aee-c7f5-4013-9c34-80a4dc321638</stp>
-        <tr r="G35" s="4"/>
-      </tp>
-      <tp>
-        <v>1</v>
-        <stp/>
-        <stp>de0d9157-bea8-4204-b7dd-1e3c62770aa4</stp>
-        <tr r="G24" s="1"/>
-      </tp>
-    </main>
-    <main first="rtdsrv.4b8ef99e016b447da4df1f9adeb95e96">
-      <tp>
-        <v>1</v>
-        <stp/>
-        <stp>e3b96405-cf09-4807-ac9a-f910d3788301</stp>
-        <tr r="G45" s="4"/>
-      </tp>
-      <tp>
-        <v>1</v>
-        <stp/>
-        <stp>24e2d18f-48ce-4cf4-8914-9ef68226412e</stp>
-        <tr r="G24" s="4"/>
-      </tp>
-    </main>
-    <main first="rtdsrv.4b8ef99e016b447da4df1f9adeb95e96">
-      <tp>
-        <v>1</v>
-        <stp/>
-        <stp>a99f1cad-dbb1-4d0b-87d2-37a1ceb188fb</stp>
-        <tr r="G47" s="4"/>
-      </tp>
-      <tp>
-        <v>1</v>
-        <stp/>
-        <stp>dfe1bc29-d3b7-44be-a4ed-15290cd27b46</stp>
-        <tr r="G41" s="4"/>
-      </tp>
-    </main>
-    <main first="rtdsrv.4b8ef99e016b447da4df1f9adeb95e96">
-      <tp>
-        <v>1</v>
-        <stp/>
-        <stp>e2fb3df6-7928-4ed2-8d99-4288b8aa348e</stp>
-        <tr r="G51" s="4"/>
-      </tp>
-      <tp>
-        <v>1</v>
-        <stp/>
-        <stp>b06dd595-b7b5-404f-80bc-57d58bb87b99</stp>
-        <tr r="G30" s="4"/>
-      </tp>
-    </main>
-    <main first="rtdsrv.4b8ef99e016b447da4df1f9adeb95e96">
-      <tp>
-        <v>1</v>
-        <stp/>
-        <stp>75eb7dcb-1240-4813-b3cd-ef943785f6ce</stp>
-        <tr r="G47" s="1"/>
-      </tp>
-      <tp>
-        <v>1</v>
-        <stp/>
-        <stp>1fc5db0e-0951-487a-b35f-6615274cf683</stp>
-        <tr r="G28" s="4"/>
-      </tp>
-      <tp>
-        <v>1</v>
-        <stp/>
-        <stp>3f7b3da9-67a8-4255-b1be-ae7e3397cbab</stp>
-        <tr r="G37" s="4"/>
-      </tp>
-      <tp>
-        <v>1</v>
-        <stp/>
-        <stp>5f50dafc-460c-4064-833d-a02370dd9c49</stp>
-        <tr r="G21" s="4"/>
-      </tp>
-      <tp>
-        <v>1</v>
-        <stp/>
-        <stp>bcbafea3-e434-44bc-be00-e66713672c7e</stp>
-        <tr r="G50" s="1"/>
-      </tp>
-      <tp>
-        <v>1</v>
-        <stp/>
-        <stp>a1062289-db09-428b-8629-af3da22f05da</stp>
-        <tr r="G54" s="1"/>
-      </tp>
-    </main>
-    <main first="rtdsrv.4b8ef99e016b447da4df1f9adeb95e96">
-      <tp>
-        <v>1</v>
-        <stp/>
-        <stp>707587d9-6fc6-4bc9-9b16-c8ffd6afbafd</stp>
-        <tr r="G43" s="4"/>
-      </tp>
-      <tp>
-        <v>1</v>
-        <stp/>
-        <stp>e18d8c9e-c7ef-4783-8616-b9c95aaafb8b</stp>
-        <tr r="G42" s="4"/>
-      </tp>
-      <tp>
-        <v>1</v>
-        <stp/>
-        <stp>d6663a89-5a23-4a77-ab92-71ebb7412c5d</stp>
-        <tr r="G49" s="4"/>
-      </tp>
-      <tp>
-        <v>1</v>
-        <stp/>
-        <stp>286aafc8-7969-4e4a-8158-37f692fa413a</stp>
-        <tr r="F6" s="1"/>
-      </tp>
-    </main>
-    <main first="rtdsrv.4b8ef99e016b447da4df1f9adeb95e96">
-      <tp>
-        <v>1</v>
-        <stp/>
-        <stp>b422dca2-8e2c-4b43-9da5-ba427a1f059b</stp>
-        <tr r="I19" s="1"/>
-      </tp>
-      <tp>
-        <v>1</v>
-        <stp/>
-        <stp>973f232f-a5fe-4d22-87e0-492d5091f33a</stp>
-        <tr r="G52" s="4"/>
-      </tp>
-      <tp>
-        <v>1</v>
-        <stp/>
-        <stp>dfc230f6-10a5-4eda-aa34-c9b742da8661</stp>
-        <tr r="G22" s="1"/>
-      </tp>
-      <tp>
-        <v>1</v>
-        <stp/>
-        <stp>0168d52e-0b73-4b49-998d-c7f218970209</stp>
-        <tr r="G48" s="1"/>
-      </tp>
-    </main>
-    <main first="rtdsrv.4b8ef99e016b447da4df1f9adeb95e96">
-      <tp>
-        <v>1</v>
-        <stp/>
-        <stp>b4d8df59-58b8-4ca4-831e-c49829f09db5</stp>
-        <tr r="G46" s="1"/>
-      </tp>
-      <tp>
-        <v>1</v>
-        <stp/>
-        <stp>e86b73fe-6b46-4c47-8271-abf34dc84018</stp>
-        <tr r="G30" s="1"/>
-      </tp>
-      <tp>
-        <v>1</v>
-        <stp/>
-        <stp>417fc574-e091-4fdb-a48d-f67ad5e8c32e</stp>
-        <tr r="G45" s="1"/>
-      </tp>
-      <tp>
-        <v>1</v>
-        <stp/>
-        <stp>865af7e0-1550-485c-b1a5-218d1075a9da</stp>
-        <tr r="G37" s="1"/>
-      </tp>
-      <tp>
-        <v>1</v>
-        <stp/>
-        <stp>76b07320-f83c-4689-894b-6c28860fe15b</stp>
-        <tr r="G36" s="1"/>
-      </tp>
-    </main>
-    <main first="rtdsrv.4b8ef99e016b447da4df1f9adeb95e96">
-      <tp>
-        <v>1</v>
-        <stp/>
-        <stp>6b449903-bc31-4f60-95aa-7dc19c10ee4e</stp>
-        <tr r="G57" s="4"/>
-      </tp>
-    </main>
-    <main first="rtdsrv.4b8ef99e016b447da4df1f9adeb95e96">
-      <tp>
-        <v>1</v>
-        <stp/>
-        <stp>ea1c0135-b590-4337-8ab2-961da8091d6b</stp>
-        <tr r="G39" s="1"/>
-      </tp>
-    </main>
-    <main first="rtdsrv.4b8ef99e016b447da4df1f9adeb95e96">
-      <tp>
-        <v>1</v>
-        <stp/>
-        <stp>939e3515-f4df-4f0b-b75c-65eb29c357c5</stp>
-        <tr r="I28" s="4"/>
-      </tp>
-    </main>
-    <main first="rtdsrv.4b8ef99e016b447da4df1f9adeb95e96">
-      <tp>
-        <v>1</v>
-        <stp/>
-        <stp>fc7bacc0-7b10-4c5a-ac91-a0d0be715610</stp>
-        <tr r="G46" s="4"/>
-      </tp>
-    </main>
-    <main first="rtdsrv.4b8ef99e016b447da4df1f9adeb95e96">
-      <tp>
-        <v>1</v>
-        <stp/>
-        <stp>36e58f36-0b31-4d70-8478-59c7f352eb23</stp>
-        <tr r="G19" s="4"/>
-      </tp>
-    </main>
-    <main first="rtdsrv.4b8ef99e016b447da4df1f9adeb95e96">
-      <tp>
-        <v>1</v>
-        <stp/>
-        <stp>a27287b1-9ad8-4cdd-a84f-9163a71d1d9f</stp>
-        <tr r="G56" s="4"/>
-      </tp>
-      <tp>
-        <v>1</v>
-        <stp/>
-        <stp>4f4f6569-5531-4084-8239-b724ae377229</stp>
-        <tr r="G35" s="1"/>
-      </tp>
-      <tp>
-        <v>1</v>
-        <stp/>
-        <stp>d686cd8e-4bda-4864-a9a4-8fec273e7c27</stp>
-        <tr r="G29" s="4"/>
-      </tp>
-      <tp>
-        <v>1</v>
-        <stp/>
-        <stp>bb76ab39-1507-4cd5-8ffc-5a599d4b8f8e</stp>
-        <tr r="G50" s="4"/>
-      </tp>
-      <tp>
-        <v>1</v>
-        <stp/>
-        <stp>737fdd70-fa54-4068-bb99-a5a3dbd02f5a</stp>
-        <tr r="G44" s="1"/>
-      </tp>
-      <tp>
-        <v>1</v>
-        <stp/>
-        <stp>9319eabb-8ddd-43c6-9111-e02b98c07d5e</stp>
-        <tr r="G44" s="4"/>
-      </tp>
-      <tp>
-        <v>1</v>
-        <stp/>
-        <stp>bebc2de1-60ea-40bb-8a46-521efe0f458e</stp>
-        <tr r="G41" s="1"/>
-      </tp>
-      <tp>
-        <v>1</v>
-        <stp/>
-        <stp>29f95f6a-8c35-4d6b-9c18-f67c942ba582</stp>
+        <stp>db3a0ca7-52e1-4b1f-8b6e-1391133a786f</stp>
+        <tr r="E4" s="3"/>
+      </tp>
+      <tp>
+        <v>1</v>
+        <stp/>
+        <stp>ca953b95-c8cc-4728-8e32-5181bc039e00</stp>
         <tr r="G22" s="4"/>
-      </tp>
-      <tp>
-        <v>1</v>
-        <stp/>
-        <stp>21f26eb4-332f-4579-a19f-7b05db019d10</stp>
-        <tr r="E4" s="3"/>
-      </tp>
-      <tp>
-        <v>1</v>
-        <stp/>
-        <stp>45f70452-a4c1-48af-8087-beebc9e9fa7e</stp>
-        <tr r="G38" s="4"/>
-      </tp>
-      <tp>
-        <v>1</v>
-        <stp/>
-        <stp>cb75bec1-4e61-4348-b7c1-7d0d579e9979</stp>
-        <tr r="G26" s="1"/>
-      </tp>
-    </main>
-    <main first="rtdsrv.4b8ef99e016b447da4df1f9adeb95e96">
-      <tp>
-        <v>1</v>
-        <stp/>
-        <stp>d40bbdc3-504c-43f0-a54d-e58652259d10</stp>
-        <tr r="G34" s="1"/>
-      </tp>
-      <tp>
-        <v>1</v>
-        <stp/>
-        <stp>000049d3-ca0c-4109-a973-0713aa7ad004</stp>
-        <tr r="G23" s="1"/>
-      </tp>
-      <tp>
-        <v>101</v>
-        <stp/>
-        <stp>a0770d64-0cc0-4d63-a9c0-72192be5bf75</stp>
-        <tr r="E7" s="3"/>
-      </tp>
-      <tp>
-        <v>1</v>
-        <stp/>
-        <stp>9f0b6f53-f245-405d-83f1-d57507822dbc</stp>
-        <tr r="I19" s="4"/>
-      </tp>
-      <tp>
-        <v>1</v>
-        <stp/>
-        <stp>6e91c3b5-e1e9-4efe-93bb-46c26a0a6a2c</stp>
-        <tr r="G51" s="1"/>
-      </tp>
-      <tp>
-        <v>1</v>
-        <stp/>
-        <stp>f91acaf9-ab77-44af-9389-6eef20a9a0ac</stp>
-        <tr r="G53" s="4"/>
-      </tp>
-    </main>
-    <main first="rtdsrv.4b8ef99e016b447da4df1f9adeb95e96">
-      <tp>
-        <v>1</v>
-        <stp/>
-        <stp>1e20d4de-2006-41bf-9f80-48b93da56c4b</stp>
-        <tr r="G23" s="4"/>
-      </tp>
-      <tp>
-        <v>1</v>
-        <stp/>
-        <stp>ce261162-24ce-4c6d-a0ab-2cd83d335a7c</stp>
-        <tr r="G34" s="4"/>
-      </tp>
-      <tp>
-        <v>1</v>
-        <stp/>
-        <stp>1fe8571a-1322-4957-a257-27722b06f2ec</stp>
-        <tr r="F1" s="4"/>
-      </tp>
-      <tp>
-        <v>1</v>
-        <stp/>
-        <stp>6ab7d9c1-044d-4c95-8eee-209aa8eda5dc</stp>
-        <tr r="G32" s="4"/>
-      </tp>
-    </main>
-    <main first="rtdsrv.4b8ef99e016b447da4df1f9adeb95e96">
-      <tp>
-        <v>1</v>
-        <stp/>
-        <stp>50a5dade-ed33-482e-a207-4ac937b8d260</stp>
-        <tr r="G43" s="1"/>
-      </tp>
-      <tp>
-        <v>1</v>
-        <stp/>
-        <stp>9b1b9ee4-4a7f-4a10-9faf-e205c6243c5a</stp>
-        <tr r="G33" s="1"/>
-      </tp>
-      <tp>
-        <v>1</v>
-        <stp/>
-        <stp>10487dcd-ca18-4168-91ef-9969c4be5c62</stp>
-        <tr r="G29" s="1"/>
-      </tp>
-    </main>
-    <main first="rtdsrv.4b8ef99e016b447da4df1f9adeb95e96">
-      <tp>
-        <v>1</v>
-        <stp/>
-        <stp>68817488-5a6f-4517-8f05-abe5eae029a3</stp>
-        <tr r="G55" s="4"/>
-      </tp>
-    </main>
-    <main first="rtdsrv.4b8ef99e016b447da4df1f9adeb95e96">
-      <tp>
-        <v>1</v>
-        <stp/>
-        <stp>5dd97d21-88d3-495d-a3ec-ab00bd0b884d</stp>
-        <tr r="F1" s="1"/>
-      </tp>
-    </main>
-    <main first="rtdsrv.4b8ef99e016b447da4df1f9adeb95e96">
-      <tp>
-        <v>1</v>
-        <stp/>
-        <stp>ec33074b-202c-4cda-8fd4-da68ad1c0a3f</stp>
-        <tr r="I28" s="1"/>
-      </tp>
-    </main>
-    <main first="rtdsrv.4b8ef99e016b447da4df1f9adeb95e96">
-      <tp>
-        <v>1</v>
-        <stp/>
-        <stp>2ed72686-3229-4c7b-9b5a-2dabef48625d</stp>
-        <tr r="G28" s="1"/>
-      </tp>
-      <tp>
-        <v>1</v>
-        <stp/>
-        <stp>ad36159f-d95a-408b-a01c-a0ad60f46a87</stp>
-        <tr r="G40" s="1"/>
-      </tp>
-      <tp>
-        <v>1</v>
-        <stp/>
-        <stp>3b855b64-7082-46e7-9617-789a87d58986</stp>
-        <tr r="G54" s="4"/>
-      </tp>
-    </main>
-    <main first="rtdsrv.4b8ef99e016b447da4df1f9adeb95e96">
-      <tp>
-        <v>1</v>
-        <stp/>
-        <stp>4fca72d5-313d-4a80-ac8b-cde084ac485b</stp>
-        <tr r="G39" s="4"/>
-      </tp>
-    </main>
-    <main first="rtdsrv.4b8ef99e016b447da4df1f9adeb95e96">
-      <tp>
-        <v>1</v>
-        <stp/>
-        <stp>a28a91ab-2972-417f-8575-1cd8af371c3f</stp>
-        <tr r="G48" s="4"/>
-      </tp>
-    </main>
-    <main first="rtdsrv.4b8ef99e016b447da4df1f9adeb95e96">
-      <tp>
-        <v>1</v>
-        <stp/>
-        <stp>ca9757e3-7740-4471-bd1f-59b2b8403f6c</stp>
-        <tr r="G55" s="1"/>
       </tp>
     </main>
   </volType>
@@ -1471,11 +1577,11 @@
       </c>
       <c r="F1" t="str" cm="1">
         <f t="array" ref="F1">_xll.ExLibris.Json.CreateJsonObject(E3:F6)</f>
-        <v>JsonObject:BE1FC4FB-547E-4869-A7F0-521890319C3A</v>
+        <v>JsonObject:D9546E1A-85CD-4E6B-9AF3-523AE7DBD289</v>
       </c>
       <c r="K1" t="str">
         <f>EXLIBRIS_CONFIGURATION</f>
-        <v>ExLibris.Core.ExLibrisConfiguration:78976E74-B484-403F-9AE1-F5D51D57D63F</v>
+        <v>ExLibris.Core.ExLibrisConfiguration:4C2DB07D-02CB-4C76-9A7E-AE031E5570ED</v>
       </c>
     </row>
     <row r="2" spans="2:25" x14ac:dyDescent="0.4">
@@ -1545,7 +1651,7 @@
       </c>
       <c r="F6" t="str" cm="1">
         <f t="array" ref="F6">_xll.ExLibris.Json.CreateJsonArray(E8:J14)</f>
-        <v>JsonObject:7FD63C57-393E-49CA-A58E-C4F2225A9BAA</v>
+        <v>JsonObject:D595CB16-7EE7-48F3-B7F5-1DC76697DC3E</v>
       </c>
       <c r="L6" t="s">
         <v>68</v>
@@ -1770,7 +1876,7 @@
       </c>
       <c r="I19" t="str" cm="1">
         <f t="array" ref="I19">_xll.ExLibris.Json.GetJsonValue(F1,E6)</f>
-        <v>JsonObject:854737B1-0B9E-4F70-9A82-B16823CD8333</v>
+        <v>JsonObject:F5BA49B4-54BA-482E-BB40-1CCA69ED4A88</v>
       </c>
       <c r="P19" t="s">
         <v>14</v>
@@ -2492,7 +2598,7 @@
       </c>
       <c r="I28" t="str" cm="1">
         <f t="array" ref="I28">_xll.ExLibris.Json.GetJsonValue(I19,"[2]")</f>
-        <v>JsonObject:1676224C-EAA0-4A14-9F89-A758F8BDAE9D</v>
+        <v>JsonObject:CEF2AE64-4D67-41FA-ACD8-1DF0DFF2AAA0</v>
       </c>
       <c r="P28" t="s">
         <v>38</v>
@@ -3628,11 +3734,11 @@
       </c>
       <c r="F1" t="str" cm="1">
         <f t="array" ref="F1">_xll.ExLibris.Json.CreateJsonObject(E3:F6, EXLIBRIS_CONFIGURATION)</f>
-        <v>JsonObject:503E7613-4E07-4006-B2A7-CB6401DF8B02</v>
+        <v>JsonObject:4E0DA391-E32A-4907-87DB-4ACB7798D168</v>
       </c>
       <c r="K1" t="str">
         <f>EXLIBRIS_CONFIGURATION</f>
-        <v>ExLibris.Core.ExLibrisConfiguration:78976E74-B484-403F-9AE1-F5D51D57D63F</v>
+        <v>ExLibris.Core.ExLibrisConfiguration:4C2DB07D-02CB-4C76-9A7E-AE031E5570ED</v>
       </c>
     </row>
     <row r="2" spans="2:25" x14ac:dyDescent="0.4">
@@ -3702,7 +3808,7 @@
       </c>
       <c r="F6" t="str" cm="1">
         <f t="array" ref="F6">_xll.ExLibris.Json.CreateJsonArray(E8:J14, EXLIBRIS_CONFIGURATION)</f>
-        <v>JsonObject:16334072-DD2A-4369-8330-48716197076D</v>
+        <v>JsonObject:1160F4EE-5F11-4DFA-8155-76BE404E3252</v>
       </c>
       <c r="L6" t="s">
         <v>68</v>
@@ -3927,7 +4033,7 @@
       </c>
       <c r="I19" t="str" cm="1">
         <f t="array" ref="I19">_xll.ExLibris.Json.GetJsonValue(F1,E6, EXLIBRIS_CONFIGURATION)</f>
-        <v>JsonObject:CF6400C5-7AED-47FD-98B7-BD0CD6EEF736</v>
+        <v>JsonObject:632DADF0-F7D3-4231-A0E3-06B44F2048FD</v>
       </c>
       <c r="P19" t="s">
         <v>14</v>
@@ -4649,7 +4755,7 @@
       </c>
       <c r="I28" t="str" cm="1">
         <f t="array" ref="I28">_xll.ExLibris.Json.GetJsonValue(I19,"[2]", EXLIBRIS_CONFIGURATION)</f>
-        <v>JsonObject:391EFAB2-D899-4E8E-B0E6-36E35FB16A7E</v>
+        <v>JsonObject:BC8324FF-7E00-485C-86D8-1B4C5ED69517</v>
       </c>
       <c r="P28" t="s">
         <v>38</v>
@@ -5760,7 +5866,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C0D3ACF1-D52B-4405-9E6D-D2579DCD0199}">
-  <dimension ref="B2:E15"/>
+  <dimension ref="B2:E28"/>
   <sheetFormatPr defaultRowHeight="18.75" x14ac:dyDescent="0.4"/>
   <cols>
     <col min="1" max="1" width="2.25" customWidth="1"/>
@@ -5779,8 +5885,8 @@
         <v>111</v>
       </c>
       <c r="E4" t="str" cm="1">
-        <f t="array" ref="E4">_xll.ExLibris.WebSockets.OpenWebSocket("ws://localhost:10101",D4)</f>
-        <v>ExLibris.Core.WebSockets.WebsocketClient:AF651CF1-1F52-4171-B6DA-EE452997DBD2</v>
+        <f t="array" ref="E4">_xll.ExLibris.WebSockets.OpenWebSocket("ws://localhost:10101",,D4)</f>
+        <v>ExLibris.Core.WebSockets.WebsocketClient:D7607EC4-3BC7-4E96-9A35-B113B197CBB7</v>
       </c>
     </row>
     <row r="6" spans="2:5" x14ac:dyDescent="0.4">
@@ -5789,79 +5895,169 @@
       </c>
       <c r="E6" t="str" cm="1">
         <f t="array" ref="E6">_xll.ExLibris.WebSockets.ObserveWebSocketStatus(E4,1000)</f>
-        <v>Open</v>
+        <v>Closed</v>
       </c>
     </row>
     <row r="7" spans="2:5" x14ac:dyDescent="0.4">
       <c r="D7" t="s">
         <v>103</v>
       </c>
-      <c r="E7" t="str" cm="1">
+      <c r="E7" t="e" cm="1">
         <f t="array" ref="E7">_xll.ExLibris.WebSockets.ObserveWebSocketMessage(E4)</f>
-        <v>push_event 22:04:25</v>
+        <v>#N/A</v>
       </c>
     </row>
     <row r="9" spans="2:5" x14ac:dyDescent="0.4">
       <c r="D9" t="s">
         <v>104</v>
       </c>
-      <c r="E9" t="str" cm="1">
+      <c r="E9" t="e" cm="1">
         <f t="array" ref="E9">_xll.ExLibris.WebSockets.SendWebSocketMessage(E4,"test "&amp;D9,E6="Open")</f>
-        <v>message sent : 2021-09-20T10:01:04.926</v>
+        <v>#N/A</v>
       </c>
     </row>
     <row r="10" spans="2:5" x14ac:dyDescent="0.4">
       <c r="D10" t="s">
         <v>105</v>
       </c>
-      <c r="E10" t="str" cm="1">
+      <c r="E10" t="e" cm="1">
         <f t="array" ref="E10">_xll.ExLibris.WebSockets.SendWebSocketMessage($E$4,"test next "&amp;D10,E9)</f>
-        <v>message sent : 2021-09-20T10:01:04.927</v>
+        <v>#N/A</v>
       </c>
     </row>
     <row r="11" spans="2:5" x14ac:dyDescent="0.4">
       <c r="D11" t="s">
         <v>106</v>
       </c>
-      <c r="E11" t="str" cm="1">
+      <c r="E11" t="e" cm="1">
         <f t="array" ref="E11">_xll.ExLibris.WebSockets.SendWebSocketMessage($E$4,"test next "&amp;D11,E10)</f>
-        <v>message sent : 2021-09-20T10:01:04.931</v>
+        <v>#N/A</v>
       </c>
     </row>
     <row r="12" spans="2:5" x14ac:dyDescent="0.4">
       <c r="D12" t="s">
         <v>107</v>
       </c>
-      <c r="E12" t="str" cm="1">
+      <c r="E12" t="e" cm="1">
         <f t="array" ref="E12">_xll.ExLibris.WebSockets.SendWebSocketMessage($E$4,"test next "&amp;D12,E11)</f>
-        <v>message sent : 2021-09-20T10:01:04.932</v>
+        <v>#N/A</v>
       </c>
     </row>
     <row r="13" spans="2:5" x14ac:dyDescent="0.4">
       <c r="D13" t="s">
         <v>108</v>
       </c>
-      <c r="E13" t="str" cm="1">
+      <c r="E13" t="e" cm="1">
         <f t="array" ref="E13">_xll.ExLibris.WebSockets.SendWebSocketMessage($E$4,"test next "&amp;D13,E12)</f>
-        <v>message sent : 2021-09-20T10:01:04.946</v>
+        <v>#N/A</v>
       </c>
     </row>
     <row r="14" spans="2:5" x14ac:dyDescent="0.4">
       <c r="D14" t="s">
         <v>109</v>
       </c>
-      <c r="E14" t="str" cm="1">
+      <c r="E14" t="e" cm="1">
         <f t="array" ref="E14">_xll.ExLibris.WebSockets.SendWebSocketMessage($E$4,"test next "&amp;D14,E13)</f>
-        <v>message sent : 2021-09-20T10:01:04.946</v>
+        <v>#N/A</v>
       </c>
     </row>
     <row r="15" spans="2:5" x14ac:dyDescent="0.4">
       <c r="D15" t="s">
         <v>110</v>
       </c>
-      <c r="E15" t="str" cm="1">
+      <c r="E15" t="e" cm="1">
         <f t="array" ref="E15">_xll.ExLibris.WebSockets.SendWebSocketMessage($E$4,"test next "&amp;D15,E14)</f>
-        <v>message sent : 2021-09-20T10:01:04.947</v>
+        <v>#N/A</v>
+      </c>
+    </row>
+    <row r="17" spans="4:5" x14ac:dyDescent="0.4">
+      <c r="D17" t="s">
+        <v>113</v>
+      </c>
+      <c r="E17" t="str" cm="1">
+        <f t="array" ref="E17">_xll.ExLibris.WebSockets.OpenWebSocket("ws://localhost:10101",,D17)</f>
+        <v>ExLibris.Core.WebSockets.WebsocketClient:90B5A407-38E2-420E-9E87-435302544694</v>
+      </c>
+    </row>
+    <row r="19" spans="4:5" x14ac:dyDescent="0.4">
+      <c r="D19" t="s">
+        <v>102</v>
+      </c>
+      <c r="E19" t="str" cm="1">
+        <f t="array" ref="E19">_xll.ExLibris.WebSockets.ObserveWebSocketStatus(E17,1000)</f>
+        <v>Closed</v>
+      </c>
+    </row>
+    <row r="20" spans="4:5" x14ac:dyDescent="0.4">
+      <c r="D20" t="s">
+        <v>103</v>
+      </c>
+      <c r="E20" t="str" cm="1">
+        <f t="array" ref="E20">_xll.ExLibris.WebSockets.ObserveWebSocketMessage(E17)</f>
+        <v>push_event 22:36:20</v>
+      </c>
+    </row>
+    <row r="22" spans="4:5" x14ac:dyDescent="0.4">
+      <c r="D22" t="s">
+        <v>104</v>
+      </c>
+      <c r="E22" t="e" cm="1">
+        <f t="array" ref="E22">_xll.ExLibris.WebSockets.SendWebSocketMessage(E17,"test "&amp;D22,E19="Open")</f>
+        <v>#N/A</v>
+      </c>
+    </row>
+    <row r="23" spans="4:5" x14ac:dyDescent="0.4">
+      <c r="D23" t="s">
+        <v>105</v>
+      </c>
+      <c r="E23" t="e" cm="1">
+        <f t="array" ref="E23">_xll.ExLibris.WebSockets.SendWebSocketMessage($E$4,"test next "&amp;D23,E22)</f>
+        <v>#N/A</v>
+      </c>
+    </row>
+    <row r="24" spans="4:5" x14ac:dyDescent="0.4">
+      <c r="D24" t="s">
+        <v>106</v>
+      </c>
+      <c r="E24" t="e" cm="1">
+        <f t="array" ref="E24">_xll.ExLibris.WebSockets.SendWebSocketMessage($E$4,"test next "&amp;D24,E23)</f>
+        <v>#N/A</v>
+      </c>
+    </row>
+    <row r="25" spans="4:5" x14ac:dyDescent="0.4">
+      <c r="D25" t="s">
+        <v>107</v>
+      </c>
+      <c r="E25" t="e" cm="1">
+        <f t="array" ref="E25">_xll.ExLibris.WebSockets.SendWebSocketMessage($E$4,"test next "&amp;D25,E24)</f>
+        <v>#N/A</v>
+      </c>
+    </row>
+    <row r="26" spans="4:5" x14ac:dyDescent="0.4">
+      <c r="D26" t="s">
+        <v>108</v>
+      </c>
+      <c r="E26" t="e" cm="1">
+        <f t="array" ref="E26">_xll.ExLibris.WebSockets.SendWebSocketMessage($E$4,"test next "&amp;D26,E25)</f>
+        <v>#N/A</v>
+      </c>
+    </row>
+    <row r="27" spans="4:5" x14ac:dyDescent="0.4">
+      <c r="D27" t="s">
+        <v>109</v>
+      </c>
+      <c r="E27" t="e" cm="1">
+        <f t="array" ref="E27">_xll.ExLibris.WebSockets.SendWebSocketMessage($E$4,"test next "&amp;D27,E26)</f>
+        <v>#N/A</v>
+      </c>
+    </row>
+    <row r="28" spans="4:5" x14ac:dyDescent="0.4">
+      <c r="D28" t="s">
+        <v>110</v>
+      </c>
+      <c r="E28" t="e" cm="1">
+        <f t="array" ref="E28">_xll.ExLibris.WebSockets.SendWebSocketMessage($E$4,"test next "&amp;D28,E27)</f>
+        <v>#N/A</v>
       </c>
     </row>
   </sheetData>
@@ -5888,7 +6084,7 @@
       </c>
       <c r="C2" t="str" cm="1">
         <f t="array" ref="C2">_xll.ExLibris.LoadConfiguration(B6:C15)</f>
-        <v>ExLibris.Core.ExLibrisConfiguration:78976E74-B484-403F-9AE1-F5D51D57D63F</v>
+        <v>ExLibris.Core.ExLibrisConfiguration:4C2DB07D-02CB-4C76-9A7E-AE031E5570ED</v>
       </c>
     </row>
     <row r="4" spans="2:6" s="4" customFormat="1" ht="18" x14ac:dyDescent="0.4">

</xml_diff>

<commit_message>
search elements from json array
</commit_message>
<xml_diff>
--- a/ExLibris/test_excel/exlibris_test.xlsx
+++ b/ExLibris/test_excel/exlibris_test.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\mugen\git\ex-libris\ExLibris\test_excel\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{52877A10-F1B3-45C7-B3B3-63F3316701B7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A09AF23E-B13E-4D3F-AA6B-2751D4DADB9A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{705CD0B7-27A9-4291-85BD-6034C0FEE3E4}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" activeTab="1" xr2:uid="{705CD0B7-27A9-4291-85BD-6034C0FEE3E4}"/>
   </bookViews>
   <sheets>
     <sheet name="json_test" sheetId="1" r:id="rId1"/>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/metadata.xml><?xml version="1.0" encoding="utf-8"?>
-<metadata xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xda="http://schemas.microsoft.com/office/spreadsheetml/2017/dynamicarray">
+<metadata xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xlrd="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata" xmlns:xda="http://schemas.microsoft.com/office/spreadsheetml/2017/dynamicarray">
   <metadataTypes count="1">
     <metadataType name="XLDAPR" minSupportedVersion="120000" copy="1" pasteAll="1" pasteValues="1" merge="1" splitFirst="1" rowColShift="1" clearFormats="1" clearComments="1" assign="1" coerce="1" cellMeta="1"/>
   </metadataTypes>
@@ -62,7 +62,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="379" uniqueCount="116">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="407" uniqueCount="120">
   <si>
     <t>payment _date</t>
   </si>
@@ -394,9 +394,6 @@
     <t>2024-08-28</t>
   </si>
   <si>
-    <t>{"trade_code":"money_00001","couter_party":"CP00001","fixed_leg":{"pay_or_recieve":"Receive","cashflows":[{"payment _date":"2022-03-12","start_date":"2021-09-13","end_date":"2022-03-12","day_count_type":"ACT/360","amout":10000000,"fixed_rate":0.001},{"payment _date":"2022-09-08","start_date":"2022-03-12","end_date":"2022-09-08","day_count_type":"ACT/360","amout":11000000,"fixed_rate":0.001},{"payment _date":"2023-03-07","start_date":"2022-09-08","end_date":"2023-03-07","day_count_type":"ACT/360","amout":12000000,"fixed_rate":0.001},{"payment _date":"2023-09-03","start_date":"2023-03-07","end_date":"2023-09-03","day_count_type":"ACT/360","amout":13000000,"fixed_rate":0.001},{"payment _date":"2024-03-01","start_date":"2023-09-03","end_date":"2024-03-01","day_count_type":"ACT/360","amout":14000000,"fixed_rate":0.001},{"payment _date":"2024-08-28","start_date":"2024-03-01","end_date":"2024-08-28","day_count_type":"ACT/360","amout":15000000,"fixed_rate":0.001}]}}</t>
-  </si>
-  <si>
     <t>client</t>
     <phoneticPr fontId="1"/>
   </si>
@@ -447,6 +444,24 @@
   </si>
   <si>
     <t>table3</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>{"trade_code":"money_00001","couter_party":"CP00001","fixed_leg":{"pay_or_recieve":"Receive","cashflows":[{"payment _date":"2022-03-12","start_date":"2021-09-13","end_date":"2022-03-12","day_count_type":"ACT/360","amout":10000000,"fixed_rate":0.001},{"payment _date":"2022-09-08","start_date":"2022-03-12","end_date":"2022-09-08","day_count_type":"ACT/360","amout":10000000,"fixed_rate":0.0011},{"payment _date":"2023-03-07","start_date":"2022-09-08","end_date":"2023-03-07","day_count_type":"ACT/360","amout":11000000,"fixed_rate":0.0012000000000000001},{"payment _date":"2023-09-03","start_date":"2023-03-07","end_date":"2023-09-03","day_count_type":"ACT/360","amout":11000000,"fixed_rate":0.0013000000000000002},{"payment _date":"2024-03-01","start_date":"2023-09-03","end_date":"2024-03-01","day_count_type":"ACT/360","amout":12000000,"fixed_rate":0.0014000000000000002},{"payment _date":"2024-08-28","start_date":"2024-03-01","end_date":"2024-08-28","day_count_type":"ACT/360","amout":12000000,"fixed_rate":0.0015000000000000002}]}}</t>
+  </si>
+  <si>
+    <t/>
+  </si>
+  <si>
+    <t>search</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>search1</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>search2</t>
     <phoneticPr fontId="1"/>
   </si>
 </sst>
@@ -553,660 +568,695 @@
 <file path=xl/volatileDependencies.xml><?xml version="1.0" encoding="utf-8"?>
 <volTypes xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <volType type="realTimeData">
-    <main first="rtdsrv.4f71aace325a499b836bfd0f6b877e4c">
-      <tp>
-        <v>1</v>
-        <stp/>
-        <stp>8b266871-b605-451c-9340-96dd10bd8976</stp>
+    <main first="rtdsrv.0283c6361b6f4b11963d8af96e32e10b">
+      <tp>
+        <v>1</v>
+        <stp/>
+        <stp>0a5b767d-2c0d-4667-b21e-681ebdb69761</stp>
+        <tr r="G37" s="4"/>
+      </tp>
+      <tp>
+        <v>1</v>
+        <stp/>
+        <stp>79bb9cc5-ab9d-4b90-98b1-c384a6508df6</stp>
+        <tr r="G32" s="4"/>
+      </tp>
+      <tp>
+        <v>1</v>
+        <stp/>
+        <stp>2c075992-a4a9-4c1d-81a2-293828bca7ac</stp>
+        <tr r="G35" s="1"/>
+      </tp>
+    </main>
+    <main first="rtdsrv.0283c6361b6f4b11963d8af96e32e10b">
+      <tp>
+        <v>1</v>
+        <stp/>
+        <stp>9d75c974-4696-4850-a778-5110e5d04c69</stp>
+        <tr r="G48" s="1"/>
+      </tp>
+    </main>
+    <main first="rtdsrv.0283c6361b6f4b11963d8af96e32e10b">
+      <tp>
+        <v>1</v>
+        <stp/>
+        <stp>11c4a480-bf05-44ff-b422-afa33e54f953</stp>
+        <tr r="G41" s="4"/>
+      </tp>
+    </main>
+    <main first="rtdsrv.0283c6361b6f4b11963d8af96e32e10b">
+      <tp>
+        <v>1</v>
+        <stp/>
+        <stp>71964b75-97bb-48e6-814e-fd6edf65ecfd</stp>
+        <tr r="G35" s="4"/>
+      </tp>
+      <tp>
+        <v>1</v>
+        <stp/>
+        <stp>ad9d6985-9ef3-471f-848b-d4b2e5ccf264</stp>
+        <tr r="G20" s="1"/>
+      </tp>
+      <tp>
+        <v>1</v>
+        <stp/>
+        <stp>1a26cff1-62dd-46a9-bc02-da6ee3c2ec2d</stp>
+        <tr r="G56" s="1"/>
+      </tp>
+    </main>
+    <main first="rtdsrv.0283c6361b6f4b11963d8af96e32e10b">
+      <tp>
+        <v>1</v>
+        <stp/>
+        <stp>494cb52c-09ee-451d-9707-bdab376cb11f</stp>
+        <tr r="G45" s="1"/>
+      </tp>
+    </main>
+    <main first="rtdsrv.0283c6361b6f4b11963d8af96e32e10b">
+      <tp>
+        <v>1</v>
+        <stp/>
+        <stp>a7fc733b-4306-47f1-b303-91a0733bd96e</stp>
+        <tr r="G24" s="4"/>
+      </tp>
+    </main>
+    <main first="rtdsrv.0283c6361b6f4b11963d8af96e32e10b">
+      <tp>
+        <v>1</v>
+        <stp/>
+        <stp>5e89c57d-823d-40ee-803b-ee158b0ad298</stp>
+        <tr r="G23" s="4"/>
+      </tp>
+    </main>
+    <main first="rtdsrv.0283c6361b6f4b11963d8af96e32e10b">
+      <tp>
+        <v>1</v>
+        <stp/>
+        <stp>9e19ad3e-8ac7-4540-a626-24556bba9f46</stp>
+        <tr r="G38" s="1"/>
+      </tp>
+      <tp>
+        <v>1</v>
+        <stp/>
+        <stp>50f7d0ee-ed0a-4314-8706-0a90d5e3f9d4</stp>
+        <tr r="G52" s="4"/>
+      </tp>
+      <tp>
+        <v>1</v>
+        <stp/>
+        <stp>eab1819a-b8ac-4b37-8420-c97e9d574f97</stp>
+        <tr r="G55" s="4"/>
+      </tp>
+    </main>
+    <main first="rtdsrv.0283c6361b6f4b11963d8af96e32e10b">
+      <tp>
+        <v>1</v>
+        <stp/>
+        <stp>ba63b3ea-c5d4-457c-aa45-bb2ac9fb61ef</stp>
+        <tr r="G47" s="4"/>
+      </tp>
+      <tp>
+        <v>1</v>
+        <stp/>
+        <stp>df270489-bf85-4e88-9ec6-21b4203c1f13</stp>
+        <tr r="G49" s="1"/>
+      </tp>
+    </main>
+    <main first="rtdsrv.0283c6361b6f4b11963d8af96e32e10b">
+      <tp>
+        <v>1</v>
+        <stp/>
+        <stp>576c96bd-78ac-4139-8ff4-6e3bc28a92f0</stp>
+        <tr r="C2" s="2"/>
+      </tp>
+    </main>
+    <main first="rtdsrv.0283c6361b6f4b11963d8af96e32e10b">
+      <tp>
+        <v>1</v>
+        <stp/>
+        <stp>80ea02ff-4bf0-4ce4-8769-aef7c93d8e5b</stp>
+        <tr r="I28" s="4"/>
+      </tp>
+    </main>
+    <main first="rtdsrv.0283c6361b6f4b11963d8af96e32e10b">
+      <tp>
+        <v>1</v>
+        <stp/>
+        <stp>f72b93fc-57da-4a79-8c8d-1d0eac79d898</stp>
+        <tr r="G46" s="4"/>
+      </tp>
+    </main>
+    <main first="rtdsrv.0283c6361b6f4b11963d8af96e32e10b">
+      <tp>
+        <v>1</v>
+        <stp/>
+        <stp>9cf72df3-cfa0-496d-9f52-f558b698c9bf</stp>
+        <tr r="I28" s="1"/>
+      </tp>
+      <tp>
+        <v>1</v>
+        <stp/>
+        <stp>a69edd2b-5938-4346-941a-536bbda6083c</stp>
+        <tr r="G53" s="1"/>
+      </tp>
+    </main>
+    <main first="rtdsrv.0283c6361b6f4b11963d8af96e32e10b">
+      <tp>
+        <v>139</v>
+        <stp/>
+        <stp>e1927053-d5ef-4d92-b827-bad9a722f355</stp>
+        <tr r="E20" s="3"/>
+      </tp>
+      <tp>
+        <v>1</v>
+        <stp/>
+        <stp>24ae9bbb-adb5-46e7-9cdc-ea5ef0d95525</stp>
+        <tr r="G22" s="1"/>
+      </tp>
+    </main>
+    <main first="rtdsrv.0283c6361b6f4b11963d8af96e32e10b">
+      <tp>
+        <v>1</v>
+        <stp/>
+        <stp>f91521ea-7295-4df7-913b-f04f08850313</stp>
+        <tr r="G28" s="1"/>
+      </tp>
+      <tp>
+        <v>1</v>
+        <stp/>
+        <stp>d3e0ba7e-11f4-4ded-93ad-f0af33e02e07</stp>
+        <tr r="G23" s="1"/>
+      </tp>
+    </main>
+    <main first="rtdsrv.0283c6361b6f4b11963d8af96e32e10b">
+      <tp>
+        <v>1</v>
+        <stp/>
+        <stp>45ab64ca-418f-4176-9d1e-bb0c000ddac6</stp>
+        <tr r="E4" s="3"/>
+      </tp>
+      <tp>
+        <v>1</v>
+        <stp/>
+        <stp>278c9eff-de88-4e97-b96d-f54f1460b440</stp>
+        <tr r="G28" s="4"/>
+      </tp>
+      <tp>
+        <v>1</v>
+        <stp/>
+        <stp>9f6ecca5-15eb-4707-971f-c7b66c809d05</stp>
+        <tr r="G54" s="1"/>
+      </tp>
+      <tp>
+        <v>1</v>
+        <stp/>
+        <stp>ad40027b-b0cf-42c3-b21e-6270d5cf1389</stp>
+        <tr r="G51" s="1"/>
+      </tp>
+    </main>
+    <main first="rtdsrv.0283c6361b6f4b11963d8af96e32e10b">
+      <tp>
+        <v>2</v>
+        <stp/>
+        <stp>609e9975-c42e-41c3-a60e-320dbafcd898</stp>
+        <tr r="E19" s="3"/>
+      </tp>
+    </main>
+    <main first="rtdsrv.0283c6361b6f4b11963d8af96e32e10b">
+      <tp>
+        <v>1</v>
+        <stp/>
+        <stp>66e3f1a7-dc82-4c18-848e-3f138dbaeccd</stp>
+        <tr r="G48" s="4"/>
+      </tp>
+    </main>
+    <main first="rtdsrv.0283c6361b6f4b11963d8af96e32e10b">
+      <tp>
+        <v>1</v>
+        <stp/>
+        <stp>2e80f495-6d23-4931-8c10-9bcbef252a35</stp>
+        <tr r="G22" s="4"/>
+      </tp>
+    </main>
+    <main first="rtdsrv.0283c6361b6f4b11963d8af96e32e10b">
+      <tp>
+        <v>1</v>
+        <stp/>
+        <stp>9dc87f22-e789-498b-887f-e87ae0db0980</stp>
+        <tr r="G42" s="1"/>
+      </tp>
+    </main>
+    <main first="rtdsrv.0283c6361b6f4b11963d8af96e32e10b">
+      <tp>
+        <v>1</v>
+        <stp/>
+        <stp>a655e98a-9dac-47cf-87ef-6724f5c7840f</stp>
+        <tr r="G24" s="1"/>
+      </tp>
+    </main>
+    <main first="rtdsrv.0283c6361b6f4b11963d8af96e32e10b">
+      <tp>
+        <v>1</v>
+        <stp/>
+        <stp>8e830847-c845-41bb-be9e-5a243184011c</stp>
+        <tr r="G25" s="1"/>
+      </tp>
+      <tp>
+        <v>1</v>
+        <stp/>
+        <stp>9d2fd18b-6a30-4fb8-bd59-485c503e5b4e</stp>
+        <tr r="P19" s="1"/>
+      </tp>
+    </main>
+    <main first="rtdsrv.0283c6361b6f4b11963d8af96e32e10b">
+      <tp>
+        <v>1</v>
+        <stp/>
+        <stp>1c60dd64-2466-49d3-9918-45ff2e7b9c9d</stp>
+        <tr r="G21" s="4"/>
+      </tp>
+      <tp>
+        <v>1</v>
+        <stp/>
+        <stp>ff5c22c2-369f-4487-8e10-b8915ea6382b</stp>
+        <tr r="I42" s="4"/>
+      </tp>
+      <tp>
+        <v>1</v>
+        <stp/>
+        <stp>85c15001-f38a-4ac1-bddb-cc15c02b6a00</stp>
+        <tr r="G36" s="1"/>
+      </tp>
+      <tp>
+        <v>1</v>
+        <stp/>
+        <stp>9ffbd7bb-ffa9-4fcb-848e-fce2f9c0833e</stp>
+        <tr r="G57" s="4"/>
+      </tp>
+      <tp>
+        <v>1</v>
+        <stp/>
+        <stp>c138934d-7354-4caf-9caf-42ad97fb7248</stp>
+        <tr r="G19" s="4"/>
+      </tp>
+    </main>
+    <main first="rtdsrv.0283c6361b6f4b11963d8af96e32e10b">
+      <tp>
+        <v>1</v>
+        <stp/>
+        <stp>cbbe6ba9-2680-41e4-913e-bfcf2a0aa77f</stp>
+        <tr r="G44" s="4"/>
+      </tp>
+      <tp>
+        <v>1</v>
+        <stp/>
+        <stp>4a7bcb66-77cd-4970-9a01-f2ceab246b8b</stp>
+        <tr r="G53" s="4"/>
+      </tp>
+      <tp>
+        <v>1</v>
+        <stp/>
+        <stp>6f4a615d-aa46-434c-9ab4-df19ed2e4335</stp>
+        <tr r="G39" s="4"/>
+      </tp>
+    </main>
+    <main first="rtdsrv.0283c6361b6f4b11963d8af96e32e10b">
+      <tp>
+        <v>1</v>
+        <stp/>
+        <stp>f8929a55-a88b-44db-9885-7a81f572303f</stp>
+        <tr r="G40" s="4"/>
+      </tp>
+    </main>
+    <main first="rtdsrv.0283c6361b6f4b11963d8af96e32e10b">
+      <tp>
+        <v>1</v>
+        <stp/>
+        <stp>b2716693-b771-4d35-a494-64c03823aa58</stp>
+        <tr r="G39" s="1"/>
+      </tp>
+    </main>
+    <main first="rtdsrv.0283c6361b6f4b11963d8af96e32e10b">
+      <tp>
+        <v>1</v>
+        <stp/>
+        <stp>33af8016-04e7-4377-a471-ce4f8af9d018</stp>
+        <tr r="G26" s="4"/>
+      </tp>
+    </main>
+    <main first="rtdsrv.0283c6361b6f4b11963d8af96e32e10b">
+      <tp>
+        <v>1</v>
+        <stp/>
+        <stp>a3f90695-9d61-4ed8-b31e-c8b1bbe0977a</stp>
+        <tr r="G42" s="4"/>
+      </tp>
+      <tp>
+        <v>1</v>
+        <stp/>
+        <stp>5c9ad030-821b-4f1c-895b-6e5e999b9971</stp>
+        <tr r="E7" s="3"/>
+      </tp>
+      <tp>
+        <v>1</v>
+        <stp/>
+        <stp>99bfbf6f-23ef-4990-ab6f-549cdfb64a9a</stp>
+        <tr r="G32" s="1"/>
+      </tp>
+      <tp>
+        <v>1</v>
+        <stp/>
+        <stp>08c5cdbd-f323-4cee-b022-4032ca3c8dce</stp>
+        <tr r="G40" s="1"/>
+      </tp>
+      <tp>
+        <v>1</v>
+        <stp/>
+        <stp>a39a21d3-9a80-4d66-97aa-9727121e71c7</stp>
+        <tr r="G27" s="4"/>
+      </tp>
+      <tp>
+        <v>1</v>
+        <stp/>
+        <stp>a2134fa5-d7d4-4355-9dc4-b4cf637f9982</stp>
+        <tr r="G26" s="1"/>
+      </tp>
+    </main>
+    <main first="rtdsrv.0283c6361b6f4b11963d8af96e32e10b">
+      <tp>
+        <v>1</v>
+        <stp/>
+        <stp>b2d1bb5e-37ec-4e68-a11b-75a887d91109</stp>
+        <tr r="G55" s="1"/>
+      </tp>
+    </main>
+    <main first="rtdsrv.0283c6361b6f4b11963d8af96e32e10b">
+      <tp>
+        <v>1</v>
+        <stp/>
+        <stp>d61d9e4b-241f-49f8-bf8d-4c55fa97b90e</stp>
+        <tr r="E17" s="3"/>
+      </tp>
+      <tp>
+        <v>1</v>
+        <stp/>
+        <stp>86e458ad-7840-4a40-b408-d2d5cb9f7393</stp>
+        <tr r="G25" s="4"/>
+      </tp>
+      <tp>
+        <v>1</v>
+        <stp/>
+        <stp>56c2fa54-9bbc-4552-9d34-60b07c8ecf8a</stp>
+        <tr r="G47" s="1"/>
+      </tp>
+    </main>
+    <main first="rtdsrv.0283c6361b6f4b11963d8af96e32e10b">
+      <tp>
+        <v>1</v>
+        <stp/>
+        <stp>e963b4d4-dc60-4de2-815a-ac34c4325b7c</stp>
+        <tr r="G20" s="4"/>
+      </tp>
+      <tp>
+        <v>1</v>
+        <stp/>
+        <stp>9937bbaa-a783-4863-abc3-1477619f5356</stp>
+        <tr r="P29" s="1"/>
+      </tp>
+    </main>
+    <main first="rtdsrv.0283c6361b6f4b11963d8af96e32e10b">
+      <tp>
+        <v>1</v>
+        <stp/>
+        <stp>11a4f85d-10ab-4f5b-a609-43d62c900fb2</stp>
+        <tr r="G21" s="1"/>
+      </tp>
+    </main>
+    <main first="rtdsrv.0283c6361b6f4b11963d8af96e32e10b">
+      <tp>
+        <v>3</v>
+        <stp/>
+        <stp>a36ca0cf-060a-4d10-8b5f-0505df02792e</stp>
         <tr r="E6" s="3"/>
       </tp>
-      <tp>
-        <v>1</v>
-        <stp/>
-        <stp>4bae0147-0d67-4488-8d65-e83c8e1dbace</stp>
-        <tr r="G47" s="1"/>
-      </tp>
-      <tp>
-        <v>1</v>
-        <stp/>
-        <stp>57a29ce7-243a-49ee-8a54-baf4fb7bbd34</stp>
-        <tr r="G55" s="1"/>
-      </tp>
     </main>
-    <main first="rtdsrv.4f71aace325a499b836bfd0f6b877e4c">
-      <tp>
-        <v>1</v>
-        <stp/>
-        <stp>4163b705-a18d-4b6d-b35d-ae46066c14e9</stp>
+    <main first="rtdsrv.0283c6361b6f4b11963d8af96e32e10b">
+      <tp>
+        <v>1</v>
+        <stp/>
+        <stp>f5147f57-e942-477b-bc5d-d5be92025832</stp>
+        <tr r="G33" s="4"/>
+      </tp>
+    </main>
+    <main first="rtdsrv.0283c6361b6f4b11963d8af96e32e10b">
+      <tp>
+        <v>1</v>
+        <stp/>
+        <stp>c3cb2885-40fe-449d-bbf7-1b654249c3da</stp>
+        <tr r="F6" s="4"/>
+      </tp>
+      <tp>
+        <v>1</v>
+        <stp/>
+        <stp>0ff35af1-3ec5-4775-91ca-f3220917168b</stp>
+        <tr r="G30" s="1"/>
+      </tp>
+      <tp>
+        <v>1</v>
+        <stp/>
+        <stp>79970d27-e740-4c17-af5f-b3af2d3eb38c</stp>
+        <tr r="G29" s="1"/>
+      </tp>
+      <tp>
+        <v>1</v>
+        <stp/>
+        <stp>141a1fed-1759-426b-b780-8a548c72ceeb</stp>
+        <tr r="I33" s="4"/>
+      </tp>
+    </main>
+    <main first="rtdsrv.0283c6361b6f4b11963d8af96e32e10b">
+      <tp>
+        <v>1</v>
+        <stp/>
+        <stp>f641ffaa-0cd0-4a39-b80a-1c589a79243e</stp>
+        <tr r="G56" s="4"/>
+      </tp>
+      <tp>
+        <v>1</v>
+        <stp/>
+        <stp>d9bce48c-a145-4bc3-8f59-da1aa1b0ae58</stp>
+        <tr r="G57" s="1"/>
+      </tp>
+      <tp>
+        <v>1</v>
+        <stp/>
+        <stp>2f3d2bf1-108c-419c-93df-b01dfd54a90a</stp>
+        <tr r="G44" s="1"/>
+      </tp>
+    </main>
+    <main first="rtdsrv.0283c6361b6f4b11963d8af96e32e10b">
+      <tp>
+        <v>1</v>
+        <stp/>
+        <stp>b8e04dcb-f9a2-4623-9693-f0295ca4a34c</stp>
+        <tr r="G52" s="1"/>
+      </tp>
+    </main>
+    <main first="rtdsrv.0283c6361b6f4b11963d8af96e32e10b">
+      <tp>
+        <v>1</v>
+        <stp/>
+        <stp>f20ed68b-d0e4-45e0-9135-c16e52bf1090</stp>
+        <tr r="G43" s="1"/>
+      </tp>
+      <tp>
+        <v>1</v>
+        <stp/>
+        <stp>6a3813d9-0763-484d-b451-4de952f9851b</stp>
+        <tr r="G54" s="4"/>
+      </tp>
+      <tp>
+        <v>1</v>
+        <stp/>
+        <stp>753f90eb-abb2-4537-adad-cc80deb23d2f</stp>
+        <tr r="G41" s="1"/>
+      </tp>
+    </main>
+    <main first="rtdsrv.0283c6361b6f4b11963d8af96e32e10b">
+      <tp>
+        <v>1</v>
+        <stp/>
+        <stp>60df1138-c085-4b4c-b3d0-ea8b94607ac9</stp>
+        <tr r="G31" s="4"/>
+      </tp>
+      <tp>
+        <v>1</v>
+        <stp/>
+        <stp>d8cb59d9-e18e-4c40-9210-a2c4f78441c6</stp>
         <tr r="G43" s="4"/>
       </tp>
       <tp>
         <v>1</v>
         <stp/>
-        <stp>6a6b9490-09b5-4900-891f-9c78bddaf25b</stp>
-        <tr r="G54" s="4"/>
+        <stp>355d1bf7-cde7-4353-bd2e-4bd530e246c6</stp>
+        <tr r="F6" s="1"/>
       </tp>
     </main>
-    <main first="rtdsrv.4f71aace325a499b836bfd0f6b877e4c">
-      <tp>
-        <v>1</v>
-        <stp/>
-        <stp>1addcbe8-55cc-414b-8019-be397cb481b7</stp>
-        <tr r="G23" s="4"/>
+    <main first="rtdsrv.0283c6361b6f4b11963d8af96e32e10b">
+      <tp>
+        <v>1</v>
+        <stp/>
+        <stp>272954a3-5628-403c-aa41-1e8f15653c49</stp>
+        <tr r="G45" s="4"/>
       </tp>
     </main>
-    <main first="rtdsrv.4f71aace325a499b836bfd0f6b877e4c">
-      <tp>
-        <v>1</v>
-        <stp/>
-        <stp>fb1214e3-b538-48b3-9e44-8d40314db522</stp>
-        <tr r="I28" s="4"/>
+    <main first="rtdsrv.0283c6361b6f4b11963d8af96e32e10b">
+      <tp>
+        <v>1</v>
+        <stp/>
+        <stp>086581e9-ff31-4301-a5fa-c84c13d55a84</stp>
+        <tr r="F1" s="4"/>
+      </tp>
+      <tp>
+        <v>1</v>
+        <stp/>
+        <stp>f7f67aaa-40a7-41fe-b9f4-8241e90c4883</stp>
+        <tr r="G49" s="4"/>
+      </tp>
+      <tp>
+        <v>1</v>
+        <stp/>
+        <stp>3b5ca16b-7f32-40ad-9284-90ba68954b58</stp>
+        <tr r="G27" s="1"/>
       </tp>
     </main>
-    <main first="rtdsrv.4f71aace325a499b836bfd0f6b877e4c">
-      <tp>
-        <v>1</v>
-        <stp/>
-        <stp>1f155c50-bf1e-4b8a-9d25-1b1cc08c4238</stp>
+    <main first="rtdsrv.0283c6361b6f4b11963d8af96e32e10b">
+      <tp>
+        <v>1</v>
+        <stp/>
+        <stp>1d52dc5d-def5-48a4-b0e0-136c77f4cee8</stp>
+        <tr r="G34" s="4"/>
+      </tp>
+    </main>
+    <main first="rtdsrv.0283c6361b6f4b11963d8af96e32e10b">
+      <tp>
+        <v>1</v>
+        <stp/>
+        <stp>8d81f2d5-48c3-44b6-89fa-788f2a6b787b</stp>
+        <tr r="I19" s="1"/>
+      </tp>
+      <tp>
+        <v>1</v>
+        <stp/>
+        <stp>11b79eb1-60dc-4082-83e3-512865d2bbac</stp>
+        <tr r="G30" s="4"/>
+      </tp>
+    </main>
+    <main first="rtdsrv.0283c6361b6f4b11963d8af96e32e10b">
+      <tp>
+        <v>1</v>
+        <stp/>
+        <stp>6e00cf5e-d87a-4774-a2c3-26e9532c1a99</stp>
+        <tr r="G36" s="4"/>
+      </tp>
+      <tp>
+        <v>1</v>
+        <stp/>
+        <stp>33b718fa-1d0a-46b9-b22d-ad3aedfb6e2c</stp>
+        <tr r="G34" s="1"/>
+      </tp>
+      <tp>
+        <v>1</v>
+        <stp/>
+        <stp>edee6b00-035b-4a47-b7bd-504d71d07643</stp>
+        <tr r="I38" s="4"/>
+      </tp>
+    </main>
+    <main first="rtdsrv.0283c6361b6f4b11963d8af96e32e10b">
+      <tp>
+        <v>1</v>
+        <stp/>
+        <stp>e0efa2c1-1305-4fd7-8f2c-4f86b795c3fa</stp>
+        <tr r="F1" s="1"/>
+      </tp>
+      <tp>
+        <v>1</v>
+        <stp/>
+        <stp>26b72fdc-0088-4f80-aac6-22bc27e07b25</stp>
+        <tr r="G50" s="1"/>
+      </tp>
+    </main>
+    <main first="rtdsrv.0283c6361b6f4b11963d8af96e32e10b">
+      <tp>
+        <v>1</v>
+        <stp/>
+        <stp>8be0a774-7476-4540-82fd-f7712f7e00af</stp>
+        <tr r="G46" s="1"/>
+      </tp>
+    </main>
+    <main first="rtdsrv.0283c6361b6f4b11963d8af96e32e10b">
+      <tp>
+        <v>1</v>
+        <stp/>
+        <stp>377f1767-bdeb-456a-bfa8-da20e30ade9c</stp>
+        <tr r="I32" s="4"/>
         <tr r="I19" s="4"/>
       </tp>
       <tp>
         <v>1</v>
         <stp/>
-        <stp>587faa86-a1fa-4931-8150-247ab8dd5d05</stp>
-        <tr r="G46" s="1"/>
+        <stp>d4f7c6e5-4bcf-4a5b-986f-444caa822b37</stp>
+        <tr r="G31" s="1"/>
       </tp>
     </main>
-    <main first="rtdsrv.4f71aace325a499b836bfd0f6b877e4c">
-      <tp>
-        <v>1</v>
-        <stp/>
-        <stp>9d9901ba-c07c-4de4-89ef-2287d79a869e</stp>
-        <tr r="F1" s="4"/>
-      </tp>
-      <tp>
-        <v>1</v>
-        <stp/>
-        <stp>17533588-4af8-4e69-9195-8c878e79ee77</stp>
-        <tr r="G45" s="1"/>
+    <main first="rtdsrv.0283c6361b6f4b11963d8af96e32e10b">
+      <tp>
+        <v>1</v>
+        <stp/>
+        <stp>0a165bec-66a7-4967-930d-9ce67bad1e9d</stp>
+        <tr r="G38" s="4"/>
       </tp>
     </main>
-    <main first="rtdsrv.4f71aace325a499b836bfd0f6b877e4c">
-      <tp>
-        <v>1</v>
-        <stp/>
-        <stp>c2eff6ec-90e0-43c7-a185-60a52ee6621e</stp>
-        <tr r="G44" s="4"/>
+    <main first="rtdsrv.0283c6361b6f4b11963d8af96e32e10b">
+      <tp>
+        <v>1</v>
+        <stp/>
+        <stp>6e255841-2f77-4868-8904-c2b69a9fbcd6</stp>
+        <tr r="G33" s="1"/>
+      </tp>
+      <tp>
+        <v>1</v>
+        <stp/>
+        <stp>bdfe15f5-d962-4809-a052-51f8695ddf26</stp>
+        <tr r="G19" s="1"/>
       </tp>
     </main>
-    <main first="rtdsrv.4f71aace325a499b836bfd0f6b877e4c">
-      <tp>
-        <v>1</v>
-        <stp/>
-        <stp>349ebc8d-c6a1-436d-bbd5-e8700b499866</stp>
-        <tr r="G33" s="4"/>
+    <main first="rtdsrv.0283c6361b6f4b11963d8af96e32e10b">
+      <tp>
+        <v>1</v>
+        <stp/>
+        <stp>00199060-f9af-4630-b20a-f4efbfbcecd4</stp>
+        <tr r="G50" s="4"/>
+      </tp>
+      <tp>
+        <v>1</v>
+        <stp/>
+        <stp>c23fc26f-fa90-4b0e-8c3c-310977890a04</stp>
+        <tr r="G37" s="1"/>
       </tp>
     </main>
-    <main first="rtdsrv.4f71aace325a499b836bfd0f6b877e4c">
-      <tp>
-        <v>1</v>
-        <stp/>
-        <stp>83b38bd8-f4a2-46d8-b09c-acfa62cb302c</stp>
-        <tr r="G31" s="4"/>
-      </tp>
-      <tp>
-        <v>1</v>
-        <stp/>
-        <stp>295aa45c-0223-43dd-98a2-4ef1c9816374</stp>
-        <tr r="G40" s="4"/>
-      </tp>
-    </main>
-    <main first="rtdsrv.4f71aace325a499b836bfd0f6b877e4c">
-      <tp>
-        <v>1</v>
-        <stp/>
-        <stp>6194f773-4e58-446d-8a9c-9604b85816b0</stp>
-        <tr r="G23" s="1"/>
-      </tp>
-      <tp>
-        <v>1</v>
-        <stp/>
-        <stp>113f6e08-0927-4ae5-9fc7-ef710a470b9f</stp>
-        <tr r="G24" s="1"/>
-      </tp>
-      <tp>
-        <v>1</v>
-        <stp/>
-        <stp>cdaa407f-a2d2-4306-86ec-fd706aa994f2</stp>
-        <tr r="G50" s="4"/>
-      </tp>
-    </main>
-    <main first="rtdsrv.4f71aace325a499b836bfd0f6b877e4c">
-      <tp>
-        <v>1</v>
-        <stp/>
-        <stp>821072e5-bc6d-474c-bcc8-5b70aa3249c9</stp>
-        <tr r="G52" s="4"/>
-      </tp>
-    </main>
-    <main first="rtdsrv.4f71aace325a499b836bfd0f6b877e4c">
-      <tp>
-        <v>1</v>
-        <stp/>
-        <stp>b70d8356-6cd7-4ee5-a98f-7358766a3c20</stp>
-        <tr r="G38" s="4"/>
-      </tp>
-    </main>
-    <main first="rtdsrv.4f71aace325a499b836bfd0f6b877e4c">
-      <tp>
-        <v>1</v>
-        <stp/>
-        <stp>da984842-f31f-4be3-b8d8-f96252e8b973</stp>
-        <tr r="G26" s="4"/>
-      </tp>
-    </main>
-    <main first="rtdsrv.4f71aace325a499b836bfd0f6b877e4c">
-      <tp>
-        <v>1</v>
-        <stp/>
-        <stp>1c11f703-7eb2-4001-bafd-dcfb15ad6873</stp>
-        <tr r="G48" s="4"/>
-      </tp>
-      <tp>
-        <v>1</v>
-        <stp/>
-        <stp>89bb6b5e-59c0-45b0-92a4-c2383b9e95a1</stp>
-        <tr r="G51" s="1"/>
-      </tp>
-    </main>
-    <main first="rtdsrv.4f71aace325a499b836bfd0f6b877e4c">
-      <tp>
-        <v>1</v>
-        <stp/>
-        <stp>cf645a20-1d65-4640-af2c-119808173f09</stp>
-        <tr r="G54" s="1"/>
-      </tp>
-      <tp>
-        <v>2</v>
-        <stp/>
-        <stp>71f9e4a4-0cc6-4c54-8615-402fad66e852</stp>
-        <tr r="E19" s="3"/>
-      </tp>
-      <tp>
-        <v>1</v>
-        <stp/>
-        <stp>545e4b14-faec-4e48-a313-414ecd277031</stp>
-        <tr r="G50" s="1"/>
-      </tp>
-      <tp>
-        <v>1</v>
-        <stp/>
-        <stp>718d3480-f185-4049-95e9-f7df1d060082</stp>
-        <tr r="P19" s="1"/>
-      </tp>
-    </main>
-    <main first="rtdsrv.4f71aace325a499b836bfd0f6b877e4c">
-      <tp>
-        <v>1</v>
-        <stp/>
-        <stp>ba67df44-c074-425a-8cc3-aa341b13692b</stp>
-        <tr r="G45" s="4"/>
-      </tp>
-      <tp>
-        <v>1</v>
-        <stp/>
-        <stp>7a5a7273-0481-4883-885b-58ea48478972</stp>
-        <tr r="G57" s="1"/>
-      </tp>
-    </main>
-    <main first="rtdsrv.4f71aace325a499b836bfd0f6b877e4c">
-      <tp>
-        <v>1</v>
-        <stp/>
-        <stp>c17002ae-dab7-488f-b2b3-a80ec529e28b</stp>
-        <tr r="G26" s="1"/>
-      </tp>
-      <tp>
-        <v>1</v>
-        <stp/>
-        <stp>b9339e3b-b03e-454d-a6d8-de99cd99dc74</stp>
-        <tr r="G19" s="4"/>
-      </tp>
-    </main>
-    <main first="rtdsrv.4f71aace325a499b836bfd0f6b877e4c">
-      <tp>
-        <v>1</v>
-        <stp/>
-        <stp>2c30cd29-e878-40d7-8b73-e86902795517</stp>
-        <tr r="F1" s="1"/>
-      </tp>
-      <tp>
-        <v>1</v>
-        <stp/>
-        <stp>430d5d6f-5494-4da3-84e8-c9688bc8f2b2</stp>
-        <tr r="G39" s="1"/>
-      </tp>
-    </main>
-    <main first="rtdsrv.4f71aace325a499b836bfd0f6b877e4c">
-      <tp>
-        <v>1</v>
-        <stp/>
-        <stp>255fd695-c436-4249-a688-1bc98e2a7841</stp>
-        <tr r="G27" s="4"/>
-      </tp>
-      <tp>
-        <v>1</v>
-        <stp/>
-        <stp>2552e3eb-539e-48ed-ae7e-7a6779f35f03</stp>
-        <tr r="I28" s="1"/>
-      </tp>
-    </main>
-    <main first="rtdsrv.4f71aace325a499b836bfd0f6b877e4c">
-      <tp>
-        <v>1</v>
-        <stp/>
-        <stp>27842b44-08dd-48b0-8995-c47c85544349</stp>
-        <tr r="G38" s="1"/>
-      </tp>
-      <tp>
-        <v>1</v>
-        <stp/>
-        <stp>3a79f843-312b-43c2-b855-23589ed93d35</stp>
-        <tr r="G47" s="4"/>
-      </tp>
-    </main>
-    <main first="rtdsrv.4f71aace325a499b836bfd0f6b877e4c">
-      <tp>
-        <v>1</v>
-        <stp/>
-        <stp>80416d9d-0d03-4b19-b1e8-0dbf166e5545</stp>
-        <tr r="G43" s="1"/>
-      </tp>
-      <tp>
-        <v>1</v>
-        <stp/>
-        <stp>c43bd51b-f5e1-4c2e-a4ea-1516fa6d2317</stp>
-        <tr r="G42" s="1"/>
-      </tp>
-      <tp>
-        <v>1</v>
-        <stp/>
-        <stp>e2f3b2bf-24e1-4295-a12b-b54a4e7b5e08</stp>
-        <tr r="G24" s="4"/>
-      </tp>
-      <tp>
-        <v>1</v>
-        <stp/>
-        <stp>27c232a8-357e-43ab-bd06-fd79baf7ea18</stp>
-        <tr r="G21" s="4"/>
-      </tp>
-      <tp>
-        <v>1</v>
-        <stp/>
-        <stp>2ba53cec-7cd6-4cb6-b922-6269fe63fe15</stp>
-        <tr r="G44" s="1"/>
-      </tp>
-      <tp>
-        <v>1</v>
-        <stp/>
-        <stp>f8f83b47-ea59-46c5-a64f-91699659090e</stp>
+    <main first="rtdsrv.0283c6361b6f4b11963d8af96e32e10b">
+      <tp>
+        <v>1</v>
+        <stp/>
+        <stp>fd6544de-9255-4888-a540-0eb35adf36cd</stp>
+        <tr r="G29" s="4"/>
+      </tp>
+      <tp>
+        <v>1</v>
+        <stp/>
+        <stp>e2d2ba5b-bf0f-4538-bc3f-586c04ca0a37</stp>
         <tr r="G51" s="4"/>
-      </tp>
-    </main>
-    <main first="rtdsrv.4f71aace325a499b836bfd0f6b877e4c">
-      <tp>
-        <v>1</v>
-        <stp/>
-        <stp>11f5c004-d32f-4149-9ca2-56c22874e323</stp>
-        <tr r="G34" s="1"/>
-      </tp>
-    </main>
-    <main first="rtdsrv.4f71aace325a499b836bfd0f6b877e4c">
-      <tp>
-        <v>1</v>
-        <stp/>
-        <stp>1d79f584-c29e-4de4-b624-15b5ee65adf1</stp>
-        <tr r="G56" s="4"/>
-      </tp>
-      <tp>
-        <v>1</v>
-        <stp/>
-        <stp>d17dfc9e-23f0-4de5-9e7e-40029141ccc3</stp>
-        <tr r="G40" s="1"/>
-      </tp>
-      <tp>
-        <v>1</v>
-        <stp/>
-        <stp>2de5d6bf-5e35-4b52-98f6-151d34349329</stp>
-        <tr r="G41" s="1"/>
-      </tp>
-    </main>
-    <main first="rtdsrv.4f71aace325a499b836bfd0f6b877e4c">
-      <tp>
-        <v>1</v>
-        <stp/>
-        <stp>999925e6-a973-424b-af08-70c7062b38ac</stp>
-        <tr r="G35" s="4"/>
-      </tp>
-      <tp>
-        <v>1</v>
-        <stp/>
-        <stp>3c295dff-e4a8-4646-b617-57f78c68103e</stp>
-        <tr r="F6" s="4"/>
-      </tp>
-    </main>
-    <main first="rtdsrv.4f71aace325a499b836bfd0f6b877e4c">
-      <tp>
-        <v>1</v>
-        <stp/>
-        <stp>8186f115-44c6-4a76-bd13-8dc1a2335de3</stp>
-        <tr r="G22" s="1"/>
-      </tp>
-      <tp>
-        <v>1</v>
-        <stp/>
-        <stp>0c614bc8-4770-4416-bddd-8185d58aaace</stp>
-        <tr r="G25" s="1"/>
-      </tp>
-      <tp>
-        <v>1</v>
-        <stp/>
-        <stp>f2f1c59c-6121-484d-b9fc-1bab5c609020</stp>
-        <tr r="G29" s="4"/>
-      </tp>
-      <tp>
-        <v>1</v>
-        <stp/>
-        <stp>07a4e063-4ab1-4f12-aca8-ecd724bbe5ae</stp>
-        <tr r="G21" s="1"/>
-      </tp>
-      <tp>
-        <v>1</v>
-        <stp/>
-        <stp>4173253c-bf00-4e35-833c-9dc6261c90c7</stp>
-        <tr r="G25" s="4"/>
-      </tp>
-    </main>
-    <main first="rtdsrv.4f71aace325a499b836bfd0f6b877e4c">
-      <tp>
-        <v>1</v>
-        <stp/>
-        <stp>3a8c2ea4-d8f3-4bb9-8115-3ff5054908f3</stp>
-        <tr r="G29" s="1"/>
-      </tp>
-      <tp>
-        <v>1</v>
-        <stp/>
-        <stp>bd129158-f05a-4fc8-8dc4-441dff7089f4</stp>
-        <tr r="G55" s="4"/>
-      </tp>
-      <tp>
-        <v>1</v>
-        <stp/>
-        <stp>f0cc7e91-339e-4f31-8822-bffc89a39912</stp>
-        <tr r="G48" s="1"/>
-      </tp>
-    </main>
-    <main first="rtdsrv.4f71aace325a499b836bfd0f6b877e4c">
-      <tp>
-        <v>1</v>
-        <stp/>
-        <stp>79a457b1-4de5-4861-be04-92fcd904d39b</stp>
-        <tr r="G19" s="1"/>
-      </tp>
-      <tp>
-        <v>1</v>
-        <stp/>
-        <stp>efe3f7c9-0873-426b-be51-2a0b0083ad86</stp>
-        <tr r="G37" s="4"/>
-      </tp>
-      <tp>
-        <v>1</v>
-        <stp/>
-        <stp>113287e1-07d9-4572-bb63-040a416a636e</stp>
-        <tr r="G52" s="1"/>
-      </tp>
-    </main>
-    <main first="rtdsrv.4f71aace325a499b836bfd0f6b877e4c">
-      <tp>
-        <v>1</v>
-        <stp/>
-        <stp>1729ab4b-7e8b-4ea4-ad68-939ca28f6e58</stp>
-        <tr r="G27" s="1"/>
-      </tp>
-      <tp>
-        <v>1</v>
-        <stp/>
-        <stp>0ca64ebb-4e8e-44b5-a2b4-bab88805c837</stp>
-        <tr r="G32" s="1"/>
-      </tp>
-      <tp>
-        <v>1</v>
-        <stp/>
-        <stp>501c11c1-722f-4e42-81f4-967d23408cbd</stp>
-        <tr r="F6" s="1"/>
-      </tp>
-      <tp>
-        <v>1</v>
-        <stp/>
-        <stp>d2cacac1-e787-484c-99fd-91bff247d43b</stp>
-        <tr r="G36" s="4"/>
-      </tp>
-      <tp>
-        <v>1</v>
-        <stp/>
-        <stp>f8777e23-40cd-443b-b9c2-c901937c5f89</stp>
-        <tr r="G49" s="4"/>
-      </tp>
-      <tp>
-        <v>1</v>
-        <stp/>
-        <stp>217763d1-4754-4cd8-b282-a90cd8b3d2d2</stp>
-        <tr r="G20" s="1"/>
-      </tp>
-    </main>
-    <main first="rtdsrv.4f71aace325a499b836bfd0f6b877e4c">
-      <tp>
-        <v>1</v>
-        <stp/>
-        <stp>85d8af6a-be03-4cd5-a225-7b515b12f361</stp>
-        <tr r="G34" s="4"/>
-      </tp>
-      <tp>
-        <v>1</v>
-        <stp/>
-        <stp>8612f0e6-cf52-4782-821c-037cb6f41f17</stp>
-        <tr r="G36" s="1"/>
-      </tp>
-      <tp>
-        <v>1</v>
-        <stp/>
-        <stp>609151f1-2a33-444f-9d3a-7c7104a7548b</stp>
-        <tr r="G20" s="4"/>
-      </tp>
-    </main>
-    <main first="rtdsrv.4f71aace325a499b836bfd0f6b877e4c">
-      <tp>
-        <v>1</v>
-        <stp/>
-        <stp>75fef74d-a48a-4dc3-b1f4-5436afb16a63</stp>
-        <tr r="G53" s="1"/>
-      </tp>
-    </main>
-    <main first="rtdsrv.4f71aace325a499b836bfd0f6b877e4c">
-      <tp>
-        <v>1</v>
-        <stp/>
-        <stp>ad2254d2-ca1a-43cb-bda4-803023ca64b4</stp>
-        <tr r="E7" s="3"/>
-      </tp>
-      <tp>
-        <v>1</v>
-        <stp/>
-        <stp>c6fc1df5-7ac8-4402-8a52-2b7f03a2744d</stp>
-        <tr r="G53" s="4"/>
-      </tp>
-    </main>
-    <main first="rtdsrv.4f71aace325a499b836bfd0f6b877e4c">
-      <tp>
-        <v>1</v>
-        <stp/>
-        <stp>ead48723-45fa-4c0e-b2e6-02f66d230397</stp>
-        <tr r="G30" s="4"/>
-      </tp>
-      <tp>
-        <v>1</v>
-        <stp/>
-        <stp>1a5a3ccf-95ee-4d79-aeb5-0f6da58084d4</stp>
-        <tr r="G57" s="4"/>
-      </tp>
-      <tp>
-        <v>1</v>
-        <stp/>
-        <stp>11b17745-1d84-434d-85d9-685775c8025d</stp>
-        <tr r="P29" s="1"/>
-      </tp>
-    </main>
-    <main first="rtdsrv.4f71aace325a499b836bfd0f6b877e4c">
-      <tp>
-        <v>1</v>
-        <stp/>
-        <stp>75d38090-2134-470f-b49f-9d4b95b411f3</stp>
-        <tr r="G28" s="4"/>
-      </tp>
-      <tp>
-        <v>1</v>
-        <stp/>
-        <stp>b07346bb-75c5-4c80-8a6e-a6a52934c137</stp>
-        <tr r="G28" s="1"/>
-      </tp>
-      <tp>
-        <v>1</v>
-        <stp/>
-        <stp>2be77c6d-9869-4513-bdb7-93e931415bf1</stp>
-        <tr r="G46" s="4"/>
-      </tp>
-      <tp>
-        <v>1</v>
-        <stp/>
-        <stp>c13a6b84-56f3-40f0-85a0-5ca489f23df6</stp>
-        <tr r="E17" s="3"/>
-      </tp>
-    </main>
-    <main first="rtdsrv.4f71aace325a499b836bfd0f6b877e4c">
-      <tp>
-        <v>1</v>
-        <stp/>
-        <stp>149b894e-2c91-48e1-b85d-2d6cdb2de450</stp>
-        <tr r="G39" s="4"/>
-      </tp>
-    </main>
-    <main first="rtdsrv.4f71aace325a499b836bfd0f6b877e4c">
-      <tp>
-        <v>1</v>
-        <stp/>
-        <stp>6903d874-73eb-49fa-82da-d8c82552345f</stp>
-        <tr r="G30" s="1"/>
-      </tp>
-      <tp>
-        <v>1</v>
-        <stp/>
-        <stp>e8678673-243c-47b4-aa09-3a2852e4bab3</stp>
-        <tr r="G56" s="1"/>
-      </tp>
-      <tp>
-        <v>1</v>
-        <stp/>
-        <stp>67c5d08c-e50f-4d3b-b18f-21b601ec7240</stp>
-        <tr r="C2" s="2"/>
-      </tp>
-    </main>
-    <main first="rtdsrv.4f71aace325a499b836bfd0f6b877e4c">
-      <tp>
-        <v>1</v>
-        <stp/>
-        <stp>d28ab38a-3a2c-4d58-9720-101e85c856c1</stp>
-        <tr r="G31" s="1"/>
-      </tp>
-    </main>
-    <main first="rtdsrv.4f71aace325a499b836bfd0f6b877e4c">
-      <tp>
-        <v>1</v>
-        <stp/>
-        <stp>6108a201-d12b-4544-8121-dad2e9b80251</stp>
-        <tr r="G35" s="1"/>
-      </tp>
-      <tp>
-        <v>1</v>
-        <stp/>
-        <stp>288837ab-cad4-4a96-8c70-975c8e85943d</stp>
-        <tr r="G32" s="4"/>
-      </tp>
-      <tp>
-        <v>1</v>
-        <stp/>
-        <stp>74053748-6a7e-4921-b32a-7095b2b71887</stp>
-        <tr r="G22" s="4"/>
-      </tp>
-    </main>
-    <main first="rtdsrv.4f71aace325a499b836bfd0f6b877e4c">
-      <tp>
-        <v>33</v>
-        <stp/>
-        <stp>c3ad1f91-6114-461c-a7f7-09efed5357a5</stp>
-        <tr r="E20" s="3"/>
-      </tp>
-    </main>
-    <main first="rtdsrv.4f71aace325a499b836bfd0f6b877e4c">
-      <tp>
-        <v>1</v>
-        <stp/>
-        <stp>48820364-459b-4994-8570-ec8d11700b8c</stp>
-        <tr r="E4" s="3"/>
-      </tp>
-      <tp>
-        <v>1</v>
-        <stp/>
-        <stp>3d62ac29-391a-459c-adc8-924fd94e12d3</stp>
-        <tr r="I19" s="1"/>
-      </tp>
-    </main>
-    <main first="rtdsrv.4f71aace325a499b836bfd0f6b877e4c">
-      <tp>
-        <v>1</v>
-        <stp/>
-        <stp>e286e8a0-42e1-4b02-a729-3e26ab08f77c</stp>
-        <tr r="G49" s="1"/>
-      </tp>
-      <tp>
-        <v>1</v>
-        <stp/>
-        <stp>055c55a9-295e-48c2-9596-31bcbca2ce01</stp>
-        <tr r="G41" s="4"/>
-      </tp>
-    </main>
-    <main first="rtdsrv.4f71aace325a499b836bfd0f6b877e4c">
-      <tp>
-        <v>1</v>
-        <stp/>
-        <stp>9f669866-ecfd-4851-9fea-d15f95cc3ec4</stp>
-        <tr r="G42" s="4"/>
-      </tp>
-    </main>
-    <main first="rtdsrv.4f71aace325a499b836bfd0f6b877e4c">
-      <tp>
-        <v>1</v>
-        <stp/>
-        <stp>332597c7-85d4-431f-aadd-07cdaef72ca0</stp>
-        <tr r="G33" s="1"/>
-      </tp>
-    </main>
-    <main first="rtdsrv.4f71aace325a499b836bfd0f6b877e4c">
-      <tp>
-        <v>1</v>
-        <stp/>
-        <stp>7210d7af-f60e-4f7f-a176-f86d3f8e7cac</stp>
-        <tr r="G37" s="1"/>
       </tp>
     </main>
   </volType>
@@ -1540,11 +1590,11 @@
       </c>
       <c r="F1" t="str" cm="1">
         <f t="array" ref="F1">_xll.ExLibris.Json.CreateJsonObject(E3:F6)</f>
-        <v>JsonObject:A90E9D9A-D769-488B-BA4A-7DC68DDAE374</v>
+        <v>JsonObject:76876AD4-5002-4E2F-B04C-A3891F489D96</v>
       </c>
       <c r="K1" t="str">
         <f>EXLIBRIS_CONFIGURATION</f>
-        <v>ExLibris.Core.ExLibrisConfiguration:3DBC2D14-284C-4875-833A-7330C5C56AB2</v>
+        <v>ExLibris.Core.ExLibrisConfiguration:23598F7C-BC8C-460B-B094-6B7B1D5D478C</v>
       </c>
     </row>
     <row r="2" spans="2:28" x14ac:dyDescent="0.4">
@@ -1614,7 +1664,7 @@
       </c>
       <c r="F6" t="str" cm="1">
         <f t="array" ref="F6">_xll.ExLibris.Json.CreateJsonArray(E8:J14)</f>
-        <v>JsonObject:05B87254-C6AC-4550-9DAB-537F01796631</v>
+        <v>JsonObject:335D9DA4-5359-4486-9EB4-A04CE9A9E1A3</v>
       </c>
       <c r="L6" t="s">
         <v>68</v>
@@ -1626,7 +1676,7 @@
     </row>
     <row r="7" spans="2:28" x14ac:dyDescent="0.4">
       <c r="B7" s="6" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="C7" s="6">
         <f>COUNTIF(AR19:AS21,FALSE)</f>
@@ -1636,12 +1686,12 @@
         <v>74</v>
       </c>
       <c r="M7" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
     </row>
     <row r="8" spans="2:28" x14ac:dyDescent="0.4">
       <c r="B8" s="6" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="C8" s="6">
         <f>COUNTIF(AR30:AS65,FALSE)</f>
@@ -1853,7 +1903,7 @@
       </c>
       <c r="I19" t="str" cm="1">
         <f t="array" ref="I19">_xll.ExLibris.Json.GetJsonValue(F1,E6)</f>
-        <v>JsonObject:726D8B20-9BBE-486A-89AE-24693B6C9A94</v>
+        <v>JsonObject:A1901F1D-E8FA-4D73-9D81-905B827A439D</v>
       </c>
       <c r="P19" t="str" cm="1">
         <f t="array" ref="P19:Q27">_xll.ExLibris.Json.GetJsonKeyValues(F1,,3)</f>
@@ -2158,7 +2208,7 @@
         <v>fixed_leg.cashflows.[0]</v>
       </c>
       <c r="Q22" t="str">
-        <v>JsonObject:0BCBA1E4-04F2-4A64-BE7A-7CC302F24F93</v>
+        <v>JsonObject:2E45E8C0-4857-4BBC-8F67-F07DF8F104DE</v>
       </c>
       <c r="S22" t="s">
         <v>32</v>
@@ -2257,7 +2307,7 @@
         <v>fixed_leg.cashflows.[1]</v>
       </c>
       <c r="Q23" t="str">
-        <v>JsonObject:E05AC574-6535-4FD8-8C3A-311EC3318237</v>
+        <v>JsonObject:0D99B359-988F-4603-B7A3-85B0D393EA96</v>
       </c>
       <c r="S23" t="s">
         <v>33</v>
@@ -2356,7 +2406,7 @@
         <v>fixed_leg.cashflows.[2]</v>
       </c>
       <c r="Q24" t="str">
-        <v>JsonObject:35843975-D2C9-4969-AB74-971876A5041B</v>
+        <v>JsonObject:926A79F0-EE6A-4898-AEED-998440594C6B</v>
       </c>
       <c r="S24" t="s">
         <v>34</v>
@@ -2455,7 +2505,7 @@
         <v>fixed_leg.cashflows.[3]</v>
       </c>
       <c r="Q25" t="str">
-        <v>JsonObject:A19E2369-7E3C-4840-A99D-0730DC46FD2F</v>
+        <v>JsonObject:168243F9-DBCC-4C09-A9BC-805ABAEF10AA</v>
       </c>
       <c r="S25" t="s">
         <v>35</v>
@@ -2554,7 +2604,7 @@
         <v>fixed_leg.cashflows.[4]</v>
       </c>
       <c r="Q26" t="str">
-        <v>JsonObject:9E3A70AD-EDDD-4C62-A87A-400B8D84BFA4</v>
+        <v>JsonObject:D7FB3BD5-B53F-4337-81ED-4A956008BD00</v>
       </c>
       <c r="S26" t="s">
         <v>36</v>
@@ -2635,7 +2685,7 @@
         <v>fixed_leg.cashflows.[5]</v>
       </c>
       <c r="Q27" t="str">
-        <v>JsonObject:33F26FF0-6428-4583-A96F-22A67FB214A3</v>
+        <v>JsonObject:EF9CA57C-7F7D-4997-B8CE-C3458BA2C48E</v>
       </c>
       <c r="S27" t="s">
         <v>37</v>
@@ -2672,7 +2722,7 @@
       </c>
       <c r="I28" t="str" cm="1">
         <f t="array" ref="I28">_xll.ExLibris.Json.GetJsonValue(I19,"[2]")</f>
-        <v>JsonObject:033FD9F7-EF14-42CA-952E-A63F2C7DC36A</v>
+        <v>JsonObject:3B3BE114-1984-48B4-B95C-8BF7D4F473B5</v>
       </c>
       <c r="S28" t="s">
         <v>38</v>
@@ -2728,7 +2778,7 @@
       </c>
       <c r="P29" t="str" cm="1">
         <f t="array" ref="P29">_xll.ExLibris.Json.CreateJsonObject(P22:Q27)</f>
-        <v>JsonObject:56EAB903-BAA2-479F-910A-6BF19D91752D</v>
+        <v>JsonObject:0825B6B7-9C64-4EE8-A992-0A914261D6AD</v>
       </c>
       <c r="S29" t="s">
         <v>39</v>
@@ -4528,6 +4578,7 @@
   <sheetFormatPr defaultRowHeight="18.75" x14ac:dyDescent="0.4"/>
   <cols>
     <col min="1" max="1" width="2.25" customWidth="1"/>
+    <col min="2" max="2" width="11" customWidth="1"/>
     <col min="4" max="4" width="2.125" customWidth="1"/>
     <col min="5" max="5" width="38.125" bestFit="1" customWidth="1"/>
     <col min="6" max="7" width="13.25" customWidth="1"/>
@@ -4549,11 +4600,11 @@
       </c>
       <c r="F1" t="str" cm="1">
         <f t="array" ref="F1">_xll.ExLibris.Json.CreateJsonObject(E3:F6, EXLIBRIS_CONFIGURATION)</f>
-        <v>JsonObject:86C5E29F-D324-48A8-9522-F1FA8030568E</v>
+        <v>JsonObject:008E0007-AECB-42C1-8068-149FAC93578D</v>
       </c>
       <c r="K1" t="str">
         <f>EXLIBRIS_CONFIGURATION</f>
-        <v>ExLibris.Core.ExLibrisConfiguration:3DBC2D14-284C-4875-833A-7330C5C56AB2</v>
+        <v>ExLibris.Core.ExLibrisConfiguration:23598F7C-BC8C-460B-B094-6B7B1D5D478C</v>
       </c>
     </row>
     <row r="2" spans="2:25" x14ac:dyDescent="0.4">
@@ -4623,25 +4674,39 @@
       </c>
       <c r="F6" t="str" cm="1">
         <f t="array" ref="F6">_xll.ExLibris.Json.CreateJsonArray(E8:J14, EXLIBRIS_CONFIGURATION)</f>
-        <v>JsonObject:C6663F5F-000E-4D61-B837-BC7ABB53F0F9</v>
+        <v>JsonObject:CA60A2AE-6AFA-4219-846F-D2F18716D018</v>
       </c>
       <c r="L6" t="s">
         <v>68</v>
       </c>
       <c r="M6" t="str" cm="1">
         <f t="array" ref="M6">_xll.ExLibris.Json.ShowJsonText(F1)</f>
-        <v>{"trade_code":"money_00001","couter_party":"CP00001","fixed_leg":{"pay_or_recieve":"Receive","cashflows":[{"payment _date":"2022-03-12","start_date":"2021-09-13","end_date":"2022-03-12","day_count_type":"ACT/360","amout":10000000,"fixed_rate":0.001},{"payment _date":"2022-09-08","start_date":"2022-03-12","end_date":"2022-09-08","day_count_type":"ACT/360","amout":11000000,"fixed_rate":0.001},{"payment _date":"2023-03-07","start_date":"2022-09-08","end_date":"2023-03-07","day_count_type":"ACT/360","amout":12000000,"fixed_rate":0.001},{"payment _date":"2023-09-03","start_date":"2023-03-07","end_date":"2023-09-03","day_count_type":"ACT/360","amout":13000000,"fixed_rate":0.001},{"payment _date":"2024-03-01","start_date":"2023-09-03","end_date":"2024-03-01","day_count_type":"ACT/360","amout":14000000,"fixed_rate":0.001},{"payment _date":"2024-08-28","start_date":"2024-03-01","end_date":"2024-08-28","day_count_type":"ACT/360","amout":15000000,"fixed_rate":0.001}]}}</v>
+        <v>{"trade_code":"money_00001","couter_party":"CP00001","fixed_leg":{"pay_or_recieve":"Receive","cashflows":[{"payment _date":"2022-03-12","start_date":"2021-09-13","end_date":"2022-03-12","day_count_type":"ACT/360","amout":10000000,"fixed_rate":0.001},{"payment _date":"2022-09-08","start_date":"2022-03-12","end_date":"2022-09-08","day_count_type":"ACT/360","amout":10000000,"fixed_rate":0.0011},{"payment _date":"2023-03-07","start_date":"2022-09-08","end_date":"2023-03-07","day_count_type":"ACT/360","amout":11000000,"fixed_rate":0.0012000000000000001},{"payment _date":"2023-09-03","start_date":"2023-03-07","end_date":"2023-09-03","day_count_type":"ACT/360","amout":11000000,"fixed_rate":0.0013000000000000002},{"payment _date":"2024-03-01","start_date":"2023-09-03","end_date":"2024-03-01","day_count_type":"ACT/360","amout":12000000,"fixed_rate":0.0014000000000000002},{"payment _date":"2024-08-28","start_date":"2024-03-01","end_date":"2024-08-28","day_count_type":"ACT/360","amout":12000000,"fixed_rate":0.0015000000000000002}]}}</v>
       </c>
     </row>
     <row r="7" spans="2:25" x14ac:dyDescent="0.4">
+      <c r="B7" s="6" t="s">
+        <v>117</v>
+      </c>
+      <c r="C7" s="6">
+        <f>COUNTIF(AE34:AJ36,FALSE)</f>
+        <v>0</v>
+      </c>
       <c r="L7" t="s">
         <v>74</v>
       </c>
       <c r="M7" t="s">
-        <v>100</v>
+        <v>115</v>
       </c>
     </row>
     <row r="8" spans="2:25" x14ac:dyDescent="0.4">
+      <c r="B8" s="6" t="s">
+        <v>118</v>
+      </c>
+      <c r="C8" s="6">
+        <f>COUNTIF(AE39:AJ40,FALSE)</f>
+        <v>0</v>
+      </c>
       <c r="E8" t="s">
         <v>1</v>
       </c>
@@ -4662,6 +4727,13 @@
       </c>
     </row>
     <row r="9" spans="2:25" x14ac:dyDescent="0.4">
+      <c r="B9" s="6" t="s">
+        <v>119</v>
+      </c>
+      <c r="C9" s="6">
+        <f>COUNTIF(AE43,FALSE)</f>
+        <v>0</v>
+      </c>
       <c r="E9" s="1">
         <f>G9</f>
         <v>44632</v>
@@ -4700,11 +4772,12 @@
         <v>9</v>
       </c>
       <c r="I10" s="2">
-        <f>I9+1000000</f>
-        <v>11000000</v>
+        <f>I9</f>
+        <v>10000000</v>
       </c>
       <c r="J10" s="3">
-        <v>1E-3</v>
+        <f>J9+0.0001</f>
+        <v>1.1000000000000001E-3</v>
       </c>
     </row>
     <row r="11" spans="2:25" x14ac:dyDescent="0.4">
@@ -4724,11 +4797,12 @@
         <v>9</v>
       </c>
       <c r="I11" s="2">
-        <f t="shared" ref="I11:I14" si="3">I10+1000000</f>
-        <v>12000000</v>
+        <f t="shared" ref="I11:I13" si="3">I10+1000000</f>
+        <v>11000000</v>
       </c>
       <c r="J11" s="3">
-        <v>1E-3</v>
+        <f t="shared" ref="J11:J14" si="4">J10+0.0001</f>
+        <v>1.2000000000000001E-3</v>
       </c>
     </row>
     <row r="12" spans="2:25" x14ac:dyDescent="0.4">
@@ -4748,11 +4822,12 @@
         <v>9</v>
       </c>
       <c r="I12" s="2">
-        <f t="shared" si="3"/>
-        <v>13000000</v>
+        <f>I11</f>
+        <v>11000000</v>
       </c>
       <c r="J12" s="3">
-        <v>1E-3</v>
+        <f t="shared" si="4"/>
+        <v>1.3000000000000002E-3</v>
       </c>
     </row>
     <row r="13" spans="2:25" x14ac:dyDescent="0.4">
@@ -4773,10 +4848,11 @@
       </c>
       <c r="I13" s="2">
         <f t="shared" si="3"/>
-        <v>14000000</v>
+        <v>12000000</v>
       </c>
       <c r="J13" s="3">
-        <v>1E-3</v>
+        <f t="shared" si="4"/>
+        <v>1.4000000000000002E-3</v>
       </c>
     </row>
     <row r="14" spans="2:25" x14ac:dyDescent="0.4">
@@ -4796,11 +4872,12 @@
         <v>9</v>
       </c>
       <c r="I14" s="2">
-        <f t="shared" si="3"/>
-        <v>15000000</v>
+        <f>I13</f>
+        <v>12000000</v>
       </c>
       <c r="J14" s="3">
-        <v>1E-3</v>
+        <f t="shared" si="4"/>
+        <v>1.5000000000000002E-3</v>
       </c>
     </row>
     <row r="16" spans="2:25" s="4" customFormat="1" ht="18" x14ac:dyDescent="0.4">
@@ -4848,7 +4925,7 @@
       </c>
       <c r="I19" t="str" cm="1">
         <f t="array" ref="I19">_xll.ExLibris.Json.GetJsonValue(F1,E6, EXLIBRIS_CONFIGURATION)</f>
-        <v>JsonObject:4AF288B1-6716-40F0-9D27-F704DDFB7A50</v>
+        <v>JsonObject:F4BE569E-7806-4DA7-A070-484C307ECDE3</v>
       </c>
       <c r="P19" t="s">
         <v>14</v>
@@ -4860,15 +4937,15 @@
         <v>16</v>
       </c>
       <c r="AA19" t="b">
-        <f t="shared" ref="AA19:AA57" si="4">E19=P19</f>
+        <f t="shared" ref="AA19:AA57" si="5">E19=P19</f>
         <v>1</v>
       </c>
       <c r="AB19" t="b">
-        <f t="shared" ref="AB19:AC57" si="5">E19=P19</f>
+        <f t="shared" ref="AB19:AC57" si="6">E19=P19</f>
         <v>1</v>
       </c>
       <c r="AC19" t="b">
-        <f t="shared" si="5"/>
+        <f t="shared" si="6"/>
         <v>1</v>
       </c>
     </row>
@@ -4930,39 +5007,39 @@
         <v>12</v>
       </c>
       <c r="AA20" t="b">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v>1</v>
       </c>
       <c r="AB20" t="b">
-        <f t="shared" si="5"/>
+        <f t="shared" si="6"/>
         <v>1</v>
       </c>
       <c r="AC20" t="b">
-        <f t="shared" si="5"/>
+        <f t="shared" si="6"/>
         <v>1</v>
       </c>
       <c r="AE20" t="b">
-        <f t="shared" ref="AE20:AJ26" si="6">I20=T20</f>
+        <f t="shared" ref="AE20:AJ26" si="7">I20=T20</f>
         <v>1</v>
       </c>
       <c r="AF20" t="b">
-        <f t="shared" si="6"/>
+        <f t="shared" si="7"/>
         <v>1</v>
       </c>
       <c r="AG20" t="b">
-        <f t="shared" si="6"/>
+        <f t="shared" si="7"/>
         <v>1</v>
       </c>
       <c r="AH20" t="b">
-        <f t="shared" si="6"/>
+        <f t="shared" si="7"/>
         <v>1</v>
       </c>
       <c r="AI20" t="b">
-        <f t="shared" si="6"/>
+        <f t="shared" si="7"/>
         <v>1</v>
       </c>
       <c r="AJ20" t="b">
-        <f t="shared" si="6"/>
+        <f t="shared" si="7"/>
         <v>1</v>
       </c>
     </row>
@@ -5023,39 +5100,39 @@
         <v>1E-3</v>
       </c>
       <c r="AA21" t="b">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v>1</v>
       </c>
       <c r="AB21" t="b">
-        <f t="shared" si="5"/>
+        <f t="shared" si="6"/>
         <v>1</v>
       </c>
       <c r="AC21" t="b">
-        <f t="shared" si="5"/>
+        <f t="shared" si="6"/>
         <v>1</v>
       </c>
       <c r="AE21" t="b">
-        <f t="shared" si="6"/>
+        <f t="shared" si="7"/>
         <v>1</v>
       </c>
       <c r="AF21" t="b">
-        <f t="shared" si="6"/>
+        <f t="shared" si="7"/>
         <v>1</v>
       </c>
       <c r="AG21" t="b">
-        <f t="shared" si="6"/>
+        <f t="shared" si="7"/>
         <v>1</v>
       </c>
       <c r="AH21" t="b">
-        <f t="shared" si="6"/>
+        <f t="shared" si="7"/>
         <v>1</v>
       </c>
       <c r="AI21" t="b">
-        <f t="shared" si="6"/>
+        <f t="shared" si="7"/>
         <v>1</v>
       </c>
       <c r="AJ21" t="b">
-        <f t="shared" si="6"/>
+        <f t="shared" si="7"/>
         <v>1</v>
       </c>
     </row>
@@ -5083,10 +5160,10 @@
         <v>ACT/360</v>
       </c>
       <c r="M22">
-        <v>11000000</v>
+        <v>10000000</v>
       </c>
       <c r="N22">
-        <v>1E-3</v>
+        <v>1.1000000000000001E-3</v>
       </c>
       <c r="P22" t="s">
         <v>32</v>
@@ -5110,45 +5187,45 @@
         <v>8</v>
       </c>
       <c r="X22">
-        <v>11000000</v>
+        <v>10000000</v>
       </c>
       <c r="Y22">
-        <v>1E-3</v>
+        <v>1.1000000000000001E-3</v>
       </c>
       <c r="AA22" t="b">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v>1</v>
       </c>
       <c r="AB22" t="b">
-        <f t="shared" si="5"/>
+        <f t="shared" si="6"/>
         <v>1</v>
       </c>
       <c r="AC22" t="b">
-        <f t="shared" si="5"/>
+        <f t="shared" si="6"/>
         <v>1</v>
       </c>
       <c r="AE22" t="b">
-        <f t="shared" si="6"/>
+        <f t="shared" si="7"/>
         <v>1</v>
       </c>
       <c r="AF22" t="b">
-        <f t="shared" si="6"/>
+        <f t="shared" si="7"/>
         <v>1</v>
       </c>
       <c r="AG22" t="b">
-        <f t="shared" si="6"/>
+        <f t="shared" si="7"/>
         <v>1</v>
       </c>
       <c r="AH22" t="b">
-        <f t="shared" si="6"/>
+        <f t="shared" si="7"/>
         <v>1</v>
       </c>
       <c r="AI22" t="b">
-        <f t="shared" si="6"/>
+        <f t="shared" si="7"/>
         <v>1</v>
       </c>
       <c r="AJ22" t="b">
-        <f t="shared" si="6"/>
+        <f t="shared" si="7"/>
         <v>1</v>
       </c>
     </row>
@@ -5176,10 +5253,10 @@
         <v>ACT/360</v>
       </c>
       <c r="M23">
-        <v>12000000</v>
+        <v>11000000</v>
       </c>
       <c r="N23">
-        <v>1E-3</v>
+        <v>1.2000000000000001E-3</v>
       </c>
       <c r="P23" t="s">
         <v>33</v>
@@ -5203,45 +5280,45 @@
         <v>8</v>
       </c>
       <c r="X23">
-        <v>12000000</v>
+        <v>11000000</v>
       </c>
       <c r="Y23">
-        <v>1E-3</v>
+        <v>1.2000000000000001E-3</v>
       </c>
       <c r="AA23" t="b">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v>1</v>
       </c>
       <c r="AB23" t="b">
-        <f t="shared" si="5"/>
+        <f t="shared" si="6"/>
         <v>1</v>
       </c>
       <c r="AC23" t="b">
-        <f t="shared" si="5"/>
+        <f t="shared" si="6"/>
         <v>1</v>
       </c>
       <c r="AE23" t="b">
-        <f t="shared" si="6"/>
+        <f t="shared" si="7"/>
         <v>1</v>
       </c>
       <c r="AF23" t="b">
-        <f t="shared" si="6"/>
+        <f t="shared" si="7"/>
         <v>1</v>
       </c>
       <c r="AG23" t="b">
-        <f t="shared" si="6"/>
+        <f t="shared" si="7"/>
         <v>1</v>
       </c>
       <c r="AH23" t="b">
-        <f t="shared" si="6"/>
+        <f t="shared" si="7"/>
         <v>1</v>
       </c>
       <c r="AI23" t="b">
-        <f t="shared" si="6"/>
+        <f t="shared" si="7"/>
         <v>1</v>
       </c>
       <c r="AJ23" t="b">
-        <f t="shared" si="6"/>
+        <f t="shared" si="7"/>
         <v>1</v>
       </c>
     </row>
@@ -5269,10 +5346,10 @@
         <v>ACT/360</v>
       </c>
       <c r="M24">
-        <v>13000000</v>
+        <v>11000000</v>
       </c>
       <c r="N24">
-        <v>1E-3</v>
+        <v>1.3000000000000002E-3</v>
       </c>
       <c r="P24" t="s">
         <v>34</v>
@@ -5296,45 +5373,45 @@
         <v>8</v>
       </c>
       <c r="X24">
-        <v>13000000</v>
+        <v>11000000</v>
       </c>
       <c r="Y24">
-        <v>1E-3</v>
+        <v>1.3000000000000002E-3</v>
       </c>
       <c r="AA24" t="b">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v>1</v>
       </c>
       <c r="AB24" t="b">
-        <f t="shared" si="5"/>
+        <f t="shared" si="6"/>
         <v>1</v>
       </c>
       <c r="AC24" t="b">
-        <f t="shared" si="5"/>
+        <f t="shared" si="6"/>
         <v>1</v>
       </c>
       <c r="AE24" t="b">
-        <f t="shared" si="6"/>
+        <f t="shared" si="7"/>
         <v>1</v>
       </c>
       <c r="AF24" t="b">
-        <f t="shared" si="6"/>
+        <f t="shared" si="7"/>
         <v>1</v>
       </c>
       <c r="AG24" t="b">
-        <f t="shared" si="6"/>
+        <f t="shared" si="7"/>
         <v>1</v>
       </c>
       <c r="AH24" t="b">
-        <f t="shared" si="6"/>
+        <f t="shared" si="7"/>
         <v>1</v>
       </c>
       <c r="AI24" t="b">
-        <f t="shared" si="6"/>
+        <f t="shared" si="7"/>
         <v>1</v>
       </c>
       <c r="AJ24" t="b">
-        <f t="shared" si="6"/>
+        <f t="shared" si="7"/>
         <v>1</v>
       </c>
     </row>
@@ -5362,10 +5439,10 @@
         <v>ACT/360</v>
       </c>
       <c r="M25">
-        <v>14000000</v>
+        <v>12000000</v>
       </c>
       <c r="N25">
-        <v>1E-3</v>
+        <v>1.4000000000000002E-3</v>
       </c>
       <c r="P25" t="s">
         <v>35</v>
@@ -5389,45 +5466,45 @@
         <v>8</v>
       </c>
       <c r="X25">
-        <v>14000000</v>
+        <v>12000000</v>
       </c>
       <c r="Y25">
-        <v>1E-3</v>
+        <v>1.4000000000000002E-3</v>
       </c>
       <c r="AA25" t="b">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v>1</v>
       </c>
       <c r="AB25" t="b">
-        <f t="shared" si="5"/>
+        <f t="shared" si="6"/>
         <v>1</v>
       </c>
       <c r="AC25" t="b">
-        <f t="shared" si="5"/>
+        <f t="shared" si="6"/>
         <v>1</v>
       </c>
       <c r="AE25" t="b">
-        <f t="shared" si="6"/>
+        <f t="shared" si="7"/>
         <v>1</v>
       </c>
       <c r="AF25" t="b">
-        <f t="shared" si="6"/>
+        <f t="shared" si="7"/>
         <v>1</v>
       </c>
       <c r="AG25" t="b">
-        <f t="shared" si="6"/>
+        <f t="shared" si="7"/>
         <v>1</v>
       </c>
       <c r="AH25" t="b">
-        <f t="shared" si="6"/>
+        <f t="shared" si="7"/>
         <v>1</v>
       </c>
       <c r="AI25" t="b">
-        <f t="shared" si="6"/>
+        <f t="shared" si="7"/>
         <v>1</v>
       </c>
       <c r="AJ25" t="b">
-        <f t="shared" si="6"/>
+        <f t="shared" si="7"/>
         <v>1</v>
       </c>
     </row>
@@ -5455,10 +5532,10 @@
         <v>ACT/360</v>
       </c>
       <c r="M26">
-        <v>15000000</v>
+        <v>12000000</v>
       </c>
       <c r="N26">
-        <v>1E-3</v>
+        <v>1.5000000000000002E-3</v>
       </c>
       <c r="P26" t="s">
         <v>36</v>
@@ -5482,45 +5559,45 @@
         <v>8</v>
       </c>
       <c r="X26">
-        <v>15000000</v>
+        <v>12000000</v>
       </c>
       <c r="Y26">
-        <v>1E-3</v>
+        <v>1.5000000000000002E-3</v>
       </c>
       <c r="AA26" t="b">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v>1</v>
       </c>
       <c r="AB26" t="b">
-        <f t="shared" si="5"/>
+        <f t="shared" si="6"/>
         <v>1</v>
       </c>
       <c r="AC26" t="b">
-        <f t="shared" si="5"/>
+        <f t="shared" si="6"/>
         <v>1</v>
       </c>
       <c r="AE26" t="b">
-        <f t="shared" si="6"/>
+        <f t="shared" si="7"/>
         <v>1</v>
       </c>
       <c r="AF26" t="b">
-        <f t="shared" si="6"/>
+        <f t="shared" si="7"/>
         <v>1</v>
       </c>
       <c r="AG26" t="b">
-        <f t="shared" si="6"/>
+        <f t="shared" si="7"/>
         <v>1</v>
       </c>
       <c r="AH26" t="b">
-        <f t="shared" si="6"/>
+        <f t="shared" si="7"/>
         <v>1</v>
       </c>
       <c r="AI26" t="b">
-        <f t="shared" si="6"/>
+        <f t="shared" si="7"/>
         <v>1</v>
       </c>
       <c r="AJ26" t="b">
-        <f t="shared" si="6"/>
+        <f t="shared" si="7"/>
         <v>1</v>
       </c>
     </row>
@@ -5545,15 +5622,15 @@
         <v>1E-3</v>
       </c>
       <c r="AA27" t="b">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v>1</v>
       </c>
       <c r="AB27" t="b">
-        <f t="shared" si="5"/>
+        <f t="shared" si="6"/>
         <v>1</v>
       </c>
       <c r="AC27" t="b">
-        <f t="shared" si="5"/>
+        <f t="shared" si="6"/>
         <v>1</v>
       </c>
     </row>
@@ -5570,7 +5647,7 @@
       </c>
       <c r="I28" t="str" cm="1">
         <f t="array" ref="I28">_xll.ExLibris.Json.GetJsonValue(I19,"[2]", EXLIBRIS_CONFIGURATION)</f>
-        <v>JsonObject:281CC426-AAFB-4A91-BC34-F8660F1D2F1C</v>
+        <v>JsonObject:F5491BB0-47BB-4609-B55B-B44DFFC9B9EC</v>
       </c>
       <c r="P28" t="s">
         <v>38</v>
@@ -5582,15 +5659,15 @@
         <v>95</v>
       </c>
       <c r="AA28" t="b">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v>1</v>
       </c>
       <c r="AB28" t="b">
-        <f t="shared" si="5"/>
+        <f t="shared" si="6"/>
         <v>1</v>
       </c>
       <c r="AC28" t="b">
-        <f t="shared" si="5"/>
+        <f t="shared" si="6"/>
         <v>1</v>
       </c>
     </row>
@@ -5652,39 +5729,39 @@
         <v>12</v>
       </c>
       <c r="AA29" t="b">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v>1</v>
       </c>
       <c r="AB29" t="b">
-        <f t="shared" si="5"/>
+        <f t="shared" si="6"/>
         <v>1</v>
       </c>
       <c r="AC29" t="b">
-        <f t="shared" si="5"/>
+        <f t="shared" si="6"/>
         <v>1</v>
       </c>
       <c r="AE29" t="b">
-        <f t="shared" ref="AE29:AJ30" si="7">I29=T29</f>
+        <f t="shared" ref="AE29:AJ30" si="8">I29=T29</f>
         <v>1</v>
       </c>
       <c r="AF29" t="b">
-        <f t="shared" si="7"/>
+        <f t="shared" si="8"/>
         <v>1</v>
       </c>
       <c r="AG29" t="b">
-        <f t="shared" si="7"/>
+        <f t="shared" si="8"/>
         <v>1</v>
       </c>
       <c r="AH29" t="b">
-        <f t="shared" si="7"/>
+        <f t="shared" si="8"/>
         <v>1</v>
       </c>
       <c r="AI29" t="b">
-        <f t="shared" si="7"/>
+        <f t="shared" si="8"/>
         <v>1</v>
       </c>
       <c r="AJ29" t="b">
-        <f t="shared" si="7"/>
+        <f t="shared" si="8"/>
         <v>1</v>
       </c>
     </row>
@@ -5712,10 +5789,10 @@
         <v>ACT/360</v>
       </c>
       <c r="M30">
-        <v>12000000</v>
+        <v>11000000</v>
       </c>
       <c r="N30">
-        <v>1E-3</v>
+        <v>1.2000000000000001E-3</v>
       </c>
       <c r="P30" t="s">
         <v>40</v>
@@ -5739,45 +5816,45 @@
         <v>8</v>
       </c>
       <c r="X30">
-        <v>12000000</v>
+        <v>11000000</v>
       </c>
       <c r="Y30">
-        <v>1E-3</v>
+        <v>1.2000000000000001E-3</v>
       </c>
       <c r="AA30" t="b">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v>1</v>
       </c>
       <c r="AB30" t="b">
-        <f t="shared" si="5"/>
+        <f t="shared" si="6"/>
         <v>1</v>
       </c>
       <c r="AC30" t="b">
-        <f t="shared" si="5"/>
+        <f t="shared" si="6"/>
         <v>1</v>
       </c>
       <c r="AE30" t="b">
-        <f t="shared" si="7"/>
+        <f t="shared" si="8"/>
         <v>1</v>
       </c>
       <c r="AF30" t="b">
-        <f t="shared" si="7"/>
+        <f t="shared" si="8"/>
         <v>1</v>
       </c>
       <c r="AG30" t="b">
-        <f t="shared" si="7"/>
+        <f t="shared" si="8"/>
         <v>1</v>
       </c>
       <c r="AH30" t="b">
-        <f t="shared" si="7"/>
+        <f t="shared" si="8"/>
         <v>1</v>
       </c>
       <c r="AI30" t="b">
-        <f t="shared" si="7"/>
+        <f t="shared" si="8"/>
         <v>1</v>
       </c>
       <c r="AJ30" t="b">
-        <f t="shared" si="7"/>
+        <f t="shared" si="8"/>
         <v>1</v>
       </c>
     </row>
@@ -5802,15 +5879,15 @@
         <v>8</v>
       </c>
       <c r="AA31" t="b">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v>1</v>
       </c>
       <c r="AB31" t="b">
-        <f t="shared" si="5"/>
+        <f t="shared" si="6"/>
         <v>1</v>
       </c>
       <c r="AC31" t="b">
-        <f t="shared" si="5"/>
+        <f t="shared" si="6"/>
         <v>1</v>
       </c>
     </row>
@@ -5819,68 +5896,76 @@
         <v>fixed_leg.cashflows.[1].amout</v>
       </c>
       <c r="F32">
-        <v>11000000</v>
+        <v>10000000</v>
       </c>
       <c r="G32" cm="1">
         <f t="array" ref="G32">_xll.ExLibris.Json.GetJsonValue($F$1,E32, EXLIBRIS_CONFIGURATION)</f>
-        <v>11000000</v>
+        <v>10000000</v>
+      </c>
+      <c r="I32" t="str" cm="1">
+        <f t="array" ref="I32">_xll.ExLibris.Json.GetJsonValue(F1,E6,EXLIBRIS_CONFIGURATION)</f>
+        <v>JsonObject:F4BE569E-7806-4DA7-A070-484C307ECDE3</v>
       </c>
       <c r="P32" t="s">
         <v>42</v>
       </c>
       <c r="Q32">
-        <v>11000000</v>
+        <v>10000000</v>
       </c>
       <c r="R32">
-        <v>11000000</v>
+        <v>10000000</v>
       </c>
       <c r="AA32" t="b">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v>1</v>
       </c>
       <c r="AB32" t="b">
-        <f t="shared" si="5"/>
+        <f t="shared" si="6"/>
         <v>1</v>
       </c>
       <c r="AC32" t="b">
-        <f t="shared" si="5"/>
-        <v>1</v>
-      </c>
-    </row>
-    <row r="33" spans="5:29" x14ac:dyDescent="0.4">
+        <f t="shared" si="6"/>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="33" spans="5:36" x14ac:dyDescent="0.4">
       <c r="E33" t="str">
         <v>fixed_leg.cashflows.[1].fixed_rate</v>
       </c>
       <c r="F33">
-        <v>1E-3</v>
+        <v>1.1000000000000001E-3</v>
       </c>
       <c r="G33" cm="1">
         <f t="array" ref="G33">_xll.ExLibris.Json.GetJsonValue($F$1,E33, EXLIBRIS_CONFIGURATION)</f>
-        <v>1E-3</v>
+        <v>1.1000000000000001E-3</v>
+      </c>
+      <c r="I33" t="str" cm="1">
+        <f t="array" ref="I33">_xll.ExLibris.Json.SeachJsonArrayElements(I32,I8,I11,EXLIBRIS_CONFIGURATION)</f>
+        <v>JsonObject:D262EE96-6677-4E9A-A2A2-262853EC37BD</v>
       </c>
       <c r="P33" t="s">
         <v>43</v>
       </c>
       <c r="Q33">
-        <v>1E-3</v>
+        <v>1.1000000000000001E-3</v>
       </c>
       <c r="R33">
-        <v>1E-3</v>
+        <v>1.1000000000000001E-3</v>
       </c>
       <c r="AA33" t="b">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v>1</v>
       </c>
       <c r="AB33" t="b">
-        <f t="shared" si="5"/>
+        <f t="shared" si="6"/>
         <v>1</v>
       </c>
       <c r="AC33" t="b">
-        <f t="shared" si="5"/>
-        <v>1</v>
-      </c>
-    </row>
-    <row r="34" spans="5:29" x14ac:dyDescent="0.4">
+        <f t="shared" si="6"/>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="34" spans="5:36" x14ac:dyDescent="0.4">
       <c r="E34" t="str">
         <v>fixed_leg.cashflows.[2].payment _date</v>
       </c>
@@ -5891,6 +5976,25 @@
         <f t="array" ref="G34">_xll.ExLibris.Json.GetJsonValue($F$1,E34, EXLIBRIS_CONFIGURATION)</f>
         <v>2023-03-07</v>
       </c>
+      <c r="I34" t="str" cm="1">
+        <f t="array" ref="I34:N36">_xll.ExLibris.Json.GetJsonTable(I33, EXLIBRIS_CONFIGURATION)</f>
+        <v>payment _date</v>
+      </c>
+      <c r="J34" t="str">
+        <v>start_date</v>
+      </c>
+      <c r="K34" t="str">
+        <v>end_date</v>
+      </c>
+      <c r="L34" t="str">
+        <v>day_count_type</v>
+      </c>
+      <c r="M34" t="str">
+        <v>amout</v>
+      </c>
+      <c r="N34" t="str">
+        <v>fixed_rate</v>
+      </c>
       <c r="P34" t="s">
         <v>44</v>
       </c>
@@ -5900,20 +6004,62 @@
       <c r="R34" t="s">
         <v>96</v>
       </c>
+      <c r="T34" t="s">
+        <v>0</v>
+      </c>
+      <c r="U34" t="s">
+        <v>2</v>
+      </c>
+      <c r="V34" t="s">
+        <v>4</v>
+      </c>
+      <c r="W34" t="s">
+        <v>6</v>
+      </c>
+      <c r="X34" t="s">
+        <v>10</v>
+      </c>
+      <c r="Y34" t="s">
+        <v>12</v>
+      </c>
       <c r="AA34" t="b">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v>1</v>
       </c>
       <c r="AB34" t="b">
-        <f t="shared" si="5"/>
+        <f t="shared" si="6"/>
         <v>1</v>
       </c>
       <c r="AC34" t="b">
-        <f t="shared" si="5"/>
-        <v>1</v>
-      </c>
-    </row>
-    <row r="35" spans="5:29" x14ac:dyDescent="0.4">
+        <f t="shared" si="6"/>
+        <v>1</v>
+      </c>
+      <c r="AE34" t="b">
+        <f t="shared" ref="AE34:AE36" si="9">I34=T34</f>
+        <v>1</v>
+      </c>
+      <c r="AF34" t="b">
+        <f t="shared" ref="AF34:AF36" si="10">J34=U34</f>
+        <v>1</v>
+      </c>
+      <c r="AG34" t="b">
+        <f t="shared" ref="AG34:AG36" si="11">K34=V34</f>
+        <v>1</v>
+      </c>
+      <c r="AH34" t="b">
+        <f t="shared" ref="AH34:AH36" si="12">L34=W34</f>
+        <v>1</v>
+      </c>
+      <c r="AI34" t="b">
+        <f t="shared" ref="AI34:AI36" si="13">M34=X34</f>
+        <v>1</v>
+      </c>
+      <c r="AJ34" t="b">
+        <f t="shared" ref="AJ34:AJ36" si="14">N34=Y34</f>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="35" spans="5:36" x14ac:dyDescent="0.4">
       <c r="E35" t="str">
         <v>fixed_leg.cashflows.[2].start_date</v>
       </c>
@@ -5924,6 +6070,24 @@
         <f t="array" ref="G35">_xll.ExLibris.Json.GetJsonValue($F$1,E35, EXLIBRIS_CONFIGURATION)</f>
         <v>2022-09-08</v>
       </c>
+      <c r="I35" t="str">
+        <v>2023-03-07</v>
+      </c>
+      <c r="J35" t="str">
+        <v>2022-09-08</v>
+      </c>
+      <c r="K35" t="str">
+        <v>2023-03-07</v>
+      </c>
+      <c r="L35" t="str">
+        <v>ACT/360</v>
+      </c>
+      <c r="M35">
+        <v>11000000</v>
+      </c>
+      <c r="N35">
+        <v>1.2000000000000001E-3</v>
+      </c>
       <c r="P35" t="s">
         <v>45</v>
       </c>
@@ -5933,20 +6097,62 @@
       <c r="R35" t="s">
         <v>95</v>
       </c>
+      <c r="T35" t="s">
+        <v>96</v>
+      </c>
+      <c r="U35" t="s">
+        <v>95</v>
+      </c>
+      <c r="V35" t="s">
+        <v>96</v>
+      </c>
+      <c r="W35" t="s">
+        <v>8</v>
+      </c>
+      <c r="X35">
+        <v>11000000</v>
+      </c>
+      <c r="Y35">
+        <v>1.2000000000000001E-3</v>
+      </c>
       <c r="AA35" t="b">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v>1</v>
       </c>
       <c r="AB35" t="b">
-        <f t="shared" si="5"/>
+        <f t="shared" si="6"/>
         <v>1</v>
       </c>
       <c r="AC35" t="b">
-        <f t="shared" si="5"/>
-        <v>1</v>
-      </c>
-    </row>
-    <row r="36" spans="5:29" x14ac:dyDescent="0.4">
+        <f t="shared" si="6"/>
+        <v>1</v>
+      </c>
+      <c r="AE35" t="b">
+        <f t="shared" si="9"/>
+        <v>1</v>
+      </c>
+      <c r="AF35" t="b">
+        <f t="shared" si="10"/>
+        <v>1</v>
+      </c>
+      <c r="AG35" t="b">
+        <f t="shared" si="11"/>
+        <v>1</v>
+      </c>
+      <c r="AH35" t="b">
+        <f t="shared" si="12"/>
+        <v>1</v>
+      </c>
+      <c r="AI35" t="b">
+        <f t="shared" si="13"/>
+        <v>1</v>
+      </c>
+      <c r="AJ35" t="b">
+        <f t="shared" si="14"/>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="36" spans="5:36" x14ac:dyDescent="0.4">
       <c r="E36" t="str">
         <v>fixed_leg.cashflows.[2].end_date</v>
       </c>
@@ -5957,6 +6163,24 @@
         <f t="array" ref="G36">_xll.ExLibris.Json.GetJsonValue($F$1,E36, EXLIBRIS_CONFIGURATION)</f>
         <v>2023-03-07</v>
       </c>
+      <c r="I36" t="str">
+        <v>2023-09-03</v>
+      </c>
+      <c r="J36" t="str">
+        <v>2023-03-07</v>
+      </c>
+      <c r="K36" t="str">
+        <v>2023-09-03</v>
+      </c>
+      <c r="L36" t="str">
+        <v>ACT/360</v>
+      </c>
+      <c r="M36">
+        <v>11000000</v>
+      </c>
+      <c r="N36">
+        <v>1.3000000000000002E-3</v>
+      </c>
       <c r="P36" t="s">
         <v>46</v>
       </c>
@@ -5966,20 +6190,62 @@
       <c r="R36" t="s">
         <v>96</v>
       </c>
+      <c r="T36" t="s">
+        <v>97</v>
+      </c>
+      <c r="U36" t="s">
+        <v>96</v>
+      </c>
+      <c r="V36" t="s">
+        <v>97</v>
+      </c>
+      <c r="W36" t="s">
+        <v>8</v>
+      </c>
+      <c r="X36">
+        <v>11000000</v>
+      </c>
+      <c r="Y36">
+        <v>1.3000000000000002E-3</v>
+      </c>
       <c r="AA36" t="b">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v>1</v>
       </c>
       <c r="AB36" t="b">
-        <f t="shared" si="5"/>
+        <f t="shared" si="6"/>
         <v>1</v>
       </c>
       <c r="AC36" t="b">
-        <f t="shared" si="5"/>
-        <v>1</v>
-      </c>
-    </row>
-    <row r="37" spans="5:29" x14ac:dyDescent="0.4">
+        <f t="shared" si="6"/>
+        <v>1</v>
+      </c>
+      <c r="AE36" t="b">
+        <f t="shared" si="9"/>
+        <v>1</v>
+      </c>
+      <c r="AF36" t="b">
+        <f t="shared" si="10"/>
+        <v>1</v>
+      </c>
+      <c r="AG36" t="b">
+        <f t="shared" si="11"/>
+        <v>1</v>
+      </c>
+      <c r="AH36" t="b">
+        <f t="shared" si="12"/>
+        <v>1</v>
+      </c>
+      <c r="AI36" t="b">
+        <f t="shared" si="13"/>
+        <v>1</v>
+      </c>
+      <c r="AJ36" t="b">
+        <f t="shared" si="14"/>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="37" spans="5:36" x14ac:dyDescent="0.4">
       <c r="E37" t="str">
         <v>fixed_leg.cashflows.[2].day_count_type</v>
       </c>
@@ -6000,85 +6266,150 @@
         <v>8</v>
       </c>
       <c r="AA37" t="b">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v>1</v>
       </c>
       <c r="AB37" t="b">
-        <f t="shared" si="5"/>
+        <f t="shared" si="6"/>
         <v>1</v>
       </c>
       <c r="AC37" t="b">
-        <f t="shared" si="5"/>
-        <v>1</v>
-      </c>
-    </row>
-    <row r="38" spans="5:29" x14ac:dyDescent="0.4">
+        <f t="shared" si="6"/>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="38" spans="5:36" x14ac:dyDescent="0.4">
       <c r="E38" t="str">
         <v>fixed_leg.cashflows.[2].amout</v>
       </c>
       <c r="F38">
-        <v>12000000</v>
+        <v>11000000</v>
       </c>
       <c r="G38" cm="1">
         <f t="array" ref="G38">_xll.ExLibris.Json.GetJsonValue($F$1,E38, EXLIBRIS_CONFIGURATION)</f>
-        <v>12000000</v>
+        <v>11000000</v>
+      </c>
+      <c r="I38" t="str" cm="1">
+        <f t="array" ref="I38">_xll.ExLibris.Json.SeachJsonArrayElements(I32,J8,J11,EXLIBRIS_CONFIGURATION)</f>
+        <v>JsonObject:4CB3FEA9-E981-4454-9AD1-627AF904785E</v>
       </c>
       <c r="P38" t="s">
         <v>48</v>
       </c>
       <c r="Q38">
-        <v>12000000</v>
+        <v>11000000</v>
       </c>
       <c r="R38">
-        <v>12000000</v>
+        <v>11000000</v>
       </c>
       <c r="AA38" t="b">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v>1</v>
       </c>
       <c r="AB38" t="b">
-        <f t="shared" si="5"/>
+        <f t="shared" si="6"/>
         <v>1</v>
       </c>
       <c r="AC38" t="b">
-        <f t="shared" si="5"/>
-        <v>1</v>
-      </c>
-    </row>
-    <row r="39" spans="5:29" x14ac:dyDescent="0.4">
+        <f t="shared" si="6"/>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="39" spans="5:36" x14ac:dyDescent="0.4">
       <c r="E39" t="str">
         <v>fixed_leg.cashflows.[2].fixed_rate</v>
       </c>
       <c r="F39">
-        <v>1E-3</v>
+        <v>1.2000000000000001E-3</v>
       </c>
       <c r="G39" cm="1">
         <f t="array" ref="G39">_xll.ExLibris.Json.GetJsonValue($F$1,E39, EXLIBRIS_CONFIGURATION)</f>
-        <v>1E-3</v>
+        <v>1.2000000000000001E-3</v>
+      </c>
+      <c r="I39" t="str" cm="1">
+        <f t="array" ref="I39:N40">_xll.ExLibris.Json.GetJsonTable(I38, EXLIBRIS_CONFIGURATION)</f>
+        <v>payment _date</v>
+      </c>
+      <c r="J39" t="str">
+        <v>start_date</v>
+      </c>
+      <c r="K39" t="str">
+        <v>end_date</v>
+      </c>
+      <c r="L39" t="str">
+        <v>day_count_type</v>
+      </c>
+      <c r="M39" t="str">
+        <v>amout</v>
+      </c>
+      <c r="N39" t="str">
+        <v>fixed_rate</v>
       </c>
       <c r="P39" t="s">
         <v>49</v>
       </c>
       <c r="Q39">
-        <v>1E-3</v>
+        <v>1.2000000000000001E-3</v>
       </c>
       <c r="R39">
-        <v>1E-3</v>
+        <v>1.2000000000000001E-3</v>
+      </c>
+      <c r="T39" t="s">
+        <v>0</v>
+      </c>
+      <c r="U39" t="s">
+        <v>2</v>
+      </c>
+      <c r="V39" t="s">
+        <v>4</v>
+      </c>
+      <c r="W39" t="s">
+        <v>6</v>
+      </c>
+      <c r="X39" t="s">
+        <v>10</v>
+      </c>
+      <c r="Y39" t="s">
+        <v>12</v>
       </c>
       <c r="AA39" t="b">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v>1</v>
       </c>
       <c r="AB39" t="b">
-        <f t="shared" si="5"/>
+        <f t="shared" si="6"/>
         <v>1</v>
       </c>
       <c r="AC39" t="b">
-        <f t="shared" si="5"/>
-        <v>1</v>
-      </c>
-    </row>
-    <row r="40" spans="5:29" x14ac:dyDescent="0.4">
+        <f t="shared" si="6"/>
+        <v>1</v>
+      </c>
+      <c r="AE39" t="b">
+        <f t="shared" ref="AE39:AE40" si="15">I39=T39</f>
+        <v>1</v>
+      </c>
+      <c r="AF39" t="b">
+        <f t="shared" ref="AF39:AF40" si="16">J39=U39</f>
+        <v>1</v>
+      </c>
+      <c r="AG39" t="b">
+        <f t="shared" ref="AG39:AG40" si="17">K39=V39</f>
+        <v>1</v>
+      </c>
+      <c r="AH39" t="b">
+        <f t="shared" ref="AH39:AH40" si="18">L39=W39</f>
+        <v>1</v>
+      </c>
+      <c r="AI39" t="b">
+        <f t="shared" ref="AI39:AI40" si="19">M39=X39</f>
+        <v>1</v>
+      </c>
+      <c r="AJ39" t="b">
+        <f t="shared" ref="AJ39:AJ40" si="20">N39=Y39</f>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="40" spans="5:36" x14ac:dyDescent="0.4">
       <c r="E40" t="str">
         <v>fixed_leg.cashflows.[3].payment _date</v>
       </c>
@@ -6089,6 +6420,24 @@
         <f t="array" ref="G40">_xll.ExLibris.Json.GetJsonValue($F$1,E40, EXLIBRIS_CONFIGURATION)</f>
         <v>2023-09-03</v>
       </c>
+      <c r="I40" t="str">
+        <v>2023-03-07</v>
+      </c>
+      <c r="J40" t="str">
+        <v>2022-09-08</v>
+      </c>
+      <c r="K40" t="str">
+        <v>2023-03-07</v>
+      </c>
+      <c r="L40" t="str">
+        <v>ACT/360</v>
+      </c>
+      <c r="M40">
+        <v>11000000</v>
+      </c>
+      <c r="N40">
+        <v>1.2000000000000001E-3</v>
+      </c>
       <c r="P40" t="s">
         <v>50</v>
       </c>
@@ -6098,20 +6447,62 @@
       <c r="R40" t="s">
         <v>97</v>
       </c>
+      <c r="T40" t="s">
+        <v>96</v>
+      </c>
+      <c r="U40" t="s">
+        <v>95</v>
+      </c>
+      <c r="V40" t="s">
+        <v>96</v>
+      </c>
+      <c r="W40" t="s">
+        <v>8</v>
+      </c>
+      <c r="X40">
+        <v>11000000</v>
+      </c>
+      <c r="Y40">
+        <v>1.2000000000000001E-3</v>
+      </c>
       <c r="AA40" t="b">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v>1</v>
       </c>
       <c r="AB40" t="b">
-        <f t="shared" si="5"/>
+        <f t="shared" si="6"/>
         <v>1</v>
       </c>
       <c r="AC40" t="b">
-        <f t="shared" si="5"/>
-        <v>1</v>
-      </c>
-    </row>
-    <row r="41" spans="5:29" x14ac:dyDescent="0.4">
+        <f t="shared" si="6"/>
+        <v>1</v>
+      </c>
+      <c r="AE40" t="b">
+        <f t="shared" si="15"/>
+        <v>1</v>
+      </c>
+      <c r="AF40" t="b">
+        <f t="shared" si="16"/>
+        <v>1</v>
+      </c>
+      <c r="AG40" t="b">
+        <f t="shared" si="17"/>
+        <v>1</v>
+      </c>
+      <c r="AH40" t="b">
+        <f t="shared" si="18"/>
+        <v>1</v>
+      </c>
+      <c r="AI40" t="b">
+        <f t="shared" si="19"/>
+        <v>1</v>
+      </c>
+      <c r="AJ40" t="b">
+        <f t="shared" si="20"/>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="41" spans="5:36" x14ac:dyDescent="0.4">
       <c r="E41" t="str">
         <v>fixed_leg.cashflows.[3].start_date</v>
       </c>
@@ -6132,19 +6523,19 @@
         <v>96</v>
       </c>
       <c r="AA41" t="b">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v>1</v>
       </c>
       <c r="AB41" t="b">
-        <f t="shared" si="5"/>
+        <f t="shared" si="6"/>
         <v>1</v>
       </c>
       <c r="AC41" t="b">
-        <f t="shared" si="5"/>
-        <v>1</v>
-      </c>
-    </row>
-    <row r="42" spans="5:29" x14ac:dyDescent="0.4">
+        <f t="shared" si="6"/>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="42" spans="5:36" x14ac:dyDescent="0.4">
       <c r="E42" t="str">
         <v>fixed_leg.cashflows.[3].end_date</v>
       </c>
@@ -6155,6 +6546,10 @@
         <f t="array" ref="G42">_xll.ExLibris.Json.GetJsonValue($F$1,E42, EXLIBRIS_CONFIGURATION)</f>
         <v>2023-09-03</v>
       </c>
+      <c r="I42" t="str" cm="1">
+        <f t="array" ref="I42">_xll.ExLibris.Json.SeachJsonArrayElements(I32,J8,,EXLIBRIS_CONFIGURATION)</f>
+        <v>JsonObject:6AF0E31F-7F9D-4D16-9302-6AF3FF5BAD64</v>
+      </c>
       <c r="P42" t="s">
         <v>52</v>
       </c>
@@ -6165,19 +6560,19 @@
         <v>97</v>
       </c>
       <c r="AA42" t="b">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v>1</v>
       </c>
       <c r="AB42" t="b">
-        <f t="shared" si="5"/>
+        <f t="shared" si="6"/>
         <v>1</v>
       </c>
       <c r="AC42" t="b">
-        <f t="shared" si="5"/>
-        <v>1</v>
-      </c>
-    </row>
-    <row r="43" spans="5:29" x14ac:dyDescent="0.4">
+        <f t="shared" si="6"/>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="43" spans="5:36" x14ac:dyDescent="0.4">
       <c r="E43" t="str">
         <v>fixed_leg.cashflows.[3].day_count_type</v>
       </c>
@@ -6188,6 +6583,10 @@
         <f t="array" ref="G43">_xll.ExLibris.Json.GetJsonValue($F$1,E43, EXLIBRIS_CONFIGURATION)</f>
         <v>ACT/360</v>
       </c>
+      <c r="I43" t="str" cm="1">
+        <f t="array" ref="I43">_xll.ExLibris.Json.GetJsonTable(I42, EXLIBRIS_CONFIGURATION)</f>
+        <v/>
+      </c>
       <c r="P43" t="s">
         <v>53</v>
       </c>
@@ -6197,86 +6596,93 @@
       <c r="R43" t="s">
         <v>8</v>
       </c>
+      <c r="T43" t="s">
+        <v>116</v>
+      </c>
       <c r="AA43" t="b">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v>1</v>
       </c>
       <c r="AB43" t="b">
-        <f t="shared" si="5"/>
+        <f t="shared" si="6"/>
         <v>1</v>
       </c>
       <c r="AC43" t="b">
-        <f t="shared" si="5"/>
-        <v>1</v>
-      </c>
-    </row>
-    <row r="44" spans="5:29" x14ac:dyDescent="0.4">
+        <f t="shared" si="6"/>
+        <v>1</v>
+      </c>
+      <c r="AE43" t="b">
+        <f t="shared" ref="AE43" si="21">I43=T43</f>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="44" spans="5:36" x14ac:dyDescent="0.4">
       <c r="E44" t="str">
         <v>fixed_leg.cashflows.[3].amout</v>
       </c>
       <c r="F44">
-        <v>13000000</v>
+        <v>11000000</v>
       </c>
       <c r="G44" cm="1">
         <f t="array" ref="G44">_xll.ExLibris.Json.GetJsonValue($F$1,E44, EXLIBRIS_CONFIGURATION)</f>
-        <v>13000000</v>
+        <v>11000000</v>
       </c>
       <c r="P44" t="s">
         <v>54</v>
       </c>
       <c r="Q44">
-        <v>13000000</v>
+        <v>11000000</v>
       </c>
       <c r="R44">
-        <v>13000000</v>
+        <v>11000000</v>
       </c>
       <c r="AA44" t="b">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v>1</v>
       </c>
       <c r="AB44" t="b">
-        <f t="shared" si="5"/>
+        <f t="shared" si="6"/>
         <v>1</v>
       </c>
       <c r="AC44" t="b">
-        <f t="shared" si="5"/>
-        <v>1</v>
-      </c>
-    </row>
-    <row r="45" spans="5:29" x14ac:dyDescent="0.4">
+        <f t="shared" si="6"/>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="45" spans="5:36" x14ac:dyDescent="0.4">
       <c r="E45" t="str">
         <v>fixed_leg.cashflows.[3].fixed_rate</v>
       </c>
       <c r="F45">
-        <v>1E-3</v>
+        <v>1.3000000000000002E-3</v>
       </c>
       <c r="G45" cm="1">
         <f t="array" ref="G45">_xll.ExLibris.Json.GetJsonValue($F$1,E45, EXLIBRIS_CONFIGURATION)</f>
-        <v>1E-3</v>
+        <v>1.3000000000000002E-3</v>
       </c>
       <c r="P45" t="s">
         <v>55</v>
       </c>
       <c r="Q45">
-        <v>1E-3</v>
+        <v>1.3000000000000002E-3</v>
       </c>
       <c r="R45">
-        <v>1E-3</v>
+        <v>1.3000000000000002E-3</v>
       </c>
       <c r="AA45" t="b">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v>1</v>
       </c>
       <c r="AB45" t="b">
-        <f t="shared" si="5"/>
+        <f t="shared" si="6"/>
         <v>1</v>
       </c>
       <c r="AC45" t="b">
-        <f t="shared" si="5"/>
-        <v>1</v>
-      </c>
-    </row>
-    <row r="46" spans="5:29" x14ac:dyDescent="0.4">
+        <f t="shared" si="6"/>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="46" spans="5:36" x14ac:dyDescent="0.4">
       <c r="E46" t="str">
         <v>fixed_leg.cashflows.[4].payment _date</v>
       </c>
@@ -6297,19 +6703,19 @@
         <v>98</v>
       </c>
       <c r="AA46" t="b">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v>1</v>
       </c>
       <c r="AB46" t="b">
-        <f t="shared" si="5"/>
+        <f t="shared" si="6"/>
         <v>1</v>
       </c>
       <c r="AC46" t="b">
-        <f t="shared" si="5"/>
-        <v>1</v>
-      </c>
-    </row>
-    <row r="47" spans="5:29" x14ac:dyDescent="0.4">
+        <f t="shared" si="6"/>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="47" spans="5:36" x14ac:dyDescent="0.4">
       <c r="E47" t="str">
         <v>fixed_leg.cashflows.[4].start_date</v>
       </c>
@@ -6330,19 +6736,19 @@
         <v>97</v>
       </c>
       <c r="AA47" t="b">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v>1</v>
       </c>
       <c r="AB47" t="b">
-        <f t="shared" si="5"/>
+        <f t="shared" si="6"/>
         <v>1</v>
       </c>
       <c r="AC47" t="b">
-        <f t="shared" si="5"/>
-        <v>1</v>
-      </c>
-    </row>
-    <row r="48" spans="5:29" x14ac:dyDescent="0.4">
+        <f t="shared" si="6"/>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="48" spans="5:36" x14ac:dyDescent="0.4">
       <c r="E48" t="str">
         <v>fixed_leg.cashflows.[4].end_date</v>
       </c>
@@ -6363,15 +6769,15 @@
         <v>98</v>
       </c>
       <c r="AA48" t="b">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v>1</v>
       </c>
       <c r="AB48" t="b">
-        <f t="shared" si="5"/>
+        <f t="shared" si="6"/>
         <v>1</v>
       </c>
       <c r="AC48" t="b">
-        <f t="shared" si="5"/>
+        <f t="shared" si="6"/>
         <v>1</v>
       </c>
     </row>
@@ -6396,15 +6802,15 @@
         <v>8</v>
       </c>
       <c r="AA49" t="b">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v>1</v>
       </c>
       <c r="AB49" t="b">
-        <f t="shared" si="5"/>
+        <f t="shared" si="6"/>
         <v>1</v>
       </c>
       <c r="AC49" t="b">
-        <f t="shared" si="5"/>
+        <f t="shared" si="6"/>
         <v>1</v>
       </c>
     </row>
@@ -6413,31 +6819,31 @@
         <v>fixed_leg.cashflows.[4].amout</v>
       </c>
       <c r="F50">
-        <v>14000000</v>
+        <v>12000000</v>
       </c>
       <c r="G50" cm="1">
         <f t="array" ref="G50">_xll.ExLibris.Json.GetJsonValue($F$1,E50, EXLIBRIS_CONFIGURATION)</f>
-        <v>14000000</v>
+        <v>12000000</v>
       </c>
       <c r="P50" t="s">
         <v>60</v>
       </c>
       <c r="Q50">
-        <v>14000000</v>
+        <v>12000000</v>
       </c>
       <c r="R50">
-        <v>14000000</v>
+        <v>12000000</v>
       </c>
       <c r="AA50" t="b">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v>1</v>
       </c>
       <c r="AB50" t="b">
-        <f t="shared" si="5"/>
+        <f t="shared" si="6"/>
         <v>1</v>
       </c>
       <c r="AC50" t="b">
-        <f t="shared" si="5"/>
+        <f t="shared" si="6"/>
         <v>1</v>
       </c>
     </row>
@@ -6446,31 +6852,31 @@
         <v>fixed_leg.cashflows.[4].fixed_rate</v>
       </c>
       <c r="F51">
-        <v>1E-3</v>
+        <v>1.4000000000000002E-3</v>
       </c>
       <c r="G51" cm="1">
         <f t="array" ref="G51">_xll.ExLibris.Json.GetJsonValue($F$1,E51, EXLIBRIS_CONFIGURATION)</f>
-        <v>1E-3</v>
+        <v>1.4000000000000002E-3</v>
       </c>
       <c r="P51" t="s">
         <v>61</v>
       </c>
       <c r="Q51">
-        <v>1E-3</v>
+        <v>1.4000000000000002E-3</v>
       </c>
       <c r="R51">
-        <v>1E-3</v>
+        <v>1.4000000000000002E-3</v>
       </c>
       <c r="AA51" t="b">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v>1</v>
       </c>
       <c r="AB51" t="b">
-        <f t="shared" si="5"/>
+        <f t="shared" si="6"/>
         <v>1</v>
       </c>
       <c r="AC51" t="b">
-        <f t="shared" si="5"/>
+        <f t="shared" si="6"/>
         <v>1</v>
       </c>
     </row>
@@ -6495,15 +6901,15 @@
         <v>99</v>
       </c>
       <c r="AA52" t="b">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v>1</v>
       </c>
       <c r="AB52" t="b">
-        <f t="shared" si="5"/>
+        <f t="shared" si="6"/>
         <v>1</v>
       </c>
       <c r="AC52" t="b">
-        <f t="shared" si="5"/>
+        <f t="shared" si="6"/>
         <v>1</v>
       </c>
     </row>
@@ -6528,15 +6934,15 @@
         <v>98</v>
       </c>
       <c r="AA53" t="b">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v>1</v>
       </c>
       <c r="AB53" t="b">
-        <f t="shared" si="5"/>
+        <f t="shared" si="6"/>
         <v>1</v>
       </c>
       <c r="AC53" t="b">
-        <f t="shared" si="5"/>
+        <f t="shared" si="6"/>
         <v>1</v>
       </c>
     </row>
@@ -6561,15 +6967,15 @@
         <v>99</v>
       </c>
       <c r="AA54" t="b">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v>1</v>
       </c>
       <c r="AB54" t="b">
-        <f t="shared" si="5"/>
+        <f t="shared" si="6"/>
         <v>1</v>
       </c>
       <c r="AC54" t="b">
-        <f t="shared" si="5"/>
+        <f t="shared" si="6"/>
         <v>1</v>
       </c>
     </row>
@@ -6594,15 +7000,15 @@
         <v>8</v>
       </c>
       <c r="AA55" t="b">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v>1</v>
       </c>
       <c r="AB55" t="b">
-        <f t="shared" si="5"/>
+        <f t="shared" si="6"/>
         <v>1</v>
       </c>
       <c r="AC55" t="b">
-        <f t="shared" si="5"/>
+        <f t="shared" si="6"/>
         <v>1</v>
       </c>
     </row>
@@ -6611,31 +7017,31 @@
         <v>fixed_leg.cashflows.[5].amout</v>
       </c>
       <c r="F56">
-        <v>15000000</v>
+        <v>12000000</v>
       </c>
       <c r="G56" cm="1">
         <f t="array" ref="G56">_xll.ExLibris.Json.GetJsonValue($F$1,E56, EXLIBRIS_CONFIGURATION)</f>
-        <v>15000000</v>
+        <v>12000000</v>
       </c>
       <c r="P56" t="s">
         <v>66</v>
       </c>
       <c r="Q56">
-        <v>15000000</v>
+        <v>12000000</v>
       </c>
       <c r="R56">
-        <v>15000000</v>
+        <v>12000000</v>
       </c>
       <c r="AA56" t="b">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v>1</v>
       </c>
       <c r="AB56" t="b">
-        <f t="shared" si="5"/>
+        <f t="shared" si="6"/>
         <v>1</v>
       </c>
       <c r="AC56" t="b">
-        <f t="shared" si="5"/>
+        <f t="shared" si="6"/>
         <v>1</v>
       </c>
     </row>
@@ -6644,31 +7050,31 @@
         <v>fixed_leg.cashflows.[5].fixed_rate</v>
       </c>
       <c r="F57">
-        <v>1E-3</v>
+        <v>1.5000000000000002E-3</v>
       </c>
       <c r="G57" cm="1">
         <f t="array" ref="G57">_xll.ExLibris.Json.GetJsonValue($F$1,E57, EXLIBRIS_CONFIGURATION)</f>
-        <v>1E-3</v>
+        <v>1.5000000000000002E-3</v>
       </c>
       <c r="P57" t="s">
         <v>67</v>
       </c>
       <c r="Q57">
-        <v>1E-3</v>
+        <v>1.5000000000000002E-3</v>
       </c>
       <c r="R57">
-        <v>1E-3</v>
+        <v>1.5000000000000002E-3</v>
       </c>
       <c r="AA57" t="b">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v>1</v>
       </c>
       <c r="AB57" t="b">
-        <f t="shared" si="5"/>
+        <f t="shared" si="6"/>
         <v>1</v>
       </c>
       <c r="AC57" t="b">
-        <f t="shared" si="5"/>
+        <f t="shared" si="6"/>
         <v>1</v>
       </c>
     </row>
@@ -6696,7 +7102,7 @@
       </c>
       <c r="C2" t="str" cm="1">
         <f t="array" ref="C2">_xll.ExLibris.LoadConfiguration(B6:C15)</f>
-        <v>ExLibris.Core.ExLibrisConfiguration:3DBC2D14-284C-4875-833A-7330C5C56AB2</v>
+        <v>ExLibris.Core.ExLibrisConfiguration:23598F7C-BC8C-460B-B094-6B7B1D5D478C</v>
       </c>
     </row>
     <row r="4" spans="2:6" s="4" customFormat="1" ht="18" x14ac:dyDescent="0.4">
@@ -6868,30 +7274,30 @@
   <sheetData>
     <row r="2" spans="2:5" s="4" customFormat="1" ht="18" x14ac:dyDescent="0.4">
       <c r="B2" s="4" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
     </row>
     <row r="4" spans="2:5" x14ac:dyDescent="0.4">
       <c r="D4" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="E4" t="str" cm="1">
         <f t="array" ref="E4">_xll.ExLibris.WebSockets.OpenWebSocket("ws://localhost:10101",,D4)</f>
-        <v>ExLibris.Core.WebSockets.WebsocketClient:2A1B90EA-4103-4F63-A62D-8F47A3FDC4C9</v>
+        <v>ExLibris.Core.WebSockets.WebsocketClient:5A633BFF-4691-4566-A934-9DDD80FC2D74</v>
       </c>
     </row>
     <row r="6" spans="2:5" x14ac:dyDescent="0.4">
       <c r="D6" t="s">
-        <v>102</v>
-      </c>
-      <c r="E6" t="e" cm="1">
+        <v>101</v>
+      </c>
+      <c r="E6" t="str" cm="1">
         <f t="array" ref="E6">_xll.ExLibris.WebSockets.ObserveWebSocketStatus(E4,1000)</f>
-        <v>#N/A</v>
+        <v>Closed</v>
       </c>
     </row>
     <row r="7" spans="2:5" x14ac:dyDescent="0.4">
       <c r="D7" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="E7" t="e" cm="1">
         <f t="array" ref="E7">_xll.ExLibris.WebSockets.ObserveWebSocketMessage(E4)</f>
@@ -6900,7 +7306,7 @@
     </row>
     <row r="9" spans="2:5" x14ac:dyDescent="0.4">
       <c r="D9" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="E9" t="e" cm="1">
         <f t="array" ref="E9">_xll.ExLibris.WebSockets.SendWebSocketMessage(E4,"test "&amp;D9,E6="Open")</f>
@@ -6909,7 +7315,7 @@
     </row>
     <row r="10" spans="2:5" x14ac:dyDescent="0.4">
       <c r="D10" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="E10" t="e" cm="1">
         <f t="array" ref="E10">_xll.ExLibris.WebSockets.SendWebSocketMessage($E$4,"test next "&amp;D10,E9)</f>
@@ -6918,7 +7324,7 @@
     </row>
     <row r="11" spans="2:5" x14ac:dyDescent="0.4">
       <c r="D11" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="E11" t="e" cm="1">
         <f t="array" ref="E11">_xll.ExLibris.WebSockets.SendWebSocketMessage($E$4,"test next "&amp;D11,E10)</f>
@@ -6927,7 +7333,7 @@
     </row>
     <row r="12" spans="2:5" x14ac:dyDescent="0.4">
       <c r="D12" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="E12" t="e" cm="1">
         <f t="array" ref="E12">_xll.ExLibris.WebSockets.SendWebSocketMessage($E$4,"test next "&amp;D12,E11)</f>
@@ -6936,7 +7342,7 @@
     </row>
     <row r="13" spans="2:5" x14ac:dyDescent="0.4">
       <c r="D13" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="E13" t="e" cm="1">
         <f t="array" ref="E13">_xll.ExLibris.WebSockets.SendWebSocketMessage($E$4,"test next "&amp;D13,E12)</f>
@@ -6945,7 +7351,7 @@
     </row>
     <row r="14" spans="2:5" x14ac:dyDescent="0.4">
       <c r="D14" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="E14" t="e" cm="1">
         <f t="array" ref="E14">_xll.ExLibris.WebSockets.SendWebSocketMessage($E$4,"test next "&amp;D14,E13)</f>
@@ -6954,7 +7360,7 @@
     </row>
     <row r="15" spans="2:5" x14ac:dyDescent="0.4">
       <c r="D15" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="E15" t="e" cm="1">
         <f t="array" ref="E15">_xll.ExLibris.WebSockets.SendWebSocketMessage($E$4,"test next "&amp;D15,E14)</f>
@@ -6963,16 +7369,16 @@
     </row>
     <row r="17" spans="4:5" x14ac:dyDescent="0.4">
       <c r="D17" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="E17" t="str" cm="1">
         <f t="array" ref="E17">_xll.ExLibris.WebSockets.OpenWebSocket("ws://localhost:10101",,D17)</f>
-        <v>ExLibris.Core.WebSockets.WebsocketClient:30B6D814-1245-4F5D-9185-59306DE1A74C</v>
+        <v>ExLibris.Core.WebSockets.WebsocketClient:6F42C26C-72F1-4ED5-B8A4-01C93DB2F850</v>
       </c>
     </row>
     <row r="19" spans="4:5" x14ac:dyDescent="0.4">
       <c r="D19" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="E19" t="str" cm="1">
         <f t="array" ref="E19">_xll.ExLibris.WebSockets.ObserveWebSocketStatus(E17,1000)</f>
@@ -6981,74 +7387,74 @@
     </row>
     <row r="20" spans="4:5" x14ac:dyDescent="0.4">
       <c r="D20" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="E20" t="str" cm="1">
         <f t="array" ref="E20">_xll.ExLibris.WebSockets.ObserveWebSocketMessage(E17)</f>
-        <v>push_event 22:43:08</v>
+        <v>push_event 23:13:14</v>
       </c>
     </row>
     <row r="22" spans="4:5" x14ac:dyDescent="0.4">
       <c r="D22" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="E22" t="str" cm="1">
         <f t="array" ref="E22">_xll.ExLibris.WebSockets.SendWebSocketMessage(E17,"test "&amp;D22,E19="Open")</f>
-        <v>message sent : 2021-09-21T10:42:23.782</v>
+        <v>message sent : 2021-09-21T11:08:38.139</v>
       </c>
     </row>
     <row r="23" spans="4:5" x14ac:dyDescent="0.4">
       <c r="D23" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="E23" t="str" cm="1">
         <f t="array" ref="E23">_xll.ExLibris.WebSockets.SendWebSocketMessage($E$4,"test next "&amp;D23,E22)</f>
-        <v>message sent : 2021-09-21T10:42:23.801</v>
+        <v>message sent : 2021-09-21T11:08:38.157</v>
       </c>
     </row>
     <row r="24" spans="4:5" x14ac:dyDescent="0.4">
       <c r="D24" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="E24" t="str" cm="1">
         <f t="array" ref="E24">_xll.ExLibris.WebSockets.SendWebSocketMessage($E$4,"test next "&amp;D24,E23)</f>
-        <v>message sent : 2021-09-21T10:42:23.801</v>
+        <v>message sent : 2021-09-21T11:08:38.188</v>
       </c>
     </row>
     <row r="25" spans="4:5" x14ac:dyDescent="0.4">
       <c r="D25" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="E25" t="str" cm="1">
         <f t="array" ref="E25">_xll.ExLibris.WebSockets.SendWebSocketMessage($E$4,"test next "&amp;D25,E24)</f>
-        <v>message sent : 2021-09-21T10:42:23.818</v>
+        <v>message sent : 2021-09-21T11:08:38.208</v>
       </c>
     </row>
     <row r="26" spans="4:5" x14ac:dyDescent="0.4">
       <c r="D26" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="E26" t="str" cm="1">
         <f t="array" ref="E26">_xll.ExLibris.WebSockets.SendWebSocketMessage($E$4,"test next "&amp;D26,E25)</f>
-        <v>message sent : 2021-09-21T10:42:23.861</v>
+        <v>message sent : 2021-09-21T11:08:38.217</v>
       </c>
     </row>
     <row r="27" spans="4:5" x14ac:dyDescent="0.4">
       <c r="D27" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="E27" t="str" cm="1">
         <f t="array" ref="E27">_xll.ExLibris.WebSockets.SendWebSocketMessage($E$4,"test next "&amp;D27,E26)</f>
-        <v>message sent : 2021-09-21T10:42:23.878</v>
+        <v>message sent : 2021-09-21T11:08:38.238</v>
       </c>
     </row>
     <row r="28" spans="4:5" x14ac:dyDescent="0.4">
       <c r="D28" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="E28" t="str" cm="1">
         <f t="array" ref="E28">_xll.ExLibris.WebSockets.SendWebSocketMessage($E$4,"test next "&amp;D28,E27)</f>
-        <v>message sent : 2021-09-21T10:42:23.886</v>
+        <v>message sent : 2021-09-21T11:08:38.276</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
keys of registered objects
</commit_message>
<xml_diff>
--- a/ExLibris/test_excel/exlibris_test.xlsx
+++ b/ExLibris/test_excel/exlibris_test.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\mugen\git\ex-libris\ExLibris\test_excel\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A09AF23E-B13E-4D3F-AA6B-2751D4DADB9A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{89A03140-CF45-4D3C-820E-F40428F495FA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" activeTab="1" xr2:uid="{705CD0B7-27A9-4291-85BD-6034C0FEE3E4}"/>
   </bookViews>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/metadata.xml><?xml version="1.0" encoding="utf-8"?>
-<metadata xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xlrd="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata" xmlns:xda="http://schemas.microsoft.com/office/spreadsheetml/2017/dynamicarray">
+<metadata xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xda="http://schemas.microsoft.com/office/spreadsheetml/2017/dynamicarray">
   <metadataTypes count="1">
     <metadataType name="XLDAPR" minSupportedVersion="120000" copy="1" pasteAll="1" pasteValues="1" merge="1" splitFirst="1" rowColShift="1" clearFormats="1" clearComments="1" assign="1" coerce="1" cellMeta="1"/>
   </metadataTypes>
@@ -568,695 +568,709 @@
 <file path=xl/volatileDependencies.xml><?xml version="1.0" encoding="utf-8"?>
 <volTypes xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <volType type="realTimeData">
-    <main first="rtdsrv.0283c6361b6f4b11963d8af96e32e10b">
-      <tp>
-        <v>1</v>
-        <stp/>
-        <stp>0a5b767d-2c0d-4667-b21e-681ebdb69761</stp>
-        <tr r="G37" s="4"/>
-      </tp>
-      <tp>
-        <v>1</v>
-        <stp/>
-        <stp>79bb9cc5-ab9d-4b90-98b1-c384a6508df6</stp>
-        <tr r="G32" s="4"/>
-      </tp>
-      <tp>
-        <v>1</v>
-        <stp/>
-        <stp>2c075992-a4a9-4c1d-81a2-293828bca7ac</stp>
-        <tr r="G35" s="1"/>
+    <main first="rtdsrv.4d0052b8a95742c6a15f6fa4fe5ede69">
+      <tp>
+        <v>1</v>
+        <stp/>
+        <stp>2b11cf95-fd63-461a-8a73-c443748e2d60</stp>
+        <tr r="G36" s="1"/>
       </tp>
     </main>
-    <main first="rtdsrv.0283c6361b6f4b11963d8af96e32e10b">
-      <tp>
-        <v>1</v>
-        <stp/>
-        <stp>9d75c974-4696-4850-a778-5110e5d04c69</stp>
-        <tr r="G48" s="1"/>
+    <main first="rtdsrv.4d0052b8a95742c6a15f6fa4fe5ede69">
+      <tp>
+        <v>1</v>
+        <stp/>
+        <stp>e4f013b8-fb2d-492e-98a7-752ecaa58a30</stp>
+        <tr r="G31" s="1"/>
       </tp>
     </main>
-    <main first="rtdsrv.0283c6361b6f4b11963d8af96e32e10b">
-      <tp>
-        <v>1</v>
-        <stp/>
-        <stp>11c4a480-bf05-44ff-b422-afa33e54f953</stp>
-        <tr r="G41" s="4"/>
+    <main first="rtdsrv.4d0052b8a95742c6a15f6fa4fe5ede69">
+      <tp>
+        <v>1</v>
+        <stp/>
+        <stp>46b1f2fc-6178-45e4-a65e-825eb27d9b2c</stp>
+        <tr r="G29" s="1"/>
       </tp>
     </main>
-    <main first="rtdsrv.0283c6361b6f4b11963d8af96e32e10b">
-      <tp>
-        <v>1</v>
-        <stp/>
-        <stp>71964b75-97bb-48e6-814e-fd6edf65ecfd</stp>
-        <tr r="G35" s="4"/>
-      </tp>
-      <tp>
-        <v>1</v>
-        <stp/>
-        <stp>ad9d6985-9ef3-471f-848b-d4b2e5ccf264</stp>
+    <main first="rtdsrv.4d0052b8a95742c6a15f6fa4fe5ede69">
+      <tp>
+        <v>1</v>
+        <stp/>
+        <stp>4cf63580-055e-42ae-8a95-e9d5b3431bec</stp>
+        <tr r="E17" s="3"/>
+      </tp>
+    </main>
+    <main first="rtdsrv.4d0052b8a95742c6a15f6fa4fe5ede69">
+      <tp>
+        <v>1</v>
+        <stp/>
+        <stp>6029f4af-5828-4a06-9df0-5ffa9e0331eb</stp>
+        <tr r="G25" s="1"/>
+      </tp>
+    </main>
+    <main first="rtdsrv.4d0052b8a95742c6a15f6fa4fe5ede69">
+      <tp>
+        <v>1</v>
+        <stp/>
+        <stp>5bc05b15-10d6-48f4-a731-b4db87fcef44</stp>
+        <tr r="G33" s="4"/>
+      </tp>
+      <tp>
+        <v>1</v>
+        <stp/>
+        <stp>a55683b4-3907-48f0-acf9-40a493fa7318</stp>
+        <tr r="G28" s="4"/>
+      </tp>
+      <tp>
+        <v>1</v>
+        <stp/>
+        <stp>d2b5ad53-87c2-44d9-b164-ff6192fd6f1c</stp>
+        <tr r="G19" s="1"/>
+      </tp>
+    </main>
+    <main first="rtdsrv.4d0052b8a95742c6a15f6fa4fe5ede69">
+      <tp>
+        <v>1</v>
+        <stp/>
+        <stp>670c4cb8-d842-40bc-ba41-bb86a5a8cdfc</stp>
+        <tr r="I28" s="4"/>
+      </tp>
+    </main>
+    <main first="rtdsrv.4d0052b8a95742c6a15f6fa4fe5ede69">
+      <tp>
+        <v>1</v>
+        <stp/>
+        <stp>d56ea897-e572-41b9-a6cb-c16b9f57a1cb</stp>
+        <tr r="G53" s="4"/>
+      </tp>
+    </main>
+    <main first="rtdsrv.4d0052b8a95742c6a15f6fa4fe5ede69">
+      <tp>
+        <v>1</v>
+        <stp/>
+        <stp>0714adcc-9276-4742-aea9-9882c612db90</stp>
+        <tr r="G27" s="4"/>
+      </tp>
+    </main>
+    <main first="rtdsrv.4d0052b8a95742c6a15f6fa4fe5ede69">
+      <tp>
+        <v>1</v>
+        <stp/>
+        <stp>0315530b-2cdd-4eed-8529-909b18b279c9</stp>
+        <tr r="G48" s="4"/>
+      </tp>
+      <tp>
+        <v>1</v>
+        <stp/>
+        <stp>77fd5d79-dd7d-4a94-b809-b7d64de3f55b</stp>
+        <tr r="P29" s="1"/>
+      </tp>
+    </main>
+    <main first="rtdsrv.4d0052b8a95742c6a15f6fa4fe5ede69">
+      <tp>
+        <v>1</v>
+        <stp/>
+        <stp>b87b5514-0119-4e95-b5f2-69fe71c00321</stp>
+        <tr r="G37" s="1"/>
+      </tp>
+    </main>
+    <main first="rtdsrv.4d0052b8a95742c6a15f6fa4fe5ede69">
+      <tp>
+        <v>1</v>
+        <stp/>
+        <stp>c6929708-2854-47e1-99e7-5e62e0ec2d43</stp>
+        <tr r="G51" s="4"/>
+      </tp>
+      <tp>
+        <v>1</v>
+        <stp/>
+        <stp>b8e741da-0361-4ba3-be92-be9a80544021</stp>
+        <tr r="G50" s="4"/>
+      </tp>
+    </main>
+    <main first="rtdsrv.4d0052b8a95742c6a15f6fa4fe5ede69">
+      <tp>
+        <v>2</v>
+        <stp/>
+        <stp>ebef0892-d459-4436-8685-93d757951b1b</stp>
+        <tr r="E6" s="3"/>
+      </tp>
+    </main>
+    <main first="rtdsrv.4d0052b8a95742c6a15f6fa4fe5ede69">
+      <tp>
+        <v>1</v>
+        <stp/>
+        <stp>cdb18f07-052d-4f9b-a404-c2c36186e458</stp>
+        <tr r="G47" s="1"/>
+      </tp>
+      <tp>
+        <v>1</v>
+        <stp/>
+        <stp>69b80b53-5886-4660-91f0-e8545cb3c457</stp>
+        <tr r="I33" s="4"/>
+      </tp>
+    </main>
+    <main first="rtdsrv.4d0052b8a95742c6a15f6fa4fe5ede69">
+      <tp>
+        <v>1</v>
+        <stp/>
+        <stp>4c0cb919-a736-4c2f-850b-98e3d4fe96c4</stp>
         <tr r="G20" s="1"/>
       </tp>
-      <tp>
-        <v>1</v>
-        <stp/>
-        <stp>1a26cff1-62dd-46a9-bc02-da6ee3c2ec2d</stp>
-        <tr r="G56" s="1"/>
-      </tp>
     </main>
-    <main first="rtdsrv.0283c6361b6f4b11963d8af96e32e10b">
-      <tp>
-        <v>1</v>
-        <stp/>
-        <stp>494cb52c-09ee-451d-9707-bdab376cb11f</stp>
-        <tr r="G45" s="1"/>
+    <main first="rtdsrv.4d0052b8a95742c6a15f6fa4fe5ede69">
+      <tp>
+        <v>1</v>
+        <stp/>
+        <stp>104b40a4-e355-4695-b0cf-a680d69bbd7f</stp>
+        <tr r="G38" s="4"/>
       </tp>
     </main>
-    <main first="rtdsrv.0283c6361b6f4b11963d8af96e32e10b">
-      <tp>
-        <v>1</v>
-        <stp/>
-        <stp>a7fc733b-4306-47f1-b303-91a0733bd96e</stp>
+    <main first="rtdsrv.4d0052b8a95742c6a15f6fa4fe5ede69">
+      <tp>
+        <v>1</v>
+        <stp/>
+        <stp>98849fdc-61d6-4757-be5e-0114b68765a6</stp>
+        <tr r="G30" s="4"/>
+      </tp>
+      <tp>
+        <v>1</v>
+        <stp/>
+        <stp>49c5511b-68bb-4a9d-8b76-eecc84110ec0</stp>
+        <tr r="G24" s="1"/>
+      </tp>
+      <tp>
+        <v>1</v>
+        <stp/>
+        <stp>6d7b2c38-8216-4059-ae04-c6209ab42874</stp>
+        <tr r="F6" s="4"/>
+      </tp>
+    </main>
+    <main first="rtdsrv.4d0052b8a95742c6a15f6fa4fe5ede69">
+      <tp>
+        <v>1</v>
+        <stp/>
+        <stp>d3983292-18bc-4393-b6fc-c6fdd8f68186</stp>
         <tr r="G24" s="4"/>
       </tp>
+      <tp>
+        <v>1</v>
+        <stp/>
+        <stp>e8414323-1a0f-48d4-ac51-86f4ef86413c</stp>
+        <tr r="G49" s="4"/>
+      </tp>
     </main>
-    <main first="rtdsrv.0283c6361b6f4b11963d8af96e32e10b">
-      <tp>
-        <v>1</v>
-        <stp/>
-        <stp>5e89c57d-823d-40ee-803b-ee158b0ad298</stp>
-        <tr r="G23" s="4"/>
-      </tp>
-    </main>
-    <main first="rtdsrv.0283c6361b6f4b11963d8af96e32e10b">
-      <tp>
-        <v>1</v>
-        <stp/>
-        <stp>9e19ad3e-8ac7-4540-a626-24556bba9f46</stp>
-        <tr r="G38" s="1"/>
-      </tp>
-      <tp>
-        <v>1</v>
-        <stp/>
-        <stp>50f7d0ee-ed0a-4314-8706-0a90d5e3f9d4</stp>
-        <tr r="G52" s="4"/>
-      </tp>
-      <tp>
-        <v>1</v>
-        <stp/>
-        <stp>eab1819a-b8ac-4b37-8420-c97e9d574f97</stp>
-        <tr r="G55" s="4"/>
-      </tp>
-    </main>
-    <main first="rtdsrv.0283c6361b6f4b11963d8af96e32e10b">
-      <tp>
-        <v>1</v>
-        <stp/>
-        <stp>ba63b3ea-c5d4-457c-aa45-bb2ac9fb61ef</stp>
-        <tr r="G47" s="4"/>
-      </tp>
-      <tp>
-        <v>1</v>
-        <stp/>
-        <stp>df270489-bf85-4e88-9ec6-21b4203c1f13</stp>
-        <tr r="G49" s="1"/>
-      </tp>
-    </main>
-    <main first="rtdsrv.0283c6361b6f4b11963d8af96e32e10b">
-      <tp>
-        <v>1</v>
-        <stp/>
-        <stp>576c96bd-78ac-4139-8ff4-6e3bc28a92f0</stp>
-        <tr r="C2" s="2"/>
-      </tp>
-    </main>
-    <main first="rtdsrv.0283c6361b6f4b11963d8af96e32e10b">
-      <tp>
-        <v>1</v>
-        <stp/>
-        <stp>80ea02ff-4bf0-4ce4-8769-aef7c93d8e5b</stp>
-        <tr r="I28" s="4"/>
-      </tp>
-    </main>
-    <main first="rtdsrv.0283c6361b6f4b11963d8af96e32e10b">
-      <tp>
-        <v>1</v>
-        <stp/>
-        <stp>f72b93fc-57da-4a79-8c8d-1d0eac79d898</stp>
-        <tr r="G46" s="4"/>
-      </tp>
-    </main>
-    <main first="rtdsrv.0283c6361b6f4b11963d8af96e32e10b">
-      <tp>
-        <v>1</v>
-        <stp/>
-        <stp>9cf72df3-cfa0-496d-9f52-f558b698c9bf</stp>
-        <tr r="I28" s="1"/>
-      </tp>
-      <tp>
-        <v>1</v>
-        <stp/>
-        <stp>a69edd2b-5938-4346-941a-536bbda6083c</stp>
-        <tr r="G53" s="1"/>
-      </tp>
-    </main>
-    <main first="rtdsrv.0283c6361b6f4b11963d8af96e32e10b">
-      <tp>
-        <v>139</v>
-        <stp/>
-        <stp>e1927053-d5ef-4d92-b827-bad9a722f355</stp>
+    <main first="rtdsrv.4d0052b8a95742c6a15f6fa4fe5ede69">
+      <tp>
+        <v>57</v>
+        <stp/>
+        <stp>dad8bdbe-9037-492b-b484-385430b984b7</stp>
         <tr r="E20" s="3"/>
       </tp>
       <tp>
         <v>1</v>
         <stp/>
-        <stp>24ae9bbb-adb5-46e7-9cdc-ea5ef0d95525</stp>
-        <tr r="G22" s="1"/>
-      </tp>
-    </main>
-    <main first="rtdsrv.0283c6361b6f4b11963d8af96e32e10b">
-      <tp>
-        <v>1</v>
-        <stp/>
-        <stp>f91521ea-7295-4df7-913b-f04f08850313</stp>
-        <tr r="G28" s="1"/>
-      </tp>
-      <tp>
-        <v>1</v>
-        <stp/>
-        <stp>d3e0ba7e-11f4-4ded-93ad-f0af33e02e07</stp>
-        <tr r="G23" s="1"/>
-      </tp>
-    </main>
-    <main first="rtdsrv.0283c6361b6f4b11963d8af96e32e10b">
-      <tp>
-        <v>1</v>
-        <stp/>
-        <stp>45ab64ca-418f-4176-9d1e-bb0c000ddac6</stp>
-        <tr r="E4" s="3"/>
-      </tp>
-      <tp>
-        <v>1</v>
-        <stp/>
-        <stp>278c9eff-de88-4e97-b96d-f54f1460b440</stp>
-        <tr r="G28" s="4"/>
-      </tp>
-      <tp>
-        <v>1</v>
-        <stp/>
-        <stp>9f6ecca5-15eb-4707-971f-c7b66c809d05</stp>
-        <tr r="G54" s="1"/>
-      </tp>
-      <tp>
-        <v>1</v>
-        <stp/>
-        <stp>ad40027b-b0cf-42c3-b21e-6270d5cf1389</stp>
-        <tr r="G51" s="1"/>
-      </tp>
-    </main>
-    <main first="rtdsrv.0283c6361b6f4b11963d8af96e32e10b">
-      <tp>
-        <v>2</v>
-        <stp/>
-        <stp>609e9975-c42e-41c3-a60e-320dbafcd898</stp>
-        <tr r="E19" s="3"/>
-      </tp>
-    </main>
-    <main first="rtdsrv.0283c6361b6f4b11963d8af96e32e10b">
-      <tp>
-        <v>1</v>
-        <stp/>
-        <stp>66e3f1a7-dc82-4c18-848e-3f138dbaeccd</stp>
-        <tr r="G48" s="4"/>
-      </tp>
-    </main>
-    <main first="rtdsrv.0283c6361b6f4b11963d8af96e32e10b">
-      <tp>
-        <v>1</v>
-        <stp/>
-        <stp>2e80f495-6d23-4931-8c10-9bcbef252a35</stp>
-        <tr r="G22" s="4"/>
-      </tp>
-    </main>
-    <main first="rtdsrv.0283c6361b6f4b11963d8af96e32e10b">
-      <tp>
-        <v>1</v>
-        <stp/>
-        <stp>9dc87f22-e789-498b-887f-e87ae0db0980</stp>
-        <tr r="G42" s="1"/>
-      </tp>
-    </main>
-    <main first="rtdsrv.0283c6361b6f4b11963d8af96e32e10b">
-      <tp>
-        <v>1</v>
-        <stp/>
-        <stp>a655e98a-9dac-47cf-87ef-6724f5c7840f</stp>
-        <tr r="G24" s="1"/>
-      </tp>
-    </main>
-    <main first="rtdsrv.0283c6361b6f4b11963d8af96e32e10b">
-      <tp>
-        <v>1</v>
-        <stp/>
-        <stp>8e830847-c845-41bb-be9e-5a243184011c</stp>
-        <tr r="G25" s="1"/>
-      </tp>
-      <tp>
-        <v>1</v>
-        <stp/>
-        <stp>9d2fd18b-6a30-4fb8-bd59-485c503e5b4e</stp>
-        <tr r="P19" s="1"/>
-      </tp>
-    </main>
-    <main first="rtdsrv.0283c6361b6f4b11963d8af96e32e10b">
-      <tp>
-        <v>1</v>
-        <stp/>
-        <stp>1c60dd64-2466-49d3-9918-45ff2e7b9c9d</stp>
-        <tr r="G21" s="4"/>
-      </tp>
-      <tp>
-        <v>1</v>
-        <stp/>
-        <stp>ff5c22c2-369f-4487-8e10-b8915ea6382b</stp>
-        <tr r="I42" s="4"/>
-      </tp>
-      <tp>
-        <v>1</v>
-        <stp/>
-        <stp>85c15001-f38a-4ac1-bddb-cc15c02b6a00</stp>
-        <tr r="G36" s="1"/>
-      </tp>
-      <tp>
-        <v>1</v>
-        <stp/>
-        <stp>9ffbd7bb-ffa9-4fcb-848e-fce2f9c0833e</stp>
-        <tr r="G57" s="4"/>
-      </tp>
-      <tp>
-        <v>1</v>
-        <stp/>
-        <stp>c138934d-7354-4caf-9caf-42ad97fb7248</stp>
-        <tr r="G19" s="4"/>
-      </tp>
-    </main>
-    <main first="rtdsrv.0283c6361b6f4b11963d8af96e32e10b">
-      <tp>
-        <v>1</v>
-        <stp/>
-        <stp>cbbe6ba9-2680-41e4-913e-bfcf2a0aa77f</stp>
+        <stp>aa35dd33-8bec-4727-b0f0-86a70c918bdd</stp>
         <tr r="G44" s="4"/>
       </tp>
       <tp>
         <v>1</v>
         <stp/>
-        <stp>4a7bcb66-77cd-4970-9a01-f2ceab246b8b</stp>
-        <tr r="G53" s="4"/>
-      </tp>
-      <tp>
-        <v>1</v>
-        <stp/>
-        <stp>6f4a615d-aa46-434c-9ab4-df19ed2e4335</stp>
-        <tr r="G39" s="4"/>
-      </tp>
-    </main>
-    <main first="rtdsrv.0283c6361b6f4b11963d8af96e32e10b">
-      <tp>
-        <v>1</v>
-        <stp/>
-        <stp>f8929a55-a88b-44db-9885-7a81f572303f</stp>
-        <tr r="G40" s="4"/>
-      </tp>
-    </main>
-    <main first="rtdsrv.0283c6361b6f4b11963d8af96e32e10b">
-      <tp>
-        <v>1</v>
-        <stp/>
-        <stp>b2716693-b771-4d35-a494-64c03823aa58</stp>
-        <tr r="G39" s="1"/>
-      </tp>
-    </main>
-    <main first="rtdsrv.0283c6361b6f4b11963d8af96e32e10b">
-      <tp>
-        <v>1</v>
-        <stp/>
-        <stp>33af8016-04e7-4377-a471-ce4f8af9d018</stp>
-        <tr r="G26" s="4"/>
-      </tp>
-    </main>
-    <main first="rtdsrv.0283c6361b6f4b11963d8af96e32e10b">
-      <tp>
-        <v>1</v>
-        <stp/>
-        <stp>a3f90695-9d61-4ed8-b31e-c8b1bbe0977a</stp>
-        <tr r="G42" s="4"/>
-      </tp>
-      <tp>
-        <v>1</v>
-        <stp/>
-        <stp>5c9ad030-821b-4f1c-895b-6e5e999b9971</stp>
-        <tr r="E7" s="3"/>
-      </tp>
-      <tp>
-        <v>1</v>
-        <stp/>
-        <stp>99bfbf6f-23ef-4990-ab6f-549cdfb64a9a</stp>
-        <tr r="G32" s="1"/>
-      </tp>
-      <tp>
-        <v>1</v>
-        <stp/>
-        <stp>08c5cdbd-f323-4cee-b022-4032ca3c8dce</stp>
-        <tr r="G40" s="1"/>
-      </tp>
-      <tp>
-        <v>1</v>
-        <stp/>
-        <stp>a39a21d3-9a80-4d66-97aa-9727121e71c7</stp>
-        <tr r="G27" s="4"/>
-      </tp>
-      <tp>
-        <v>1</v>
-        <stp/>
-        <stp>a2134fa5-d7d4-4355-9dc4-b4cf637f9982</stp>
+        <stp>6b0179ab-43e2-44c3-9d8b-435c84c0989a</stp>
         <tr r="G26" s="1"/>
       </tp>
-    </main>
-    <main first="rtdsrv.0283c6361b6f4b11963d8af96e32e10b">
-      <tp>
-        <v>1</v>
-        <stp/>
-        <stp>b2d1bb5e-37ec-4e68-a11b-75a887d91109</stp>
-        <tr r="G55" s="1"/>
-      </tp>
-    </main>
-    <main first="rtdsrv.0283c6361b6f4b11963d8af96e32e10b">
-      <tp>
-        <v>1</v>
-        <stp/>
-        <stp>d61d9e4b-241f-49f8-bf8d-4c55fa97b90e</stp>
-        <tr r="E17" s="3"/>
-      </tp>
-      <tp>
-        <v>1</v>
-        <stp/>
-        <stp>86e458ad-7840-4a40-b408-d2d5cb9f7393</stp>
-        <tr r="G25" s="4"/>
-      </tp>
-      <tp>
-        <v>1</v>
-        <stp/>
-        <stp>56c2fa54-9bbc-4552-9d34-60b07c8ecf8a</stp>
-        <tr r="G47" s="1"/>
-      </tp>
-    </main>
-    <main first="rtdsrv.0283c6361b6f4b11963d8af96e32e10b">
-      <tp>
-        <v>1</v>
-        <stp/>
-        <stp>e963b4d4-dc60-4de2-815a-ac34c4325b7c</stp>
-        <tr r="G20" s="4"/>
-      </tp>
-      <tp>
-        <v>1</v>
-        <stp/>
-        <stp>9937bbaa-a783-4863-abc3-1477619f5356</stp>
-        <tr r="P29" s="1"/>
-      </tp>
-    </main>
-    <main first="rtdsrv.0283c6361b6f4b11963d8af96e32e10b">
-      <tp>
-        <v>1</v>
-        <stp/>
-        <stp>11a4f85d-10ab-4f5b-a609-43d62c900fb2</stp>
-        <tr r="G21" s="1"/>
-      </tp>
-    </main>
-    <main first="rtdsrv.0283c6361b6f4b11963d8af96e32e10b">
-      <tp>
-        <v>3</v>
-        <stp/>
-        <stp>a36ca0cf-060a-4d10-8b5f-0505df02792e</stp>
-        <tr r="E6" s="3"/>
-      </tp>
-    </main>
-    <main first="rtdsrv.0283c6361b6f4b11963d8af96e32e10b">
-      <tp>
-        <v>1</v>
-        <stp/>
-        <stp>f5147f57-e942-477b-bc5d-d5be92025832</stp>
-        <tr r="G33" s="4"/>
-      </tp>
-    </main>
-    <main first="rtdsrv.0283c6361b6f4b11963d8af96e32e10b">
-      <tp>
-        <v>1</v>
-        <stp/>
-        <stp>c3cb2885-40fe-449d-bbf7-1b654249c3da</stp>
-        <tr r="F6" s="4"/>
-      </tp>
-      <tp>
-        <v>1</v>
-        <stp/>
-        <stp>0ff35af1-3ec5-4775-91ca-f3220917168b</stp>
-        <tr r="G30" s="1"/>
-      </tp>
-      <tp>
-        <v>1</v>
-        <stp/>
-        <stp>79970d27-e740-4c17-af5f-b3af2d3eb38c</stp>
-        <tr r="G29" s="1"/>
-      </tp>
-      <tp>
-        <v>1</v>
-        <stp/>
-        <stp>141a1fed-1759-426b-b780-8a548c72ceeb</stp>
-        <tr r="I33" s="4"/>
-      </tp>
-    </main>
-    <main first="rtdsrv.0283c6361b6f4b11963d8af96e32e10b">
-      <tp>
-        <v>1</v>
-        <stp/>
-        <stp>f641ffaa-0cd0-4a39-b80a-1c589a79243e</stp>
-        <tr r="G56" s="4"/>
-      </tp>
-      <tp>
-        <v>1</v>
-        <stp/>
-        <stp>d9bce48c-a145-4bc3-8f59-da1aa1b0ae58</stp>
-        <tr r="G57" s="1"/>
-      </tp>
-      <tp>
-        <v>1</v>
-        <stp/>
-        <stp>2f3d2bf1-108c-419c-93df-b01dfd54a90a</stp>
-        <tr r="G44" s="1"/>
-      </tp>
-    </main>
-    <main first="rtdsrv.0283c6361b6f4b11963d8af96e32e10b">
-      <tp>
-        <v>1</v>
-        <stp/>
-        <stp>b8e04dcb-f9a2-4623-9693-f0295ca4a34c</stp>
-        <tr r="G52" s="1"/>
-      </tp>
-    </main>
-    <main first="rtdsrv.0283c6361b6f4b11963d8af96e32e10b">
-      <tp>
-        <v>1</v>
-        <stp/>
-        <stp>f20ed68b-d0e4-45e0-9135-c16e52bf1090</stp>
-        <tr r="G43" s="1"/>
-      </tp>
-      <tp>
-        <v>1</v>
-        <stp/>
-        <stp>6a3813d9-0763-484d-b451-4de952f9851b</stp>
-        <tr r="G54" s="4"/>
-      </tp>
-      <tp>
-        <v>1</v>
-        <stp/>
-        <stp>753f90eb-abb2-4537-adad-cc80deb23d2f</stp>
-        <tr r="G41" s="1"/>
-      </tp>
-    </main>
-    <main first="rtdsrv.0283c6361b6f4b11963d8af96e32e10b">
-      <tp>
-        <v>1</v>
-        <stp/>
-        <stp>60df1138-c085-4b4c-b3d0-ea8b94607ac9</stp>
-        <tr r="G31" s="4"/>
-      </tp>
-      <tp>
-        <v>1</v>
-        <stp/>
-        <stp>d8cb59d9-e18e-4c40-9210-a2c4f78441c6</stp>
-        <tr r="G43" s="4"/>
-      </tp>
-      <tp>
-        <v>1</v>
-        <stp/>
-        <stp>355d1bf7-cde7-4353-bd2e-4bd530e246c6</stp>
-        <tr r="F6" s="1"/>
-      </tp>
-    </main>
-    <main first="rtdsrv.0283c6361b6f4b11963d8af96e32e10b">
-      <tp>
-        <v>1</v>
-        <stp/>
-        <stp>272954a3-5628-403c-aa41-1e8f15653c49</stp>
-        <tr r="G45" s="4"/>
-      </tp>
-    </main>
-    <main first="rtdsrv.0283c6361b6f4b11963d8af96e32e10b">
-      <tp>
-        <v>1</v>
-        <stp/>
-        <stp>086581e9-ff31-4301-a5fa-c84c13d55a84</stp>
-        <tr r="F1" s="4"/>
-      </tp>
-      <tp>
-        <v>1</v>
-        <stp/>
-        <stp>f7f67aaa-40a7-41fe-b9f4-8241e90c4883</stp>
-        <tr r="G49" s="4"/>
-      </tp>
-      <tp>
-        <v>1</v>
-        <stp/>
-        <stp>3b5ca16b-7f32-40ad-9284-90ba68954b58</stp>
-        <tr r="G27" s="1"/>
-      </tp>
-    </main>
-    <main first="rtdsrv.0283c6361b6f4b11963d8af96e32e10b">
-      <tp>
-        <v>1</v>
-        <stp/>
-        <stp>1d52dc5d-def5-48a4-b0e0-136c77f4cee8</stp>
-        <tr r="G34" s="4"/>
-      </tp>
-    </main>
-    <main first="rtdsrv.0283c6361b6f4b11963d8af96e32e10b">
-      <tp>
-        <v>1</v>
-        <stp/>
-        <stp>8d81f2d5-48c3-44b6-89fa-788f2a6b787b</stp>
-        <tr r="I19" s="1"/>
-      </tp>
-      <tp>
-        <v>1</v>
-        <stp/>
-        <stp>11b79eb1-60dc-4082-83e3-512865d2bbac</stp>
-        <tr r="G30" s="4"/>
-      </tp>
-    </main>
-    <main first="rtdsrv.0283c6361b6f4b11963d8af96e32e10b">
-      <tp>
-        <v>1</v>
-        <stp/>
-        <stp>6e00cf5e-d87a-4774-a2c3-26e9532c1a99</stp>
-        <tr r="G36" s="4"/>
-      </tp>
-      <tp>
-        <v>1</v>
-        <stp/>
-        <stp>33b718fa-1d0a-46b9-b22d-ad3aedfb6e2c</stp>
-        <tr r="G34" s="1"/>
-      </tp>
-      <tp>
-        <v>1</v>
-        <stp/>
-        <stp>edee6b00-035b-4a47-b7bd-504d71d07643</stp>
-        <tr r="I38" s="4"/>
-      </tp>
-    </main>
-    <main first="rtdsrv.0283c6361b6f4b11963d8af96e32e10b">
-      <tp>
-        <v>1</v>
-        <stp/>
-        <stp>e0efa2c1-1305-4fd7-8f2c-4f86b795c3fa</stp>
-        <tr r="F1" s="1"/>
-      </tp>
-      <tp>
-        <v>1</v>
-        <stp/>
-        <stp>26b72fdc-0088-4f80-aac6-22bc27e07b25</stp>
-        <tr r="G50" s="1"/>
-      </tp>
-    </main>
-    <main first="rtdsrv.0283c6361b6f4b11963d8af96e32e10b">
-      <tp>
-        <v>1</v>
-        <stp/>
-        <stp>8be0a774-7476-4540-82fd-f7712f7e00af</stp>
-        <tr r="G46" s="1"/>
-      </tp>
-    </main>
-    <main first="rtdsrv.0283c6361b6f4b11963d8af96e32e10b">
-      <tp>
-        <v>1</v>
-        <stp/>
-        <stp>377f1767-bdeb-456a-bfa8-da20e30ade9c</stp>
+      <tp>
+        <v>1</v>
+        <stp/>
+        <stp>a5377819-58f7-4b92-89b7-0ca6e658af6a</stp>
         <tr r="I32" s="4"/>
         <tr r="I19" s="4"/>
       </tp>
       <tp>
         <v>1</v>
         <stp/>
-        <stp>d4f7c6e5-4bcf-4a5b-986f-444caa822b37</stp>
-        <tr r="G31" s="1"/>
+        <stp>0f42f9a3-1016-4858-b6dd-06889fd9c942</stp>
+        <tr r="G40" s="4"/>
       </tp>
     </main>
-    <main first="rtdsrv.0283c6361b6f4b11963d8af96e32e10b">
-      <tp>
-        <v>1</v>
-        <stp/>
-        <stp>0a165bec-66a7-4967-930d-9ce67bad1e9d</stp>
-        <tr r="G38" s="4"/>
+    <main first="rtdsrv.4d0052b8a95742c6a15f6fa4fe5ede69">
+      <tp>
+        <v>1</v>
+        <stp/>
+        <stp>c2520d9d-7d37-4849-adf9-bf1e6f9a5b54</stp>
+        <tr r="F1" s="4"/>
       </tp>
     </main>
-    <main first="rtdsrv.0283c6361b6f4b11963d8af96e32e10b">
-      <tp>
-        <v>1</v>
-        <stp/>
-        <stp>6e255841-2f77-4868-8904-c2b69a9fbcd6</stp>
+    <main first="rtdsrv.4d0052b8a95742c6a15f6fa4fe5ede69">
+      <tp>
+        <v>1</v>
+        <stp/>
+        <stp>aac33ceb-d988-4ec2-b85e-38621011f570</stp>
+        <tr r="G49" s="1"/>
+      </tp>
+    </main>
+    <main first="rtdsrv.4d0052b8a95742c6a15f6fa4fe5ede69">
+      <tp>
+        <v>1</v>
+        <stp/>
+        <stp>ca633845-4280-4e32-9d46-94feee492f29</stp>
+        <tr r="G21" s="1"/>
+      </tp>
+      <tp>
+        <v>1</v>
+        <stp/>
+        <stp>704427e6-3ac1-4dd7-847c-443e7efd99e4</stp>
+        <tr r="G36" s="4"/>
+      </tp>
+      <tp>
+        <v>1</v>
+        <stp/>
+        <stp>2e741680-ff78-4a04-b096-7dbed428b497</stp>
+        <tr r="G52" s="4"/>
+      </tp>
+      <tp>
+        <v>1</v>
+        <stp/>
+        <stp>be5991eb-a186-4f01-86ba-bad63908ac29</stp>
+        <tr r="G47" s="4"/>
+      </tp>
+      <tp>
+        <v>1</v>
+        <stp/>
+        <stp>b22c7e46-dac5-466b-b893-7a2146e20b5f</stp>
+        <tr r="G32" s="4"/>
+      </tp>
+    </main>
+    <main first="rtdsrv.4d0052b8a95742c6a15f6fa4fe5ede69">
+      <tp>
+        <v>1</v>
+        <stp/>
+        <stp>d124d935-7ac7-43a0-85a3-134d60c5b3b2</stp>
+        <tr r="F1" s="1"/>
+      </tp>
+    </main>
+    <main first="rtdsrv.4d0052b8a95742c6a15f6fa4fe5ede69">
+      <tp>
+        <v>1</v>
+        <stp/>
+        <stp>33639009-6595-4ef9-b218-59e189f2bc86</stp>
+        <tr r="G45" s="4"/>
+      </tp>
+      <tp>
+        <v>1</v>
+        <stp/>
+        <stp>0bc113f6-2c51-4179-ac4b-8d6a21363e1d</stp>
+        <tr r="G22" s="1"/>
+      </tp>
+      <tp>
+        <v>1</v>
+        <stp/>
+        <stp>1e3e57bc-d24e-434b-88dc-4bb5054979d9</stp>
+        <tr r="G43" s="1"/>
+      </tp>
+      <tp>
+        <v>1</v>
+        <stp/>
+        <stp>4229dc0b-b766-4729-85d1-9d02c1dbfecb</stp>
+        <tr r="G39" s="4"/>
+      </tp>
+      <tp>
+        <v>1</v>
+        <stp/>
+        <stp>e7095731-0036-4536-a072-09af1c0e25c2</stp>
+        <tr r="G27" s="1"/>
+      </tp>
+    </main>
+    <main first="rtdsrv.4d0052b8a95742c6a15f6fa4fe5ede69">
+      <tp>
+        <v>1</v>
+        <stp/>
+        <stp>4885ad71-26a0-4b08-bcac-f83f71092a97</stp>
+        <tr r="G53" s="1"/>
+      </tp>
+      <tp>
+        <v>1</v>
+        <stp/>
+        <stp>bdcb95dd-8bb0-460b-93da-622af106f3fe</stp>
+        <tr r="G21" s="4"/>
+      </tp>
+      <tp>
+        <v>1</v>
+        <stp/>
+        <stp>dbca8b14-9afb-4546-a752-241940120aba</stp>
+        <tr r="G41" s="4"/>
+      </tp>
+    </main>
+    <main first="rtdsrv.4d0052b8a95742c6a15f6fa4fe5ede69">
+      <tp>
+        <v>1</v>
+        <stp/>
+        <stp>d0d03c74-a6b1-4907-8de6-253bfc86e6e0</stp>
+        <tr r="G57" s="1"/>
+      </tp>
+    </main>
+    <main first="rtdsrv.4d0052b8a95742c6a15f6fa4fe5ede69">
+      <tp>
+        <v>1</v>
+        <stp/>
+        <stp>7843cc4c-28e1-40a1-afbb-04242859677e</stp>
+        <tr r="G55" s="1"/>
+      </tp>
+    </main>
+    <main first="rtdsrv.4d0052b8a95742c6a15f6fa4fe5ede69">
+      <tp>
+        <v>1</v>
+        <stp/>
+        <stp>7e978fba-cda3-4efd-ad41-6b275572ff44</stp>
+        <tr r="G56" s="4"/>
+      </tp>
+    </main>
+    <main first="rtdsrv.4d0052b8a95742c6a15f6fa4fe5ede69">
+      <tp>
+        <v>1</v>
+        <stp/>
+        <stp>df39a10f-63cc-4fd5-9ee4-7ce02a7b72c5</stp>
+        <tr r="G45" s="1"/>
+      </tp>
+      <tp>
+        <v>1</v>
+        <stp/>
+        <stp>1e71f983-acb9-4ada-962e-91835850bf16</stp>
+        <tr r="G39" s="1"/>
+      </tp>
+    </main>
+    <main first="rtdsrv.4d0052b8a95742c6a15f6fa4fe5ede69">
+      <tp>
+        <v>1</v>
+        <stp/>
+        <stp>84668846-63a6-4dae-814f-a07188280bb7</stp>
+        <tr r="I19" s="1"/>
+      </tp>
+    </main>
+    <main first="rtdsrv.4d0052b8a95742c6a15f6fa4fe5ede69">
+      <tp>
+        <v>1</v>
+        <stp/>
+        <stp>aa0eed66-b424-4048-9f9d-e21e830ace80</stp>
+        <tr r="G38" s="1"/>
+      </tp>
+      <tp>
+        <v>1</v>
+        <stp/>
+        <stp>a88bdb55-0a4c-4a61-861c-dbd399c33398</stp>
+        <tr r="I38" s="4"/>
+      </tp>
+    </main>
+    <main first="rtdsrv.4d0052b8a95742c6a15f6fa4fe5ede69">
+      <tp>
+        <v>1</v>
+        <stp/>
+        <stp>c0e0f610-d4c5-429e-8856-f48d66b9e3ad</stp>
+        <tr r="E4" s="3"/>
+      </tp>
+      <tp>
+        <v>1</v>
+        <stp/>
+        <stp>3ced1629-20dc-475a-bbff-f5b92285dd23</stp>
+        <tr r="P19" s="1"/>
+      </tp>
+    </main>
+    <main first="rtdsrv.4d0052b8a95742c6a15f6fa4fe5ede69">
+      <tp>
+        <v>1</v>
+        <stp/>
+        <stp>cd4fd604-3e94-4b9a-9423-eaf8cfc7e67d</stp>
+        <tr r="G20" s="4"/>
+      </tp>
+      <tp>
+        <v>2</v>
+        <stp/>
+        <stp>1cf3d21f-1caf-446b-a59d-9cf02cd4b814</stp>
+        <tr r="E19" s="3"/>
+      </tp>
+      <tp>
+        <v>1</v>
+        <stp/>
+        <stp>bd95a4a0-87eb-45a5-ac93-40742fbbf156</stp>
+        <tr r="G54" s="1"/>
+      </tp>
+    </main>
+    <main first="rtdsrv.4d0052b8a95742c6a15f6fa4fe5ede69">
+      <tp>
+        <v>1</v>
+        <stp/>
+        <stp>38220e8f-0685-4b83-8ac1-8c6458172e04</stp>
+        <tr r="I42" s="4"/>
+      </tp>
+      <tp>
+        <v>1</v>
+        <stp/>
+        <stp>49c00da1-a096-4e7f-91b8-d2481993f023</stp>
+        <tr r="C2" s="2"/>
+      </tp>
+      <tp>
+        <v>1</v>
+        <stp/>
+        <stp>6c6c41bf-25b7-462b-b644-46d44bacdac6</stp>
+        <tr r="G23" s="1"/>
+      </tp>
+      <tp>
+        <v>1</v>
+        <stp/>
+        <stp>f20d93e1-e24c-484f-91c2-8b74c60996a4</stp>
+        <tr r="G56" s="1"/>
+      </tp>
+    </main>
+    <main first="rtdsrv.4d0052b8a95742c6a15f6fa4fe5ede69">
+      <tp>
+        <v>1</v>
+        <stp/>
+        <stp>0a6b14f8-22e6-4bff-84be-df8132c393d3</stp>
+        <tr r="G28" s="1"/>
+      </tp>
+      <tp>
+        <v>1</v>
+        <stp/>
+        <stp>422e3368-3c6b-4429-b696-d1d72128b679</stp>
+        <tr r="I28" s="1"/>
+      </tp>
+    </main>
+    <main first="rtdsrv.4d0052b8a95742c6a15f6fa4fe5ede69">
+      <tp>
+        <v>1</v>
+        <stp/>
+        <stp>0a00d53d-2e3e-47a6-89b7-dc15d7fc3ccd</stp>
+        <tr r="G35" s="1"/>
+      </tp>
+      <tp>
+        <v>1</v>
+        <stp/>
+        <stp>a5bc2f0f-8ac7-4f29-813b-d504178adfe8</stp>
+        <tr r="G54" s="4"/>
+      </tp>
+    </main>
+    <main first="rtdsrv.4d0052b8a95742c6a15f6fa4fe5ede69">
+      <tp>
+        <v>1</v>
+        <stp/>
+        <stp>716a72bc-3530-430a-9f94-ac838536b83b</stp>
+        <tr r="G41" s="1"/>
+      </tp>
+    </main>
+    <main first="rtdsrv.4d0052b8a95742c6a15f6fa4fe5ede69">
+      <tp>
+        <v>1</v>
+        <stp/>
+        <stp>4d8ea511-0a26-4b3d-bf58-adf10ee4a71a</stp>
+        <tr r="E7" s="3"/>
+      </tp>
+    </main>
+    <main first="rtdsrv.4d0052b8a95742c6a15f6fa4fe5ede69">
+      <tp>
+        <v>1</v>
+        <stp/>
+        <stp>af2d159d-ae8b-49d9-9f5f-4b066b40e834</stp>
+        <tr r="G25" s="4"/>
+      </tp>
+    </main>
+    <main first="rtdsrv.4d0052b8a95742c6a15f6fa4fe5ede69">
+      <tp>
+        <v>1</v>
+        <stp/>
+        <stp>d66cdeb8-c5bf-4525-898d-b473d726e826</stp>
+        <tr r="G40" s="1"/>
+      </tp>
+    </main>
+    <main first="rtdsrv.4d0052b8a95742c6a15f6fa4fe5ede69">
+      <tp>
+        <v>1</v>
+        <stp/>
+        <stp>999e73b9-4e72-44aa-9bf2-08c8aeba7ce8</stp>
+        <tr r="G48" s="1"/>
+      </tp>
+      <tp>
+        <v>1</v>
+        <stp/>
+        <stp>8b6f1a54-e3f4-4a23-b4ff-5c1f5d14936a</stp>
+        <tr r="G31" s="4"/>
+      </tp>
+    </main>
+    <main first="rtdsrv.4d0052b8a95742c6a15f6fa4fe5ede69">
+      <tp>
+        <v>1</v>
+        <stp/>
+        <stp>1b61cf71-f764-4b64-905d-3634217a5ce9</stp>
+        <tr r="G42" s="4"/>
+      </tp>
+    </main>
+    <main first="rtdsrv.4d0052b8a95742c6a15f6fa4fe5ede69">
+      <tp>
+        <v>1</v>
+        <stp/>
+        <stp>294b4d63-9edc-4184-aa8e-819fadfcb522</stp>
+        <tr r="G19" s="4"/>
+      </tp>
+      <tp>
+        <v>1</v>
+        <stp/>
+        <stp>53c35579-790e-41c5-843a-fcaaddf1885e</stp>
+        <tr r="G30" s="1"/>
+      </tp>
+    </main>
+    <main first="rtdsrv.4d0052b8a95742c6a15f6fa4fe5ede69">
+      <tp>
+        <v>1</v>
+        <stp/>
+        <stp>c74fdf9f-64a9-42df-96df-8da3f018b95d</stp>
+        <tr r="G29" s="4"/>
+      </tp>
+    </main>
+    <main first="rtdsrv.4d0052b8a95742c6a15f6fa4fe5ede69">
+      <tp>
+        <v>1</v>
+        <stp/>
+        <stp>cf45dac4-f22e-46d9-87ac-f4d4bcfddf36</stp>
+        <tr r="G51" s="1"/>
+      </tp>
+    </main>
+    <main first="rtdsrv.4d0052b8a95742c6a15f6fa4fe5ede69">
+      <tp>
+        <v>1</v>
+        <stp/>
+        <stp>ce96b86c-95a4-4f56-b840-1c95b8336520</stp>
+        <tr r="G57" s="4"/>
+      </tp>
+    </main>
+    <main first="rtdsrv.4d0052b8a95742c6a15f6fa4fe5ede69">
+      <tp>
+        <v>1</v>
+        <stp/>
+        <stp>a5f8b11b-42cd-4e13-b32c-d901ec028c5c</stp>
+        <tr r="G23" s="4"/>
+      </tp>
+    </main>
+    <main first="rtdsrv.4d0052b8a95742c6a15f6fa4fe5ede69">
+      <tp>
+        <v>2</v>
+        <stp/>
+        <stp>7f1ba27b-53e4-4b7e-a782-0853694564bd</stp>
+        <tr r="H6" s="2"/>
+      </tp>
+      <tp>
+        <v>1</v>
+        <stp/>
+        <stp>0217233c-e4cc-418a-bbb6-9ed0c2667971</stp>
+        <tr r="G52" s="1"/>
+      </tp>
+      <tp>
+        <v>1</v>
+        <stp/>
+        <stp>c889e564-cfaa-4c9a-9b0f-fa586e6ca1a7</stp>
         <tr r="G33" s="1"/>
       </tp>
-      <tp>
-        <v>1</v>
-        <stp/>
-        <stp>bdfe15f5-d962-4809-a052-51f8695ddf26</stp>
-        <tr r="G19" s="1"/>
-      </tp>
     </main>
-    <main first="rtdsrv.0283c6361b6f4b11963d8af96e32e10b">
-      <tp>
-        <v>1</v>
-        <stp/>
-        <stp>00199060-f9af-4630-b20a-f4efbfbcecd4</stp>
-        <tr r="G50" s="4"/>
-      </tp>
-      <tp>
-        <v>1</v>
-        <stp/>
-        <stp>c23fc26f-fa90-4b0e-8c3c-310977890a04</stp>
-        <tr r="G37" s="1"/>
+    <main first="rtdsrv.4d0052b8a95742c6a15f6fa4fe5ede69">
+      <tp>
+        <v>1</v>
+        <stp/>
+        <stp>4646bd6e-bd49-4737-8f15-d3f6690f864c</stp>
+        <tr r="G42" s="1"/>
+      </tp>
+      <tp>
+        <v>1</v>
+        <stp/>
+        <stp>02805fa5-347c-4a4c-859b-f0b5332c45f5</stp>
+        <tr r="G46" s="1"/>
+      </tp>
+      <tp>
+        <v>1</v>
+        <stp/>
+        <stp>91771e1e-9de6-41fd-8441-1581b3cae7fb</stp>
+        <tr r="G50" s="1"/>
+      </tp>
+      <tp>
+        <v>1</v>
+        <stp/>
+        <stp>45919176-eaa4-41e9-ae69-145ab3addeba</stp>
+        <tr r="G37" s="4"/>
       </tp>
     </main>
-    <main first="rtdsrv.0283c6361b6f4b11963d8af96e32e10b">
-      <tp>
-        <v>1</v>
-        <stp/>
-        <stp>fd6544de-9255-4888-a540-0eb35adf36cd</stp>
-        <tr r="G29" s="4"/>
-      </tp>
-      <tp>
-        <v>1</v>
-        <stp/>
-        <stp>e2d2ba5b-bf0f-4538-bc3f-586c04ca0a37</stp>
-        <tr r="G51" s="4"/>
+    <main first="rtdsrv.4d0052b8a95742c6a15f6fa4fe5ede69">
+      <tp>
+        <v>1</v>
+        <stp/>
+        <stp>736da762-5192-4140-ac9d-5e80acdbb289</stp>
+        <tr r="G34" s="1"/>
+      </tp>
+      <tp>
+        <v>1</v>
+        <stp/>
+        <stp>0d295b6a-26e9-4909-aecc-d0053e431683</stp>
+        <tr r="G32" s="1"/>
+      </tp>
+    </main>
+    <main first="rtdsrv.4d0052b8a95742c6a15f6fa4fe5ede69">
+      <tp>
+        <v>1</v>
+        <stp/>
+        <stp>b0a4f77f-f6ab-4c4d-8a7b-ac72ceb75904</stp>
+        <tr r="G26" s="4"/>
+      </tp>
+      <tp>
+        <v>1</v>
+        <stp/>
+        <stp>20c7e7a9-8c6f-4062-b9a7-eed5f17025de</stp>
+        <tr r="G22" s="4"/>
+      </tp>
+    </main>
+    <main first="rtdsrv.4d0052b8a95742c6a15f6fa4fe5ede69">
+      <tp>
+        <v>1</v>
+        <stp/>
+        <stp>83350920-cda7-4980-9abc-220e374c8375</stp>
+        <tr r="G43" s="4"/>
+      </tp>
+      <tp>
+        <v>1</v>
+        <stp/>
+        <stp>dfd99da8-a579-4632-9b75-0b7ac886f185</stp>
+        <tr r="G34" s="4"/>
+      </tp>
+      <tp>
+        <v>1</v>
+        <stp/>
+        <stp>c6d48c6d-0904-4c4a-99b1-99e4aac1803a</stp>
+        <tr r="G44" s="1"/>
+      </tp>
+      <tp>
+        <v>1</v>
+        <stp/>
+        <stp>cdc845c4-7ae1-4c39-903b-d5d55d7cd351</stp>
+        <tr r="G55" s="4"/>
+      </tp>
+    </main>
+    <main first="rtdsrv.4d0052b8a95742c6a15f6fa4fe5ede69">
+      <tp>
+        <v>1</v>
+        <stp/>
+        <stp>6c0392bc-a65f-40b4-99c5-cba623987800</stp>
+        <tr r="F6" s="1"/>
+      </tp>
+    </main>
+    <main first="rtdsrv.4d0052b8a95742c6a15f6fa4fe5ede69">
+      <tp>
+        <v>1</v>
+        <stp/>
+        <stp>dca6c031-6ce2-45b7-8756-8c148817433f</stp>
+        <tr r="G46" s="4"/>
+      </tp>
+    </main>
+    <main first="rtdsrv.4d0052b8a95742c6a15f6fa4fe5ede69">
+      <tp>
+        <v>1</v>
+        <stp/>
+        <stp>9cd863de-990f-4e1c-ab9f-a19e9903b4e6</stp>
+        <tr r="G35" s="4"/>
       </tp>
     </main>
   </volType>
@@ -1590,11 +1604,11 @@
       </c>
       <c r="F1" t="str" cm="1">
         <f t="array" ref="F1">_xll.ExLibris.Json.CreateJsonObject(E3:F6)</f>
-        <v>JsonObject:76876AD4-5002-4E2F-B04C-A3891F489D96</v>
+        <v>JsonObject:094034A9-8F2E-4DB9-BBA4-B1B6A2AEA0DB</v>
       </c>
       <c r="K1" t="str">
         <f>EXLIBRIS_CONFIGURATION</f>
-        <v>ExLibris.Core.ExLibrisConfiguration:23598F7C-BC8C-460B-B094-6B7B1D5D478C</v>
+        <v>ExLibris.Core.ExLibrisConfiguration:6708C3D9-DE2D-47BE-9248-773006E26782</v>
       </c>
     </row>
     <row r="2" spans="2:28" x14ac:dyDescent="0.4">
@@ -1664,7 +1678,7 @@
       </c>
       <c r="F6" t="str" cm="1">
         <f t="array" ref="F6">_xll.ExLibris.Json.CreateJsonArray(E8:J14)</f>
-        <v>JsonObject:335D9DA4-5359-4486-9EB4-A04CE9A9E1A3</v>
+        <v>JsonObject:4E615853-43E8-41FC-83FD-467E8A931C27</v>
       </c>
       <c r="L6" t="s">
         <v>68</v>
@@ -1903,7 +1917,7 @@
       </c>
       <c r="I19" t="str" cm="1">
         <f t="array" ref="I19">_xll.ExLibris.Json.GetJsonValue(F1,E6)</f>
-        <v>JsonObject:A1901F1D-E8FA-4D73-9D81-905B827A439D</v>
+        <v>JsonObject:2E68A39D-A156-4D80-9D04-AF626B72E3DA</v>
       </c>
       <c r="P19" t="str" cm="1">
         <f t="array" ref="P19:Q27">_xll.ExLibris.Json.GetJsonKeyValues(F1,,3)</f>
@@ -2208,7 +2222,7 @@
         <v>fixed_leg.cashflows.[0]</v>
       </c>
       <c r="Q22" t="str">
-        <v>JsonObject:2E45E8C0-4857-4BBC-8F67-F07DF8F104DE</v>
+        <v>JsonObject:7798C1E6-BB2E-45F5-A0D0-276268D6B6BA</v>
       </c>
       <c r="S22" t="s">
         <v>32</v>
@@ -2307,7 +2321,7 @@
         <v>fixed_leg.cashflows.[1]</v>
       </c>
       <c r="Q23" t="str">
-        <v>JsonObject:0D99B359-988F-4603-B7A3-85B0D393EA96</v>
+        <v>JsonObject:DD53F82E-862B-4076-A9BD-4C94E106716B</v>
       </c>
       <c r="S23" t="s">
         <v>33</v>
@@ -2406,7 +2420,7 @@
         <v>fixed_leg.cashflows.[2]</v>
       </c>
       <c r="Q24" t="str">
-        <v>JsonObject:926A79F0-EE6A-4898-AEED-998440594C6B</v>
+        <v>JsonObject:BD189982-E6DC-45DB-847E-1B555AAB0E0E</v>
       </c>
       <c r="S24" t="s">
         <v>34</v>
@@ -2505,7 +2519,7 @@
         <v>fixed_leg.cashflows.[3]</v>
       </c>
       <c r="Q25" t="str">
-        <v>JsonObject:168243F9-DBCC-4C09-A9BC-805ABAEF10AA</v>
+        <v>JsonObject:468191F2-CEAB-4D55-9615-D6D8FC66E157</v>
       </c>
       <c r="S25" t="s">
         <v>35</v>
@@ -2604,7 +2618,7 @@
         <v>fixed_leg.cashflows.[4]</v>
       </c>
       <c r="Q26" t="str">
-        <v>JsonObject:D7FB3BD5-B53F-4337-81ED-4A956008BD00</v>
+        <v>JsonObject:DA744F30-C5A8-4DB8-8CD0-9A3A26BA7A41</v>
       </c>
       <c r="S26" t="s">
         <v>36</v>
@@ -2685,7 +2699,7 @@
         <v>fixed_leg.cashflows.[5]</v>
       </c>
       <c r="Q27" t="str">
-        <v>JsonObject:EF9CA57C-7F7D-4997-B8CE-C3458BA2C48E</v>
+        <v>JsonObject:3D0ED9D9-1E8A-4EEB-BA45-D0DBE00F1401</v>
       </c>
       <c r="S27" t="s">
         <v>37</v>
@@ -2722,7 +2736,7 @@
       </c>
       <c r="I28" t="str" cm="1">
         <f t="array" ref="I28">_xll.ExLibris.Json.GetJsonValue(I19,"[2]")</f>
-        <v>JsonObject:3B3BE114-1984-48B4-B95C-8BF7D4F473B5</v>
+        <v>JsonObject:06B3FFA1-06C3-451D-9A1E-52B904CFCBEE</v>
       </c>
       <c r="S28" t="s">
         <v>38</v>
@@ -2778,7 +2792,7 @@
       </c>
       <c r="P29" t="str" cm="1">
         <f t="array" ref="P29">_xll.ExLibris.Json.CreateJsonObject(P22:Q27)</f>
-        <v>JsonObject:0825B6B7-9C64-4EE8-A992-0A914261D6AD</v>
+        <v>JsonObject:D3A31ED2-5743-47BC-A580-72FDB5020433</v>
       </c>
       <c r="S29" t="s">
         <v>39</v>
@@ -4600,11 +4614,11 @@
       </c>
       <c r="F1" t="str" cm="1">
         <f t="array" ref="F1">_xll.ExLibris.Json.CreateJsonObject(E3:F6, EXLIBRIS_CONFIGURATION)</f>
-        <v>JsonObject:008E0007-AECB-42C1-8068-149FAC93578D</v>
+        <v>JsonObject:BF1B6B6F-9EEE-4DC6-91F4-424E7E9A56F3</v>
       </c>
       <c r="K1" t="str">
         <f>EXLIBRIS_CONFIGURATION</f>
-        <v>ExLibris.Core.ExLibrisConfiguration:23598F7C-BC8C-460B-B094-6B7B1D5D478C</v>
+        <v>ExLibris.Core.ExLibrisConfiguration:6708C3D9-DE2D-47BE-9248-773006E26782</v>
       </c>
     </row>
     <row r="2" spans="2:25" x14ac:dyDescent="0.4">
@@ -4674,7 +4688,7 @@
       </c>
       <c r="F6" t="str" cm="1">
         <f t="array" ref="F6">_xll.ExLibris.Json.CreateJsonArray(E8:J14, EXLIBRIS_CONFIGURATION)</f>
-        <v>JsonObject:CA60A2AE-6AFA-4219-846F-D2F18716D018</v>
+        <v>JsonObject:5FC16F5F-D218-4EEF-9A28-7A9B1B612039</v>
       </c>
       <c r="L6" t="s">
         <v>68</v>
@@ -4925,7 +4939,7 @@
       </c>
       <c r="I19" t="str" cm="1">
         <f t="array" ref="I19">_xll.ExLibris.Json.GetJsonValue(F1,E6, EXLIBRIS_CONFIGURATION)</f>
-        <v>JsonObject:F4BE569E-7806-4DA7-A070-484C307ECDE3</v>
+        <v>JsonObject:7F17AEF2-D9B8-44C3-A108-FA6737E6A206</v>
       </c>
       <c r="P19" t="s">
         <v>14</v>
@@ -5647,7 +5661,7 @@
       </c>
       <c r="I28" t="str" cm="1">
         <f t="array" ref="I28">_xll.ExLibris.Json.GetJsonValue(I19,"[2]", EXLIBRIS_CONFIGURATION)</f>
-        <v>JsonObject:F5491BB0-47BB-4609-B55B-B44DFFC9B9EC</v>
+        <v>JsonObject:DA126573-71F3-4949-B529-2FCCDED3A4C0</v>
       </c>
       <c r="P28" t="s">
         <v>38</v>
@@ -5904,7 +5918,7 @@
       </c>
       <c r="I32" t="str" cm="1">
         <f t="array" ref="I32">_xll.ExLibris.Json.GetJsonValue(F1,E6,EXLIBRIS_CONFIGURATION)</f>
-        <v>JsonObject:F4BE569E-7806-4DA7-A070-484C307ECDE3</v>
+        <v>JsonObject:7F17AEF2-D9B8-44C3-A108-FA6737E6A206</v>
       </c>
       <c r="P32" t="s">
         <v>42</v>
@@ -5941,7 +5955,7 @@
       </c>
       <c r="I33" t="str" cm="1">
         <f t="array" ref="I33">_xll.ExLibris.Json.SeachJsonArrayElements(I32,I8,I11,EXLIBRIS_CONFIGURATION)</f>
-        <v>JsonObject:D262EE96-6677-4E9A-A2A2-262853EC37BD</v>
+        <v>JsonObject:2F58EA90-CBB0-43E2-89BE-AD985FEEAE8C</v>
       </c>
       <c r="P33" t="s">
         <v>43</v>
@@ -6291,7 +6305,7 @@
       </c>
       <c r="I38" t="str" cm="1">
         <f t="array" ref="I38">_xll.ExLibris.Json.SeachJsonArrayElements(I32,J8,J11,EXLIBRIS_CONFIGURATION)</f>
-        <v>JsonObject:4CB3FEA9-E981-4454-9AD1-627AF904785E</v>
+        <v>JsonObject:520EC172-D3BC-49D2-AD96-04ADF51E0CE1</v>
       </c>
       <c r="P38" t="s">
         <v>48</v>
@@ -6548,7 +6562,7 @@
       </c>
       <c r="I42" t="str" cm="1">
         <f t="array" ref="I42">_xll.ExLibris.Json.SeachJsonArrayElements(I32,J8,,EXLIBRIS_CONFIGURATION)</f>
-        <v>JsonObject:6AF0E31F-7F9D-4D16-9302-6AF3FF5BAD64</v>
+        <v>JsonObject:FD2CC247-CD79-4796-8F03-426C6562740F</v>
       </c>
       <c r="P42" t="s">
         <v>52</v>
@@ -7087,7 +7101,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{92C31E65-5244-494C-A4E6-E2042CA25001}">
-  <dimension ref="B2:F15"/>
+  <dimension ref="B2:H26"/>
   <sheetFormatPr defaultRowHeight="18.75" x14ac:dyDescent="0.4"/>
   <cols>
     <col min="1" max="1" width="3.5" customWidth="1"/>
@@ -7096,16 +7110,16 @@
     <col min="5" max="5" width="39.625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="2:6" x14ac:dyDescent="0.4">
+    <row r="2" spans="2:8" x14ac:dyDescent="0.4">
       <c r="B2" t="s">
         <v>84</v>
       </c>
       <c r="C2" t="str" cm="1">
         <f t="array" ref="C2">_xll.ExLibris.LoadConfiguration(B6:C15)</f>
-        <v>ExLibris.Core.ExLibrisConfiguration:23598F7C-BC8C-460B-B094-6B7B1D5D478C</v>
-      </c>
-    </row>
-    <row r="4" spans="2:6" s="4" customFormat="1" ht="18" x14ac:dyDescent="0.4">
+        <v>ExLibris.Core.ExLibrisConfiguration:6708C3D9-DE2D-47BE-9248-773006E26782</v>
+      </c>
+    </row>
+    <row r="4" spans="2:8" s="4" customFormat="1" ht="18" x14ac:dyDescent="0.4">
       <c r="B4" s="4" t="s">
         <v>86</v>
       </c>
@@ -7113,7 +7127,7 @@
         <v>85</v>
       </c>
     </row>
-    <row r="6" spans="2:6" x14ac:dyDescent="0.4">
+    <row r="6" spans="2:8" x14ac:dyDescent="0.4">
       <c r="B6" t="s">
         <v>76</v>
       </c>
@@ -7121,14 +7135,18 @@
         <v>77</v>
       </c>
       <c r="E6" t="str" cm="1">
-        <f t="array" ref="E6:F15">_xll.DumpObject(EXLIBRIS_CONFIGURATION)</f>
+        <f t="array" ref="E6:F15">_xll.ExLibris.DumpObject(EXLIBRIS_CONFIGURATION)</f>
         <v>excel_value.excel_error_to</v>
       </c>
       <c r="F6" t="str">
         <v>Error</v>
       </c>
-    </row>
-    <row r="7" spans="2:6" x14ac:dyDescent="0.4">
+      <c r="H6" t="str" cm="1">
+        <f t="array" ref="H6:H26">_xll.ExLibris.ObserveRegisteredObjects()</f>
+        <v>JsonObject:4E615853-43E8-41FC-83FD-467E8A931C27</v>
+      </c>
+    </row>
+    <row r="7" spans="2:8" x14ac:dyDescent="0.4">
       <c r="B7" t="s">
         <v>78</v>
       </c>
@@ -7141,8 +7159,11 @@
       <c r="F7" t="str">
         <v>Null</v>
       </c>
-    </row>
-    <row r="8" spans="2:6" x14ac:dyDescent="0.4">
+      <c r="H7" t="str">
+        <v>JsonObject:3D0ED9D9-1E8A-4EEB-BA45-D0DBE00F1401</v>
+      </c>
+    </row>
+    <row r="8" spans="2:8" x14ac:dyDescent="0.4">
       <c r="B8" t="s">
         <v>80</v>
       </c>
@@ -7155,8 +7176,11 @@
       <c r="F8" t="str">
         <v>Null</v>
       </c>
-    </row>
-    <row r="9" spans="2:6" x14ac:dyDescent="0.4">
+      <c r="H8" t="str">
+        <v>JsonObject:468191F2-CEAB-4D55-9615-D6D8FC66E157</v>
+      </c>
+    </row>
+    <row r="9" spans="2:8" x14ac:dyDescent="0.4">
       <c r="B9" t="s">
         <v>81</v>
       </c>
@@ -7169,8 +7193,11 @@
       <c r="F9" t="str">
         <v>Null</v>
       </c>
-    </row>
-    <row r="10" spans="2:6" x14ac:dyDescent="0.4">
+      <c r="H9" t="str">
+        <v>JsonObject:BD189982-E6DC-45DB-847E-1B555AAB0E0E</v>
+      </c>
+    </row>
+    <row r="10" spans="2:8" x14ac:dyDescent="0.4">
       <c r="B10" t="s">
         <v>82</v>
       </c>
@@ -7183,8 +7210,11 @@
       <c r="F10" t="str">
         <v>StringEmpty</v>
       </c>
-    </row>
-    <row r="11" spans="2:6" x14ac:dyDescent="0.4">
+      <c r="H10" t="str">
+        <v>JsonObject:7F17AEF2-D9B8-44C3-A108-FA6737E6A206</v>
+      </c>
+    </row>
+    <row r="11" spans="2:8" x14ac:dyDescent="0.4">
       <c r="B11" t="s">
         <v>83</v>
       </c>
@@ -7197,8 +7227,11 @@
       <c r="F11" t="str">
         <v>StringEmpty</v>
       </c>
-    </row>
-    <row r="12" spans="2:6" x14ac:dyDescent="0.4">
+      <c r="H11" t="str">
+        <v>JsonObject:7798C1E6-BB2E-45F5-A0D0-276268D6B6BA</v>
+      </c>
+    </row>
+    <row r="12" spans="2:8" x14ac:dyDescent="0.4">
       <c r="B12" t="s">
         <v>88</v>
       </c>
@@ -7211,8 +7244,11 @@
       <c r="F12" t="str">
         <v>yyyy-MM-dd</v>
       </c>
-    </row>
-    <row r="13" spans="2:6" x14ac:dyDescent="0.4">
+      <c r="H12" t="str">
+        <v>JsonObject:D3A31ED2-5743-47BC-A580-72FDB5020433</v>
+      </c>
+    </row>
+    <row r="13" spans="2:8" x14ac:dyDescent="0.4">
       <c r="B13" t="s">
         <v>90</v>
       </c>
@@ -7225,8 +7261,11 @@
       <c r="F13" t="str">
         <v>payment _date</v>
       </c>
-    </row>
-    <row r="14" spans="2:6" x14ac:dyDescent="0.4">
+      <c r="H13" t="str">
+        <v>JsonObject:DA744F30-C5A8-4DB8-8CD0-9A3A26BA7A41</v>
+      </c>
+    </row>
+    <row r="14" spans="2:8" x14ac:dyDescent="0.4">
       <c r="B14" t="s">
         <v>91</v>
       </c>
@@ -7239,8 +7278,11 @@
       <c r="F14" t="str">
         <v>start_date</v>
       </c>
-    </row>
-    <row r="15" spans="2:6" x14ac:dyDescent="0.4">
+      <c r="H14" t="str">
+        <v>JsonObject:06B3FFA1-06C3-451D-9A1E-52B904CFCBEE</v>
+      </c>
+    </row>
+    <row r="15" spans="2:8" x14ac:dyDescent="0.4">
       <c r="B15" t="s">
         <v>92</v>
       </c>
@@ -7252,6 +7294,64 @@
       </c>
       <c r="F15" t="str">
         <v>end_date</v>
+      </c>
+      <c r="H15" t="str">
+        <v>JsonObject:2F58EA90-CBB0-43E2-89BE-AD985FEEAE8C</v>
+      </c>
+    </row>
+    <row r="16" spans="2:8" x14ac:dyDescent="0.4">
+      <c r="H16" t="str">
+        <v>JsonObject:DA126573-71F3-4949-B529-2FCCDED3A4C0</v>
+      </c>
+    </row>
+    <row r="17" spans="8:8" x14ac:dyDescent="0.4">
+      <c r="H17" t="str">
+        <v>JsonObject:FD2CC247-CD79-4796-8F03-426C6562740F</v>
+      </c>
+    </row>
+    <row r="18" spans="8:8" x14ac:dyDescent="0.4">
+      <c r="H18" t="str">
+        <v>JsonObject:2E68A39D-A156-4D80-9D04-AF626B72E3DA</v>
+      </c>
+    </row>
+    <row r="19" spans="8:8" x14ac:dyDescent="0.4">
+      <c r="H19" t="str">
+        <v>ExLibris.Core.WebSockets.WebsocketClient:01F5B277-9E73-4634-9E37-43F25E0BF6AF</v>
+      </c>
+    </row>
+    <row r="20" spans="8:8" x14ac:dyDescent="0.4">
+      <c r="H20" t="str">
+        <v>JsonObject:5FC16F5F-D218-4EEF-9A28-7A9B1B612039</v>
+      </c>
+    </row>
+    <row r="21" spans="8:8" x14ac:dyDescent="0.4">
+      <c r="H21" t="str">
+        <v>JsonObject:520EC172-D3BC-49D2-AD96-04ADF51E0CE1</v>
+      </c>
+    </row>
+    <row r="22" spans="8:8" x14ac:dyDescent="0.4">
+      <c r="H22" t="str">
+        <v>JsonObject:BF1B6B6F-9EEE-4DC6-91F4-424E7E9A56F3</v>
+      </c>
+    </row>
+    <row r="23" spans="8:8" x14ac:dyDescent="0.4">
+      <c r="H23" t="str">
+        <v>ExLibris.Core.ExLibrisConfiguration:6708C3D9-DE2D-47BE-9248-773006E26782</v>
+      </c>
+    </row>
+    <row r="24" spans="8:8" x14ac:dyDescent="0.4">
+      <c r="H24" t="str">
+        <v>JsonObject:094034A9-8F2E-4DB9-BBA4-B1B6A2AEA0DB</v>
+      </c>
+    </row>
+    <row r="25" spans="8:8" x14ac:dyDescent="0.4">
+      <c r="H25" t="str">
+        <v>JsonObject:DD53F82E-862B-4076-A9BD-4C94E106716B</v>
+      </c>
+    </row>
+    <row r="26" spans="8:8" x14ac:dyDescent="0.4">
+      <c r="H26" t="str">
+        <v>ExLibris.Core.WebSockets.WebsocketClient:387BB5DF-1F1C-489B-B0E3-E5546217F5ED</v>
       </c>
     </row>
   </sheetData>
@@ -7283,7 +7383,7 @@
       </c>
       <c r="E4" t="str" cm="1">
         <f t="array" ref="E4">_xll.ExLibris.WebSockets.OpenWebSocket("ws://localhost:10101",,D4)</f>
-        <v>ExLibris.Core.WebSockets.WebsocketClient:5A633BFF-4691-4566-A934-9DDD80FC2D74</v>
+        <v>ExLibris.Core.WebSockets.WebsocketClient:387BB5DF-1F1C-489B-B0E3-E5546217F5ED</v>
       </c>
     </row>
     <row r="6" spans="2:5" x14ac:dyDescent="0.4">
@@ -7292,7 +7392,7 @@
       </c>
       <c r="E6" t="str" cm="1">
         <f t="array" ref="E6">_xll.ExLibris.WebSockets.ObserveWebSocketStatus(E4,1000)</f>
-        <v>Closed</v>
+        <v>Connecting</v>
       </c>
     </row>
     <row r="7" spans="2:5" x14ac:dyDescent="0.4">
@@ -7373,7 +7473,7 @@
       </c>
       <c r="E17" t="str" cm="1">
         <f t="array" ref="E17">_xll.ExLibris.WebSockets.OpenWebSocket("ws://localhost:10101",,D17)</f>
-        <v>ExLibris.Core.WebSockets.WebsocketClient:6F42C26C-72F1-4ED5-B8A4-01C93DB2F850</v>
+        <v>ExLibris.Core.WebSockets.WebsocketClient:01F5B277-9E73-4634-9E37-43F25E0BF6AF</v>
       </c>
     </row>
     <row r="19" spans="4:5" x14ac:dyDescent="0.4">
@@ -7391,7 +7491,7 @@
       </c>
       <c r="E20" t="str" cm="1">
         <f t="array" ref="E20">_xll.ExLibris.WebSockets.ObserveWebSocketMessage(E17)</f>
-        <v>push_event 23:13:14</v>
+        <v>push_event 23:39:46</v>
       </c>
     </row>
     <row r="22" spans="4:5" x14ac:dyDescent="0.4">
@@ -7400,7 +7500,7 @@
       </c>
       <c r="E22" t="str" cm="1">
         <f t="array" ref="E22">_xll.ExLibris.WebSockets.SendWebSocketMessage(E17,"test "&amp;D22,E19="Open")</f>
-        <v>message sent : 2021-09-21T11:08:38.139</v>
+        <v>message sent : 2021-09-21T11:37:55.121</v>
       </c>
     </row>
     <row r="23" spans="4:5" x14ac:dyDescent="0.4">
@@ -7409,7 +7509,7 @@
       </c>
       <c r="E23" t="str" cm="1">
         <f t="array" ref="E23">_xll.ExLibris.WebSockets.SendWebSocketMessage($E$4,"test next "&amp;D23,E22)</f>
-        <v>message sent : 2021-09-21T11:08:38.157</v>
+        <v>message sent : 2021-09-21T11:37:55.138</v>
       </c>
     </row>
     <row r="24" spans="4:5" x14ac:dyDescent="0.4">
@@ -7418,7 +7518,7 @@
       </c>
       <c r="E24" t="str" cm="1">
         <f t="array" ref="E24">_xll.ExLibris.WebSockets.SendWebSocketMessage($E$4,"test next "&amp;D24,E23)</f>
-        <v>message sent : 2021-09-21T11:08:38.188</v>
+        <v>message sent : 2021-09-21T11:37:55.154</v>
       </c>
     </row>
     <row r="25" spans="4:5" x14ac:dyDescent="0.4">
@@ -7427,7 +7527,7 @@
       </c>
       <c r="E25" t="str" cm="1">
         <f t="array" ref="E25">_xll.ExLibris.WebSockets.SendWebSocketMessage($E$4,"test next "&amp;D25,E24)</f>
-        <v>message sent : 2021-09-21T11:08:38.208</v>
+        <v>message sent : 2021-09-21T11:37:55.169</v>
       </c>
     </row>
     <row r="26" spans="4:5" x14ac:dyDescent="0.4">
@@ -7436,7 +7536,7 @@
       </c>
       <c r="E26" t="str" cm="1">
         <f t="array" ref="E26">_xll.ExLibris.WebSockets.SendWebSocketMessage($E$4,"test next "&amp;D26,E25)</f>
-        <v>message sent : 2021-09-21T11:08:38.217</v>
+        <v>message sent : 2021-09-21T11:37:55.182</v>
       </c>
     </row>
     <row r="27" spans="4:5" x14ac:dyDescent="0.4">
@@ -7445,7 +7545,7 @@
       </c>
       <c r="E27" t="str" cm="1">
         <f t="array" ref="E27">_xll.ExLibris.WebSockets.SendWebSocketMessage($E$4,"test next "&amp;D27,E26)</f>
-        <v>message sent : 2021-09-21T11:08:38.238</v>
+        <v>message sent : 2021-09-21T11:37:55.198</v>
       </c>
     </row>
     <row r="28" spans="4:5" x14ac:dyDescent="0.4">
@@ -7454,7 +7554,7 @@
       </c>
       <c r="E28" t="str" cm="1">
         <f t="array" ref="E28">_xll.ExLibris.WebSockets.SendWebSocketMessage($E$4,"test next "&amp;D28,E27)</f>
-        <v>message sent : 2021-09-21T11:08:38.276</v>
+        <v>message sent : 2021-09-21T11:37:55.234</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
refactoring : webapi GET
</commit_message>
<xml_diff>
--- a/ExLibris/test_excel/exlibris_test.xlsx
+++ b/ExLibris/test_excel/exlibris_test.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\mugen\git\ex-libris\ExLibris\test_excel\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BC78540B-8D62-4125-989F-DFA06D02F6F5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{09D918CE-A7AD-4DBE-B942-98CF6D7FE251}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" activeTab="4" xr2:uid="{705CD0B7-27A9-4291-85BD-6034C0FEE3E4}"/>
   </bookViews>
@@ -660,799 +660,791 @@
 <file path=xl/volatileDependencies.xml><?xml version="1.0" encoding="utf-8"?>
 <volTypes xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <volType type="realTimeData">
-    <main first="rtdsrv.d1787fac4db647738cc71ff32b237324">
-      <tp>
-        <v>1</v>
-        <stp/>
-        <stp>caa7bd7e-f827-44b0-a781-5b3c066c55ff</stp>
-        <tr r="G29" s="4"/>
+    <main first="rtdsrv.fec3502cf85349c38b0a9636c87dce5f">
+      <tp>
+        <v>1</v>
+        <stp/>
+        <stp>41d37bd5-da93-4034-9b17-8a1cb81e9999</stp>
+        <tr r="G49" s="1"/>
+      </tp>
+      <tp>
+        <v>1</v>
+        <stp/>
+        <stp>c1c81a94-1d0c-402e-9a72-118505064ebe</stp>
+        <tr r="G32" s="4"/>
       </tp>
     </main>
-    <main first="rtdsrv.d1787fac4db647738cc71ff32b237324">
-      <tp>
-        <v>1</v>
-        <stp/>
-        <stp>bacdec7f-c0e6-420a-884a-e9e1ac473ecd</stp>
-        <tr r="I28" s="4"/>
-      </tp>
-      <tp>
-        <v>2</v>
-        <stp/>
-        <stp>b8b471e6-5f6b-4e06-90a8-f773bcab5453</stp>
-        <tr r="E6" s="3"/>
-      </tp>
-      <tp>
-        <v>1</v>
-        <stp/>
-        <stp>4e2c944d-3621-488b-a882-cb108cc0a239</stp>
-        <tr r="G32" s="4"/>
-      </tp>
-      <tp>
-        <v>1</v>
-        <stp/>
-        <stp>0178fa67-8dbf-4a7b-8a1e-891d583f51cf</stp>
-        <tr r="G34" s="4"/>
-      </tp>
-      <tp>
-        <v>1</v>
-        <stp/>
-        <stp>2f6c2586-7143-424c-af0a-fad44924bdd9</stp>
-        <tr r="G41" s="4"/>
+    <main first="rtdsrv.fec3502cf85349c38b0a9636c87dce5f">
+      <tp>
+        <v>1</v>
+        <stp/>
+        <stp>6e5ee5dc-9dd0-4717-b348-8de188135e40</stp>
+        <tr r="G55" s="4"/>
       </tp>
     </main>
-    <main first="rtdsrv.d1787fac4db647738cc71ff32b237324">
-      <tp>
-        <v>1</v>
-        <stp/>
-        <stp>a09a100c-b691-4212-b36c-f88c43e60e55</stp>
-        <tr r="G53" s="4"/>
+    <main first="rtdsrv.fec3502cf85349c38b0a9636c87dce5f">
+      <tp>
+        <v>1</v>
+        <stp/>
+        <stp>25d87983-8abc-42fb-a075-5f6fcda0f07f</stp>
+        <tr r="F6" s="4"/>
+      </tp>
+      <tp>
+        <v>1</v>
+        <stp/>
+        <stp>1f3c2185-6dc6-4ece-a427-eab3c23106ba</stp>
+        <tr r="G38" s="4"/>
       </tp>
     </main>
-    <main first="rtdsrv.d1787fac4db647738cc71ff32b237324">
-      <tp>
-        <v>1</v>
-        <stp/>
-        <stp>39315191-2204-4ab1-97d5-95e93b830096</stp>
-        <tr r="G38" s="1"/>
-      </tp>
-      <tp>
-        <v>1</v>
-        <stp/>
-        <stp>49ae780b-df4a-46f9-bffa-a03aaaf10b1d</stp>
-        <tr r="G35" s="1"/>
+    <main first="rtdsrv.fec3502cf85349c38b0a9636c87dce5f">
+      <tp>
+        <v>1</v>
+        <stp/>
+        <stp>f07f42be-2bec-44ea-a97a-255795c925b3</stp>
+        <tr r="G45" s="1"/>
+      </tp>
+      <tp>
+        <v>1</v>
+        <stp/>
+        <stp>cdef52d2-03c0-4254-9337-95f136fcb181</stp>
+        <tr r="G22" s="1"/>
       </tp>
     </main>
-    <main first="rtdsrv.d1787fac4db647738cc71ff32b237324">
-      <tp>
-        <v>1</v>
-        <stp/>
-        <stp>bc984b94-eee1-4519-a96e-25eff55a2bcf</stp>
-        <tr r="G37" s="4"/>
+    <main first="rtdsrv.fec3502cf85349c38b0a9636c87dce5f">
+      <tp>
+        <v>1</v>
+        <stp/>
+        <stp>df963bfc-b4c5-40f6-a26b-3f604f264526</stp>
+        <tr r="G52" s="1"/>
       </tp>
     </main>
-    <main first="rtdsrv.d1787fac4db647738cc71ff32b237324">
-      <tp>
-        <v>1</v>
-        <stp/>
-        <stp>f0c4cc0b-0c22-420a-af1b-480dd2c7f09b</stp>
+    <main first="rtdsrv.fec3502cf85349c38b0a9636c87dce5f">
+      <tp>
+        <v>1</v>
+        <stp/>
+        <stp>df549754-6680-4a5d-9407-a4244e8d1159</stp>
+        <tr r="G27" s="1"/>
+      </tp>
+    </main>
+    <main first="rtdsrv.fec3502cf85349c38b0a9636c87dce5f">
+      <tp>
+        <v>1</v>
+        <stp/>
+        <stp>7686c814-9b05-4399-9d64-3bfc728119e6</stp>
+        <tr r="G47" s="4"/>
+      </tp>
+    </main>
+    <main first="rtdsrv.fec3502cf85349c38b0a9636c87dce5f">
+      <tp>
+        <v>1</v>
+        <stp/>
+        <stp>f7cdaf6c-1f42-4f3d-bf27-bed8a160a3e7</stp>
+        <tr r="G54" s="4"/>
+      </tp>
+      <tp>
+        <v>1</v>
+        <stp/>
+        <stp>fe04cf25-f2f9-4097-a2ff-376d70a62b30</stp>
         <tr r="G46" s="4"/>
       </tp>
+      <tp>
+        <v>1</v>
+        <stp/>
+        <stp>3efdff68-009e-4e93-9a13-5713ca3796cd</stp>
+        <tr r="I38" s="4"/>
+      </tp>
     </main>
-    <main first="rtdsrv.d1787fac4db647738cc71ff32b237324">
-      <tp>
-        <v>1</v>
-        <stp/>
-        <stp>2f438f7d-8958-4729-8797-243153f6a692</stp>
-        <tr r="G51" s="4"/>
-      </tp>
-      <tp>
-        <v>1</v>
-        <stp/>
-        <stp>074b24bf-4522-4af6-8fdf-8764cc0e68fb</stp>
-        <tr r="G44" s="1"/>
-      </tp>
-      <tp>
-        <v>1</v>
-        <stp/>
-        <stp>248bb63e-82d2-4f23-9de6-916d3d6280f3</stp>
-        <tr r="G19" s="1"/>
-      </tp>
-      <tp>
-        <v>1</v>
-        <stp/>
-        <stp>b7450be8-e5c3-4a5a-81cb-1d880960bff9</stp>
-        <tr r="D15" s="5"/>
-      </tp>
-      <tp>
-        <v>1</v>
-        <stp/>
-        <stp>88cc5982-f9e0-4a89-844f-8d7eec22ec29</stp>
-        <tr r="G21" s="1"/>
-      </tp>
-      <tp>
-        <v>1</v>
-        <stp/>
-        <stp>a194e105-62ee-4109-9d63-fc1751cd9eee</stp>
-        <tr r="G49" s="1"/>
-      </tp>
-    </main>
-    <main first="rtdsrv.d1787fac4db647738cc71ff32b237324">
-      <tp>
-        <v>1</v>
-        <stp/>
-        <stp>24d669c0-9031-4849-8a0a-2f9eba732439</stp>
-        <tr r="G48" s="1"/>
-      </tp>
-    </main>
-    <main first="rtdsrv.d1787fac4db647738cc71ff32b237324">
-      <tp>
-        <v>1</v>
-        <stp/>
-        <stp>afc1f8fe-31ef-47ea-93ce-a6b717c87af7</stp>
+    <main first="rtdsrv.fec3502cf85349c38b0a9636c87dce5f">
+      <tp>
+        <v>1</v>
+        <stp/>
+        <stp>c05e99df-b6ab-45e3-8c6d-71d3202a0902</stp>
         <tr r="I19" s="4"/>
         <tr r="I32" s="4"/>
       </tp>
+    </main>
+    <main first="rtdsrv.fec3502cf85349c38b0a9636c87dce5f">
+      <tp>
+        <v>1</v>
+        <stp/>
+        <stp>0b560688-ea4c-4ea3-805e-3596e0560d9f</stp>
+        <tr r="G50" s="1"/>
+      </tp>
+      <tp>
+        <v>1</v>
+        <stp/>
+        <stp>6a22f092-3c96-4c57-ac5e-d2ae2f665baf</stp>
+        <tr r="G20" s="4"/>
+      </tp>
+    </main>
+    <main first="rtdsrv.fec3502cf85349c38b0a9636c87dce5f">
+      <tp>
+        <v>1</v>
+        <stp/>
+        <stp>5ca38746-802e-4fcf-89d3-f57de854c5cb</stp>
+        <tr r="G29" s="1"/>
+      </tp>
+    </main>
+    <main first="rtdsrv.fec3502cf85349c38b0a9636c87dce5f">
+      <tp>
+        <v>1</v>
+        <stp/>
+        <stp>bd502f1f-cbbb-4523-bffa-62225d9f16dc</stp>
+        <tr r="G45" s="4"/>
+      </tp>
+    </main>
+    <main first="rtdsrv.fec3502cf85349c38b0a9636c87dce5f">
+      <tp>
+        <v>1</v>
+        <stp/>
+        <stp>c318d0ef-8e21-482f-9079-de70d9c97be0</stp>
+        <tr r="G31" s="4"/>
+      </tp>
+    </main>
+    <main first="rtdsrv.fec3502cf85349c38b0a9636c87dce5f">
+      <tp>
+        <v>1</v>
+        <stp/>
+        <stp>8d322247-b76a-4d4a-afc9-aa6f76b3d427</stp>
+        <tr r="P19" s="1"/>
+      </tp>
+    </main>
+    <main first="rtdsrv.fec3502cf85349c38b0a9636c87dce5f">
+      <tp>
+        <v>3</v>
+        <stp/>
+        <stp>f57b3145-43df-48eb-b5f8-32a09235fa2d</stp>
+        <tr r="E6" s="3"/>
+      </tp>
+      <tp>
+        <v>1</v>
+        <stp/>
+        <stp>3d2c34ce-7fe8-4afa-8170-863f47147ec5</stp>
+        <tr r="G32" s="1"/>
+      </tp>
+    </main>
+    <main first="rtdsrv.fec3502cf85349c38b0a9636c87dce5f">
+      <tp>
+        <v>1</v>
+        <stp/>
+        <stp>3961e80a-b6ad-46e0-9a47-ac2b3a720083</stp>
+        <tr r="G34" s="4"/>
+      </tp>
+    </main>
+    <main first="rtdsrv.fec3502cf85349c38b0a9636c87dce5f">
+      <tp>
+        <v>1</v>
+        <stp/>
+        <stp>d011d82a-8fb8-4b67-95dd-61dbd5a0122e</stp>
+        <tr r="G57" s="1"/>
+      </tp>
+      <tp>
+        <v>1</v>
+        <stp/>
+        <stp>36594df7-e5f8-4773-b74f-6af48ea81a65</stp>
+        <tr r="G24" s="4"/>
+      </tp>
+    </main>
+    <main first="rtdsrv.fec3502cf85349c38b0a9636c87dce5f">
+      <tp>
+        <v>1</v>
+        <stp/>
+        <stp>6e691c8f-859c-4e1c-9ce3-fffa863ad250</stp>
+        <tr r="G36" s="4"/>
+      </tp>
+      <tp>
+        <v>1</v>
+        <stp/>
+        <stp>0ad5b270-8e7d-40ae-947a-24ddcdb3b37e</stp>
+        <tr r="G21" s="4"/>
+      </tp>
+      <tp>
+        <v>1</v>
+        <stp/>
+        <stp>af00cae3-7ae0-4d4b-868f-fcdab0124cf9</stp>
+        <tr r="G42" s="4"/>
+      </tp>
+    </main>
+    <main first="rtdsrv.fec3502cf85349c38b0a9636c87dce5f">
+      <tp>
+        <v>1</v>
+        <stp/>
+        <stp>2155bb00-9eca-4c3b-adfe-766badf7efbf</stp>
+        <tr r="G19" s="1"/>
+      </tp>
+      <tp>
+        <v>1</v>
+        <stp/>
+        <stp>12f51600-8f94-4a27-ab01-802fb532fd30</stp>
+        <tr r="G29" s="4"/>
+      </tp>
+    </main>
+    <main first="rtdsrv.fec3502cf85349c38b0a9636c87dce5f">
+      <tp>
+        <v>1</v>
+        <stp/>
+        <stp>b7993e25-d405-437e-b995-ed1ad3d87f13</stp>
+        <tr r="F1" s="1"/>
+      </tp>
+      <tp>
+        <v>1</v>
+        <stp/>
+        <stp>6f595ac6-6aec-472d-aa65-462c0814f6dd</stp>
+        <tr r="G40" s="4"/>
+      </tp>
+      <tp>
+        <v>1</v>
+        <stp/>
+        <stp>79014e27-9281-4701-b2b9-3cdf984c468b</stp>
+        <tr r="E7" s="3"/>
+      </tp>
+    </main>
+    <main first="rtdsrv.fec3502cf85349c38b0a9636c87dce5f">
+      <tp>
+        <v>1</v>
+        <stp/>
+        <stp>ac903392-5fec-4aeb-b7ba-2f6709773a92</stp>
+        <tr r="G51" s="1"/>
+      </tp>
+      <tp>
+        <v>1</v>
+        <stp/>
+        <stp>9e066c9e-9519-468d-94eb-cf2c514c42c4</stp>
+        <tr r="G57" s="4"/>
+      </tp>
+    </main>
+    <main first="rtdsrv.fec3502cf85349c38b0a9636c87dce5f">
+      <tp>
+        <v>1</v>
+        <stp/>
+        <stp>4cdc7e09-6580-4c54-99fb-e823aad3ac96</stp>
+        <tr r="G41" s="4"/>
+      </tp>
+      <tp>
+        <v>1</v>
+        <stp/>
+        <stp>17d656fd-dcab-4f4e-8ecd-5a90bb42b8df</stp>
+        <tr r="G43" s="1"/>
+      </tp>
+    </main>
+    <main first="rtdsrv.fec3502cf85349c38b0a9636c87dce5f">
+      <tp>
+        <v>3</v>
+        <stp/>
+        <stp>aafa0d76-b534-42bb-9446-a8ddb4800e10</stp>
+        <tr r="E19" s="3"/>
+      </tp>
+    </main>
+    <main first="rtdsrv.fec3502cf85349c38b0a9636c87dce5f">
+      <tp>
+        <v>1</v>
+        <stp/>
+        <stp>a038f868-aa17-4423-9075-d7d850e962e4</stp>
+        <tr r="G23" s="4"/>
+      </tp>
+      <tp>
+        <v>1</v>
+        <stp/>
+        <stp>60a099c2-461d-4573-83f2-048bcf2abb96</stp>
+        <tr r="G27" s="4"/>
+      </tp>
+      <tp>
+        <v>1</v>
+        <stp/>
+        <stp>aafa770e-0be5-4204-909a-69a7394f632e</stp>
+        <tr r="F1" s="4"/>
+      </tp>
+    </main>
+    <main first="rtdsrv.fec3502cf85349c38b0a9636c87dce5f">
+      <tp>
+        <v>1</v>
+        <stp/>
+        <stp>2ae078fe-f70f-4bbd-aea5-fed1d40bd28f</stp>
+        <tr r="G40" s="1"/>
+      </tp>
+    </main>
+    <main first="rtdsrv.fec3502cf85349c38b0a9636c87dce5f">
+      <tp>
+        <v>1</v>
+        <stp/>
+        <stp>5cc015a7-5f49-4357-9791-cba5cec8b33f</stp>
+        <tr r="G44" s="1"/>
+      </tp>
+      <tp>
+        <v>1</v>
+        <stp/>
+        <stp>af58d94b-f369-498b-b153-76a3217ec078</stp>
+        <tr r="D50" s="5"/>
+      </tp>
+      <tp>
+        <v>1</v>
+        <stp/>
+        <stp>e9faecb7-34e9-40b6-a1db-acefc1f7e022</stp>
+        <tr r="G44" s="4"/>
+      </tp>
+      <tp>
+        <v>1</v>
+        <stp/>
+        <stp>6089cecb-c592-4dba-acf3-8d4715bcd927</stp>
+        <tr r="G24" s="1"/>
+      </tp>
+    </main>
+    <main first="rtdsrv.fec3502cf85349c38b0a9636c87dce5f">
+      <tp>
+        <v>1</v>
+        <stp/>
+        <stp>d9422ab3-329c-4380-822e-e5f150433337</stp>
+        <tr r="D7" s="5"/>
+      </tp>
+    </main>
+    <main first="rtdsrv.fec3502cf85349c38b0a9636c87dce5f">
+      <tp>
+        <v>1</v>
+        <stp/>
+        <stp>51b68aff-8bc7-439f-a1b7-8565e1cdf494</stp>
+        <tr r="G30" s="4"/>
+      </tp>
+    </main>
+    <main first="rtdsrv.fec3502cf85349c38b0a9636c87dce5f">
+      <tp>
+        <v>1</v>
+        <stp/>
+        <stp>6007b537-953e-4c48-838f-c11b02f83c71</stp>
+        <tr r="G26" s="4"/>
+      </tp>
+    </main>
+    <main first="rtdsrv.fec3502cf85349c38b0a9636c87dce5f">
+      <tp>
+        <v>1</v>
+        <stp/>
+        <stp>7444a875-7b1f-4cb1-bbe9-5542f604018b</stp>
+        <tr r="G48" s="4"/>
+      </tp>
+      <tp>
+        <v>1</v>
+        <stp/>
+        <stp>b5856513-1ffa-4575-a040-593b7191ce2d</stp>
+        <tr r="D15" s="5"/>
+      </tp>
+    </main>
+    <main first="rtdsrv.fec3502cf85349c38b0a9636c87dce5f">
+      <tp>
+        <v>1</v>
+        <stp/>
+        <stp>4123f829-c8e5-4646-aa5f-7330e15b36a3</stp>
+        <tr r="G36" s="1"/>
+      </tp>
+    </main>
+    <main first="rtdsrv.fec3502cf85349c38b0a9636c87dce5f">
+      <tp>
+        <v>1</v>
+        <stp/>
+        <stp>905651c1-d07d-4697-91be-f9b0202fadad</stp>
+        <tr r="D25" s="5"/>
+      </tp>
+      <tp>
+        <v>1</v>
+        <stp/>
+        <stp>a7763fce-5e70-42dd-bca1-c869fb9869ce</stp>
+        <tr r="G41" s="1"/>
+      </tp>
+      <tp>
+        <v>1</v>
+        <stp/>
+        <stp>cc97de46-ac94-41d5-976d-53f9bf20a360</stp>
+        <tr r="E17" s="3"/>
+      </tp>
+    </main>
+    <main first="rtdsrv.fec3502cf85349c38b0a9636c87dce5f">
+      <tp>
+        <v>1</v>
+        <stp/>
+        <stp>d3a23e72-47ef-48ec-97b0-84c6af6c83c6</stp>
+        <tr r="G46" s="1"/>
+      </tp>
+      <tp>
+        <v>1</v>
+        <stp/>
+        <stp>6f3ee88a-d720-4c2e-9552-b938d0871aee</stp>
+        <tr r="G28" s="1"/>
+      </tp>
+    </main>
+    <main first="rtdsrv.fec3502cf85349c38b0a9636c87dce5f">
+      <tp>
+        <v>1</v>
+        <stp/>
+        <stp>349317df-9dc9-452b-bcc1-893a1db20de2</stp>
+        <tr r="C23" s="5"/>
+      </tp>
+      <tp>
+        <v>1</v>
+        <stp/>
+        <stp>5e4dd906-30e3-4740-9bcc-95df69624207</stp>
+        <tr r="G47" s="1"/>
+      </tp>
+      <tp>
+        <v>1</v>
+        <stp/>
+        <stp>16a60fdc-5c95-4cc7-9de8-057034eea48c</stp>
+        <tr r="G37" s="1"/>
+      </tp>
+      <tp>
+        <v>1</v>
+        <stp/>
+        <stp>97e2d439-9c30-43d8-9be6-bf16ed5dafe3</stp>
+        <tr r="G43" s="4"/>
+      </tp>
+    </main>
+    <main first="rtdsrv.fec3502cf85349c38b0a9636c87dce5f">
+      <tp>
+        <v>1</v>
+        <stp/>
+        <stp>138032a9-f0e1-48f7-b6b9-4add3f12f644</stp>
+        <tr r="G30" s="1"/>
+      </tp>
+      <tp>
+        <v>1</v>
+        <stp/>
+        <stp>1163c23c-4c7e-4462-bb16-fef7d5bbed92</stp>
+        <tr r="E4" s="3"/>
+      </tp>
+      <tp>
+        <v>1</v>
+        <stp/>
+        <stp>4b6a515f-6f83-4e05-ace9-6f3a1b110174</stp>
+        <tr r="C13" s="5"/>
+      </tp>
+    </main>
+    <main first="rtdsrv.fec3502cf85349c38b0a9636c87dce5f">
+      <tp>
+        <v>1</v>
+        <stp/>
+        <stp>4637dc13-60df-4a9a-aded-a31fbceed781</stp>
+        <tr r="I28" s="1"/>
+      </tp>
+    </main>
+    <main first="rtdsrv.fec3502cf85349c38b0a9636c87dce5f">
+      <tp>
+        <v>1</v>
+        <stp/>
+        <stp>3954c03c-daae-494c-8c17-726fe50e599e</stp>
+        <tr r="G38" s="1"/>
+      </tp>
+    </main>
+    <main first="rtdsrv.fec3502cf85349c38b0a9636c87dce5f">
+      <tp>
+        <v>1</v>
+        <stp/>
+        <stp>454e9412-5346-47ef-abf8-565197ae130a</stp>
+        <tr r="G52" s="4"/>
+      </tp>
+      <tp>
+        <v>1</v>
+        <stp/>
+        <stp>68dc244b-60a3-4386-8394-b5e5d20534f3</stp>
+        <tr r="G23" s="1"/>
+      </tp>
+    </main>
+    <main first="rtdsrv.fec3502cf85349c38b0a9636c87dce5f">
+      <tp>
+        <v>1</v>
+        <stp/>
+        <stp>f238d34b-3ca4-4a64-98e7-a402c5303e3b</stp>
+        <tr r="G39" s="1"/>
+      </tp>
+      <tp>
+        <v>1</v>
+        <stp/>
+        <stp>d2e8ea0d-041c-4b47-801d-1c868db2cebc</stp>
+        <tr r="G34" s="1"/>
+      </tp>
+      <tp>
+        <v>1</v>
+        <stp/>
+        <stp>fec3ff6a-5ba7-41ca-9240-8b9e9f3edcb1</stp>
+        <tr r="C2" s="2"/>
+      </tp>
+    </main>
+    <main first="rtdsrv.fec3502cf85349c38b0a9636c87dce5f">
+      <tp>
+        <v>1</v>
+        <stp/>
+        <stp>1ade31fd-ca3a-47f4-8d05-dba8a2ec5c8d</stp>
+        <tr r="C5" s="5"/>
+      </tp>
+      <tp>
+        <v>1</v>
+        <stp/>
+        <stp>8d180003-bb94-4981-8e42-62ee56b4235a</stp>
+        <tr r="G51" s="4"/>
+      </tp>
+    </main>
+    <main first="rtdsrv.fec3502cf85349c38b0a9636c87dce5f">
+      <tp>
+        <v>1</v>
+        <stp/>
+        <stp>40e1d5d2-24cd-4b37-8c06-7ffe76edaeed</stp>
+        <tr r="N47" s="5"/>
+      </tp>
+    </main>
+    <main first="rtdsrv.fec3502cf85349c38b0a9636c87dce5f">
+      <tp>
+        <v>1</v>
+        <stp/>
+        <stp>8ac09a24-fb87-4c7c-a07b-696f8978e76f</stp>
+        <tr r="G33" s="4"/>
+      </tp>
       <tp>
         <v>2</v>
         <stp/>
-        <stp>598e351b-0511-4553-b2d3-13f2f41cfcfc</stp>
+        <stp>7a41143d-32f7-435f-9eff-d8776ce868a7</stp>
         <tr r="H6" s="2"/>
       </tp>
+      <tp>
+        <v>1</v>
+        <stp/>
+        <stp>2e6a7105-8bba-42b9-84cc-a6dbb2e5f7d2</stp>
+        <tr r="I42" s="4"/>
+      </tp>
     </main>
-    <main first="rtdsrv.d1787fac4db647738cc71ff32b237324">
-      <tp>
-        <v>1</v>
-        <stp/>
-        <stp>0c97422d-6cfd-41c1-bd55-68fb862f3bf3</stp>
-        <tr r="P19" s="1"/>
+    <main first="rtdsrv.fec3502cf85349c38b0a9636c87dce5f">
+      <tp>
+        <v>1</v>
+        <stp/>
+        <stp>14395c78-0b5e-45cc-a957-131e32fc6505</stp>
+        <tr r="G25" s="4"/>
+      </tp>
+      <tp>
+        <v>1</v>
+        <stp/>
+        <stp>558062cd-9e9a-40cb-9570-97b98513bc24</stp>
+        <tr r="G28" s="4"/>
+      </tp>
+      <tp>
+        <v>1</v>
+        <stp/>
+        <stp>e656fdf3-cc4a-4c28-853d-b36c77bd74e3</stp>
+        <tr r="G19" s="4"/>
       </tp>
     </main>
-    <main first="rtdsrv.d1787fac4db647738cc71ff32b237324">
-      <tp>
-        <v>1</v>
-        <stp/>
-        <stp>4ef1d119-33d1-4f0b-bbdd-4980f2044f06</stp>
+    <main first="rtdsrv.fec3502cf85349c38b0a9636c87dce5f">
+      <tp>
+        <v>1</v>
+        <stp/>
+        <stp>f5672198-62a1-458d-a933-48a512633ef4</stp>
+        <tr r="I33" s="4"/>
+      </tp>
+    </main>
+    <main first="rtdsrv.fec3502cf85349c38b0a9636c87dce5f">
+      <tp>
+        <v>1</v>
+        <stp/>
+        <stp>ae8bdb0d-809a-4223-93cd-bf5bb6134415</stp>
+        <tr r="G35" s="4"/>
+      </tp>
+    </main>
+    <main first="rtdsrv.fec3502cf85349c38b0a9636c87dce5f">
+      <tp>
+        <v>1</v>
+        <stp/>
+        <stp>eb470802-e367-4cd5-b92a-c6015534701c</stp>
+        <tr r="I19" s="1"/>
+      </tp>
+      <tp>
+        <v>1</v>
+        <stp/>
+        <stp>2c786e63-556d-45d9-81f0-177401c82a4b</stp>
+        <tr r="G21" s="1"/>
+      </tp>
+    </main>
+    <main first="rtdsrv.fec3502cf85349c38b0a9636c87dce5f">
+      <tp>
+        <v>1</v>
+        <stp/>
+        <stp>c539fcad-c7b3-45c0-bc54-813613f449ee</stp>
+        <tr r="G48" s="1"/>
+      </tp>
+    </main>
+    <main first="rtdsrv.fec3502cf85349c38b0a9636c87dce5f">
+      <tp>
+        <v>1</v>
+        <stp/>
+        <stp>84395e62-0a8e-4850-9f82-6b006a28db8e</stp>
+        <tr r="C48" s="5"/>
+      </tp>
+      <tp>
+        <v>1</v>
+        <stp/>
+        <stp>767836ff-bcb0-46d4-b37f-e8d86fc18788</stp>
+        <tr r="G55" s="1"/>
+      </tp>
+      <tp>
+        <v>1</v>
+        <stp/>
+        <stp>e2609d9a-ae73-4236-9acb-dcc7b1c748b8</stp>
+        <tr r="D36" s="5"/>
+      </tp>
+    </main>
+    <main first="rtdsrv.fec3502cf85349c38b0a9636c87dce5f">
+      <tp>
+        <v>1</v>
+        <stp/>
+        <stp>30c8a90d-1380-4b65-854a-7fab7e95029b</stp>
+        <tr r="F6" s="1"/>
+      </tp>
+    </main>
+    <main first="rtdsrv.fec3502cf85349c38b0a9636c87dce5f">
+      <tp>
+        <v>1</v>
+        <stp/>
+        <stp>5210af78-0c8d-4c99-807b-8d5c3c8aee51</stp>
+        <tr r="G37" s="4"/>
+      </tp>
+    </main>
+    <main first="rtdsrv.fec3502cf85349c38b0a9636c87dce5f">
+      <tp>
+        <v>1</v>
+        <stp/>
+        <stp>9818e04b-bd86-47bf-936b-0d53662b0a88</stp>
+        <tr r="G20" s="1"/>
+      </tp>
+    </main>
+    <main first="rtdsrv.fec3502cf85349c38b0a9636c87dce5f">
+      <tp>
+        <v>1</v>
+        <stp/>
+        <stp>7c2bf98a-033b-4a45-8aee-62fccb5f2c76</stp>
+        <tr r="G26" s="1"/>
+      </tp>
+      <tp>
+        <v>1</v>
+        <stp/>
+        <stp>f731062d-ec50-440b-8f19-fce5dca60926</stp>
+        <tr r="G33" s="1"/>
+      </tp>
+    </main>
+    <main first="rtdsrv.fec3502cf85349c38b0a9636c87dce5f">
+      <tp>
+        <v>1</v>
+        <stp/>
+        <stp>fe415089-983b-444d-9911-bec3cf26d479</stp>
+        <tr r="G49" s="4"/>
+      </tp>
+      <tp>
+        <v>1</v>
+        <stp/>
+        <stp>e29b84d7-53bf-45e8-9ab9-46116dd2054f</stp>
+        <tr r="P29" s="1"/>
+      </tp>
+    </main>
+    <main first="rtdsrv.fec3502cf85349c38b0a9636c87dce5f">
+      <tp>
+        <v>1</v>
+        <stp/>
+        <stp>6d5f1f89-55bd-482d-b11e-c4b49ab6480f</stp>
+        <tr r="G39" s="4"/>
+      </tp>
+      <tp>
+        <v>1</v>
+        <stp/>
+        <stp>b200d3d9-4c82-45b9-a0b7-92ed87b39daf</stp>
+        <tr r="E20" s="3"/>
+      </tp>
+      <tp>
+        <v>1</v>
+        <stp/>
+        <stp>b131af93-c104-4245-879c-fb9e3e541024</stp>
+        <tr r="G25" s="1"/>
+      </tp>
+      <tp>
+        <v>1</v>
+        <stp/>
+        <stp>737afef3-585f-49e5-81fe-8577c264b814</stp>
+        <tr r="G22" s="4"/>
+      </tp>
+      <tp>
+        <v>1</v>
+        <stp/>
+        <stp>579dc3d5-cff8-42df-bcfb-a81e065dbfab</stp>
+        <tr r="G56" s="1"/>
+      </tp>
+    </main>
+    <main first="rtdsrv.fec3502cf85349c38b0a9636c87dce5f">
+      <tp>
+        <v>1</v>
+        <stp/>
+        <stp>674d49e4-a63f-451b-b85e-d410efecbeca</stp>
+        <tr r="G54" s="1"/>
+      </tp>
+    </main>
+    <main first="rtdsrv.fec3502cf85349c38b0a9636c87dce5f">
+      <tp>
+        <v>1</v>
+        <stp/>
+        <stp>221b33c6-aaa0-4d3f-af7f-28a2f0b926d9</stp>
+        <tr r="G53" s="4"/>
+      </tp>
+      <tp>
+        <v>1</v>
+        <stp/>
+        <stp>0c04faa2-04e7-4237-9fea-b4cf09672bc3</stp>
+        <tr r="G53" s="1"/>
+      </tp>
+    </main>
+    <main first="rtdsrv.fec3502cf85349c38b0a9636c87dce5f">
+      <tp>
+        <v>1</v>
+        <stp/>
+        <stp>2d4c38a1-b42e-4515-bdd9-4e44db3c3d10</stp>
+        <tr r="G50" s="4"/>
+      </tp>
+      <tp>
+        <v>1</v>
+        <stp/>
+        <stp>677609c3-5d6e-49ba-a9a4-175bd8176885</stp>
+        <tr r="G35" s="1"/>
+      </tp>
+    </main>
+    <main first="rtdsrv.fec3502cf85349c38b0a9636c87dce5f">
+      <tp>
+        <v>1</v>
+        <stp/>
+        <stp>e9b8c83b-21b1-439d-a6a1-f8a1dafbccd1</stp>
+        <tr r="C34" s="5"/>
+      </tp>
+      <tp>
+        <v>1</v>
+        <stp/>
+        <stp>24ace882-361d-4fac-bb7d-9a5b5e04cbff</stp>
         <tr r="G42" s="1"/>
       </tp>
     </main>
-    <main first="rtdsrv.d1787fac4db647738cc71ff32b237324">
-      <tp>
-        <v>1</v>
-        <stp/>
-        <stp>3011bca9-87db-4964-b79c-6c34d98550c4</stp>
-        <tr r="G29" s="1"/>
-      </tp>
-      <tp>
-        <v>1</v>
-        <stp/>
-        <stp>7ca5075b-7583-4be1-8207-cfd9c8bda1a0</stp>
-        <tr r="G33" s="4"/>
-      </tp>
-      <tp>
-        <v>1</v>
-        <stp/>
-        <stp>ede3a8a3-2cb5-407e-b7d4-b95b18dfdc31</stp>
-        <tr r="G42" s="4"/>
+    <main first="rtdsrv.fec3502cf85349c38b0a9636c87dce5f">
+      <tp>
+        <v>1</v>
+        <stp/>
+        <stp>2ebdbb89-8465-4edd-b47b-ff3740be3753</stp>
+        <tr r="G56" s="4"/>
+      </tp>
+      <tp>
+        <v>1</v>
+        <stp/>
+        <stp>6ecdd236-4e1c-48e4-8564-fd266915f1ef</stp>
+        <tr r="I28" s="4"/>
+      </tp>
+      <tp>
+        <v>1</v>
+        <stp/>
+        <stp>0b799bba-31f0-4a3e-ac53-ff694042586c</stp>
+        <tr r="G31" s="1"/>
       </tp>
     </main>
-    <main first="rtdsrv.d1787fac4db647738cc71ff32b237324">
-      <tp>
-        <v>1</v>
-        <stp/>
-        <stp>6d90f83c-0186-47ea-bc60-4dd6670a2eff</stp>
-        <tr r="C48" s="5"/>
-      </tp>
-      <tp>
-        <v>1</v>
-        <stp/>
-        <stp>a299abb1-9eb6-4331-b3ca-dd363be48071</stp>
-        <tr r="G55" s="1"/>
-      </tp>
-    </main>
-    <main first="rtdsrv.d1787fac4db647738cc71ff32b237324">
-      <tp>
-        <v>1</v>
-        <stp/>
-        <stp>bb8858a9-dce4-4547-90de-f48c72f45fb1</stp>
-        <tr r="G53" s="1"/>
-      </tp>
-    </main>
-    <main first="rtdsrv.d1787fac4db647738cc71ff32b237324">
-      <tp>
-        <v>1</v>
-        <stp/>
-        <stp>18ffae04-c5f1-43b0-8cf7-8f8761c262d7</stp>
-        <tr r="P29" s="1"/>
-      </tp>
-      <tp>
-        <v>1</v>
-        <stp/>
-        <stp>97cf1f5a-9e31-4726-a191-d8b168a7ae02</stp>
-        <tr r="E20" s="3"/>
-      </tp>
-    </main>
-    <main first="rtdsrv.d1787fac4db647738cc71ff32b237324">
-      <tp>
-        <v>1</v>
-        <stp/>
-        <stp>1b55c51c-1d63-44b2-91f5-8ccd226f5af2</stp>
-        <tr r="G40" s="1"/>
-      </tp>
-    </main>
-    <main first="rtdsrv.d1787fac4db647738cc71ff32b237324">
-      <tp>
-        <v>1</v>
-        <stp/>
-        <stp>aca3f687-a8bf-4ba2-9160-62944838086a</stp>
-        <tr r="G39" s="4"/>
-      </tp>
-      <tp>
-        <v>1</v>
-        <stp/>
-        <stp>59364c00-63d4-4c89-beaf-4df71cf180f5</stp>
-        <tr r="G26" s="4"/>
-      </tp>
-    </main>
-    <main first="rtdsrv.d1787fac4db647738cc71ff32b237324">
-      <tp>
-        <v>1</v>
-        <stp/>
-        <stp>f0ae5515-cea0-4915-9609-7d25210a450d</stp>
-        <tr r="G37" s="1"/>
-      </tp>
-      <tp>
-        <v>1</v>
-        <stp/>
-        <stp>4a3d8d02-28db-412f-a106-2c54cea44de2</stp>
-        <tr r="G49" s="4"/>
-      </tp>
-    </main>
-    <main first="rtdsrv.d1787fac4db647738cc71ff32b237324">
-      <tp>
-        <v>1</v>
-        <stp/>
-        <stp>6ec9afa5-d160-40b0-88b2-0f9d16861fc5</stp>
-        <tr r="G23" s="4"/>
-      </tp>
-    </main>
-    <main first="rtdsrv.d1787fac4db647738cc71ff32b237324">
-      <tp>
-        <v>1</v>
-        <stp/>
-        <stp>f193db98-ef88-495e-bb62-735c507e2e34</stp>
-        <tr r="G52" s="4"/>
-      </tp>
-      <tp>
-        <v>1</v>
-        <stp/>
-        <stp>8fa4f63c-ba99-4232-a48e-cca0ab55397f</stp>
-        <tr r="G25" s="4"/>
-      </tp>
-    </main>
-    <main first="rtdsrv.d1787fac4db647738cc71ff32b237324">
-      <tp>
-        <v>1</v>
-        <stp/>
-        <stp>81102e16-3a3b-4e8a-b4c7-c09cdc44e6ce</stp>
-        <tr r="G56" s="1"/>
-      </tp>
-    </main>
-    <main first="rtdsrv.d1787fac4db647738cc71ff32b237324">
-      <tp>
-        <v>1</v>
-        <stp/>
-        <stp>e1904003-b047-4eac-8bff-66f7faa401a6</stp>
-        <tr r="G41" s="1"/>
-      </tp>
-      <tp>
-        <v>1</v>
-        <stp/>
-        <stp>fa213f58-161b-48fe-8fc9-d4c274ae3073</stp>
-        <tr r="C5" s="5"/>
-      </tp>
-      <tp>
-        <v>1</v>
-        <stp/>
-        <stp>2d8da6e6-9894-4d88-8f40-41495eb6b3aa</stp>
-        <tr r="G57" s="1"/>
-      </tp>
-    </main>
-    <main first="rtdsrv.d1787fac4db647738cc71ff32b237324">
-      <tp>
-        <v>1</v>
-        <stp/>
-        <stp>fc72a9bc-0a8f-4112-ae75-59a68cc135ba</stp>
-        <tr r="G39" s="1"/>
-      </tp>
-    </main>
-    <main first="rtdsrv.d1787fac4db647738cc71ff32b237324">
-      <tp>
-        <v>1</v>
-        <stp/>
-        <stp>c0dc28dd-bb47-4642-82ae-ddcbc81b5e87</stp>
-        <tr r="G36" s="4"/>
-      </tp>
-      <tp>
-        <v>1</v>
-        <stp/>
-        <stp>d9cbe40e-0c58-4bb2-b873-60cbd1abd829</stp>
-        <tr r="C23" s="5"/>
-      </tp>
-      <tp>
-        <v>1</v>
-        <stp/>
-        <stp>b3e287d8-7454-4b2c-bc3a-3c0eec3e6bfc</stp>
-        <tr r="E7" s="3"/>
-      </tp>
-      <tp>
-        <v>1</v>
-        <stp/>
-        <stp>4e20341a-1c7e-403b-994d-96a7d12230a1</stp>
-        <tr r="G50" s="1"/>
-      </tp>
-    </main>
-    <main first="rtdsrv.d1787fac4db647738cc71ff32b237324">
-      <tp>
-        <v>1</v>
-        <stp/>
-        <stp>932fd7c3-4b0a-4153-9261-82e0d80699d0</stp>
-        <tr r="G45" s="1"/>
-      </tp>
-      <tp>
-        <v>1</v>
-        <stp/>
-        <stp>ecd1a62e-93e3-4350-bcc6-04a6b4734963</stp>
-        <tr r="G20" s="1"/>
-      </tp>
-      <tp>
-        <v>1</v>
-        <stp/>
-        <stp>34896d5a-4988-4d2b-a8ac-d2c8cf0d3531</stp>
-        <tr r="G31" s="4"/>
-      </tp>
-      <tp>
-        <v>1</v>
-        <stp/>
-        <stp>5a0dcc88-65ff-4bee-963c-079d1b4fa1fb</stp>
-        <tr r="G24" s="4"/>
-      </tp>
-      <tp>
-        <v>1</v>
-        <stp/>
-        <stp>4171b93b-b652-482e-b41a-c60b681a3646</stp>
-        <tr r="G22" s="1"/>
-      </tp>
-    </main>
-    <main first="rtdsrv.d1787fac4db647738cc71ff32b237324">
-      <tp>
-        <v>1</v>
-        <stp/>
-        <stp>bc8948d6-8083-4210-b085-59453d4a402b</stp>
-        <tr r="G22" s="4"/>
-      </tp>
-    </main>
-    <main first="rtdsrv.d1787fac4db647738cc71ff32b237324">
-      <tp>
-        <v>1</v>
-        <stp/>
-        <stp>fe5a5bb5-4781-4fae-8f0e-9d21ba75dd33</stp>
-        <tr r="D36" s="5"/>
-      </tp>
-    </main>
-    <main first="rtdsrv.d1787fac4db647738cc71ff32b237324">
-      <tp>
-        <v>1</v>
-        <stp/>
-        <stp>ceab6afd-eb63-4ec5-b168-3bd684cd13be</stp>
-        <tr r="G21" s="4"/>
-      </tp>
-    </main>
-    <main first="rtdsrv.d1787fac4db647738cc71ff32b237324">
-      <tp>
-        <v>1</v>
-        <stp/>
-        <stp>37d19242-febf-48c6-b819-24fc2bdc3523</stp>
-        <tr r="G19" s="4"/>
-      </tp>
-      <tp>
-        <v>1</v>
-        <stp/>
-        <stp>fbc9db33-f764-4c2d-a12f-de883bacd0dd</stp>
-        <tr r="G27" s="4"/>
-      </tp>
-      <tp>
-        <v>1</v>
-        <stp/>
-        <stp>bdebd685-5eea-43b0-8b15-610c5434dde4</stp>
-        <tr r="F1" s="1"/>
-      </tp>
-      <tp>
-        <v>1</v>
-        <stp/>
-        <stp>36971736-cf58-448e-9ba4-5aa2965c06e7</stp>
-        <tr r="G57" s="4"/>
-      </tp>
-    </main>
-    <main first="rtdsrv.d1787fac4db647738cc71ff32b237324">
-      <tp>
-        <v>1</v>
-        <stp/>
-        <stp>7e707116-7f40-48a1-ad0b-bea805dd9636</stp>
-        <tr r="G44" s="4"/>
-      </tp>
-    </main>
-    <main first="rtdsrv.d1787fac4db647738cc71ff32b237324">
-      <tp>
-        <v>1</v>
-        <stp/>
-        <stp>105f7372-f40e-4116-a971-2ae30d3dce0b</stp>
-        <tr r="G27" s="1"/>
-      </tp>
-      <tp>
-        <v>1</v>
-        <stp/>
-        <stp>9d6da1f8-5e8e-4b7c-83c7-4b704dbb0b8f</stp>
-        <tr r="G30" s="4"/>
-      </tp>
-      <tp>
-        <v>1</v>
-        <stp/>
-        <stp>85ba3259-11b9-4f1e-be47-3bd7d867f80f</stp>
-        <tr r="G20" s="4"/>
-      </tp>
-    </main>
-    <main first="rtdsrv.d1787fac4db647738cc71ff32b237324">
-      <tp>
-        <v>1</v>
-        <stp/>
-        <stp>52aa4d2f-a92b-4441-a763-068a64d527fb</stp>
-        <tr r="F6" s="1"/>
-      </tp>
-    </main>
-    <main first="rtdsrv.d1787fac4db647738cc71ff32b237324">
-      <tp>
-        <v>1</v>
-        <stp/>
-        <stp>bbfd060e-a779-4150-ad5d-aaaeaded90f3</stp>
-        <tr r="G23" s="1"/>
-      </tp>
-    </main>
-    <main first="rtdsrv.d1787fac4db647738cc71ff32b237324">
-      <tp>
-        <v>1</v>
-        <stp/>
-        <stp>a4f31b3f-b425-41f8-bbc0-0f3e691ab589</stp>
-        <tr r="G28" s="4"/>
-      </tp>
-    </main>
-    <main first="rtdsrv.d1787fac4db647738cc71ff32b237324">
-      <tp>
-        <v>1</v>
-        <stp/>
-        <stp>bdb5bbc5-4ff6-4065-be9d-341f21ec9ac6</stp>
-        <tr r="G47" s="4"/>
-      </tp>
-      <tp>
-        <v>1</v>
-        <stp/>
-        <stp>3cb26f99-e2cd-4188-aed4-33001ff02373</stp>
-        <tr r="D7" s="5"/>
-      </tp>
-    </main>
-    <main first="rtdsrv.d1787fac4db647738cc71ff32b237324">
-      <tp>
-        <v>1</v>
-        <stp/>
-        <stp>0268655a-1b26-495a-8607-589e7404c06d</stp>
-        <tr r="C2" s="2"/>
-      </tp>
-    </main>
-    <main first="rtdsrv.d1787fac4db647738cc71ff32b237324">
-      <tp>
-        <v>1</v>
-        <stp/>
-        <stp>6c9a97ee-7646-4edb-b18d-fb65f6cdc5ff</stp>
-        <tr r="N47" s="5"/>
-      </tp>
-    </main>
-    <main first="rtdsrv.d1787fac4db647738cc71ff32b237324">
-      <tp>
-        <v>1</v>
-        <stp/>
-        <stp>37ffc880-f745-4166-bf76-5023c97ff917</stp>
-        <tr r="G36" s="1"/>
-      </tp>
-      <tp>
-        <v>1</v>
-        <stp/>
-        <stp>cab723cc-ffcd-4895-8fa0-818a28a281a9</stp>
-        <tr r="I42" s="4"/>
-      </tp>
-    </main>
-    <main first="rtdsrv.d1787fac4db647738cc71ff32b237324">
-      <tp>
-        <v>1</v>
-        <stp/>
-        <stp>c8b1fead-72de-4389-9c00-b21a09bc96a6</stp>
-        <tr r="G54" s="4"/>
-      </tp>
-      <tp>
-        <v>1</v>
-        <stp/>
-        <stp>417c8a1a-acc6-49ad-b11e-f80e4d90cf89</stp>
-        <tr r="G48" s="4"/>
-      </tp>
-    </main>
-    <main first="rtdsrv.d1787fac4db647738cc71ff32b237324">
-      <tp>
-        <v>1</v>
-        <stp/>
-        <stp>405f1312-aa43-41d1-beda-dba8138c58ae</stp>
-        <tr r="G54" s="1"/>
-      </tp>
-    </main>
-    <main first="rtdsrv.d1787fac4db647738cc71ff32b237324">
-      <tp>
-        <v>1</v>
-        <stp/>
-        <stp>c03b1621-588e-4f3f-8db4-c22a6ce3387e</stp>
-        <tr r="G55" s="4"/>
-      </tp>
-    </main>
-    <main first="rtdsrv.d1787fac4db647738cc71ff32b237324">
-      <tp>
-        <v>1</v>
-        <stp/>
-        <stp>c5ceb666-ef12-4dbc-9606-dd1fc91cc792</stp>
-        <tr r="G38" s="4"/>
-      </tp>
-    </main>
-    <main first="rtdsrv.d1787fac4db647738cc71ff32b237324">
-      <tp>
-        <v>1</v>
-        <stp/>
-        <stp>8e8fb2dc-6821-4c6c-998f-1ebebae84b21</stp>
-        <tr r="G45" s="4"/>
-      </tp>
-    </main>
-    <main first="rtdsrv.d1787fac4db647738cc71ff32b237324">
-      <tp>
-        <v>1</v>
-        <stp/>
-        <stp>3925f836-cadf-4ff8-bd54-84ae5d035c86</stp>
-        <tr r="G35" s="4"/>
-      </tp>
-    </main>
-    <main first="rtdsrv.d1787fac4db647738cc71ff32b237324">
-      <tp>
-        <v>1</v>
-        <stp/>
-        <stp>c7eef671-ab7d-4c5f-abea-7cbe893a7d24</stp>
-        <tr r="G52" s="1"/>
-      </tp>
-      <tp>
-        <v>1</v>
-        <stp/>
-        <stp>20e4e851-e435-46e3-babc-55d3bb1c76a2</stp>
-        <tr r="C34" s="5"/>
-      </tp>
-    </main>
-    <main first="rtdsrv.d1787fac4db647738cc71ff32b237324">
-      <tp>
-        <v>1</v>
-        <stp/>
-        <stp>72544104-8729-4c43-afc8-8d6f2ae313c1</stp>
-        <tr r="I19" s="1"/>
-      </tp>
-      <tp>
-        <v>1</v>
-        <stp/>
-        <stp>c9303e59-adc8-4ce4-9a69-f280345a3d2c</stp>
-        <tr r="F1" s="4"/>
-      </tp>
-    </main>
-    <main first="rtdsrv.d1787fac4db647738cc71ff32b237324">
-      <tp>
-        <v>1</v>
-        <stp/>
-        <stp>fcc016aa-c2cc-4936-9151-cf599159d085</stp>
-        <tr r="G24" s="1"/>
-      </tp>
-    </main>
-    <main first="rtdsrv.d1787fac4db647738cc71ff32b237324">
-      <tp>
-        <v>1</v>
-        <stp/>
-        <stp>a77f35d2-b944-4c9a-9263-0a2fd1c0a5c1</stp>
-        <tr r="G30" s="1"/>
-      </tp>
-      <tp>
-        <v>1</v>
-        <stp/>
-        <stp>8e66f66c-153b-4c57-84c9-5538976c9fab</stp>
-        <tr r="G32" s="1"/>
-      </tp>
-    </main>
-    <main first="rtdsrv.d1787fac4db647738cc71ff32b237324">
-      <tp>
-        <v>1</v>
-        <stp/>
-        <stp>19f1ee8e-7484-4c66-adee-ef3954852929</stp>
-        <tr r="E17" s="3"/>
-      </tp>
-    </main>
-    <main first="rtdsrv.d1787fac4db647738cc71ff32b237324">
-      <tp>
-        <v>1</v>
-        <stp/>
-        <stp>8f4f3d0a-4d63-4d9d-a42a-b5712c582e99</stp>
-        <tr r="G34" s="1"/>
-      </tp>
-    </main>
-    <main first="rtdsrv.d1787fac4db647738cc71ff32b237324">
-      <tp>
-        <v>1</v>
-        <stp/>
-        <stp>71a7a642-ae38-45e3-b328-4d2b04475d64</stp>
-        <tr r="D25" s="5"/>
-      </tp>
-    </main>
-    <main first="rtdsrv.d1787fac4db647738cc71ff32b237324">
-      <tp>
-        <v>1</v>
-        <stp/>
-        <stp>b66efb31-3ca7-4fcf-8e44-6558b1a9da41</stp>
-        <tr r="G31" s="1"/>
-      </tp>
-    </main>
-    <main first="rtdsrv.d1787fac4db647738cc71ff32b237324">
-      <tp>
-        <v>1</v>
-        <stp/>
-        <stp>3a4de821-b3d3-427e-9add-5b9fb97171aa</stp>
-        <tr r="G46" s="1"/>
-      </tp>
-    </main>
-    <main first="rtdsrv.d1787fac4db647738cc71ff32b237324">
-      <tp>
-        <v>1</v>
-        <stp/>
-        <stp>f28b4a67-da7b-42c7-aa97-7df9758298e0</stp>
-        <tr r="I28" s="1"/>
-      </tp>
-    </main>
-    <main first="rtdsrv.d1787fac4db647738cc71ff32b237324">
-      <tp>
-        <v>1</v>
-        <stp/>
-        <stp>602d787a-b016-49de-aaa6-5c5a3d79182f</stp>
-        <tr r="G26" s="1"/>
-      </tp>
-      <tp>
-        <v>1</v>
-        <stp/>
-        <stp>30a31a4e-6790-4656-a95e-4f8dbb811171</stp>
-        <tr r="G33" s="1"/>
-      </tp>
-      <tp>
-        <v>3</v>
-        <stp/>
-        <stp>7cc161e9-59ac-4aec-9cc0-d2831451c029</stp>
-        <tr r="E19" s="3"/>
-      </tp>
-    </main>
-    <main first="rtdsrv.d1787fac4db647738cc71ff32b237324">
-      <tp>
-        <v>1</v>
-        <stp/>
-        <stp>70d129b8-4b00-4370-83c4-3b7168b3ce04</stp>
+    <main first="rtdsrv.fec3502cf85349c38b0a9636c87dce5f">
+      <tp>
+        <v>1</v>
+        <stp/>
+        <stp>d876a44f-64bd-483f-82e9-c75310b9c3a1</stp>
         <tr r="N33" s="5"/>
-      </tp>
-    </main>
-    <main first="rtdsrv.d1787fac4db647738cc71ff32b237324">
-      <tp>
-        <v>1</v>
-        <stp/>
-        <stp>9d2c464a-e2a8-4982-905d-bc58755f6722</stp>
-        <tr r="G50" s="4"/>
-      </tp>
-    </main>
-    <main first="rtdsrv.d1787fac4db647738cc71ff32b237324">
-      <tp>
-        <v>1</v>
-        <stp/>
-        <stp>a34c74a5-6e01-4553-be1c-97f3bd2591ab</stp>
-        <tr r="G43" s="1"/>
-      </tp>
-    </main>
-    <main first="rtdsrv.d1787fac4db647738cc71ff32b237324">
-      <tp>
-        <v>1</v>
-        <stp/>
-        <stp>1af37226-3c80-4cb3-9815-855187700657</stp>
-        <tr r="G51" s="1"/>
-      </tp>
-    </main>
-    <main first="rtdsrv.d1787fac4db647738cc71ff32b237324">
-      <tp>
-        <v>1</v>
-        <stp/>
-        <stp>25beeffa-2e2c-49a3-ac7a-c7f0050be0dd</stp>
-        <tr r="G25" s="1"/>
-      </tp>
-      <tp>
-        <v>1</v>
-        <stp/>
-        <stp>8589e631-5f79-45a9-a521-e92dad0bb788</stp>
-        <tr r="G47" s="1"/>
-      </tp>
-      <tp>
-        <v>1</v>
-        <stp/>
-        <stp>f9dd498b-d00c-457f-a008-1256a4749c14</stp>
-        <tr r="C13" s="5"/>
-      </tp>
-    </main>
-    <main first="rtdsrv.d1787fac4db647738cc71ff32b237324">
-      <tp>
-        <v>1</v>
-        <stp/>
-        <stp>ee58db56-6b7b-40e2-9909-eaddc12c44ba</stp>
-        <tr r="F6" s="4"/>
-      </tp>
-      <tp>
-        <v>1</v>
-        <stp/>
-        <stp>ed97f581-3276-414a-8587-012009c04d80</stp>
-        <tr r="G40" s="4"/>
-      </tp>
-      <tp>
-        <v>1</v>
-        <stp/>
-        <stp>aa9527dd-9290-408b-8ea9-d9ad66620722</stp>
-        <tr r="E4" s="3"/>
-      </tp>
-    </main>
-    <main first="rtdsrv.d1787fac4db647738cc71ff32b237324">
-      <tp>
-        <v>1</v>
-        <stp/>
-        <stp>2c3cdeaf-7d41-4be2-9fc4-840be121e1eb</stp>
-        <tr r="D50" s="5"/>
-      </tp>
-      <tp>
-        <v>1</v>
-        <stp/>
-        <stp>c7907278-6fec-4d69-80e1-0cdb59116ae4</stp>
-        <tr r="I38" s="4"/>
-      </tp>
-      <tp>
-        <v>1</v>
-        <stp/>
-        <stp>dd0af438-5e43-4ce0-8428-842cad0a4c20</stp>
-        <tr r="G43" s="4"/>
-      </tp>
-    </main>
-    <main first="rtdsrv.d1787fac4db647738cc71ff32b237324">
-      <tp>
-        <v>1</v>
-        <stp/>
-        <stp>05eca21a-ec78-4780-a9bc-f21df0942f05</stp>
-        <tr r="I33" s="4"/>
-      </tp>
-      <tp>
-        <v>1</v>
-        <stp/>
-        <stp>bbc5cd80-bdfa-4290-9ddc-6f99ee6f4fdc</stp>
-        <tr r="G56" s="4"/>
-      </tp>
-    </main>
-    <main first="rtdsrv.d1787fac4db647738cc71ff32b237324">
-      <tp>
-        <v>1</v>
-        <stp/>
-        <stp>af26cd98-701c-473b-a893-af4038df8ed0</stp>
-        <tr r="G28" s="1"/>
       </tp>
     </main>
   </volType>
@@ -1786,11 +1778,11 @@
       </c>
       <c r="F1" t="str" cm="1">
         <f t="array" ref="F1">_xll.ExLibris.Json.CreateJsonObject(E3:F6)</f>
-        <v>JsonObject:FEAF55B6-F256-4256-9161-1D1B64DEE139</v>
+        <v>JsonObject:623F6835-4451-4CC3-B87E-D5E03AD80608</v>
       </c>
       <c r="K1" t="str">
         <f>EXLIBRIS_CONFIGURATION</f>
-        <v>ExLibris.Core.ExLibrisConfiguration:24ADB25B-B7A4-4556-8E21-DF7CFC2AF75C</v>
+        <v>ExLibris.Core.ExLibrisConfiguration:A169F21B-3C75-4067-A8E9-C01650919406</v>
       </c>
     </row>
     <row r="2" spans="2:28" x14ac:dyDescent="0.4">
@@ -1860,7 +1852,7 @@
       </c>
       <c r="F6" t="str" cm="1">
         <f t="array" ref="F6">_xll.ExLibris.Json.CreateJsonArray(E8:J14)</f>
-        <v>JsonObject:0FB264D1-4D53-4D49-AAA9-52061311CDDC</v>
+        <v>JsonObject:69FE46EE-7BAD-44EE-A051-A35E12DB58A2</v>
       </c>
       <c r="L6" t="s">
         <v>68</v>
@@ -2099,7 +2091,7 @@
       </c>
       <c r="I19" t="str" cm="1">
         <f t="array" ref="I19">_xll.ExLibris.Json.GetJsonValue(F1,E6)</f>
-        <v>JsonObject:87C48750-5BE7-49D9-9F62-C2D7B06B7A24</v>
+        <v>JsonObject:3EEFC1CF-3E90-4341-B907-92CB5E1CF38C</v>
       </c>
       <c r="P19" t="str" cm="1">
         <f t="array" ref="P19:Q27">_xll.ExLibris.Json.GetJsonKeyValues(F1,,3)</f>
@@ -2404,7 +2396,7 @@
         <v>fixed_leg.cashflows.[0]</v>
       </c>
       <c r="Q22" t="str">
-        <v>JsonObject:DE5EACA0-1A4E-463B-89BA-0EFE2C25DD86</v>
+        <v>JsonObject:1212F87C-E83E-4EA3-B39B-C69E89770D3A</v>
       </c>
       <c r="S22" t="s">
         <v>32</v>
@@ -2503,7 +2495,7 @@
         <v>fixed_leg.cashflows.[1]</v>
       </c>
       <c r="Q23" t="str">
-        <v>JsonObject:57B6C87F-0B66-4F3A-8868-045D0C2F18C7</v>
+        <v>JsonObject:EEADEA6E-CC19-4756-BF0E-EB6D8A376D13</v>
       </c>
       <c r="S23" t="s">
         <v>33</v>
@@ -2602,7 +2594,7 @@
         <v>fixed_leg.cashflows.[2]</v>
       </c>
       <c r="Q24" t="str">
-        <v>JsonObject:5D27BF30-066D-4852-A63E-C2080A7BCCCB</v>
+        <v>JsonObject:7EE00EE0-F021-48CC-AF30-46DFD63C56CC</v>
       </c>
       <c r="S24" t="s">
         <v>34</v>
@@ -2701,7 +2693,7 @@
         <v>fixed_leg.cashflows.[3]</v>
       </c>
       <c r="Q25" t="str">
-        <v>JsonObject:D81B8AE9-7ED3-4E79-AF7E-74CA81157E43</v>
+        <v>JsonObject:66A47F1E-B96C-4129-BD6F-EC5FBA11C55D</v>
       </c>
       <c r="S25" t="s">
         <v>35</v>
@@ -2800,7 +2792,7 @@
         <v>fixed_leg.cashflows.[4]</v>
       </c>
       <c r="Q26" t="str">
-        <v>JsonObject:D3798F61-C738-4505-9FA5-B176C37C2C4E</v>
+        <v>JsonObject:877FF99A-D53A-4294-AF80-8AD15E0507C5</v>
       </c>
       <c r="S26" t="s">
         <v>36</v>
@@ -2881,7 +2873,7 @@
         <v>fixed_leg.cashflows.[5]</v>
       </c>
       <c r="Q27" t="str">
-        <v>JsonObject:1835D640-7BAD-4911-9240-482839F49999</v>
+        <v>JsonObject:C28BD98F-9EA9-45E9-BF1C-568A1FD0DEAF</v>
       </c>
       <c r="S27" t="s">
         <v>37</v>
@@ -2918,7 +2910,7 @@
       </c>
       <c r="I28" t="str" cm="1">
         <f t="array" ref="I28">_xll.ExLibris.Json.GetJsonValue(I19,"[2]")</f>
-        <v>JsonObject:CD15D726-92C0-4486-9C36-EEF6F80FE91F</v>
+        <v>JsonObject:C0CEBDDA-B9C4-4979-A93C-C5BD82F613A9</v>
       </c>
       <c r="S28" t="s">
         <v>38</v>
@@ -2974,7 +2966,7 @@
       </c>
       <c r="P29" t="str" cm="1">
         <f t="array" ref="P29">_xll.ExLibris.Json.CreateJsonObject(P22:Q27)</f>
-        <v>JsonObject:F856625E-56F8-4FD8-9FBF-EC1651BD6EFE</v>
+        <v>JsonObject:622C3500-D38A-451D-ACD1-FCF6CD1ADC11</v>
       </c>
       <c r="S29" t="s">
         <v>39</v>
@@ -4796,11 +4788,11 @@
       </c>
       <c r="F1" t="str" cm="1">
         <f t="array" ref="F1">_xll.ExLibris.Json.CreateJsonObject(E3:F6, EXLIBRIS_CONFIGURATION)</f>
-        <v>JsonObject:01C35595-5E97-44D0-AF9B-401ED84F14E7</v>
+        <v>JsonObject:6705B80E-340C-4216-B581-6E92DEBEB39B</v>
       </c>
       <c r="K1" t="str">
         <f>EXLIBRIS_CONFIGURATION</f>
-        <v>ExLibris.Core.ExLibrisConfiguration:24ADB25B-B7A4-4556-8E21-DF7CFC2AF75C</v>
+        <v>ExLibris.Core.ExLibrisConfiguration:A169F21B-3C75-4067-A8E9-C01650919406</v>
       </c>
     </row>
     <row r="2" spans="2:25" x14ac:dyDescent="0.4">
@@ -4870,7 +4862,7 @@
       </c>
       <c r="F6" t="str" cm="1">
         <f t="array" ref="F6">_xll.ExLibris.Json.CreateJsonArray(E8:J14, EXLIBRIS_CONFIGURATION)</f>
-        <v>JsonObject:531CBB1A-AAB5-46C7-8765-D2CF539D73C0</v>
+        <v>JsonObject:EA8A377D-2E23-4FA7-8D86-08096F3DE6A3</v>
       </c>
       <c r="L6" t="s">
         <v>68</v>
@@ -5121,7 +5113,7 @@
       </c>
       <c r="I19" t="str" cm="1">
         <f t="array" ref="I19">_xll.ExLibris.Json.GetJsonValue(F1,E6, EXLIBRIS_CONFIGURATION)</f>
-        <v>JsonObject:327669E4-FD13-41AA-BD7F-9D7BD82647D3</v>
+        <v>JsonObject:AF929A4D-B3EC-4AAA-8C0D-1FD0C1B57C7D</v>
       </c>
       <c r="P19" t="s">
         <v>14</v>
@@ -5843,7 +5835,7 @@
       </c>
       <c r="I28" t="str" cm="1">
         <f t="array" ref="I28">_xll.ExLibris.Json.GetJsonValue(I19,"[2]", EXLIBRIS_CONFIGURATION)</f>
-        <v>JsonObject:E0ACD3ED-F103-4688-9674-8F620C7B4846</v>
+        <v>JsonObject:E9D6A6A1-229F-4E2B-AB2F-0BE7C53A5C9D</v>
       </c>
       <c r="P28" t="s">
         <v>38</v>
@@ -6100,7 +6092,7 @@
       </c>
       <c r="I32" t="str" cm="1">
         <f t="array" ref="I32">_xll.ExLibris.Json.GetJsonValue(F1,E6,EXLIBRIS_CONFIGURATION)</f>
-        <v>JsonObject:327669E4-FD13-41AA-BD7F-9D7BD82647D3</v>
+        <v>JsonObject:AF929A4D-B3EC-4AAA-8C0D-1FD0C1B57C7D</v>
       </c>
       <c r="P32" t="s">
         <v>42</v>
@@ -6137,7 +6129,7 @@
       </c>
       <c r="I33" t="str" cm="1">
         <f t="array" ref="I33">_xll.ExLibris.Json.SeachJsonArrayElements(I32,I8,I11,EXLIBRIS_CONFIGURATION)</f>
-        <v>JsonObject:30472878-CE6C-4467-AE39-6ABB050A7208</v>
+        <v>JsonObject:AEE131CD-9E63-49B1-8B47-E63629B8575C</v>
       </c>
       <c r="P33" t="s">
         <v>43</v>
@@ -6487,7 +6479,7 @@
       </c>
       <c r="I38" t="str" cm="1">
         <f t="array" ref="I38">_xll.ExLibris.Json.SeachJsonArrayElements(I32,J8,J11,EXLIBRIS_CONFIGURATION)</f>
-        <v>JsonObject:5469C72A-CE31-47BF-ADD4-DA535D9A5668</v>
+        <v>JsonObject:89622B6F-33BC-48C9-B001-3FE96B312D1A</v>
       </c>
       <c r="P38" t="s">
         <v>48</v>
@@ -6744,7 +6736,7 @@
       </c>
       <c r="I42" t="str" cm="1">
         <f t="array" ref="I42">_xll.ExLibris.Json.SeachJsonArrayElements(I32,J8,,EXLIBRIS_CONFIGURATION)</f>
-        <v>JsonObject:0E63F8CA-CBEB-4495-8244-C5DCCA769678</v>
+        <v>JsonObject:C7740020-3253-41F8-8F7D-56E87CFD0734</v>
       </c>
       <c r="P42" t="s">
         <v>52</v>
@@ -7298,7 +7290,7 @@
       </c>
       <c r="C2" t="str" cm="1">
         <f t="array" ref="C2">_xll.ExLibris.LoadConfiguration(B6:C15)</f>
-        <v>ExLibris.Core.ExLibrisConfiguration:24ADB25B-B7A4-4556-8E21-DF7CFC2AF75C</v>
+        <v>ExLibris.Core.ExLibrisConfiguration:A169F21B-3C75-4067-A8E9-C01650919406</v>
       </c>
     </row>
     <row r="4" spans="2:8" s="4" customFormat="1" ht="18" x14ac:dyDescent="0.4">
@@ -7324,8 +7316,8 @@
         <v>Error</v>
       </c>
       <c r="H6" t="str" cm="1">
-        <f t="array" ref="H6:H10">_xll.ExLibris.ObserveRegisteredObjects()</f>
-        <v>ExLibris.Core.WebSockets.WebsocketClient:775383A7-EAAC-425F-BBF2-5B1060DBD59B</v>
+        <f t="array" ref="H6:H14">_xll.ExLibris.ObserveRegisteredObjects()</f>
+        <v>ExLibris.Core.WebAPIs.WebAPI:DE93CF18-3BBD-402F-A843-CEF41861F596</v>
       </c>
     </row>
     <row r="7" spans="2:8" x14ac:dyDescent="0.4">
@@ -7342,7 +7334,7 @@
         <v>Null</v>
       </c>
       <c r="H7" t="str">
-        <v>JsonObject:13CCC74E-74C5-4157-A96C-DFA57E671E4C</v>
+        <v>ExLibris.Core.WebAPIs.WebAPI:F992A6ED-9AB5-4908-840B-718FBDF7535A</v>
       </c>
     </row>
     <row r="8" spans="2:8" x14ac:dyDescent="0.4">
@@ -7359,7 +7351,7 @@
         <v>Null</v>
       </c>
       <c r="H8" t="str">
-        <v>JsonObject:D560D4B9-72BB-4BFE-826E-E16F2B223BFE</v>
+        <v>JsonObject:2A58B27D-675E-4034-AD59-7B57491E800E</v>
       </c>
     </row>
     <row r="9" spans="2:8" x14ac:dyDescent="0.4">
@@ -7376,7 +7368,7 @@
         <v>Null</v>
       </c>
       <c r="H9" t="str">
-        <v>ExLibris.Core.ExLibrisConfiguration:24ADB25B-B7A4-4556-8E21-DF7CFC2AF75C</v>
+        <v>ExLibris.Core.WebSockets.WebsocketClient:34127D7E-4CD6-41C6-82F8-0E63D38248E6</v>
       </c>
     </row>
     <row r="10" spans="2:8" x14ac:dyDescent="0.4">
@@ -7393,7 +7385,7 @@
         <v>StringEmpty</v>
       </c>
       <c r="H10" t="str">
-        <v>ExLibris.Core.WebAPIs.WebAPI:FCC762F8-ED4C-4FF8-95E7-CC84EAA249C2</v>
+        <v>ExLibris.Core.WebSockets.WebsocketClient:FA73B600-4A27-4BF1-952F-90C5D53BC9C9</v>
       </c>
     </row>
     <row r="11" spans="2:8" x14ac:dyDescent="0.4">
@@ -7409,6 +7401,9 @@
       <c r="F11" t="str">
         <v>StringEmpty</v>
       </c>
+      <c r="H11" t="str">
+        <v>ExLibris.Core.WebAPIs.WebAPI:2E9B4D0E-91E8-4953-AB2F-AB683EE9AD80</v>
+      </c>
     </row>
     <row r="12" spans="2:8" x14ac:dyDescent="0.4">
       <c r="B12" t="s">
@@ -7423,6 +7418,9 @@
       <c r="F12" t="str">
         <v>yyyy-MM-dd</v>
       </c>
+      <c r="H12" t="str">
+        <v>ExLibris.Core.ExLibrisConfiguration:A169F21B-3C75-4067-A8E9-C01650919406</v>
+      </c>
     </row>
     <row r="13" spans="2:8" x14ac:dyDescent="0.4">
       <c r="B13" t="s">
@@ -7437,6 +7435,9 @@
       <c r="F13" t="str">
         <v>payment _date</v>
       </c>
+      <c r="H13" t="str">
+        <v>ExLibris.Core.WebAPIs.WebAPI:A77102A5-4736-4B3B-9940-2D0470A6736C</v>
+      </c>
     </row>
     <row r="14" spans="2:8" x14ac:dyDescent="0.4">
       <c r="B14" t="s">
@@ -7450,6 +7451,9 @@
       </c>
       <c r="F14" t="str">
         <v>start_date</v>
+      </c>
+      <c r="H14" t="str">
+        <v>JsonObject:E062079A-A1E7-4DA8-9EE1-3BE1C4EE4FD6</v>
       </c>
     </row>
     <row r="15" spans="2:8" x14ac:dyDescent="0.4">
@@ -7495,7 +7499,7 @@
       </c>
       <c r="E4" t="str" cm="1">
         <f t="array" ref="E4">_xll.ExLibris.WebSockets.OpenWebSocket("ws://localhost:10101",,D4)</f>
-        <v>ExLibris.Core.WebSockets.WebsocketClient:022610D8-7DA7-4027-B75A-69F26CB9C36C</v>
+        <v>ExLibris.Core.WebSockets.WebsocketClient:34127D7E-4CD6-41C6-82F8-0E63D38248E6</v>
       </c>
     </row>
     <row r="6" spans="2:5" x14ac:dyDescent="0.4">
@@ -7585,7 +7589,7 @@
       </c>
       <c r="E17" t="str" cm="1">
         <f t="array" ref="E17">_xll.ExLibris.WebSockets.OpenWebSocket("ws://localhost:10101",,D17)</f>
-        <v>ExLibris.Core.WebSockets.WebsocketClient:775383A7-EAAC-425F-BBF2-5B1060DBD59B</v>
+        <v>ExLibris.Core.WebSockets.WebsocketClient:FA73B600-4A27-4BF1-952F-90C5D53BC9C9</v>
       </c>
     </row>
     <row r="19" spans="4:5" x14ac:dyDescent="0.4">
@@ -7700,7 +7704,7 @@
       </c>
       <c r="C5" t="str" cm="1">
         <f t="array" ref="C5">_xll.ExLibris.WebAPIs.OpenWebSocket($C$2,B5)</f>
-        <v>ExLibris.Core.WebAPIs.WebAPI:3A2163D7-BDD0-4F94-B890-D0345078D963</v>
+        <v>ExLibris.Core.WebAPIs.WebAPI:DE93CF18-3BBD-402F-A843-CEF41861F596</v>
       </c>
     </row>
     <row r="6" spans="2:4" x14ac:dyDescent="0.4">
@@ -7720,7 +7724,7 @@
       </c>
       <c r="D7" t="str" cm="1">
         <f t="array" ref="D7">_xll.ExLibris.WebAPIs.WebAPIGet(C5,D6)</f>
-        <v>ExLibris.Core.WebAPIs.Response:3211004F-4F9A-4CBA-9B3D-795D9363CFC7</v>
+        <v>ExLibris.Core.WebAPIs.Response:B88BDE11-5F0D-4ED5-9E92-B1610492CA6F</v>
       </c>
     </row>
     <row r="8" spans="2:4" x14ac:dyDescent="0.4">
@@ -7729,76 +7733,6 @@
       </c>
       <c r="D8" t="str" cm="1">
         <f t="array" ref="D8">_xll.ExLibris.WebAPIs.WebAPIRequestContent(D7)</f>
-        <v xml:space="preserve">{
-  "args": {}, 
-  "headers": {
-    "Host": "localhost"
-  }, 
-  "origin": "172.17.0.1", 
-  "url": "http://localhost/get"
-}
-</v>
-      </c>
-    </row>
-    <row r="9" spans="2:4" x14ac:dyDescent="0.4">
-      <c r="C9" t="s">
-        <v>101</v>
-      </c>
-      <c r="D9" t="str" cm="1">
-        <f t="array" ref="D9">_xll.ExLibris.WebAPIs.WebAPIResponseStatus(D7)</f>
-        <v>OK(200)</v>
-      </c>
-    </row>
-    <row r="10" spans="2:4" x14ac:dyDescent="0.4">
-      <c r="C10" t="s">
-        <v>138</v>
-      </c>
-      <c r="D10" t="str" cm="1">
-        <f t="array" ref="D10">_xll.ExLibris.WebAPIs.WebAPIResponseHeader(D7)</f>
-        <v xml:space="preserve">Connection: keep-alive_x000D_
-Access-Control-Allow-Origin: *_x000D_
-Access-Control-Allow-Credentials: true_x000D_
-Date: Thu, 23 Sep 2021 11:55:16 GMT_x000D_
-Server: gunicorn/19.9.0_x000D_
-</v>
-      </c>
-    </row>
-    <row r="13" spans="2:4" x14ac:dyDescent="0.4">
-      <c r="B13" t="s">
-        <v>128</v>
-      </c>
-      <c r="C13" t="str" cm="1">
-        <f t="array" ref="C13">_xll.ExLibris.WebAPIs.OpenWebSocket(,B13)</f>
-        <v>ExLibris.Core.WebAPIs.WebAPI:4FB1F122-7BD2-4DFC-89EF-2AE6C87CBE6E</v>
-      </c>
-    </row>
-    <row r="14" spans="2:4" x14ac:dyDescent="0.4">
-      <c r="B14" t="s">
-        <v>125</v>
-      </c>
-      <c r="C14" t="s">
-        <v>124</v>
-      </c>
-      <c r="D14" t="str">
-        <f>$C$2&amp;"get"</f>
-        <v>http://localhost:80/get</v>
-      </c>
-    </row>
-    <row r="15" spans="2:4" x14ac:dyDescent="0.4">
-      <c r="C15" t="s">
-        <v>122</v>
-      </c>
-      <c r="D15" t="str" cm="1">
-        <f t="array" ref="D15">_xll.ExLibris.WebAPIs.WebAPIGet(C13,D14,,C13)</f>
-        <v>ExLibris.Core.WebAPIs.Response:A0D930E7-8868-4534-B857-D12DAE3EA0A9</v>
-      </c>
-    </row>
-    <row r="16" spans="2:4" x14ac:dyDescent="0.4">
-      <c r="C16" t="s">
-        <v>123</v>
-      </c>
-      <c r="D16" t="str" cm="1">
-        <f t="array" ref="D16">_xll.ExLibris.WebAPIs.WebAPIRequestContent(D15)</f>
         <v xml:space="preserve">{
   "args": {}, 
   "headers": {
@@ -7811,6 +7745,76 @@
 </v>
       </c>
     </row>
+    <row r="9" spans="2:4" x14ac:dyDescent="0.4">
+      <c r="C9" t="s">
+        <v>101</v>
+      </c>
+      <c r="D9" t="str" cm="1">
+        <f t="array" ref="D9">_xll.ExLibris.WebAPIs.WebAPIResponseStatus(D7)</f>
+        <v>OK(200)</v>
+      </c>
+    </row>
+    <row r="10" spans="2:4" x14ac:dyDescent="0.4">
+      <c r="C10" t="s">
+        <v>138</v>
+      </c>
+      <c r="D10" t="str" cm="1">
+        <f t="array" ref="D10">_xll.ExLibris.WebAPIs.WebAPIResponseHeader(D7)</f>
+        <v xml:space="preserve">Connection: keep-alive_x000D_
+Access-Control-Allow-Origin: *_x000D_
+Access-Control-Allow-Credentials: true_x000D_
+Date: Thu, 23 Sep 2021 13:10:44 GMT_x000D_
+Server: gunicorn/19.9.0_x000D_
+</v>
+      </c>
+    </row>
+    <row r="13" spans="2:4" x14ac:dyDescent="0.4">
+      <c r="B13" t="s">
+        <v>128</v>
+      </c>
+      <c r="C13" t="str" cm="1">
+        <f t="array" ref="C13">_xll.ExLibris.WebAPIs.OpenWebSocket(,B13)</f>
+        <v>ExLibris.Core.WebAPIs.WebAPI:F992A6ED-9AB5-4908-840B-718FBDF7535A</v>
+      </c>
+    </row>
+    <row r="14" spans="2:4" x14ac:dyDescent="0.4">
+      <c r="B14" t="s">
+        <v>125</v>
+      </c>
+      <c r="C14" t="s">
+        <v>124</v>
+      </c>
+      <c r="D14" t="str">
+        <f>$C$2&amp;"get"</f>
+        <v>http://localhost:80/get</v>
+      </c>
+    </row>
+    <row r="15" spans="2:4" x14ac:dyDescent="0.4">
+      <c r="C15" t="s">
+        <v>122</v>
+      </c>
+      <c r="D15" t="str" cm="1">
+        <f t="array" ref="D15">_xll.ExLibris.WebAPIs.WebAPIGet(C13,D14,C13)</f>
+        <v>ExLibris.Core.WebAPIs.Response:416876DD-FF98-41E3-B602-5ACC625EEBB3</v>
+      </c>
+    </row>
+    <row r="16" spans="2:4" x14ac:dyDescent="0.4">
+      <c r="C16" t="s">
+        <v>123</v>
+      </c>
+      <c r="D16" t="str" cm="1">
+        <f t="array" ref="D16">_xll.ExLibris.WebAPIs.WebAPIRequestContent(D15)</f>
+        <v xml:space="preserve">{
+  "args": {}, 
+  "headers": {
+    "Host": "localhost"
+  }, 
+  "origin": "172.17.0.1", 
+  "url": "http://localhost/get"
+}
+</v>
+      </c>
+    </row>
     <row r="17" spans="2:14" x14ac:dyDescent="0.4">
       <c r="C17" t="s">
         <v>101</v>
@@ -7829,7 +7833,7 @@
         <v xml:space="preserve">Connection: keep-alive_x000D_
 Access-Control-Allow-Origin: *_x000D_
 Access-Control-Allow-Credentials: true_x000D_
-Date: Thu, 23 Sep 2021 11:55:16 GMT_x000D_
+Date: Thu, 23 Sep 2021 13:11:14 GMT_x000D_
 Server: gunicorn/19.9.0_x000D_
 </v>
       </c>
@@ -7845,7 +7849,7 @@
       </c>
       <c r="C23" t="str" cm="1">
         <f t="array" ref="C23">_xll.ExLibris.WebAPIs.OpenWebSocket(,B23)</f>
-        <v>ExLibris.Core.WebAPIs.WebAPI:FCC762F8-ED4C-4FF8-95E7-CC84EAA249C2</v>
+        <v>ExLibris.Core.WebAPIs.WebAPI:C4D65701-6655-47E4-8DE3-5312399F01C0</v>
       </c>
       <c r="M23" t="s">
         <v>131</v>
@@ -7862,9 +7866,9 @@
       <c r="C24" t="s">
         <v>124</v>
       </c>
-      <c r="D24" t="str">
-        <f>$C$2&amp;"get"</f>
-        <v>http://localhost:80/get</v>
+      <c r="D24" t="str" cm="1">
+        <f t="array" ref="D24">_xll.ExLibris.WebAPIs.BuildUri($C$2&amp;"get",M23:N25)</f>
+        <v>http://localhost:80/get?key0=WebAPI2&amp;key1.int=1&amp;key1.string=value1</v>
       </c>
       <c r="M24" t="s">
         <v>132</v>
@@ -7878,8 +7882,8 @@
         <v>122</v>
       </c>
       <c r="D25" t="str" cm="1">
-        <f t="array" ref="D25">_xll.ExLibris.WebAPIs.WebAPIGet(C23,D24,M23:N25,C23)</f>
-        <v>ExLibris.Core.WebAPIs.Response:500713E6-4D22-42AD-A816-74BBB81DC4F2</v>
+        <f t="array" ref="D25">_xll.ExLibris.WebAPIs.WebAPIGet(C23,D24,C23)</f>
+        <v>ExLibris.Core.WebAPIs.Response:B6B8BE68-E323-4FE4-923E-7D8A039C22DF</v>
       </c>
       <c r="M25" t="s">
         <v>133</v>
@@ -7927,7 +7931,7 @@
         <v xml:space="preserve">Connection: keep-alive_x000D_
 Access-Control-Allow-Origin: *_x000D_
 Access-Control-Allow-Credentials: true_x000D_
-Date: Thu, 23 Sep 2021 11:55:16 GMT_x000D_
+Date: Thu, 23 Sep 2021 13:11:53 GMT_x000D_
 Server: gunicorn/19.9.0_x000D_
 </v>
       </c>
@@ -7938,7 +7942,7 @@
       </c>
       <c r="N33" t="str" cm="1">
         <f t="array" ref="N33">_xll.ExLibris.Json.CreateJsonObject(M34:N36)</f>
-        <v>JsonObject:13CCC74E-74C5-4157-A96C-DFA57E671E4C</v>
+        <v>JsonObject:2A58B27D-675E-4034-AD59-7B57491E800E</v>
       </c>
     </row>
     <row r="34" spans="2:14" x14ac:dyDescent="0.4">
@@ -7947,7 +7951,7 @@
       </c>
       <c r="C34" t="str" cm="1">
         <f t="array" ref="C34">_xll.ExLibris.WebAPIs.OpenWebSocket(,B34)</f>
-        <v>ExLibris.Core.WebAPIs.WebAPI:17739D45-05ED-4F05-A16C-4AD8D03E4741</v>
+        <v>ExLibris.Core.WebAPIs.WebAPI:A77102A5-4736-4B3B-9940-2D0470A6736C</v>
       </c>
       <c r="M34" t="s">
         <v>131</v>
@@ -7964,9 +7968,9 @@
       <c r="C35" t="s">
         <v>124</v>
       </c>
-      <c r="D35" t="str">
-        <f>$C$2&amp;"get"</f>
-        <v>http://localhost:80/get</v>
+      <c r="D35" t="str" cm="1">
+        <f t="array" ref="D35">_xll.ExLibris.WebAPIs.BuildUri($C$2&amp;"get",N33)</f>
+        <v>http://localhost:80/get?key0=WebAPI3&amp;key1.int=1&amp;key1.string=value1</v>
       </c>
       <c r="M35" t="s">
         <v>132</v>
@@ -7980,8 +7984,8 @@
         <v>122</v>
       </c>
       <c r="D36" t="str" cm="1">
-        <f t="array" ref="D36">_xll.ExLibris.WebAPIs.WebAPIGet(C34,D35,N33,C34)</f>
-        <v>ExLibris.Core.WebAPIs.Response:F145C1E6-F6D5-4239-83E0-3C1B0B662900</v>
+        <f t="array" ref="D36">_xll.ExLibris.WebAPIs.WebAPIGet(C34,D35,C34)</f>
+        <v>ExLibris.Core.WebAPIs.Response:371B0CC6-5ACB-4BFA-8A99-58422DEE2F75</v>
       </c>
       <c r="M36" t="s">
         <v>133</v>
@@ -8029,7 +8033,7 @@
         <v xml:space="preserve">Connection: keep-alive_x000D_
 Access-Control-Allow-Origin: *_x000D_
 Access-Control-Allow-Credentials: true_x000D_
-Date: Thu, 23 Sep 2021 11:55:16 GMT_x000D_
+Date: Thu, 23 Sep 2021 13:12:27 GMT_x000D_
 Server: gunicorn/19.9.0_x000D_
 </v>
       </c>
@@ -8040,7 +8044,7 @@
       </c>
       <c r="N47" t="str" cm="1">
         <f t="array" ref="N47">_xll.ExLibris.Json.CreateJsonObject(M48:N50)</f>
-        <v>JsonObject:D560D4B9-72BB-4BFE-826E-E16F2B223BFE</v>
+        <v>JsonObject:E062079A-A1E7-4DA8-9EE1-3BE1C4EE4FD6</v>
       </c>
     </row>
     <row r="48" spans="2:14" x14ac:dyDescent="0.4">
@@ -8049,7 +8053,7 @@
       </c>
       <c r="C48" t="str" cm="1">
         <f t="array" ref="C48">_xll.ExLibris.WebAPIs.OpenWebSocket(D49,B48)</f>
-        <v>ExLibris.Core.WebAPIs.WebAPI:6D1287A6-84BB-4684-B03F-030C69FB9A82</v>
+        <v>ExLibris.Core.WebAPIs.WebAPI:34E5C5F6-BCA3-4834-AB59-8A3501EB8FD7</v>
       </c>
       <c r="M48" t="s">
         <v>131</v>
@@ -8066,9 +8070,9 @@
       <c r="C49" t="s">
         <v>124</v>
       </c>
-      <c r="D49" t="str">
-        <f>$C$2&amp;"get"</f>
-        <v>http://localhost:80/get</v>
+      <c r="D49" t="str" cm="1">
+        <f t="array" ref="D49">_xll.ExLibris.WebAPIs.BuildUri($C$2&amp;"get",N47)</f>
+        <v>http://localhost:80/get?key0=WebAPI4&amp;key1.int=1&amp;key1.string=value1</v>
       </c>
       <c r="M49" t="s">
         <v>132</v>
@@ -8082,8 +8086,8 @@
         <v>122</v>
       </c>
       <c r="D50" t="str" cm="1">
-        <f t="array" ref="D50">_xll.ExLibris.WebAPIs.WebAPIGet(C48,,N47,C48)</f>
-        <v>ExLibris.Core.WebAPIs.Response:05290E9E-A98E-473E-AD23-5B88BC02A0CF</v>
+        <f t="array" ref="D50">_xll.ExLibris.WebAPIs.WebAPIGet(C48,,C48)</f>
+        <v>ExLibris.Core.WebAPIs.Response:0185E35B-6629-4388-8ECE-0D96F025740F</v>
       </c>
       <c r="M50" t="s">
         <v>133</v>

</xml_diff>

<commit_message>
snapshot of registered objects
</commit_message>
<xml_diff>
--- a/ExLibris/test_excel/exlibris_test.xlsx
+++ b/ExLibris/test_excel/exlibris_test.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\mugen\git\ex-libris\ExLibris\test_excel\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{39F7EBFE-6F85-4584-AD95-D2DC17508E93}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{82B7008D-AD48-47A1-918F-440DC17078EE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" activeTab="4" xr2:uid="{705CD0B7-27A9-4291-85BD-6034C0FEE3E4}"/>
   </bookViews>
@@ -42,7 +42,7 @@
 </file>
 
 <file path=xl/metadata.xml><?xml version="1.0" encoding="utf-8"?>
-<metadata xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xda="http://schemas.microsoft.com/office/spreadsheetml/2017/dynamicarray">
+<metadata xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xlrd="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata" xmlns:xda="http://schemas.microsoft.com/office/spreadsheetml/2017/dynamicarray">
   <metadataTypes count="1">
     <metadataType name="XLDAPR" minSupportedVersion="120000" copy="1" pasteAll="1" pasteValues="1" merge="1" splitFirst="1" rowColShift="1" clearFormats="1" clearComments="1" assign="1" coerce="1" cellMeta="1"/>
   </metadataTypes>
@@ -720,849 +720,771 @@
 <file path=xl/volatileDependencies.xml><?xml version="1.0" encoding="utf-8"?>
 <volTypes xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <volType type="realTimeData">
-    <main first="rtdsrv.e3b84d0ff4f547568288363859b2eb81">
-      <tp>
-        <v>2</v>
-        <stp/>
-        <stp>c24a2331-6a3e-4180-b913-237d3934e5f4</stp>
+    <main first="rtdsrv.6a4f66642a534248940068305b780441">
+      <tp>
+        <v>2</v>
+        <stp/>
+        <stp>ee7e3b1d-b980-4c43-94a0-2f4c23320ea0</stp>
+        <tr r="F6" s="4"/>
+      </tp>
+    </main>
+    <main first="rtdsrv.6a4f66642a534248940068305b780441">
+      <tp>
+        <v>2</v>
+        <stp/>
+        <stp>aee70c88-7b43-4e86-b50c-1de45ebe2146</stp>
+        <tr r="D39" s="5"/>
+      </tp>
+    </main>
+    <main first="rtdsrv.6a4f66642a534248940068305b780441">
+      <tp>
+        <v>2</v>
+        <stp/>
+        <stp>356fb4d0-c41c-4bf3-8bfe-87849cbbfdad</stp>
+        <tr r="G25" s="1"/>
+      </tp>
+      <tp>
+        <v>2</v>
+        <stp/>
+        <stp>bea44935-05e7-41e6-84a4-185cb26d7708</stp>
+        <tr r="D29" s="5"/>
+      </tp>
+    </main>
+    <main first="rtdsrv.6a4f66642a534248940068305b780441">
+      <tp>
+        <v>2</v>
+        <stp/>
+        <stp>a09e3ca5-544f-4b23-9f1d-e3c820913adc</stp>
+        <tr r="G55" s="4"/>
+      </tp>
+    </main>
+    <main first="rtdsrv.6a4f66642a534248940068305b780441">
+      <tp>
+        <v>2</v>
+        <stp/>
+        <stp>c14eb4e9-314f-4b26-8219-62da8347a640</stp>
+        <tr r="G47" s="1"/>
+      </tp>
+      <tp>
+        <v>2</v>
+        <stp/>
+        <stp>b0ecbcb4-8cef-49b3-8e4b-a129baa4593e</stp>
+        <tr r="G26" s="4"/>
+      </tp>
+      <tp>
+        <v>2</v>
+        <stp/>
+        <stp>58312168-87db-4d5b-b83b-7f3420a6d3d0</stp>
+        <tr r="G52" s="4"/>
+      </tp>
+      <tp>
+        <v>2</v>
+        <stp/>
+        <stp>aff3d7e7-c70a-4f62-ab87-11a8398d7520</stp>
+        <tr r="G21" s="4"/>
+      </tp>
+      <tp>
+        <v>2</v>
+        <stp/>
+        <stp>825a1c03-be1e-4d71-86c6-5c81a1722643</stp>
+        <tr r="I38" s="4"/>
+      </tp>
+      <tp>
+        <v>2</v>
+        <stp/>
+        <stp>bdc63699-4c53-4e31-9737-74e11493caa8</stp>
+        <tr r="G46" s="4"/>
+      </tp>
+    </main>
+    <main first="rtdsrv.6a4f66642a534248940068305b780441">
+      <tp>
+        <v>2</v>
+        <stp/>
+        <stp>6afd3141-ee5b-43c1-bf51-3bff8054ffa7</stp>
+        <tr r="G38" s="1"/>
+      </tp>
+      <tp>
+        <v>2</v>
+        <stp/>
+        <stp>0a553bbb-4599-4f34-a35e-33df3c3e7cfa</stp>
+        <tr r="G22" s="4"/>
+      </tp>
+      <tp>
+        <v>2</v>
+        <stp/>
+        <stp>78690c09-4258-4169-8f3b-d6c7caff27ee</stp>
+        <tr r="G35" s="4"/>
+      </tp>
+      <tp>
+        <v>2</v>
+        <stp/>
+        <stp>0d9abeba-a503-4e82-a5e7-4d0147b46a76</stp>
+        <tr r="P19" s="1"/>
+      </tp>
+    </main>
+    <main first="rtdsrv.6a4f66642a534248940068305b780441">
+      <tp>
+        <v>2</v>
+        <stp/>
+        <stp>f42171cc-149d-4171-b20f-172db7b4e104</stp>
+        <tr r="G31" s="1"/>
+      </tp>
+      <tp>
+        <v>2</v>
+        <stp/>
+        <stp>4f048712-2cb9-492f-b6b3-563f64905a90</stp>
         <tr r="G53" s="4"/>
       </tp>
-      <tp>
-        <v>2</v>
-        <stp/>
-        <stp>2c8a3f35-1cc3-414d-b950-288d1a1ab5a1</stp>
-        <tr r="G37" s="1"/>
-      </tp>
     </main>
-    <main first="rtdsrv.e3b84d0ff4f547568288363859b2eb81">
-      <tp>
-        <v>2</v>
-        <stp/>
-        <stp>64e9d8d9-541d-46d3-a223-05858754f394</stp>
+    <main first="rtdsrv.6a4f66642a534248940068305b780441">
+      <tp>
+        <v>2</v>
+        <stp/>
+        <stp>930fab66-8cc1-4219-8201-1b327ea13ca9</stp>
+        <tr r="G41" s="1"/>
+      </tp>
+    </main>
+    <main first="rtdsrv.6a4f66642a534248940068305b780441">
+      <tp>
+        <v>2</v>
+        <stp/>
+        <stp>baa96e19-1f5b-461c-9dd3-b66af36153cf</stp>
+        <tr r="G40" s="4"/>
+      </tp>
+    </main>
+    <main first="rtdsrv.6a4f66642a534248940068305b780441">
+      <tp>
+        <v>2</v>
+        <stp/>
+        <stp>99a8cad4-8a9f-4973-a109-e1a6cff5c007</stp>
+        <tr r="E17" s="3"/>
+      </tp>
+    </main>
+    <main first="rtdsrv.6a4f66642a534248940068305b780441">
+      <tp>
+        <v>2</v>
+        <stp/>
+        <stp>0a69e6ed-e9ee-4e2c-9964-326132c77d59</stp>
+        <tr r="G32" s="1"/>
+      </tp>
+    </main>
+    <main first="rtdsrv.6a4f66642a534248940068305b780441">
+      <tp>
+        <v>2</v>
+        <stp/>
+        <stp>caf852fc-611d-4896-b0ff-f61f02537083</stp>
+        <tr r="G30" s="1"/>
+      </tp>
+      <tp>
+        <v>2</v>
+        <stp/>
+        <stp>6a5b1d68-7037-47e5-85a6-82dede849044</stp>
         <tr r="G40" s="1"/>
       </tp>
+      <tp>
+        <v>2</v>
+        <stp/>
+        <stp>3dc85ad6-f283-4299-b8a9-1531a841d786</stp>
+        <tr r="B5" s="5"/>
+      </tp>
+      <tp>
+        <v>2</v>
+        <stp/>
+        <stp>6ff4e3ec-d8dc-4dba-b34b-46b020417c89</stp>
+        <tr r="G36" s="4"/>
+      </tp>
+      <tp>
+        <v>2</v>
+        <stp/>
+        <stp>7d3b00cf-d5d9-4bbf-95bd-7e8fef0ba641</stp>
+        <tr r="G51" s="1"/>
+      </tp>
+      <tp>
+        <v>2</v>
+        <stp/>
+        <stp>7d622a0e-5091-4c7d-ac30-cd361b3e0adb</stp>
+        <tr r="G42" s="4"/>
+      </tp>
+      <tp>
+        <v>2</v>
+        <stp/>
+        <stp>9dd625e1-8881-43d5-8352-c9d59b70f22a</stp>
+        <tr r="H5" s="5"/>
+      </tp>
+      <tp>
+        <v>2</v>
+        <stp/>
+        <stp>1d90a2c6-0b6b-47df-a6d4-0134fb2377bf</stp>
+        <tr r="B2" s="6"/>
+      </tp>
+      <tp>
+        <v>2</v>
+        <stp/>
+        <stp>c96f1af6-b6d4-4c98-a20f-fc54cdbf65db</stp>
+        <tr r="G21" s="1"/>
+      </tp>
     </main>
-    <main first="rtdsrv.e3b84d0ff4f547568288363859b2eb81">
-      <tp>
-        <v>2</v>
-        <stp/>
-        <stp>60ba10a9-1d97-44ca-a05b-179289c0cbe0</stp>
-        <tr r="G31" s="1"/>
-      </tp>
-      <tp>
-        <v>2</v>
-        <stp/>
-        <stp>23a89722-6aa6-4107-9f61-cf178d53e8ac</stp>
-        <tr r="D34" s="5"/>
-      </tp>
-      <tp>
-        <v>2</v>
-        <stp/>
-        <stp>12d6de75-b075-4884-b7c8-9d47889a4755</stp>
+    <main first="rtdsrv.6a4f66642a534248940068305b780441">
+      <tp>
+        <v>2</v>
+        <stp/>
+        <stp>8b1b99ae-eb98-456b-a812-bb833750b7aa</stp>
+        <tr r="G27" s="4"/>
+      </tp>
+      <tp>
+        <v>2</v>
+        <stp/>
+        <stp>a2b66973-557e-4c8d-896e-1cc5e9188847</stp>
+        <tr r="G50" s="1"/>
+      </tp>
+      <tp>
+        <v>2</v>
+        <stp/>
+        <stp>a5df89d6-57c5-407d-adcc-92783d71cf7c</stp>
+        <tr r="G25" s="4"/>
+      </tp>
+      <tp>
+        <v>2</v>
+        <stp/>
+        <stp>4d853aec-2444-4b24-ad6c-b54d869248ef</stp>
+        <tr r="G39" s="1"/>
+      </tp>
+    </main>
+    <main first="rtdsrv.6a4f66642a534248940068305b780441">
+      <tp>
+        <v>2</v>
+        <stp/>
+        <stp>2d00a897-5188-4fc4-bd37-138a5a9b92eb</stp>
+        <tr r="P29" s="1"/>
+      </tp>
+      <tp>
+        <v>2</v>
+        <stp/>
+        <stp>a7d6cf37-91ff-4bc1-afad-e2b40431809c</stp>
+        <tr r="G19" s="4"/>
+      </tp>
+    </main>
+    <main first="rtdsrv.6a4f66642a534248940068305b780441">
+      <tp>
+        <v>2</v>
+        <stp/>
+        <stp>7127a5cb-bc1b-43e8-8821-be143771008c</stp>
+        <tr r="G47" s="4"/>
+      </tp>
+      <tp>
+        <v>2</v>
+        <stp/>
+        <stp>7bd768f8-54a1-4213-a054-fbd93b879d7b</stp>
+        <tr r="G54" s="4"/>
+      </tp>
+    </main>
+    <main first="rtdsrv.6a4f66642a534248940068305b780441">
+      <tp>
+        <v>2</v>
+        <stp/>
+        <stp>a075f88a-691a-438c-ab30-8689aa3fb4b2</stp>
+        <tr r="G56" s="4"/>
+      </tp>
+    </main>
+    <main first="rtdsrv.6a4f66642a534248940068305b780441">
+      <tp>
+        <v>2</v>
+        <stp/>
+        <stp>85791df0-6fd6-40cb-a6e5-47c1c8106c43</stp>
+        <tr r="G45" s="4"/>
+      </tp>
+    </main>
+    <main first="rtdsrv.6a4f66642a534248940068305b780441">
+      <tp>
+        <v>2</v>
+        <stp/>
+        <stp>5faed0c3-f5ad-44f1-9e65-9b4538be8aee</stp>
         <tr r="E4" s="3"/>
       </tp>
+      <tp>
+        <v>2</v>
+        <stp/>
+        <stp>439a9a35-9b3f-4326-b4e2-5b3977d77a66</stp>
+        <tr r="G49" s="1"/>
+      </tp>
+      <tp>
+        <v>1</v>
+        <stp/>
+        <stp>4386d816-1731-4bdf-a370-c29a26272de7</stp>
+        <tr r="E20" s="3"/>
+      </tp>
     </main>
-    <main first="rtdsrv.e3b84d0ff4f547568288363859b2eb81">
-      <tp>
-        <v>1</v>
-        <stp/>
-        <stp>a478182a-ff84-4d0c-8442-86877c6a8a2d</stp>
-        <tr r="H6" s="2"/>
+    <main first="rtdsrv.6a4f66642a534248940068305b780441">
+      <tp>
+        <v>2</v>
+        <stp/>
+        <stp>d84ad232-20cd-4f55-a042-9bfaef311699</stp>
+        <tr r="G22" s="1"/>
       </tp>
     </main>
-    <main first="rtdsrv.e3b84d0ff4f547568288363859b2eb81">
-      <tp>
-        <v>1</v>
-        <stp/>
-        <stp>b06e52c4-088f-4cf3-9689-53ec07b4449c</stp>
-        <tr r="E20" s="3"/>
-      </tp>
-      <tp>
-        <v>2</v>
-        <stp/>
-        <stp>0d80d83e-d2c7-4537-bb88-e78510ba6910</stp>
-        <tr r="G46" s="4"/>
+    <main first="rtdsrv.6a4f66642a534248940068305b780441">
+      <tp>
+        <v>2</v>
+        <stp/>
+        <stp>46d02a19-c413-4424-a1cd-19791439de81</stp>
+        <tr r="G27" s="1"/>
       </tp>
     </main>
-    <main first="rtdsrv.e3b84d0ff4f547568288363859b2eb81">
-      <tp>
-        <v>2</v>
-        <stp/>
-        <stp>eddabb02-4015-40c4-af83-2a0d55633b36</stp>
-        <tr r="G54" s="1"/>
+    <main first="rtdsrv.6a4f66642a534248940068305b780441">
+      <tp>
+        <v>2</v>
+        <stp/>
+        <stp>48151ec3-673f-48af-ba12-a21767a5e3b1</stp>
+        <tr r="G53" s="1"/>
+      </tp>
+      <tp>
+        <v>2</v>
+        <stp/>
+        <stp>12bbd3de-3a05-4f62-899b-0544cdb7bb4f</stp>
+        <tr r="G50" s="4"/>
+      </tp>
+      <tp>
+        <v>2</v>
+        <stp/>
+        <stp>701034f6-d378-4a68-a638-a56cfc95c782</stp>
+        <tr r="F1" s="4"/>
+      </tp>
+      <tp>
+        <v>2</v>
+        <stp/>
+        <stp>42105dc3-e174-42eb-8669-8a8a95706994</stp>
+        <tr r="F1" s="1"/>
       </tp>
     </main>
-    <main first="rtdsrv.e3b84d0ff4f547568288363859b2eb81">
-      <tp>
-        <v>2</v>
-        <stp/>
-        <stp>4e1959d1-c2f1-41e3-9bbc-1656529b3ba8</stp>
-        <tr r="D39" s="5"/>
-      </tp>
-      <tp>
-        <v>2</v>
-        <stp/>
-        <stp>d6331de3-06e9-4ff1-ac93-423ddc3df0d7</stp>
-        <tr r="G20" s="1"/>
+    <main first="rtdsrv.6a4f66642a534248940068305b780441">
+      <tp>
+        <v>2</v>
+        <stp/>
+        <stp>c091a543-3a9d-495f-9212-c967fbc9a027</stp>
+        <tr r="G42" s="1"/>
       </tp>
     </main>
-    <main first="rtdsrv.e3b84d0ff4f547568288363859b2eb81">
-      <tp>
-        <v>2</v>
-        <stp/>
-        <stp>8e828674-d74e-40d6-b6f6-d8c3aed8c1c9</stp>
-        <tr r="I28" s="4"/>
+    <main first="rtdsrv.6a4f66642a534248940068305b780441">
+      <tp>
+        <v>2</v>
+        <stp/>
+        <stp>a0756196-8176-4d0e-9255-9c620159e2c5</stp>
+        <tr r="G20" s="4"/>
       </tp>
     </main>
-    <main first="rtdsrv.e3b84d0ff4f547568288363859b2eb81">
-      <tp>
-        <v>2</v>
-        <stp/>
-        <stp>782764ef-fc63-41b5-bcee-03744ae25b38</stp>
-        <tr r="G39" s="4"/>
+    <main first="rtdsrv.6a4f66642a534248940068305b780441">
+      <tp>
+        <v>2</v>
+        <stp/>
+        <stp>418f86d6-eceb-48a9-bae4-a46127758430</stp>
+        <tr r="G43" s="4"/>
+      </tp>
+      <tp>
+        <v>2</v>
+        <stp/>
+        <stp>652a7953-6ec0-46bc-b3d4-ac116ab3569d</stp>
+        <tr r="G36" s="1"/>
+      </tp>
+      <tp>
+        <v>2</v>
+        <stp/>
+        <stp>b12bcf4c-5e65-4445-aa4e-e19e88d8bce2</stp>
+        <tr r="G44" s="4"/>
+      </tp>
+      <tp>
+        <v>2</v>
+        <stp/>
+        <stp>ae7f0fea-7cac-4b7c-93bc-b81237d782e7</stp>
+        <tr r="I28" s="1"/>
+      </tp>
+      <tp>
+        <v>2</v>
+        <stp/>
+        <stp>d8ea4c75-8416-43c7-a03a-c33e5e8fa9c1</stp>
+        <tr r="G56" s="1"/>
       </tp>
     </main>
-    <main first="rtdsrv.e3b84d0ff4f547568288363859b2eb81">
-      <tp>
-        <v>2</v>
-        <stp/>
-        <stp>8e71947f-282d-4275-9b59-8be1e958724d</stp>
-        <tr r="G51" s="4"/>
-      </tp>
-      <tp>
-        <v>2</v>
-        <stp/>
-        <stp>5f6fd2f8-16d1-4c2a-998b-8a0845ba8b37</stp>
-        <tr r="G49" s="1"/>
-      </tp>
-    </main>
-    <main first="rtdsrv.e3b84d0ff4f547568288363859b2eb81">
-      <tp>
-        <v>2</v>
-        <stp/>
-        <stp>d7efc1c8-21b5-4d89-950b-8d72e7f1ddf7</stp>
-        <tr r="G26" s="4"/>
-      </tp>
-    </main>
-    <main first="rtdsrv.e3b84d0ff4f547568288363859b2eb81">
-      <tp>
-        <v>2</v>
-        <stp/>
-        <stp>0770a83b-c8db-4355-b530-b66c93ddbe64</stp>
-        <tr r="G54" s="4"/>
-      </tp>
-    </main>
-    <main first="rtdsrv.e3b84d0ff4f547568288363859b2eb81">
-      <tp>
-        <v>2</v>
-        <stp/>
-        <stp>96b58b05-c181-41c0-b78c-9f7f86798b5b</stp>
-        <tr r="D44" s="5"/>
-      </tp>
-    </main>
-    <main first="rtdsrv.e3b84d0ff4f547568288363859b2eb81">
-      <tp>
-        <v>2</v>
-        <stp/>
-        <stp>9d00bb7a-8565-4a78-b13f-cbc788cf9b12</stp>
-        <tr r="G55" s="4"/>
-      </tp>
-    </main>
-    <main first="rtdsrv.e3b84d0ff4f547568288363859b2eb81">
-      <tp>
-        <v>2</v>
-        <stp/>
-        <stp>38065485-c5b8-40c2-9623-8435d3956d0c</stp>
-        <tr r="G35" s="1"/>
-      </tp>
-      <tp>
-        <v>2</v>
-        <stp/>
-        <stp>14d281b2-a561-4c14-959b-26fbd5cb4fb1</stp>
-        <tr r="G52" s="4"/>
-      </tp>
-    </main>
-    <main first="rtdsrv.e3b84d0ff4f547568288363859b2eb81">
-      <tp>
-        <v>2</v>
-        <stp/>
-        <stp>86015f1c-6fad-45f8-89e1-7f47266d8dae</stp>
-        <tr r="G26" s="1"/>
-      </tp>
-    </main>
-    <main first="rtdsrv.e3b84d0ff4f547568288363859b2eb81">
-      <tp>
-        <v>2</v>
-        <stp/>
-        <stp>448233f1-754e-4141-8e10-3875f11816ce</stp>
-        <tr r="G38" s="4"/>
-      </tp>
-    </main>
-    <main first="rtdsrv.e3b84d0ff4f547568288363859b2eb81">
-      <tp>
-        <v>2</v>
-        <stp/>
-        <stp>4c8cdf9c-7b48-4a98-ab2c-9efda4589f53</stp>
-        <tr r="G45" s="1"/>
-      </tp>
-      <tp>
-        <v>2</v>
-        <stp/>
-        <stp>d8acd443-b62d-49cd-9b4f-7bc5c151eb2d</stp>
-        <tr r="G22" s="4"/>
-      </tp>
-    </main>
-    <main first="rtdsrv.e3b84d0ff4f547568288363859b2eb81">
-      <tp>
-        <v>2</v>
-        <stp/>
-        <stp>467ffe5a-d420-4a83-a165-b07ec897e5ae</stp>
-        <tr r="F6" s="1"/>
-      </tp>
-    </main>
-    <main first="rtdsrv.e3b84d0ff4f547568288363859b2eb81">
-      <tp>
-        <v>2</v>
-        <stp/>
-        <stp>ef1ab567-8def-4d6a-8434-c7fd4d0b1def</stp>
-        <tr r="G38" s="1"/>
-      </tp>
-    </main>
-    <main first="rtdsrv.e3b84d0ff4f547568288363859b2eb81">
-      <tp>
-        <v>2</v>
-        <stp/>
-        <stp>fae96250-15fc-457a-be96-a85c6235f1e3</stp>
-        <tr r="G41" s="4"/>
-      </tp>
-    </main>
-    <main first="rtdsrv.e3b84d0ff4f547568288363859b2eb81">
-      <tp>
-        <v>2</v>
-        <stp/>
-        <stp>dbc577b3-e80c-42a5-b4ae-adb8516ca078</stp>
-        <tr r="G44" s="1"/>
-      </tp>
-      <tp>
-        <v>2</v>
-        <stp/>
-        <stp>a634d33d-6f09-47bf-8e7f-befc274e5165</stp>
-        <tr r="D29" s="5"/>
-      </tp>
-    </main>
-    <main first="rtdsrv.e3b84d0ff4f547568288363859b2eb81">
-      <tp>
-        <v>2</v>
-        <stp/>
-        <stp>81ea4ef0-4d90-4ff7-82ec-ea730ecf86a5</stp>
-        <tr r="G19" s="4"/>
-      </tp>
-    </main>
-    <main first="rtdsrv.e3b84d0ff4f547568288363859b2eb81">
-      <tp>
-        <v>2</v>
-        <stp/>
-        <stp>d2d284db-e95d-40a4-81d5-dacc0a6393f8</stp>
-        <tr r="G34" s="4"/>
-      </tp>
-    </main>
-    <main first="rtdsrv.e3b84d0ff4f547568288363859b2eb81">
-      <tp>
-        <v>2</v>
-        <stp/>
-        <stp>1334892e-c562-4c7b-8dc9-6208b959bcef</stp>
-        <tr r="E19" s="3"/>
-      </tp>
-      <tp>
-        <v>2</v>
-        <stp/>
-        <stp>bb9a7cad-bad0-41af-bab4-441625c7ef33</stp>
-        <tr r="G35" s="4"/>
-      </tp>
-    </main>
-    <main first="rtdsrv.e3b84d0ff4f547568288363859b2eb81">
-      <tp>
-        <v>2</v>
-        <stp/>
-        <stp>72769766-4f27-45bc-9164-806555646cb4</stp>
-        <tr r="G23" s="1"/>
-      </tp>
-    </main>
-    <main first="rtdsrv.e3b84d0ff4f547568288363859b2eb81">
-      <tp>
-        <v>2</v>
-        <stp/>
-        <stp>0563962a-e893-4760-9512-c7155e69970d</stp>
-        <tr r="G22" s="1"/>
-      </tp>
-    </main>
-    <main first="rtdsrv.e3b84d0ff4f547568288363859b2eb81">
-      <tp>
-        <v>2</v>
-        <stp/>
-        <stp>9c21e1f9-59e1-4b87-b02b-214002da1c9e</stp>
-        <tr r="G20" s="4"/>
-      </tp>
-    </main>
-    <main first="rtdsrv.e3b84d0ff4f547568288363859b2eb81">
-      <tp>
-        <v>2</v>
-        <stp/>
-        <stp>f11c90bf-79a6-40ed-882c-800e2e0937c5</stp>
-        <tr r="G24" s="1"/>
-      </tp>
-    </main>
-    <main first="rtdsrv.e3b84d0ff4f547568288363859b2eb81">
-      <tp>
-        <v>2</v>
-        <stp/>
-        <stp>cd4aaf54-6385-48b2-8b66-4b3b1f55913c</stp>
-        <tr r="G32" s="1"/>
-      </tp>
-    </main>
-    <main first="rtdsrv.e3b84d0ff4f547568288363859b2eb81">
-      <tp>
-        <v>2</v>
-        <stp/>
-        <stp>17e213ba-5ec6-4086-9129-fa4da3065bfb</stp>
-        <tr r="G40" s="4"/>
-      </tp>
-    </main>
-    <main first="rtdsrv.e3b84d0ff4f547568288363859b2eb81">
-      <tp>
-        <v>2</v>
-        <stp/>
-        <stp>d2fcf694-483e-4234-ad07-21dbf9198827</stp>
-        <tr r="I42" s="4"/>
-      </tp>
-    </main>
-    <main first="rtdsrv.e3b84d0ff4f547568288363859b2eb81">
-      <tp>
-        <v>2</v>
-        <stp/>
-        <stp>15a0fcdb-770c-4a03-80ca-d2e2aa704f9c</stp>
-        <tr r="G24" s="4"/>
-      </tp>
-    </main>
-    <main first="rtdsrv.e3b84d0ff4f547568288363859b2eb81">
-      <tp>
-        <v>2</v>
-        <stp/>
-        <stp>f0e682e2-04c6-44a5-bc5d-47e45d0d2ebf</stp>
-        <tr r="G32" s="4"/>
-      </tp>
-    </main>
-    <main first="rtdsrv.e3b84d0ff4f547568288363859b2eb81">
-      <tp>
-        <v>2</v>
-        <stp/>
-        <stp>7c9a0e78-2a09-444e-a14d-0ddfa42b5109</stp>
-        <tr r="G21" s="1"/>
-      </tp>
-    </main>
-    <main first="rtdsrv.e3b84d0ff4f547568288363859b2eb81">
-      <tp>
-        <v>2</v>
-        <stp/>
-        <stp>c959962e-79b9-41f5-a712-b9534eab0d0d</stp>
-        <tr r="G19" s="1"/>
-      </tp>
-    </main>
-    <main first="rtdsrv.e3b84d0ff4f547568288363859b2eb81">
-      <tp>
-        <v>2</v>
-        <stp/>
-        <stp>74775668-6f67-47ec-8b0f-24b167096c7c</stp>
-        <tr r="F6" s="4"/>
-      </tp>
-      <tp>
-        <v>2</v>
-        <stp/>
-        <stp>3b170a04-9169-4dd5-927f-3bdbb8dfae01</stp>
-        <tr r="G52" s="1"/>
-      </tp>
-    </main>
-    <main first="rtdsrv.e3b84d0ff4f547568288363859b2eb81">
-      <tp>
-        <v>2</v>
-        <stp/>
-        <stp>7955972d-5de8-4f69-aa64-4efb8bff2483</stp>
-        <tr r="G48" s="4"/>
-      </tp>
-      <tp>
-        <v>2</v>
-        <stp/>
-        <stp>6966ef87-230f-4a2a-bf8e-43878511558e</stp>
-        <tr r="G37" s="4"/>
-      </tp>
-    </main>
-    <main first="rtdsrv.e3b84d0ff4f547568288363859b2eb81">
-      <tp>
-        <v>2</v>
-        <stp/>
-        <stp>c20be7f7-7c9c-4895-816b-66a552279376</stp>
-        <tr r="D19" s="5"/>
-      </tp>
-    </main>
-    <main first="rtdsrv.e3b84d0ff4f547568288363859b2eb81">
-      <tp>
-        <v>2</v>
-        <stp/>
-        <stp>7645f762-f62c-4517-9cc9-10cc5aa4fda0</stp>
-        <tr r="B2" s="6"/>
-      </tp>
-    </main>
-    <main first="rtdsrv.e3b84d0ff4f547568288363859b2eb81">
-      <tp>
-        <v>2</v>
-        <stp/>
-        <stp>60a5baee-d7c8-47a8-8757-2edddecd0af6</stp>
-        <tr r="G57" s="4"/>
-      </tp>
-    </main>
-    <main first="rtdsrv.e3b84d0ff4f547568288363859b2eb81">
-      <tp>
-        <v>2</v>
-        <stp/>
-        <stp>a41a02cd-d837-4239-8246-e471ba557c30</stp>
-        <tr r="G47" s="1"/>
-      </tp>
-    </main>
-    <main first="rtdsrv.e3b84d0ff4f547568288363859b2eb81">
-      <tp>
-        <v>2</v>
-        <stp/>
-        <stp>7e2a1044-1480-48be-aa6b-438a7d3cf95b</stp>
-        <tr r="G23" s="4"/>
-      </tp>
-    </main>
-    <main first="rtdsrv.e3b84d0ff4f547568288363859b2eb81">
-      <tp>
-        <v>2</v>
-        <stp/>
-        <stp>36c05d82-6619-4a80-a09e-63b95300041b</stp>
-        <tr r="G30" s="1"/>
-      </tp>
-      <tp>
-        <v>2</v>
-        <stp/>
-        <stp>ae6f8ab1-dda2-4fff-8e97-ce46d5afc7d1</stp>
-        <tr r="G50" s="1"/>
-      </tp>
-    </main>
-    <main first="rtdsrv.e3b84d0ff4f547568288363859b2eb81">
-      <tp>
-        <v>2</v>
-        <stp/>
-        <stp>35cc9dd4-9994-4a25-bc61-8b3697a73f3d</stp>
-        <tr r="D14" s="5"/>
-      </tp>
-      <tp>
-        <v>2</v>
-        <stp/>
-        <stp>bb196fcf-5984-4554-8efb-5a4cecad292b</stp>
-        <tr r="G27" s="4"/>
-      </tp>
-    </main>
-    <main first="rtdsrv.e3b84d0ff4f547568288363859b2eb81">
-      <tp>
-        <v>2</v>
-        <stp/>
-        <stp>115d4b0b-56a0-4734-bf63-8582d8c1c2e7</stp>
-        <tr r="G28" s="4"/>
-      </tp>
-    </main>
-    <main first="rtdsrv.e3b84d0ff4f547568288363859b2eb81">
-      <tp>
-        <v>2</v>
-        <stp/>
-        <stp>2f464534-e7bc-43d6-b88e-8228c5695d42</stp>
-        <tr r="I33" s="4"/>
-      </tp>
-    </main>
-    <main first="rtdsrv.e3b84d0ff4f547568288363859b2eb81">
-      <tp>
-        <v>2</v>
-        <stp/>
-        <stp>9b91be05-82dc-494f-b72e-aeba4fe6738d</stp>
-        <tr r="G28" s="1"/>
-      </tp>
-    </main>
-    <main first="rtdsrv.e3b84d0ff4f547568288363859b2eb81">
-      <tp>
-        <v>2</v>
-        <stp/>
-        <stp>74788970-ff67-49de-b0e2-4ee9c61ccbe7</stp>
-        <tr r="G45" s="4"/>
-      </tp>
-      <tp>
-        <v>2</v>
-        <stp/>
-        <stp>422d7492-2b28-49e6-8a38-565239571d46</stp>
-        <tr r="G43" s="1"/>
-      </tp>
-    </main>
-    <main first="rtdsrv.e3b84d0ff4f547568288363859b2eb81">
-      <tp>
-        <v>2</v>
-        <stp/>
-        <stp>d5ed8957-e9ba-4c3f-a538-311192577bbc</stp>
-        <tr r="G56" s="1"/>
-      </tp>
-      <tp>
-        <v>2</v>
-        <stp/>
-        <stp>48f13015-1560-41b2-8ef6-d2e4d4174666</stp>
-        <tr r="G27" s="1"/>
-      </tp>
-      <tp>
-        <v>2</v>
-        <stp/>
-        <stp>1e3a4e7e-c070-4901-a186-02a15da8ba3c</stp>
-        <tr r="P29" s="1"/>
-      </tp>
-    </main>
-    <main first="rtdsrv.e3b84d0ff4f547568288363859b2eb81">
-      <tp>
-        <v>2</v>
-        <stp/>
-        <stp>553cfe98-bd2d-47f8-bcb5-814defb14b2e</stp>
-        <tr r="I28" s="1"/>
-      </tp>
-    </main>
-    <main first="rtdsrv.e3b84d0ff4f547568288363859b2eb81">
-      <tp>
-        <v>2</v>
-        <stp/>
-        <stp>90b1a822-fc75-4076-afa6-3ad056c3a39c</stp>
-        <tr r="F1" s="4"/>
-      </tp>
-      <tp>
-        <v>2</v>
-        <stp/>
-        <stp>cbd8a8e7-6f94-47be-af43-928c43e51a39</stp>
-        <tr r="G47" s="4"/>
-      </tp>
-      <tp>
-        <v>1</v>
-        <stp/>
-        <stp>ac43b3a7-906b-440f-a32c-e78c43883dd1</stp>
-        <tr r="E7" s="3"/>
-      </tp>
-      <tp>
-        <v>2</v>
-        <stp/>
-        <stp>63316de9-7667-412a-9690-fe617d7f7d30</stp>
-        <tr r="G29" s="4"/>
-      </tp>
-    </main>
-    <main first="rtdsrv.e3b84d0ff4f547568288363859b2eb81">
-      <tp>
-        <v>2</v>
-        <stp/>
-        <stp>2f8caf5e-9864-4e34-8ce1-f4b61e976d50</stp>
+    <main first="rtdsrv.6a4f66642a534248940068305b780441">
+      <tp>
+        <v>2</v>
+        <stp/>
+        <stp>37bbf2cb-d3f7-4680-9d97-c088efffb6e3</stp>
         <tr r="I19" s="4"/>
         <tr r="I32" s="4"/>
       </tp>
     </main>
-    <main first="rtdsrv.e3b84d0ff4f547568288363859b2eb81">
-      <tp>
-        <v>2</v>
-        <stp/>
-        <stp>fe38122f-ab84-41a9-a17b-8ca96d7b6c1f</stp>
-        <tr r="G25" s="4"/>
-      </tp>
-      <tp>
-        <v>2</v>
-        <stp/>
-        <stp>f10d6a3f-e5ff-4dca-983a-ffc768d30e8e</stp>
+    <main first="rtdsrv.6a4f66642a534248940068305b780441">
+      <tp>
+        <v>2</v>
+        <stp/>
+        <stp>8c0ce693-dbdc-41ef-8463-6b9d4ce437ca</stp>
+        <tr r="G29" s="4"/>
+      </tp>
+      <tp>
+        <v>2</v>
+        <stp/>
+        <stp>aa0af78b-7497-4460-9803-ce06654e0fa3</stp>
+        <tr r="G33" s="4"/>
+      </tp>
+    </main>
+    <main first="rtdsrv.6a4f66642a534248940068305b780441">
+      <tp>
+        <v>2</v>
+        <stp/>
+        <stp>50ecc000-3a59-4e7d-b0a7-ff1c7d8e9c99</stp>
+        <tr r="I42" s="4"/>
+      </tp>
+      <tp>
+        <v>2</v>
+        <stp/>
+        <stp>0dbdc069-3591-4d83-9ce8-1524e693befb</stp>
+        <tr r="D14" s="5"/>
+      </tp>
+      <tp>
+        <v>2</v>
+        <stp/>
+        <stp>d30a6524-c921-4a69-a570-cf6eec05494f</stp>
+        <tr r="C6" s="6"/>
+      </tp>
+    </main>
+    <main first="rtdsrv.6a4f66642a534248940068305b780441">
+      <tp>
+        <v>2</v>
+        <stp/>
+        <stp>3c6b425e-2e69-4d21-ac76-9d1dc3526d79</stp>
+        <tr r="G48" s="1"/>
+      </tp>
+      <tp>
+        <v>2</v>
+        <stp/>
+        <stp>4265b603-3e48-4c6e-a9f5-2a37468ad543</stp>
+        <tr r="C10" s="6"/>
+      </tp>
+    </main>
+    <main first="rtdsrv.6a4f66642a534248940068305b780441">
+      <tp>
+        <v>2</v>
+        <stp/>
+        <stp>9018c59e-e47b-4cac-840f-394a8dee98f2</stp>
+        <tr r="G26" s="1"/>
+      </tp>
+      <tp>
+        <v>2</v>
+        <stp/>
+        <stp>34cdae90-53b2-4310-a551-f6ceedf94e35</stp>
+        <tr r="D49" s="5"/>
+      </tp>
+      <tp>
+        <v>2</v>
+        <stp/>
+        <stp>59548fcc-663c-4748-8664-2151eb510bf0</stp>
+        <tr r="G35" s="1"/>
+      </tp>
+    </main>
+    <main first="rtdsrv.6a4f66642a534248940068305b780441">
+      <tp>
+        <v>2</v>
+        <stp/>
+        <stp>73733752-e6a3-4c65-84cd-229067a16d38</stp>
+        <tr r="G45" s="1"/>
+      </tp>
+    </main>
+    <main first="rtdsrv.6a4f66642a534248940068305b780441">
+      <tp>
+        <v>2</v>
+        <stp/>
+        <stp>885d432b-a6fa-4421-8c9f-30c6f081340b</stp>
+        <tr r="I28" s="4"/>
+      </tp>
+      <tp>
+        <v>2</v>
+        <stp/>
+        <stp>47111983-8c9b-4c45-bef4-f39524f4f7bd</stp>
+        <tr r="D19" s="5"/>
+      </tp>
+    </main>
+    <main first="rtdsrv.6a4f66642a534248940068305b780441">
+      <tp>
+        <v>-2</v>
+        <stp/>
+        <stp>88c4c9ce-32be-49d0-bb1d-10a04459cb98</stp>
+        <tr r="D29" s="5"/>
+      </tp>
+      <tp>
+        <v>2</v>
+        <stp/>
+        <stp>1601aaa6-8147-442c-84da-9b69effa6802</stp>
+        <tr r="G23" s="4"/>
+      </tp>
+      <tp>
+        <v>2</v>
+        <stp/>
+        <stp>a371ad28-0ff6-4e8d-b4e5-8cbd0e7de4b9</stp>
+        <tr r="G39" s="4"/>
+      </tp>
+      <tp>
+        <v>2</v>
+        <stp/>
+        <stp>10654141-9620-477e-a19d-0d406a56554c</stp>
+        <tr r="G19" s="1"/>
+      </tp>
+      <tp>
+        <v>2</v>
+        <stp/>
+        <stp>5adbdd05-3a3a-4e85-8872-61b42f02f701</stp>
+        <tr r="G34" s="4"/>
+      </tp>
+      <tp>
+        <v>2</v>
+        <stp/>
+        <stp>983e71d1-9638-497c-9358-97283f14cc7c</stp>
+        <tr r="G32" s="4"/>
+      </tp>
+      <tp>
+        <v>1</v>
+        <stp/>
+        <stp>ad7e8775-765c-415f-94ca-b6b46791d49d</stp>
+        <tr r="E7" s="3"/>
+      </tp>
+      <tp>
+        <v>2</v>
+        <stp/>
+        <stp>13a0607d-6418-4340-8f39-ef519f5d4bb8</stp>
+        <tr r="G51" s="4"/>
+      </tp>
+      <tp>
+        <v>2</v>
+        <stp/>
+        <stp>62f1a499-a3b3-4e51-96ef-de554f18dd5d</stp>
+        <tr r="G28" s="1"/>
+      </tp>
+      <tp>
+        <v>2</v>
+        <stp/>
+        <stp>15ed5ab8-0aa8-4e7f-b9f9-27681fe3ea11</stp>
+        <tr r="G38" s="4"/>
+      </tp>
+    </main>
+    <main first="rtdsrv.6a4f66642a534248940068305b780441">
+      <tp>
+        <v>2</v>
+        <stp/>
+        <stp>30ba0bad-7fae-485d-becc-3a35a3845ce6</stp>
+        <tr r="G43" s="1"/>
+      </tp>
+      <tp>
+        <v>2</v>
+        <stp/>
+        <stp>6c62cb0a-6aaa-4614-a0f3-ec638c91461f</stp>
+        <tr r="G33" s="1"/>
+      </tp>
+      <tp>
+        <v>2</v>
+        <stp/>
+        <stp>a0fb582e-ea55-4eaa-bf80-ce0d7dcf1f97</stp>
+        <tr r="G37" s="4"/>
+      </tp>
+    </main>
+    <main first="rtdsrv.6a4f66642a534248940068305b780441">
+      <tp>
+        <v>2</v>
+        <stp/>
+        <stp>65a1974c-0a6a-42ab-b575-b44ba05d4045</stp>
+        <tr r="G41" s="4"/>
+      </tp>
+      <tp>
+        <v>2</v>
+        <stp/>
+        <stp>89fbd583-7d1d-4995-b372-beeff8b5574f</stp>
+        <tr r="E19" s="3"/>
+      </tp>
+    </main>
+    <main first="rtdsrv.6a4f66642a534248940068305b780441">
+      <tp>
+        <v>2</v>
+        <stp/>
+        <stp>af0240fc-27b9-41eb-823f-6459a2543a35</stp>
+        <tr r="G23" s="1"/>
+      </tp>
+    </main>
+    <main first="rtdsrv.6a4f66642a534248940068305b780441">
+      <tp>
+        <v>2</v>
+        <stp/>
+        <stp>8dc2dc53-9e2f-4ab6-a09c-87f33605aaa1</stp>
+        <tr r="G20" s="1"/>
+      </tp>
+      <tp>
+        <v>2</v>
+        <stp/>
+        <stp>2fbf7492-55b5-424c-9bf8-5ac67f6eb48e</stp>
+        <tr r="G57" s="1"/>
+      </tp>
+      <tp>
+        <v>2</v>
+        <stp/>
+        <stp>90799d96-14a3-41ed-8719-f74e5c90853e</stp>
+        <tr r="I33" s="4"/>
+      </tp>
+      <tp>
+        <v>2</v>
+        <stp/>
+        <stp>cb891a64-c0df-4996-9df3-8df487a3925e</stp>
+        <tr r="D24" s="5"/>
+      </tp>
+      <tp>
+        <v>2</v>
+        <stp/>
+        <stp>5d562e93-9309-45af-88fe-38b63a06306c</stp>
+        <tr r="G24" s="1"/>
+      </tp>
+    </main>
+    <main first="rtdsrv.6a4f66642a534248940068305b780441">
+      <tp>
+        <v>2</v>
+        <stp/>
+        <stp>0657eee8-fa37-4bc2-aec3-b74ec6d425f4</stp>
+        <tr r="F6" s="1"/>
+      </tp>
+      <tp>
+        <v>2</v>
+        <stp/>
+        <stp>ff14cee9-e81f-48e9-b969-cbd04905cb82</stp>
+        <tr r="G48" s="4"/>
+      </tp>
+      <tp>
+        <v>2</v>
+        <stp/>
+        <stp>aa8070e6-683d-48c1-b741-1a81cdc3a776</stp>
+        <tr r="D44" s="5"/>
+      </tp>
+    </main>
+    <main first="rtdsrv.6a4f66642a534248940068305b780441">
+      <tp>
+        <v>2</v>
+        <stp/>
+        <stp>b3ae7651-168c-4d41-95bb-7c3acb91d8a9</stp>
+        <tr r="G57" s="4"/>
+      </tp>
+      <tp>
+        <v>2</v>
+        <stp/>
+        <stp>35d84d75-61cf-46f3-b9f1-01b07dc989bd</stp>
+        <tr r="D34" s="5"/>
+      </tp>
+    </main>
+    <main first="rtdsrv.6a4f66642a534248940068305b780441">
+      <tp>
+        <v>2</v>
+        <stp/>
+        <stp>b888e74a-d059-45fe-b7e5-eafceecb1138</stp>
+        <tr r="G24" s="4"/>
+      </tp>
+    </main>
+    <main first="rtdsrv.6a4f66642a534248940068305b780441">
+      <tp>
+        <v>2</v>
+        <stp/>
+        <stp>35be3459-21bb-449e-b25e-161e30fdc870</stp>
+        <tr r="E6" s="3"/>
+      </tp>
+      <tp>
+        <v>2</v>
+        <stp/>
+        <stp>d7a7ea9c-e555-4bdd-befe-6ccb79085690</stp>
+        <tr r="G30" s="4"/>
+      </tp>
+    </main>
+    <main first="rtdsrv.6a4f66642a534248940068305b780441">
+      <tp>
+        <v>2</v>
+        <stp/>
+        <stp>206ba408-e454-41d9-8be1-7dff7677d2b8</stp>
         <tr r="G55" s="1"/>
       </tp>
       <tp>
         <v>2</v>
         <stp/>
-        <stp>2d768c9e-e6c7-45f7-addf-4c9d354178eb</stp>
-        <tr r="F1" s="1"/>
-      </tp>
-      <tp>
-        <v>2</v>
-        <stp/>
-        <stp>e814c67c-fdb9-4db4-b4fd-b0bfa3610fcd</stp>
-        <tr r="G41" s="1"/>
+        <stp>24065492-7305-4ad9-95ef-b3b6ca924d7b</stp>
+        <tr r="G52" s="1"/>
       </tp>
     </main>
-    <main first="rtdsrv.e3b84d0ff4f547568288363859b2eb81">
-      <tp>
-        <v>2</v>
-        <stp/>
-        <stp>594ef50b-a8c0-4fc4-8064-960a91b047b7</stp>
-        <tr r="I38" s="4"/>
+    <main first="rtdsrv.6a4f66642a534248940068305b780441">
+      <tp>
+        <v>2</v>
+        <stp/>
+        <stp>7874d624-fbda-417d-833f-431501894ace</stp>
+        <tr r="G29" s="1"/>
       </tp>
     </main>
-    <main first="rtdsrv.e3b84d0ff4f547568288363859b2eb81">
-      <tp>
-        <v>2</v>
-        <stp/>
-        <stp>93c0c697-ed4e-469b-8bc5-25ce78b2b3c2</stp>
-        <tr r="C6" s="6"/>
+    <main first="rtdsrv.6a4f66642a534248940068305b780441">
+      <tp>
+        <v>2</v>
+        <stp/>
+        <stp>c17aa4e2-09cd-4418-805e-05e30cf71227</stp>
+        <tr r="G54" s="1"/>
+      </tp>
+      <tp>
+        <v>2</v>
+        <stp/>
+        <stp>90df8329-56d8-48fe-8f67-b97cb66e917f</stp>
+        <tr r="G44" s="1"/>
       </tp>
     </main>
-    <main first="rtdsrv.e3b84d0ff4f547568288363859b2eb81">
-      <tp>
-        <v>-2</v>
-        <stp/>
-        <stp>2407616c-6ca6-4c2b-9050-8af4ab946917</stp>
-        <tr r="D29" s="5"/>
+    <main first="rtdsrv.6a4f66642a534248940068305b780441">
+      <tp>
+        <v>2</v>
+        <stp/>
+        <stp>dad7c63d-175e-4339-9c52-a78dbcf33d43</stp>
+        <tr r="G28" s="4"/>
+      </tp>
+      <tp>
+        <v>2</v>
+        <stp/>
+        <stp>203f4b23-8178-40c1-8c29-3b3ba20dbc15</stp>
+        <tr r="I19" s="1"/>
       </tp>
     </main>
-    <main first="rtdsrv.e3b84d0ff4f547568288363859b2eb81">
-      <tp>
-        <v>2</v>
-        <stp/>
-        <stp>8645952f-0425-4c4c-a290-96503087a1e5</stp>
+    <main first="rtdsrv.6a4f66642a534248940068305b780441">
+      <tp>
+        <v>2</v>
+        <stp/>
+        <stp>b672a17a-16a7-4868-9509-6b71fc542fda</stp>
+        <tr r="G37" s="1"/>
+      </tp>
+      <tp>
+        <v>2</v>
+        <stp/>
+        <stp>2d7e06e2-1707-4fc5-8291-74f14a920cc3</stp>
+        <tr r="C2" s="2"/>
+      </tp>
+    </main>
+    <main first="rtdsrv.6a4f66642a534248940068305b780441">
+      <tp>
+        <v>2</v>
+        <stp/>
+        <stp>fa27ec2f-bb1f-424c-bd09-9db0593bf73b</stp>
+        <tr r="G49" s="4"/>
+      </tp>
+    </main>
+    <main first="rtdsrv.6a4f66642a534248940068305b780441">
+      <tp>
+        <v>2</v>
+        <stp/>
+        <stp>22f105d6-b6ea-4ccf-a7c1-9bba0b02e88c</stp>
         <tr r="G31" s="4"/>
       </tp>
       <tp>
         <v>2</v>
         <stp/>
-        <stp>5dd91fc6-1122-4429-bca9-d9024baf4ab8</stp>
-        <tr r="G33" s="4"/>
-      </tp>
-      <tp>
-        <v>2</v>
-        <stp/>
-        <stp>a5c5938e-918c-4733-a9a3-3624c3cf5913</stp>
-        <tr r="D24" s="5"/>
-      </tp>
-    </main>
-    <main first="rtdsrv.e3b84d0ff4f547568288363859b2eb81">
-      <tp>
-        <v>2</v>
-        <stp/>
-        <stp>17466afe-b35d-4bd9-bb7a-1909f3189aba</stp>
-        <tr r="G53" s="1"/>
-      </tp>
-      <tp>
-        <v>2</v>
-        <stp/>
-        <stp>2f6a3e7b-3a10-4f77-8750-ebe22bd0ec96</stp>
-        <tr r="G36" s="1"/>
-      </tp>
-      <tp>
-        <v>2</v>
-        <stp/>
-        <stp>0badfa8f-92c6-44c9-be33-c85fe8219a50</stp>
-        <tr r="G50" s="4"/>
-      </tp>
-    </main>
-    <main first="rtdsrv.e3b84d0ff4f547568288363859b2eb81">
-      <tp>
-        <v>2</v>
-        <stp/>
-        <stp>17f69531-7014-4132-b95f-d15e4eaf262b</stp>
-        <tr r="I19" s="1"/>
-      </tp>
-    </main>
-    <main first="rtdsrv.e3b84d0ff4f547568288363859b2eb81">
-      <tp>
-        <v>2</v>
-        <stp/>
-        <stp>3869ee95-7d22-434a-a7e4-2348a5303837</stp>
-        <tr r="G42" s="1"/>
-      </tp>
-    </main>
-    <main first="rtdsrv.e3b84d0ff4f547568288363859b2eb81">
-      <tp>
-        <v>2</v>
-        <stp/>
-        <stp>cbf15a28-a299-4cc5-8b21-4a21c4d67c0c</stp>
-        <tr r="G39" s="1"/>
-      </tp>
-    </main>
-    <main first="rtdsrv.e3b84d0ff4f547568288363859b2eb81">
-      <tp>
-        <v>2</v>
-        <stp/>
-        <stp>54f26ab6-79b8-485a-a8e1-f5e9558d45b1</stp>
-        <tr r="G36" s="4"/>
-      </tp>
-      <tp>
-        <v>2</v>
-        <stp/>
-        <stp>9781b416-22f5-472e-b3fe-2406bb2027a4</stp>
-        <tr r="G49" s="4"/>
-      </tp>
-    </main>
-    <main first="rtdsrv.e3b84d0ff4f547568288363859b2eb81">
-      <tp>
-        <v>2</v>
-        <stp/>
-        <stp>0c67571b-03c8-4330-9e17-1a87ad84b387</stp>
-        <tr r="C2" s="2"/>
-      </tp>
-    </main>
-    <main first="rtdsrv.e3b84d0ff4f547568288363859b2eb81">
-      <tp>
-        <v>2</v>
-        <stp/>
-        <stp>680bcefb-4dba-4d4d-ab29-3d2381320903</stp>
-        <tr r="G33" s="1"/>
-      </tp>
-    </main>
-    <main first="rtdsrv.e3b84d0ff4f547568288363859b2eb81">
-      <tp>
-        <v>2</v>
-        <stp/>
-        <stp>6904654c-4313-47e9-8056-7d4dd4e8e727</stp>
-        <tr r="G30" s="4"/>
-      </tp>
-    </main>
-    <main first="rtdsrv.e3b84d0ff4f547568288363859b2eb81">
-      <tp>
-        <v>2</v>
-        <stp/>
-        <stp>25f4164c-62fd-4b4b-a32f-d8be574508e2</stp>
-        <tr r="G51" s="1"/>
-      </tp>
-    </main>
-    <main first="rtdsrv.e3b84d0ff4f547568288363859b2eb81">
-      <tp>
-        <v>2</v>
-        <stp/>
-        <stp>56d0f7c1-bb6c-4d3f-8fb0-9e27e3807cfd</stp>
-        <tr r="G44" s="4"/>
-      </tp>
-    </main>
-    <main first="rtdsrv.e3b84d0ff4f547568288363859b2eb81">
-      <tp>
-        <v>2</v>
-        <stp/>
-        <stp>49cbca3f-8bbb-4dac-8eb2-970665bfd134</stp>
-        <tr r="G57" s="1"/>
-      </tp>
-    </main>
-    <main first="rtdsrv.e3b84d0ff4f547568288363859b2eb81">
-      <tp>
-        <v>2</v>
-        <stp/>
-        <stp>41d028b6-5f77-4ce0-8a11-07752a4f190d</stp>
-        <tr r="C10" s="6"/>
-      </tp>
-    </main>
-    <main first="rtdsrv.e3b84d0ff4f547568288363859b2eb81">
-      <tp>
-        <v>2</v>
-        <stp/>
-        <stp>233fed79-dab5-4ca2-94b3-6edad0ed7cea</stp>
-        <tr r="E6" s="3"/>
-      </tp>
-    </main>
-    <main first="rtdsrv.e3b84d0ff4f547568288363859b2eb81">
-      <tp>
-        <v>2</v>
-        <stp/>
-        <stp>226672b7-0b1a-4b92-bdb8-c638e0dcc3ff</stp>
-        <tr r="G29" s="1"/>
-      </tp>
-    </main>
-    <main first="rtdsrv.e3b84d0ff4f547568288363859b2eb81">
-      <tp>
-        <v>2</v>
-        <stp/>
-        <stp>5cd4ec68-a996-499c-995b-6bf7a21012d7</stp>
+        <stp>7e01c20d-9646-425e-af6c-16acf2609a36</stp>
+        <tr r="G46" s="1"/>
+      </tp>
+      <tp>
+        <v>2</v>
+        <stp/>
+        <stp>5c30f848-f178-406d-a170-1b9a3de1d0dc</stp>
         <tr r="G34" s="1"/>
-      </tp>
-    </main>
-    <main first="rtdsrv.e3b84d0ff4f547568288363859b2eb81">
-      <tp>
-        <v>2</v>
-        <stp/>
-        <stp>e6ec6272-f199-4aca-94a1-7458723d10d0</stp>
-        <tr r="B5" s="5"/>
-      </tp>
-    </main>
-    <main first="rtdsrv.e3b84d0ff4f547568288363859b2eb81">
-      <tp>
-        <v>2</v>
-        <stp/>
-        <stp>03d23fe4-42f7-48e7-9d14-709d364ec5e1</stp>
-        <tr r="G25" s="1"/>
-      </tp>
-    </main>
-    <main first="rtdsrv.e3b84d0ff4f547568288363859b2eb81">
-      <tp>
-        <v>2</v>
-        <stp/>
-        <stp>a5ec7aae-b051-4c35-a2ab-36ee3b859baa</stp>
-        <tr r="G42" s="4"/>
-      </tp>
-    </main>
-    <main first="rtdsrv.e3b84d0ff4f547568288363859b2eb81">
-      <tp>
-        <v>2</v>
-        <stp/>
-        <stp>5bf2e12d-f9c2-4836-bc2e-a4a55c7481f2</stp>
-        <tr r="E17" s="3"/>
-      </tp>
-    </main>
-    <main first="rtdsrv.e3b84d0ff4f547568288363859b2eb81">
-      <tp>
-        <v>2</v>
-        <stp/>
-        <stp>98ac2d89-5152-40c4-86d5-98866fd700c6</stp>
-        <tr r="G43" s="4"/>
-      </tp>
-    </main>
-    <main first="rtdsrv.e3b84d0ff4f547568288363859b2eb81">
-      <tp>
-        <v>2</v>
-        <stp/>
-        <stp>1bbdfb1b-762b-4f94-b974-8c3a8681c654</stp>
-        <tr r="G46" s="1"/>
-      </tp>
-    </main>
-    <main first="rtdsrv.e3b84d0ff4f547568288363859b2eb81">
-      <tp>
-        <v>2</v>
-        <stp/>
-        <stp>8ec697d3-81bc-4268-90a9-0d31a6985717</stp>
-        <tr r="G56" s="4"/>
-      </tp>
-    </main>
-    <main first="rtdsrv.e3b84d0ff4f547568288363859b2eb81">
-      <tp>
-        <v>2</v>
-        <stp/>
-        <stp>972f91f6-038b-4adc-8b2c-7a42ef77a665</stp>
-        <tr r="G21" s="4"/>
-      </tp>
-      <tp>
-        <v>2</v>
-        <stp/>
-        <stp>87efaec5-0d6c-4adb-9941-44191ae9d754</stp>
-        <tr r="D49" s="5"/>
-      </tp>
-      <tp>
-        <v>2</v>
-        <stp/>
-        <stp>02c08c1c-0f61-4842-9813-bf062455ef09</stp>
-        <tr r="P19" s="1"/>
-      </tp>
-    </main>
-    <main first="rtdsrv.e3b84d0ff4f547568288363859b2eb81">
-      <tp>
-        <v>2</v>
-        <stp/>
-        <stp>7f0f8a02-5e35-428d-b998-2450193644bb</stp>
-        <tr r="G48" s="1"/>
-      </tp>
-    </main>
-    <main first="rtdsrv.e3b84d0ff4f547568288363859b2eb81">
-      <tp>
-        <v>2</v>
-        <stp/>
-        <stp>546f1c05-7064-4761-8f32-53c061488621</stp>
-        <tr r="H5" s="5"/>
       </tp>
     </main>
   </volType>
@@ -1896,11 +1818,11 @@
       </c>
       <c r="F1" t="str" cm="1">
         <f t="array" ref="F1">_xll.ExLibris.Json.CreateJsonObject(E3:F6)</f>
-        <v>JsonObject:FF9A2D33-E1E5-47FC-91D1-7E27784C049A</v>
+        <v>JsonObject:4B303AE7-F025-4345-904C-CA73B1BDC7AF</v>
       </c>
       <c r="K1" t="str">
         <f>EXLIBRIS_CONFIGURATION</f>
-        <v>ExLibris.Core.ExLibrisConfiguration:0D0AC951-C4F0-4C41-BE04-012B566C8134</v>
+        <v>ExLibris.Core.ExLibrisConfiguration:C0F780BA-4B29-4017-A1D0-C6FF1EFE3B1D</v>
       </c>
     </row>
     <row r="2" spans="2:28" x14ac:dyDescent="0.4">
@@ -1970,7 +1892,7 @@
       </c>
       <c r="F6" t="str" cm="1">
         <f t="array" ref="F6">_xll.ExLibris.Json.CreateJsonArray(E8:J14)</f>
-        <v>JsonObject:648AAEC4-A20C-42B9-8CF0-0F53899756B7</v>
+        <v>JsonObject:E52497FB-79B9-4902-87C0-31307B818C5B</v>
       </c>
       <c r="L6" t="s">
         <v>68</v>
@@ -1986,7 +1908,7 @@
       </c>
       <c r="C7" s="6">
         <f>COUNTIF(AR19:AS21,FALSE)</f>
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="L7" t="s">
         <v>74</v>
@@ -2001,7 +1923,7 @@
       </c>
       <c r="C8" s="6">
         <f>COUNTIF(AR30:AS65,FALSE)</f>
-        <v>72</v>
+        <v>0</v>
       </c>
       <c r="E8" t="s">
         <v>1</v>
@@ -2209,11 +2131,14 @@
       </c>
       <c r="I19" t="str" cm="1">
         <f t="array" ref="I19">_xll.ExLibris.Json.GetJsonValue(F1,E6)</f>
-        <v>JsonObject:4D34F86F-E10E-452C-BF61-6C5775E63352</v>
+        <v>JsonObject:A0C5C8B2-4DD8-40E9-952C-9A88D3C0CF51</v>
       </c>
       <c r="P19" t="str" cm="1">
-        <f t="array" ref="P19">_xll.ExLibris.Json.GetJsonKeyValues(F1,,3)</f>
-        <v>JsonObject:FA028524-4421-47B8-B9EC-8A797E52830E</v>
+        <f t="array" ref="P19:Q27">_xll.ExLibris.Json.GetJsonKeyValues(F1,,3)</f>
+        <v>trade_code</v>
+      </c>
+      <c r="Q19" t="str">
+        <v>money_00001</v>
       </c>
       <c r="S19" t="s">
         <v>14</v>
@@ -2244,11 +2169,11 @@
       </c>
       <c r="AR19" t="b">
         <f t="shared" ref="AR19:AS21" si="7">P19=AD19</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AS19" t="b">
         <f t="shared" si="7"/>
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="20" spans="5:45" x14ac:dyDescent="0.4">
@@ -2281,6 +2206,12 @@
       <c r="N20" t="str">
         <v>fixed_rate</v>
       </c>
+      <c r="P20" t="str">
+        <v>couter_party</v>
+      </c>
+      <c r="Q20" t="str">
+        <v>CP00001</v>
+      </c>
       <c r="S20" t="s">
         <v>18</v>
       </c>
@@ -2352,11 +2283,11 @@
       </c>
       <c r="AR20" t="b">
         <f t="shared" si="7"/>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AS20" t="b">
         <f t="shared" si="7"/>
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="21" spans="5:45" x14ac:dyDescent="0.4">
@@ -2388,6 +2319,12 @@
       <c r="N21">
         <v>1E-3</v>
       </c>
+      <c r="P21" t="str">
+        <v>fixed_leg.pay_or_recieve</v>
+      </c>
+      <c r="Q21" t="str">
+        <v>Receive</v>
+      </c>
       <c r="S21" t="s">
         <v>22</v>
       </c>
@@ -2459,11 +2396,11 @@
       </c>
       <c r="AR21" t="b">
         <f t="shared" si="7"/>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AS21" t="b">
         <f t="shared" si="7"/>
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="22" spans="5:45" x14ac:dyDescent="0.4">
@@ -2495,6 +2432,12 @@
       <c r="N22">
         <v>1E-3</v>
       </c>
+      <c r="P22" t="str">
+        <v>fixed_leg.cashflows.[0]</v>
+      </c>
+      <c r="Q22" t="str">
+        <v>JsonObject:5CA95493-BCDD-42E1-95DA-1A797A349F8C</v>
+      </c>
       <c r="S22" t="s">
         <v>32</v>
       </c>
@@ -2588,6 +2531,12 @@
       <c r="N23">
         <v>1E-3</v>
       </c>
+      <c r="P23" t="str">
+        <v>fixed_leg.cashflows.[1]</v>
+      </c>
+      <c r="Q23" t="str">
+        <v>JsonObject:1DF73157-EE0E-4BC2-BC0E-884CF0EFC5AD</v>
+      </c>
       <c r="S23" t="s">
         <v>33</v>
       </c>
@@ -2681,6 +2630,12 @@
       <c r="N24">
         <v>1E-3</v>
       </c>
+      <c r="P24" t="str">
+        <v>fixed_leg.cashflows.[2]</v>
+      </c>
+      <c r="Q24" t="str">
+        <v>JsonObject:303467F1-E599-48BD-919D-6BB66306CA35</v>
+      </c>
       <c r="S24" t="s">
         <v>34</v>
       </c>
@@ -2774,6 +2729,12 @@
       <c r="N25">
         <v>1E-3</v>
       </c>
+      <c r="P25" t="str">
+        <v>fixed_leg.cashflows.[3]</v>
+      </c>
+      <c r="Q25" t="str">
+        <v>JsonObject:FC669D92-DED6-4649-9AA5-0813D186BE88</v>
+      </c>
       <c r="S25" t="s">
         <v>35</v>
       </c>
@@ -2867,6 +2828,12 @@
       <c r="N26">
         <v>1E-3</v>
       </c>
+      <c r="P26" t="str">
+        <v>fixed_leg.cashflows.[4]</v>
+      </c>
+      <c r="Q26" t="str">
+        <v>JsonObject:417C0C38-32FD-4229-A077-E96256864B15</v>
+      </c>
       <c r="S26" t="s">
         <v>36</v>
       </c>
@@ -2942,6 +2909,12 @@
         <f t="array" ref="G27">_xll.ExLibris.Json.GetJsonValue($F$1,E27)</f>
         <v>1E-3</v>
       </c>
+      <c r="P27" t="str">
+        <v>fixed_leg.cashflows.[5]</v>
+      </c>
+      <c r="Q27" t="str">
+        <v>JsonObject:AE1581A1-B8AA-4CA7-BDCC-3FB5364EDF93</v>
+      </c>
       <c r="S27" t="s">
         <v>37</v>
       </c>
@@ -2977,7 +2950,7 @@
       </c>
       <c r="I28" t="str" cm="1">
         <f t="array" ref="I28">_xll.ExLibris.Json.GetJsonValue(I19,"[2]")</f>
-        <v>JsonObject:699010F5-A0E8-473A-A5E9-0FB770CBE636</v>
+        <v>JsonObject:2513CF49-C6B8-48EC-8145-FD7C8DE2416F</v>
       </c>
       <c r="S28" t="s">
         <v>38</v>
@@ -3033,7 +3006,7 @@
       </c>
       <c r="P29" t="str" cm="1">
         <f t="array" ref="P29">_xll.ExLibris.Json.CreateJsonObject(P22:Q27)</f>
-        <v>JsonObject:3773B381-F04F-4EE7-A556-3D87B8740A4F</v>
+        <v>JsonObject:244CEA73-398D-4F01-9E8D-73CDF9F9F730</v>
       </c>
       <c r="S29" t="s">
         <v>39</v>
@@ -3128,12 +3101,12 @@
       <c r="N30">
         <v>1E-3</v>
       </c>
-      <c r="P30" cm="1">
-        <f t="array" ref="P30:Q30">_xll.ExLibris.Json.GetJsonKeyValues(P29)</f>
-        <v>0</v>
+      <c r="P30" t="str" cm="1">
+        <f t="array" ref="P30:Q65">_xll.ExLibris.Json.GetJsonKeyValues(P29)</f>
+        <v>fixed_leg.cashflows.[0].payment _date</v>
       </c>
       <c r="Q30">
-        <v>0</v>
+        <v>44632</v>
       </c>
       <c r="S30" t="s">
         <v>40</v>
@@ -3206,11 +3179,11 @@
       </c>
       <c r="AR30" t="b">
         <f t="shared" ref="AR30:AR64" si="10">P30=AD30</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AS30" t="b">
         <f t="shared" ref="AS30:AS64" si="11">Q30=AE30</f>
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="31" spans="5:45" x14ac:dyDescent="0.4">
@@ -3224,6 +3197,12 @@
         <f t="array" ref="G31">_xll.ExLibris.Json.GetJsonValue($F$1,E31)</f>
         <v>ACT/360</v>
       </c>
+      <c r="P31" t="str">
+        <v>fixed_leg.cashflows.[0].start_date</v>
+      </c>
+      <c r="Q31">
+        <v>44452</v>
+      </c>
       <c r="S31" t="s">
         <v>41</v>
       </c>
@@ -3253,11 +3232,11 @@
       </c>
       <c r="AR31" t="b">
         <f t="shared" si="10"/>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AS31" t="b">
         <f t="shared" si="11"/>
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="32" spans="5:45" x14ac:dyDescent="0.4">
@@ -3271,6 +3250,12 @@
         <f t="array" ref="G32">_xll.ExLibris.Json.GetJsonValue($F$1,E32)</f>
         <v>11000000</v>
       </c>
+      <c r="P32" t="str">
+        <v>fixed_leg.cashflows.[0].end_date</v>
+      </c>
+      <c r="Q32">
+        <v>44632</v>
+      </c>
       <c r="S32" t="s">
         <v>42</v>
       </c>
@@ -3300,11 +3285,11 @@
       </c>
       <c r="AR32" t="b">
         <f t="shared" si="10"/>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AS32" t="b">
         <f t="shared" si="11"/>
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="33" spans="5:45" x14ac:dyDescent="0.4">
@@ -3318,6 +3303,12 @@
         <f t="array" ref="G33">_xll.ExLibris.Json.GetJsonValue($F$1,E33)</f>
         <v>1E-3</v>
       </c>
+      <c r="P33" t="str">
+        <v>fixed_leg.cashflows.[0].day_count_type</v>
+      </c>
+      <c r="Q33" t="str">
+        <v>ACT/360</v>
+      </c>
       <c r="S33" t="s">
         <v>43</v>
       </c>
@@ -3347,11 +3338,11 @@
       </c>
       <c r="AR33" t="b">
         <f t="shared" si="10"/>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AS33" t="b">
         <f t="shared" si="11"/>
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="34" spans="5:45" x14ac:dyDescent="0.4">
@@ -3365,6 +3356,12 @@
         <f t="array" ref="G34">_xll.ExLibris.Json.GetJsonValue($F$1,E34)</f>
         <v>44992</v>
       </c>
+      <c r="P34" t="str">
+        <v>fixed_leg.cashflows.[0].amout</v>
+      </c>
+      <c r="Q34">
+        <v>10000000</v>
+      </c>
       <c r="S34" t="s">
         <v>44</v>
       </c>
@@ -3394,11 +3391,11 @@
       </c>
       <c r="AR34" t="b">
         <f t="shared" si="10"/>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AS34" t="b">
         <f t="shared" si="11"/>
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="35" spans="5:45" x14ac:dyDescent="0.4">
@@ -3412,6 +3409,12 @@
         <f t="array" ref="G35">_xll.ExLibris.Json.GetJsonValue($F$1,E35)</f>
         <v>44812</v>
       </c>
+      <c r="P35" t="str">
+        <v>fixed_leg.cashflows.[0].fixed_rate</v>
+      </c>
+      <c r="Q35">
+        <v>1E-3</v>
+      </c>
       <c r="S35" t="s">
         <v>45</v>
       </c>
@@ -3441,11 +3444,11 @@
       </c>
       <c r="AR35" t="b">
         <f t="shared" si="10"/>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AS35" t="b">
         <f t="shared" si="11"/>
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="36" spans="5:45" x14ac:dyDescent="0.4">
@@ -3459,6 +3462,12 @@
         <f t="array" ref="G36">_xll.ExLibris.Json.GetJsonValue($F$1,E36)</f>
         <v>44992</v>
       </c>
+      <c r="P36" t="str">
+        <v>fixed_leg.cashflows.[1].payment _date</v>
+      </c>
+      <c r="Q36">
+        <v>44812</v>
+      </c>
       <c r="S36" t="s">
         <v>46</v>
       </c>
@@ -3488,11 +3497,11 @@
       </c>
       <c r="AR36" t="b">
         <f t="shared" si="10"/>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AS36" t="b">
         <f t="shared" si="11"/>
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="37" spans="5:45" x14ac:dyDescent="0.4">
@@ -3506,6 +3515,12 @@
         <f t="array" ref="G37">_xll.ExLibris.Json.GetJsonValue($F$1,E37)</f>
         <v>ACT/360</v>
       </c>
+      <c r="P37" t="str">
+        <v>fixed_leg.cashflows.[1].start_date</v>
+      </c>
+      <c r="Q37">
+        <v>44632</v>
+      </c>
       <c r="S37" t="s">
         <v>47</v>
       </c>
@@ -3535,11 +3550,11 @@
       </c>
       <c r="AR37" t="b">
         <f t="shared" si="10"/>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AS37" t="b">
         <f t="shared" si="11"/>
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="38" spans="5:45" x14ac:dyDescent="0.4">
@@ -3553,6 +3568,12 @@
         <f t="array" ref="G38">_xll.ExLibris.Json.GetJsonValue($F$1,E38)</f>
         <v>12000000</v>
       </c>
+      <c r="P38" t="str">
+        <v>fixed_leg.cashflows.[1].end_date</v>
+      </c>
+      <c r="Q38">
+        <v>44812</v>
+      </c>
       <c r="S38" t="s">
         <v>48</v>
       </c>
@@ -3582,11 +3603,11 @@
       </c>
       <c r="AR38" t="b">
         <f t="shared" si="10"/>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AS38" t="b">
         <f t="shared" si="11"/>
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="39" spans="5:45" x14ac:dyDescent="0.4">
@@ -3600,6 +3621,12 @@
         <f t="array" ref="G39">_xll.ExLibris.Json.GetJsonValue($F$1,E39)</f>
         <v>1E-3</v>
       </c>
+      <c r="P39" t="str">
+        <v>fixed_leg.cashflows.[1].day_count_type</v>
+      </c>
+      <c r="Q39" t="str">
+        <v>ACT/360</v>
+      </c>
       <c r="S39" t="s">
         <v>49</v>
       </c>
@@ -3629,11 +3656,11 @@
       </c>
       <c r="AR39" t="b">
         <f t="shared" si="10"/>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AS39" t="b">
         <f t="shared" si="11"/>
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="40" spans="5:45" x14ac:dyDescent="0.4">
@@ -3647,6 +3674,12 @@
         <f t="array" ref="G40">_xll.ExLibris.Json.GetJsonValue($F$1,E40)</f>
         <v>45172</v>
       </c>
+      <c r="P40" t="str">
+        <v>fixed_leg.cashflows.[1].amout</v>
+      </c>
+      <c r="Q40">
+        <v>11000000</v>
+      </c>
       <c r="S40" t="s">
         <v>50</v>
       </c>
@@ -3676,11 +3709,11 @@
       </c>
       <c r="AR40" t="b">
         <f t="shared" si="10"/>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AS40" t="b">
         <f t="shared" si="11"/>
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="41" spans="5:45" x14ac:dyDescent="0.4">
@@ -3694,6 +3727,12 @@
         <f t="array" ref="G41">_xll.ExLibris.Json.GetJsonValue($F$1,E41)</f>
         <v>44992</v>
       </c>
+      <c r="P41" t="str">
+        <v>fixed_leg.cashflows.[1].fixed_rate</v>
+      </c>
+      <c r="Q41">
+        <v>1E-3</v>
+      </c>
       <c r="S41" t="s">
         <v>51</v>
       </c>
@@ -3723,11 +3762,11 @@
       </c>
       <c r="AR41" t="b">
         <f t="shared" si="10"/>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AS41" t="b">
         <f t="shared" si="11"/>
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="42" spans="5:45" x14ac:dyDescent="0.4">
@@ -3741,6 +3780,12 @@
         <f t="array" ref="G42">_xll.ExLibris.Json.GetJsonValue($F$1,E42)</f>
         <v>45172</v>
       </c>
+      <c r="P42" t="str">
+        <v>fixed_leg.cashflows.[2].payment _date</v>
+      </c>
+      <c r="Q42">
+        <v>44992</v>
+      </c>
       <c r="S42" t="s">
         <v>52</v>
       </c>
@@ -3770,11 +3815,11 @@
       </c>
       <c r="AR42" t="b">
         <f t="shared" si="10"/>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AS42" t="b">
         <f t="shared" si="11"/>
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="43" spans="5:45" x14ac:dyDescent="0.4">
@@ -3788,6 +3833,12 @@
         <f t="array" ref="G43">_xll.ExLibris.Json.GetJsonValue($F$1,E43)</f>
         <v>ACT/360</v>
       </c>
+      <c r="P43" t="str">
+        <v>fixed_leg.cashflows.[2].start_date</v>
+      </c>
+      <c r="Q43">
+        <v>44812</v>
+      </c>
       <c r="S43" t="s">
         <v>53</v>
       </c>
@@ -3817,11 +3868,11 @@
       </c>
       <c r="AR43" t="b">
         <f t="shared" si="10"/>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AS43" t="b">
         <f t="shared" si="11"/>
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="44" spans="5:45" x14ac:dyDescent="0.4">
@@ -3835,6 +3886,12 @@
         <f t="array" ref="G44">_xll.ExLibris.Json.GetJsonValue($F$1,E44)</f>
         <v>13000000</v>
       </c>
+      <c r="P44" t="str">
+        <v>fixed_leg.cashflows.[2].end_date</v>
+      </c>
+      <c r="Q44">
+        <v>44992</v>
+      </c>
       <c r="S44" t="s">
         <v>54</v>
       </c>
@@ -3864,11 +3921,11 @@
       </c>
       <c r="AR44" t="b">
         <f t="shared" si="10"/>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AS44" t="b">
         <f t="shared" si="11"/>
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="45" spans="5:45" x14ac:dyDescent="0.4">
@@ -3882,6 +3939,12 @@
         <f t="array" ref="G45">_xll.ExLibris.Json.GetJsonValue($F$1,E45)</f>
         <v>1E-3</v>
       </c>
+      <c r="P45" t="str">
+        <v>fixed_leg.cashflows.[2].day_count_type</v>
+      </c>
+      <c r="Q45" t="str">
+        <v>ACT/360</v>
+      </c>
       <c r="S45" t="s">
         <v>55</v>
       </c>
@@ -3911,11 +3974,11 @@
       </c>
       <c r="AR45" t="b">
         <f t="shared" si="10"/>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AS45" t="b">
         <f t="shared" si="11"/>
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="46" spans="5:45" x14ac:dyDescent="0.4">
@@ -3929,6 +3992,12 @@
         <f t="array" ref="G46">_xll.ExLibris.Json.GetJsonValue($F$1,E46)</f>
         <v>45352</v>
       </c>
+      <c r="P46" t="str">
+        <v>fixed_leg.cashflows.[2].amout</v>
+      </c>
+      <c r="Q46">
+        <v>12000000</v>
+      </c>
       <c r="S46" t="s">
         <v>56</v>
       </c>
@@ -3958,11 +4027,11 @@
       </c>
       <c r="AR46" t="b">
         <f t="shared" si="10"/>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AS46" t="b">
         <f t="shared" si="11"/>
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="47" spans="5:45" x14ac:dyDescent="0.4">
@@ -3976,6 +4045,12 @@
         <f t="array" ref="G47">_xll.ExLibris.Json.GetJsonValue($F$1,E47)</f>
         <v>45172</v>
       </c>
+      <c r="P47" t="str">
+        <v>fixed_leg.cashflows.[2].fixed_rate</v>
+      </c>
+      <c r="Q47">
+        <v>1E-3</v>
+      </c>
       <c r="S47" t="s">
         <v>57</v>
       </c>
@@ -4005,11 +4080,11 @@
       </c>
       <c r="AR47" t="b">
         <f t="shared" si="10"/>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AS47" t="b">
         <f t="shared" si="11"/>
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="48" spans="5:45" x14ac:dyDescent="0.4">
@@ -4023,6 +4098,12 @@
         <f t="array" ref="G48">_xll.ExLibris.Json.GetJsonValue($F$1,E48)</f>
         <v>45352</v>
       </c>
+      <c r="P48" t="str">
+        <v>fixed_leg.cashflows.[3].payment _date</v>
+      </c>
+      <c r="Q48">
+        <v>45172</v>
+      </c>
       <c r="S48" t="s">
         <v>58</v>
       </c>
@@ -4052,11 +4133,11 @@
       </c>
       <c r="AR48" t="b">
         <f t="shared" si="10"/>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AS48" t="b">
         <f t="shared" si="11"/>
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="49" spans="5:45" x14ac:dyDescent="0.4">
@@ -4070,6 +4151,12 @@
         <f t="array" ref="G49">_xll.ExLibris.Json.GetJsonValue($F$1,E49)</f>
         <v>ACT/360</v>
       </c>
+      <c r="P49" t="str">
+        <v>fixed_leg.cashflows.[3].start_date</v>
+      </c>
+      <c r="Q49">
+        <v>44992</v>
+      </c>
       <c r="S49" t="s">
         <v>59</v>
       </c>
@@ -4099,11 +4186,11 @@
       </c>
       <c r="AR49" t="b">
         <f t="shared" si="10"/>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AS49" t="b">
         <f t="shared" si="11"/>
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="50" spans="5:45" x14ac:dyDescent="0.4">
@@ -4117,6 +4204,12 @@
         <f t="array" ref="G50">_xll.ExLibris.Json.GetJsonValue($F$1,E50)</f>
         <v>14000000</v>
       </c>
+      <c r="P50" t="str">
+        <v>fixed_leg.cashflows.[3].end_date</v>
+      </c>
+      <c r="Q50">
+        <v>45172</v>
+      </c>
       <c r="S50" t="s">
         <v>60</v>
       </c>
@@ -4146,11 +4239,11 @@
       </c>
       <c r="AR50" t="b">
         <f t="shared" si="10"/>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AS50" t="b">
         <f t="shared" si="11"/>
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="51" spans="5:45" x14ac:dyDescent="0.4">
@@ -4164,6 +4257,12 @@
         <f t="array" ref="G51">_xll.ExLibris.Json.GetJsonValue($F$1,E51)</f>
         <v>1E-3</v>
       </c>
+      <c r="P51" t="str">
+        <v>fixed_leg.cashflows.[3].day_count_type</v>
+      </c>
+      <c r="Q51" t="str">
+        <v>ACT/360</v>
+      </c>
       <c r="S51" t="s">
         <v>61</v>
       </c>
@@ -4193,11 +4292,11 @@
       </c>
       <c r="AR51" t="b">
         <f t="shared" si="10"/>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AS51" t="b">
         <f t="shared" si="11"/>
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="52" spans="5:45" x14ac:dyDescent="0.4">
@@ -4211,6 +4310,12 @@
         <f t="array" ref="G52">_xll.ExLibris.Json.GetJsonValue($F$1,E52)</f>
         <v>45532</v>
       </c>
+      <c r="P52" t="str">
+        <v>fixed_leg.cashflows.[3].amout</v>
+      </c>
+      <c r="Q52">
+        <v>13000000</v>
+      </c>
       <c r="S52" t="s">
         <v>62</v>
       </c>
@@ -4240,11 +4345,11 @@
       </c>
       <c r="AR52" t="b">
         <f t="shared" si="10"/>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AS52" t="b">
         <f t="shared" si="11"/>
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="53" spans="5:45" x14ac:dyDescent="0.4">
@@ -4258,6 +4363,12 @@
         <f t="array" ref="G53">_xll.ExLibris.Json.GetJsonValue($F$1,E53)</f>
         <v>45352</v>
       </c>
+      <c r="P53" t="str">
+        <v>fixed_leg.cashflows.[3].fixed_rate</v>
+      </c>
+      <c r="Q53">
+        <v>1E-3</v>
+      </c>
       <c r="S53" t="s">
         <v>63</v>
       </c>
@@ -4287,11 +4398,11 @@
       </c>
       <c r="AR53" t="b">
         <f t="shared" si="10"/>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AS53" t="b">
         <f t="shared" si="11"/>
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="54" spans="5:45" x14ac:dyDescent="0.4">
@@ -4305,6 +4416,12 @@
         <f t="array" ref="G54">_xll.ExLibris.Json.GetJsonValue($F$1,E54)</f>
         <v>45532</v>
       </c>
+      <c r="P54" t="str">
+        <v>fixed_leg.cashflows.[4].payment _date</v>
+      </c>
+      <c r="Q54">
+        <v>45352</v>
+      </c>
       <c r="S54" t="s">
         <v>64</v>
       </c>
@@ -4334,11 +4451,11 @@
       </c>
       <c r="AR54" t="b">
         <f t="shared" si="10"/>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AS54" t="b">
         <f t="shared" si="11"/>
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="55" spans="5:45" x14ac:dyDescent="0.4">
@@ -4352,6 +4469,12 @@
         <f t="array" ref="G55">_xll.ExLibris.Json.GetJsonValue($F$1,E55)</f>
         <v>ACT/360</v>
       </c>
+      <c r="P55" t="str">
+        <v>fixed_leg.cashflows.[4].start_date</v>
+      </c>
+      <c r="Q55">
+        <v>45172</v>
+      </c>
       <c r="S55" t="s">
         <v>65</v>
       </c>
@@ -4381,11 +4504,11 @@
       </c>
       <c r="AR55" t="b">
         <f t="shared" si="10"/>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AS55" t="b">
         <f t="shared" si="11"/>
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="56" spans="5:45" x14ac:dyDescent="0.4">
@@ -4399,6 +4522,12 @@
         <f t="array" ref="G56">_xll.ExLibris.Json.GetJsonValue($F$1,E56)</f>
         <v>15000000</v>
       </c>
+      <c r="P56" t="str">
+        <v>fixed_leg.cashflows.[4].end_date</v>
+      </c>
+      <c r="Q56">
+        <v>45352</v>
+      </c>
       <c r="S56" t="s">
         <v>66</v>
       </c>
@@ -4428,11 +4557,11 @@
       </c>
       <c r="AR56" t="b">
         <f t="shared" si="10"/>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AS56" t="b">
         <f t="shared" si="11"/>
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="57" spans="5:45" x14ac:dyDescent="0.4">
@@ -4446,6 +4575,12 @@
         <f t="array" ref="G57">_xll.ExLibris.Json.GetJsonValue($F$1,E57)</f>
         <v>1E-3</v>
       </c>
+      <c r="P57" t="str">
+        <v>fixed_leg.cashflows.[4].day_count_type</v>
+      </c>
+      <c r="Q57" t="str">
+        <v>ACT/360</v>
+      </c>
       <c r="S57" t="s">
         <v>67</v>
       </c>
@@ -4475,14 +4610,20 @@
       </c>
       <c r="AR57" t="b">
         <f t="shared" si="10"/>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AS57" t="b">
         <f t="shared" si="11"/>
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="58" spans="5:45" x14ac:dyDescent="0.4">
+      <c r="P58" t="str">
+        <v>fixed_leg.cashflows.[4].amout</v>
+      </c>
+      <c r="Q58">
+        <v>14000000</v>
+      </c>
       <c r="AD58" t="s">
         <v>60</v>
       </c>
@@ -4491,14 +4632,20 @@
       </c>
       <c r="AR58" t="b">
         <f t="shared" si="10"/>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AS58" t="b">
         <f t="shared" si="11"/>
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="59" spans="5:45" x14ac:dyDescent="0.4">
+      <c r="P59" t="str">
+        <v>fixed_leg.cashflows.[4].fixed_rate</v>
+      </c>
+      <c r="Q59">
+        <v>1E-3</v>
+      </c>
       <c r="AD59" t="s">
         <v>61</v>
       </c>
@@ -4507,14 +4654,20 @@
       </c>
       <c r="AR59" t="b">
         <f t="shared" si="10"/>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AS59" t="b">
         <f t="shared" si="11"/>
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="60" spans="5:45" x14ac:dyDescent="0.4">
+      <c r="P60" t="str">
+        <v>fixed_leg.cashflows.[5].payment _date</v>
+      </c>
+      <c r="Q60">
+        <v>45532</v>
+      </c>
       <c r="AD60" t="s">
         <v>62</v>
       </c>
@@ -4523,14 +4676,20 @@
       </c>
       <c r="AR60" t="b">
         <f t="shared" si="10"/>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AS60" t="b">
         <f t="shared" si="11"/>
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="61" spans="5:45" x14ac:dyDescent="0.4">
+      <c r="P61" t="str">
+        <v>fixed_leg.cashflows.[5].start_date</v>
+      </c>
+      <c r="Q61">
+        <v>45352</v>
+      </c>
       <c r="AD61" t="s">
         <v>63</v>
       </c>
@@ -4539,14 +4698,20 @@
       </c>
       <c r="AR61" t="b">
         <f t="shared" si="10"/>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AS61" t="b">
         <f t="shared" si="11"/>
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="62" spans="5:45" x14ac:dyDescent="0.4">
+      <c r="P62" t="str">
+        <v>fixed_leg.cashflows.[5].end_date</v>
+      </c>
+      <c r="Q62">
+        <v>45532</v>
+      </c>
       <c r="AD62" t="s">
         <v>64</v>
       </c>
@@ -4555,14 +4720,20 @@
       </c>
       <c r="AR62" t="b">
         <f t="shared" si="10"/>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AS62" t="b">
         <f t="shared" si="11"/>
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="63" spans="5:45" x14ac:dyDescent="0.4">
+      <c r="P63" t="str">
+        <v>fixed_leg.cashflows.[5].day_count_type</v>
+      </c>
+      <c r="Q63" t="str">
+        <v>ACT/360</v>
+      </c>
       <c r="AD63" t="s">
         <v>65</v>
       </c>
@@ -4571,14 +4742,20 @@
       </c>
       <c r="AR63" t="b">
         <f t="shared" si="10"/>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AS63" t="b">
         <f t="shared" si="11"/>
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="64" spans="5:45" x14ac:dyDescent="0.4">
+      <c r="P64" t="str">
+        <v>fixed_leg.cashflows.[5].amout</v>
+      </c>
+      <c r="Q64">
+        <v>15000000</v>
+      </c>
       <c r="AD64" t="s">
         <v>66</v>
       </c>
@@ -4587,14 +4764,20 @@
       </c>
       <c r="AR64" t="b">
         <f t="shared" si="10"/>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AS64" t="b">
         <f t="shared" si="11"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="65" spans="30:45" x14ac:dyDescent="0.4">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="65" spans="16:45" x14ac:dyDescent="0.4">
+      <c r="P65" t="str">
+        <v>fixed_leg.cashflows.[5].fixed_rate</v>
+      </c>
+      <c r="Q65">
+        <v>1E-3</v>
+      </c>
       <c r="AD65" t="s">
         <v>67</v>
       </c>
@@ -4603,11 +4786,11 @@
       </c>
       <c r="AR65" t="b">
         <f>P65=AD65</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AS65" t="b">
         <f>Q65=AE65</f>
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
   </sheetData>
@@ -4645,11 +4828,11 @@
       </c>
       <c r="F1" t="str" cm="1">
         <f t="array" ref="F1">_xll.ExLibris.Json.CreateJsonObject(E3:F6, EXLIBRIS_CONFIGURATION)</f>
-        <v>JsonObject:EED117AD-EBFD-46BD-A224-D289146B930F</v>
+        <v>JsonObject:B3554340-300F-4248-82C4-19856042659F</v>
       </c>
       <c r="K1" t="str">
         <f>EXLIBRIS_CONFIGURATION</f>
-        <v>ExLibris.Core.ExLibrisConfiguration:0D0AC951-C4F0-4C41-BE04-012B566C8134</v>
+        <v>ExLibris.Core.ExLibrisConfiguration:C0F780BA-4B29-4017-A1D0-C6FF1EFE3B1D</v>
       </c>
     </row>
     <row r="2" spans="2:25" x14ac:dyDescent="0.4">
@@ -4719,7 +4902,7 @@
       </c>
       <c r="F6" t="str" cm="1">
         <f t="array" ref="F6">_xll.ExLibris.Json.CreateJsonArray(E8:J14, EXLIBRIS_CONFIGURATION)</f>
-        <v>JsonObject:290B9A4C-37A4-489C-85C3-3E5EA50711D1</v>
+        <v>JsonObject:9D3CD2B8-A9F9-460A-BE6D-866958829FBA</v>
       </c>
       <c r="L6" t="s">
         <v>68</v>
@@ -4970,7 +5153,7 @@
       </c>
       <c r="I19" t="str" cm="1">
         <f t="array" ref="I19">_xll.ExLibris.Json.GetJsonValue(F1,E6, EXLIBRIS_CONFIGURATION)</f>
-        <v>JsonObject:53B031D7-1A79-4C8D-8898-650D2BB46401</v>
+        <v>JsonObject:48ACA65A-EAC8-4DAD-8832-6C494B258E03</v>
       </c>
       <c r="P19" t="s">
         <v>14</v>
@@ -5692,7 +5875,7 @@
       </c>
       <c r="I28" t="str" cm="1">
         <f t="array" ref="I28">_xll.ExLibris.Json.GetJsonValue(I19,"[2]", EXLIBRIS_CONFIGURATION)</f>
-        <v>JsonObject:DB19D96E-89DA-4165-BE8A-10784DE0B016</v>
+        <v>JsonObject:8967CB41-FC4A-459C-A24C-E016AA6263C7</v>
       </c>
       <c r="P28" t="s">
         <v>38</v>
@@ -5949,7 +6132,7 @@
       </c>
       <c r="I32" t="str" cm="1">
         <f t="array" ref="I32">_xll.ExLibris.Json.GetJsonValue(F1,E6,EXLIBRIS_CONFIGURATION)</f>
-        <v>JsonObject:53B031D7-1A79-4C8D-8898-650D2BB46401</v>
+        <v>JsonObject:48ACA65A-EAC8-4DAD-8832-6C494B258E03</v>
       </c>
       <c r="P32" t="s">
         <v>42</v>
@@ -5986,7 +6169,7 @@
       </c>
       <c r="I33" t="str" cm="1">
         <f t="array" ref="I33">_xll.ExLibris.Json.SeachJsonArrayElements(I32,I8,I11,EXLIBRIS_CONFIGURATION)</f>
-        <v>JsonObject:E38A0DD4-84AF-45DF-8C65-1FD9755B66BA</v>
+        <v>JsonObject:DD5BD8CE-ADD0-4733-B742-5E992CA9D30D</v>
       </c>
       <c r="P33" t="s">
         <v>43</v>
@@ -6336,7 +6519,7 @@
       </c>
       <c r="I38" t="str" cm="1">
         <f t="array" ref="I38">_xll.ExLibris.Json.SeachJsonArrayElements(I32,J8,J11,EXLIBRIS_CONFIGURATION)</f>
-        <v>JsonObject:F79B0B4A-7DAF-4F5F-A598-9D67C0551214</v>
+        <v>JsonObject:3248F93E-A594-417C-8309-34778C42BACA</v>
       </c>
       <c r="P38" t="s">
         <v>48</v>
@@ -6593,7 +6776,7 @@
       </c>
       <c r="I42" t="str" cm="1">
         <f t="array" ref="I42">_xll.ExLibris.Json.SeachJsonArrayElements(I32,J8,,EXLIBRIS_CONFIGURATION)</f>
-        <v>JsonObject:3C304BE1-A20E-4773-9F55-F33916538F99</v>
+        <v>JsonObject:FF6C4EEB-95AE-4EE9-A6A0-A26325A99DF4</v>
       </c>
       <c r="P42" t="s">
         <v>52</v>
@@ -7132,7 +7315,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{92C31E65-5244-494C-A4E6-E2042CA25001}">
-  <dimension ref="B2:H15"/>
+  <dimension ref="B2:F15"/>
   <sheetFormatPr defaultRowHeight="18.75" x14ac:dyDescent="0.4"/>
   <cols>
     <col min="1" max="1" width="3.5" customWidth="1"/>
@@ -7141,16 +7324,16 @@
     <col min="5" max="5" width="39.625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="2:8" x14ac:dyDescent="0.4">
+    <row r="2" spans="2:6" x14ac:dyDescent="0.4">
       <c r="B2" t="s">
         <v>84</v>
       </c>
       <c r="C2" t="str" cm="1">
         <f t="array" ref="C2">_xll.ExLibris.LoadConfiguration(B6:C15)</f>
-        <v>ExLibris.Core.ExLibrisConfiguration:0D0AC951-C4F0-4C41-BE04-012B566C8134</v>
-      </c>
-    </row>
-    <row r="4" spans="2:8" s="4" customFormat="1" ht="18" x14ac:dyDescent="0.4">
+        <v>ExLibris.Core.ExLibrisConfiguration:C0F780BA-4B29-4017-A1D0-C6FF1EFE3B1D</v>
+      </c>
+    </row>
+    <row r="4" spans="2:6" s="4" customFormat="1" ht="18" x14ac:dyDescent="0.4">
       <c r="B4" s="4" t="s">
         <v>86</v>
       </c>
@@ -7158,7 +7341,7 @@
         <v>85</v>
       </c>
     </row>
-    <row r="6" spans="2:8" x14ac:dyDescent="0.4">
+    <row r="6" spans="2:6" x14ac:dyDescent="0.4">
       <c r="B6" t="s">
         <v>76</v>
       </c>
@@ -7172,12 +7355,8 @@
       <c r="F6" t="str">
         <v>Error</v>
       </c>
-      <c r="H6" t="e" cm="1">
-        <f t="array" ref="H6">_xll.ExLibris.ObserveRegisteredObjects()</f>
-        <v>#N/A</v>
-      </c>
-    </row>
-    <row r="7" spans="2:8" x14ac:dyDescent="0.4">
+    </row>
+    <row r="7" spans="2:6" x14ac:dyDescent="0.4">
       <c r="B7" t="s">
         <v>78</v>
       </c>
@@ -7191,7 +7370,7 @@
         <v>Null</v>
       </c>
     </row>
-    <row r="8" spans="2:8" x14ac:dyDescent="0.4">
+    <row r="8" spans="2:6" x14ac:dyDescent="0.4">
       <c r="B8" t="s">
         <v>80</v>
       </c>
@@ -7205,7 +7384,7 @@
         <v>Null</v>
       </c>
     </row>
-    <row r="9" spans="2:8" x14ac:dyDescent="0.4">
+    <row r="9" spans="2:6" x14ac:dyDescent="0.4">
       <c r="B9" t="s">
         <v>81</v>
       </c>
@@ -7219,7 +7398,7 @@
         <v>Null</v>
       </c>
     </row>
-    <row r="10" spans="2:8" x14ac:dyDescent="0.4">
+    <row r="10" spans="2:6" x14ac:dyDescent="0.4">
       <c r="B10" t="s">
         <v>82</v>
       </c>
@@ -7233,7 +7412,7 @@
         <v>StringEmpty</v>
       </c>
     </row>
-    <row r="11" spans="2:8" x14ac:dyDescent="0.4">
+    <row r="11" spans="2:6" x14ac:dyDescent="0.4">
       <c r="B11" t="s">
         <v>83</v>
       </c>
@@ -7247,7 +7426,7 @@
         <v>StringEmpty</v>
       </c>
     </row>
-    <row r="12" spans="2:8" x14ac:dyDescent="0.4">
+    <row r="12" spans="2:6" x14ac:dyDescent="0.4">
       <c r="B12" t="s">
         <v>88</v>
       </c>
@@ -7261,7 +7440,7 @@
         <v>yyyy-MM-dd</v>
       </c>
     </row>
-    <row r="13" spans="2:8" x14ac:dyDescent="0.4">
+    <row r="13" spans="2:6" x14ac:dyDescent="0.4">
       <c r="B13" t="s">
         <v>90</v>
       </c>
@@ -7275,7 +7454,7 @@
         <v>payment _date</v>
       </c>
     </row>
-    <row r="14" spans="2:8" x14ac:dyDescent="0.4">
+    <row r="14" spans="2:6" x14ac:dyDescent="0.4">
       <c r="B14" t="s">
         <v>91</v>
       </c>
@@ -7289,7 +7468,7 @@
         <v>start_date</v>
       </c>
     </row>
-    <row r="15" spans="2:8" x14ac:dyDescent="0.4">
+    <row r="15" spans="2:6" x14ac:dyDescent="0.4">
       <c r="B15" t="s">
         <v>92</v>
       </c>
@@ -7332,7 +7511,7 @@
       </c>
       <c r="E4" t="str" cm="1">
         <f t="array" ref="E4">_xll.ExLibris.WebSockets.OpenWebSocket("ws://localhost:10101",,D4)</f>
-        <v>ExLibris.Core.WebSockets.WebsocketClient:64A5F749-80A8-4374-9287-C09A2113E56C</v>
+        <v>ExLibris.Core.WebSockets.WebsocketClient:AB2FB975-0CCA-4021-925E-95538E68EEE2</v>
       </c>
     </row>
     <row r="6" spans="2:5" x14ac:dyDescent="0.4">
@@ -7422,7 +7601,7 @@
       </c>
       <c r="E17" t="str" cm="1">
         <f t="array" ref="E17">_xll.ExLibris.WebSockets.OpenWebSocket("ws://localhost:10101",,D17)</f>
-        <v>ExLibris.Core.WebSockets.WebsocketClient:BF6644FA-B4E5-4246-9A45-E096A059B7B9</v>
+        <v>ExLibris.Core.WebSockets.WebsocketClient:9ED2A033-BB2A-4015-BB16-5217FF5981DD</v>
       </c>
     </row>
     <row r="19" spans="4:5" x14ac:dyDescent="0.4">
@@ -7543,11 +7722,11 @@
     <row r="5" spans="2:9" x14ac:dyDescent="0.4">
       <c r="B5" t="str" cm="1">
         <f t="array" ref="B5">_xll.ExLibris.WebAPIs.CreateHeaders(B6:C10)</f>
-        <v>ExLibris.Core.WebAPIs.WebAPIHeaders:607A1A5A-615E-4478-A924-6EEEA6541D4C</v>
+        <v>ExLibris.Core.WebAPIs.WebAPIHeaders:7D220D4A-2728-4D06-8EE0-256E966F762A</v>
       </c>
       <c r="H5" t="str" cm="1">
         <f t="array" ref="H5">_xll.ExLibris.Json.CreateJsonObject(H6:I11)</f>
-        <v>JsonObject:01D58A43-E47B-4D68-91D5-77539870CD9B</v>
+        <v>JsonObject:33C27AA8-AC41-4D56-8606-1074506B7926</v>
       </c>
     </row>
     <row r="6" spans="2:9" x14ac:dyDescent="0.4">
@@ -7649,7 +7828,7 @@
       </c>
       <c r="D14" t="str" cm="1">
         <f t="array" ref="D14">_xll.ExLibris.WebAPIs.GET(D13)</f>
-        <v>ExLibris.Core.WebAPIs.Response:3422AB6A-AD26-4E9F-AECF-068391C0CF11</v>
+        <v>ExLibris.Core.WebAPIs.Response:D765FAFA-CFE3-4296-9E30-F02598C32B0F</v>
       </c>
     </row>
     <row r="15" spans="2:9" x14ac:dyDescent="0.4">
@@ -7696,7 +7875,7 @@
       </c>
       <c r="D19" t="str" cm="1">
         <f t="array" ref="D19">_xll.ExLibris.WebAPIs.POST(D18)</f>
-        <v>ExLibris.Core.WebAPIs.Response:D2E0241D-F272-47A9-BC83-264C38DB11B4</v>
+        <v>ExLibris.Core.WebAPIs.Response:144C2A18-4FEF-421F-8961-FD3E2B892543</v>
       </c>
     </row>
     <row r="20" spans="2:4" x14ac:dyDescent="0.4">
@@ -7720,6 +7899,7 @@
   "files": {}, 
   "form": {}, 
   "headers": {
+    "Connection": "Keep-Alive", 
     "Content-Length": "0", 
     "Host": "localhost"
   }, 
@@ -7748,7 +7928,7 @@
       </c>
       <c r="D24" t="str" cm="1">
         <f t="array" ref="D24">_xll.ExLibris.WebAPIs.GET(D23,$B$5)</f>
-        <v>ExLibris.Core.WebAPIs.Response:28D413B8-3384-44C5-A8AE-65466649C73B</v>
+        <v>ExLibris.Core.WebAPIs.Response:079F80DA-196F-4A51-975A-BD2B1CCC7C0B</v>
       </c>
     </row>
     <row r="25" spans="2:4" x14ac:dyDescent="0.4">
@@ -7791,7 +7971,7 @@
       </c>
       <c r="D29" t="str" cm="1">
         <f t="array" ref="D29">_xll.ExLibris.WebAPIs.POST(D28,_xll.ExLibris.Json.ShowJsonText(H5),,$B$5)</f>
-        <v>ExLibris.Core.WebAPIs.Response:D542C13C-E967-48F3-B47B-DC9F20305133</v>
+        <v>ExLibris.Core.WebAPIs.Response:D924CFF8-9704-43C3-AAC5-A434FB913AA2</v>
       </c>
     </row>
     <row r="30" spans="2:4" x14ac:dyDescent="0.4">
@@ -7857,7 +8037,7 @@
       </c>
       <c r="D34" t="str" cm="1">
         <f t="array" ref="D34">_xll.ExLibris.WebAPIs.POST(D33,H5,TRUE,$B$5)</f>
-        <v>ExLibris.Core.WebAPIs.Response:4E53B07D-0595-4CD3-84EA-7AA2F5C1A0B8</v>
+        <v>ExLibris.Core.WebAPIs.Response:DEB3F378-D556-40DC-B099-B9F45F93BEF6</v>
       </c>
     </row>
     <row r="35" spans="2:4" x14ac:dyDescent="0.4">
@@ -7921,7 +8101,7 @@
       </c>
       <c r="D39" t="str" cm="1">
         <f t="array" ref="D39">_xll.ExLibris.WebAPIs.POST(D38,H6:I11,TRUE,$B$5)</f>
-        <v>ExLibris.Core.WebAPIs.Response:71ACDFA3-7B6F-423F-A66F-3B2F38787FE9</v>
+        <v>ExLibris.Core.WebAPIs.Response:EAE099CF-2684-44D2-9AEE-3D6B5CBEDFD3</v>
       </c>
     </row>
     <row r="40" spans="2:4" x14ac:dyDescent="0.4">
@@ -7992,7 +8172,7 @@
       </c>
       <c r="D44" t="str" cm="1">
         <f t="array" ref="D44">_xll.ExLibris.WebAPIs.GET(D43)</f>
-        <v>ExLibris.Core.WebAPIs.Response:A8C44C1F-63C1-498F-A66D-BD891367955D</v>
+        <v>ExLibris.Core.WebAPIs.Response:E38D6823-BA7F-4A29-ABAC-663259DF3427</v>
       </c>
     </row>
     <row r="45" spans="2:4" x14ac:dyDescent="0.4">
@@ -8020,6 +8200,7 @@
     "strike": "108.5"
   }, 
   "headers": {
+    "Connection": "Keep-Alive", 
     "Host": "localhost"
   }, 
   "origin": "172.17.0.1", 
@@ -8046,7 +8227,7 @@
       </c>
       <c r="D49" t="str" cm="1">
         <f t="array" ref="D49">_xll.ExLibris.WebAPIs.GET(D48)</f>
-        <v>ExLibris.Core.WebAPIs.Response:FFFECBC7-200C-42C6-AEAC-67E3D66D9592</v>
+        <v>ExLibris.Core.WebAPIs.Response:1E65B074-72E8-4407-85F1-4C0F94C1B13F</v>
       </c>
     </row>
     <row r="50" spans="3:4" x14ac:dyDescent="0.4">
@@ -8070,6 +8251,7 @@
   "files": {}, 
   "form": {}, 
   "headers": {
+    "Connection": "Keep-Alive", 
     "Host": "localhost"
   }, 
   "origin": "172.17.0.1", 
@@ -8099,7 +8281,7 @@
     <row r="2" spans="2:4" x14ac:dyDescent="0.4">
       <c r="B2" t="str" cm="1">
         <f t="array" ref="B2">_xll.ExLibris.WebAPIs.CreateHeaders(B3:C3)</f>
-        <v>ExLibris.Core.WebAPIs.WebAPIHeaders:23264D0A-C894-44C1-A933-7234EAD7ABDD</v>
+        <v>ExLibris.Core.WebAPIs.WebAPIHeaders:665F0DD1-DB43-4FAA-9DEA-35D5F9E40BB3</v>
       </c>
     </row>
     <row r="3" spans="2:4" x14ac:dyDescent="0.4">
@@ -8125,7 +8307,7 @@
       </c>
       <c r="C6" t="str" cm="1">
         <f t="array" ref="C6">_xll.ExLibris.WebAPIs.GET(C5,B2)</f>
-        <v>ExLibris.Core.WebAPIs.Response:6BD702DC-C4E7-486F-A4BA-8814D286CDB6</v>
+        <v>ExLibris.Core.WebAPIs.Response:F20EA3B2-D4D7-4CFD-81DD-EB4598D11A81</v>
       </c>
     </row>
     <row r="7" spans="2:4" x14ac:dyDescent="0.4">
@@ -8149,7 +8331,7 @@
     <row r="10" spans="2:4" x14ac:dyDescent="0.4">
       <c r="C10" t="str" cm="1">
         <f t="array" ref="C10">_xll.ExLibris.Json.CreateJsonObject(C8)</f>
-        <v>JsonObject:226378C9-B698-4112-B3DE-F839054F1465</v>
+        <v>JsonObject:E2431071-56E5-4E55-9723-67F38579DCAB</v>
       </c>
     </row>
     <row r="11" spans="2:4" x14ac:dyDescent="0.4">

</xml_diff>

<commit_message>
get json key values
</commit_message>
<xml_diff>
--- a/ExLibris/test_excel/exlibris_test.xlsx
+++ b/ExLibris/test_excel/exlibris_test.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\mugen\git\ex-libris\ExLibris\test_excel\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A9379E99-0DA2-46B0-BD79-4DF8DC18760A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6CD0F803-07AD-4DCD-A8FD-1953ACC33668}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{705CD0B7-27A9-4291-85BD-6034C0FEE3E4}"/>
   </bookViews>
@@ -43,7 +43,7 @@
 </file>
 
 <file path=xl/metadata.xml><?xml version="1.0" encoding="utf-8"?>
-<metadata xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xda="http://schemas.microsoft.com/office/spreadsheetml/2017/dynamicarray">
+<metadata xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xlrd="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata" xmlns:xda="http://schemas.microsoft.com/office/spreadsheetml/2017/dynamicarray">
   <metadataTypes count="1">
     <metadataType name="XLDAPR" minSupportedVersion="120000" copy="1" pasteAll="1" pasteValues="1" merge="1" splitFirst="1" rowColShift="1" clearFormats="1" clearComments="1" assign="1" coerce="1" cellMeta="1"/>
   </metadataTypes>
@@ -65,7 +65,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="661" uniqueCount="181">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="691" uniqueCount="183">
   <si>
     <t>payment _date</t>
   </si>
@@ -814,6 +814,14 @@
   "url": "http://localhost/post"
 }
 </t>
+  </si>
+  <si>
+    <t>keyvalues2</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>keyvalues3</t>
+    <phoneticPr fontId="1"/>
   </si>
 </sst>
 </file>
@@ -944,1199 +952,1213 @@
 <file path=xl/volatileDependencies.xml><?xml version="1.0" encoding="utf-8"?>
 <volTypes xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <volType type="realTimeData">
-    <main first="rtdsrv.e91a2bf1ca1e4425853080e41816bb7b">
+    <main first="rtdsrv.83aaa2cc90e24b62bd47ab1283cce962">
       <tp>
         <v>2</v>
         <stp/>
-        <stp>6eaef360-c5fb-40a8-a98e-634d423d7346</stp>
+        <stp>781cc7f2-9f82-48b6-8c87-989b4d997e01</stp>
+        <tr r="G53" s="4"/>
+      </tp>
+      <tp>
+        <v>2</v>
+        <stp/>
+        <stp>9455518a-323a-4960-9aea-330b0d12d5ae</stp>
+        <tr r="G41" s="4"/>
+      </tp>
+    </main>
+    <main first="rtdsrv.83aaa2cc90e24b62bd47ab1283cce962">
+      <tp>
+        <v>2</v>
+        <stp/>
+        <stp>3a7bac21-0343-49b1-aaa7-3751df1103a1</stp>
+        <tr r="D35" s="5"/>
+      </tp>
+    </main>
+    <main first="rtdsrv.83aaa2cc90e24b62bd47ab1283cce962">
+      <tp>
+        <v>2</v>
+        <stp/>
+        <stp>be7e2e83-ffac-4fac-be04-0f59a2d03ab0</stp>
+        <tr r="G45" s="1"/>
+      </tp>
+      <tp>
+        <v>1</v>
+        <stp/>
+        <stp>cb16e582-aaf8-41cd-a1c8-16d31594f288</stp>
+        <tr r="G45" s="7"/>
+      </tp>
+      <tp>
+        <v>2</v>
+        <stp/>
+        <stp>05e760a5-b10e-43f2-b9af-8327cf786af3</stp>
+        <tr r="D45" s="5"/>
+      </tp>
+      <tp>
+        <v>2</v>
+        <stp/>
+        <stp>419e2edc-71eb-4db4-925a-da17f73e043d</stp>
+        <tr r="G41" s="1"/>
+      </tp>
+    </main>
+    <main first="rtdsrv.83aaa2cc90e24b62bd47ab1283cce962">
+      <tp>
+        <v>2</v>
+        <stp/>
+        <stp>3ac7c14d-ec11-4de8-9296-1d64ac61d0ec</stp>
+        <tr r="G50" s="4"/>
+      </tp>
+      <tp>
+        <v>1</v>
+        <stp/>
+        <stp>ba1004bc-af6e-41f2-bd3a-0e1980346c3a</stp>
+        <tr r="G21" s="7"/>
+      </tp>
+    </main>
+    <main first="rtdsrv.83aaa2cc90e24b62bd47ab1283cce962">
+      <tp>
+        <v>2</v>
+        <stp/>
+        <stp>d5943d92-2aba-4a6f-993e-acfa6e83e347</stp>
+        <tr r="G48" s="1"/>
+      </tp>
+      <tp>
+        <v>1</v>
+        <stp/>
+        <stp>39452744-12b2-4713-85ca-c99b87c81bbc</stp>
+        <tr r="G56" s="7"/>
+      </tp>
+      <tp>
+        <v>2</v>
+        <stp/>
+        <stp>ddf990ca-f2cf-4d07-bfb8-e6ede4436f57</stp>
+        <tr r="I38" s="4"/>
+      </tp>
+      <tp>
+        <v>2</v>
+        <stp/>
+        <stp>a5cb6c46-bc63-4c50-a6ef-b2c78c9d83aa</stp>
+        <tr r="D40" s="5"/>
+      </tp>
+    </main>
+    <main first="rtdsrv.83aaa2cc90e24b62bd47ab1283cce962">
+      <tp>
+        <v>1</v>
+        <stp/>
+        <stp>ae4bdd0d-d3f3-45ac-a373-1fe3602b2da4</stp>
+        <tr r="G20" s="7"/>
+      </tp>
+      <tp>
+        <v>2</v>
+        <stp/>
+        <stp>b7f99f94-b33f-4613-97f4-8fa54320204d</stp>
+        <tr r="D7" s="3"/>
+      </tp>
+      <tp>
+        <v>2</v>
+        <stp/>
+        <stp>97ef3fe0-b52c-4e33-8318-a422347b3252</stp>
+        <tr r="F6" s="1"/>
+      </tp>
+    </main>
+    <main first="rtdsrv.83aaa2cc90e24b62bd47ab1283cce962">
+      <tp>
+        <v>2</v>
+        <stp/>
+        <stp>77f7ddb4-945b-460a-ac4f-cabaeeacc906</stp>
+        <tr r="I19" s="1"/>
+      </tp>
+    </main>
+    <main first="rtdsrv.83aaa2cc90e24b62bd47ab1283cce962">
+      <tp>
+        <v>1</v>
+        <stp/>
+        <stp>2a254403-2440-4f1b-9258-43eb176a5647</stp>
+        <tr r="G48" s="7"/>
+      </tp>
+      <tp>
+        <v>2</v>
+        <stp/>
+        <stp>d472073e-d335-4c99-b06c-a83ee6d92d48</stp>
+        <tr r="G49" s="4"/>
+      </tp>
+      <tp>
+        <v>2</v>
+        <stp/>
+        <stp>6ff01800-1c9f-4738-aa51-6ffb9712067f</stp>
+        <tr r="G22" s="4"/>
+      </tp>
+    </main>
+    <main first="rtdsrv.83aaa2cc90e24b62bd47ab1283cce962">
+      <tp>
+        <v>2</v>
+        <stp/>
+        <stp>a0697226-393a-4eb6-9bf7-c72b31e57b70</stp>
+        <tr r="G38" s="4"/>
+      </tp>
+      <tp>
+        <v>2</v>
+        <stp/>
+        <stp>9cc097cc-78e3-483a-8a68-c7b776e6b00a</stp>
+        <tr r="B2" s="6"/>
+      </tp>
+    </main>
+    <main first="rtdsrv.83aaa2cc90e24b62bd47ab1283cce962">
+      <tp>
+        <v>2</v>
+        <stp/>
+        <stp>f4dc9a7a-0d57-4696-852c-2a6aa13614cd</stp>
+        <tr r="F8" s="3"/>
+      </tp>
+      <tp>
+        <v>2</v>
+        <stp/>
+        <stp>98ec348c-c302-41d1-bfd2-d0e4d97b0614</stp>
+        <tr r="G35" s="1"/>
+      </tp>
+    </main>
+    <main first="rtdsrv.83aaa2cc90e24b62bd47ab1283cce962">
+      <tp>
+        <v>2</v>
+        <stp/>
+        <stp>78939997-bf23-4bd1-a616-8b648c739f5d</stp>
+        <tr r="F1" s="4"/>
+      </tp>
+    </main>
+    <main first="rtdsrv.83aaa2cc90e24b62bd47ab1283cce962">
+      <tp>
+        <v>2</v>
+        <stp/>
+        <stp>03b474ee-2eb9-4143-a233-b23682097133</stp>
         <tr r="G19" s="4"/>
       </tp>
-      <tp>
-        <v>1</v>
-        <stp/>
-        <stp>eaa60cc1-c804-4b2c-b31d-9adbbb77c789</stp>
+    </main>
+    <main first="rtdsrv.83aaa2cc90e24b62bd47ab1283cce962">
+      <tp>
+        <v>2</v>
+        <stp/>
+        <stp>918a4a19-e41d-4cb3-9fd0-9ddd63c811c5</stp>
+        <tr r="G47" s="1"/>
+      </tp>
+      <tp>
+        <v>1</v>
+        <stp/>
+        <stp>5da1a095-0329-4964-8f62-ac88845765b0</stp>
+        <tr r="G25" s="7"/>
+      </tp>
+      <tp>
+        <v>1</v>
+        <stp/>
+        <stp>39c959e5-2798-4bc8-a793-6fb1a2247cbe</stp>
+        <tr r="G39" s="7"/>
+      </tp>
+      <tp>
+        <v>2</v>
+        <stp/>
+        <stp>4999c6e7-c231-4c9e-9a1f-9e5e2a976846</stp>
+        <tr r="G33" s="1"/>
+      </tp>
+    </main>
+    <main first="rtdsrv.83aaa2cc90e24b62bd47ab1283cce962">
+      <tp>
+        <v>1</v>
+        <stp/>
+        <stp>ab69a5ad-76db-4d3e-a3b3-e288ce5224da</stp>
+        <tr r="P74" s="7"/>
+      </tp>
+      <tp>
+        <v>2</v>
+        <stp/>
+        <stp>fdc49044-43e1-4b3e-bac2-4b9f990e59d5</stp>
+        <tr r="G27" s="1"/>
+      </tp>
+      <tp>
+        <v>2</v>
+        <stp/>
+        <stp>c053bc4e-a82e-4f87-b162-92c476f1234c</stp>
+        <tr r="G54" s="4"/>
+      </tp>
+    </main>
+    <main first="rtdsrv.83aaa2cc90e24b62bd47ab1283cce962">
+      <tp>
+        <v>2</v>
+        <stp/>
+        <stp>c17a4710-84cb-4ae1-aa06-08852f021e47</stp>
+        <tr r="P29" s="1"/>
+      </tp>
+      <tp>
+        <v>2</v>
+        <stp/>
+        <stp>e4bbc09f-64b9-4722-9d77-cb209c6da189</stp>
+        <tr r="G33" s="4"/>
+      </tp>
+      <tp>
+        <v>2</v>
+        <stp/>
+        <stp>b6ca0360-5a86-4753-9115-dbb4b5cd8bce</stp>
+        <tr r="B5" s="5"/>
+      </tp>
+      <tp>
+        <v>2</v>
+        <stp/>
+        <stp>43b53dff-3c07-461f-b5ad-ce0d969077f2</stp>
+        <tr r="G46" s="4"/>
+      </tp>
+      <tp>
+        <v>2</v>
+        <stp/>
+        <stp>2c7766e6-ce1a-462f-b530-20905dcf2015</stp>
+        <tr r="G37" s="4"/>
+      </tp>
+    </main>
+    <main first="rtdsrv.83aaa2cc90e24b62bd47ab1283cce962">
+      <tp>
+        <v>2</v>
+        <stp/>
+        <stp>73c66fca-3b4c-4740-80fd-8ccca63cebbc</stp>
+        <tr r="G49" s="1"/>
+      </tp>
+      <tp>
+        <v>2</v>
+        <stp/>
+        <stp>8923ca10-38f3-4acb-9ec4-c2126981cf59</stp>
+        <tr r="G42" s="4"/>
+      </tp>
+      <tp>
+        <v>1</v>
+        <stp/>
+        <stp>007939f4-730e-43bc-965c-69748b21a461</stp>
+        <tr r="G6" s="3"/>
+      </tp>
+      <tp>
+        <v>2</v>
+        <stp/>
+        <stp>83a7e6f4-4a94-4bd9-9a86-ab556a9df4e9</stp>
+        <tr r="G43" s="1"/>
+      </tp>
+    </main>
+    <main first="rtdsrv.83aaa2cc90e24b62bd47ab1283cce962">
+      <tp>
+        <v>2</v>
+        <stp/>
+        <stp>b35adbf1-0099-4a4c-90d4-92639bf5d0e9</stp>
+        <tr r="G50" s="1"/>
+      </tp>
+      <tp>
+        <v>1</v>
+        <stp/>
+        <stp>a680c21a-0332-4f0a-91e2-30950db84b32</stp>
+        <tr r="G31" s="7"/>
+      </tp>
+      <tp>
+        <v>1</v>
+        <stp/>
+        <stp>914b9964-dba4-47ce-9831-4c0589290f39</stp>
+        <tr r="I19" s="7"/>
+      </tp>
+    </main>
+    <main first="rtdsrv.83aaa2cc90e24b62bd47ab1283cce962">
+      <tp>
+        <v>1</v>
+        <stp/>
+        <stp>765c024f-4fc5-4d03-a940-0dddcc5e6600</stp>
+        <tr r="G37" s="7"/>
+      </tp>
+    </main>
+    <main first="rtdsrv.83aaa2cc90e24b62bd47ab1283cce962">
+      <tp>
+        <v>2</v>
+        <stp/>
+        <stp>0adb5746-4494-41a6-81d5-6c082c3596be</stp>
+        <tr r="P19" s="1"/>
+      </tp>
+      <tp>
+        <v>1</v>
+        <stp/>
+        <stp>832e845a-b9f0-411b-8632-df6c1a46155c</stp>
+        <tr r="H5" s="3"/>
+      </tp>
+    </main>
+    <main first="rtdsrv.83aaa2cc90e24b62bd47ab1283cce962">
+      <tp>
+        <v>2</v>
+        <stp/>
+        <stp>b588fff7-e4e6-4f53-9d08-d158779b65d6</stp>
+        <tr r="P67" s="1"/>
+      </tp>
+      <tp>
+        <v>2</v>
+        <stp/>
+        <stp>b0870767-23dd-4b28-95f6-1a72a931a576</stp>
+        <tr r="G56" s="4"/>
+      </tp>
+      <tp>
+        <v>1</v>
+        <stp/>
+        <stp>f59328b1-c341-4b0f-839b-efab85d59d73</stp>
+        <tr r="G36" s="7"/>
+      </tp>
+      <tp>
+        <v>2</v>
+        <stp/>
+        <stp>490c3bcc-54c1-4e09-8af2-5d69c9b0aeff</stp>
+        <tr r="G39" s="1"/>
+      </tp>
+      <tp>
+        <v>2</v>
+        <stp/>
+        <stp>11349109-2f9a-4564-b25b-0fa338c78dc9</stp>
+        <tr r="I28" s="4"/>
+      </tp>
+      <tp>
+        <v>2</v>
+        <stp/>
+        <stp>07fe09f7-9634-419d-8284-12209b04c2a1</stp>
+        <tr r="G29" s="1"/>
+      </tp>
+    </main>
+    <main first="rtdsrv.83aaa2cc90e24b62bd47ab1283cce962">
+      <tp>
+        <v>2</v>
+        <stp/>
+        <stp>4f9d77f0-7437-4a0c-88be-18d21cbb95b0</stp>
+        <tr r="G51" s="1"/>
+      </tp>
+      <tp>
+        <v>1</v>
+        <stp/>
+        <stp>2534f438-5d7e-431c-add8-2823ed6caf16</stp>
+        <tr r="G30" s="7"/>
+      </tp>
+      <tp>
+        <v>2</v>
+        <stp/>
+        <stp>1b94d221-881d-43ee-b340-72e727ac1529</stp>
+        <tr r="G45" s="4"/>
+      </tp>
+    </main>
+    <main first="rtdsrv.83aaa2cc90e24b62bd47ab1283cce962">
+      <tp>
+        <v>2</v>
+        <stp/>
+        <stp>d2a92545-35eb-4f24-99b7-6ccff062d830</stp>
+        <tr r="G38" s="1"/>
+      </tp>
+      <tp>
+        <v>2</v>
+        <stp/>
+        <stp>fd35b8b1-6ec0-4db7-8126-b3a97a1b4554</stp>
+        <tr r="G26" s="4"/>
+      </tp>
+    </main>
+    <main first="rtdsrv.83aaa2cc90e24b62bd47ab1283cce962">
+      <tp>
+        <v>1</v>
+        <stp/>
+        <stp>f6978cff-96e9-44eb-b466-6e917ba497be</stp>
+        <tr r="P19" s="7"/>
+      </tp>
+    </main>
+    <main first="rtdsrv.83aaa2cc90e24b62bd47ab1283cce962">
+      <tp>
+        <v>1</v>
+        <stp/>
+        <stp>a9afdcb2-1b97-413d-aba5-9a0bea2cdf72</stp>
+        <tr r="G41" s="7"/>
+      </tp>
+    </main>
+    <main first="rtdsrv.83aaa2cc90e24b62bd47ab1283cce962">
+      <tp>
+        <v>2</v>
+        <stp/>
+        <stp>b8bae2b1-e03a-46cf-af78-dc657f5503fc</stp>
+        <tr r="D30" s="5"/>
+      </tp>
+    </main>
+    <main first="rtdsrv.83aaa2cc90e24b62bd47ab1283cce962">
+      <tp>
+        <v>2</v>
+        <stp/>
+        <stp>8b38cfa6-9ab7-4eaa-b13b-d3af9adfe603</stp>
+        <tr r="G24" s="1"/>
+      </tp>
+    </main>
+    <main first="rtdsrv.83aaa2cc90e24b62bd47ab1283cce962">
+      <tp>
+        <v>1</v>
+        <stp/>
+        <stp>495e377f-a691-42af-bad7-2c1de40f61fb</stp>
+        <tr r="G43" s="7"/>
+      </tp>
+    </main>
+    <main first="rtdsrv.83aaa2cc90e24b62bd47ab1283cce962">
+      <tp>
+        <v>2</v>
+        <stp/>
+        <stp>643a4760-9e38-4a72-95ca-3ceaf34810de</stp>
+        <tr r="D8" s="3"/>
+      </tp>
+      <tp>
+        <v>2</v>
+        <stp/>
+        <stp>0ec90c5d-7325-4e10-b064-b782d92072e8</stp>
+        <tr r="G55" s="1"/>
+      </tp>
+      <tp>
+        <v>2</v>
+        <stp/>
+        <stp>0325835e-7032-41cb-9124-52bb1f8c18ec</stp>
+        <tr r="F5" s="3"/>
+      </tp>
+    </main>
+    <main first="rtdsrv.83aaa2cc90e24b62bd47ab1283cce962">
+      <tp>
+        <v>2</v>
+        <stp/>
+        <stp>4bb79eb0-e82a-48a8-a4a8-6c8b41081ccf</stp>
+        <tr r="G32" s="4"/>
+      </tp>
+    </main>
+    <main first="rtdsrv.83aaa2cc90e24b62bd47ab1283cce962">
+      <tp>
+        <v>2</v>
+        <stp/>
+        <stp>9dd91f9f-dbfc-4fbc-b690-8a676142bf86</stp>
+        <tr r="G31" s="4"/>
+      </tp>
+      <tp>
+        <v>1</v>
+        <stp/>
+        <stp>6d826bdb-8abe-4f71-b677-270c446dd147</stp>
+        <tr r="G28" s="7"/>
+      </tp>
+    </main>
+    <main first="rtdsrv.83aaa2cc90e24b62bd47ab1283cce962">
+      <tp>
+        <v>2</v>
+        <stp/>
+        <stp>faec576b-9edf-4454-8143-77114de48124</stp>
+        <tr r="G56" s="1"/>
+      </tp>
+      <tp>
+        <v>1</v>
+        <stp/>
+        <stp>c524c195-2c21-4b30-b830-bfeeaf8478d2</stp>
+        <tr r="G8" s="3"/>
+      </tp>
+    </main>
+    <main first="rtdsrv.83aaa2cc90e24b62bd47ab1283cce962">
+      <tp>
+        <v>2</v>
+        <stp/>
+        <stp>c6fbae5b-5405-4ce4-8256-4fb75932d54e</stp>
+        <tr r="G23" s="4"/>
+      </tp>
+      <tp>
+        <v>2</v>
+        <stp/>
+        <stp>a61118d6-20f2-4d4c-b566-93df9dfd53c8</stp>
+        <tr r="G28" s="4"/>
+      </tp>
+    </main>
+    <main first="rtdsrv.83aaa2cc90e24b62bd47ab1283cce962">
+      <tp>
+        <v>2</v>
+        <stp/>
+        <stp>9ef2f2ed-4c3a-4177-9783-d3570a4db3b5</stp>
+        <tr r="G57" s="1"/>
+      </tp>
+    </main>
+    <main first="rtdsrv.83aaa2cc90e24b62bd47ab1283cce962">
+      <tp>
+        <v>2</v>
+        <stp/>
+        <stp>365e1290-0f5d-4958-b8c0-91d20fbd245f</stp>
+        <tr r="I42" s="4"/>
+      </tp>
+      <tp>
+        <v>1</v>
+        <stp/>
+        <stp>3a1c3389-a8ab-43da-9adb-33831016f920</stp>
+        <tr r="G23" s="7"/>
+      </tp>
+    </main>
+    <main first="rtdsrv.83aaa2cc90e24b62bd47ab1283cce962">
+      <tp>
+        <v>1</v>
+        <stp/>
+        <stp>085bc341-11e5-41a0-9e9c-ea0cd9364d55</stp>
+        <tr r="G29" s="7"/>
+      </tp>
+    </main>
+    <main first="rtdsrv.83aaa2cc90e24b62bd47ab1283cce962">
+      <tp>
+        <v>2</v>
+        <stp/>
+        <stp>a8ad7b3b-7967-46ff-82fe-229964ad1d2c</stp>
+        <tr r="G36" s="4"/>
+      </tp>
+    </main>
+    <main first="rtdsrv.83aaa2cc90e24b62bd47ab1283cce962">
+      <tp>
+        <v>2</v>
+        <stp/>
+        <stp>d754fe3d-dc8f-4fe9-90af-7d99b76a62b0</stp>
+        <tr r="F6" s="4"/>
+      </tp>
+    </main>
+    <main first="rtdsrv.83aaa2cc90e24b62bd47ab1283cce962">
+      <tp>
+        <v>1</v>
+        <stp/>
+        <stp>b144271f-8998-40f1-91e9-c43fd3852bed</stp>
+        <tr r="I28" s="7"/>
+      </tp>
+    </main>
+    <main first="rtdsrv.83aaa2cc90e24b62bd47ab1283cce962">
+      <tp>
+        <v>2</v>
+        <stp/>
+        <stp>bbc659f8-154e-4472-a2ee-1ba613bbacf7</stp>
+        <tr r="G22" s="1"/>
+      </tp>
+    </main>
+    <main first="rtdsrv.83aaa2cc90e24b62bd47ab1283cce962">
+      <tp>
+        <v>1</v>
+        <stp/>
+        <stp>2856504c-b560-4495-a0f6-3a9d133b9d1a</stp>
+        <tr r="G46" s="7"/>
+      </tp>
+    </main>
+    <main first="rtdsrv.83aaa2cc90e24b62bd47ab1283cce962">
+      <tp>
+        <v>2</v>
+        <stp/>
+        <stp>6c626d03-a81e-4eb7-8cc0-05acf84ee10f</stp>
+        <tr r="G40" s="1"/>
+      </tp>
+    </main>
+    <main first="rtdsrv.83aaa2cc90e24b62bd47ab1283cce962">
+      <tp>
+        <v>1</v>
+        <stp/>
+        <stp>51251472-b147-4282-8b3c-b8a16d03544e</stp>
+        <tr r="F1" s="7"/>
+      </tp>
+      <tp>
+        <v>1</v>
+        <stp/>
+        <stp>cbcb5a2d-56e4-4408-9ec1-33283e5345aa</stp>
+        <tr r="G53" s="7"/>
+      </tp>
+      <tp>
+        <v>2</v>
+        <stp/>
+        <stp>9c138950-08be-4624-830d-603b7ab9c161</stp>
+        <tr r="G54" s="1"/>
+      </tp>
+    </main>
+    <main first="rtdsrv.83aaa2cc90e24b62bd47ab1283cce962">
+      <tp>
+        <v>2</v>
+        <stp/>
+        <stp>34d8ad6a-0d28-43e7-8766-5d7c47771cb8</stp>
+        <tr r="G29" s="4"/>
+      </tp>
+      <tp>
+        <v>1</v>
+        <stp/>
+        <stp>b582e0a2-6544-420a-984e-a0098fa2ca8e</stp>
+        <tr r="G26" s="7"/>
+      </tp>
+    </main>
+    <main first="rtdsrv.83aaa2cc90e24b62bd47ab1283cce962">
+      <tp>
+        <v>2</v>
+        <stp/>
+        <stp>12f25685-c754-40e4-b58b-e9e2745cb707</stp>
+        <tr r="I19" s="4"/>
+        <tr r="I32" s="4"/>
+      </tp>
+      <tp>
+        <v>2</v>
+        <stp/>
+        <stp>54104e83-a292-4af5-9760-7de40ec9acec</stp>
+        <tr r="G55" s="4"/>
+      </tp>
+      <tp>
+        <v>1</v>
+        <stp/>
+        <stp>97942f62-c6c6-462e-827d-35d096834271</stp>
+        <tr r="G47" s="7"/>
+      </tp>
+    </main>
+    <main first="rtdsrv.83aaa2cc90e24b62bd47ab1283cce962">
+      <tp>
+        <v>1</v>
+        <stp/>
+        <stp>80d281e4-c137-4e7c-a4cf-b2c5d1f1717e</stp>
+        <tr r="G19" s="7"/>
+      </tp>
+      <tp>
+        <v>2</v>
+        <stp/>
+        <stp>56405802-9cbe-4aaf-9615-403ec25ef26a</stp>
+        <tr r="G31" s="1"/>
+      </tp>
+      <tp>
+        <v>2</v>
+        <stp/>
+        <stp>8d4e1cce-ff6f-4fb4-98a1-3c6a9c1a7df1</stp>
+        <tr r="G21" s="4"/>
+      </tp>
+      <tp>
+        <v>2</v>
+        <stp/>
+        <stp>7194aea8-f0b3-47a0-9f05-f7f21e0db0de</stp>
+        <tr r="G19" s="1"/>
+      </tp>
+    </main>
+    <main first="rtdsrv.83aaa2cc90e24b62bd47ab1283cce962">
+      <tp>
+        <v>1</v>
+        <stp/>
+        <stp>d5719053-a00a-4a59-a667-a8717ae68b88</stp>
+        <tr r="G50" s="7"/>
+      </tp>
+    </main>
+    <main first="rtdsrv.83aaa2cc90e24b62bd47ab1283cce962">
+      <tp>
+        <v>1</v>
+        <stp/>
+        <stp>7621dfbf-a44f-4417-bed7-4db05b594472</stp>
+        <tr r="H4" s="3"/>
+      </tp>
+    </main>
+    <main first="rtdsrv.83aaa2cc90e24b62bd47ab1283cce962">
+      <tp>
+        <v>1</v>
+        <stp/>
+        <stp>ae800841-553b-40b7-a890-eba54bbca609</stp>
+        <tr r="G54" s="7"/>
+      </tp>
+      <tp>
+        <v>2</v>
+        <stp/>
+        <stp>a1de132e-e0bd-4b0a-8e3d-840aac3be1c8</stp>
+        <tr r="D50" s="5"/>
+      </tp>
+      <tp>
+        <v>2</v>
+        <stp/>
+        <stp>677ff6f7-ed92-4a22-846b-8e64b7282a80</stp>
+        <tr r="G25" s="1"/>
+      </tp>
+    </main>
+    <main first="rtdsrv.83aaa2cc90e24b62bd47ab1283cce962">
+      <tp>
+        <v>1</v>
+        <stp/>
+        <stp>21ad7d21-7c38-45e9-81ea-9932dd73913e</stp>
+        <tr r="P67" s="7"/>
+      </tp>
+      <tp>
+        <v>1</v>
+        <stp/>
+        <stp>b497b1b5-7988-4a6e-986b-3a66aeaa972b</stp>
+        <tr r="G42" s="7"/>
+      </tp>
+      <tp>
+        <v>1</v>
+        <stp/>
+        <stp>ce5c65ba-c916-49f6-bcaa-9b760d93f0da</stp>
+        <tr r="H8" s="3"/>
+      </tp>
+      <tp>
+        <v>2</v>
+        <stp/>
+        <stp>53f90b58-339c-4db9-b706-960cb991962b</stp>
+        <tr r="C6" s="6"/>
+      </tp>
+    </main>
+    <main first="rtdsrv.83aaa2cc90e24b62bd47ab1283cce962">
+      <tp>
+        <v>2</v>
+        <stp/>
+        <stp>24de8fa0-c8b4-455d-8997-7b3c493a0ef2</stp>
+        <tr r="D6" s="3"/>
+      </tp>
+      <tp>
+        <v>2</v>
+        <stp/>
+        <stp>f149b172-8151-4da1-8e8c-a3075cb9430e</stp>
+        <tr r="G44" s="1"/>
+      </tp>
+    </main>
+    <main first="rtdsrv.83aaa2cc90e24b62bd47ab1283cce962">
+      <tp>
+        <v>1</v>
+        <stp/>
+        <stp>618daed7-5bf1-454e-8f05-e6a7a5df9e7b</stp>
+        <tr r="H7" s="3"/>
+      </tp>
+      <tp>
+        <v>1</v>
+        <stp/>
+        <stp>dadb8c1a-9154-4b85-858a-3742bec82147</stp>
+        <tr r="G7" s="3"/>
+      </tp>
+      <tp>
+        <v>1</v>
+        <stp/>
+        <stp>65b794ab-1da3-492f-98e6-4e46942e6729</stp>
+        <tr r="G51" s="7"/>
+      </tp>
+      <tp>
+        <v>1</v>
+        <stp/>
+        <stp>e6f560ed-c8d5-47e5-8b5c-d309309cb352</stp>
+        <tr r="G34" s="7"/>
+      </tp>
+      <tp>
+        <v>1</v>
+        <stp/>
+        <stp>cd4f845c-3a08-4656-8ad1-9636011ddc09</stp>
+        <tr r="G40" s="7"/>
+      </tp>
+      <tp>
+        <v>2</v>
+        <stp/>
+        <stp>80376dc9-71e9-4b83-aaf6-64563d50f360</stp>
+        <tr r="I28" s="1"/>
+      </tp>
+    </main>
+    <main first="rtdsrv.83aaa2cc90e24b62bd47ab1283cce962">
+      <tp>
+        <v>1</v>
+        <stp/>
+        <stp>6161bfe8-6390-49f7-b024-5f45da83667d</stp>
+        <tr r="G44" s="7"/>
+      </tp>
+      <tp>
+        <v>1</v>
+        <stp/>
+        <stp>5d50a53b-d5e1-4d22-b0a0-4797856031ad</stp>
+        <tr r="G22" s="7"/>
+      </tp>
+    </main>
+    <main first="rtdsrv.83aaa2cc90e24b62bd47ab1283cce962">
+      <tp>
+        <v>2</v>
+        <stp/>
+        <stp>c16130d5-4518-4fc7-98ff-6dee9ca5a62d</stp>
+        <tr r="G40" s="4"/>
+      </tp>
+    </main>
+    <main first="rtdsrv.83aaa2cc90e24b62bd47ab1283cce962">
+      <tp>
+        <v>2</v>
+        <stp/>
+        <stp>9b0683ca-f6b5-4a6e-a466-ee2a9ce56760</stp>
+        <tr r="G44" s="4"/>
+      </tp>
+      <tp>
+        <v>2</v>
+        <stp/>
+        <stp>d6b4dafa-ca11-4041-9f4a-45708f6bb743</stp>
+        <tr r="G20" s="4"/>
+      </tp>
+    </main>
+    <main first="rtdsrv.83aaa2cc90e24b62bd47ab1283cce962">
+      <tp>
+        <v>1</v>
+        <stp/>
+        <stp>b3c38031-d704-421a-95ab-964971d0d40f</stp>
+        <tr r="G5" s="3"/>
+      </tp>
+    </main>
+    <main first="rtdsrv.83aaa2cc90e24b62bd47ab1283cce962">
+      <tp>
+        <v>2</v>
+        <stp/>
+        <stp>7f042a02-1e97-420e-885a-9a95cf9e3532</stp>
+        <tr r="G20" s="1"/>
+      </tp>
+      <tp>
+        <v>2</v>
+        <stp/>
+        <stp>40b47595-09d8-4883-8d2b-1d5ec2e1f6df</stp>
+        <tr r="D15" s="5"/>
+      </tp>
+    </main>
+    <main first="rtdsrv.83aaa2cc90e24b62bd47ab1283cce962">
+      <tp>
+        <v>2</v>
+        <stp/>
+        <stp>c8ce3fc5-3698-404d-ba8d-5a2d67b580e9</stp>
+        <tr r="G47" s="4"/>
+      </tp>
+    </main>
+    <main first="rtdsrv.83aaa2cc90e24b62bd47ab1283cce962">
+      <tp>
+        <v>2</v>
+        <stp/>
+        <stp>afa8cb13-4010-45f3-8c36-1e364c078a77</stp>
+        <tr r="G30" s="1"/>
+      </tp>
+      <tp>
+        <v>2</v>
+        <stp/>
+        <stp>be60c153-8997-4a59-b75f-3ff57bc7438e</stp>
+        <tr r="G51" s="4"/>
+      </tp>
+      <tp>
+        <v>2</v>
+        <stp/>
+        <stp>77e8dc46-f3c5-4e6d-9bbd-3a2d730981d7</stp>
+        <tr r="G53" s="1"/>
+      </tp>
+      <tp>
+        <v>2</v>
+        <stp/>
+        <stp>2270fba7-2a34-4bfd-ac27-fabde0997241</stp>
+        <tr r="F1" s="1"/>
+      </tp>
+    </main>
+    <main first="rtdsrv.83aaa2cc90e24b62bd47ab1283cce962">
+      <tp>
+        <v>1</v>
+        <stp/>
+        <stp>8f9d736a-065b-4aa4-a082-0ef5abbd59f6</stp>
+        <tr r="F6" s="7"/>
+      </tp>
+      <tp>
+        <v>1</v>
+        <stp/>
+        <stp>4cde677b-3a9b-4788-b633-581f703f1308</stp>
+        <tr r="G4" s="3"/>
+      </tp>
+      <tp>
+        <v>2</v>
+        <stp/>
+        <stp>effd1f44-2e12-4994-a271-db7f9262c665</stp>
+        <tr r="G30" s="4"/>
+      </tp>
+      <tp>
+        <v>2</v>
+        <stp/>
+        <stp>ddb1e70f-5baa-4ae1-8bab-43d903b5aad1</stp>
+        <tr r="G28" s="1"/>
+      </tp>
+      <tp>
+        <v>1</v>
+        <stp/>
+        <stp>4d895941-1672-47c9-9b89-f30b2908a08a</stp>
+        <tr r="G55" s="7"/>
+      </tp>
+      <tp>
+        <v>2</v>
+        <stp/>
+        <stp>728689c8-f7a8-4d10-b688-4c764a4ca12f</stp>
+        <tr r="G37" s="1"/>
+      </tp>
+    </main>
+    <main first="rtdsrv.83aaa2cc90e24b62bd47ab1283cce962">
+      <tp>
+        <v>2</v>
+        <stp/>
+        <stp>3c048cf7-9f17-413b-a2f8-a4343f74a9b1</stp>
+        <tr r="G25" s="4"/>
+      </tp>
+    </main>
+    <main first="rtdsrv.83aaa2cc90e24b62bd47ab1283cce962">
+      <tp>
+        <v>1</v>
+        <stp/>
+        <stp>ca04e0d4-0988-4967-8b93-061c3753f82f</stp>
+        <tr r="G35" s="7"/>
+      </tp>
+      <tp>
+        <v>2</v>
+        <stp/>
+        <stp>5a39b747-d5a1-4fe8-9a80-6167eb3a8701</stp>
+        <tr r="P74" s="1"/>
+      </tp>
+      <tp>
+        <v>2</v>
+        <stp/>
+        <stp>cfb861b2-be8c-4a60-9ab0-bee2ff7bf20b</stp>
+        <tr r="G52" s="1"/>
+      </tp>
+      <tp>
+        <v>2</v>
+        <stp/>
+        <stp>a652de85-b9e4-4178-b103-23cad8203de8</stp>
+        <tr r="G35" s="4"/>
+      </tp>
+      <tp>
+        <v>2</v>
+        <stp/>
+        <stp>2d8eeeba-940b-418d-8289-d2a93674d63e</stp>
+        <tr r="F6" s="3"/>
+      </tp>
+    </main>
+    <main first="rtdsrv.83aaa2cc90e24b62bd47ab1283cce962">
+      <tp>
+        <v>2</v>
+        <stp/>
+        <stp>521585f4-87e8-4ea8-9c31-34f4f8c58a73</stp>
+        <tr r="G26" s="1"/>
+      </tp>
+    </main>
+    <main first="rtdsrv.83aaa2cc90e24b62bd47ab1283cce962">
+      <tp>
+        <v>1</v>
+        <stp/>
+        <stp>804be10c-f896-4b82-b1b9-90973f65c8fa</stp>
+        <tr r="G33" s="7"/>
+      </tp>
+      <tp>
+        <v>2</v>
+        <stp/>
+        <stp>50d4749e-8d82-47b4-9153-658e5b697300</stp>
+        <tr r="F7" s="3"/>
+      </tp>
+      <tp>
+        <v>2</v>
+        <stp/>
+        <stp>fe6346ae-1995-46b1-b016-517f533829c8</stp>
+        <tr r="G39" s="4"/>
+      </tp>
+      <tp>
+        <v>1</v>
+        <stp/>
+        <stp>06d2b4b8-bb38-4585-9ff9-d7f5fd392952</stp>
+        <tr r="G52" s="7"/>
+      </tp>
+    </main>
+    <main first="rtdsrv.83aaa2cc90e24b62bd47ab1283cce962">
+      <tp>
+        <v>2</v>
+        <stp/>
+        <stp>261951ad-d32a-4223-ad36-8d73192d2f37</stp>
+        <tr r="G34" s="1"/>
+      </tp>
+      <tp>
+        <v>2</v>
+        <stp/>
+        <stp>82cf6b27-9feb-4c95-ad57-2ad78cff23cb</stp>
+        <tr r="G48" s="4"/>
+      </tp>
+    </main>
+    <main first="rtdsrv.83aaa2cc90e24b62bd47ab1283cce962">
+      <tp>
+        <v>1</v>
+        <stp/>
+        <stp>41d5d345-c4e1-4ba7-8d4b-89b14784c468</stp>
+        <tr r="H6" s="3"/>
+      </tp>
+    </main>
+    <main first="rtdsrv.83aaa2cc90e24b62bd47ab1283cce962">
+      <tp>
+        <v>2</v>
+        <stp/>
+        <stp>9ad3795c-a5a1-4e7d-9f14-3f7934998fc7</stp>
+        <tr r="G52" s="4"/>
+      </tp>
+    </main>
+    <main first="rtdsrv.83aaa2cc90e24b62bd47ab1283cce962">
+      <tp>
+        <v>2</v>
+        <stp/>
+        <stp>c770669e-5e30-493f-9a41-a9a1c41ab320</stp>
+        <tr r="G36" s="1"/>
+      </tp>
+      <tp>
+        <v>2</v>
+        <stp/>
+        <stp>b6e72c8b-569c-450f-b6c5-7e449977eae7</stp>
+        <tr r="C10" s="6"/>
+      </tp>
+      <tp>
+        <v>1</v>
+        <stp/>
+        <stp>860b2f55-bdbd-4d54-ac3e-9fbe781d7099</stp>
+        <tr r="G49" s="7"/>
+      </tp>
+    </main>
+    <main first="rtdsrv.83aaa2cc90e24b62bd47ab1283cce962">
+      <tp>
+        <v>2</v>
+        <stp/>
+        <stp>4ff250ab-753e-4504-9f1b-95e9696ce37c</stp>
+        <tr r="G21" s="1"/>
+      </tp>
+    </main>
+    <main first="rtdsrv.83aaa2cc90e24b62bd47ab1283cce962">
+      <tp>
+        <v>2</v>
+        <stp/>
+        <stp>25225206-73de-4ec5-b781-0386afd6d3f2</stp>
+        <tr r="G24" s="4"/>
+      </tp>
+    </main>
+    <main first="rtdsrv.83aaa2cc90e24b62bd47ab1283cce962">
+      <tp>
+        <v>2</v>
+        <stp/>
+        <stp>460658cf-5a8b-4c00-8528-12e57c718290</stp>
+        <tr r="C2" s="2"/>
+      </tp>
+      <tp>
+        <v>2</v>
+        <stp/>
+        <stp>81559fed-c7c7-452c-aabf-79783ce95532</stp>
+        <tr r="G32" s="1"/>
+      </tp>
+      <tp>
+        <v>2</v>
+        <stp/>
+        <stp>f7900452-2601-4ca2-b955-d9b1b04b8e6f</stp>
+        <tr r="G42" s="1"/>
+      </tp>
+    </main>
+    <main first="rtdsrv.83aaa2cc90e24b62bd47ab1283cce962">
+      <tp>
+        <v>2</v>
+        <stp/>
+        <stp>78f24e7d-9eee-4279-bf94-54666998a3fa</stp>
+        <tr r="G46" s="1"/>
+      </tp>
+    </main>
+    <main first="rtdsrv.83aaa2cc90e24b62bd47ab1283cce962">
+      <tp>
+        <v>2</v>
+        <stp/>
+        <stp>9da6abb2-9e2a-4244-b5b3-0be944a9aed0</stp>
+        <tr r="F4" s="3"/>
+      </tp>
+    </main>
+    <main first="rtdsrv.83aaa2cc90e24b62bd47ab1283cce962">
+      <tp>
+        <v>2</v>
+        <stp/>
+        <stp>d3ab0b41-cd35-48f0-ae28-81110bc069e9</stp>
+        <tr r="G43" s="4"/>
+      </tp>
+      <tp>
+        <v>2</v>
+        <stp/>
+        <stp>664c82a6-975c-48a1-9c95-34b329bf8e83</stp>
+        <tr r="D20" s="5"/>
+      </tp>
+    </main>
+    <main first="rtdsrv.83aaa2cc90e24b62bd47ab1283cce962">
+      <tp>
+        <v>1</v>
+        <stp/>
+        <stp>b9f5addd-14ad-4bfb-88f4-c3413b6ddd2a</stp>
+        <tr r="P29" s="7"/>
+      </tp>
+      <tp>
+        <v>2</v>
+        <stp/>
+        <stp>202a6caa-4d36-4fe8-97a3-95529f637056</stp>
+        <tr r="G27" s="4"/>
+      </tp>
+      <tp>
+        <v>2</v>
+        <stp/>
+        <stp>3d4b3a8c-d8b9-4f08-8d15-8ee3be71c5af</stp>
+        <tr r="H5" s="5"/>
+      </tp>
+      <tp>
+        <v>1</v>
+        <stp/>
+        <stp>542c0d5e-e930-4832-8d18-984846478e70</stp>
+        <tr r="G32" s="7"/>
+      </tp>
+    </main>
+    <main first="rtdsrv.83aaa2cc90e24b62bd47ab1283cce962">
+      <tp>
+        <v>2</v>
+        <stp/>
+        <stp>62339259-8700-4371-88db-ba1504643d86</stp>
+        <tr r="G23" s="1"/>
+      </tp>
+      <tp>
+        <v>2</v>
+        <stp/>
+        <stp>47a5aad5-7e21-4b17-bc40-763801d6492c</stp>
+        <tr r="D5" s="3"/>
+      </tp>
+    </main>
+    <main first="rtdsrv.83aaa2cc90e24b62bd47ab1283cce962">
+      <tp>
+        <v>2</v>
+        <stp/>
+        <stp>ef462004-a430-4ab6-ba8e-c506e7c9eda6</stp>
+        <tr r="D25" s="5"/>
+      </tp>
+      <tp>
+        <v>1</v>
+        <stp/>
+        <stp>19f1bc79-01e9-4276-9842-e5b3ddd74f6a</stp>
+        <tr r="G24" s="7"/>
+      </tp>
+    </main>
+    <main first="rtdsrv.83aaa2cc90e24b62bd47ab1283cce962">
+      <tp>
+        <v>2</v>
+        <stp/>
+        <stp>c0ed8746-a0aa-4903-8a5c-1d9e0b05a9a1</stp>
+        <tr r="D4" s="3"/>
+      </tp>
+      <tp>
+        <v>2</v>
+        <stp/>
+        <stp>72440ac0-408c-4689-9208-875920581667</stp>
+        <tr r="G57" s="4"/>
+      </tp>
+    </main>
+    <main first="rtdsrv.83aaa2cc90e24b62bd47ab1283cce962">
+      <tp>
+        <v>2</v>
+        <stp/>
+        <stp>ce440cb2-7dfa-4123-b5b8-b917ee7d6c99</stp>
+        <tr r="I33" s="4"/>
+      </tp>
+    </main>
+    <main first="rtdsrv.83aaa2cc90e24b62bd47ab1283cce962">
+      <tp>
+        <v>2</v>
+        <stp/>
+        <stp>090239e0-1970-4333-8ba8-4ae3ad829977</stp>
+        <tr r="G34" s="4"/>
+      </tp>
+    </main>
+    <main first="rtdsrv.83aaa2cc90e24b62bd47ab1283cce962">
+      <tp>
+        <v>1</v>
+        <stp/>
+        <stp>92957b87-942a-4eb8-8892-0507a7b5846b</stp>
+        <tr r="G27" s="7"/>
+      </tp>
+    </main>
+    <main first="rtdsrv.83aaa2cc90e24b62bd47ab1283cce962">
+      <tp>
+        <v>1</v>
+        <stp/>
+        <stp>716f7f52-d2ca-42a4-a797-ac4ab49cf7c5</stp>
         <tr r="G38" s="7"/>
       </tp>
     </main>
-    <main first="rtdsrv.e91a2bf1ca1e4425853080e41816bb7b">
-      <tp>
-        <v>1</v>
-        <stp/>
-        <stp>7c0193f4-eda0-47a4-8cec-f11bfba640ea</stp>
-        <tr r="F1" s="7"/>
-      </tp>
-    </main>
-    <main first="rtdsrv.e91a2bf1ca1e4425853080e41816bb7b">
-      <tp>
-        <v>2</v>
-        <stp/>
-        <stp>5481a29e-2b05-4e83-980b-87127fd11a17</stp>
-        <tr r="D7" s="3"/>
-      </tp>
-    </main>
-    <main first="rtdsrv.e91a2bf1ca1e4425853080e41816bb7b">
-      <tp>
-        <v>2</v>
-        <stp/>
-        <stp>be7bf41e-40b6-45b0-a1f0-1510d2888211</stp>
-        <tr r="G49" s="4"/>
-      </tp>
-      <tp>
-        <v>1</v>
-        <stp/>
-        <stp>1e7a0e30-9363-45f7-896c-d14e788af7fa</stp>
-        <tr r="G44" s="7"/>
-      </tp>
-    </main>
-    <main first="rtdsrv.e91a2bf1ca1e4425853080e41816bb7b">
-      <tp>
-        <v>1</v>
-        <stp/>
-        <stp>1a475449-68b6-4707-bed3-d1a746f9d155</stp>
-        <tr r="G40" s="7"/>
-      </tp>
-    </main>
-    <main first="rtdsrv.e91a2bf1ca1e4425853080e41816bb7b">
-      <tp>
-        <v>2</v>
-        <stp/>
-        <stp>2ed23e70-63ba-468f-9807-60a2caab5757</stp>
-        <tr r="C10" s="6"/>
-      </tp>
-      <tp>
-        <v>1</v>
-        <stp/>
-        <stp>b38c1181-a49a-4320-865e-44644a685527</stp>
-        <tr r="G19" s="7"/>
-      </tp>
-      <tp>
-        <v>2</v>
-        <stp/>
-        <stp>f7183241-a8a5-4bcd-b516-540562cf7185</stp>
-        <tr r="G25" s="4"/>
-      </tp>
-      <tp>
-        <v>2</v>
-        <stp/>
-        <stp>8f73b731-4e5d-4ee1-92c1-1d7ef3bc5e85</stp>
-        <tr r="C6" s="6"/>
-      </tp>
-      <tp>
-        <v>2</v>
-        <stp/>
-        <stp>849de138-ae66-4bbb-b20d-d0acffaf6e1b</stp>
-        <tr r="G35" s="4"/>
-      </tp>
-    </main>
-    <main first="rtdsrv.e91a2bf1ca1e4425853080e41816bb7b">
-      <tp>
-        <v>1</v>
-        <stp/>
-        <stp>40176a28-c6a0-4609-be18-8958de2dac27</stp>
-        <tr r="H4" s="3"/>
-      </tp>
-    </main>
-    <main first="rtdsrv.e91a2bf1ca1e4425853080e41816bb7b">
-      <tp>
-        <v>2</v>
-        <stp/>
-        <stp>f13641b9-5075-4b03-a2d4-a5bb9a6ce38a</stp>
-        <tr r="F1" s="1"/>
-      </tp>
-      <tp>
-        <v>1</v>
-        <stp/>
-        <stp>672e9e28-eb76-482c-9738-33f952faaccc</stp>
-        <tr r="G34" s="7"/>
-      </tp>
-    </main>
-    <main first="rtdsrv.e91a2bf1ca1e4425853080e41816bb7b">
-      <tp>
-        <v>2</v>
-        <stp/>
-        <stp>122a563d-e2f6-4cbe-8ed1-0754f6b5ad8b</stp>
-        <tr r="B2" s="6"/>
-      </tp>
-    </main>
-    <main first="rtdsrv.e91a2bf1ca1e4425853080e41816bb7b">
-      <tp>
-        <v>2</v>
-        <stp/>
-        <stp>f026c58b-495e-4413-9240-edf8ec11046b</stp>
-        <tr r="P19" s="1"/>
-      </tp>
-    </main>
-    <main first="rtdsrv.e91a2bf1ca1e4425853080e41816bb7b">
-      <tp>
-        <v>2</v>
-        <stp/>
-        <stp>f3b4e123-8824-4580-812a-a4e8b1c10922</stp>
-        <tr r="G37" s="4"/>
-      </tp>
-      <tp>
-        <v>2</v>
-        <stp/>
-        <stp>a3e2faa5-2078-491c-bf53-79cda3f5b895</stp>
-        <tr r="D35" s="5"/>
-      </tp>
-      <tp>
-        <v>2</v>
-        <stp/>
-        <stp>d8e4bf55-986a-42f5-825c-c70721a26eb6</stp>
-        <tr r="G39" s="4"/>
-      </tp>
-      <tp>
-        <v>2</v>
-        <stp/>
-        <stp>630bc26c-5865-4ff2-a4fe-dcfd8dfbdcb1</stp>
-        <tr r="G51" s="4"/>
-      </tp>
-      <tp>
-        <v>1</v>
-        <stp/>
-        <stp>8711411f-c307-4607-a130-fd4138b899af</stp>
-        <tr r="G28" s="7"/>
-      </tp>
-      <tp>
-        <v>1</v>
-        <stp/>
-        <stp>fe3f49c9-8561-4026-9ccc-2a6e4fdc52af</stp>
-        <tr r="G54" s="7"/>
-      </tp>
-      <tp>
-        <v>2</v>
-        <stp/>
-        <stp>f0299d1d-0a16-4e80-8e74-bfcbb0a471ac</stp>
-        <tr r="G57" s="1"/>
-      </tp>
-    </main>
-    <main first="rtdsrv.e91a2bf1ca1e4425853080e41816bb7b">
-      <tp>
-        <v>1</v>
-        <stp/>
-        <stp>125a602d-9f8a-41ef-9999-80fd4ef3b2a8</stp>
-        <tr r="G42" s="7"/>
-      </tp>
-      <tp>
-        <v>2</v>
-        <stp/>
-        <stp>0cbe7bed-47ee-4269-ad98-40819b142d80</stp>
-        <tr r="G26" s="4"/>
-      </tp>
-      <tp>
-        <v>1</v>
-        <stp/>
-        <stp>c35e13b5-5f9e-4093-a42b-1b6a6cbbb612</stp>
-        <tr r="G26" s="7"/>
-      </tp>
-    </main>
-    <main first="rtdsrv.e91a2bf1ca1e4425853080e41816bb7b">
-      <tp>
-        <v>2</v>
-        <stp/>
-        <stp>4c74147e-fbac-4857-86fd-b05f52cceab0</stp>
-        <tr r="D5" s="3"/>
-      </tp>
-    </main>
-    <main first="rtdsrv.e91a2bf1ca1e4425853080e41816bb7b">
-      <tp>
-        <v>2</v>
-        <stp/>
-        <stp>7b83883b-8362-488e-9c7c-685a1855230f</stp>
-        <tr r="G38" s="4"/>
-      </tp>
-      <tp>
-        <v>1</v>
-        <stp/>
-        <stp>589c3e2b-5743-41b1-b30f-bb2a68e5e12b</stp>
-        <tr r="G35" s="7"/>
-      </tp>
-    </main>
-    <main first="rtdsrv.e91a2bf1ca1e4425853080e41816bb7b">
-      <tp>
-        <v>2</v>
-        <stp/>
-        <stp>9387df30-9c25-4727-a94d-9fade9ae8249</stp>
-        <tr r="G31" s="1"/>
-      </tp>
-    </main>
-    <main first="rtdsrv.e91a2bf1ca1e4425853080e41816bb7b">
-      <tp>
-        <v>2</v>
-        <stp/>
-        <stp>86c4e9d1-e75e-4b29-aca1-a3764bdafaf7</stp>
-        <tr r="G42" s="4"/>
-      </tp>
-    </main>
-    <main first="rtdsrv.e91a2bf1ca1e4425853080e41816bb7b">
-      <tp>
-        <v>2</v>
-        <stp/>
-        <stp>7c8990af-4f65-4721-9dee-717e7732778d</stp>
-        <tr r="G50" s="1"/>
-      </tp>
-      <tp>
-        <v>2</v>
-        <stp/>
-        <stp>62b83423-9913-49a4-9aef-6e9180a35921</stp>
-        <tr r="I38" s="4"/>
-      </tp>
-      <tp>
-        <v>1</v>
-        <stp/>
-        <stp>f52438f3-96eb-47c3-96d7-55c027d15c21</stp>
-        <tr r="G50" s="7"/>
-      </tp>
-      <tp>
-        <v>2</v>
-        <stp/>
-        <stp>89f06ee3-3e41-4885-999b-7bb4b34ec3c9</stp>
-        <tr r="D6" s="3"/>
-      </tp>
-      <tp>
-        <v>2</v>
-        <stp/>
-        <stp>d05e4422-6206-4ebd-942f-cb844dd06caf</stp>
-        <tr r="I33" s="4"/>
-      </tp>
-    </main>
-    <main first="rtdsrv.e91a2bf1ca1e4425853080e41816bb7b">
-      <tp>
-        <v>1</v>
-        <stp/>
-        <stp>55348686-3f0b-4d50-8e0e-17b28baebe40</stp>
-        <tr r="G8" s="3"/>
-      </tp>
-      <tp>
-        <v>2</v>
-        <stp/>
-        <stp>40fe8dfa-6aa7-4b25-b13d-c005cf40023e</stp>
-        <tr r="G29" s="4"/>
-      </tp>
-      <tp>
-        <v>2</v>
-        <stp/>
-        <stp>2a52ddad-7901-4190-b251-3723ded68ecc</stp>
-        <tr r="D8" s="3"/>
-      </tp>
-    </main>
-    <main first="rtdsrv.e91a2bf1ca1e4425853080e41816bb7b">
-      <tp>
-        <v>1</v>
-        <stp/>
-        <stp>fc33611f-3dc4-444c-b95c-62ca8274f72c</stp>
-        <tr r="H7" s="3"/>
-      </tp>
-    </main>
-    <main first="rtdsrv.e91a2bf1ca1e4425853080e41816bb7b">
-      <tp>
-        <v>2</v>
-        <stp/>
-        <stp>b17dc94d-4063-4b8e-8a35-9612b79b4d93</stp>
-        <tr r="G50" s="4"/>
-      </tp>
-    </main>
-    <main first="rtdsrv.e91a2bf1ca1e4425853080e41816bb7b">
-      <tp>
-        <v>1</v>
-        <stp/>
-        <stp>3d9885e6-45bd-49e1-9a8f-5269b3b82b34</stp>
-        <tr r="G32" s="7"/>
-      </tp>
-    </main>
-    <main first="rtdsrv.e91a2bf1ca1e4425853080e41816bb7b">
-      <tp>
-        <v>2</v>
-        <stp/>
-        <stp>b9791b92-c539-49c7-8d1c-dc6bb2491ad7</stp>
-        <tr r="G19" s="1"/>
-      </tp>
-    </main>
-    <main first="rtdsrv.e91a2bf1ca1e4425853080e41816bb7b">
-      <tp>
-        <v>1</v>
-        <stp/>
-        <stp>375be6c5-9016-4637-bbb2-b0f17a63129e</stp>
-        <tr r="G7" s="3"/>
-      </tp>
-      <tp>
-        <v>2</v>
-        <stp/>
-        <stp>09ef696a-87c2-4bc4-99ba-8ae75d8f0ebe</stp>
-        <tr r="G55" s="4"/>
-      </tp>
-      <tp>
-        <v>2</v>
-        <stp/>
-        <stp>dee96407-8c90-4763-84ed-639385e4b775</stp>
-        <tr r="G37" s="1"/>
-      </tp>
-    </main>
-    <main first="rtdsrv.e91a2bf1ca1e4425853080e41816bb7b">
-      <tp>
-        <v>1</v>
-        <stp/>
-        <stp>db9abfd2-6edf-477a-8e07-8cc04871267b</stp>
-        <tr r="G47" s="7"/>
-      </tp>
-      <tp>
-        <v>2</v>
-        <stp/>
-        <stp>a172ed83-87a8-4cfb-8940-a3fb2c0c0e26</stp>
-        <tr r="F1" s="4"/>
-      </tp>
-      <tp>
-        <v>2</v>
-        <stp/>
-        <stp>fb8e0de9-d16b-4268-8ad6-bfaa7a7377af</stp>
-        <tr r="G56" s="1"/>
-      </tp>
-      <tp>
-        <v>1</v>
-        <stp/>
-        <stp>a89691df-8775-426d-97db-39b01eb12ccd</stp>
-        <tr r="G4" s="3"/>
-      </tp>
-      <tp>
-        <v>2</v>
-        <stp/>
-        <stp>45bd4d6a-f652-4c88-96b9-714d4b7a0011</stp>
-        <tr r="G20" s="4"/>
-      </tp>
-    </main>
-    <main first="rtdsrv.e91a2bf1ca1e4425853080e41816bb7b">
-      <tp>
-        <v>2</v>
-        <stp/>
-        <stp>9e1e2108-f142-4a0f-88ba-b020e28539f4</stp>
-        <tr r="G28" s="4"/>
-      </tp>
-    </main>
-    <main first="rtdsrv.e91a2bf1ca1e4425853080e41816bb7b">
-      <tp>
-        <v>1</v>
-        <stp/>
-        <stp>6fdf178b-a857-47c2-8888-fc8881deae2b</stp>
-        <tr r="G33" s="7"/>
-      </tp>
-    </main>
-    <main first="rtdsrv.e91a2bf1ca1e4425853080e41816bb7b">
-      <tp>
-        <v>1</v>
-        <stp/>
-        <stp>ffbe8731-f4fd-4568-86ff-efdec4ed16ab</stp>
-        <tr r="I28" s="7"/>
-      </tp>
-      <tp>
-        <v>2</v>
-        <stp/>
-        <stp>ead5256c-7c1b-42f4-bd99-9bc890361187</stp>
-        <tr r="F6" s="3"/>
-      </tp>
-      <tp>
-        <v>1</v>
-        <stp/>
-        <stp>816db770-d1de-45da-8b86-359efa0fbc21</stp>
-        <tr r="G41" s="7"/>
-      </tp>
-      <tp>
-        <v>1</v>
-        <stp/>
-        <stp>07bcb521-e3dc-4b6c-a3e9-4bd08722d88c</stp>
-        <tr r="G27" s="7"/>
-      </tp>
-    </main>
-    <main first="rtdsrv.e91a2bf1ca1e4425853080e41816bb7b">
-      <tp>
-        <v>1</v>
-        <stp/>
-        <stp>a086a178-18a3-417f-a83c-a5c6be7d9938</stp>
-        <tr r="G6" s="3"/>
-      </tp>
-      <tp>
-        <v>2</v>
-        <stp/>
-        <stp>4cec28f3-cd5a-4189-b49d-fe0f3f6b4750</stp>
-        <tr r="G27" s="4"/>
-      </tp>
-      <tp>
-        <v>2</v>
-        <stp/>
-        <stp>06508cd3-e3a6-4c3b-a716-35c7684acb31</stp>
-        <tr r="D45" s="5"/>
-      </tp>
-    </main>
-    <main first="rtdsrv.e91a2bf1ca1e4425853080e41816bb7b">
-      <tp>
-        <v>2</v>
-        <stp/>
-        <stp>49a04724-098f-4100-a6a1-8a2df247c7ca</stp>
-        <tr r="G40" s="4"/>
-      </tp>
-      <tp>
-        <v>2</v>
-        <stp/>
-        <stp>2e48e8ca-aa73-478f-a16f-f674fba46392</stp>
-        <tr r="G23" s="1"/>
-      </tp>
-      <tp>
-        <v>2</v>
-        <stp/>
-        <stp>6aa75921-65ad-4b07-ade2-cb1333cb1f98</stp>
-        <tr r="G34" s="1"/>
-      </tp>
-    </main>
-    <main first="rtdsrv.e91a2bf1ca1e4425853080e41816bb7b">
-      <tp>
-        <v>2</v>
-        <stp/>
-        <stp>3667a29f-ef97-4a03-9836-2a8a12fd692f</stp>
-        <tr r="G57" s="4"/>
-      </tp>
-    </main>
-    <main first="rtdsrv.e91a2bf1ca1e4425853080e41816bb7b">
-      <tp>
-        <v>2</v>
-        <stp/>
-        <stp>980c0fb5-b348-4820-af35-b1bb76f4e392</stp>
-        <tr r="G21" s="4"/>
-      </tp>
-    </main>
-    <main first="rtdsrv.e91a2bf1ca1e4425853080e41816bb7b">
-      <tp>
-        <v>2</v>
-        <stp/>
-        <stp>a8582a43-4f2f-4f60-b02d-bfad376af510</stp>
-        <tr r="H5" s="5"/>
-      </tp>
-    </main>
-    <main first="rtdsrv.e91a2bf1ca1e4425853080e41816bb7b">
-      <tp>
-        <v>2</v>
-        <stp/>
-        <stp>5153b8b4-caf6-4405-afb1-8694a5eb458f</stp>
-        <tr r="G32" s="4"/>
-      </tp>
-    </main>
-    <main first="rtdsrv.e91a2bf1ca1e4425853080e41816bb7b">
-      <tp>
-        <v>2</v>
-        <stp/>
-        <stp>abeb2d7b-a6aa-461b-b688-87a78ef61ee8</stp>
-        <tr r="G20" s="1"/>
-      </tp>
-    </main>
-    <main first="rtdsrv.e91a2bf1ca1e4425853080e41816bb7b">
-      <tp>
-        <v>2</v>
-        <stp/>
-        <stp>e0247dd1-819d-4ed4-8acc-8cf60a1003c9</stp>
-        <tr r="D40" s="5"/>
-      </tp>
-      <tp>
-        <v>1</v>
-        <stp/>
-        <stp>9eca985a-67bb-4bc0-b3bb-701052c651a0</stp>
-        <tr r="G24" s="7"/>
-      </tp>
-    </main>
-    <main first="rtdsrv.e91a2bf1ca1e4425853080e41816bb7b">
-      <tp>
-        <v>1</v>
-        <stp/>
-        <stp>ece48c6e-8326-4ad0-95d2-6f2a221c7257</stp>
-        <tr r="G52" s="7"/>
-      </tp>
-    </main>
-    <main first="rtdsrv.e91a2bf1ca1e4425853080e41816bb7b">
-      <tp>
-        <v>2</v>
-        <stp/>
-        <stp>88ccba31-420d-4acf-9ec9-ba91cf3f2e15</stp>
-        <tr r="G32" s="1"/>
-      </tp>
-      <tp>
-        <v>1</v>
-        <stp/>
-        <stp>08f5f323-2ea5-4faa-a7fc-a95999a444f4</stp>
-        <tr r="G55" s="7"/>
-      </tp>
-      <tp>
-        <v>1</v>
-        <stp/>
-        <stp>84c4c9e8-0355-417b-84af-7634d3fb8283</stp>
-        <tr r="G30" s="7"/>
-      </tp>
-      <tp>
-        <v>1</v>
-        <stp/>
-        <stp>b831ac8d-046f-428f-8fac-702a80649ed2</stp>
-        <tr r="G5" s="3"/>
-      </tp>
-      <tp>
-        <v>2</v>
-        <stp/>
-        <stp>ded141e6-fe97-4c48-83e8-936d27eb6b2e</stp>
-        <tr r="G41" s="4"/>
-      </tp>
-    </main>
-    <main first="rtdsrv.e91a2bf1ca1e4425853080e41816bb7b">
-      <tp>
-        <v>1</v>
-        <stp/>
-        <stp>1fd46bd6-eb4d-4eba-be8f-f5193bd36ffc</stp>
-        <tr r="H5" s="3"/>
-      </tp>
-    </main>
-    <main first="rtdsrv.e91a2bf1ca1e4425853080e41816bb7b">
-      <tp>
-        <v>2</v>
-        <stp/>
-        <stp>0e541858-15ef-4685-89b8-9a88d1aebba4</stp>
-        <tr r="I28" s="1"/>
-      </tp>
-    </main>
-    <main first="rtdsrv.e91a2bf1ca1e4425853080e41816bb7b">
-      <tp>
-        <v>2</v>
-        <stp/>
-        <stp>280945b5-761a-4b65-aee9-e82618c3acc2</stp>
-        <tr r="D50" s="5"/>
-      </tp>
-      <tp>
-        <v>1</v>
-        <stp/>
-        <stp>f96780a5-8d6e-4507-8c1d-b2e018a8644b</stp>
-        <tr r="G51" s="7"/>
-      </tp>
-    </main>
-    <main first="rtdsrv.e91a2bf1ca1e4425853080e41816bb7b">
-      <tp>
-        <v>2</v>
-        <stp/>
-        <stp>56e9ee2d-ae92-4fee-8ccc-81b26562783e</stp>
-        <tr r="G22" s="4"/>
-      </tp>
-    </main>
-    <main first="rtdsrv.e91a2bf1ca1e4425853080e41816bb7b">
-      <tp>
-        <v>2</v>
-        <stp/>
-        <stp>88bc3314-4495-4b8c-a4e9-8c251a73531a</stp>
-        <tr r="G53" s="1"/>
-      </tp>
-      <tp>
-        <v>2</v>
-        <stp/>
-        <stp>daee27e1-135c-4c38-9743-dc6fede65d11</stp>
-        <tr r="G48" s="1"/>
-      </tp>
-      <tp>
-        <v>2</v>
-        <stp/>
-        <stp>803d85a0-df34-4c3a-bca2-ac9fe6462c5a</stp>
-        <tr r="G47" s="4"/>
-      </tp>
-    </main>
-    <main first="rtdsrv.e91a2bf1ca1e4425853080e41816bb7b">
-      <tp>
-        <v>2</v>
-        <stp/>
-        <stp>b72de556-e764-409c-84ac-b4a124883231</stp>
-        <tr r="G34" s="4"/>
-      </tp>
-    </main>
-    <main first="rtdsrv.e91a2bf1ca1e4425853080e41816bb7b">
-      <tp>
-        <v>2</v>
-        <stp/>
-        <stp>780a5e52-af70-4cc1-9cab-a1c833d06939</stp>
-        <tr r="G33" s="1"/>
-      </tp>
-    </main>
-    <main first="rtdsrv.e91a2bf1ca1e4425853080e41816bb7b">
-      <tp>
-        <v>2</v>
-        <stp/>
-        <stp>7f9f530a-f2f4-4b02-bba3-a3e0221f2633</stp>
-        <tr r="G46" s="1"/>
-      </tp>
-    </main>
-    <main first="rtdsrv.e91a2bf1ca1e4425853080e41816bb7b">
-      <tp>
-        <v>2</v>
-        <stp/>
-        <stp>02a1a1e0-f7e3-4b0d-93b6-d124e36196fa</stp>
-        <tr r="D15" s="5"/>
-      </tp>
-      <tp>
-        <v>2</v>
-        <stp/>
-        <stp>c3e774ee-7c75-4828-a8b1-6d9bca54389e</stp>
-        <tr r="G38" s="1"/>
-      </tp>
-      <tp>
-        <v>2</v>
-        <stp/>
-        <stp>ca3ac737-133d-4892-a5a1-cc9532fd1299</stp>
-        <tr r="G33" s="4"/>
-      </tp>
-    </main>
-    <main first="rtdsrv.e91a2bf1ca1e4425853080e41816bb7b">
-      <tp>
-        <v>1</v>
-        <stp/>
-        <stp>bb5b7681-0456-49b7-9ac0-cfe6f1b7b184</stp>
-        <tr r="G37" s="7"/>
-      </tp>
-    </main>
-    <main first="rtdsrv.e91a2bf1ca1e4425853080e41816bb7b">
-      <tp>
-        <v>2</v>
-        <stp/>
-        <stp>5ed70c66-31db-48b0-872d-4b3aa6e595f0</stp>
-        <tr r="G36" s="4"/>
-      </tp>
-    </main>
-    <main first="rtdsrv.e91a2bf1ca1e4425853080e41816bb7b">
-      <tp>
-        <v>2</v>
-        <stp/>
-        <stp>0545b6c7-2921-4fcb-88c8-9aded2b875e6</stp>
-        <tr r="G49" s="1"/>
-      </tp>
-    </main>
-    <main first="rtdsrv.e91a2bf1ca1e4425853080e41816bb7b">
-      <tp>
-        <v>2</v>
-        <stp/>
-        <stp>8e3c1621-e367-48e7-a7ba-af43b2248a31</stp>
-        <tr r="G44" s="1"/>
-      </tp>
-      <tp>
-        <v>2</v>
-        <stp/>
-        <stp>ab551407-8702-43f6-ab37-d7c1638c0985</stp>
-        <tr r="G35" s="1"/>
-      </tp>
-      <tp>
-        <v>1</v>
-        <stp/>
-        <stp>b3ddb51f-a888-4ce2-a56e-8dc420496a88</stp>
-        <tr r="P19" s="7"/>
-      </tp>
-    </main>
-    <main first="rtdsrv.e91a2bf1ca1e4425853080e41816bb7b">
-      <tp>
-        <v>2</v>
-        <stp/>
-        <stp>bcda11bb-56fd-41c7-af62-eba232391ccf</stp>
-        <tr r="B5" s="5"/>
-      </tp>
-      <tp>
-        <v>2</v>
-        <stp/>
-        <stp>f27b0066-4167-4ae3-b27b-c4b251a75bb2</stp>
-        <tr r="D30" s="5"/>
-      </tp>
-      <tp>
-        <v>2</v>
-        <stp/>
-        <stp>1a9fed76-60fc-4da6-9f3e-6cf87d8c4d5c</stp>
-        <tr r="G45" s="4"/>
-      </tp>
-    </main>
-    <main first="rtdsrv.e91a2bf1ca1e4425853080e41816bb7b">
-      <tp>
-        <v>1</v>
-        <stp/>
-        <stp>982b784e-48a6-459a-8240-54baec0dcc1e</stp>
-        <tr r="G22" s="7"/>
-      </tp>
-      <tp>
-        <v>2</v>
-        <stp/>
-        <stp>33a39252-a7e1-4921-8445-c1166799964f</stp>
-        <tr r="G28" s="1"/>
-      </tp>
-      <tp>
-        <v>1</v>
-        <stp/>
-        <stp>e068f5c0-c1d7-4736-a4b2-6e67b0544229</stp>
-        <tr r="G20" s="7"/>
-      </tp>
-      <tp>
-        <v>2</v>
-        <stp/>
-        <stp>9445c45b-13e2-4067-83f2-1a5edeaf9172</stp>
-        <tr r="D20" s="5"/>
-      </tp>
-      <tp>
-        <v>2</v>
-        <stp/>
-        <stp>6a7d72ee-170a-4eb4-af66-ab65dfa401db</stp>
-        <tr r="F7" s="3"/>
-      </tp>
-      <tp>
-        <v>2</v>
-        <stp/>
-        <stp>ea5690f0-c08b-44fd-8930-3ded9113cef3</stp>
-        <tr r="G54" s="1"/>
-      </tp>
-    </main>
-    <main first="rtdsrv.e91a2bf1ca1e4425853080e41816bb7b">
-      <tp>
-        <v>1</v>
-        <stp/>
-        <stp>dad37e2f-6ff2-4ad7-89f2-b1d7610727cc</stp>
-        <tr r="F6" s="7"/>
-      </tp>
-    </main>
-    <main first="rtdsrv.e91a2bf1ca1e4425853080e41816bb7b">
-      <tp>
-        <v>2</v>
-        <stp/>
-        <stp>6f15ca21-eeef-4d92-953f-b6eca5a7c4bd</stp>
-        <tr r="G55" s="1"/>
-      </tp>
-    </main>
-    <main first="rtdsrv.e91a2bf1ca1e4425853080e41816bb7b">
-      <tp>
-        <v>1</v>
-        <stp/>
-        <stp>d4a82a9f-6ab7-45ed-b903-cca4a852f89e</stp>
-        <tr r="G21" s="7"/>
-      </tp>
-    </main>
-    <main first="rtdsrv.e91a2bf1ca1e4425853080e41816bb7b">
-      <tp>
-        <v>1</v>
-        <stp/>
-        <stp>2d831470-fb21-4ef4-ba8a-a4d229c6bd27</stp>
-        <tr r="G49" s="7"/>
-      </tp>
-    </main>
-    <main first="rtdsrv.e91a2bf1ca1e4425853080e41816bb7b">
-      <tp>
-        <v>2</v>
-        <stp/>
-        <stp>2feaffaf-2642-4579-a7dc-875b131928fe</stp>
-        <tr r="I42" s="4"/>
-      </tp>
-      <tp>
-        <v>2</v>
-        <stp/>
-        <stp>11764cbb-1e2f-430a-9267-6a4d618a778e</stp>
-        <tr r="G52" s="1"/>
-      </tp>
-      <tp>
-        <v>1</v>
-        <stp/>
-        <stp>64aa74f5-2d77-4355-a3de-b1b7ec6d8bb6</stp>
-        <tr r="G31" s="7"/>
-      </tp>
-    </main>
-    <main first="rtdsrv.e91a2bf1ca1e4425853080e41816bb7b">
-      <tp>
-        <v>2</v>
-        <stp/>
-        <stp>8bd127b9-4752-45e4-ad4f-7d8fbdebb2e9</stp>
-        <tr r="G25" s="1"/>
-      </tp>
-      <tp>
-        <v>1</v>
-        <stp/>
-        <stp>0b3f895f-92df-4edf-89bc-45d1c4e23498</stp>
-        <tr r="G23" s="7"/>
-      </tp>
-    </main>
-    <main first="rtdsrv.e91a2bf1ca1e4425853080e41816bb7b">
-      <tp>
-        <v>1</v>
-        <stp/>
-        <stp>659027a3-0ddd-4f1b-a507-d29b71d5100f</stp>
-        <tr r="G36" s="7"/>
-      </tp>
-      <tp>
-        <v>2</v>
-        <stp/>
-        <stp>e09fdb37-b9cb-4f52-957d-f6b47240abc6</stp>
-        <tr r="C2" s="2"/>
-      </tp>
-    </main>
-    <main first="rtdsrv.e91a2bf1ca1e4425853080e41816bb7b">
-      <tp>
-        <v>2</v>
-        <stp/>
-        <stp>ff1e2d00-b307-49fc-a9a0-937c70d0f226</stp>
-        <tr r="G23" s="4"/>
-      </tp>
-    </main>
-    <main first="rtdsrv.e91a2bf1ca1e4425853080e41816bb7b">
-      <tp>
-        <v>2</v>
-        <stp/>
-        <stp>c051a473-ff27-499e-874c-e270c67e9dd7</stp>
-        <tr r="G39" s="1"/>
-      </tp>
-      <tp>
-        <v>2</v>
-        <stp/>
-        <stp>48efdd40-2dc5-45f3-8fa5-23ca4eadf9bc</stp>
-        <tr r="D4" s="3"/>
-      </tp>
-    </main>
-    <main first="rtdsrv.e91a2bf1ca1e4425853080e41816bb7b">
-      <tp>
-        <v>1</v>
-        <stp/>
-        <stp>49f80794-5b5e-4fb8-acfc-3c0a46f70b08</stp>
-        <tr r="P29" s="7"/>
-      </tp>
-      <tp>
-        <v>2</v>
-        <stp/>
-        <stp>7c3f3146-a0f2-4e8a-a752-1c4ccf431014</stp>
-        <tr r="G26" s="1"/>
-      </tp>
-    </main>
-    <main first="rtdsrv.e91a2bf1ca1e4425853080e41816bb7b">
-      <tp>
-        <v>2</v>
-        <stp/>
-        <stp>8db3c620-0d68-4efb-bc1c-ef6d5de9ead3</stp>
-        <tr r="I19" s="1"/>
-      </tp>
-      <tp>
-        <v>2</v>
-        <stp/>
-        <stp>5d527713-f32b-4137-bd27-6d368a835d73</stp>
-        <tr r="G51" s="1"/>
-      </tp>
-      <tp>
-        <v>2</v>
-        <stp/>
-        <stp>b0659a46-a5a3-45ff-8201-049a46748520</stp>
-        <tr r="G21" s="1"/>
-      </tp>
-    </main>
-    <main first="rtdsrv.e91a2bf1ca1e4425853080e41816bb7b">
-      <tp>
-        <v>2</v>
-        <stp/>
-        <stp>fea94141-54b1-4c62-8fdf-50571e07f36d</stp>
-        <tr r="I28" s="4"/>
-      </tp>
-      <tp>
-        <v>2</v>
-        <stp/>
-        <stp>f0c4da8d-6acc-4984-95b4-2d1a009a0429</stp>
-        <tr r="G27" s="1"/>
-      </tp>
-    </main>
-    <main first="rtdsrv.e91a2bf1ca1e4425853080e41816bb7b">
-      <tp>
-        <v>1</v>
-        <stp/>
-        <stp>25c6bf0e-eb84-4137-a21b-3366a7a1de77</stp>
-        <tr r="G56" s="7"/>
-      </tp>
-    </main>
-    <main first="rtdsrv.e91a2bf1ca1e4425853080e41816bb7b">
-      <tp>
-        <v>2</v>
-        <stp/>
-        <stp>2c9dbaf7-ff4d-47bb-ab4e-2d7507fdd156</stp>
-        <tr r="G47" s="1"/>
-      </tp>
-    </main>
-    <main first="rtdsrv.e91a2bf1ca1e4425853080e41816bb7b">
-      <tp>
-        <v>1</v>
-        <stp/>
-        <stp>1aeed1e9-aa44-497b-ac03-91a760541244</stp>
-        <tr r="H8" s="3"/>
-      </tp>
-    </main>
-    <main first="rtdsrv.e91a2bf1ca1e4425853080e41816bb7b">
-      <tp>
-        <v>2</v>
-        <stp/>
-        <stp>a855ad58-8793-4358-b2da-582a4b47c297</stp>
-        <tr r="G53" s="4"/>
-      </tp>
-      <tp>
-        <v>2</v>
-        <stp/>
-        <stp>47ca01c6-4e3e-4763-8902-5dd767fd6208</stp>
-        <tr r="G31" s="4"/>
-      </tp>
-      <tp>
-        <v>2</v>
-        <stp/>
-        <stp>8cce1b30-e8a1-4fca-8324-58153dd58478</stp>
-        <tr r="G54" s="4"/>
-      </tp>
-    </main>
-    <main first="rtdsrv.e91a2bf1ca1e4425853080e41816bb7b">
-      <tp>
-        <v>2</v>
-        <stp/>
-        <stp>f90b7290-071e-43ac-a632-54ccd5bfb50c</stp>
-        <tr r="G24" s="4"/>
-      </tp>
-      <tp>
-        <v>1</v>
-        <stp/>
-        <stp>1d8cb5ba-6afc-4206-8485-3c2edb6c073a</stp>
-        <tr r="G29" s="7"/>
-      </tp>
-      <tp>
-        <v>2</v>
-        <stp/>
-        <stp>ee458c4d-70c4-4d53-bf75-3c361995c086</stp>
-        <tr r="G48" s="4"/>
-      </tp>
-    </main>
-    <main first="rtdsrv.e91a2bf1ca1e4425853080e41816bb7b">
-      <tp>
-        <v>1</v>
-        <stp/>
-        <stp>c5a16031-d5c2-45ab-9273-f90484fb3fac</stp>
+    <main first="rtdsrv.83aaa2cc90e24b62bd47ab1283cce962">
+      <tp>
+        <v>1</v>
+        <stp/>
+        <stp>8d3b9ff1-8eb7-4055-bb3c-fce76481357a</stp>
         <tr r="G57" s="7"/>
-      </tp>
-    </main>
-    <main first="rtdsrv.e91a2bf1ca1e4425853080e41816bb7b">
-      <tp>
-        <v>2</v>
-        <stp/>
-        <stp>1d962afc-24b1-4218-b6dc-6f4c52136a2b</stp>
-        <tr r="G41" s="1"/>
-      </tp>
-      <tp>
-        <v>2</v>
-        <stp/>
-        <stp>c54cb856-929c-47cf-825e-f340a39bb9f9</stp>
-        <tr r="I32" s="4"/>
-        <tr r="I19" s="4"/>
-      </tp>
-      <tp>
-        <v>1</v>
-        <stp/>
-        <stp>17c7f19d-a193-4512-8480-0cf4eb09d282</stp>
-        <tr r="H6" s="3"/>
-      </tp>
-    </main>
-    <main first="rtdsrv.e91a2bf1ca1e4425853080e41816bb7b">
-      <tp>
-        <v>1</v>
-        <stp/>
-        <stp>b45f8936-b007-49ba-8d78-912b3ea6f310</stp>
-        <tr r="G25" s="7"/>
-      </tp>
-    </main>
-    <main first="rtdsrv.e91a2bf1ca1e4425853080e41816bb7b">
-      <tp>
-        <v>2</v>
-        <stp/>
-        <stp>632f156c-8d26-4f9e-b499-94601978d127</stp>
-        <tr r="G52" s="4"/>
-      </tp>
-      <tp>
-        <v>2</v>
-        <stp/>
-        <stp>110785ba-36e4-4607-bc85-8f3186bc06d3</stp>
-        <tr r="G46" s="4"/>
-      </tp>
-      <tp>
-        <v>1</v>
-        <stp/>
-        <stp>892969df-8a5a-4075-94d2-2ea577e3aed1</stp>
-        <tr r="G45" s="7"/>
-      </tp>
-    </main>
-    <main first="rtdsrv.e91a2bf1ca1e4425853080e41816bb7b">
-      <tp>
-        <v>2</v>
-        <stp/>
-        <stp>2cab6761-c25b-43c0-94db-a2bb290675f1</stp>
-        <tr r="F6" s="4"/>
-      </tp>
-      <tp>
-        <v>2</v>
-        <stp/>
-        <stp>d830ea8e-cebd-4055-b387-18ae9a86a335</stp>
-        <tr r="G40" s="1"/>
-      </tp>
-    </main>
-    <main first="rtdsrv.e91a2bf1ca1e4425853080e41816bb7b">
-      <tp>
-        <v>2</v>
-        <stp/>
-        <stp>88202da2-efbd-4eb8-9bb4-c889e79541fc</stp>
-        <tr r="G24" s="1"/>
-      </tp>
-      <tp>
-        <v>2</v>
-        <stp/>
-        <stp>7a801bdd-1969-4439-9217-46d5d0fe8a33</stp>
-        <tr r="P29" s="1"/>
-      </tp>
-    </main>
-    <main first="rtdsrv.e91a2bf1ca1e4425853080e41816bb7b">
-      <tp>
-        <v>2</v>
-        <stp/>
-        <stp>6d7ff179-dca0-465e-9679-c85a947003cb</stp>
-        <tr r="G56" s="4"/>
-      </tp>
-    </main>
-    <main first="rtdsrv.e91a2bf1ca1e4425853080e41816bb7b">
-      <tp>
-        <v>2</v>
-        <stp/>
-        <stp>2a7416b4-4f6c-400d-9cab-2533e6d2394c</stp>
-        <tr r="D25" s="5"/>
-      </tp>
-      <tp>
-        <v>2</v>
-        <stp/>
-        <stp>f847316d-048e-476c-a9dc-d06f57e90e50</stp>
-        <tr r="G29" s="1"/>
-      </tp>
-      <tp>
-        <v>2</v>
-        <stp/>
-        <stp>3518c879-97ad-446f-ad9b-851b0dbc0f03</stp>
-        <tr r="G30" s="1"/>
-      </tp>
-    </main>
-    <main first="rtdsrv.e91a2bf1ca1e4425853080e41816bb7b">
-      <tp>
-        <v>2</v>
-        <stp/>
-        <stp>a70e9c66-6f5d-4975-b287-b401e442c394</stp>
-        <tr r="G45" s="1"/>
-      </tp>
-    </main>
-    <main first="rtdsrv.e91a2bf1ca1e4425853080e41816bb7b">
-      <tp>
-        <v>1</v>
-        <stp/>
-        <stp>e832e3d5-9a86-4f66-8198-5d203c20ca9d</stp>
-        <tr r="G43" s="7"/>
-      </tp>
-      <tp>
-        <v>1</v>
-        <stp/>
-        <stp>f3aa15cd-4dad-4112-a78e-e5e88da8a231</stp>
-        <tr r="G48" s="7"/>
-      </tp>
-    </main>
-    <main first="rtdsrv.e91a2bf1ca1e4425853080e41816bb7b">
-      <tp>
-        <v>2</v>
-        <stp/>
-        <stp>5beca35a-4ce1-4829-8b54-3a4ce23adaef</stp>
-        <tr r="G44" s="4"/>
-      </tp>
-      <tp>
-        <v>2</v>
-        <stp/>
-        <stp>16a7220e-00ca-429a-932c-7dc92a15c93c</stp>
-        <tr r="G22" s="1"/>
-      </tp>
-    </main>
-    <main first="rtdsrv.e91a2bf1ca1e4425853080e41816bb7b">
-      <tp>
-        <v>1</v>
-        <stp/>
-        <stp>2425e602-f6fd-46ea-a4ca-0932c0f2b54d</stp>
-        <tr r="G39" s="7"/>
-      </tp>
-      <tp>
-        <v>2</v>
-        <stp/>
-        <stp>545b3ea1-0f7d-4286-b753-e95f2dc37ecd</stp>
-        <tr r="G43" s="1"/>
-      </tp>
-    </main>
-    <main first="rtdsrv.e91a2bf1ca1e4425853080e41816bb7b">
-      <tp>
-        <v>1</v>
-        <stp/>
-        <stp>fe569efc-4812-4199-bb2a-b65f6c6aa0d4</stp>
-        <tr r="G53" s="7"/>
-      </tp>
-      <tp>
-        <v>2</v>
-        <stp/>
-        <stp>794bfc42-730b-42e2-b2bc-3a04408e1621</stp>
-        <tr r="G36" s="1"/>
-      </tp>
-    </main>
-    <main first="rtdsrv.e91a2bf1ca1e4425853080e41816bb7b">
-      <tp>
-        <v>2</v>
-        <stp/>
-        <stp>0323dba1-868e-4bbf-8f30-6776635cdb59</stp>
-        <tr r="G30" s="4"/>
-      </tp>
-      <tp>
-        <v>2</v>
-        <stp/>
-        <stp>da3140d5-2543-425b-b003-ba2011d9c809</stp>
-        <tr r="F8" s="3"/>
-      </tp>
-      <tp>
-        <v>1</v>
-        <stp/>
-        <stp>7eeb9f54-e650-4532-b266-3e737fc5180e</stp>
-        <tr r="G46" s="7"/>
-      </tp>
-    </main>
-    <main first="rtdsrv.e91a2bf1ca1e4425853080e41816bb7b">
-      <tp>
-        <v>2</v>
-        <stp/>
-        <stp>9d2ea3c5-6a8c-45fc-a388-7250c4fcae53</stp>
-        <tr r="G43" s="4"/>
-      </tp>
-      <tp>
-        <v>1</v>
-        <stp/>
-        <stp>ac3d5812-c37a-470c-b241-348700fa3206</stp>
-        <tr r="I19" s="7"/>
-      </tp>
-    </main>
-    <main first="rtdsrv.e91a2bf1ca1e4425853080e41816bb7b">
-      <tp>
-        <v>2</v>
-        <stp/>
-        <stp>01694f3a-a023-4d9e-bbe9-577f39d89a6d</stp>
-        <tr r="F4" s="3"/>
-      </tp>
-      <tp>
-        <v>2</v>
-        <stp/>
-        <stp>69308b63-ffde-4724-8bbf-0cd7a7490f63</stp>
-        <tr r="F6" s="1"/>
-      </tp>
-    </main>
-    <main first="rtdsrv.e91a2bf1ca1e4425853080e41816bb7b">
-      <tp>
-        <v>2</v>
-        <stp/>
-        <stp>2f200a3c-874c-4f0d-9a05-30102646e57e</stp>
-        <tr r="F5" s="3"/>
-      </tp>
-    </main>
-    <main first="rtdsrv.e91a2bf1ca1e4425853080e41816bb7b">
-      <tp>
-        <v>2</v>
-        <stp/>
-        <stp>42de0596-f89f-4d80-9b31-243e590fc74a</stp>
-        <tr r="G42" s="1"/>
       </tp>
     </main>
   </volType>
@@ -2440,7 +2462,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{04DB3D96-2BED-447F-BDEB-F8DD83959477}">
-  <dimension ref="B1:AS65"/>
+  <dimension ref="B1:AS79"/>
   <sheetFormatPr defaultRowHeight="18.75" x14ac:dyDescent="0.4"/>
   <cols>
     <col min="1" max="1" width="2.25" customWidth="1"/>
@@ -2471,11 +2493,11 @@
       </c>
       <c r="F1" t="str" cm="1">
         <f t="array" ref="F1">_xll.ExLibris.Json.CreateJsonObject(E3:F6)</f>
-        <v>JsonObject:B5B4CCE3-96AE-40E7-B7C2-DE061F03E641</v>
+        <v>JsonObject:52A2F858-3F74-4672-A31D-B7422A404FBB</v>
       </c>
       <c r="K1" t="str">
         <f>EXLIBRIS_CONFIGURATION</f>
-        <v>ExLibris.Core.ExLibrisConfiguration:A3505878-8022-4705-B0DF-ED091E6A34F4</v>
+        <v>ExLibris.Core.ExLibrisConfiguration:F0DF99F8-61E4-463E-9654-9F1DC8890D33</v>
       </c>
     </row>
     <row r="2" spans="2:28" x14ac:dyDescent="0.4">
@@ -2545,7 +2567,7 @@
       </c>
       <c r="F6" t="str" cm="1">
         <f t="array" ref="F6">_xll.ExLibris.Json.CreateJsonArray(E8:J14)</f>
-        <v>JsonObject:DCB7A87F-40A1-446F-BC48-D6727DF6D996</v>
+        <v>JsonObject:CB96C2F4-B2BE-4E54-9E6C-3D4C6042F495</v>
       </c>
       <c r="L6" t="s">
         <v>68</v>
@@ -2598,6 +2620,13 @@
       </c>
     </row>
     <row r="9" spans="2:28" x14ac:dyDescent="0.4">
+      <c r="B9" s="6" t="s">
+        <v>181</v>
+      </c>
+      <c r="C9" s="6">
+        <f>COUNTIF(AR67:AS72,FALSE)</f>
+        <v>0</v>
+      </c>
       <c r="E9" s="1">
         <f>G9</f>
         <v>44632</v>
@@ -2620,6 +2649,13 @@
       </c>
     </row>
     <row r="10" spans="2:28" x14ac:dyDescent="0.4">
+      <c r="B10" s="6" t="s">
+        <v>182</v>
+      </c>
+      <c r="C10" s="6">
+        <f>COUNTIF(AR74:AS79,FALSE)</f>
+        <v>0</v>
+      </c>
       <c r="E10" s="1">
         <f>G10</f>
         <v>44812</v>
@@ -2784,10 +2820,10 @@
       </c>
       <c r="I19" t="str" cm="1">
         <f t="array" ref="I19">_xll.ExLibris.Json.GetJsonValue(F1,E6)</f>
-        <v>JsonObject:D3EFBB05-8438-415B-925D-3931CC155DD0</v>
+        <v>JsonObject:EF404BC8-9ABB-4928-92CC-B46882D34EB7</v>
       </c>
       <c r="P19" t="str" cm="1">
-        <f t="array" ref="P19:Q27">_xll.ExLibris.Json.GetJsonKeyValues(F1,,3)</f>
+        <f t="array" ref="P19:Q27">_xll.ExLibris.Json.GetJsonKeyValues(F1,3)</f>
         <v>trade_code</v>
       </c>
       <c r="Q19" t="str">
@@ -3089,7 +3125,7 @@
         <v>fixed_leg.cashflows.[0]</v>
       </c>
       <c r="Q22" t="str">
-        <v>JsonObject:82BAFBD6-F740-4F07-8B72-17652EAD06CA</v>
+        <v>JsonObject:07017FCE-7D95-4189-8AE3-D4FB5AA3787E</v>
       </c>
       <c r="S22" t="s">
         <v>32</v>
@@ -3188,7 +3224,7 @@
         <v>fixed_leg.cashflows.[1]</v>
       </c>
       <c r="Q23" t="str">
-        <v>JsonObject:FB22A593-FC8A-4388-9EC5-D374F757CEC1</v>
+        <v>JsonObject:BEC9C01F-61B3-4A7B-9DBB-81496CCE3D9C</v>
       </c>
       <c r="S23" t="s">
         <v>33</v>
@@ -3287,7 +3323,7 @@
         <v>fixed_leg.cashflows.[2]</v>
       </c>
       <c r="Q24" t="str">
-        <v>JsonObject:ED5FAFFA-759F-4DB6-B195-261E8EC50B3B</v>
+        <v>JsonObject:7DDE9C87-A3FF-407B-BE23-C6B16A9692EA</v>
       </c>
       <c r="S24" t="s">
         <v>34</v>
@@ -3386,7 +3422,7 @@
         <v>fixed_leg.cashflows.[3]</v>
       </c>
       <c r="Q25" t="str">
-        <v>JsonObject:60840F80-06C2-4EAE-92DC-02D7027C10BF</v>
+        <v>JsonObject:9FA80DE3-74C6-4F33-B39E-F97A07871379</v>
       </c>
       <c r="S25" t="s">
         <v>35</v>
@@ -3485,7 +3521,7 @@
         <v>fixed_leg.cashflows.[4]</v>
       </c>
       <c r="Q26" t="str">
-        <v>JsonObject:C8E3E2A3-A650-4367-A12B-239FABC1C85A</v>
+        <v>JsonObject:C53CF65F-252C-4C0C-9D88-2DD7CEE442B4</v>
       </c>
       <c r="S26" t="s">
         <v>36</v>
@@ -3566,7 +3602,7 @@
         <v>fixed_leg.cashflows.[5]</v>
       </c>
       <c r="Q27" t="str">
-        <v>JsonObject:3781CD40-705D-484F-A6F8-5B66DE27128E</v>
+        <v>JsonObject:1FA869B2-6DE1-4CAB-9619-8052C38BEC92</v>
       </c>
       <c r="S27" t="s">
         <v>37</v>
@@ -3603,7 +3639,7 @@
       </c>
       <c r="I28" t="str" cm="1">
         <f t="array" ref="I28">_xll.ExLibris.Json.GetJsonValue(I19,"[2]")</f>
-        <v>JsonObject:9DDB565C-5CEA-459A-B30C-D60000B098A9</v>
+        <v>JsonObject:AE972D68-C821-466C-BCAB-DE624FD97744</v>
       </c>
       <c r="S28" t="s">
         <v>38</v>
@@ -3659,7 +3695,7 @@
       </c>
       <c r="P29" t="str" cm="1">
         <f t="array" ref="P29">_xll.ExLibris.Json.CreateJsonObject(P22:Q27)</f>
-        <v>JsonObject:8BC4681C-84F4-4680-90F7-E525ED5BB21B</v>
+        <v>JsonObject:697E7411-20D4-4EF3-87D7-E6644719D4E2</v>
       </c>
       <c r="S29" t="s">
         <v>39</v>
@@ -5443,6 +5479,272 @@
       </c>
       <c r="AS65" t="b">
         <f>Q65=AE65</f>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="67" spans="16:45" x14ac:dyDescent="0.4">
+      <c r="P67" t="str" cm="1">
+        <f t="array" ref="P67:Q72">_xll.ExLibris.Json.GetJsonKeyValues(F1,"fixed_leg.cashflows.*.payment _date")</f>
+        <v>fixed_leg.cashflows.[0].payment _date</v>
+      </c>
+      <c r="Q67">
+        <v>44632</v>
+      </c>
+      <c r="AD67" t="s">
+        <v>32</v>
+      </c>
+      <c r="AE67">
+        <v>44632</v>
+      </c>
+      <c r="AR67" t="b">
+        <f t="shared" ref="AR67:AR79" si="10">P67=AD67</f>
+        <v>1</v>
+      </c>
+      <c r="AS67" t="b">
+        <f t="shared" ref="AS67:AS79" si="11">Q67=AE67</f>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="68" spans="16:45" x14ac:dyDescent="0.4">
+      <c r="P68" t="str">
+        <v>fixed_leg.cashflows.[1].payment _date</v>
+      </c>
+      <c r="Q68">
+        <v>44812</v>
+      </c>
+      <c r="AD68" t="s">
+        <v>38</v>
+      </c>
+      <c r="AE68">
+        <v>44812</v>
+      </c>
+      <c r="AR68" t="b">
+        <f t="shared" si="10"/>
+        <v>1</v>
+      </c>
+      <c r="AS68" t="b">
+        <f t="shared" si="11"/>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="69" spans="16:45" x14ac:dyDescent="0.4">
+      <c r="P69" t="str">
+        <v>fixed_leg.cashflows.[2].payment _date</v>
+      </c>
+      <c r="Q69">
+        <v>44992</v>
+      </c>
+      <c r="AD69" t="s">
+        <v>44</v>
+      </c>
+      <c r="AE69">
+        <v>44992</v>
+      </c>
+      <c r="AR69" t="b">
+        <f t="shared" si="10"/>
+        <v>1</v>
+      </c>
+      <c r="AS69" t="b">
+        <f t="shared" si="11"/>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="70" spans="16:45" x14ac:dyDescent="0.4">
+      <c r="P70" t="str">
+        <v>fixed_leg.cashflows.[3].payment _date</v>
+      </c>
+      <c r="Q70">
+        <v>45172</v>
+      </c>
+      <c r="AD70" t="s">
+        <v>50</v>
+      </c>
+      <c r="AE70">
+        <v>45172</v>
+      </c>
+      <c r="AR70" t="b">
+        <f t="shared" si="10"/>
+        <v>1</v>
+      </c>
+      <c r="AS70" t="b">
+        <f t="shared" si="11"/>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="71" spans="16:45" x14ac:dyDescent="0.4">
+      <c r="P71" t="str">
+        <v>fixed_leg.cashflows.[4].payment _date</v>
+      </c>
+      <c r="Q71">
+        <v>45352</v>
+      </c>
+      <c r="AD71" t="s">
+        <v>56</v>
+      </c>
+      <c r="AE71">
+        <v>45352</v>
+      </c>
+      <c r="AR71" t="b">
+        <f t="shared" si="10"/>
+        <v>1</v>
+      </c>
+      <c r="AS71" t="b">
+        <f t="shared" si="11"/>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="72" spans="16:45" x14ac:dyDescent="0.4">
+      <c r="P72" t="str">
+        <v>fixed_leg.cashflows.[5].payment _date</v>
+      </c>
+      <c r="Q72">
+        <v>45532</v>
+      </c>
+      <c r="AD72" t="s">
+        <v>62</v>
+      </c>
+      <c r="AE72">
+        <v>45532</v>
+      </c>
+      <c r="AR72" t="b">
+        <f t="shared" si="10"/>
+        <v>1</v>
+      </c>
+      <c r="AS72" t="b">
+        <f t="shared" si="11"/>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="74" spans="16:45" x14ac:dyDescent="0.4">
+      <c r="P74" t="str" cm="1">
+        <f t="array" ref="P74:Q79">_xll.ExLibris.Json.GetJsonKeyValues(F1,"fixed_leg.cashflows.[3].*")</f>
+        <v>fixed_leg.cashflows.[3].payment _date</v>
+      </c>
+      <c r="Q74">
+        <v>45172</v>
+      </c>
+      <c r="AD74" t="s">
+        <v>50</v>
+      </c>
+      <c r="AE74">
+        <v>45172</v>
+      </c>
+      <c r="AR74" t="b">
+        <f t="shared" si="10"/>
+        <v>1</v>
+      </c>
+      <c r="AS74" t="b">
+        <f t="shared" si="11"/>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="75" spans="16:45" x14ac:dyDescent="0.4">
+      <c r="P75" t="str">
+        <v>fixed_leg.cashflows.[3].start_date</v>
+      </c>
+      <c r="Q75">
+        <v>44992</v>
+      </c>
+      <c r="AD75" t="s">
+        <v>51</v>
+      </c>
+      <c r="AE75">
+        <v>44992</v>
+      </c>
+      <c r="AR75" t="b">
+        <f t="shared" si="10"/>
+        <v>1</v>
+      </c>
+      <c r="AS75" t="b">
+        <f t="shared" si="11"/>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="76" spans="16:45" x14ac:dyDescent="0.4">
+      <c r="P76" t="str">
+        <v>fixed_leg.cashflows.[3].end_date</v>
+      </c>
+      <c r="Q76">
+        <v>45172</v>
+      </c>
+      <c r="AD76" t="s">
+        <v>52</v>
+      </c>
+      <c r="AE76">
+        <v>45172</v>
+      </c>
+      <c r="AR76" t="b">
+        <f t="shared" si="10"/>
+        <v>1</v>
+      </c>
+      <c r="AS76" t="b">
+        <f t="shared" si="11"/>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="77" spans="16:45" x14ac:dyDescent="0.4">
+      <c r="P77" t="str">
+        <v>fixed_leg.cashflows.[3].day_count_type</v>
+      </c>
+      <c r="Q77" t="str">
+        <v>ACT/360</v>
+      </c>
+      <c r="AD77" t="s">
+        <v>53</v>
+      </c>
+      <c r="AE77" t="s">
+        <v>8</v>
+      </c>
+      <c r="AR77" t="b">
+        <f t="shared" si="10"/>
+        <v>1</v>
+      </c>
+      <c r="AS77" t="b">
+        <f t="shared" si="11"/>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="78" spans="16:45" x14ac:dyDescent="0.4">
+      <c r="P78" t="str">
+        <v>fixed_leg.cashflows.[3].amout</v>
+      </c>
+      <c r="Q78">
+        <v>13000000</v>
+      </c>
+      <c r="AD78" t="s">
+        <v>54</v>
+      </c>
+      <c r="AE78">
+        <v>13000000</v>
+      </c>
+      <c r="AR78" t="b">
+        <f t="shared" si="10"/>
+        <v>1</v>
+      </c>
+      <c r="AS78" t="b">
+        <f t="shared" si="11"/>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="79" spans="16:45" x14ac:dyDescent="0.4">
+      <c r="P79" t="str">
+        <v>fixed_leg.cashflows.[3].fixed_rate</v>
+      </c>
+      <c r="Q79">
+        <v>1E-3</v>
+      </c>
+      <c r="AD79" t="s">
+        <v>55</v>
+      </c>
+      <c r="AE79">
+        <v>1E-3</v>
+      </c>
+      <c r="AR79" t="b">
+        <f t="shared" si="10"/>
+        <v>1</v>
+      </c>
+      <c r="AS79" t="b">
+        <f t="shared" si="11"/>
         <v>1</v>
       </c>
     </row>
@@ -5455,7 +5757,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{130D5E5E-1419-4F0D-AFC7-AD1DEAC9CE64}">
-  <dimension ref="B1:AS65"/>
+  <dimension ref="B1:AS79"/>
   <sheetFormatPr defaultRowHeight="18.75" x14ac:dyDescent="0.4"/>
   <cols>
     <col min="1" max="1" width="2.25" customWidth="1"/>
@@ -5486,11 +5788,11 @@
       </c>
       <c r="F1" t="str" cm="1">
         <f t="array" ref="F1">_xll.ExLibris.Json.CreateJsonObjectAsync(E3:F6)</f>
-        <v>JsonObject:3C6C8349-B49F-45AC-90E0-1C959B076691</v>
+        <v>JsonObject:2A1832AF-6F94-4519-9D6F-7AFF11A808B5</v>
       </c>
       <c r="K1" t="str">
         <f>EXLIBRIS_CONFIGURATION</f>
-        <v>ExLibris.Core.ExLibrisConfiguration:A3505878-8022-4705-B0DF-ED091E6A34F4</v>
+        <v>ExLibris.Core.ExLibrisConfiguration:F0DF99F8-61E4-463E-9654-9F1DC8890D33</v>
       </c>
     </row>
     <row r="2" spans="2:28" x14ac:dyDescent="0.4">
@@ -5560,7 +5862,7 @@
       </c>
       <c r="F6" t="str" cm="1">
         <f t="array" ref="F6">_xll.ExLibris.Json.CreateJsonArrayAsync(E8:J14)</f>
-        <v>JsonObject:0A8307F4-3F69-4E1B-9C16-7043EA734C0F</v>
+        <v>JsonObject:206F023E-4FD8-45A8-AB21-54CE69ABD566</v>
       </c>
       <c r="L6" t="s">
         <v>68</v>
@@ -5613,6 +5915,13 @@
       </c>
     </row>
     <row r="9" spans="2:28" x14ac:dyDescent="0.4">
+      <c r="B9" s="6" t="s">
+        <v>181</v>
+      </c>
+      <c r="C9" s="6">
+        <f>COUNTIF(AR67:AS72,FALSE)</f>
+        <v>0</v>
+      </c>
       <c r="E9" s="1">
         <f>G9</f>
         <v>44632</v>
@@ -5635,6 +5944,13 @@
       </c>
     </row>
     <row r="10" spans="2:28" x14ac:dyDescent="0.4">
+      <c r="B10" s="6" t="s">
+        <v>182</v>
+      </c>
+      <c r="C10" s="6">
+        <f>COUNTIF(AR74:AS79,FALSE)</f>
+        <v>0</v>
+      </c>
       <c r="E10" s="1">
         <f>G10</f>
         <v>44812</v>
@@ -5799,10 +6115,10 @@
       </c>
       <c r="I19" t="str" cm="1">
         <f t="array" ref="I19">_xll.ExLibris.Json.GetJsonValueAsync(F1,E6)</f>
-        <v>JsonObject:6C930AEF-8421-40AB-BAFF-0CB90F782945</v>
+        <v>JsonObject:EB8BC461-3C01-476B-9048-FF0DB295746A</v>
       </c>
       <c r="P19" t="str" cm="1">
-        <f t="array" ref="P19:Q27">_xll.ExLibris.Json.GetJsonKeyValuesAsync(F1,,3)</f>
+        <f t="array" ref="P19:Q27">_xll.ExLibris.Json.GetJsonKeyValuesAsync(F1,3)</f>
         <v>trade_code</v>
       </c>
       <c r="Q19" t="str">
@@ -6104,7 +6420,7 @@
         <v>fixed_leg.cashflows.[0]</v>
       </c>
       <c r="Q22" t="str">
-        <v>JsonObject:61F37CF0-86A7-43C9-8F36-CBE5A8BA9982</v>
+        <v>JsonObject:B9DA0B81-A803-4023-A5B0-ED39D1636721</v>
       </c>
       <c r="S22" t="s">
         <v>32</v>
@@ -6203,7 +6519,7 @@
         <v>fixed_leg.cashflows.[1]</v>
       </c>
       <c r="Q23" t="str">
-        <v>JsonObject:20286845-E0C5-443A-94A2-16E49B8FFCF9</v>
+        <v>JsonObject:2C3549B1-51DF-4C6F-AF04-35C341FD7F8C</v>
       </c>
       <c r="S23" t="s">
         <v>33</v>
@@ -6302,7 +6618,7 @@
         <v>fixed_leg.cashflows.[2]</v>
       </c>
       <c r="Q24" t="str">
-        <v>JsonObject:6CCF7990-888C-4451-BBE1-359E76DA2EF4</v>
+        <v>JsonObject:6F9AF213-68EF-4C6B-AB9E-3E8E9E044219</v>
       </c>
       <c r="S24" t="s">
         <v>34</v>
@@ -6401,7 +6717,7 @@
         <v>fixed_leg.cashflows.[3]</v>
       </c>
       <c r="Q25" t="str">
-        <v>JsonObject:7E41441A-F581-4936-A2E9-88E9CBC8A716</v>
+        <v>JsonObject:BCCE4269-E901-44CF-A4F0-5E0D24C861A0</v>
       </c>
       <c r="S25" t="s">
         <v>35</v>
@@ -6500,7 +6816,7 @@
         <v>fixed_leg.cashflows.[4]</v>
       </c>
       <c r="Q26" t="str">
-        <v>JsonObject:88E5773E-7315-4B4F-A4DD-6FB4D6B99DA8</v>
+        <v>JsonObject:1796A747-6F1D-4621-8C5C-987A3978B065</v>
       </c>
       <c r="S26" t="s">
         <v>36</v>
@@ -6581,7 +6897,7 @@
         <v>fixed_leg.cashflows.[5]</v>
       </c>
       <c r="Q27" t="str">
-        <v>JsonObject:6F5CDAD0-1D3B-478B-84AB-CDDFE94B3FCC</v>
+        <v>JsonObject:D2E997B2-D3DF-4862-A042-5745B76A80E7</v>
       </c>
       <c r="S27" t="s">
         <v>37</v>
@@ -6618,7 +6934,7 @@
       </c>
       <c r="I28" t="str" cm="1">
         <f t="array" ref="I28">_xll.ExLibris.Json.GetJsonValueAsync(I19,"[2]")</f>
-        <v>JsonObject:59D3B7CE-EE20-4211-911F-F1328EE23664</v>
+        <v>JsonObject:42183BC8-8C17-40A4-B1A4-628331E7B363</v>
       </c>
       <c r="S28" t="s">
         <v>38</v>
@@ -6674,7 +6990,7 @@
       </c>
       <c r="P29" t="str" cm="1">
         <f t="array" ref="P29">_xll.ExLibris.Json.CreateJsonObjectAsync(P22:Q27)</f>
-        <v>JsonObject:E4F52AA6-81C7-4154-832C-8CDEAEE32991</v>
+        <v>JsonObject:F5AD9A29-1E53-423F-A257-35EE79423841</v>
       </c>
       <c r="S29" t="s">
         <v>39</v>
@@ -8458,6 +8774,272 @@
       </c>
       <c r="AS65" t="b">
         <f>Q65=AE65</f>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="67" spans="16:45" x14ac:dyDescent="0.4">
+      <c r="P67" t="str" cm="1">
+        <f t="array" ref="P67:Q72">_xll.ExLibris.Json.GetJsonKeyValuesAsync(F1,"fixed_leg.cashflows.*.payment _date")</f>
+        <v>fixed_leg.cashflows.[0].payment _date</v>
+      </c>
+      <c r="Q67">
+        <v>44632</v>
+      </c>
+      <c r="AD67" t="s">
+        <v>32</v>
+      </c>
+      <c r="AE67">
+        <v>44632</v>
+      </c>
+      <c r="AR67" t="b">
+        <f t="shared" ref="AR67:AS79" si="12">P67=AD67</f>
+        <v>1</v>
+      </c>
+      <c r="AS67" t="b">
+        <f t="shared" si="12"/>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="68" spans="16:45" x14ac:dyDescent="0.4">
+      <c r="P68" t="str">
+        <v>fixed_leg.cashflows.[1].payment _date</v>
+      </c>
+      <c r="Q68">
+        <v>44812</v>
+      </c>
+      <c r="AD68" t="s">
+        <v>38</v>
+      </c>
+      <c r="AE68">
+        <v>44812</v>
+      </c>
+      <c r="AR68" t="b">
+        <f t="shared" si="12"/>
+        <v>1</v>
+      </c>
+      <c r="AS68" t="b">
+        <f t="shared" si="12"/>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="69" spans="16:45" x14ac:dyDescent="0.4">
+      <c r="P69" t="str">
+        <v>fixed_leg.cashflows.[2].payment _date</v>
+      </c>
+      <c r="Q69">
+        <v>44992</v>
+      </c>
+      <c r="AD69" t="s">
+        <v>44</v>
+      </c>
+      <c r="AE69">
+        <v>44992</v>
+      </c>
+      <c r="AR69" t="b">
+        <f t="shared" si="12"/>
+        <v>1</v>
+      </c>
+      <c r="AS69" t="b">
+        <f t="shared" si="12"/>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="70" spans="16:45" x14ac:dyDescent="0.4">
+      <c r="P70" t="str">
+        <v>fixed_leg.cashflows.[3].payment _date</v>
+      </c>
+      <c r="Q70">
+        <v>45172</v>
+      </c>
+      <c r="AD70" t="s">
+        <v>50</v>
+      </c>
+      <c r="AE70">
+        <v>45172</v>
+      </c>
+      <c r="AR70" t="b">
+        <f t="shared" si="12"/>
+        <v>1</v>
+      </c>
+      <c r="AS70" t="b">
+        <f t="shared" si="12"/>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="71" spans="16:45" x14ac:dyDescent="0.4">
+      <c r="P71" t="str">
+        <v>fixed_leg.cashflows.[4].payment _date</v>
+      </c>
+      <c r="Q71">
+        <v>45352</v>
+      </c>
+      <c r="AD71" t="s">
+        <v>56</v>
+      </c>
+      <c r="AE71">
+        <v>45352</v>
+      </c>
+      <c r="AR71" t="b">
+        <f t="shared" si="12"/>
+        <v>1</v>
+      </c>
+      <c r="AS71" t="b">
+        <f t="shared" si="12"/>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="72" spans="16:45" x14ac:dyDescent="0.4">
+      <c r="P72" t="str">
+        <v>fixed_leg.cashflows.[5].payment _date</v>
+      </c>
+      <c r="Q72">
+        <v>45532</v>
+      </c>
+      <c r="AD72" t="s">
+        <v>62</v>
+      </c>
+      <c r="AE72">
+        <v>45532</v>
+      </c>
+      <c r="AR72" t="b">
+        <f t="shared" si="12"/>
+        <v>1</v>
+      </c>
+      <c r="AS72" t="b">
+        <f t="shared" si="12"/>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="74" spans="16:45" x14ac:dyDescent="0.4">
+      <c r="P74" t="str" cm="1">
+        <f t="array" ref="P74:Q79">_xll.ExLibris.Json.GetJsonKeyValuesAsync(F1,"fixed_leg.cashflows.[3].*")</f>
+        <v>fixed_leg.cashflows.[3].payment _date</v>
+      </c>
+      <c r="Q74">
+        <v>45172</v>
+      </c>
+      <c r="AD74" t="s">
+        <v>50</v>
+      </c>
+      <c r="AE74">
+        <v>45172</v>
+      </c>
+      <c r="AR74" t="b">
+        <f t="shared" si="12"/>
+        <v>1</v>
+      </c>
+      <c r="AS74" t="b">
+        <f t="shared" si="12"/>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="75" spans="16:45" x14ac:dyDescent="0.4">
+      <c r="P75" t="str">
+        <v>fixed_leg.cashflows.[3].start_date</v>
+      </c>
+      <c r="Q75">
+        <v>44992</v>
+      </c>
+      <c r="AD75" t="s">
+        <v>51</v>
+      </c>
+      <c r="AE75">
+        <v>44992</v>
+      </c>
+      <c r="AR75" t="b">
+        <f t="shared" si="12"/>
+        <v>1</v>
+      </c>
+      <c r="AS75" t="b">
+        <f t="shared" si="12"/>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="76" spans="16:45" x14ac:dyDescent="0.4">
+      <c r="P76" t="str">
+        <v>fixed_leg.cashflows.[3].end_date</v>
+      </c>
+      <c r="Q76">
+        <v>45172</v>
+      </c>
+      <c r="AD76" t="s">
+        <v>52</v>
+      </c>
+      <c r="AE76">
+        <v>45172</v>
+      </c>
+      <c r="AR76" t="b">
+        <f t="shared" si="12"/>
+        <v>1</v>
+      </c>
+      <c r="AS76" t="b">
+        <f t="shared" si="12"/>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="77" spans="16:45" x14ac:dyDescent="0.4">
+      <c r="P77" t="str">
+        <v>fixed_leg.cashflows.[3].day_count_type</v>
+      </c>
+      <c r="Q77" t="str">
+        <v>ACT/360</v>
+      </c>
+      <c r="AD77" t="s">
+        <v>53</v>
+      </c>
+      <c r="AE77" t="s">
+        <v>8</v>
+      </c>
+      <c r="AR77" t="b">
+        <f t="shared" si="12"/>
+        <v>1</v>
+      </c>
+      <c r="AS77" t="b">
+        <f t="shared" si="12"/>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="78" spans="16:45" x14ac:dyDescent="0.4">
+      <c r="P78" t="str">
+        <v>fixed_leg.cashflows.[3].amout</v>
+      </c>
+      <c r="Q78">
+        <v>13000000</v>
+      </c>
+      <c r="AD78" t="s">
+        <v>54</v>
+      </c>
+      <c r="AE78">
+        <v>13000000</v>
+      </c>
+      <c r="AR78" t="b">
+        <f t="shared" si="12"/>
+        <v>1</v>
+      </c>
+      <c r="AS78" t="b">
+        <f t="shared" si="12"/>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="79" spans="16:45" x14ac:dyDescent="0.4">
+      <c r="P79" t="str">
+        <v>fixed_leg.cashflows.[3].fixed_rate</v>
+      </c>
+      <c r="Q79">
+        <v>1E-3</v>
+      </c>
+      <c r="AD79" t="s">
+        <v>55</v>
+      </c>
+      <c r="AE79">
+        <v>1E-3</v>
+      </c>
+      <c r="AR79" t="b">
+        <f t="shared" si="12"/>
+        <v>1</v>
+      </c>
+      <c r="AS79" t="b">
+        <f t="shared" si="12"/>
         <v>1</v>
       </c>
     </row>
@@ -8496,11 +9078,11 @@
       </c>
       <c r="F1" t="str" cm="1">
         <f t="array" ref="F1">_xll.ExLibris.Json.CreateJsonObjectAsync(E3:F6, EXLIBRIS_CONFIGURATION)</f>
-        <v>JsonObject:2B2A96C2-A634-4768-97AA-40BF69D427BB</v>
+        <v>JsonObject:BBECD4AA-A485-4CA4-9E97-0F7FC250627D</v>
       </c>
       <c r="K1" t="str">
         <f>EXLIBRIS_CONFIGURATION</f>
-        <v>ExLibris.Core.ExLibrisConfiguration:A3505878-8022-4705-B0DF-ED091E6A34F4</v>
+        <v>ExLibris.Core.ExLibrisConfiguration:F0DF99F8-61E4-463E-9654-9F1DC8890D33</v>
       </c>
     </row>
     <row r="2" spans="2:25" x14ac:dyDescent="0.4">
@@ -8570,7 +9152,7 @@
       </c>
       <c r="F6" t="str" cm="1">
         <f t="array" ref="F6">_xll.ExLibris.Json.CreateJsonArrayAsync(E8:J14, EXLIBRIS_CONFIGURATION)</f>
-        <v>JsonObject:A5AF79D2-AAF4-4315-A839-1A7598723ABC</v>
+        <v>JsonObject:E4760CE1-5B18-4BE6-8A2E-D54D58C331C3</v>
       </c>
       <c r="L6" t="s">
         <v>68</v>
@@ -8809,7 +9391,7 @@
     </row>
     <row r="19" spans="5:36" x14ac:dyDescent="0.4">
       <c r="E19" t="str" cm="1">
-        <f t="array" ref="E19:F57">_xll.ExLibris.Json.GetJsonKeyValuesAsync(F1, EXLIBRIS_CONFIGURATION)</f>
+        <f t="array" ref="E19:F57">_xll.ExLibris.Json.GetJsonKeyValuesAsync(F1,, EXLIBRIS_CONFIGURATION)</f>
         <v>trade_code</v>
       </c>
       <c r="F19" t="str">
@@ -8821,7 +9403,7 @@
       </c>
       <c r="I19" t="str" cm="1">
         <f t="array" ref="I19">_xll.ExLibris.Json.GetJsonValueAsync(F1,E6, EXLIBRIS_CONFIGURATION)</f>
-        <v>JsonObject:F2DDDE3E-A881-4CB2-B225-52BFE1009195</v>
+        <v>JsonObject:83CBBB06-78F8-4E96-A681-BF324E9CE363</v>
       </c>
       <c r="P19" t="s">
         <v>14</v>
@@ -9543,7 +10125,7 @@
       </c>
       <c r="I28" t="str" cm="1">
         <f t="array" ref="I28">_xll.ExLibris.Json.GetJsonValueAsync(I19,"[2]", EXLIBRIS_CONFIGURATION)</f>
-        <v>JsonObject:F36138D1-4683-4536-BDF9-3D243EABA6DB</v>
+        <v>JsonObject:B9931949-9D59-44CC-8FE2-B91CD72E9523</v>
       </c>
       <c r="P28" t="s">
         <v>38</v>
@@ -9800,7 +10382,7 @@
       </c>
       <c r="I32" t="str" cm="1">
         <f t="array" ref="I32">_xll.ExLibris.Json.GetJsonValueAsync(F1,E6,EXLIBRIS_CONFIGURATION)</f>
-        <v>JsonObject:F2DDDE3E-A881-4CB2-B225-52BFE1009195</v>
+        <v>JsonObject:83CBBB06-78F8-4E96-A681-BF324E9CE363</v>
       </c>
       <c r="P32" t="s">
         <v>42</v>
@@ -9837,7 +10419,7 @@
       </c>
       <c r="I33" t="str" cm="1">
         <f t="array" ref="I33">_xll.ExLibris.Json.SearchJsonArrayElementsAsync(I32,I8,I11,EXLIBRIS_CONFIGURATION)</f>
-        <v>JsonObject:D008CE39-6185-478A-B17E-6D4C87DBADD7</v>
+        <v>JsonObject:401E3E45-1D7F-464C-B02D-2F563EFFAFC5</v>
       </c>
       <c r="P33" t="s">
         <v>43</v>
@@ -10187,7 +10769,7 @@
       </c>
       <c r="I38" t="str" cm="1">
         <f t="array" ref="I38">_xll.ExLibris.Json.SearchJsonArrayElementsAsync(I32,J8,J11,EXLIBRIS_CONFIGURATION)</f>
-        <v>JsonObject:C4634FDF-A9C9-414E-8231-1235C2E87600</v>
+        <v>JsonObject:F78D41FE-B256-458A-8364-43AE5435BE17</v>
       </c>
       <c r="P38" t="s">
         <v>48</v>
@@ -10444,7 +11026,7 @@
       </c>
       <c r="I42" t="str" cm="1">
         <f t="array" ref="I42">_xll.ExLibris.Json.SearchJsonArrayElementsAsync(I32,J8,,EXLIBRIS_CONFIGURATION)</f>
-        <v>JsonObject:F7CEB066-2995-4133-AC88-D60949E98D8E</v>
+        <v>JsonObject:6796472E-1BC6-4551-B028-F64D8E7765AC</v>
       </c>
       <c r="P42" t="s">
         <v>52</v>
@@ -10998,7 +11580,7 @@
       </c>
       <c r="C2" t="str" cm="1">
         <f t="array" ref="C2">_xll.ExLibris.LoadConfigurationAsync(B6:C15)</f>
-        <v>ExLibris.Core.ExLibrisConfiguration:A3505878-8022-4705-B0DF-ED091E6A34F4</v>
+        <v>ExLibris.Core.ExLibrisConfiguration:F0DF99F8-61E4-463E-9654-9F1DC8890D33</v>
       </c>
     </row>
     <row r="4" spans="2:6" s="4" customFormat="1" ht="18" x14ac:dyDescent="0.4">
@@ -11201,7 +11783,7 @@
     <row r="4" spans="2:10" x14ac:dyDescent="0.4">
       <c r="D4" t="str" cm="1">
         <f t="array" ref="D4">_xll.ExLibris.WebSockets.OpenWebSocketAsync("ws://localhost:10101",,E4)</f>
-        <v>ExLibris.Core.WebSockets.WebsocketClient:659B3690-449E-4205-886D-2C084E20246F</v>
+        <v>ExLibris.Core.WebSockets.WebsocketClient:16D7337E-1A65-4898-9732-8272DF54FFEA</v>
       </c>
       <c r="E4" t="s">
         <v>102</v>
@@ -11230,7 +11812,7 @@
     <row r="5" spans="2:10" x14ac:dyDescent="0.4">
       <c r="D5" t="str" cm="1">
         <f t="array" ref="D5">_xll.ExLibris.WebSockets.OpenWebSocketAsync("ws://localhost:10101",,E5)</f>
-        <v>ExLibris.Core.WebSockets.WebsocketClient:67060E24-65ED-4CC3-AE98-AEF89A1CD3E0</v>
+        <v>ExLibris.Core.WebSockets.WebsocketClient:029ECD09-225C-49C0-AD77-AB72A4B01810</v>
       </c>
       <c r="E5" t="s">
         <v>152</v>
@@ -11259,7 +11841,7 @@
     <row r="6" spans="2:10" x14ac:dyDescent="0.4">
       <c r="D6" t="str" cm="1">
         <f t="array" ref="D6">_xll.ExLibris.WebSockets.OpenWebSocketAsync("ws://localhost:10101",,E6)</f>
-        <v>ExLibris.Core.WebSockets.WebsocketClient:7C5A7623-9A39-4799-B0B2-07D68C7AF4D0</v>
+        <v>ExLibris.Core.WebSockets.WebsocketClient:1C440D9A-89CA-424C-8668-8284097545EB</v>
       </c>
       <c r="E6" t="s">
         <v>153</v>
@@ -11288,7 +11870,7 @@
     <row r="7" spans="2:10" x14ac:dyDescent="0.4">
       <c r="D7" t="str" cm="1">
         <f t="array" ref="D7">_xll.ExLibris.WebSockets.OpenWebSocketAsync("ws://localhost:10101",,E7)</f>
-        <v>ExLibris.Core.WebSockets.WebsocketClient:2E20B24C-6F88-425B-A976-776E83DAD963</v>
+        <v>ExLibris.Core.WebSockets.WebsocketClient:15BCE862-62F6-46B6-B0CB-B3D03FFAF414</v>
       </c>
       <c r="E7" t="s">
         <v>154</v>
@@ -11317,7 +11899,7 @@
     <row r="8" spans="2:10" x14ac:dyDescent="0.4">
       <c r="D8" t="str" cm="1">
         <f t="array" ref="D8">_xll.ExLibris.WebSockets.OpenWebSocketAsync("ws://localhost:10101",,E8)</f>
-        <v>ExLibris.Core.WebSockets.WebsocketClient:1151B977-4A20-498E-A241-8352314C9F93</v>
+        <v>ExLibris.Core.WebSockets.WebsocketClient:17B5C0EE-0BED-483E-8604-510D0BE6BDF3</v>
       </c>
       <c r="E8" t="s">
         <v>155</v>
@@ -11383,11 +11965,11 @@
     <row r="5" spans="2:11" x14ac:dyDescent="0.4">
       <c r="B5" t="str" cm="1">
         <f t="array" ref="B5">_xll.ExLibris.WebAPIs.CreateHeadersAsync(B6:C10)</f>
-        <v>ExLibris.Core.WebAPIs.WebAPIHeaders:520AFD9E-7D6D-477F-AE62-12DA42BD3FE3</v>
+        <v>ExLibris.Core.WebAPIs.WebAPIHeaders:96371D18-46CF-437E-98A7-3FCEC36D9FEE</v>
       </c>
       <c r="H5" t="str" cm="1">
         <f t="array" ref="H5">_xll.ExLibris.Json.CreateJsonObjectAsync(H6:I11)</f>
-        <v>JsonObject:30D2728C-3ABD-4502-830A-356B76FF444B</v>
+        <v>JsonObject:BEC6A6FB-8692-4111-AAB8-B82C788E4C2E</v>
       </c>
     </row>
     <row r="6" spans="2:11" x14ac:dyDescent="0.4">
@@ -12012,7 +12594,7 @@
     <row r="2" spans="2:4" x14ac:dyDescent="0.4">
       <c r="B2" t="str" cm="1">
         <f t="array" ref="B2">_xll.ExLibris.WebAPIs.CreateHeadersAsync(B3:C3)</f>
-        <v>ExLibris.Core.WebAPIs.WebAPIHeaders:220864F8-C2DA-46E8-A88C-10D98A5302FC</v>
+        <v>ExLibris.Core.WebAPIs.WebAPIHeaders:048FA470-F40B-4E12-A202-7FBB2EA67477</v>
       </c>
     </row>
     <row r="3" spans="2:4" x14ac:dyDescent="0.4">
@@ -12038,7 +12620,7 @@
       </c>
       <c r="C6" t="str" cm="1">
         <f t="array" ref="C6">_xll.ExLibris.WebAPIs.GET(C5,B2)</f>
-        <v>ExLibris.Core.WebAPIs.Response:6B5DA93B-83A0-4D8E-A7C9-AC25CFAC1844</v>
+        <v>ExLibris.Core.WebAPIs.Response:983346E2-30E2-44FD-AA41-C964ED5A9BD0</v>
       </c>
     </row>
     <row r="7" spans="2:4" x14ac:dyDescent="0.4">
@@ -12056,13 +12638,13 @@
       </c>
       <c r="C8" t="str" cm="1">
         <f t="array" ref="C8">_xll.ExLibris.WebAPIs.WebAPIResponseContent(C6)</f>
-        <v>{"login":"defunkt","id":2,"node_id":"MDQ6VXNlcjI=","avatar_url":"https://avatars.githubusercontent.com/u/2?v=4","gravatar_id":"","url":"https://api.github.com/users/defunkt","html_url":"https://github.com/defunkt","followers_url":"https://api.github.com/users/defunkt/followers","following_url":"https://api.github.com/users/defunkt/following{/other_user}","gists_url":"https://api.github.com/users/defunkt/gists{/gist_id}","starred_url":"https://api.github.com/users/defunkt/starred{/owner}{/repo}","subscriptions_url":"https://api.github.com/users/defunkt/subscriptions","organizations_url":"https://api.github.com/users/defunkt/orgs","repos_url":"https://api.github.com/users/defunkt/repos","events_url":"https://api.github.com/users/defunkt/events{/privacy}","received_events_url":"https://api.github.com/users/defunkt/received_events","type":"User","site_admin":false,"name":"Chris Wanstrath","company":null,"blog":"http://chriswanstrath.com/","location":null,"email":null,"hireable":null,"bio":"🍔","twitter_username":null,"public_repos":107,"public_gists":273,"followers":21404,"following":210,"created_at":"2007-10-20T05:24:19Z","updated_at":"2022-03-29T01:48:36Z"}</v>
+        <v>{"login":"defunkt","id":2,"node_id":"MDQ6VXNlcjI=","avatar_url":"https://avatars.githubusercontent.com/u/2?v=4","gravatar_id":"","url":"https://api.github.com/users/defunkt","html_url":"https://github.com/defunkt","followers_url":"https://api.github.com/users/defunkt/followers","following_url":"https://api.github.com/users/defunkt/following{/other_user}","gists_url":"https://api.github.com/users/defunkt/gists{/gist_id}","starred_url":"https://api.github.com/users/defunkt/starred{/owner}{/repo}","subscriptions_url":"https://api.github.com/users/defunkt/subscriptions","organizations_url":"https://api.github.com/users/defunkt/orgs","repos_url":"https://api.github.com/users/defunkt/repos","events_url":"https://api.github.com/users/defunkt/events{/privacy}","received_events_url":"https://api.github.com/users/defunkt/received_events","type":"User","site_admin":false,"name":"Chris Wanstrath","company":null,"blog":"http://chriswanstrath.com/","location":null,"email":null,"hireable":null,"bio":"🍔","twitter_username":null,"public_repos":107,"public_gists":273,"followers":21402,"following":210,"created_at":"2007-10-20T05:24:19Z","updated_at":"2022-03-29T01:48:36Z"}</v>
       </c>
     </row>
     <row r="10" spans="2:4" x14ac:dyDescent="0.4">
       <c r="C10" t="str" cm="1">
         <f t="array" ref="C10">_xll.ExLibris.Json.CreateJsonObjectAsync(C8)</f>
-        <v>JsonObject:B814FCD8-AD80-49E1-8F21-1DE963EFE530</v>
+        <v>JsonObject:21E33735-F806-4566-A797-446C8DA6C4EE</v>
       </c>
     </row>
     <row r="11" spans="2:4" x14ac:dyDescent="0.4">
@@ -12295,7 +12877,7 @@
         <v>followers</v>
       </c>
       <c r="D39">
-        <v>21404</v>
+        <v>21402</v>
       </c>
     </row>
     <row r="40" spans="3:4" x14ac:dyDescent="0.4">

</xml_diff>

<commit_message>
json table without column names
</commit_message>
<xml_diff>
--- a/ExLibris/test_excel/exlibris_test.xlsx
+++ b/ExLibris/test_excel/exlibris_test.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\mugen\git\ex-libris\ExLibris\test_excel\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B7D274E7-8A72-4E44-AF45-4E50D99540E1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B9E30E08-DB83-4B2F-8176-ADF5D1F9B09B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{705CD0B7-27A9-4291-85BD-6034C0FEE3E4}"/>
   </bookViews>
@@ -43,7 +43,7 @@
 </file>
 
 <file path=xl/metadata.xml><?xml version="1.0" encoding="utf-8"?>
-<metadata xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xda="http://schemas.microsoft.com/office/spreadsheetml/2017/dynamicarray">
+<metadata xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xlrd="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata" xmlns:xda="http://schemas.microsoft.com/office/spreadsheetml/2017/dynamicarray">
   <metadataTypes count="1">
     <metadataType name="XLDAPR" minSupportedVersion="120000" copy="1" pasteAll="1" pasteValues="1" merge="1" splitFirst="1" rowColShift="1" clearFormats="1" clearComments="1" assign="1" coerce="1" cellMeta="1"/>
   </metadataTypes>
@@ -65,7 +65,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="713" uniqueCount="187">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="744" uniqueCount="189">
   <si>
     <t>payment _date</t>
   </si>
@@ -836,6 +836,14 @@
   </si>
   <si>
     <t>{"trade_code":"money_00001","couter_party":"CP00001","fixed_leg":{"pay_or_recieve":"Receive","cashflows":[{"payment _date":"2022-03-12","start_date":"2021-09-13","end_date":"2022-03-12","day_count_type":"ACT/360","amount":10000000,"fixed_rate":0.001},{"payment _date":"2022-09-08","start_date":"2022-03-12","end_date":"2022-09-08","day_count_type":"ACT/360","amount":10000000,"fixed_rate":0.0011},{"payment _date":"2023-03-07","start_date":"2022-09-08","end_date":"2023-03-07","day_count_type":"ACT/360","amount":11000000,"fixed_rate":0.0012000000000000001},{"payment _date":"2023-09-03","start_date":"2023-03-07","end_date":"2023-09-03","day_count_type":"ACT/360","amount":11000000,"fixed_rate":0.0013000000000000002},{"payment _date":"2024-03-01","start_date":"2023-09-03","end_date":"2024-03-01","day_count_type":"ACT/360","amount":12000000,"fixed_rate":0.0014000000000000002},{"payment _date":"2024-08-28","start_date":"2024-03-01","end_date":"2024-08-28","day_count_type":"ACT/360","amount":12000000,"fixed_rate":0.0015000000000000002}]}}</t>
+  </si>
+  <si>
+    <t>table w/o keys</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>table w/o keys1</t>
+    <phoneticPr fontId="1"/>
   </si>
 </sst>
 </file>
@@ -966,1227 +974,1219 @@
 <file path=xl/volatileDependencies.xml><?xml version="1.0" encoding="utf-8"?>
 <volTypes xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <volType type="realTimeData">
-    <main first="rtdsrv.e9e679e6621d402baf5d71ad7ce809cc">
-      <tp>
-        <v>1</v>
-        <stp/>
-        <stp>0221e945-fff4-483c-aa18-9fae6c5b00a8</stp>
-        <tr r="G57" s="7"/>
+    <main first="rtdsrv.f947b7ebca124db5a46086c0c9fe0cad">
+      <tp>
+        <v>2</v>
+        <stp/>
+        <stp>da48622c-71e7-4c6e-a8b3-0ca472b82609</stp>
+        <tr r="G23" s="1"/>
+      </tp>
+      <tp>
+        <v>1</v>
+        <stp/>
+        <stp>8355e164-8a52-4212-90b5-c8c062f2bdcc</stp>
+        <tr r="G23" s="7"/>
+      </tp>
+      <tp>
+        <v>2</v>
+        <stp/>
+        <stp>56e07a60-5cb1-4168-afa7-69946793216f</stp>
+        <tr r="G38" s="4"/>
       </tp>
     </main>
-    <main first="rtdsrv.e9e679e6621d402baf5d71ad7ce809cc">
+    <main first="rtdsrv.f947b7ebca124db5a46086c0c9fe0cad">
+      <tp>
+        <v>1</v>
+        <stp/>
+        <stp>65b17f35-286b-40dc-93c8-5ed5d9efb960</stp>
+        <tr r="G27" s="7"/>
+      </tp>
+    </main>
+    <main first="rtdsrv.f947b7ebca124db5a46086c0c9fe0cad">
       <tp>
         <v>2</v>
         <stp/>
-        <stp>be0e7fcd-083a-4798-9443-f785c5049700</stp>
-        <tr r="D50" s="5"/>
-      </tp>
+        <stp>8df6df43-f979-4850-9ca6-ef5d1dd3e3b4</stp>
+        <tr r="G49" s="4"/>
+      </tp>
+    </main>
+    <main first="rtdsrv.f947b7ebca124db5a46086c0c9fe0cad">
       <tp>
         <v>2</v>
         <stp/>
-        <stp>30f98b7c-a201-4dff-ae8e-afb94b9e6cc0</stp>
+        <stp>5d614a3b-e620-4c14-8ff7-6a99b3d39d73</stp>
+        <tr r="G24" s="4"/>
+      </tp>
+    </main>
+    <main first="rtdsrv.f947b7ebca124db5a46086c0c9fe0cad">
+      <tp>
+        <v>2</v>
+        <stp/>
+        <stp>77a64598-40fc-4494-aa0b-ddbb82d37a4f</stp>
+        <tr r="G20" s="4"/>
+      </tp>
+      <tp>
+        <v>2</v>
+        <stp/>
+        <stp>f85f4431-2fb6-4e58-a13c-9c952cb380c0</stp>
+        <tr r="C2" s="2"/>
+      </tp>
+    </main>
+    <main first="rtdsrv.f947b7ebca124db5a46086c0c9fe0cad">
+      <tp>
+        <v>2</v>
+        <stp/>
+        <stp>45702167-350f-43bf-9508-c3746fdd919f</stp>
+        <tr r="G36" s="4"/>
+      </tp>
+    </main>
+    <main first="rtdsrv.f947b7ebca124db5a46086c0c9fe0cad">
+      <tp>
+        <v>2</v>
+        <stp/>
+        <stp>857843ea-07f9-44b3-a633-2328d20bb26f</stp>
+        <tr r="C10" s="6"/>
+      </tp>
+    </main>
+    <main first="rtdsrv.f947b7ebca124db5a46086c0c9fe0cad">
+      <tp>
+        <v>1</v>
+        <stp/>
+        <stp>6800ddd2-e1c7-49b2-9ad5-f9a5ded5266c</stp>
+        <tr r="G53" s="7"/>
+      </tp>
+    </main>
+    <main first="rtdsrv.f947b7ebca124db5a46086c0c9fe0cad">
+      <tp>
+        <v>2</v>
+        <stp/>
+        <stp>e61e6eb5-a5d7-486a-aa46-0d134a15ddd9</stp>
+        <tr r="G45" s="4"/>
+      </tp>
+      <tp>
+        <v>2</v>
+        <stp/>
+        <stp>8ccd80c6-7841-4f6e-b18a-ea81e894efd4</stp>
+        <tr r="G43" s="1"/>
+      </tp>
+    </main>
+    <main first="rtdsrv.f947b7ebca124db5a46086c0c9fe0cad">
+      <tp>
+        <v>2</v>
+        <stp/>
+        <stp>699e5996-1c34-49a5-ae20-ea62a4401e27</stp>
+        <tr r="D8" s="3"/>
+      </tp>
+    </main>
+    <main first="rtdsrv.f947b7ebca124db5a46086c0c9fe0cad">
+      <tp>
+        <v>2</v>
+        <stp/>
+        <stp>8388d227-5797-47f0-93c5-32f2f191ecbc</stp>
+        <tr r="P19" s="1"/>
+      </tp>
+      <tp>
+        <v>2</v>
+        <stp/>
+        <stp>09a17634-3b0b-4a09-820d-23c56cd1dbec</stp>
+        <tr r="G51" s="4"/>
+      </tp>
+    </main>
+    <main first="rtdsrv.f947b7ebca124db5a46086c0c9fe0cad">
+      <tp>
+        <v>1</v>
+        <stp/>
+        <stp>6ceeee8c-dbb1-4506-bce7-a3882dcccff5</stp>
+        <tr r="G52" s="7"/>
+      </tp>
+    </main>
+    <main first="rtdsrv.f947b7ebca124db5a46086c0c9fe0cad">
+      <tp>
+        <v>1</v>
+        <stp/>
+        <stp>8b140ba1-910b-4fd9-8b78-a455566005ce</stp>
+        <tr r="G5" s="3"/>
+      </tp>
+      <tp>
+        <v>1</v>
+        <stp/>
+        <stp>125059eb-d58e-4dbb-9804-b2bec676e9c7</stp>
+        <tr r="I28" s="7"/>
+      </tp>
+      <tp>
+        <v>2</v>
+        <stp/>
+        <stp>10b6bca6-bc2d-43dc-8672-752e54f27dab</stp>
+        <tr r="G50" s="4"/>
+      </tp>
+      <tp>
+        <v>2</v>
+        <stp/>
+        <stp>31620036-d26c-4140-9d55-7f1d5cb3fe0d</stp>
+        <tr r="G33" s="1"/>
+      </tp>
+    </main>
+    <main first="rtdsrv.f947b7ebca124db5a46086c0c9fe0cad">
+      <tp>
+        <v>1</v>
+        <stp/>
+        <stp>68d767fd-3f48-4c7b-a2bd-e83114b6a03d</stp>
+        <tr r="G48" s="7"/>
+      </tp>
+      <tp>
+        <v>2</v>
+        <stp/>
+        <stp>7ca18702-9a4f-4894-92e3-f9cded169a21</stp>
+        <tr r="G55" s="1"/>
+      </tp>
+      <tp>
+        <v>2</v>
+        <stp/>
+        <stp>045d9f65-7a24-4ba6-a807-13982ecd35b3</stp>
+        <tr r="D30" s="5"/>
+      </tp>
+    </main>
+    <main first="rtdsrv.f947b7ebca124db5a46086c0c9fe0cad">
+      <tp>
+        <v>2</v>
+        <stp/>
+        <stp>e685f2e5-de19-4671-86f9-0b550c3e773f</stp>
+        <tr r="G34" s="1"/>
+      </tp>
+      <tp>
+        <v>1</v>
+        <stp/>
+        <stp>1bab10b7-64d2-4aa2-b5f6-c7ef17a5d122</stp>
+        <tr r="G39" s="7"/>
+      </tp>
+    </main>
+    <main first="rtdsrv.f947b7ebca124db5a46086c0c9fe0cad">
+      <tp>
+        <v>2</v>
+        <stp/>
+        <stp>50acd600-eeb8-4762-8b05-f3783c41d0a9</stp>
+        <tr r="G48" s="4"/>
+      </tp>
+      <tp>
+        <v>2</v>
+        <stp/>
+        <stp>2a7f5b97-6f58-42f8-8488-f7a875f7a685</stp>
+        <tr r="G51" s="1"/>
+      </tp>
+      <tp>
+        <v>2</v>
+        <stp/>
+        <stp>19ef5492-32f0-4301-8c75-e33552478868</stp>
+        <tr r="G41" s="1"/>
+      </tp>
+    </main>
+    <main first="rtdsrv.f947b7ebca124db5a46086c0c9fe0cad">
+      <tp>
+        <v>2</v>
+        <stp/>
+        <stp>1943e18a-9b90-4ee0-980d-4183022cd055</stp>
+        <tr r="G37" s="1"/>
+      </tp>
+      <tp>
+        <v>2</v>
+        <stp/>
+        <stp>4bcb3b3f-be70-4bf0-81a0-484e394a2098</stp>
+        <tr r="G42" s="4"/>
+      </tp>
+    </main>
+    <main first="rtdsrv.f947b7ebca124db5a46086c0c9fe0cad">
+      <tp>
+        <v>1</v>
+        <stp/>
+        <stp>ad777002-53d7-4e8b-8a03-7eef769c4b99</stp>
+        <tr r="G28" s="7"/>
+      </tp>
+    </main>
+    <main first="rtdsrv.f947b7ebca124db5a46086c0c9fe0cad">
+      <tp>
+        <v>2</v>
+        <stp/>
+        <stp>96dea021-e4f7-41af-901f-324d256a507d</stp>
+        <tr r="G52" s="1"/>
+      </tp>
+      <tp>
+        <v>2</v>
+        <stp/>
+        <stp>7c41e32b-a3b5-4e3f-be30-bcfe43b80734</stp>
+        <tr r="F6" s="1"/>
+      </tp>
+      <tp>
+        <v>2</v>
+        <stp/>
+        <stp>93d39973-0bc4-499d-b9f4-00e36374f8e8</stp>
+        <tr r="G31" s="4"/>
+      </tp>
+      <tp>
+        <v>1</v>
+        <stp/>
+        <stp>2bf925f1-3406-4213-b470-6d562a126f32</stp>
+        <tr r="G36" s="7"/>
+      </tp>
+      <tp>
+        <v>1</v>
+        <stp/>
+        <stp>8ae002dd-7aad-4d98-8363-f8db007fba32</stp>
+        <tr r="H7" s="3"/>
+      </tp>
+    </main>
+    <main first="rtdsrv.f947b7ebca124db5a46086c0c9fe0cad">
+      <tp>
+        <v>2</v>
+        <stp/>
+        <stp>179af7c5-23bd-45f8-bb93-197b41e0b820</stp>
+        <tr r="G35" s="1"/>
+      </tp>
+      <tp>
+        <v>2</v>
+        <stp/>
+        <stp>b07552e1-0107-4ba7-b10a-3ffaf1041a1e</stp>
+        <tr r="F1" s="1"/>
+      </tp>
+      <tp>
+        <v>2</v>
+        <stp/>
+        <stp>b590959a-3708-428b-a661-47ab465fee1d</stp>
+        <tr r="I19" s="1"/>
+      </tp>
+      <tp>
+        <v>2</v>
+        <stp/>
+        <stp>222f77c5-794f-44b1-b7f6-277615541d40</stp>
+        <tr r="G43" s="4"/>
+      </tp>
+      <tp>
+        <v>2</v>
+        <stp/>
+        <stp>0ccef164-5079-47fb-b507-37864c4fab56</stp>
+        <tr r="G54" s="4"/>
+      </tp>
+    </main>
+    <main first="rtdsrv.f947b7ebca124db5a46086c0c9fe0cad">
+      <tp>
+        <v>1</v>
+        <stp/>
+        <stp>715ee365-42c7-4690-9f29-dd86b9effeb3</stp>
+        <tr r="G49" s="7"/>
+      </tp>
+    </main>
+    <main first="rtdsrv.f947b7ebca124db5a46086c0c9fe0cad">
+      <tp>
+        <v>1</v>
+        <stp/>
+        <stp>309fb272-8ed4-4efc-bebf-9b24a7735b6e</stp>
+        <tr r="G19" s="7"/>
+      </tp>
+      <tp>
+        <v>1</v>
+        <stp/>
+        <stp>c826d994-8a4d-4aa2-bcc5-2e89095b5863</stp>
+        <tr r="G31" s="7"/>
+      </tp>
+    </main>
+    <main first="rtdsrv.f947b7ebca124db5a46086c0c9fe0cad">
+      <tp>
+        <v>2</v>
+        <stp/>
+        <stp>b5296717-70a9-4ae7-b1bd-700fd839cd2e</stp>
+        <tr r="G56" s="1"/>
+      </tp>
+      <tp>
+        <v>2</v>
+        <stp/>
+        <stp>33a34cf3-e8e1-4fe6-a319-7812b7ec2126</stp>
         <tr r="F6" s="4"/>
       </tp>
       <tp>
         <v>2</v>
         <stp/>
-        <stp>b1fb4f5d-4216-4966-800c-b95425bcdcc5</stp>
-        <tr r="G24" s="4"/>
+        <stp>62d36e69-4ef9-41b9-94dd-e15e302e539b</stp>
+        <tr r="G39" s="4"/>
+      </tp>
+      <tp>
+        <v>1</v>
+        <stp/>
+        <stp>b1c5ec70-1878-4096-bd77-d92c34e6bca0</stp>
+        <tr r="G35" s="7"/>
       </tp>
     </main>
-    <main first="rtdsrv.e9e679e6621d402baf5d71ad7ce809cc">
-      <tp>
-        <v>1</v>
-        <stp/>
-        <stp>e75657d8-9205-4917-8910-fdaa52143c2d</stp>
+    <main first="rtdsrv.f947b7ebca124db5a46086c0c9fe0cad">
+      <tp>
+        <v>2</v>
+        <stp/>
+        <stp>c7e8a5d0-517d-4aef-8b63-29b67a2b4286</stp>
+        <tr r="I33" s="4"/>
+      </tp>
+    </main>
+    <main first="rtdsrv.f947b7ebca124db5a46086c0c9fe0cad">
+      <tp>
+        <v>1</v>
+        <stp/>
+        <stp>f4ababdb-f805-481c-a225-a61b189e3a18</stp>
+        <tr r="G56" s="7"/>
+      </tp>
+    </main>
+    <main first="rtdsrv.f947b7ebca124db5a46086c0c9fe0cad">
+      <tp>
+        <v>1</v>
+        <stp/>
+        <stp>20697eb6-d9e4-4768-bdc3-72bbcb5e7449</stp>
         <tr r="G7" s="3"/>
       </tp>
       <tp>
         <v>2</v>
         <stp/>
-        <stp>d74aef44-17c6-4a26-9f62-e91a33dfba84</stp>
-        <tr r="G54" s="1"/>
+        <stp>772f485b-88c8-46eb-acc6-baaa3ae1e82c</stp>
+        <tr r="G27" s="4"/>
       </tp>
       <tp>
         <v>2</v>
         <stp/>
-        <stp>327762f6-f2cc-4efa-9078-050548aa76c1</stp>
-        <tr r="G45" s="4"/>
+        <stp>10ea3d37-ef24-4037-b385-a134b44a65dd</stp>
+        <tr r="G40" s="1"/>
       </tp>
     </main>
-    <main first="rtdsrv.e9e679e6621d402baf5d71ad7ce809cc">
+    <main first="rtdsrv.f947b7ebca124db5a46086c0c9fe0cad">
       <tp>
         <v>2</v>
         <stp/>
-        <stp>c4aa2dda-12e8-45a4-b913-bb81a589f889</stp>
-        <tr r="G23" s="1"/>
+        <stp>e28db441-8124-4353-9be1-ef8e3fbf3f90</stp>
+        <tr r="G34" s="4"/>
       </tp>
       <tp>
         <v>2</v>
         <stp/>
-        <stp>b24210b4-a755-45fc-9ca3-ba79738c18b8</stp>
-        <tr r="G23" s="4"/>
-      </tp>
+        <stp>e4cffb26-1014-42d9-a307-64ad56b46ccb</stp>
+        <tr r="G48" s="1"/>
+      </tp>
+    </main>
+    <main first="rtdsrv.f947b7ebca124db5a46086c0c9fe0cad">
       <tp>
         <v>2</v>
         <stp/>
-        <stp>d85171bc-beeb-41da-85c4-fca9f4eae596</stp>
-        <tr r="F4" s="3"/>
-      </tp>
-      <tp>
-        <v>1</v>
-        <stp/>
-        <stp>33fdf581-872b-4aa1-b27c-e3588968a925</stp>
-        <tr r="F1" s="7"/>
+        <stp>599bb0bc-7139-4c2b-9fff-95f1109b5077</stp>
+        <tr r="G42" s="1"/>
+      </tp>
+      <tp>
+        <v>1</v>
+        <stp/>
+        <stp>d096bc01-662b-4134-9529-3024595f3ed7</stp>
+        <tr r="F6" s="7"/>
       </tp>
     </main>
-    <main first="rtdsrv.e9e679e6621d402baf5d71ad7ce809cc">
+    <main first="rtdsrv.f947b7ebca124db5a46086c0c9fe0cad">
       <tp>
         <v>2</v>
         <stp/>
-        <stp>3e0d2caa-1dc3-4f22-a17f-66acf73eb871</stp>
-        <tr r="G52" s="1"/>
+        <stp>3c829717-05b3-453f-9519-97d3e27dd975</stp>
+        <tr r="P67" s="1"/>
+      </tp>
+    </main>
+    <main first="rtdsrv.f947b7ebca124db5a46086c0c9fe0cad">
+      <tp>
+        <v>1</v>
+        <stp/>
+        <stp>b50d0dae-9717-4dd7-a262-954520049c9a</stp>
+        <tr r="G55" s="7"/>
       </tp>
       <tp>
         <v>2</v>
         <stp/>
-        <stp>022d2070-d5c9-41fc-a782-e93ac9ae36ae</stp>
-        <tr r="G49" s="1"/>
+        <stp>1c4f0498-2dca-47ff-b110-7a8658e63c1e</stp>
+        <tr r="G26" s="1"/>
       </tp>
     </main>
-    <main first="rtdsrv.e9e679e6621d402baf5d71ad7ce809cc">
+    <main first="rtdsrv.f947b7ebca124db5a46086c0c9fe0cad">
       <tp>
         <v>2</v>
         <stp/>
-        <stp>233ea251-9794-4ede-b7ac-c41c676d876e</stp>
-        <tr r="G56" s="4"/>
+        <stp>b4186636-6ab1-4f72-aa01-08de3c303e57</stp>
+        <tr r="F1" s="4"/>
       </tp>
     </main>
-    <main first="rtdsrv.e9e679e6621d402baf5d71ad7ce809cc">
+    <main first="rtdsrv.f947b7ebca124db5a46086c0c9fe0cad">
       <tp>
         <v>2</v>
         <stp/>
-        <stp>cd1417b6-d08f-45ae-928e-654eade3e3b7</stp>
-        <tr r="G21" s="4"/>
+        <stp>dbd084e8-0625-4fed-af98-d335501380a6</stp>
+        <tr r="G44" s="1"/>
       </tp>
     </main>
-    <main first="rtdsrv.e9e679e6621d402baf5d71ad7ce809cc">
-      <tp>
-        <v>1</v>
-        <stp/>
-        <stp>1cb7fbb4-e043-4e89-aff3-f4f004787285</stp>
-        <tr r="G40" s="7"/>
-      </tp>
-    </main>
-    <main first="rtdsrv.e9e679e6621d402baf5d71ad7ce809cc">
-      <tp>
-        <v>1</v>
-        <stp/>
-        <stp>9e78f2bb-4ac3-489b-a141-5f6fc9dfac19</stp>
-        <tr r="G53" s="7"/>
-      </tp>
-      <tp>
-        <v>1</v>
-        <stp/>
-        <stp>29173679-d34d-410d-9e5f-4171348756bb</stp>
-        <tr r="G43" s="7"/>
-      </tp>
+    <main first="rtdsrv.f947b7ebca124db5a46086c0c9fe0cad">
       <tp>
         <v>2</v>
         <stp/>
-        <stp>60e4a127-ec42-45c4-9fbb-6d3d49d53f76</stp>
-        <tr r="G46" s="4"/>
-      </tp>
-    </main>
-    <main first="rtdsrv.e9e679e6621d402baf5d71ad7ce809cc">
-      <tp>
-        <v>2</v>
-        <stp/>
-        <stp>1941794a-23a4-4fa9-884d-a40b3cd6aa10</stp>
-        <tr r="P74" s="1"/>
-      </tp>
-      <tp>
-        <v>1</v>
-        <stp/>
-        <stp>5a3506db-b0f0-4d26-ace8-e9a034467eba</stp>
-        <tr r="G37" s="7"/>
-      </tp>
-    </main>
-    <main first="rtdsrv.e9e679e6621d402baf5d71ad7ce809cc">
-      <tp>
-        <v>2</v>
-        <stp/>
-        <stp>6d4c8086-aec7-4ca4-ae7d-c6c036d7b807</stp>
-        <tr r="G20" s="4"/>
-      </tp>
-      <tp>
-        <v>2</v>
-        <stp/>
-        <stp>e988b699-486d-4dfb-93c3-95e49dc65e6d</stp>
-        <tr r="P19" s="1"/>
-      </tp>
-      <tp>
-        <v>2</v>
-        <stp/>
-        <stp>2a3fb5d6-ba2e-40dc-a5a5-2671a853c470</stp>
-        <tr r="G33" s="1"/>
-      </tp>
-    </main>
-    <main first="rtdsrv.e9e679e6621d402baf5d71ad7ce809cc">
-      <tp>
-        <v>2</v>
-        <stp/>
-        <stp>3c43a87a-121b-4fdb-8234-c335c554b316</stp>
-        <tr r="G39" s="1"/>
-      </tp>
-      <tp>
-        <v>2</v>
-        <stp/>
-        <stp>20ca0e0a-4e1f-46e8-9e67-7c56c5acd60c</stp>
-        <tr r="G29" s="4"/>
-      </tp>
-    </main>
-    <main first="rtdsrv.e9e679e6621d402baf5d71ad7ce809cc">
-      <tp>
-        <v>2</v>
-        <stp/>
-        <stp>eef9688d-68f9-4e26-98e8-a9d0d6fc78ae</stp>
-        <tr r="G41" s="4"/>
-      </tp>
-    </main>
-    <main first="rtdsrv.e9e679e6621d402baf5d71ad7ce809cc">
-      <tp>
-        <v>2</v>
-        <stp/>
-        <stp>2473af4c-a7a5-44f1-bdc5-b870dd8651bf</stp>
-        <tr r="I33" s="4"/>
-      </tp>
-    </main>
-    <main first="rtdsrv.e9e679e6621d402baf5d71ad7ce809cc">
-      <tp>
-        <v>2</v>
-        <stp/>
-        <stp>a4329483-82d3-40ef-9897-3b1211b2d8a5</stp>
-        <tr r="G27" s="1"/>
-      </tp>
-      <tp>
-        <v>1</v>
-        <stp/>
-        <stp>8b47aec0-7947-453a-8798-b1146015eebe</stp>
-        <tr r="H7" s="3"/>
-      </tp>
-    </main>
-    <main first="rtdsrv.e9e679e6621d402baf5d71ad7ce809cc">
-      <tp>
-        <v>2</v>
-        <stp/>
-        <stp>836248d6-1a6e-4680-bb77-305a4d695da1</stp>
-        <tr r="G41" s="1"/>
-      </tp>
-      <tp>
-        <v>2</v>
-        <stp/>
-        <stp>b4491249-f6c2-4c2b-a082-895239a7b77c</stp>
-        <tr r="G57" s="4"/>
-      </tp>
-    </main>
-    <main first="rtdsrv.e9e679e6621d402baf5d71ad7ce809cc">
-      <tp>
-        <v>2</v>
-        <stp/>
-        <stp>9e163131-4a4a-4abb-9c4f-5e9a75f23d49</stp>
-        <tr r="G19" s="1"/>
-      </tp>
-      <tp>
-        <v>2</v>
-        <stp/>
-        <stp>ae319cc9-cc66-429f-bf00-d032e50414ea</stp>
-        <tr r="D35" s="5"/>
-      </tp>
-      <tp>
-        <v>2</v>
-        <stp/>
-        <stp>747cd138-c3ce-426a-8d25-a92678ca7668</stp>
-        <tr r="G28" s="1"/>
-      </tp>
-    </main>
-    <main first="rtdsrv.e9e679e6621d402baf5d71ad7ce809cc">
-      <tp>
-        <v>2</v>
-        <stp/>
-        <stp>1d5e7c68-a152-4e3f-8622-2793537ad438</stp>
-        <tr r="F1" s="1"/>
-      </tp>
-    </main>
-    <main first="rtdsrv.e9e679e6621d402baf5d71ad7ce809cc">
-      <tp>
-        <v>2</v>
-        <stp/>
-        <stp>eb4709ce-be48-4352-aa80-fff935152bde</stp>
-        <tr r="G38" s="1"/>
-      </tp>
-      <tp>
-        <v>2</v>
-        <stp/>
-        <stp>152b946a-9d6e-42e6-a0ea-781c4453fe66</stp>
-        <tr r="F6" s="3"/>
-      </tp>
-    </main>
-    <main first="rtdsrv.e9e679e6621d402baf5d71ad7ce809cc">
-      <tp>
-        <v>1</v>
-        <stp/>
-        <stp>65d6935e-d99e-4406-bace-1caf4c53b41b</stp>
-        <tr r="G33" s="7"/>
-      </tp>
-    </main>
-    <main first="rtdsrv.e9e679e6621d402baf5d71ad7ce809cc">
-      <tp>
-        <v>1</v>
-        <stp/>
-        <stp>d732be89-1a80-47cf-b3fd-13567628fe2c</stp>
-        <tr r="G8" s="3"/>
-      </tp>
-    </main>
-    <main first="rtdsrv.e9e679e6621d402baf5d71ad7ce809cc">
-      <tp>
-        <v>1</v>
-        <stp/>
-        <stp>b5590201-ab7f-4a9f-9f0a-5e7d83c5eeeb</stp>
-        <tr r="G27" s="7"/>
-      </tp>
-      <tp>
-        <v>2</v>
-        <stp/>
-        <stp>288eab39-57cd-4a32-a0aa-debc38819b68</stp>
-        <tr r="G22" s="1"/>
-      </tp>
-      <tp>
-        <v>1</v>
-        <stp/>
-        <stp>1b4a9e0d-65cc-4c16-a5b5-03de9e6fc0d7</stp>
-        <tr r="G31" s="7"/>
-      </tp>
-      <tp>
-        <v>2</v>
-        <stp/>
-        <stp>30901615-b53c-4a81-b3d3-55c22ffbebe7</stp>
-        <tr r="B5" s="5"/>
-      </tp>
-    </main>
-    <main first="rtdsrv.e9e679e6621d402baf5d71ad7ce809cc">
-      <tp>
-        <v>2</v>
-        <stp/>
-        <stp>fa89e121-159a-4d70-bfb5-197528c1d25f</stp>
-        <tr r="G46" s="1"/>
-      </tp>
-      <tp>
-        <v>2</v>
-        <stp/>
-        <stp>b55a17fe-5bdd-475c-8864-8dfcdc097e70</stp>
-        <tr r="G55" s="1"/>
-      </tp>
-    </main>
-    <main first="rtdsrv.e9e679e6621d402baf5d71ad7ce809cc">
-      <tp>
-        <v>2</v>
-        <stp/>
-        <stp>eb5810e2-608b-409f-a35d-01997b4b0d62</stp>
-        <tr r="G55" s="4"/>
-      </tp>
-    </main>
-    <main first="rtdsrv.e9e679e6621d402baf5d71ad7ce809cc">
-      <tp>
-        <v>2</v>
-        <stp/>
-        <stp>8e2b0e54-d204-4256-8ba0-8ce31e88847e</stp>
-        <tr r="G34" s="1"/>
-      </tp>
-    </main>
-    <main first="rtdsrv.e9e679e6621d402baf5d71ad7ce809cc">
-      <tp>
-        <v>2</v>
-        <stp/>
-        <stp>0fdcaa91-4b73-4512-a134-445c9400f3df</stp>
-        <tr r="P29" s="1"/>
-      </tp>
-    </main>
-    <main first="rtdsrv.e9e679e6621d402baf5d71ad7ce809cc">
-      <tp>
-        <v>1</v>
-        <stp/>
-        <stp>2285d762-d409-4296-8759-1c814f167f47</stp>
-        <tr r="G26" s="7"/>
-      </tp>
-      <tp>
-        <v>1</v>
-        <stp/>
-        <stp>b0cafb50-c1a7-4917-9fdd-9092de5b565c</stp>
-        <tr r="P29" s="7"/>
-      </tp>
-    </main>
-    <main first="rtdsrv.e9e679e6621d402baf5d71ad7ce809cc">
-      <tp>
-        <v>2</v>
-        <stp/>
-        <stp>4bab67fe-7dca-494e-951e-425b25c05788</stp>
-        <tr r="G47" s="4"/>
-      </tp>
-      <tp>
-        <v>1</v>
-        <stp/>
-        <stp>5ad2087a-8a76-4717-9b1d-9ed64a8d6ec6</stp>
-        <tr r="P74" s="7"/>
-      </tp>
-      <tp>
-        <v>1</v>
-        <stp/>
-        <stp>3b699b30-6ace-48ca-88ec-036a068481c6</stp>
-        <tr r="G54" s="7"/>
-      </tp>
-      <tp>
-        <v>2</v>
-        <stp/>
-        <stp>4089ce51-6e96-480d-aef7-33e740788df7</stp>
-        <tr r="G20" s="1"/>
-      </tp>
-      <tp>
-        <v>2</v>
-        <stp/>
-        <stp>ef61032a-2b7e-479d-8a1b-bad7035e2f21</stp>
-        <tr r="G36" s="4"/>
-      </tp>
-      <tp>
-        <v>2</v>
-        <stp/>
-        <stp>d2d231d0-47c8-4ffb-8cc5-7d1aebbb566f</stp>
-        <tr r="I38" s="4"/>
-      </tp>
-    </main>
-    <main first="rtdsrv.e9e679e6621d402baf5d71ad7ce809cc">
-      <tp>
-        <v>2</v>
-        <stp/>
-        <stp>4a6af1a3-06ea-44f2-af3d-6ce4d253566d</stp>
-        <tr r="G52" s="4"/>
-      </tp>
-      <tp>
-        <v>1</v>
-        <stp/>
-        <stp>cd8abe01-440c-47fd-b3a4-9742153dd447</stp>
-        <tr r="G34" s="7"/>
-      </tp>
-    </main>
-    <main first="rtdsrv.e9e679e6621d402baf5d71ad7ce809cc">
-      <tp>
-        <v>1</v>
-        <stp/>
-        <stp>07471017-6355-48e1-8a34-4362e68e2088</stp>
-        <tr r="G32" s="7"/>
-      </tp>
-    </main>
-    <main first="rtdsrv.e9e679e6621d402baf5d71ad7ce809cc">
-      <tp>
-        <v>1</v>
-        <stp/>
-        <stp>aa083d57-5cc6-47eb-90eb-865013d344cf</stp>
-        <tr r="G45" s="7"/>
-      </tp>
-    </main>
-    <main first="rtdsrv.e9e679e6621d402baf5d71ad7ce809cc">
-      <tp>
-        <v>1</v>
-        <stp/>
-        <stp>0f1d9e25-8562-4a69-b063-420a7bc41bf5</stp>
-        <tr r="G41" s="7"/>
-      </tp>
-      <tp>
-        <v>2</v>
-        <stp/>
-        <stp>1cd1eb24-b5a9-4962-ad0a-045580bb0ced</stp>
-        <tr r="D8" s="3"/>
-      </tp>
-    </main>
-    <main first="rtdsrv.e9e679e6621d402baf5d71ad7ce809cc">
-      <tp>
-        <v>1</v>
-        <stp/>
-        <stp>f5c74ec1-3539-4676-9bc9-46c8aeeedbbc</stp>
-        <tr r="G36" s="7"/>
-      </tp>
-      <tp>
-        <v>1</v>
-        <stp/>
-        <stp>462fd044-438f-42c2-bca7-ef859537b5af</stp>
-        <tr r="G49" s="7"/>
-      </tp>
-    </main>
-    <main first="rtdsrv.e9e679e6621d402baf5d71ad7ce809cc">
-      <tp>
-        <v>2</v>
-        <stp/>
-        <stp>d1dc9079-2d50-4ae5-b81e-74500561116f</stp>
-        <tr r="F7" s="3"/>
-      </tp>
-      <tp>
-        <v>1</v>
-        <stp/>
-        <stp>bc352835-f26b-47ca-93fe-c28b67966840</stp>
-        <tr r="G6" s="3"/>
-      </tp>
-      <tp>
-        <v>2</v>
-        <stp/>
-        <stp>0fe8c6b2-c96c-4cfb-8953-c31fe1b18ab1</stp>
-        <tr r="G31" s="4"/>
-      </tp>
-      <tp>
-        <v>2</v>
-        <stp/>
-        <stp>f858fbf7-6964-477b-ad65-09dc0020d65f</stp>
-        <tr r="G44" s="1"/>
-      </tp>
-      <tp>
-        <v>2</v>
-        <stp/>
-        <stp>805c5868-e855-41df-a739-58aff0caa798</stp>
-        <tr r="G40" s="4"/>
-      </tp>
-      <tp>
-        <v>2</v>
-        <stp/>
-        <stp>53cff610-e785-4cc1-b1ba-eecbfae27055</stp>
-        <tr r="G53" s="4"/>
-      </tp>
-    </main>
-    <main first="rtdsrv.e9e679e6621d402baf5d71ad7ce809cc">
-      <tp>
-        <v>2</v>
-        <stp/>
-        <stp>5edf0faa-64b6-462d-877f-a75a15269ccc</stp>
-        <tr r="G44" s="4"/>
-      </tp>
-    </main>
-    <main first="rtdsrv.e9e679e6621d402baf5d71ad7ce809cc">
-      <tp>
-        <v>2</v>
-        <stp/>
-        <stp>8274d1a8-f46e-49cc-8ff9-4d50484c2813</stp>
-        <tr r="G48" s="4"/>
-      </tp>
-    </main>
-    <main first="rtdsrv.e9e679e6621d402baf5d71ad7ce809cc">
-      <tp>
-        <v>2</v>
-        <stp/>
-        <stp>0a2ce789-6658-4919-8d8b-1ec974472478</stp>
-        <tr r="D25" s="5"/>
-      </tp>
-    </main>
-    <main first="rtdsrv.e9e679e6621d402baf5d71ad7ce809cc">
-      <tp>
-        <v>2</v>
-        <stp/>
-        <stp>41adec2e-7be3-4bbe-b609-a3305016b71e</stp>
-        <tr r="G25" s="1"/>
-      </tp>
-      <tp>
-        <v>1</v>
-        <stp/>
-        <stp>b3e99a89-0f07-4674-9c1c-e3f333c1acfd</stp>
-        <tr r="G47" s="7"/>
-      </tp>
-      <tp>
-        <v>1</v>
-        <stp/>
-        <stp>4058f969-9784-4281-8fe5-8f54d610603b</stp>
-        <tr r="I28" s="7"/>
-      </tp>
-      <tp>
-        <v>1</v>
-        <stp/>
-        <stp>54c3c8e2-8a46-4c9d-81ba-4de903d3ea14</stp>
-        <tr r="G5" s="3"/>
-      </tp>
-    </main>
-    <main first="rtdsrv.e9e679e6621d402baf5d71ad7ce809cc">
-      <tp>
-        <v>1</v>
-        <stp/>
-        <stp>f60de59a-475d-49cb-b5d4-6935181bf5fb</stp>
-        <tr r="F6" s="7"/>
-      </tp>
-    </main>
-    <main first="rtdsrv.e9e679e6621d402baf5d71ad7ce809cc">
-      <tp>
-        <v>2</v>
-        <stp/>
-        <stp>5ba40365-34ce-4f75-82e3-cfa53ffa170f</stp>
-        <tr r="G28" s="4"/>
-      </tp>
-    </main>
-    <main first="rtdsrv.e9e679e6621d402baf5d71ad7ce809cc">
-      <tp>
-        <v>2</v>
-        <stp/>
-        <stp>95b6fe7e-770c-4b79-bb23-c6fdd937dfe3</stp>
-        <tr r="G53" s="1"/>
-      </tp>
-      <tp>
-        <v>1</v>
-        <stp/>
-        <stp>3956bbbc-ef63-4456-a9f8-7cf6c1e92963</stp>
-        <tr r="G48" s="7"/>
-      </tp>
-      <tp>
-        <v>1</v>
-        <stp/>
-        <stp>f6681d96-7041-4e24-8200-4635410edc15</stp>
-        <tr r="G24" s="7"/>
-      </tp>
-    </main>
-    <main first="rtdsrv.e9e679e6621d402baf5d71ad7ce809cc">
-      <tp>
-        <v>2</v>
-        <stp/>
-        <stp>6ad6e353-2e97-4964-87b4-a937d0d24e9a</stp>
-        <tr r="G35" s="1"/>
-      </tp>
-    </main>
-    <main first="rtdsrv.e9e679e6621d402baf5d71ad7ce809cc">
-      <tp>
-        <v>2</v>
-        <stp/>
-        <stp>9a9d0bda-5643-442d-b140-1a5d989eeeda</stp>
-        <tr r="D30" s="5"/>
-      </tp>
-    </main>
-    <main first="rtdsrv.e9e679e6621d402baf5d71ad7ce809cc">
-      <tp>
-        <v>1</v>
-        <stp/>
-        <stp>ea46f39e-678d-4859-9705-5c83c33f1e00</stp>
-        <tr r="G19" s="7"/>
-      </tp>
-    </main>
-    <main first="rtdsrv.e9e679e6621d402baf5d71ad7ce809cc">
-      <tp>
-        <v>2</v>
-        <stp/>
-        <stp>e37e5de4-f4d1-4c12-9ee8-89d1a5bd9347</stp>
-        <tr r="G39" s="4"/>
-      </tp>
-    </main>
-    <main first="rtdsrv.e9e679e6621d402baf5d71ad7ce809cc">
-      <tp>
-        <v>1</v>
-        <stp/>
-        <stp>6fdb948b-bb8d-4f92-a37d-4979915d3d3f</stp>
-        <tr r="G50" s="7"/>
-      </tp>
-    </main>
-    <main first="rtdsrv.e9e679e6621d402baf5d71ad7ce809cc">
-      <tp>
-        <v>2</v>
-        <stp/>
-        <stp>337bf53c-4446-4d77-9593-e0ca9e1b6015</stp>
-        <tr r="D45" s="5"/>
-      </tp>
-    </main>
-    <main first="rtdsrv.e9e679e6621d402baf5d71ad7ce809cc">
-      <tp>
-        <v>1</v>
-        <stp/>
-        <stp>f2331c9d-365f-4f36-9be1-599a5bbdb34b</stp>
-        <tr r="G25" s="7"/>
-      </tp>
-    </main>
-    <main first="rtdsrv.e9e679e6621d402baf5d71ad7ce809cc">
-      <tp>
-        <v>2</v>
-        <stp/>
-        <stp>459123d1-5766-453e-be94-d2782a3a4eb0</stp>
-        <tr r="G26" s="4"/>
-      </tp>
-      <tp>
-        <v>1</v>
-        <stp/>
-        <stp>cc824bea-871a-4c9b-810b-b4159d3cdb12</stp>
-        <tr r="G21" s="7"/>
-      </tp>
-      <tp>
-        <v>1</v>
-        <stp/>
-        <stp>fcdbbfda-4f86-4243-8690-76bf02bfcfc7</stp>
-        <tr r="H6" s="3"/>
-      </tp>
-    </main>
-    <main first="rtdsrv.e9e679e6621d402baf5d71ad7ce809cc">
-      <tp>
-        <v>2</v>
-        <stp/>
-        <stp>2d980c35-94f2-445b-91a1-85415fb73010</stp>
-        <tr r="B2" s="6"/>
-      </tp>
-      <tp>
-        <v>2</v>
-        <stp/>
-        <stp>4022795b-cd70-49e1-8745-abd997425dbd</stp>
-        <tr r="G42" s="1"/>
-      </tp>
-      <tp>
-        <v>1</v>
-        <stp/>
-        <stp>1a3012b1-8ec2-4985-8ac8-140d231d9d30</stp>
-        <tr r="G46" s="7"/>
-      </tp>
-    </main>
-    <main first="rtdsrv.e9e679e6621d402baf5d71ad7ce809cc">
-      <tp>
-        <v>2</v>
-        <stp/>
-        <stp>c8776104-deb1-4245-8448-9dcac5cfbcb3</stp>
-        <tr r="G34" s="4"/>
-      </tp>
-      <tp>
-        <v>2</v>
-        <stp/>
-        <stp>beb498b7-246c-42b6-b9a5-cb719f4d0b9f</stp>
-        <tr r="G21" s="1"/>
-      </tp>
-      <tp>
-        <v>1</v>
-        <stp/>
-        <stp>c1665e7f-a000-486c-b8b9-c1cabcf0388d</stp>
-        <tr r="G55" s="7"/>
-      </tp>
-      <tp>
-        <v>1</v>
-        <stp/>
-        <stp>66955e8b-30ca-4287-9eab-ec08b275d9a9</stp>
-        <tr r="G20" s="7"/>
-      </tp>
-      <tp>
-        <v>2</v>
-        <stp/>
-        <stp>5777fa6e-23b8-4eb5-9320-16d988f0a361</stp>
-        <tr r="G37" s="1"/>
-      </tp>
-      <tp>
-        <v>2</v>
-        <stp/>
-        <stp>f5031817-6119-47f6-8016-55194d282325</stp>
-        <tr r="G30" s="1"/>
-      </tp>
-    </main>
-    <main first="rtdsrv.e9e679e6621d402baf5d71ad7ce809cc">
-      <tp>
-        <v>2</v>
-        <stp/>
-        <stp>34bd90e4-969b-4c78-891d-0bd7b9b0c1a3</stp>
-        <tr r="D6" s="3"/>
-      </tp>
-      <tp>
-        <v>1</v>
-        <stp/>
-        <stp>84cb5393-609d-4211-a6c7-13e0a86037d3</stp>
-        <tr r="G56" s="7"/>
-      </tp>
-    </main>
-    <main first="rtdsrv.e9e679e6621d402baf5d71ad7ce809cc">
-      <tp>
-        <v>2</v>
-        <stp/>
-        <stp>75c36322-ae20-4ad0-a01d-ee512d34c803</stp>
-        <tr r="G48" s="1"/>
-      </tp>
-      <tp>
-        <v>1</v>
-        <stp/>
-        <stp>96823ba7-90fc-45df-af68-b9bee8d6ec1d</stp>
-        <tr r="H8" s="3"/>
-      </tp>
-      <tp>
-        <v>2</v>
-        <stp/>
-        <stp>8ea51daa-1700-47a1-91cb-784faac6cdba</stp>
-        <tr r="G57" s="1"/>
-      </tp>
-    </main>
-    <main first="rtdsrv.e9e679e6621d402baf5d71ad7ce809cc">
-      <tp>
-        <v>1</v>
-        <stp/>
-        <stp>667e036d-b52b-49ab-b1f7-c49f50a0a8fb</stp>
-        <tr r="G42" s="7"/>
-      </tp>
-      <tp>
-        <v>1</v>
-        <stp/>
-        <stp>377a31d5-e859-4827-8ce3-f5069b3399ae</stp>
-        <tr r="G4" s="3"/>
-      </tp>
-      <tp>
-        <v>2</v>
-        <stp/>
-        <stp>5c58f884-5780-4af2-9fb1-70a7fff7177f</stp>
-        <tr r="D15" s="5"/>
-      </tp>
-      <tp>
-        <v>2</v>
-        <stp/>
-        <stp>77e135aa-3e1f-4728-8fd1-9306e587b4c3</stp>
-        <tr r="G47" s="1"/>
-      </tp>
-      <tp>
-        <v>2</v>
-        <stp/>
-        <stp>1f4798d1-a3f6-4ba3-8955-ac28135c26e0</stp>
-        <tr r="G38" s="4"/>
-      </tp>
-    </main>
-    <main first="rtdsrv.e9e679e6621d402baf5d71ad7ce809cc">
-      <tp>
-        <v>2</v>
-        <stp/>
-        <stp>d17c93f5-cd9d-41f2-906b-0f3f0ed96901</stp>
-        <tr r="I28" s="4"/>
-      </tp>
-    </main>
-    <main first="rtdsrv.e9e679e6621d402baf5d71ad7ce809cc">
-      <tp>
-        <v>2</v>
-        <stp/>
-        <stp>267a712d-7b04-4fb8-8daa-26e2d24f019b</stp>
-        <tr r="I28" s="1"/>
-      </tp>
-    </main>
-    <main first="rtdsrv.e9e679e6621d402baf5d71ad7ce809cc">
-      <tp>
-        <v>1</v>
-        <stp/>
-        <stp>037ba740-4bae-46eb-80b7-f7d6a8e0ec05</stp>
-        <tr r="G28" s="7"/>
-      </tp>
-      <tp>
-        <v>2</v>
-        <stp/>
-        <stp>982f664e-13dd-4d92-af52-6fc7837bf14b</stp>
-        <tr r="C6" s="6"/>
-      </tp>
-    </main>
-    <main first="rtdsrv.e9e679e6621d402baf5d71ad7ce809cc">
-      <tp>
-        <v>2</v>
-        <stp/>
-        <stp>158a94dc-ab63-418f-b207-11d5194ccbed</stp>
-        <tr r="C10" s="6"/>
-      </tp>
-    </main>
-    <main first="rtdsrv.e9e679e6621d402baf5d71ad7ce809cc">
-      <tp>
-        <v>2</v>
-        <stp/>
-        <stp>266bb827-38d7-4427-9d52-76ee9f6623e2</stp>
+        <stp>9f5e3b9c-479b-4d04-bcaa-8770b9c72ca5</stp>
         <tr r="I19" s="4"/>
         <tr r="I32" s="4"/>
       </tp>
     </main>
-    <main first="rtdsrv.e9e679e6621d402baf5d71ad7ce809cc">
+    <main first="rtdsrv.f947b7ebca124db5a46086c0c9fe0cad">
+      <tp>
+        <v>1</v>
+        <stp/>
+        <stp>4af39476-cca8-4084-a99f-85026b044ee8</stp>
+        <tr r="P19" s="7"/>
+      </tp>
+    </main>
+    <main first="rtdsrv.f947b7ebca124db5a46086c0c9fe0cad">
       <tp>
         <v>2</v>
         <stp/>
-        <stp>5d38ba0d-20da-46cc-a41a-6b2839e02b37</stp>
-        <tr r="G56" s="1"/>
+        <stp>bc8c654d-544f-4855-9785-35ba46817d3e</stp>
+        <tr r="D4" s="3"/>
+      </tp>
+      <tp>
+        <v>1</v>
+        <stp/>
+        <stp>de03541b-8121-4e42-ad5b-5c37819f958f</stp>
+        <tr r="G22" s="7"/>
       </tp>
     </main>
-    <main first="rtdsrv.e9e679e6621d402baf5d71ad7ce809cc">
+    <main first="rtdsrv.f947b7ebca124db5a46086c0c9fe0cad">
       <tp>
         <v>2</v>
         <stp/>
-        <stp>17121786-17bd-4da8-b260-a99049c64cf5</stp>
+        <stp>38906c11-479b-4bd4-b51c-16d7037fafeb</stp>
+        <tr r="G47" s="1"/>
+      </tp>
+    </main>
+    <main first="rtdsrv.f947b7ebca124db5a46086c0c9fe0cad">
+      <tp>
+        <v>2</v>
+        <stp/>
+        <stp>322c27e9-acf7-4a6f-a9a4-4e39f551e90f</stp>
+        <tr r="I42" s="4"/>
+      </tp>
+    </main>
+    <main first="rtdsrv.f947b7ebca124db5a46086c0c9fe0cad">
+      <tp>
+        <v>2</v>
+        <stp/>
+        <stp>14846879-1ec2-46cd-a3bd-2624807b972c</stp>
+        <tr r="G24" s="1"/>
+      </tp>
+    </main>
+    <main first="rtdsrv.f947b7ebca124db5a46086c0c9fe0cad">
+      <tp>
+        <v>1</v>
+        <stp/>
+        <stp>9fc53e1e-a024-4336-a57e-d85883774bb5</stp>
+        <tr r="G46" s="7"/>
+      </tp>
+    </main>
+    <main first="rtdsrv.f947b7ebca124db5a46086c0c9fe0cad">
+      <tp>
+        <v>2</v>
+        <stp/>
+        <stp>f08d4798-0f6d-46bc-9cc1-452d3091b865</stp>
+        <tr r="G20" s="1"/>
+      </tp>
+    </main>
+    <main first="rtdsrv.f947b7ebca124db5a46086c0c9fe0cad">
+      <tp>
+        <v>2</v>
+        <stp/>
+        <stp>c8f872f9-6991-47ec-b716-9905fe826979</stp>
+        <tr r="G53" s="1"/>
+      </tp>
+      <tp>
+        <v>2</v>
+        <stp/>
+        <stp>390a2b2b-e1ed-4867-9254-6b53ba36942a</stp>
+        <tr r="G46" s="1"/>
+      </tp>
+    </main>
+    <main first="rtdsrv.f947b7ebca124db5a46086c0c9fe0cad">
+      <tp>
+        <v>1</v>
+        <stp/>
+        <stp>4623cb07-3a25-490c-88fc-c14ea9da5a6d</stp>
+        <tr r="G47" s="7"/>
+      </tp>
+      <tp>
+        <v>2</v>
+        <stp/>
+        <stp>71a87a8b-b6a8-4758-94f1-936a82aa5fbb</stp>
+        <tr r="G30" s="4"/>
+      </tp>
+      <tp>
+        <v>2</v>
+        <stp/>
+        <stp>436a5f6b-5632-48b4-9747-b5ce07dac626</stp>
+        <tr r="G28" s="4"/>
+      </tp>
+      <tp>
+        <v>2</v>
+        <stp/>
+        <stp>645b5316-9c48-4302-b15f-b1f62eb8b919</stp>
+        <tr r="C6" s="6"/>
+      </tp>
+    </main>
+    <main first="rtdsrv.f947b7ebca124db5a46086c0c9fe0cad">
+      <tp>
+        <v>1</v>
+        <stp/>
+        <stp>b12fa1a1-734c-4044-8173-872a4f1401ad</stp>
+        <tr r="G45" s="7"/>
+      </tp>
+      <tp>
+        <v>2</v>
+        <stp/>
+        <stp>8c9971f8-1766-4a33-bec7-36e063d9abb2</stp>
+        <tr r="G52" s="4"/>
+      </tp>
+      <tp>
+        <v>1</v>
+        <stp/>
+        <stp>5460852d-44df-434a-b058-ab5cf6106a4a</stp>
+        <tr r="H5" s="3"/>
+      </tp>
+      <tp>
+        <v>2</v>
+        <stp/>
+        <stp>818ab1e6-f655-47f0-aec7-3ce5271ec53f</stp>
+        <tr r="G29" s="1"/>
+      </tp>
+      <tp>
+        <v>1</v>
+        <stp/>
+        <stp>f4cd5044-ed60-412c-a321-d7524adc727c</stp>
+        <tr r="G54" s="7"/>
+      </tp>
+      <tp>
+        <v>2</v>
+        <stp/>
+        <stp>41657bc5-e45e-402b-8e74-1b1afa6f1454</stp>
+        <tr r="G50" s="1"/>
+      </tp>
+      <tp>
+        <v>1</v>
+        <stp/>
+        <stp>110e3582-4e30-420a-8141-bf97c6ce7af6</stp>
+        <tr r="F1" s="7"/>
+      </tp>
+      <tp>
+        <v>1</v>
+        <stp/>
+        <stp>9db01a2f-053b-4990-b83c-3c5220d95156</stp>
+        <tr r="G25" s="7"/>
+      </tp>
+      <tp>
+        <v>2</v>
+        <stp/>
+        <stp>47f85db5-087e-426b-a700-70a77aa474f7</stp>
+        <tr r="G44" s="4"/>
+      </tp>
+    </main>
+    <main first="rtdsrv.f947b7ebca124db5a46086c0c9fe0cad">
+      <tp>
+        <v>1</v>
+        <stp/>
+        <stp>630d197d-d625-4d9c-ad8d-2316caab527f</stp>
+        <tr r="G21" s="7"/>
+      </tp>
+      <tp>
+        <v>2</v>
+        <stp/>
+        <stp>97b2e9d2-c6d1-42cc-b960-e7cb78a84b14</stp>
+        <tr r="B5" s="5"/>
+      </tp>
+      <tp>
+        <v>2</v>
+        <stp/>
+        <stp>6fb680ce-b314-4d8c-a57f-a0b7a49cd174</stp>
+        <tr r="G32" s="4"/>
+      </tp>
+      <tp>
+        <v>1</v>
+        <stp/>
+        <stp>dfb4f7df-a4a1-4f8b-9088-39069ef76c9d</stp>
+        <tr r="G29" s="7"/>
+      </tp>
+      <tp>
+        <v>2</v>
+        <stp/>
+        <stp>05ffd59f-f923-451a-9a0c-509f1015ebf2</stp>
+        <tr r="I28" s="1"/>
+      </tp>
+      <tp>
+        <v>2</v>
+        <stp/>
+        <stp>162cbcef-9f72-4253-ad95-84a6cb9d3fb8</stp>
+        <tr r="G30" s="1"/>
+      </tp>
+      <tp>
+        <v>2</v>
+        <stp/>
+        <stp>f90c26e9-8b3f-44e6-880c-b0628ed02298</stp>
+        <tr r="G40" s="4"/>
+      </tp>
+      <tp>
+        <v>2</v>
+        <stp/>
+        <stp>1d883798-4df3-4011-98da-209ab112ee30</stp>
+        <tr r="G47" s="4"/>
+      </tp>
+      <tp>
+        <v>2</v>
+        <stp/>
+        <stp>59954cae-4bec-48d6-b706-d35b296f6453</stp>
+        <tr r="G25" s="4"/>
+      </tp>
+      <tp>
+        <v>2</v>
+        <stp/>
+        <stp>2561c09e-8d3c-4927-941c-c393bfdc3862</stp>
+        <tr r="G36" s="1"/>
+      </tp>
+    </main>
+    <main first="rtdsrv.f947b7ebca124db5a46086c0c9fe0cad">
+      <tp>
+        <v>2</v>
+        <stp/>
+        <stp>1ba7419c-fc4c-4432-8e5d-a21030a82fc2</stp>
+        <tr r="I28" s="4"/>
+      </tp>
+      <tp>
+        <v>2</v>
+        <stp/>
+        <stp>e2faa3a3-026c-4aa8-9889-b67890122ada</stp>
+        <tr r="F4" s="3"/>
+      </tp>
+      <tp>
+        <v>1</v>
+        <stp/>
+        <stp>b0378cf4-4c40-4133-ac8e-db8159d63ade</stp>
+        <tr r="P74" s="7"/>
+      </tp>
+    </main>
+    <main first="rtdsrv.f947b7ebca124db5a46086c0c9fe0cad">
+      <tp>
+        <v>1</v>
+        <stp/>
+        <stp>575c47ff-b954-457e-8d20-979d20e50e0f</stp>
+        <tr r="G57" s="7"/>
+      </tp>
+      <tp>
+        <v>1</v>
+        <stp/>
+        <stp>432644d3-6e63-4094-ab8a-08dacb72301a</stp>
+        <tr r="G44" s="7"/>
+      </tp>
+      <tp>
+        <v>2</v>
+        <stp/>
+        <stp>f0adb8cf-cd42-486a-be72-4d28184706c2</stp>
+        <tr r="G28" s="1"/>
+      </tp>
+    </main>
+    <main first="rtdsrv.f947b7ebca124db5a46086c0c9fe0cad">
+      <tp>
+        <v>2</v>
+        <stp/>
+        <stp>91d8b6c6-b7d7-49ee-9f5a-e585a452dcb6</stp>
+        <tr r="G26" s="4"/>
+      </tp>
+      <tp>
+        <v>2</v>
+        <stp/>
+        <stp>9a504b69-a945-44f1-ab44-51e34360a2be</stp>
+        <tr r="B2" s="6"/>
+      </tp>
+    </main>
+    <main first="rtdsrv.f947b7ebca124db5a46086c0c9fe0cad">
+      <tp>
+        <v>1</v>
+        <stp/>
+        <stp>af5142b3-4bf8-431b-89a7-84f0f993a990</stp>
+        <tr r="I19" s="7"/>
+      </tp>
+      <tp>
+        <v>2</v>
+        <stp/>
+        <stp>42e1da87-f0c9-441b-9cf8-5543dad8b2a3</stp>
+        <tr r="G39" s="1"/>
+      </tp>
+    </main>
+    <main first="rtdsrv.f947b7ebca124db5a46086c0c9fe0cad">
+      <tp>
+        <v>1</v>
+        <stp/>
+        <stp>23a88f98-0ee5-4c7d-bfc2-9285dbe65e15</stp>
+        <tr r="G33" s="7"/>
+      </tp>
+    </main>
+    <main first="rtdsrv.f947b7ebca124db5a46086c0c9fe0cad">
+      <tp>
+        <v>2</v>
+        <stp/>
+        <stp>9d0891bb-5d0b-4648-87d3-703ef8c7ec9c</stp>
+        <tr r="F8" s="3"/>
+      </tp>
+    </main>
+    <main first="rtdsrv.f947b7ebca124db5a46086c0c9fe0cad">
+      <tp>
+        <v>1</v>
+        <stp/>
+        <stp>0db01588-4513-4d13-ad5b-671431e8222a</stp>
+        <tr r="H4" s="3"/>
+      </tp>
+    </main>
+    <main first="rtdsrv.f947b7ebca124db5a46086c0c9fe0cad">
+      <tp>
+        <v>2</v>
+        <stp/>
+        <stp>2e9a3567-20f9-47bf-ad6f-86097049ed87</stp>
+        <tr r="D35" s="5"/>
+      </tp>
+    </main>
+    <main first="rtdsrv.f947b7ebca124db5a46086c0c9fe0cad">
+      <tp>
+        <v>2</v>
+        <stp/>
+        <stp>8cceb3bd-ab95-491a-8c50-2568e5788557</stp>
+        <tr r="D15" s="5"/>
+      </tp>
+      <tp>
+        <v>1</v>
+        <stp/>
+        <stp>ec908f3e-ae60-4960-b5d3-5a6f8e457d9d</stp>
+        <tr r="G24" s="7"/>
+      </tp>
+    </main>
+    <main first="rtdsrv.f947b7ebca124db5a46086c0c9fe0cad">
+      <tp>
+        <v>1</v>
+        <stp/>
+        <stp>fe4d6309-e055-4021-9e52-e676d3b02b13</stp>
+        <tr r="P67" s="7"/>
+      </tp>
+      <tp>
+        <v>1</v>
+        <stp/>
+        <stp>d727f42d-6513-491a-9f5c-41f564d9c46a</stp>
+        <tr r="G43" s="7"/>
+      </tp>
+    </main>
+    <main first="rtdsrv.f947b7ebca124db5a46086c0c9fe0cad">
+      <tp>
+        <v>2</v>
+        <stp/>
+        <stp>f391ed1e-dd43-4ea5-afe8-7c74f7c81f68</stp>
+        <tr r="G57" s="1"/>
+      </tp>
+    </main>
+    <main first="rtdsrv.f947b7ebca124db5a46086c0c9fe0cad">
+      <tp>
+        <v>2</v>
+        <stp/>
+        <stp>a1755eba-e910-43b3-be25-4c25ef754dd0</stp>
+        <tr r="G29" s="4"/>
+      </tp>
+    </main>
+    <main first="rtdsrv.f947b7ebca124db5a46086c0c9fe0cad">
+      <tp>
+        <v>2</v>
+        <stp/>
+        <stp>d952c98c-38ab-439e-b6a9-a1afa4fe0cd4</stp>
+        <tr r="G37" s="4"/>
+      </tp>
+      <tp>
+        <v>2</v>
+        <stp/>
+        <stp>f6a975ff-dd82-4f31-bfb0-a195ec7d172e</stp>
+        <tr r="H5" s="5"/>
+      </tp>
+    </main>
+    <main first="rtdsrv.f947b7ebca124db5a46086c0c9fe0cad">
+      <tp>
+        <v>2</v>
+        <stp/>
+        <stp>19d71b3e-8448-4c23-982b-4a58def5d78c</stp>
+        <tr r="G32" s="1"/>
+      </tp>
+      <tp>
+        <v>2</v>
+        <stp/>
+        <stp>cff780ee-5410-43b5-b080-0907fa385d2e</stp>
+        <tr r="D5" s="3"/>
+      </tp>
+    </main>
+    <main first="rtdsrv.f947b7ebca124db5a46086c0c9fe0cad">
+      <tp>
+        <v>2</v>
+        <stp/>
+        <stp>b9799913-d92c-4d27-a569-35934d45ef71</stp>
+        <tr r="G38" s="1"/>
+      </tp>
+      <tp>
+        <v>2</v>
+        <stp/>
+        <stp>4a896586-e4d6-4f0d-81eb-6490fce03566</stp>
+        <tr r="D6" s="3"/>
+      </tp>
+      <tp>
+        <v>2</v>
+        <stp/>
+        <stp>3812a53a-b827-427a-9aba-5cc5993ddd59</stp>
+        <tr r="G54" s="1"/>
+      </tp>
+    </main>
+    <main first="rtdsrv.f947b7ebca124db5a46086c0c9fe0cad">
+      <tp>
+        <v>2</v>
+        <stp/>
+        <stp>133c73f8-6c3d-4e99-beda-ed110ed338b8</stp>
+        <tr r="G22" s="1"/>
+      </tp>
+    </main>
+    <main first="rtdsrv.f947b7ebca124db5a46086c0c9fe0cad">
+      <tp>
+        <v>1</v>
+        <stp/>
+        <stp>314a0294-bccf-4e37-b704-a28acdcf7bc4</stp>
+        <tr r="G50" s="7"/>
+      </tp>
+      <tp>
+        <v>2</v>
+        <stp/>
+        <stp>0ba9bfc8-ca15-41ff-9641-834ab15e6e0f</stp>
+        <tr r="G27" s="1"/>
+      </tp>
+    </main>
+    <main first="rtdsrv.f947b7ebca124db5a46086c0c9fe0cad">
+      <tp>
+        <v>2</v>
+        <stp/>
+        <stp>2d62c716-e580-4d75-b7e0-daa8f705ecff</stp>
+        <tr r="G21" s="1"/>
+      </tp>
+    </main>
+    <main first="rtdsrv.f947b7ebca124db5a46086c0c9fe0cad">
+      <tp>
+        <v>2</v>
+        <stp/>
+        <stp>2b1ad3b7-53ed-4e48-8b87-1b9526289c25</stp>
+        <tr r="G45" s="1"/>
+      </tp>
+    </main>
+    <main first="rtdsrv.f947b7ebca124db5a46086c0c9fe0cad">
+      <tp>
+        <v>2</v>
+        <stp/>
+        <stp>10f574ec-5b15-4851-91ec-b086f77a71d4</stp>
+        <tr r="G56" s="4"/>
+      </tp>
+      <tp>
+        <v>1</v>
+        <stp/>
+        <stp>7b3b0f55-f0aa-4dc2-bdca-6058de9e0519</stp>
+        <tr r="G51" s="7"/>
+      </tp>
+      <tp>
+        <v>2</v>
+        <stp/>
+        <stp>b3bf3a9e-28e3-41ee-90e9-d502952be326</stp>
+        <tr r="G31" s="1"/>
+      </tp>
+    </main>
+    <main first="rtdsrv.f947b7ebca124db5a46086c0c9fe0cad">
+      <tp>
+        <v>2</v>
+        <stp/>
+        <stp>e247614c-843b-49e2-a8c2-571da015811e</stp>
+        <tr r="G25" s="1"/>
+      </tp>
+      <tp>
+        <v>2</v>
+        <stp/>
+        <stp>3489830e-72fc-4526-9509-18bb3a3273ec</stp>
+        <tr r="D40" s="5"/>
+      </tp>
+      <tp>
+        <v>2</v>
+        <stp/>
+        <stp>184496fa-cc4f-411c-ae73-27077d2e160c</stp>
+        <tr r="G21" s="4"/>
+      </tp>
+    </main>
+    <main first="rtdsrv.f947b7ebca124db5a46086c0c9fe0cad">
+      <tp>
+        <v>2</v>
+        <stp/>
+        <stp>342b88b1-575f-45bd-956d-9adb428b1d73</stp>
+        <tr r="D50" s="5"/>
+      </tp>
+      <tp>
+        <v>2</v>
+        <stp/>
+        <stp>bd759504-928b-4264-a40a-a3252167328b</stp>
+        <tr r="G22" s="4"/>
+      </tp>
+    </main>
+    <main first="rtdsrv.f947b7ebca124db5a46086c0c9fe0cad">
+      <tp>
+        <v>1</v>
+        <stp/>
+        <stp>2d376dba-79c9-4105-9c00-bdcca83de2c4</stp>
+        <tr r="G38" s="7"/>
+      </tp>
+      <tp>
+        <v>2</v>
+        <stp/>
+        <stp>f0c51d1f-e552-4239-8255-7f36fd788bb7</stp>
+        <tr r="G19" s="1"/>
+      </tp>
+      <tp>
+        <v>2</v>
+        <stp/>
+        <stp>99612717-d683-46f5-85f7-ebeab51433fa</stp>
+        <tr r="G46" s="4"/>
+      </tp>
+    </main>
+    <main first="rtdsrv.f947b7ebca124db5a46086c0c9fe0cad">
+      <tp>
+        <v>2</v>
+        <stp/>
+        <stp>4f779b71-1632-4f26-8639-479a584fbb87</stp>
+        <tr r="F6" s="3"/>
+      </tp>
+      <tp>
+        <v>2</v>
+        <stp/>
+        <stp>546faadc-281d-410a-a39c-f9fcf80a4ce3</stp>
+        <tr r="I38" s="4"/>
+      </tp>
+      <tp>
+        <v>1</v>
+        <stp/>
+        <stp>4531e528-a59f-4f54-ad11-905428ea013d</stp>
+        <tr r="G6" s="3"/>
+      </tp>
+    </main>
+    <main first="rtdsrv.f947b7ebca124db5a46086c0c9fe0cad">
+      <tp>
+        <v>1</v>
+        <stp/>
+        <stp>d443590f-32f6-40b5-abc7-7554589ec8ed</stp>
+        <tr r="H8" s="3"/>
+      </tp>
+      <tp>
+        <v>1</v>
+        <stp/>
+        <stp>ed98de0a-bb6b-4c2e-b7bc-f4b41936142e</stp>
+        <tr r="G42" s="7"/>
+      </tp>
+      <tp>
+        <v>1</v>
+        <stp/>
+        <stp>17fe11df-c960-4d1e-9067-2982fc974294</stp>
+        <tr r="G4" s="3"/>
+      </tp>
+      <tp>
+        <v>2</v>
+        <stp/>
+        <stp>ae0d8d4f-d1cd-42b5-b25e-f06483e3287c</stp>
+        <tr r="G19" s="4"/>
+      </tp>
+    </main>
+    <main first="rtdsrv.f947b7ebca124db5a46086c0c9fe0cad">
+      <tp>
+        <v>1</v>
+        <stp/>
+        <stp>c8a82c79-58e2-4b37-b5bc-c043bd539141</stp>
+        <tr r="G34" s="7"/>
+      </tp>
+    </main>
+    <main first="rtdsrv.f947b7ebca124db5a46086c0c9fe0cad">
+      <tp>
+        <v>1</v>
+        <stp/>
+        <stp>8a1e1f9c-c7f2-40fa-9999-aca9be6f3ed5</stp>
+        <tr r="H6" s="3"/>
+      </tp>
+    </main>
+    <main first="rtdsrv.f947b7ebca124db5a46086c0c9fe0cad">
+      <tp>
+        <v>2</v>
+        <stp/>
+        <stp>8e9a4084-b597-44a8-812a-a048ed8256b8</stp>
+        <tr r="P29" s="1"/>
+      </tp>
+      <tp>
+        <v>2</v>
+        <stp/>
+        <stp>5774bf76-82dc-4ce0-8bab-42a3d3279ffe</stp>
+        <tr r="D45" s="5"/>
+      </tp>
+    </main>
+    <main first="rtdsrv.f947b7ebca124db5a46086c0c9fe0cad">
+      <tp>
+        <v>2</v>
+        <stp/>
+        <stp>93cfa075-b767-430d-ae8d-6401cd3502e6</stp>
+        <tr r="G57" s="4"/>
+      </tp>
+      <tp>
+        <v>1</v>
+        <stp/>
+        <stp>f75fe032-beb2-4d29-8fc5-940ba6825b26</stp>
+        <tr r="G32" s="7"/>
+      </tp>
+      <tp>
+        <v>1</v>
+        <stp/>
+        <stp>e05489d8-18ed-4166-9c20-045072dc6ed5</stp>
+        <tr r="G40" s="7"/>
+      </tp>
+      <tp>
+        <v>2</v>
+        <stp/>
+        <stp>51e9711c-beef-47af-adc1-691e238082fe</stp>
+        <tr r="D7" s="3"/>
+      </tp>
+    </main>
+    <main first="rtdsrv.f947b7ebca124db5a46086c0c9fe0cad">
+      <tp>
+        <v>2</v>
+        <stp/>
+        <stp>5d6228aa-e757-4625-b0bf-ca7dfcaeb382</stp>
         <tr r="D20" s="5"/>
       </tp>
-      <tp>
-        <v>1</v>
-        <stp/>
-        <stp>57f98e78-c621-481a-a408-88b546dca35b</stp>
-        <tr r="H5" s="3"/>
-      </tp>
     </main>
-    <main first="rtdsrv.e9e679e6621d402baf5d71ad7ce809cc">
+    <main first="rtdsrv.f947b7ebca124db5a46086c0c9fe0cad">
+      <tp>
+        <v>1</v>
+        <stp/>
+        <stp>4eee08f1-0863-4999-ac95-4130e100c587</stp>
+        <tr r="P29" s="7"/>
+      </tp>
       <tp>
         <v>2</v>
         <stp/>
-        <stp>3e631e16-a389-4c9b-8bb5-97e75952625d</stp>
-        <tr r="G50" s="4"/>
+        <stp>df23a185-e92d-4888-80ed-977e9e71fea9</stp>
+        <tr r="F5" s="3"/>
       </tp>
     </main>
-    <main first="rtdsrv.e9e679e6621d402baf5d71ad7ce809cc">
-      <tp>
-        <v>1</v>
-        <stp/>
-        <stp>de081842-4996-4452-baad-5f7f0def2e7c</stp>
-        <tr r="G35" s="7"/>
-      </tp>
+    <main first="rtdsrv.f947b7ebca124db5a46086c0c9fe0cad">
+      <tp>
+        <v>1</v>
+        <stp/>
+        <stp>5937bfa9-fd23-4765-a91c-cd06030fe238</stp>
+        <tr r="G30" s="7"/>
+      </tp>
+    </main>
+    <main first="rtdsrv.f947b7ebca124db5a46086c0c9fe0cad">
       <tp>
         <v>2</v>
         <stp/>
-        <stp>648227c9-1f26-4932-aaa3-a66268caa2e7</stp>
-        <tr r="G27" s="4"/>
+        <stp>7771dc53-eeaf-4510-91ca-e429e81117d9</stp>
+        <tr r="G55" s="4"/>
       </tp>
       <tp>
         <v>2</v>
         <stp/>
-        <stp>146f722d-1932-4321-b5be-ada5ee9a788f</stp>
-        <tr r="I42" s="4"/>
+        <stp>b4058f72-2ae7-404e-898e-e7105b51d1e9</stp>
+        <tr r="P74" s="1"/>
+      </tp>
+      <tp>
+        <v>1</v>
+        <stp/>
+        <stp>39d8741b-f8d3-4b2b-865c-5afde77ba377</stp>
+        <tr r="G37" s="7"/>
       </tp>
       <tp>
         <v>2</v>
         <stp/>
-        <stp>322d1fb3-417b-4e59-9afc-bc81c644777a</stp>
-        <tr r="F8" s="3"/>
-      </tp>
+        <stp>4ee03947-a422-45b0-bc20-303a67175bcc</stp>
+        <tr r="D25" s="5"/>
+      </tp>
+    </main>
+    <main first="rtdsrv.f947b7ebca124db5a46086c0c9fe0cad">
       <tp>
         <v>2</v>
         <stp/>
-        <stp>7ee7726f-9ca0-4f5b-8cbb-97305bc6ef7b</stp>
-        <tr r="G49" s="4"/>
+        <stp>c5914c14-4d2c-47d6-8ab9-88425cf3c79c</stp>
+        <tr r="G35" s="4"/>
       </tp>
     </main>
-    <main first="rtdsrv.e9e679e6621d402baf5d71ad7ce809cc">
+    <main first="rtdsrv.f947b7ebca124db5a46086c0c9fe0cad">
       <tp>
         <v>2</v>
         <stp/>
-        <stp>b066d117-02c7-459b-be70-cd240d329949</stp>
-        <tr r="P67" s="1"/>
+        <stp>6fb4a479-252d-4b08-8d62-c9cda81445ca</stp>
+        <tr r="G41" s="4"/>
       </tp>
     </main>
-    <main first="rtdsrv.e9e679e6621d402baf5d71ad7ce809cc">
+    <main first="rtdsrv.f947b7ebca124db5a46086c0c9fe0cad">
+      <tp>
+        <v>1</v>
+        <stp/>
+        <stp>e7c7a038-99b7-4543-b4d4-a34db0ed50cb</stp>
+        <tr r="G8" s="3"/>
+      </tp>
+    </main>
+    <main first="rtdsrv.f947b7ebca124db5a46086c0c9fe0cad">
+      <tp>
+        <v>1</v>
+        <stp/>
+        <stp>d927b72f-765d-4b19-8484-62b06e6e14e3</stp>
+        <tr r="G20" s="7"/>
+      </tp>
+    </main>
+    <main first="rtdsrv.f947b7ebca124db5a46086c0c9fe0cad">
+      <tp>
+        <v>1</v>
+        <stp/>
+        <stp>3b797f96-4510-4ac8-9b79-dd61d2d03276</stp>
+        <tr r="G41" s="7"/>
+      </tp>
+    </main>
+    <main first="rtdsrv.f947b7ebca124db5a46086c0c9fe0cad">
       <tp>
         <v>2</v>
         <stp/>
-        <stp>eb91b8ac-42ed-422a-b7cb-86a599cb21d4</stp>
-        <tr r="G24" s="1"/>
+        <stp>473456c7-8b89-40e5-a406-fcb567e313cd</stp>
+        <tr r="G23" s="4"/>
+      </tp>
+      <tp>
+        <v>2</v>
+        <stp/>
+        <stp>ab009897-04aa-4f6d-904f-722716179e95</stp>
+        <tr r="G33" s="4"/>
       </tp>
     </main>
-    <main first="rtdsrv.e9e679e6621d402baf5d71ad7ce809cc">
+    <main first="rtdsrv.f947b7ebca124db5a46086c0c9fe0cad">
       <tp>
         <v>2</v>
         <stp/>
-        <stp>3738f755-58ce-42c0-96cd-1d54dd6bb46e</stp>
-        <tr r="G32" s="4"/>
+        <stp>a78ab43c-2ac5-47e8-bce9-d798d35c5323</stp>
+        <tr r="F7" s="3"/>
+      </tp>
+    </main>
+    <main first="rtdsrv.f947b7ebca124db5a46086c0c9fe0cad">
+      <tp>
+        <v>1</v>
+        <stp/>
+        <stp>1c1641c2-5e65-4e08-8eeb-2088803fba34</stp>
+        <tr r="G26" s="7"/>
       </tp>
       <tp>
         <v>2</v>
         <stp/>
-        <stp>f5f18a63-b630-4455-9c1a-8a78d65e47a6</stp>
-        <tr r="D40" s="5"/>
-      </tp>
-    </main>
-    <main first="rtdsrv.e9e679e6621d402baf5d71ad7ce809cc">
+        <stp>0e82b2bc-6f43-42a0-b98a-6fc44f41a2d6</stp>
+        <tr r="G53" s="4"/>
+      </tp>
       <tp>
         <v>2</v>
         <stp/>
-        <stp>706d2bbd-0d20-439f-b660-44a2d15d0e75</stp>
-        <tr r="G35" s="4"/>
-      </tp>
-      <tp>
-        <v>1</v>
-        <stp/>
-        <stp>509173b7-ae7c-46fe-a7de-a76e2c07ceb0</stp>
-        <tr r="I19" s="7"/>
-      </tp>
-      <tp>
-        <v>1</v>
-        <stp/>
-        <stp>cfded6dd-4203-4c87-bef4-33366b821679</stp>
-        <tr r="G39" s="7"/>
-      </tp>
-      <tp>
-        <v>2</v>
-        <stp/>
-        <stp>75ca7530-6a25-4048-99b2-f578d26dc97d</stp>
-        <tr r="F1" s="4"/>
-      </tp>
-    </main>
-    <main first="rtdsrv.e9e679e6621d402baf5d71ad7ce809cc">
-      <tp>
-        <v>2</v>
-        <stp/>
-        <stp>3ff96d44-4451-4615-b6dc-bf2171015b0b</stp>
-        <tr r="D7" s="3"/>
-      </tp>
-      <tp>
-        <v>1</v>
-        <stp/>
-        <stp>2f542e0d-6dfd-4f94-bbdb-a5155f95bd92</stp>
-        <tr r="P19" s="7"/>
-      </tp>
-      <tp>
-        <v>2</v>
-        <stp/>
-        <stp>b82dff94-2718-494e-a028-6e973497a871</stp>
-        <tr r="G51" s="4"/>
-      </tp>
-      <tp>
-        <v>2</v>
-        <stp/>
-        <stp>9766cb65-5e60-4b71-8644-26865b27ab36</stp>
-        <tr r="G43" s="4"/>
-      </tp>
-      <tp>
-        <v>1</v>
-        <stp/>
-        <stp>1853b35b-b66b-48f2-b10c-49f8c0ab1193</stp>
-        <tr r="G29" s="7"/>
-      </tp>
-    </main>
-    <main first="rtdsrv.e9e679e6621d402baf5d71ad7ce809cc">
-      <tp>
-        <v>2</v>
-        <stp/>
-        <stp>353bbe5f-8bec-4a35-b4b6-6e7ff86f312c</stp>
-        <tr r="D4" s="3"/>
-      </tp>
-    </main>
-    <main first="rtdsrv.e9e679e6621d402baf5d71ad7ce809cc">
-      <tp>
-        <v>2</v>
-        <stp/>
-        <stp>403e9d2c-1986-40e5-97cc-9d0c6bfacf90</stp>
-        <tr r="C2" s="2"/>
-      </tp>
-      <tp>
-        <v>2</v>
-        <stp/>
-        <stp>6e380c36-3132-4c7b-bdac-4e90628542ff</stp>
-        <tr r="G45" s="1"/>
-      </tp>
-    </main>
-    <main first="rtdsrv.e9e679e6621d402baf5d71ad7ce809cc">
-      <tp>
-        <v>2</v>
-        <stp/>
-        <stp>0455aa01-e585-4bdb-9653-8033b0fa7728</stp>
-        <tr r="G50" s="1"/>
-      </tp>
-      <tp>
-        <v>1</v>
-        <stp/>
-        <stp>f87d72d6-76f5-4cb8-95a8-fc98da1b761a</stp>
-        <tr r="P67" s="7"/>
-      </tp>
-      <tp>
-        <v>1</v>
-        <stp/>
-        <stp>1c3b5a52-4e0d-405c-9dfc-c255005c3aa1</stp>
-        <tr r="G38" s="7"/>
-      </tp>
-    </main>
-    <main first="rtdsrv.e9e679e6621d402baf5d71ad7ce809cc">
-      <tp>
-        <v>1</v>
-        <stp/>
-        <stp>29c7a23c-2f95-49f1-b4f0-37a549331072</stp>
-        <tr r="G30" s="7"/>
-      </tp>
-    </main>
-    <main first="rtdsrv.e9e679e6621d402baf5d71ad7ce809cc">
-      <tp>
-        <v>2</v>
-        <stp/>
-        <stp>08e386b6-fe3e-497c-b2e1-79ce92fd65e7</stp>
-        <tr r="G51" s="1"/>
-      </tp>
-    </main>
-    <main first="rtdsrv.e9e679e6621d402baf5d71ad7ce809cc">
-      <tp>
-        <v>2</v>
-        <stp/>
-        <stp>6620f1f5-7daf-459d-92cc-273f1f533711</stp>
-        <tr r="F6" s="1"/>
-      </tp>
-    </main>
-    <main first="rtdsrv.e9e679e6621d402baf5d71ad7ce809cc">
-      <tp>
-        <v>1</v>
-        <stp/>
-        <stp>7c8591ad-6274-4b12-861e-bcc13c1996cc</stp>
-        <tr r="G23" s="7"/>
-      </tp>
-    </main>
-    <main first="rtdsrv.e9e679e6621d402baf5d71ad7ce809cc">
-      <tp>
-        <v>2</v>
-        <stp/>
-        <stp>39ae3fbe-e8ca-4341-96d1-a2b1255289e8</stp>
-        <tr r="G37" s="4"/>
-      </tp>
-      <tp>
-        <v>2</v>
-        <stp/>
-        <stp>3edb09fb-5c68-43d0-8e4f-3dbcb9076ab6</stp>
-        <tr r="D5" s="3"/>
-      </tp>
-      <tp>
-        <v>2</v>
-        <stp/>
-        <stp>51111f44-ced3-4ae2-98c1-19b7a9700452</stp>
-        <tr r="G33" s="4"/>
-      </tp>
-      <tp>
-        <v>2</v>
-        <stp/>
-        <stp>5e0ae8ac-d864-4092-ac21-e6cff80def9f</stp>
-        <tr r="G22" s="4"/>
-      </tp>
-    </main>
-    <main first="rtdsrv.e9e679e6621d402baf5d71ad7ce809cc">
-      <tp>
-        <v>2</v>
-        <stp/>
-        <stp>2a471559-6746-4ff2-bb35-a07bf60573cf</stp>
-        <tr r="I19" s="1"/>
-      </tp>
-    </main>
-    <main first="rtdsrv.e9e679e6621d402baf5d71ad7ce809cc">
-      <tp>
-        <v>1</v>
-        <stp/>
-        <stp>3c97835c-036c-4987-995e-c1d3d6f573ed</stp>
-        <tr r="G51" s="7"/>
-      </tp>
-      <tp>
-        <v>2</v>
-        <stp/>
-        <stp>e9f7e83b-e363-4fdb-8d1b-93849af023e9</stp>
-        <tr r="G32" s="1"/>
-      </tp>
-      <tp>
-        <v>2</v>
-        <stp/>
-        <stp>448d4632-211b-4f04-b0ce-ae1f46cd7b49</stp>
-        <tr r="F5" s="3"/>
-      </tp>
-    </main>
-    <main first="rtdsrv.e9e679e6621d402baf5d71ad7ce809cc">
-      <tp>
-        <v>2</v>
-        <stp/>
-        <stp>3bdfea5d-20b5-4187-8c5e-db81dc352d49</stp>
-        <tr r="G36" s="1"/>
-      </tp>
-      <tp>
-        <v>1</v>
-        <stp/>
-        <stp>ff3a81ad-4fc4-44bc-8278-57d5cc8175ce</stp>
-        <tr r="G22" s="7"/>
-      </tp>
-    </main>
-    <main first="rtdsrv.e9e679e6621d402baf5d71ad7ce809cc">
-      <tp>
-        <v>2</v>
-        <stp/>
-        <stp>118de0bb-50a9-44ac-8af8-289dddad19e4</stp>
-        <tr r="G54" s="4"/>
-      </tp>
-    </main>
-    <main first="rtdsrv.e9e679e6621d402baf5d71ad7ce809cc">
-      <tp>
-        <v>2</v>
-        <stp/>
-        <stp>bac08e65-0e7c-48d0-8010-9f1f14d0a310</stp>
-        <tr r="G43" s="1"/>
-      </tp>
-    </main>
-    <main first="rtdsrv.e9e679e6621d402baf5d71ad7ce809cc">
-      <tp>
-        <v>2</v>
-        <stp/>
-        <stp>24ef5a13-6afd-408e-a82f-b73bf2120e60</stp>
-        <tr r="G40" s="1"/>
-      </tp>
-      <tp>
-        <v>2</v>
-        <stp/>
-        <stp>074c543b-5e20-47d2-ac0b-d0f10a42e153</stp>
-        <tr r="G42" s="4"/>
-      </tp>
-      <tp>
-        <v>2</v>
-        <stp/>
-        <stp>ed80b138-a494-4a27-810d-e0299bd9c521</stp>
-        <tr r="G31" s="1"/>
-      </tp>
-    </main>
-    <main first="rtdsrv.e9e679e6621d402baf5d71ad7ce809cc">
-      <tp>
-        <v>1</v>
-        <stp/>
-        <stp>1db48b33-3357-4a98-82d0-69f8e77e636d</stp>
-        <tr r="G52" s="7"/>
-      </tp>
-      <tp>
-        <v>2</v>
-        <stp/>
-        <stp>af42a24d-5b59-4621-813a-d70aff53cf09</stp>
-        <tr r="G29" s="1"/>
-      </tp>
-    </main>
-    <main first="rtdsrv.e9e679e6621d402baf5d71ad7ce809cc">
-      <tp>
-        <v>2</v>
-        <stp/>
-        <stp>98458365-2c0e-4f98-99c1-8659f963a9bf</stp>
-        <tr r="G26" s="1"/>
-      </tp>
-    </main>
-    <main first="rtdsrv.e9e679e6621d402baf5d71ad7ce809cc">
-      <tp>
-        <v>2</v>
-        <stp/>
-        <stp>3c670a5f-f407-4de0-967b-ac39f7212b32</stp>
-        <tr r="G19" s="4"/>
-      </tp>
-    </main>
-    <main first="rtdsrv.e9e679e6621d402baf5d71ad7ce809cc">
-      <tp>
-        <v>2</v>
-        <stp/>
-        <stp>b1263af4-8565-4555-acc8-5bcd915e3822</stp>
-        <tr r="H5" s="5"/>
-      </tp>
-    </main>
-    <main first="rtdsrv.e9e679e6621d402baf5d71ad7ce809cc">
-      <tp>
-        <v>2</v>
-        <stp/>
-        <stp>65938c34-9ba1-4f89-8f8d-c9432208e004</stp>
-        <tr r="G30" s="4"/>
-      </tp>
-      <tp>
-        <v>1</v>
-        <stp/>
-        <stp>35875b55-4a77-44c6-b561-b71575b0e461</stp>
-        <tr r="H4" s="3"/>
-      </tp>
-    </main>
-    <main first="rtdsrv.e9e679e6621d402baf5d71ad7ce809cc">
-      <tp>
-        <v>1</v>
-        <stp/>
-        <stp>be8bc3dd-35bf-4372-b16e-26a6934531bf</stp>
-        <tr r="G44" s="7"/>
-      </tp>
-    </main>
-    <main first="rtdsrv.e9e679e6621d402baf5d71ad7ce809cc">
-      <tp>
-        <v>2</v>
-        <stp/>
-        <stp>5074bc93-05dd-49a4-9ba1-9ada3fc91d8f</stp>
-        <tr r="G25" s="4"/>
+        <stp>ccab1742-4781-4596-acf2-fb81a0e489f8</stp>
+        <tr r="G49" s="1"/>
       </tp>
     </main>
   </volType>
@@ -2494,7 +2494,7 @@
   <sheetFormatPr defaultRowHeight="18.75" x14ac:dyDescent="0.4"/>
   <cols>
     <col min="1" max="1" width="2.25" customWidth="1"/>
-    <col min="2" max="2" width="11" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="15.5" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="2.125" customWidth="1"/>
     <col min="5" max="5" width="38.125" bestFit="1" customWidth="1"/>
     <col min="6" max="7" width="13.25" customWidth="1"/>
@@ -2521,11 +2521,11 @@
       </c>
       <c r="F1" t="str" cm="1">
         <f t="array" ref="F1">_xll.ExLibris.Json.CreateJsonObject(E3:F6)</f>
-        <v>JsonObject:8487D676-0480-430D-9695-C9445095E295</v>
+        <v>JsonObject:653EA321-44AA-4F9A-848F-0FC246CEB0BE</v>
       </c>
       <c r="K1" t="str">
         <f>EXLIBRIS_CONFIGURATION</f>
-        <v>ExLibris.Core.ExLibrisConfiguration:309B6F05-E9D9-4A90-B78A-A8124E730131</v>
+        <v>ExLibris.Core.ExLibrisConfiguration:B757D65E-70E4-4BE1-AC2F-AD0EBE726B7C</v>
       </c>
     </row>
     <row r="2" spans="2:28" x14ac:dyDescent="0.4">
@@ -2595,7 +2595,7 @@
       </c>
       <c r="F6" t="str" cm="1">
         <f t="array" ref="F6">_xll.ExLibris.Json.CreateJsonArray(E8:J14)</f>
-        <v>JsonObject:A97E40D2-EF9D-4A05-9FA5-20553B6C306E</v>
+        <v>JsonObject:A6BB95DE-D6D4-4E3E-BD7F-83877ED0A045</v>
       </c>
       <c r="L6" t="s">
         <v>60</v>
@@ -2739,6 +2739,13 @@
       </c>
     </row>
     <row r="12" spans="2:28" x14ac:dyDescent="0.4">
+      <c r="B12" s="6" t="s">
+        <v>187</v>
+      </c>
+      <c r="C12" s="6">
+        <f>COUNTIF(AK40:AP45,FALSE)</f>
+        <v>0</v>
+      </c>
       <c r="E12" s="1">
         <f t="shared" si="0"/>
         <v>45172</v>
@@ -2763,6 +2770,13 @@
       </c>
     </row>
     <row r="13" spans="2:28" x14ac:dyDescent="0.4">
+      <c r="B13" s="6" t="s">
+        <v>188</v>
+      </c>
+      <c r="C13" s="6">
+        <f>COUNTIF(AK48:AM53,FALSE)</f>
+        <v>0</v>
+      </c>
       <c r="E13" s="1">
         <f t="shared" si="0"/>
         <v>45352</v>
@@ -2855,7 +2869,7 @@
       </c>
       <c r="I19" t="str" cm="1">
         <f t="array" ref="I19">_xll.ExLibris.Json.GetJsonValue(F1,E6)</f>
-        <v>JsonObject:2AA6FE8C-50EA-4B3A-A191-40ADDBD87401</v>
+        <v>JsonObject:DA4B7CFC-7BC8-424E-819E-6A4EA0030839</v>
       </c>
       <c r="P19" t="str" cm="1">
         <f t="array" ref="P19:Q27">_xll.ExLibris.Json.GetJsonKeyValues(F1,3)</f>
@@ -3160,7 +3174,7 @@
         <v>fixed_leg.cashflows.[0]</v>
       </c>
       <c r="Q22" t="str">
-        <v>JsonObject:88929540-3ABE-4FC8-BB47-8213930E1A1D</v>
+        <v>JsonObject:A75D6759-DC17-47A6-B967-46E32BBC25FA</v>
       </c>
       <c r="S22" t="s">
         <v>30</v>
@@ -3259,7 +3273,7 @@
         <v>fixed_leg.cashflows.[1]</v>
       </c>
       <c r="Q23" t="str">
-        <v>JsonObject:61A5A220-C39E-4D8C-BDB3-38F9E94F6039</v>
+        <v>JsonObject:F290241A-31EE-4787-9FF1-192184AFE7B5</v>
       </c>
       <c r="S23" t="s">
         <v>31</v>
@@ -3358,7 +3372,7 @@
         <v>fixed_leg.cashflows.[2]</v>
       </c>
       <c r="Q24" t="str">
-        <v>JsonObject:C0186349-E1EA-4627-A718-712F9DBC997D</v>
+        <v>JsonObject:3E22439B-A3B1-471F-B251-44792FA4D151</v>
       </c>
       <c r="S24" t="s">
         <v>32</v>
@@ -3457,7 +3471,7 @@
         <v>fixed_leg.cashflows.[3]</v>
       </c>
       <c r="Q25" t="str">
-        <v>JsonObject:F95194C4-473C-47DB-8CFD-0FA4BFBC4ACA</v>
+        <v>JsonObject:55E23224-8611-43E1-BCBC-BFE0185DD537</v>
       </c>
       <c r="S25" t="s">
         <v>33</v>
@@ -3556,7 +3570,7 @@
         <v>fixed_leg.cashflows.[4]</v>
       </c>
       <c r="Q26" t="str">
-        <v>JsonObject:2DAEA00F-9E01-43E8-B06F-4B2AA2C7E61A</v>
+        <v>JsonObject:B1A995A1-5850-42D6-BBE4-109EB818A285</v>
       </c>
       <c r="S26" t="s">
         <v>176</v>
@@ -3637,7 +3651,7 @@
         <v>fixed_leg.cashflows.[5]</v>
       </c>
       <c r="Q27" t="str">
-        <v>JsonObject:079E92FD-235C-4C34-960F-49227FDE0B77</v>
+        <v>JsonObject:F252E6F3-382B-403C-BBA8-0A81230C96D5</v>
       </c>
       <c r="S27" t="s">
         <v>34</v>
@@ -3674,7 +3688,7 @@
       </c>
       <c r="I28" t="str" cm="1">
         <f t="array" ref="I28">_xll.ExLibris.Json.GetJsonValue(I19,"[2]")</f>
-        <v>JsonObject:2CE140CF-C851-4D16-ABAC-B61A659D0BC2</v>
+        <v>JsonObject:389D722F-9AD0-4395-84B9-1B6BAD6073DC</v>
       </c>
       <c r="S28" t="s">
         <v>35</v>
@@ -3730,7 +3744,7 @@
       </c>
       <c r="P29" t="str" cm="1">
         <f t="array" ref="P29">_xll.ExLibris.Json.CreateJsonObject(P22:Q27)</f>
-        <v>JsonObject:2E8670F7-6BCC-44BD-A438-5C7B844EDD13</v>
+        <v>JsonObject:1C730280-3958-455F-8637-D1BB9C3415DB</v>
       </c>
       <c r="S29" t="s">
         <v>36</v>
@@ -4679,6 +4693,25 @@
         <f t="array" ref="G40">_xll.ExLibris.Json.GetJsonValue($F$1,E40)</f>
         <v>45172</v>
       </c>
+      <c r="I40" cm="1">
+        <f t="array" ref="I40:N45">_xll.ExLibris.Json.GetJsonTable(I19,,TRUE)</f>
+        <v>44632</v>
+      </c>
+      <c r="J40">
+        <v>44452</v>
+      </c>
+      <c r="K40">
+        <v>44632</v>
+      </c>
+      <c r="L40" t="str">
+        <v>ACT/360</v>
+      </c>
+      <c r="M40">
+        <v>10000000</v>
+      </c>
+      <c r="N40">
+        <v>1E-3</v>
+      </c>
       <c r="P40" t="str">
         <v>fixed_leg.cashflows.[1].amount</v>
       </c>
@@ -4694,6 +4727,24 @@
       <c r="U40">
         <v>45172</v>
       </c>
+      <c r="W40">
+        <v>44632</v>
+      </c>
+      <c r="X40">
+        <v>44452</v>
+      </c>
+      <c r="Y40">
+        <v>44632</v>
+      </c>
+      <c r="Z40" t="s">
+        <v>8</v>
+      </c>
+      <c r="AA40">
+        <v>10000000</v>
+      </c>
+      <c r="AB40">
+        <v>1E-3</v>
+      </c>
       <c r="AD40" t="s">
         <v>177</v>
       </c>
@@ -4710,6 +4761,30 @@
       </c>
       <c r="AI40" t="b">
         <f t="shared" si="5"/>
+        <v>1</v>
+      </c>
+      <c r="AK40" t="b">
+        <f t="shared" ref="AK40:AP45" si="14">I40=W40</f>
+        <v>1</v>
+      </c>
+      <c r="AL40" t="b">
+        <f t="shared" ref="AL40:AP45" si="15">J40=X40</f>
+        <v>1</v>
+      </c>
+      <c r="AM40" t="b">
+        <f t="shared" ref="AM40:AP45" si="16">K40=Y40</f>
+        <v>1</v>
+      </c>
+      <c r="AN40" t="b">
+        <f t="shared" ref="AN40:AP45" si="17">L40=Z40</f>
+        <v>1</v>
+      </c>
+      <c r="AO40" t="b">
+        <f t="shared" ref="AO40:AP45" si="18">M40=AA40</f>
+        <v>1</v>
+      </c>
+      <c r="AP40" t="b">
+        <f t="shared" ref="AP40:AP45" si="19">N40=AB40</f>
         <v>1</v>
       </c>
       <c r="AR40" t="b">
@@ -4732,6 +4807,24 @@
         <f t="array" ref="G41">_xll.ExLibris.Json.GetJsonValue($F$1,E41)</f>
         <v>44992</v>
       </c>
+      <c r="I41">
+        <v>44812</v>
+      </c>
+      <c r="J41">
+        <v>44632</v>
+      </c>
+      <c r="K41">
+        <v>44812</v>
+      </c>
+      <c r="L41" t="str">
+        <v>ACT/360</v>
+      </c>
+      <c r="M41">
+        <v>11000000</v>
+      </c>
+      <c r="N41">
+        <v>1E-3</v>
+      </c>
       <c r="P41" t="str">
         <v>fixed_leg.cashflows.[1].fixed_rate</v>
       </c>
@@ -4747,6 +4840,24 @@
       <c r="U41">
         <v>44992</v>
       </c>
+      <c r="W41">
+        <v>44812</v>
+      </c>
+      <c r="X41">
+        <v>44632</v>
+      </c>
+      <c r="Y41">
+        <v>44812</v>
+      </c>
+      <c r="Z41" t="s">
+        <v>8</v>
+      </c>
+      <c r="AA41">
+        <v>11000000</v>
+      </c>
+      <c r="AB41">
+        <v>1E-3</v>
+      </c>
       <c r="AD41" t="s">
         <v>39</v>
       </c>
@@ -4763,6 +4874,30 @@
       </c>
       <c r="AI41" t="b">
         <f t="shared" si="5"/>
+        <v>1</v>
+      </c>
+      <c r="AK41" t="b">
+        <f t="shared" si="14"/>
+        <v>1</v>
+      </c>
+      <c r="AL41" t="b">
+        <f t="shared" si="15"/>
+        <v>1</v>
+      </c>
+      <c r="AM41" t="b">
+        <f t="shared" si="16"/>
+        <v>1</v>
+      </c>
+      <c r="AN41" t="b">
+        <f t="shared" si="17"/>
+        <v>1</v>
+      </c>
+      <c r="AO41" t="b">
+        <f t="shared" si="18"/>
+        <v>1</v>
+      </c>
+      <c r="AP41" t="b">
+        <f t="shared" si="19"/>
         <v>1</v>
       </c>
       <c r="AR41" t="b">
@@ -4785,6 +4920,24 @@
         <f t="array" ref="G42">_xll.ExLibris.Json.GetJsonValue($F$1,E42)</f>
         <v>45172</v>
       </c>
+      <c r="I42">
+        <v>44992</v>
+      </c>
+      <c r="J42">
+        <v>44812</v>
+      </c>
+      <c r="K42">
+        <v>44992</v>
+      </c>
+      <c r="L42" t="str">
+        <v>ACT/360</v>
+      </c>
+      <c r="M42">
+        <v>12000000</v>
+      </c>
+      <c r="N42">
+        <v>1E-3</v>
+      </c>
       <c r="P42" t="str">
         <v>fixed_leg.cashflows.[2].payment _date</v>
       </c>
@@ -4800,6 +4953,24 @@
       <c r="U42">
         <v>45172</v>
       </c>
+      <c r="W42">
+        <v>44992</v>
+      </c>
+      <c r="X42">
+        <v>44812</v>
+      </c>
+      <c r="Y42">
+        <v>44992</v>
+      </c>
+      <c r="Z42" t="s">
+        <v>8</v>
+      </c>
+      <c r="AA42">
+        <v>12000000</v>
+      </c>
+      <c r="AB42">
+        <v>1E-3</v>
+      </c>
       <c r="AD42" t="s">
         <v>40</v>
       </c>
@@ -4816,6 +4987,30 @@
       </c>
       <c r="AI42" t="b">
         <f t="shared" si="5"/>
+        <v>1</v>
+      </c>
+      <c r="AK42" t="b">
+        <f t="shared" si="14"/>
+        <v>1</v>
+      </c>
+      <c r="AL42" t="b">
+        <f t="shared" si="15"/>
+        <v>1</v>
+      </c>
+      <c r="AM42" t="b">
+        <f t="shared" si="16"/>
+        <v>1</v>
+      </c>
+      <c r="AN42" t="b">
+        <f t="shared" si="17"/>
+        <v>1</v>
+      </c>
+      <c r="AO42" t="b">
+        <f t="shared" si="18"/>
+        <v>1</v>
+      </c>
+      <c r="AP42" t="b">
+        <f t="shared" si="19"/>
         <v>1</v>
       </c>
       <c r="AR42" t="b">
@@ -4838,6 +5033,24 @@
         <f t="array" ref="G43">_xll.ExLibris.Json.GetJsonValue($F$1,E43)</f>
         <v>ACT/360</v>
       </c>
+      <c r="I43">
+        <v>45172</v>
+      </c>
+      <c r="J43">
+        <v>44992</v>
+      </c>
+      <c r="K43">
+        <v>45172</v>
+      </c>
+      <c r="L43" t="str">
+        <v>ACT/360</v>
+      </c>
+      <c r="M43">
+        <v>13000000</v>
+      </c>
+      <c r="N43">
+        <v>1E-3</v>
+      </c>
       <c r="P43" t="str">
         <v>fixed_leg.cashflows.[2].start_date</v>
       </c>
@@ -4853,6 +5066,24 @@
       <c r="U43" t="s">
         <v>8</v>
       </c>
+      <c r="W43">
+        <v>45172</v>
+      </c>
+      <c r="X43">
+        <v>44992</v>
+      </c>
+      <c r="Y43">
+        <v>45172</v>
+      </c>
+      <c r="Z43" t="s">
+        <v>8</v>
+      </c>
+      <c r="AA43">
+        <v>13000000</v>
+      </c>
+      <c r="AB43">
+        <v>1E-3</v>
+      </c>
       <c r="AD43" t="s">
         <v>41</v>
       </c>
@@ -4869,6 +5100,30 @@
       </c>
       <c r="AI43" t="b">
         <f t="shared" si="5"/>
+        <v>1</v>
+      </c>
+      <c r="AK43" t="b">
+        <f t="shared" si="14"/>
+        <v>1</v>
+      </c>
+      <c r="AL43" t="b">
+        <f t="shared" si="15"/>
+        <v>1</v>
+      </c>
+      <c r="AM43" t="b">
+        <f t="shared" si="16"/>
+        <v>1</v>
+      </c>
+      <c r="AN43" t="b">
+        <f t="shared" si="17"/>
+        <v>1</v>
+      </c>
+      <c r="AO43" t="b">
+        <f t="shared" si="18"/>
+        <v>1</v>
+      </c>
+      <c r="AP43" t="b">
+        <f t="shared" si="19"/>
         <v>1</v>
       </c>
       <c r="AR43" t="b">
@@ -4891,6 +5146,24 @@
         <f t="array" ref="G44">_xll.ExLibris.Json.GetJsonValue($F$1,E44)</f>
         <v>13000000</v>
       </c>
+      <c r="I44">
+        <v>45352</v>
+      </c>
+      <c r="J44">
+        <v>45172</v>
+      </c>
+      <c r="K44">
+        <v>45352</v>
+      </c>
+      <c r="L44" t="str">
+        <v>ACT/360</v>
+      </c>
+      <c r="M44">
+        <v>14000000</v>
+      </c>
+      <c r="N44">
+        <v>1E-3</v>
+      </c>
       <c r="P44" t="str">
         <v>fixed_leg.cashflows.[2].end_date</v>
       </c>
@@ -4906,6 +5179,24 @@
       <c r="U44">
         <v>13000000</v>
       </c>
+      <c r="W44">
+        <v>45352</v>
+      </c>
+      <c r="X44">
+        <v>45172</v>
+      </c>
+      <c r="Y44">
+        <v>45352</v>
+      </c>
+      <c r="Z44" t="s">
+        <v>8</v>
+      </c>
+      <c r="AA44">
+        <v>14000000</v>
+      </c>
+      <c r="AB44">
+        <v>1E-3</v>
+      </c>
       <c r="AD44" t="s">
         <v>42</v>
       </c>
@@ -4922,6 +5213,30 @@
       </c>
       <c r="AI44" t="b">
         <f t="shared" si="5"/>
+        <v>1</v>
+      </c>
+      <c r="AK44" t="b">
+        <f t="shared" si="14"/>
+        <v>1</v>
+      </c>
+      <c r="AL44" t="b">
+        <f t="shared" si="15"/>
+        <v>1</v>
+      </c>
+      <c r="AM44" t="b">
+        <f t="shared" si="16"/>
+        <v>1</v>
+      </c>
+      <c r="AN44" t="b">
+        <f t="shared" si="17"/>
+        <v>1</v>
+      </c>
+      <c r="AO44" t="b">
+        <f t="shared" si="18"/>
+        <v>1</v>
+      </c>
+      <c r="AP44" t="b">
+        <f t="shared" si="19"/>
         <v>1</v>
       </c>
       <c r="AR44" t="b">
@@ -4944,6 +5259,24 @@
         <f t="array" ref="G45">_xll.ExLibris.Json.GetJsonValue($F$1,E45)</f>
         <v>1E-3</v>
       </c>
+      <c r="I45">
+        <v>45532</v>
+      </c>
+      <c r="J45">
+        <v>45352</v>
+      </c>
+      <c r="K45">
+        <v>45532</v>
+      </c>
+      <c r="L45" t="str">
+        <v>ACT/360</v>
+      </c>
+      <c r="M45">
+        <v>15000000</v>
+      </c>
+      <c r="N45">
+        <v>1E-3</v>
+      </c>
       <c r="P45" t="str">
         <v>fixed_leg.cashflows.[2].day_count_type</v>
       </c>
@@ -4959,6 +5292,24 @@
       <c r="U45">
         <v>1E-3</v>
       </c>
+      <c r="W45">
+        <v>45532</v>
+      </c>
+      <c r="X45">
+        <v>45352</v>
+      </c>
+      <c r="Y45">
+        <v>45532</v>
+      </c>
+      <c r="Z45" t="s">
+        <v>8</v>
+      </c>
+      <c r="AA45">
+        <v>15000000</v>
+      </c>
+      <c r="AB45">
+        <v>1E-3</v>
+      </c>
       <c r="AD45" t="s">
         <v>43</v>
       </c>
@@ -4975,6 +5326,30 @@
       </c>
       <c r="AI45" t="b">
         <f t="shared" si="5"/>
+        <v>1</v>
+      </c>
+      <c r="AK45" t="b">
+        <f t="shared" si="14"/>
+        <v>1</v>
+      </c>
+      <c r="AL45" t="b">
+        <f t="shared" si="15"/>
+        <v>1</v>
+      </c>
+      <c r="AM45" t="b">
+        <f t="shared" si="16"/>
+        <v>1</v>
+      </c>
+      <c r="AN45" t="b">
+        <f t="shared" si="17"/>
+        <v>1</v>
+      </c>
+      <c r="AO45" t="b">
+        <f t="shared" si="18"/>
+        <v>1</v>
+      </c>
+      <c r="AP45" t="b">
+        <f t="shared" si="19"/>
         <v>1</v>
       </c>
       <c r="AR45" t="b">
@@ -5050,6 +5425,18 @@
         <f t="array" ref="G47">_xll.ExLibris.Json.GetJsonValue($F$1,E47)</f>
         <v>45172</v>
       </c>
+      <c r="I47" t="str">
+        <f>E8</f>
+        <v>payment _date</v>
+      </c>
+      <c r="J47" t="str">
+        <f>H8</f>
+        <v>day_count_type</v>
+      </c>
+      <c r="K47" t="str">
+        <f>I8</f>
+        <v>amount</v>
+      </c>
       <c r="P47" t="str">
         <v>fixed_leg.cashflows.[2].fixed_rate</v>
       </c>
@@ -5064,6 +5451,15 @@
       </c>
       <c r="U47">
         <v>45172</v>
+      </c>
+      <c r="W47" t="s">
+        <v>0</v>
+      </c>
+      <c r="X47" t="s">
+        <v>6</v>
+      </c>
+      <c r="Y47" t="s">
+        <v>174</v>
       </c>
       <c r="AD47" t="s">
         <v>44</v>
@@ -5103,6 +5499,16 @@
         <f t="array" ref="G48">_xll.ExLibris.Json.GetJsonValue($F$1,E48)</f>
         <v>45352</v>
       </c>
+      <c r="I48" cm="1">
+        <f t="array" ref="I48:K53">_xll.ExLibris.Json.GetJsonTable(I19,I47:K47,TRUE)</f>
+        <v>44632</v>
+      </c>
+      <c r="J48" t="str">
+        <v>ACT/360</v>
+      </c>
+      <c r="K48">
+        <v>10000000</v>
+      </c>
       <c r="P48" t="str">
         <v>fixed_leg.cashflows.[3].payment _date</v>
       </c>
@@ -5118,6 +5524,15 @@
       <c r="U48">
         <v>45352</v>
       </c>
+      <c r="W48">
+        <v>44632</v>
+      </c>
+      <c r="X48" t="s">
+        <v>8</v>
+      </c>
+      <c r="Y48">
+        <v>10000000</v>
+      </c>
       <c r="AD48" t="s">
         <v>45</v>
       </c>
@@ -5134,6 +5549,18 @@
       </c>
       <c r="AI48" t="b">
         <f t="shared" si="5"/>
+        <v>1</v>
+      </c>
+      <c r="AK48" t="b">
+        <f t="shared" ref="AK48:AM53" si="20">I48=W48</f>
+        <v>1</v>
+      </c>
+      <c r="AL48" t="b">
+        <f t="shared" ref="AL48:AM53" si="21">J48=X48</f>
+        <v>1</v>
+      </c>
+      <c r="AM48" t="b">
+        <f t="shared" ref="AM48:AM53" si="22">K48=Y48</f>
         <v>1</v>
       </c>
       <c r="AR48" t="b">
@@ -5156,6 +5583,15 @@
         <f t="array" ref="G49">_xll.ExLibris.Json.GetJsonValue($F$1,E49)</f>
         <v>ACT/360</v>
       </c>
+      <c r="I49">
+        <v>44812</v>
+      </c>
+      <c r="J49" t="str">
+        <v>ACT/360</v>
+      </c>
+      <c r="K49">
+        <v>11000000</v>
+      </c>
       <c r="P49" t="str">
         <v>fixed_leg.cashflows.[3].start_date</v>
       </c>
@@ -5171,6 +5607,15 @@
       <c r="U49" t="s">
         <v>8</v>
       </c>
+      <c r="W49">
+        <v>44812</v>
+      </c>
+      <c r="X49" t="s">
+        <v>8</v>
+      </c>
+      <c r="Y49">
+        <v>11000000</v>
+      </c>
       <c r="AD49" t="s">
         <v>46</v>
       </c>
@@ -5187,6 +5632,18 @@
       </c>
       <c r="AI49" t="b">
         <f t="shared" si="5"/>
+        <v>1</v>
+      </c>
+      <c r="AK49" t="b">
+        <f t="shared" si="20"/>
+        <v>1</v>
+      </c>
+      <c r="AL49" t="b">
+        <f t="shared" si="21"/>
+        <v>1</v>
+      </c>
+      <c r="AM49" t="b">
+        <f t="shared" si="22"/>
         <v>1</v>
       </c>
       <c r="AR49" t="b">
@@ -5209,6 +5666,15 @@
         <f t="array" ref="G50">_xll.ExLibris.Json.GetJsonValue($F$1,E50)</f>
         <v>14000000</v>
       </c>
+      <c r="I50">
+        <v>44992</v>
+      </c>
+      <c r="J50" t="str">
+        <v>ACT/360</v>
+      </c>
+      <c r="K50">
+        <v>12000000</v>
+      </c>
       <c r="P50" t="str">
         <v>fixed_leg.cashflows.[3].end_date</v>
       </c>
@@ -5224,6 +5690,15 @@
       <c r="U50">
         <v>14000000</v>
       </c>
+      <c r="W50">
+        <v>44992</v>
+      </c>
+      <c r="X50" t="s">
+        <v>8</v>
+      </c>
+      <c r="Y50">
+        <v>12000000</v>
+      </c>
       <c r="AD50" t="s">
         <v>47</v>
       </c>
@@ -5240,6 +5715,18 @@
       </c>
       <c r="AI50" t="b">
         <f t="shared" si="5"/>
+        <v>1</v>
+      </c>
+      <c r="AK50" t="b">
+        <f t="shared" si="20"/>
+        <v>1</v>
+      </c>
+      <c r="AL50" t="b">
+        <f t="shared" si="21"/>
+        <v>1</v>
+      </c>
+      <c r="AM50" t="b">
+        <f t="shared" si="22"/>
         <v>1</v>
       </c>
       <c r="AR50" t="b">
@@ -5262,6 +5749,15 @@
         <f t="array" ref="G51">_xll.ExLibris.Json.GetJsonValue($F$1,E51)</f>
         <v>1E-3</v>
       </c>
+      <c r="I51">
+        <v>45172</v>
+      </c>
+      <c r="J51" t="str">
+        <v>ACT/360</v>
+      </c>
+      <c r="K51">
+        <v>13000000</v>
+      </c>
       <c r="P51" t="str">
         <v>fixed_leg.cashflows.[3].day_count_type</v>
       </c>
@@ -5277,6 +5773,15 @@
       <c r="U51">
         <v>1E-3</v>
       </c>
+      <c r="W51">
+        <v>45172</v>
+      </c>
+      <c r="X51" t="s">
+        <v>8</v>
+      </c>
+      <c r="Y51">
+        <v>13000000</v>
+      </c>
       <c r="AD51" t="s">
         <v>48</v>
       </c>
@@ -5293,6 +5798,18 @@
       </c>
       <c r="AI51" t="b">
         <f t="shared" si="5"/>
+        <v>1</v>
+      </c>
+      <c r="AK51" t="b">
+        <f t="shared" si="20"/>
+        <v>1</v>
+      </c>
+      <c r="AL51" t="b">
+        <f t="shared" si="21"/>
+        <v>1</v>
+      </c>
+      <c r="AM51" t="b">
+        <f t="shared" si="22"/>
         <v>1</v>
       </c>
       <c r="AR51" t="b">
@@ -5315,6 +5832,15 @@
         <f t="array" ref="G52">_xll.ExLibris.Json.GetJsonValue($F$1,E52)</f>
         <v>45532</v>
       </c>
+      <c r="I52">
+        <v>45352</v>
+      </c>
+      <c r="J52" t="str">
+        <v>ACT/360</v>
+      </c>
+      <c r="K52">
+        <v>14000000</v>
+      </c>
       <c r="P52" t="str">
         <v>fixed_leg.cashflows.[3].amount</v>
       </c>
@@ -5330,6 +5856,15 @@
       <c r="U52">
         <v>45532</v>
       </c>
+      <c r="W52">
+        <v>45352</v>
+      </c>
+      <c r="X52" t="s">
+        <v>8</v>
+      </c>
+      <c r="Y52">
+        <v>14000000</v>
+      </c>
       <c r="AD52" t="s">
         <v>179</v>
       </c>
@@ -5346,6 +5881,18 @@
       </c>
       <c r="AI52" t="b">
         <f t="shared" si="5"/>
+        <v>1</v>
+      </c>
+      <c r="AK52" t="b">
+        <f t="shared" si="20"/>
+        <v>1</v>
+      </c>
+      <c r="AL52" t="b">
+        <f t="shared" si="21"/>
+        <v>1</v>
+      </c>
+      <c r="AM52" t="b">
+        <f t="shared" si="22"/>
         <v>1</v>
       </c>
       <c r="AR52" t="b">
@@ -5368,6 +5915,15 @@
         <f t="array" ref="G53">_xll.ExLibris.Json.GetJsonValue($F$1,E53)</f>
         <v>45352</v>
       </c>
+      <c r="I53">
+        <v>45532</v>
+      </c>
+      <c r="J53" t="str">
+        <v>ACT/360</v>
+      </c>
+      <c r="K53">
+        <v>15000000</v>
+      </c>
       <c r="P53" t="str">
         <v>fixed_leg.cashflows.[3].fixed_rate</v>
       </c>
@@ -5383,6 +5939,15 @@
       <c r="U53">
         <v>45352</v>
       </c>
+      <c r="W53">
+        <v>45532</v>
+      </c>
+      <c r="X53" t="s">
+        <v>8</v>
+      </c>
+      <c r="Y53">
+        <v>15000000</v>
+      </c>
       <c r="AD53" t="s">
         <v>49</v>
       </c>
@@ -5399,6 +5964,18 @@
       </c>
       <c r="AI53" t="b">
         <f t="shared" si="5"/>
+        <v>1</v>
+      </c>
+      <c r="AK53" t="b">
+        <f t="shared" si="20"/>
+        <v>1</v>
+      </c>
+      <c r="AL53" t="b">
+        <f t="shared" si="21"/>
+        <v>1</v>
+      </c>
+      <c r="AM53" t="b">
+        <f t="shared" si="22"/>
         <v>1</v>
       </c>
       <c r="AR53" t="b">
@@ -5813,11 +6390,11 @@
         <v>44632</v>
       </c>
       <c r="AR67" t="b">
-        <f t="shared" ref="AR67:AR79" si="14">P67=AD67</f>
+        <f t="shared" ref="AR67:AR79" si="23">P67=AD67</f>
         <v>1</v>
       </c>
       <c r="AS67" t="b">
-        <f t="shared" ref="AS67:AS79" si="15">Q67=AE67</f>
+        <f t="shared" ref="AS67:AS79" si="24">Q67=AE67</f>
         <v>1</v>
       </c>
     </row>
@@ -5835,11 +6412,11 @@
         <v>44812</v>
       </c>
       <c r="AR68" t="b">
-        <f t="shared" si="14"/>
+        <f t="shared" si="23"/>
         <v>1</v>
       </c>
       <c r="AS68" t="b">
-        <f t="shared" si="15"/>
+        <f t="shared" si="24"/>
         <v>1</v>
       </c>
     </row>
@@ -5857,11 +6434,11 @@
         <v>44992</v>
       </c>
       <c r="AR69" t="b">
-        <f t="shared" si="14"/>
+        <f t="shared" si="23"/>
         <v>1</v>
       </c>
       <c r="AS69" t="b">
-        <f t="shared" si="15"/>
+        <f t="shared" si="24"/>
         <v>1</v>
       </c>
     </row>
@@ -5879,11 +6456,11 @@
         <v>45172</v>
       </c>
       <c r="AR70" t="b">
-        <f t="shared" si="14"/>
+        <f t="shared" si="23"/>
         <v>1</v>
       </c>
       <c r="AS70" t="b">
-        <f t="shared" si="15"/>
+        <f t="shared" si="24"/>
         <v>1</v>
       </c>
     </row>
@@ -5901,11 +6478,11 @@
         <v>45352</v>
       </c>
       <c r="AR71" t="b">
-        <f t="shared" si="14"/>
+        <f t="shared" si="23"/>
         <v>1</v>
       </c>
       <c r="AS71" t="b">
-        <f t="shared" si="15"/>
+        <f t="shared" si="24"/>
         <v>1</v>
       </c>
     </row>
@@ -5923,11 +6500,11 @@
         <v>45532</v>
       </c>
       <c r="AR72" t="b">
-        <f t="shared" si="14"/>
+        <f t="shared" si="23"/>
         <v>1</v>
       </c>
       <c r="AS72" t="b">
-        <f t="shared" si="15"/>
+        <f t="shared" si="24"/>
         <v>1</v>
       </c>
     </row>
@@ -5946,11 +6523,11 @@
         <v>45172</v>
       </c>
       <c r="AR74" t="b">
-        <f t="shared" si="14"/>
+        <f t="shared" si="23"/>
         <v>1</v>
       </c>
       <c r="AS74" t="b">
-        <f t="shared" si="15"/>
+        <f t="shared" si="24"/>
         <v>1</v>
       </c>
     </row>
@@ -5968,11 +6545,11 @@
         <v>44992</v>
       </c>
       <c r="AR75" t="b">
-        <f t="shared" si="14"/>
+        <f t="shared" si="23"/>
         <v>1</v>
       </c>
       <c r="AS75" t="b">
-        <f t="shared" si="15"/>
+        <f t="shared" si="24"/>
         <v>1</v>
       </c>
     </row>
@@ -5990,11 +6567,11 @@
         <v>45172</v>
       </c>
       <c r="AR76" t="b">
-        <f t="shared" si="14"/>
+        <f t="shared" si="23"/>
         <v>1</v>
       </c>
       <c r="AS76" t="b">
-        <f t="shared" si="15"/>
+        <f t="shared" si="24"/>
         <v>1</v>
       </c>
     </row>
@@ -6012,11 +6589,11 @@
         <v>8</v>
       </c>
       <c r="AR77" t="b">
-        <f t="shared" si="14"/>
+        <f t="shared" si="23"/>
         <v>1</v>
       </c>
       <c r="AS77" t="b">
-        <f t="shared" si="15"/>
+        <f t="shared" si="24"/>
         <v>1</v>
       </c>
     </row>
@@ -6034,11 +6611,11 @@
         <v>13000000</v>
       </c>
       <c r="AR78" t="b">
-        <f t="shared" si="14"/>
+        <f t="shared" si="23"/>
         <v>1</v>
       </c>
       <c r="AS78" t="b">
-        <f t="shared" si="15"/>
+        <f t="shared" si="24"/>
         <v>1</v>
       </c>
     </row>
@@ -6056,11 +6633,11 @@
         <v>1E-3</v>
       </c>
       <c r="AR79" t="b">
-        <f t="shared" si="14"/>
+        <f t="shared" si="23"/>
         <v>1</v>
       </c>
       <c r="AS79" t="b">
-        <f t="shared" si="15"/>
+        <f t="shared" si="24"/>
         <v>1</v>
       </c>
     </row>
@@ -6077,7 +6654,7 @@
   <sheetFormatPr defaultRowHeight="18.75" x14ac:dyDescent="0.4"/>
   <cols>
     <col min="1" max="1" width="2.25" customWidth="1"/>
-    <col min="2" max="2" width="11" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="15.5" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="2.125" customWidth="1"/>
     <col min="5" max="5" width="38.125" bestFit="1" customWidth="1"/>
     <col min="6" max="7" width="13.25" customWidth="1"/>
@@ -6104,11 +6681,11 @@
       </c>
       <c r="F1" t="str" cm="1">
         <f t="array" ref="F1">_xll.ExLibris.Json.CreateJsonObjectAsync(E3:F6)</f>
-        <v>JsonObject:9779E518-6FDE-4D6F-A363-4EEC79F7EC4C</v>
+        <v>JsonObject:83F8ED29-929D-492C-9032-4856AD088F8E</v>
       </c>
       <c r="K1" t="str">
         <f>EXLIBRIS_CONFIGURATION</f>
-        <v>ExLibris.Core.ExLibrisConfiguration:309B6F05-E9D9-4A90-B78A-A8124E730131</v>
+        <v>ExLibris.Core.ExLibrisConfiguration:B757D65E-70E4-4BE1-AC2F-AD0EBE726B7C</v>
       </c>
     </row>
     <row r="2" spans="2:28" x14ac:dyDescent="0.4">
@@ -6178,7 +6755,7 @@
       </c>
       <c r="F6" t="str" cm="1">
         <f t="array" ref="F6">_xll.ExLibris.Json.CreateJsonArrayAsync(E8:J14)</f>
-        <v>JsonObject:F530457B-7B3E-434F-BFAE-12901E9A2482</v>
+        <v>JsonObject:C19874F4-0741-4571-BB67-8F0380608706</v>
       </c>
       <c r="L6" t="s">
         <v>60</v>
@@ -6322,6 +6899,13 @@
       </c>
     </row>
     <row r="12" spans="2:28" x14ac:dyDescent="0.4">
+      <c r="B12" s="6" t="s">
+        <v>187</v>
+      </c>
+      <c r="C12" s="6">
+        <f>COUNTIF(AK40:AP45,FALSE)</f>
+        <v>0</v>
+      </c>
       <c r="E12" s="1">
         <f t="shared" si="0"/>
         <v>45172</v>
@@ -6346,6 +6930,13 @@
       </c>
     </row>
     <row r="13" spans="2:28" x14ac:dyDescent="0.4">
+      <c r="B13" s="6" t="s">
+        <v>188</v>
+      </c>
+      <c r="C13" s="6">
+        <f>COUNTIF(AK48:AM53,FALSE)</f>
+        <v>0</v>
+      </c>
       <c r="E13" s="1">
         <f t="shared" si="0"/>
         <v>45352</v>
@@ -6438,7 +7029,7 @@
       </c>
       <c r="I19" t="str" cm="1">
         <f t="array" ref="I19">_xll.ExLibris.Json.GetJsonValueAsync(F1,E6)</f>
-        <v>JsonObject:B6E4D12F-506F-4634-B9AB-00B8642409D6</v>
+        <v>JsonObject:78074F34-2A76-4FDD-A7A5-EA6B18BC28AF</v>
       </c>
       <c r="P19" t="str" cm="1">
         <f t="array" ref="P19:Q27">_xll.ExLibris.Json.GetJsonKeyValuesAsync(F1,3)</f>
@@ -6743,7 +7334,7 @@
         <v>fixed_leg.cashflows.[0]</v>
       </c>
       <c r="Q22" t="str">
-        <v>JsonObject:D52D8C09-F125-4B92-AFAB-36F9EC2599D0</v>
+        <v>JsonObject:3CE6B1E8-E3FA-40CD-914D-9C73489F4264</v>
       </c>
       <c r="S22" t="s">
         <v>30</v>
@@ -6842,7 +7433,7 @@
         <v>fixed_leg.cashflows.[1]</v>
       </c>
       <c r="Q23" t="str">
-        <v>JsonObject:7BEAF70D-F303-40C7-8930-C853BDAABC8E</v>
+        <v>JsonObject:24736553-4D11-4D30-9D47-3B3133D0B066</v>
       </c>
       <c r="S23" t="s">
         <v>31</v>
@@ -6941,7 +7532,7 @@
         <v>fixed_leg.cashflows.[2]</v>
       </c>
       <c r="Q24" t="str">
-        <v>JsonObject:E82F81DC-37FE-4A3E-B1E4-C11122917FD8</v>
+        <v>JsonObject:6E0B9315-7F04-4297-B548-1934524F4D0E</v>
       </c>
       <c r="S24" t="s">
         <v>32</v>
@@ -7040,7 +7631,7 @@
         <v>fixed_leg.cashflows.[3]</v>
       </c>
       <c r="Q25" t="str">
-        <v>JsonObject:12D8F8B5-0484-4360-B2AC-EC5EA8687234</v>
+        <v>JsonObject:665EF199-7C22-4BAE-9D3B-0D878C2E7653</v>
       </c>
       <c r="S25" t="s">
         <v>33</v>
@@ -7139,7 +7730,7 @@
         <v>fixed_leg.cashflows.[4]</v>
       </c>
       <c r="Q26" t="str">
-        <v>JsonObject:2BB2D9AF-6CEC-43B4-BE5B-AA91ADA0E770</v>
+        <v>JsonObject:822D5D09-9B4B-4110-841D-05BA22805051</v>
       </c>
       <c r="S26" t="s">
         <v>176</v>
@@ -7220,7 +7811,7 @@
         <v>fixed_leg.cashflows.[5]</v>
       </c>
       <c r="Q27" t="str">
-        <v>JsonObject:BFE5ECDA-617F-47FF-881E-39A63CD349D8</v>
+        <v>JsonObject:EB6EC5A4-BFDC-4B67-8B3B-E1C512D2C1B8</v>
       </c>
       <c r="S27" t="s">
         <v>34</v>
@@ -7257,7 +7848,7 @@
       </c>
       <c r="I28" t="str" cm="1">
         <f t="array" ref="I28">_xll.ExLibris.Json.GetJsonValueAsync(I19,"[2]")</f>
-        <v>JsonObject:F189FE5C-8C89-42C9-A297-98386BDB0FD5</v>
+        <v>JsonObject:2E1DD465-3B8C-4FC8-94F6-743A57E20F4F</v>
       </c>
       <c r="S28" t="s">
         <v>35</v>
@@ -7313,7 +7904,7 @@
       </c>
       <c r="P29" t="str" cm="1">
         <f t="array" ref="P29">_xll.ExLibris.Json.CreateJsonObjectAsync(P22:Q27)</f>
-        <v>JsonObject:9E1A475A-6C9E-434B-8488-82965B75B08C</v>
+        <v>JsonObject:6B012B77-5FB8-473C-8B42-FBAF8B9B9B3E</v>
       </c>
       <c r="S29" t="s">
         <v>36</v>
@@ -8262,6 +8853,25 @@
         <f t="array" ref="G40">_xll.ExLibris.Json.GetJsonValueAsync($F$1,E40)</f>
         <v>45172</v>
       </c>
+      <c r="I40" cm="1">
+        <f t="array" ref="I40:N45">_xll.ExLibris.Json.GetJsonTableAsync(I19,,TRUE)</f>
+        <v>44632</v>
+      </c>
+      <c r="J40">
+        <v>44452</v>
+      </c>
+      <c r="K40">
+        <v>44632</v>
+      </c>
+      <c r="L40" t="str">
+        <v>ACT/360</v>
+      </c>
+      <c r="M40">
+        <v>10000000</v>
+      </c>
+      <c r="N40">
+        <v>1E-3</v>
+      </c>
       <c r="P40" t="str">
         <v>fixed_leg.cashflows.[1].amount</v>
       </c>
@@ -8277,6 +8887,24 @@
       <c r="U40">
         <v>45172</v>
       </c>
+      <c r="W40">
+        <v>44632</v>
+      </c>
+      <c r="X40">
+        <v>44452</v>
+      </c>
+      <c r="Y40">
+        <v>44632</v>
+      </c>
+      <c r="Z40" t="s">
+        <v>8</v>
+      </c>
+      <c r="AA40">
+        <v>10000000</v>
+      </c>
+      <c r="AB40">
+        <v>1E-3</v>
+      </c>
       <c r="AD40" t="s">
         <v>177</v>
       </c>
@@ -8293,6 +8921,30 @@
       </c>
       <c r="AI40" t="b">
         <f t="shared" si="6"/>
+        <v>1</v>
+      </c>
+      <c r="AK40" t="b">
+        <f t="shared" ref="AK40:AP45" si="13">I40=W40</f>
+        <v>1</v>
+      </c>
+      <c r="AL40" t="b">
+        <f t="shared" ref="AL40:AP45" si="14">J40=X40</f>
+        <v>1</v>
+      </c>
+      <c r="AM40" t="b">
+        <f t="shared" ref="AM40:AP45" si="15">K40=Y40</f>
+        <v>1</v>
+      </c>
+      <c r="AN40" t="b">
+        <f t="shared" ref="AN40:AP45" si="16">L40=Z40</f>
+        <v>1</v>
+      </c>
+      <c r="AO40" t="b">
+        <f t="shared" ref="AO40:AP45" si="17">M40=AA40</f>
+        <v>1</v>
+      </c>
+      <c r="AP40" t="b">
+        <f t="shared" ref="AP40:AP45" si="18">N40=AB40</f>
         <v>1</v>
       </c>
       <c r="AR40" t="b">
@@ -8315,6 +8967,24 @@
         <f t="array" ref="G41">_xll.ExLibris.Json.GetJsonValueAsync($F$1,E41)</f>
         <v>44992</v>
       </c>
+      <c r="I41">
+        <v>44812</v>
+      </c>
+      <c r="J41">
+        <v>44632</v>
+      </c>
+      <c r="K41">
+        <v>44812</v>
+      </c>
+      <c r="L41" t="str">
+        <v>ACT/360</v>
+      </c>
+      <c r="M41">
+        <v>11000000</v>
+      </c>
+      <c r="N41">
+        <v>1E-3</v>
+      </c>
       <c r="P41" t="str">
         <v>fixed_leg.cashflows.[1].fixed_rate</v>
       </c>
@@ -8330,6 +9000,24 @@
       <c r="U41">
         <v>44992</v>
       </c>
+      <c r="W41">
+        <v>44812</v>
+      </c>
+      <c r="X41">
+        <v>44632</v>
+      </c>
+      <c r="Y41">
+        <v>44812</v>
+      </c>
+      <c r="Z41" t="s">
+        <v>8</v>
+      </c>
+      <c r="AA41">
+        <v>11000000</v>
+      </c>
+      <c r="AB41">
+        <v>1E-3</v>
+      </c>
       <c r="AD41" t="s">
         <v>39</v>
       </c>
@@ -8346,6 +9034,30 @@
       </c>
       <c r="AI41" t="b">
         <f t="shared" si="6"/>
+        <v>1</v>
+      </c>
+      <c r="AK41" t="b">
+        <f t="shared" si="13"/>
+        <v>1</v>
+      </c>
+      <c r="AL41" t="b">
+        <f t="shared" si="14"/>
+        <v>1</v>
+      </c>
+      <c r="AM41" t="b">
+        <f t="shared" si="15"/>
+        <v>1</v>
+      </c>
+      <c r="AN41" t="b">
+        <f t="shared" si="16"/>
+        <v>1</v>
+      </c>
+      <c r="AO41" t="b">
+        <f t="shared" si="17"/>
+        <v>1</v>
+      </c>
+      <c r="AP41" t="b">
+        <f t="shared" si="18"/>
         <v>1</v>
       </c>
       <c r="AR41" t="b">
@@ -8368,6 +9080,24 @@
         <f t="array" ref="G42">_xll.ExLibris.Json.GetJsonValueAsync($F$1,E42)</f>
         <v>45172</v>
       </c>
+      <c r="I42">
+        <v>44992</v>
+      </c>
+      <c r="J42">
+        <v>44812</v>
+      </c>
+      <c r="K42">
+        <v>44992</v>
+      </c>
+      <c r="L42" t="str">
+        <v>ACT/360</v>
+      </c>
+      <c r="M42">
+        <v>12000000</v>
+      </c>
+      <c r="N42">
+        <v>1E-3</v>
+      </c>
       <c r="P42" t="str">
         <v>fixed_leg.cashflows.[2].payment _date</v>
       </c>
@@ -8383,6 +9113,24 @@
       <c r="U42">
         <v>45172</v>
       </c>
+      <c r="W42">
+        <v>44992</v>
+      </c>
+      <c r="X42">
+        <v>44812</v>
+      </c>
+      <c r="Y42">
+        <v>44992</v>
+      </c>
+      <c r="Z42" t="s">
+        <v>8</v>
+      </c>
+      <c r="AA42">
+        <v>12000000</v>
+      </c>
+      <c r="AB42">
+        <v>1E-3</v>
+      </c>
       <c r="AD42" t="s">
         <v>40</v>
       </c>
@@ -8399,6 +9147,30 @@
       </c>
       <c r="AI42" t="b">
         <f t="shared" si="6"/>
+        <v>1</v>
+      </c>
+      <c r="AK42" t="b">
+        <f t="shared" si="13"/>
+        <v>1</v>
+      </c>
+      <c r="AL42" t="b">
+        <f t="shared" si="14"/>
+        <v>1</v>
+      </c>
+      <c r="AM42" t="b">
+        <f t="shared" si="15"/>
+        <v>1</v>
+      </c>
+      <c r="AN42" t="b">
+        <f t="shared" si="16"/>
+        <v>1</v>
+      </c>
+      <c r="AO42" t="b">
+        <f t="shared" si="17"/>
+        <v>1</v>
+      </c>
+      <c r="AP42" t="b">
+        <f t="shared" si="18"/>
         <v>1</v>
       </c>
       <c r="AR42" t="b">
@@ -8421,6 +9193,24 @@
         <f t="array" ref="G43">_xll.ExLibris.Json.GetJsonValueAsync($F$1,E43)</f>
         <v>ACT/360</v>
       </c>
+      <c r="I43">
+        <v>45172</v>
+      </c>
+      <c r="J43">
+        <v>44992</v>
+      </c>
+      <c r="K43">
+        <v>45172</v>
+      </c>
+      <c r="L43" t="str">
+        <v>ACT/360</v>
+      </c>
+      <c r="M43">
+        <v>13000000</v>
+      </c>
+      <c r="N43">
+        <v>1E-3</v>
+      </c>
       <c r="P43" t="str">
         <v>fixed_leg.cashflows.[2].start_date</v>
       </c>
@@ -8436,6 +9226,24 @@
       <c r="U43" t="s">
         <v>8</v>
       </c>
+      <c r="W43">
+        <v>45172</v>
+      </c>
+      <c r="X43">
+        <v>44992</v>
+      </c>
+      <c r="Y43">
+        <v>45172</v>
+      </c>
+      <c r="Z43" t="s">
+        <v>8</v>
+      </c>
+      <c r="AA43">
+        <v>13000000</v>
+      </c>
+      <c r="AB43">
+        <v>1E-3</v>
+      </c>
       <c r="AD43" t="s">
         <v>41</v>
       </c>
@@ -8452,6 +9260,30 @@
       </c>
       <c r="AI43" t="b">
         <f t="shared" si="6"/>
+        <v>1</v>
+      </c>
+      <c r="AK43" t="b">
+        <f t="shared" si="13"/>
+        <v>1</v>
+      </c>
+      <c r="AL43" t="b">
+        <f t="shared" si="14"/>
+        <v>1</v>
+      </c>
+      <c r="AM43" t="b">
+        <f t="shared" si="15"/>
+        <v>1</v>
+      </c>
+      <c r="AN43" t="b">
+        <f t="shared" si="16"/>
+        <v>1</v>
+      </c>
+      <c r="AO43" t="b">
+        <f t="shared" si="17"/>
+        <v>1</v>
+      </c>
+      <c r="AP43" t="b">
+        <f t="shared" si="18"/>
         <v>1</v>
       </c>
       <c r="AR43" t="b">
@@ -8474,6 +9306,24 @@
         <f t="array" ref="G44">_xll.ExLibris.Json.GetJsonValueAsync($F$1,E44)</f>
         <v>13000000</v>
       </c>
+      <c r="I44">
+        <v>45352</v>
+      </c>
+      <c r="J44">
+        <v>45172</v>
+      </c>
+      <c r="K44">
+        <v>45352</v>
+      </c>
+      <c r="L44" t="str">
+        <v>ACT/360</v>
+      </c>
+      <c r="M44">
+        <v>14000000</v>
+      </c>
+      <c r="N44">
+        <v>1E-3</v>
+      </c>
       <c r="P44" t="str">
         <v>fixed_leg.cashflows.[2].end_date</v>
       </c>
@@ -8489,6 +9339,24 @@
       <c r="U44">
         <v>13000000</v>
       </c>
+      <c r="W44">
+        <v>45352</v>
+      </c>
+      <c r="X44">
+        <v>45172</v>
+      </c>
+      <c r="Y44">
+        <v>45352</v>
+      </c>
+      <c r="Z44" t="s">
+        <v>8</v>
+      </c>
+      <c r="AA44">
+        <v>14000000</v>
+      </c>
+      <c r="AB44">
+        <v>1E-3</v>
+      </c>
       <c r="AD44" t="s">
         <v>42</v>
       </c>
@@ -8505,6 +9373,30 @@
       </c>
       <c r="AI44" t="b">
         <f t="shared" si="6"/>
+        <v>1</v>
+      </c>
+      <c r="AK44" t="b">
+        <f t="shared" si="13"/>
+        <v>1</v>
+      </c>
+      <c r="AL44" t="b">
+        <f t="shared" si="14"/>
+        <v>1</v>
+      </c>
+      <c r="AM44" t="b">
+        <f t="shared" si="15"/>
+        <v>1</v>
+      </c>
+      <c r="AN44" t="b">
+        <f t="shared" si="16"/>
+        <v>1</v>
+      </c>
+      <c r="AO44" t="b">
+        <f t="shared" si="17"/>
+        <v>1</v>
+      </c>
+      <c r="AP44" t="b">
+        <f t="shared" si="18"/>
         <v>1</v>
       </c>
       <c r="AR44" t="b">
@@ -8527,6 +9419,24 @@
         <f t="array" ref="G45">_xll.ExLibris.Json.GetJsonValueAsync($F$1,E45)</f>
         <v>1E-3</v>
       </c>
+      <c r="I45">
+        <v>45532</v>
+      </c>
+      <c r="J45">
+        <v>45352</v>
+      </c>
+      <c r="K45">
+        <v>45532</v>
+      </c>
+      <c r="L45" t="str">
+        <v>ACT/360</v>
+      </c>
+      <c r="M45">
+        <v>15000000</v>
+      </c>
+      <c r="N45">
+        <v>1E-3</v>
+      </c>
       <c r="P45" t="str">
         <v>fixed_leg.cashflows.[2].day_count_type</v>
       </c>
@@ -8542,6 +9452,24 @@
       <c r="U45">
         <v>1E-3</v>
       </c>
+      <c r="W45">
+        <v>45532</v>
+      </c>
+      <c r="X45">
+        <v>45352</v>
+      </c>
+      <c r="Y45">
+        <v>45532</v>
+      </c>
+      <c r="Z45" t="s">
+        <v>8</v>
+      </c>
+      <c r="AA45">
+        <v>15000000</v>
+      </c>
+      <c r="AB45">
+        <v>1E-3</v>
+      </c>
       <c r="AD45" t="s">
         <v>43</v>
       </c>
@@ -8558,6 +9486,30 @@
       </c>
       <c r="AI45" t="b">
         <f t="shared" si="6"/>
+        <v>1</v>
+      </c>
+      <c r="AK45" t="b">
+        <f t="shared" si="13"/>
+        <v>1</v>
+      </c>
+      <c r="AL45" t="b">
+        <f t="shared" si="14"/>
+        <v>1</v>
+      </c>
+      <c r="AM45" t="b">
+        <f t="shared" si="15"/>
+        <v>1</v>
+      </c>
+      <c r="AN45" t="b">
+        <f t="shared" si="16"/>
+        <v>1</v>
+      </c>
+      <c r="AO45" t="b">
+        <f t="shared" si="17"/>
+        <v>1</v>
+      </c>
+      <c r="AP45" t="b">
+        <f t="shared" si="18"/>
         <v>1</v>
       </c>
       <c r="AR45" t="b">
@@ -8633,6 +9585,18 @@
         <f t="array" ref="G47">_xll.ExLibris.Json.GetJsonValueAsync($F$1,E47)</f>
         <v>45172</v>
       </c>
+      <c r="I47" t="str">
+        <f>E8</f>
+        <v>payment _date</v>
+      </c>
+      <c r="J47" t="str">
+        <f>H8</f>
+        <v>day_count_type</v>
+      </c>
+      <c r="K47" t="str">
+        <f>I8</f>
+        <v>amount</v>
+      </c>
       <c r="P47" t="str">
         <v>fixed_leg.cashflows.[2].fixed_rate</v>
       </c>
@@ -8686,6 +9650,16 @@
         <f t="array" ref="G48">_xll.ExLibris.Json.GetJsonValueAsync($F$1,E48)</f>
         <v>45352</v>
       </c>
+      <c r="I48" cm="1">
+        <f t="array" ref="I48:K53">_xll.ExLibris.Json.GetJsonTableAsync(I19,I47:K47,TRUE)</f>
+        <v>44632</v>
+      </c>
+      <c r="J48" t="str">
+        <v>ACT/360</v>
+      </c>
+      <c r="K48">
+        <v>10000000</v>
+      </c>
       <c r="P48" t="str">
         <v>fixed_leg.cashflows.[3].payment _date</v>
       </c>
@@ -8701,6 +9675,15 @@
       <c r="U48">
         <v>45352</v>
       </c>
+      <c r="W48">
+        <v>44632</v>
+      </c>
+      <c r="X48" t="s">
+        <v>8</v>
+      </c>
+      <c r="Y48">
+        <v>10000000</v>
+      </c>
       <c r="AD48" t="s">
         <v>45</v>
       </c>
@@ -8717,6 +9700,18 @@
       </c>
       <c r="AI48" t="b">
         <f t="shared" si="6"/>
+        <v>1</v>
+      </c>
+      <c r="AK48" t="b">
+        <f t="shared" ref="AK48:AM53" si="19">I48=W48</f>
+        <v>1</v>
+      </c>
+      <c r="AL48" t="b">
+        <f t="shared" ref="AL48:AM53" si="20">J48=X48</f>
+        <v>1</v>
+      </c>
+      <c r="AM48" t="b">
+        <f t="shared" ref="AM48:AM53" si="21">K48=Y48</f>
         <v>1</v>
       </c>
       <c r="AR48" t="b">
@@ -8739,6 +9734,15 @@
         <f t="array" ref="G49">_xll.ExLibris.Json.GetJsonValueAsync($F$1,E49)</f>
         <v>ACT/360</v>
       </c>
+      <c r="I49">
+        <v>44812</v>
+      </c>
+      <c r="J49" t="str">
+        <v>ACT/360</v>
+      </c>
+      <c r="K49">
+        <v>11000000</v>
+      </c>
       <c r="P49" t="str">
         <v>fixed_leg.cashflows.[3].start_date</v>
       </c>
@@ -8754,6 +9758,15 @@
       <c r="U49" t="s">
         <v>8</v>
       </c>
+      <c r="W49">
+        <v>44812</v>
+      </c>
+      <c r="X49" t="s">
+        <v>8</v>
+      </c>
+      <c r="Y49">
+        <v>11000000</v>
+      </c>
       <c r="AD49" t="s">
         <v>46</v>
       </c>
@@ -8770,6 +9783,18 @@
       </c>
       <c r="AI49" t="b">
         <f t="shared" si="6"/>
+        <v>1</v>
+      </c>
+      <c r="AK49" t="b">
+        <f t="shared" si="19"/>
+        <v>1</v>
+      </c>
+      <c r="AL49" t="b">
+        <f t="shared" si="20"/>
+        <v>1</v>
+      </c>
+      <c r="AM49" t="b">
+        <f t="shared" si="21"/>
         <v>1</v>
       </c>
       <c r="AR49" t="b">
@@ -8792,6 +9817,15 @@
         <f t="array" ref="G50">_xll.ExLibris.Json.GetJsonValueAsync($F$1,E50)</f>
         <v>14000000</v>
       </c>
+      <c r="I50">
+        <v>44992</v>
+      </c>
+      <c r="J50" t="str">
+        <v>ACT/360</v>
+      </c>
+      <c r="K50">
+        <v>12000000</v>
+      </c>
       <c r="P50" t="str">
         <v>fixed_leg.cashflows.[3].end_date</v>
       </c>
@@ -8807,6 +9841,15 @@
       <c r="U50">
         <v>14000000</v>
       </c>
+      <c r="W50">
+        <v>44992</v>
+      </c>
+      <c r="X50" t="s">
+        <v>8</v>
+      </c>
+      <c r="Y50">
+        <v>12000000</v>
+      </c>
       <c r="AD50" t="s">
         <v>47</v>
       </c>
@@ -8823,6 +9866,18 @@
       </c>
       <c r="AI50" t="b">
         <f t="shared" si="6"/>
+        <v>1</v>
+      </c>
+      <c r="AK50" t="b">
+        <f t="shared" si="19"/>
+        <v>1</v>
+      </c>
+      <c r="AL50" t="b">
+        <f t="shared" si="20"/>
+        <v>1</v>
+      </c>
+      <c r="AM50" t="b">
+        <f t="shared" si="21"/>
         <v>1</v>
       </c>
       <c r="AR50" t="b">
@@ -8845,6 +9900,15 @@
         <f t="array" ref="G51">_xll.ExLibris.Json.GetJsonValueAsync($F$1,E51)</f>
         <v>1E-3</v>
       </c>
+      <c r="I51">
+        <v>45172</v>
+      </c>
+      <c r="J51" t="str">
+        <v>ACT/360</v>
+      </c>
+      <c r="K51">
+        <v>13000000</v>
+      </c>
       <c r="P51" t="str">
         <v>fixed_leg.cashflows.[3].day_count_type</v>
       </c>
@@ -8860,6 +9924,15 @@
       <c r="U51">
         <v>1E-3</v>
       </c>
+      <c r="W51">
+        <v>45172</v>
+      </c>
+      <c r="X51" t="s">
+        <v>8</v>
+      </c>
+      <c r="Y51">
+        <v>13000000</v>
+      </c>
       <c r="AD51" t="s">
         <v>48</v>
       </c>
@@ -8876,6 +9949,18 @@
       </c>
       <c r="AI51" t="b">
         <f t="shared" si="6"/>
+        <v>1</v>
+      </c>
+      <c r="AK51" t="b">
+        <f t="shared" si="19"/>
+        <v>1</v>
+      </c>
+      <c r="AL51" t="b">
+        <f t="shared" si="20"/>
+        <v>1</v>
+      </c>
+      <c r="AM51" t="b">
+        <f t="shared" si="21"/>
         <v>1</v>
       </c>
       <c r="AR51" t="b">
@@ -8898,6 +9983,15 @@
         <f t="array" ref="G52">_xll.ExLibris.Json.GetJsonValueAsync($F$1,E52)</f>
         <v>45532</v>
       </c>
+      <c r="I52">
+        <v>45352</v>
+      </c>
+      <c r="J52" t="str">
+        <v>ACT/360</v>
+      </c>
+      <c r="K52">
+        <v>14000000</v>
+      </c>
       <c r="P52" t="str">
         <v>fixed_leg.cashflows.[3].amount</v>
       </c>
@@ -8913,6 +10007,15 @@
       <c r="U52">
         <v>45532</v>
       </c>
+      <c r="W52">
+        <v>45352</v>
+      </c>
+      <c r="X52" t="s">
+        <v>8</v>
+      </c>
+      <c r="Y52">
+        <v>14000000</v>
+      </c>
       <c r="AD52" t="s">
         <v>179</v>
       </c>
@@ -8929,6 +10032,18 @@
       </c>
       <c r="AI52" t="b">
         <f t="shared" si="6"/>
+        <v>1</v>
+      </c>
+      <c r="AK52" t="b">
+        <f t="shared" si="19"/>
+        <v>1</v>
+      </c>
+      <c r="AL52" t="b">
+        <f t="shared" si="20"/>
+        <v>1</v>
+      </c>
+      <c r="AM52" t="b">
+        <f t="shared" si="21"/>
         <v>1</v>
       </c>
       <c r="AR52" t="b">
@@ -8951,6 +10066,15 @@
         <f t="array" ref="G53">_xll.ExLibris.Json.GetJsonValueAsync($F$1,E53)</f>
         <v>45352</v>
       </c>
+      <c r="I53">
+        <v>45532</v>
+      </c>
+      <c r="J53" t="str">
+        <v>ACT/360</v>
+      </c>
+      <c r="K53">
+        <v>15000000</v>
+      </c>
       <c r="P53" t="str">
         <v>fixed_leg.cashflows.[3].fixed_rate</v>
       </c>
@@ -8966,6 +10090,15 @@
       <c r="U53">
         <v>45352</v>
       </c>
+      <c r="W53">
+        <v>45532</v>
+      </c>
+      <c r="X53" t="s">
+        <v>8</v>
+      </c>
+      <c r="Y53">
+        <v>15000000</v>
+      </c>
       <c r="AD53" t="s">
         <v>49</v>
       </c>
@@ -8982,6 +10115,18 @@
       </c>
       <c r="AI53" t="b">
         <f t="shared" si="6"/>
+        <v>1</v>
+      </c>
+      <c r="AK53" t="b">
+        <f t="shared" si="19"/>
+        <v>1</v>
+      </c>
+      <c r="AL53" t="b">
+        <f t="shared" si="20"/>
+        <v>1</v>
+      </c>
+      <c r="AM53" t="b">
+        <f t="shared" si="21"/>
         <v>1</v>
       </c>
       <c r="AR53" t="b">
@@ -9396,11 +10541,11 @@
         <v>44632</v>
       </c>
       <c r="AR67" t="b">
-        <f t="shared" ref="AR67:AS79" si="13">P67=AD67</f>
+        <f t="shared" ref="AR67:AS79" si="22">P67=AD67</f>
         <v>1</v>
       </c>
       <c r="AS67" t="b">
-        <f t="shared" si="13"/>
+        <f t="shared" si="22"/>
         <v>1</v>
       </c>
     </row>
@@ -9418,11 +10563,11 @@
         <v>44812</v>
       </c>
       <c r="AR68" t="b">
-        <f t="shared" si="13"/>
+        <f t="shared" si="22"/>
         <v>1</v>
       </c>
       <c r="AS68" t="b">
-        <f t="shared" si="13"/>
+        <f t="shared" si="22"/>
         <v>1</v>
       </c>
     </row>
@@ -9440,11 +10585,11 @@
         <v>44992</v>
       </c>
       <c r="AR69" t="b">
-        <f t="shared" si="13"/>
+        <f t="shared" si="22"/>
         <v>1</v>
       </c>
       <c r="AS69" t="b">
-        <f t="shared" si="13"/>
+        <f t="shared" si="22"/>
         <v>1</v>
       </c>
     </row>
@@ -9462,11 +10607,11 @@
         <v>45172</v>
       </c>
       <c r="AR70" t="b">
-        <f t="shared" si="13"/>
+        <f t="shared" si="22"/>
         <v>1</v>
       </c>
       <c r="AS70" t="b">
-        <f t="shared" si="13"/>
+        <f t="shared" si="22"/>
         <v>1</v>
       </c>
     </row>
@@ -9484,11 +10629,11 @@
         <v>45352</v>
       </c>
       <c r="AR71" t="b">
-        <f t="shared" si="13"/>
+        <f t="shared" si="22"/>
         <v>1</v>
       </c>
       <c r="AS71" t="b">
-        <f t="shared" si="13"/>
+        <f t="shared" si="22"/>
         <v>1</v>
       </c>
     </row>
@@ -9506,11 +10651,11 @@
         <v>45532</v>
       </c>
       <c r="AR72" t="b">
-        <f t="shared" si="13"/>
+        <f t="shared" si="22"/>
         <v>1</v>
       </c>
       <c r="AS72" t="b">
-        <f t="shared" si="13"/>
+        <f t="shared" si="22"/>
         <v>1</v>
       </c>
     </row>
@@ -9529,11 +10674,11 @@
         <v>45172</v>
       </c>
       <c r="AR74" t="b">
-        <f t="shared" si="13"/>
+        <f t="shared" si="22"/>
         <v>1</v>
       </c>
       <c r="AS74" t="b">
-        <f t="shared" si="13"/>
+        <f t="shared" si="22"/>
         <v>1</v>
       </c>
     </row>
@@ -9551,11 +10696,11 @@
         <v>44992</v>
       </c>
       <c r="AR75" t="b">
-        <f t="shared" si="13"/>
+        <f t="shared" si="22"/>
         <v>1</v>
       </c>
       <c r="AS75" t="b">
-        <f t="shared" si="13"/>
+        <f t="shared" si="22"/>
         <v>1</v>
       </c>
     </row>
@@ -9573,11 +10718,11 @@
         <v>45172</v>
       </c>
       <c r="AR76" t="b">
-        <f t="shared" si="13"/>
+        <f t="shared" si="22"/>
         <v>1</v>
       </c>
       <c r="AS76" t="b">
-        <f t="shared" si="13"/>
+        <f t="shared" si="22"/>
         <v>1</v>
       </c>
     </row>
@@ -9595,11 +10740,11 @@
         <v>8</v>
       </c>
       <c r="AR77" t="b">
-        <f t="shared" si="13"/>
+        <f t="shared" si="22"/>
         <v>1</v>
       </c>
       <c r="AS77" t="b">
-        <f t="shared" si="13"/>
+        <f t="shared" si="22"/>
         <v>1</v>
       </c>
     </row>
@@ -9617,11 +10762,11 @@
         <v>13000000</v>
       </c>
       <c r="AR78" t="b">
-        <f t="shared" si="13"/>
+        <f t="shared" si="22"/>
         <v>1</v>
       </c>
       <c r="AS78" t="b">
-        <f t="shared" si="13"/>
+        <f t="shared" si="22"/>
         <v>1</v>
       </c>
     </row>
@@ -9639,11 +10784,11 @@
         <v>1E-3</v>
       </c>
       <c r="AR79" t="b">
-        <f t="shared" si="13"/>
+        <f t="shared" si="22"/>
         <v>1</v>
       </c>
       <c r="AS79" t="b">
-        <f t="shared" si="13"/>
+        <f t="shared" si="22"/>
         <v>1</v>
       </c>
     </row>
@@ -9682,11 +10827,11 @@
       </c>
       <c r="F1" t="str" cm="1">
         <f t="array" ref="F1">_xll.ExLibris.Json.CreateJsonObjectAsync(E3:F6, EXLIBRIS_CONFIGURATION)</f>
-        <v>JsonObject:E022D8CD-4072-4F20-BB6D-9EB3A047AE3F</v>
+        <v>JsonObject:2689C2FA-2F6D-4A03-91A8-7BAC6D40ED38</v>
       </c>
       <c r="K1" t="str">
         <f>EXLIBRIS_CONFIGURATION</f>
-        <v>ExLibris.Core.ExLibrisConfiguration:309B6F05-E9D9-4A90-B78A-A8124E730131</v>
+        <v>ExLibris.Core.ExLibrisConfiguration:B757D65E-70E4-4BE1-AC2F-AD0EBE726B7C</v>
       </c>
     </row>
     <row r="2" spans="2:25" x14ac:dyDescent="0.4">
@@ -9756,7 +10901,7 @@
       </c>
       <c r="F6" t="str" cm="1">
         <f t="array" ref="F6">_xll.ExLibris.Json.CreateJsonArrayAsync(E8:J14, EXLIBRIS_CONFIGURATION)</f>
-        <v>JsonObject:FD6D4ACC-D566-422D-8354-506E7A48EA6C</v>
+        <v>JsonObject:F31AE2FF-4CCA-40E5-8DEF-3106A237C82C</v>
       </c>
       <c r="L6" t="s">
         <v>60</v>
@@ -10007,7 +11152,7 @@
       </c>
       <c r="I19" t="str" cm="1">
         <f t="array" ref="I19">_xll.ExLibris.Json.GetJsonValueAsync(F1,E6, EXLIBRIS_CONFIGURATION)</f>
-        <v>JsonObject:F3085FBE-9F79-46CE-9165-745350A21E70</v>
+        <v>JsonObject:614EAC64-A164-47D8-B2BA-9F9D8C0759A9</v>
       </c>
       <c r="P19" t="s">
         <v>12</v>
@@ -10043,7 +11188,7 @@
         <v>CP00001</v>
       </c>
       <c r="I20" t="str" cm="1">
-        <f t="array" ref="I20:N26">_xll.ExLibris.Json.GetJsonTableAsync(I19,,EXLIBRIS_CONFIGURATION)</f>
+        <f t="array" ref="I20:N26">_xll.ExLibris.Json.GetJsonTableAsync(I19,,,EXLIBRIS_CONFIGURATION)</f>
         <v>payment _date</v>
       </c>
       <c r="J20" t="str">
@@ -10729,7 +11874,7 @@
       </c>
       <c r="I28" t="str" cm="1">
         <f t="array" ref="I28">_xll.ExLibris.Json.GetJsonValueAsync(I19,"[2]", EXLIBRIS_CONFIGURATION)</f>
-        <v>JsonObject:45DE8A71-7DB4-4C8A-91FA-74E6271057AC</v>
+        <v>JsonObject:1F1EDFBE-2CE2-4991-9C98-F3F76E4B793C</v>
       </c>
       <c r="P28" t="s">
         <v>35</v>
@@ -10765,7 +11910,7 @@
         <v>2022-03-12</v>
       </c>
       <c r="I29" t="str" cm="1">
-        <f t="array" ref="I29:N30">_xll.ExLibris.Json.GetJsonTableAsync(I28,,EXLIBRIS_CONFIGURATION)</f>
+        <f t="array" ref="I29:N30">_xll.ExLibris.Json.GetJsonTableAsync(I28,,,EXLIBRIS_CONFIGURATION)</f>
         <v>payment _date</v>
       </c>
       <c r="J29" t="str">
@@ -10986,7 +12131,7 @@
       </c>
       <c r="I32" t="str" cm="1">
         <f t="array" ref="I32">_xll.ExLibris.Json.GetJsonValueAsync(F1,E6,EXLIBRIS_CONFIGURATION)</f>
-        <v>JsonObject:F3085FBE-9F79-46CE-9165-745350A21E70</v>
+        <v>JsonObject:614EAC64-A164-47D8-B2BA-9F9D8C0759A9</v>
       </c>
       <c r="P32" t="s">
         <v>177</v>
@@ -11023,7 +12168,7 @@
       </c>
       <c r="I33" t="str" cm="1">
         <f t="array" ref="I33">_xll.ExLibris.Json.SearchJsonArrayElementsAsync(I32,I8,I11,EXLIBRIS_CONFIGURATION)</f>
-        <v>JsonObject:50F505B9-A50D-416A-A11D-E9C4CCC85B68</v>
+        <v>JsonObject:6E4DB88E-191B-43CE-9B84-31D60AAFA0ED</v>
       </c>
       <c r="P33" t="s">
         <v>39</v>
@@ -11059,7 +12204,7 @@
         <v>2023-03-07</v>
       </c>
       <c r="I34" t="str" cm="1">
-        <f t="array" ref="I34:N36">_xll.ExLibris.Json.GetJsonTableAsync(I33,,EXLIBRIS_CONFIGURATION)</f>
+        <f t="array" ref="I34:N36">_xll.ExLibris.Json.GetJsonTableAsync(I33,,,EXLIBRIS_CONFIGURATION)</f>
         <v>payment _date</v>
       </c>
       <c r="J34" t="str">
@@ -11373,7 +12518,7 @@
       </c>
       <c r="I38" t="str" cm="1">
         <f t="array" ref="I38">_xll.ExLibris.Json.SearchJsonArrayElementsAsync(I32,J8,J11,EXLIBRIS_CONFIGURATION)</f>
-        <v>JsonObject:B32771EE-A881-4C5F-BEB9-6759F851ED5D</v>
+        <v>JsonObject:C0257BD0-DC6E-4852-AB2A-9C24A270EAF1</v>
       </c>
       <c r="P38" t="s">
         <v>178</v>
@@ -11409,7 +12554,7 @@
         <v>1.2000000000000001E-3</v>
       </c>
       <c r="I39" t="str" cm="1">
-        <f t="array" ref="I39:N40">_xll.ExLibris.Json.GetJsonTableAsync(I38,,EXLIBRIS_CONFIGURATION)</f>
+        <f t="array" ref="I39:N40">_xll.ExLibris.Json.GetJsonTableAsync(I38,,,EXLIBRIS_CONFIGURATION)</f>
         <v>payment _date</v>
       </c>
       <c r="J39" t="str">
@@ -11630,7 +12775,7 @@
       </c>
       <c r="I42" t="str" cm="1">
         <f t="array" ref="I42">_xll.ExLibris.Json.SearchJsonArrayElementsAsync(I32,J8,,EXLIBRIS_CONFIGURATION)</f>
-        <v>JsonObject:174C6349-530C-4DE9-8DB7-189DD28430E0</v>
+        <v>JsonObject:FB1D8EB7-FA68-42D7-9DB6-D3CA93BD59DA</v>
       </c>
       <c r="P42" t="s">
         <v>47</v>
@@ -11666,7 +12811,7 @@
         <v>ACT/360</v>
       </c>
       <c r="I43" t="str" cm="1">
-        <f t="array" ref="I43">_xll.ExLibris.Json.GetJsonTableAsync(I42,,EXLIBRIS_CONFIGURATION)</f>
+        <f t="array" ref="I43">_xll.ExLibris.Json.GetJsonTableAsync(I42,,,EXLIBRIS_CONFIGURATION)</f>
         <v/>
       </c>
       <c r="P43" t="s">
@@ -12184,7 +13329,7 @@
       </c>
       <c r="C2" t="str" cm="1">
         <f t="array" ref="C2">_xll.ExLibris.LoadConfigurationAsync(B6:C15)</f>
-        <v>ExLibris.Core.ExLibrisConfiguration:309B6F05-E9D9-4A90-B78A-A8124E730131</v>
+        <v>ExLibris.Core.ExLibrisConfiguration:B757D65E-70E4-4BE1-AC2F-AD0EBE726B7C</v>
       </c>
     </row>
     <row r="4" spans="2:6" s="4" customFormat="1" ht="18" x14ac:dyDescent="0.4">
@@ -12387,7 +13532,7 @@
     <row r="4" spans="2:10" x14ac:dyDescent="0.4">
       <c r="D4" t="str" cm="1">
         <f t="array" ref="D4">_xll.ExLibris.WebSockets.OpenWebSocketAsync("ws://localhost:10101",,E4)</f>
-        <v>ExLibris.Core.WebSockets.WebsocketClient:5B1E523E-555E-4404-96B3-3C764D3008A0</v>
+        <v>ExLibris.Core.WebSockets.WebsocketClient:FC8CD32E-B5EE-4B59-BF8C-2512FF6A7D9E</v>
       </c>
       <c r="E4" t="s">
         <v>94</v>
@@ -12416,7 +13561,7 @@
     <row r="5" spans="2:10" x14ac:dyDescent="0.4">
       <c r="D5" t="str" cm="1">
         <f t="array" ref="D5">_xll.ExLibris.WebSockets.OpenWebSocketAsync("ws://localhost:10101",,E5)</f>
-        <v>ExLibris.Core.WebSockets.WebsocketClient:A518D726-DC07-4306-BCB1-D0135534C7EC</v>
+        <v>ExLibris.Core.WebSockets.WebsocketClient:98D2FC76-FEF6-4D84-8DEF-A9099C946C06</v>
       </c>
       <c r="E5" t="s">
         <v>142</v>
@@ -12445,7 +13590,7 @@
     <row r="6" spans="2:10" x14ac:dyDescent="0.4">
       <c r="D6" t="str" cm="1">
         <f t="array" ref="D6">_xll.ExLibris.WebSockets.OpenWebSocketAsync("ws://localhost:10101",,E6)</f>
-        <v>ExLibris.Core.WebSockets.WebsocketClient:DBEA9D7A-51E0-4C64-BC61-FD2E5484DA2A</v>
+        <v>ExLibris.Core.WebSockets.WebsocketClient:60572BB0-D57F-4A28-A61B-A565815F3194</v>
       </c>
       <c r="E6" t="s">
         <v>143</v>
@@ -12474,7 +13619,7 @@
     <row r="7" spans="2:10" x14ac:dyDescent="0.4">
       <c r="D7" t="str" cm="1">
         <f t="array" ref="D7">_xll.ExLibris.WebSockets.OpenWebSocketAsync("ws://localhost:10101",,E7)</f>
-        <v>ExLibris.Core.WebSockets.WebsocketClient:9DC5558A-02DD-4C67-8851-A182FE9FED6F</v>
+        <v>ExLibris.Core.WebSockets.WebsocketClient:149A3688-4522-4337-8796-F87C8A42227D</v>
       </c>
       <c r="E7" t="s">
         <v>144</v>
@@ -12503,7 +13648,7 @@
     <row r="8" spans="2:10" x14ac:dyDescent="0.4">
       <c r="D8" t="str" cm="1">
         <f t="array" ref="D8">_xll.ExLibris.WebSockets.OpenWebSocketAsync("ws://localhost:10101",,E8)</f>
-        <v>ExLibris.Core.WebSockets.WebsocketClient:1CA6C4EE-A57C-44DF-9C79-13606AA3EBA2</v>
+        <v>ExLibris.Core.WebSockets.WebsocketClient:0AE14383-970D-4356-AA96-C4C2DED24B88</v>
       </c>
       <c r="E8" t="s">
         <v>145</v>
@@ -12569,11 +13714,11 @@
     <row r="5" spans="2:11" x14ac:dyDescent="0.4">
       <c r="B5" t="str" cm="1">
         <f t="array" ref="B5">_xll.ExLibris.WebAPIs.CreateHeadersAsync(B6:C10)</f>
-        <v>ExLibris.Core.WebAPIs.WebAPIHeaders:6D21A553-B5A3-4AAE-95D7-CF8B8DEA2C16</v>
+        <v>ExLibris.Core.WebAPIs.WebAPIHeaders:760CC286-9664-4A11-81DD-AC5873477A75</v>
       </c>
       <c r="H5" t="str" cm="1">
         <f t="array" ref="H5">_xll.ExLibris.Json.CreateJsonObjectAsync(H6:I11)</f>
-        <v>JsonObject:CC773D14-6DA7-4AE4-96D3-C02C76114111</v>
+        <v>JsonObject:26F9F0BF-9B62-4A0E-A353-6F9AB0289536</v>
       </c>
     </row>
     <row r="6" spans="2:11" x14ac:dyDescent="0.4">
@@ -13198,7 +14343,7 @@
     <row r="2" spans="2:4" x14ac:dyDescent="0.4">
       <c r="B2" t="str" cm="1">
         <f t="array" ref="B2">_xll.ExLibris.WebAPIs.CreateHeadersAsync(B3:C3)</f>
-        <v>ExLibris.Core.WebAPIs.WebAPIHeaders:A0A27A5E-8C97-4C45-967C-B54F4B58A126</v>
+        <v>ExLibris.Core.WebAPIs.WebAPIHeaders:99456C6A-DD30-4D3F-A155-84C89E618C48</v>
       </c>
     </row>
     <row r="3" spans="2:4" x14ac:dyDescent="0.4">
@@ -13224,7 +14369,7 @@
       </c>
       <c r="C6" t="str" cm="1">
         <f t="array" ref="C6">_xll.ExLibris.WebAPIs.GET(C5,B2)</f>
-        <v>ExLibris.Core.WebAPIs.Response:F72CC60D-61BA-42C7-89E1-5231EA610786</v>
+        <v>ExLibris.Core.WebAPIs.Response:7B6CE83E-1713-4AD2-BF20-B4CFC8A7502A</v>
       </c>
     </row>
     <row r="7" spans="2:4" x14ac:dyDescent="0.4">
@@ -13248,7 +14393,7 @@
     <row r="10" spans="2:4" x14ac:dyDescent="0.4">
       <c r="C10" t="str" cm="1">
         <f t="array" ref="C10">_xll.ExLibris.Json.CreateJsonObjectAsync(C8)</f>
-        <v>JsonObject:FB80924F-3D29-4993-A6F3-A4AE5BBF05AC</v>
+        <v>JsonObject:3818E816-2167-4F03-B522-8402A1114104</v>
       </c>
     </row>
     <row r="11" spans="2:4" x14ac:dyDescent="0.4">

</xml_diff>